<commit_message>
Modernize flagship fallacy entries
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4088beb924b14588"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rd39a76922e234f2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rafc964cff2114eac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbb06db31815a441b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R37f93d70b5094a44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R348c512875f343ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -321,7 +321,8 @@
         <x:v>The fact that you did not see me at your birthday party does not mean I was not there!</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>&lt;br /&gt;&amp;nbsp;&lt;br /&gt;&lt;blockquote&gt;&lt;i&gt;The absence of evidence it not evidence of absence.&lt;/i&gt;&lt;/blockquote&gt;This argument, attributed to Carl Sagan, is often invoked when claims of a god comes under scrutiny. While the absence of evidence is not proof of absence, it is, to varying degrees, evidence of absence. The degree of evidence an absence of evidence is for the absence of anything will depend on the context. If there is no evidence of thing &lt;i&gt;X&lt;/i&gt; in a location &lt;i&gt;Y&lt;/i&gt;, the degree that will constitute evidence for the absence of that thing depends upon how we substantiate the variables. Is &lt;i&gt;X&lt;/i&gt; a molecule, mouse or monster? Is &lt;i&gt;Y&lt;/i&gt; a cup, couch or continent?</x:v>
+        <x:v>The absence of evidence it not evidence of absence.
+This argument, attributed to Carl Sagan, is often invoked when claims of a god comes under scrutiny. While the absence of evidence is not proof of absence, it is, to varying degrees, evidence of absence. The degree of evidence an absence of evidence is for the absence of anything will depend on the context. If there is no evidence of thing X in a location Y, the degree that will constitute evidence for the absence of that thing depends upon how we substantiate the variables. Is X a molecule, mouse or monster? Is Y a cup, couch or continent?</x:v>
       </x:c>
       <x:c r="M2" t="str">
         <x:v>After a Harvard Medical School study on the effects of prayer on heart surgery patients showed no statistical advantage of prayer, it was argued that "the absence of evidence is not evidence of absence".</x:v>
@@ -399,7 +400,7 @@
         <x:v>The law of gravity says that two objects of mass attract each other, so when physicists say gravity can repel, they don't know what they're talking about.</x:v>
       </x:c>
       <x:c r="L4" t="str">
-        <x:v>In the gravity example, the very physicist who christened the "law of gravity" also believe it repels in some cases. Each law is only reliable to the extent of its predictive success, and may come with stipulations. This is a type of faulty generalization that arises when induction justifiably categorizes an event or state extremely improbable. The fallacy arises when we say something that is physically improbable is logically impossible. A more detailed treatment of faulty generalizations can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+        <x:v>In the gravity example, the very physicist who christened the "law of gravity" also believe it repels in some cases. Each law is only reliable to the extent of its predictive success, and may come with stipulations. This is a type of faulty generalization that arises when induction justifiably categorizes an event or state extremely improbable. The fallacy arises when we say something that is physically improbable is logically impossible. A more detailed treatment of faulty generalizations can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M4" t="str">
         <x:v>Consider the Law of Reciprocity. This law describes how healthy societies find cohesion when a critical level of altruism is reached among its constituents. However, its descriptive power does not in any way imply that societies will actualize cohesion based on altruism.</x:v>
@@ -408,7 +409,7 @@
         <x:v>The Law of Diminishing Returns is another good example. This law is an inductive generalization from our economic interactions. This law does not constrain economics, nor is prior to it, but rather economic phenomena restrict our formulation of economic laws.</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>Moore's Law which states that the number of transistors that can be inexpensively placed on a circuit board doubles about every 2 years is another example. Due to physical constraints, this law is expected to fail at some point. This is also a type of &lt;a href="http://logfall.wordpress.com/human-standard-fallacy/"&gt;human standard fallacy&lt;/a&gt; in which an artifact of human abstraction is given more authority than is warranted.</x:v>
+        <x:v>Moore's Law which states that the number of transistors that can be inexpensively placed on a circuit board doubles about every 2 years is another example. Due to physical constraints, this law is expected to fail at some point. This is also a type of human standard fallacy in which an artifact of human abstraction is given more authority than is warranted.</x:v>
       </x:c>
       <x:c r="P4" t="str"/>
       <x:c r="Q4" t="str"/>
@@ -441,21 +442,25 @@
       <x:c r="H5" t="str"/>
       <x:c r="I5" t="str"/>
       <x:c r="J5" t="str">
-        <x:v>Attacking the person instead of the argument.</x:v>
+        <x:v>Occurs when someone treats an attack on a person's character, motives, class, or biography as if it were a refutation of that person's argument.</x:v>
       </x:c>
       <x:c r="K5" t="str">
-        <x:v>What would you know about economics? You filed for bankruptcy last year!</x:v>
+        <x:v>An economist presents data against a tariff proposal, and the reply is: 'Why listen to her? She is an Ivy League elitist who has never worked a real job.'</x:v>
       </x:c>
       <x:c r="L5" t="str">
-        <x:v>"Ad hominem" means "to the individual", and is often used as either a distraction from the main argument, or as a hostile emotional release against an opponent. This does not invalidate any argument it accompanies, but is generally considered poor form.</x:v>
-      </x:c>
-      <x:c r="M5" t="str"/>
-      <x:c r="N5" t="str"/>
+        <x:v>Character can matter when credibility itself is at issue, such as fraud, conflicts of interest, or proven dishonesty. The fallacy appears when those personal facts are used instead of answering the actual reasons or evidence.</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>In the June 27, 2024 Biden-Trump debate, policy exchanges repeatedly slid into attacks on each candidate's age, criminal exposure, or family rather than sustained engagement with the argument on the table.</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>Online discussion of climate, vaccines, and AI policy often substitutes labels such as 'shill,' 'grifter,' or 'elitist' for any serious response to the evidence.</x:v>
+      </x:c>
       <x:c r="O5" t="str"/>
       <x:c r="P5" t="str"/>
       <x:c r="Q5" t="str"/>
       <x:c r="R5" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -485,11 +490,13 @@
         <x:v>I don't eat meat. People who eat meat have no compassion. Therefore, I have compassion.</x:v>
       </x:c>
       <x:c r="L6" t="str">
-        <x:v>&lt;br /&gt;&amp;nbsp;&lt;br /&gt;&lt;blockquote&gt;If A ⊄ B and B ⊄ C then A ⊂ C.&lt;/blockquote&gt;
-This fallacy is made clear when we follow this same form and say "If I'm not a goose, and geese don't play bingo, therefore I play bingo.".</x:v>
+        <x:v>If A ⊄ B and B ⊄ C then A ⊂ C.
+This fallacy is made clear when we follow this same form and say "If I'm not a goose, and geese don't play bingo, therefore I play bingo."</x:v>
       </x:c>
       <x:c r="M6" t="str">
-        <x:v>This fallacy is often a part of tribalism in which the following type of argument is implicitly made.&lt;blockquote&gt;We don't do that. &lt;br /&gt;People who do that are bad. &lt;br /&gt;Therefore, we are good.&lt;/blockquote&gt;.</x:v>
+        <x:v>This fallacy is often a part of tribalism in which the following type of argument is implicitly made.We don't do that.
+People who do that are bad.
+Therefore, we are good.</x:v>
       </x:c>
       <x:c r="N6" t="str"/>
       <x:c r="O6" t="str"/>
@@ -528,8 +535,11 @@
         <x:v>My new neighbor looked so happy, I knew he had either a girlfriend or a wife. He told me he has a wife, so I know he does not have a girlfriend.</x:v>
       </x:c>
       <x:c r="L7" t="str">
-        <x:v>&lt;br /&gt;&amp;nbsp;&lt;br /&gt;&lt;blockquote&gt;P or Q &lt;br /&gt; P &lt;br /&gt;Therefore, not Q &lt;/blockquote&gt;
-This fallacy is made clear when when follow this same form and say "To have a girlfriend like Tom's, you have to be either rich or famous. He's rich, so he can't be famous." &lt;br /&gt;Note that this fallacy does not hold for exclusive disjunctions where P and Q cannot both be true.</x:v>
+        <x:v>P or Q
+P
+Therefore, not Q
+This fallacy is made clear when when follow this same form and say "To have a girlfriend like Tom's, you have to be either rich or famous. He's rich, so he can't be famous."
+Note that this fallacy does not hold for exclusive disjunctions where P and Q cannot both be true.</x:v>
       </x:c>
       <x:c r="M7" t="str">
         <x:v>Some politicians might argue that, to lower the deficit, we'll need to either cut programs or raise taxes, then suggest that, since they've already cut taxes, cutting programs wouldn't also contribute to alleviating the problem.</x:v>
@@ -571,10 +581,12 @@
         <x:v>Whenever it rains, people carry umbrellas. People are carrying umbrellas, so it must be raining.</x:v>
       </x:c>
       <x:c r="L8" t="str">
-        <x:v>&lt;br /&gt;&amp;nbsp;&lt;br /&gt;&lt;blockquote&gt;If P, then Q &lt;br /&gt;Q &lt;br /&gt;Therefore, P&lt;/blockquote&gt;.</x:v>
+        <x:v>If P, then Q
+Q
+Therefore, P.</x:v>
       </x:c>
       <x:c r="M8" t="str">
-        <x:v>If Tom says "All ducks can fly", and Bob responds "Not true. Bats can fly and they're not ducks", Bob has fallaciously affirmed the consequent of Tom's statement as if Tom had said "This animal can fly and is therefore a duck.".</x:v>
+        <x:v>If Tom says "All ducks can fly", and Bob responds "Not true. Bats can fly and they're not ducks", Bob has fallaciously affirmed the consequent of Tom's statement as if Tom had said "This animal can fly and is therefore a duck."</x:v>
       </x:c>
       <x:c r="N8" t="str"/>
       <x:c r="O8" t="str"/>
@@ -697,25 +709,25 @@
         <x:v>ad verecundiam</x:v>
       </x:c>
       <x:c r="J11" t="str">
-        <x:v>Occurs when an claim is deemed true because of the position, authority or esteem of the person asserting it.</x:v>
+        <x:v>Occurs when someone treats an authority's endorsement as if it settled the issue, even when the authority is unqualified, the field is divided, or the claim still requires evidence.</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>My sociology professor says globalization has had a net negative effect on humanity, so it is obviously true.</x:v>
+        <x:v>A wellness influencer says a supplement works because a famous surgeon on a podcast called it 'a game changer,' so listeners treat the endorsement as proof.</x:v>
       </x:c>
       <x:c r="L11" t="str">
-        <x:v>If an authority gained their status or position due to a track record of success, then we have more warrant to prioritize consideration of their arguments. However, it is their actual arguments that must ultimately be considered. Taking credible authorities at their word is a useful heuristic, but it is a weaker form of evidence that is no real substitute for the actual arguments those authorities make.&lt;br /&gt;&amp;nbsp;&lt;br /&gt;&lt;blockquote&gt;&lt;i&gt;[I]t is not &lt;i&gt;what&lt;/i&gt; the man of science believes that distinguishes him, but &lt;i&gt;how&lt;/i&gt; and &lt;i&gt;why&lt;/i&gt; he believes it. His beliefs are tentative, not dogmatic; they are based on evidence, not on authority or intuition.&lt;/i&gt;&lt;br /&gt;&lt;sub&gt;Bertrand Russell, &lt;i&gt;A History of Western Philosophy&lt;/i&gt; (Book-of-the-Month Club, 1995), p. 527. &lt;/sub&gt;&lt;/blockquote&gt;.</x:v>
+        <x:v>Expert testimony can be good evidence when the authority is relevant, the expertise is genuine, and the claim fits the expert consensus. The fallacy appears when prestige replaces argument.</x:v>
       </x:c>
       <x:c r="M11" t="str">
-        <x:v>If the mayor of your town is in favor of legalizing marijuana, that is, in itself, not an argument in favor of legalizing marijuana.</x:v>
+        <x:v>Debates about nutrition, vaccines, crypto, and AI frequently lean on celebrity experts or founders speaking outside their strongest field, while the underlying studies and uncertainties get little attention.</x:v>
       </x:c>
       <x:c r="N11" t="str">
-        <x:v>If your hitherto reliable doctor recommends a certain type of cold medicine, you are warranted in accepting his recommendation. This does not, however, substitute for doing your own research if you have the time.</x:v>
+        <x:v>In public discussion of AI safety and capability, people often present a famous CEO's confidence level as if it were itself a substitute for technical evidence or broad expert agreement.</x:v>
       </x:c>
       <x:c r="O11" t="str"/>
       <x:c r="P11" t="str"/>
       <x:c r="Q11" t="str"/>
       <x:c r="R11" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -799,7 +811,7 @@
         <x:v>It would be awesome to know that we were not alone in the universe. I can't help but believe space aliens exist out there somewhere.</x:v>
       </x:c>
       <x:c r="L13" t="str">
-        <x:v>This fallacy has itself been categorized as a tactical fallacy, but is a parent category for specific appeals to emotion that are not listed among the primary fallacies. &lt;ul&gt;&lt;li&gt;&lt;a href="http://logfall.wordpress.com/?s=*emot"&gt;All appeal to emotion fallacies&lt;/a&gt;&lt;/li&gt;&lt;/ul&gt;.</x:v>
+        <x:v>This fallacy has itself been categorized as a tactical fallacy, but is a parent category for specific appeals to emotion that are not listed among the primary fallacies. - All appeal to emotion fallacies.</x:v>
       </x:c>
       <x:c r="M13" t="str"/>
       <x:c r="N13" t="str"/>
@@ -971,7 +983,8 @@
         <x:v>Birds are monogamous. Therefore, humans should also be monogamous.</x:v>
       </x:c>
       <x:c r="L17" t="str">
-        <x:v>It does not take much exploration of nature to realize that it is not a very coherent or desirable standard for human conduct. Nor is nature, as is, very amenable to human survival. This is why medicine perennially combats the influenza virus, and would eradicate it if possible. Interestingly, the most "natural" of all actions inherent to life is the striving for survival. This puts humans at odds with the rest of nature and what is "natural". This is why we ingest neither natural hemlock nor synthetic poisons.&lt;br /&gt;&lt;br /&gt;In many cases, once the act that is deemed "unnatural" is scrutinized, it is discovered that the act is merely emotionally unpalatable to the person making the categorization.</x:v>
+        <x:v>It does not take much exploration of nature to realize that it is not a very coherent or desirable standard for human conduct. Nor is nature, as is, very amenable to human survival. This is why medicine perennially combats the influenza virus, and would eradicate it if possible. Interestingly, the most "natural" of all actions inherent to life is the striving for survival. This puts humans at odds with the rest of nature and what is "natural". This is why we ingest neither natural hemlock nor synthetic poisons.
+In many cases, once the act that is deemed "unnatural" is scrutinized, it is discovered that the act is merely emotionally unpalatable to the person making the categorization.</x:v>
       </x:c>
       <x:c r="M17" t="str">
         <x:v>Some claim that genetically modified crops are "wrong" for the sole reason that they are not what nature has naturally produced. There may be good reason for caution in growing genetically-modified crops, but the fact that they are merely "unnatural" is not good reason.</x:v>
@@ -1103,7 +1116,7 @@
         <x:v>He can be trusted due to his humble upbringing in a one-room cabin deep in the mountains.</x:v>
       </x:c>
       <x:c r="L20" t="str">
-        <x:v>The converse of this fallacy is the &lt;a href="logfall.wordpress.com/appeal-to-wealth/"&gt;appeal to wealth&lt;/a&gt; fallacy.</x:v>
+        <x:v>The converse of this fallacy is the appeal to wealth fallacy.</x:v>
       </x:c>
       <x:c r="M20" t="str">
         <x:v>The humble beginnings of many political candidates are often emphasized in an attempt to get the common citizen to identify with the candidate.</x:v>
@@ -1315,7 +1328,7 @@
         <x:v>If your ideas had any real merit, you'd be rich by now.</x:v>
       </x:c>
       <x:c r="L25" t="str">
-        <x:v>The converse of this fallacy is the &lt;a href="logfall.wordpress.com/appeal-to-poverty/"&gt;appeal to poverty&lt;/a&gt; fallacy.</x:v>
+        <x:v>The converse of this fallacy is the appeal to poverty fallacy.</x:v>
       </x:c>
       <x:c r="M25" t="str">
         <x:v>The financial success of an individual is often cited as evidence for their competency to take the helm of additional ventures, some of which may require skills other than what a successful business person can offer.</x:v>
@@ -1397,7 +1410,8 @@
         <x:v>Fairies must exist since we've seen no evidence falsifying their existence.</x:v>
       </x:c>
       <x:c r="L27" t="str">
-        <x:v>Phrases that often accompany this fallacy include "What are the odds!" and "Explain that!" The inability of the (or a particular) human brain to grasp the stochastic or conceptual complexities of a particular concept do not warrant the introduction of magic or a god or luck as an explanation.&lt;hr /&gt;Note that there is warrant to dismiss out-of-hand claims that are logically or physically impossible. If I claim I possess a square triangle, or a flying reindeer, you are warranted in stating unequivocally that I am wrong.</x:v>
+        <x:v>Phrases that often accompany this fallacy include "What are the odds!" and "Explain that!" The inability of the (or a particular) human brain to grasp the stochastic or conceptual complexities of a particular concept do not warrant the introduction of magic or a god or luck as an explanation.
+Note that there is warrant to dismiss out-of-hand claims that are logically or physically impossible. If I claim I possess a square triangle, or a flying reindeer, you are warranted in stating unequivocally that I am wrong.</x:v>
       </x:c>
       <x:c r="M27" t="str">
         <x:v>Some say we are warranted in believing that the Loch Ness Monster exists since there is no evidence to the contrary.</x:v>
@@ -1487,7 +1501,7 @@
         <x:v>Because my opponent failed to address my point, my point is validated.</x:v>
       </x:c>
       <x:c r="L29" t="str">
-        <x:v>If a point is not addressed, rarely does it become anything other than an unaddressed point. However, this is context-dependent. If you see a vampire sitting across from you on the subway, and none of the other passengers seem interested, you might first consider what medication you might have taken that morning before wielding your wooden stake since the silence of the other passengers in such a setting would be unusual. The key question to ask is "How unusual is this silence?".</x:v>
+        <x:v>If a point is not addressed, rarely does it become anything other than an unaddressed point. However, this is context-dependent. If you see a vampire sitting across from you on the subway, and none of the other passengers seem interested, you might first consider what medication you might have taken that morning before wielding your wooden stake since the silence of the other passengers in such a setting would be unusual. The key question to ask is "How unusual is this silence?"</x:v>
       </x:c>
       <x:c r="M29" t="str">
         <x:v>The disinterest and subsequent silence of doctors on the claims of dubious medial remedies is often spun to imply their tacit support, or at minimum, their lack of opposition.</x:v>
@@ -1668,7 +1682,7 @@
       </x:c>
       <x:c r="L33" t="str">
         <x:v>There may, however, be a relevant association between two qualities. If, for example, you note that pianists have long fingers, there may be a causal relationship between long fingers and pianists, though this needs to be substantiated with evidence and argumentation.
-This is a type of proof by example fallacy. A more detailed treatment of proof by example fallacies can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+This is a type of proof by example fallacy. A more detailed treatment of proof by example fallacies can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M33" t="str">
         <x:v>If you argue that, because Japanese are polite, they would never push each other, you have not seen a rush hour subway train in Tokyo. Pushing does not necessarily entail impoliteness..</x:v>
@@ -1708,11 +1722,11 @@
         <x:v>My father Is 3 meters tall. Your father is only 1 meter tall. Therefore my father is taller than your father.</x:v>
       </x:c>
       <x:c r="L34" t="str">
-        <x:v>This fallacy is often accompanies by a phrase such as "Trust me." It might be considered a self-referential &lt;a href="http://logfall.wordpress.com/appeal-to-authority/"&gt;appeal to authority&lt;/a&gt;. A more rigorous and constrained discussion might allow you to ask "What is you evidence for that claim?" However, when bare assertions are constantly thrown out as red herrings, it may be best to abandon any hope of real dialog. &lt;blockquote&gt;"&lt;i&gt;When I use a word" Humpty Dumpty said, "...it means just what I choose it to mean-neither more nor less.&lt;/i&gt;"&lt;br /&gt;
-&lt;sup&gt;Lewis Carroll, Through the Looking Glass. &lt;/sup&gt;&lt;/blockquote&gt;.</x:v>
+        <x:v>This fallacy is often accompanies by a phrase such as "Trust me." It might be considered a self-referential appeal to authority. A more rigorous and constrained discussion might allow you to ask "What is you evidence for that claim?" However, when bare assertions are constantly thrown out as red herrings, it may be best to abandon any hope of real dialog. "When I use a word" Humpty Dumpty said, "...it means just what I choose it to mean-neither more nor less."
+Lewis Carroll, Through the Looking Glass.</x:v>
       </x:c>
       <x:c r="M34" t="str">
-        <x:v>Many economic or political arguments begin with bare assertions such as "The economy can't grow without tax breaks, so we need to...".</x:v>
+        <x:v>Many economic or political arguments begin with bare assertions such as "The economy can't grow without tax breaks, so we need to..."</x:v>
       </x:c>
       <x:c r="N34" t="str"/>
       <x:c r="O34" t="str"/>
@@ -1783,27 +1797,25 @@
         <x:v>petitio principii</x:v>
       </x:c>
       <x:c r="J36" t="str">
-        <x:v>Occurs when the conclusion of an argument is implicitly or explicitly assumed in one of the premises.</x:v>
+        <x:v>Occurs when an argument quietly assumes the very point it is supposed to prove, so the conclusion is built into the premises.</x:v>
       </x:c>
       <x:c r="K36" t="str">
-        <x:v>This medicine will definitely make you well since it can cure your disease.</x:v>
+        <x:v>This source is trustworthy because it tells the truth, and we know it tells the truth because it is a trustworthy source.</x:v>
       </x:c>
       <x:c r="L36" t="str">
-        <x:v>This fallacy employs circularity, and is usually a disguised tautology.</x:v>
+        <x:v>Circularity can be obvious, but it is often hidden behind rewording, loaded descriptions, or a chain of claims that loops back to the start. The argument feels like support has been offered when the conclusion has only been restated.</x:v>
       </x:c>
       <x:c r="M36" t="str">
-        <x:v>It's been argued that p1) holy books claim that a god can perform miracles, but p2) miracles are impossible, and C) therefore the holy books are wrong. This is begging the question in that you are essentially saying even though it is claimed that miracles are possible, miracles are not possible. A more precise definition of "miracle" might be called for here, then a demonstration of why p2 is true, perhaps not an easy task.</x:v>
+        <x:v>Conspiracy-style reasoning often treats the absence of confirming evidence as proof that the conspiracy is powerful enough to hide the evidence, which assumes the conclusion inside the explanation.</x:v>
       </x:c>
       <x:c r="N36" t="str">
-        <x:v>Some might beg the question by arguing that abortion is the unjustified killing of a human being and is therefore murder. Murder is illegal. So abortion should be made illegal.</x:v>
-      </x:c>
-      <x:c r="O36" t="str">
-        <x:v>Others might beg the question by arguing "Paranormal phenomena exist because I have had experiences that have transcended what is normal.".</x:v>
-      </x:c>
+        <x:v>Debates about 'real journalism' or 'real science' sometimes define the trustworthy outlet or institution as whichever one already agrees with the speaker's preferred view.</x:v>
+      </x:c>
+      <x:c r="O36" t="str"/>
       <x:c r="P36" t="str"/>
       <x:c r="Q36" t="str"/>
       <x:c r="R36" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -1833,7 +1845,7 @@
         <x:v>Bankers are jerks, and because my neighbor is a banker, he must be a jerk.</x:v>
       </x:c>
       <x:c r="L37" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M37" t="str">
         <x:v>If you learn that you have a tumor, the fact that many tumors are malignant, inoperable and fatal does not mean that you should despair since many tumors can be successfully treated. More information about the type and stage of the tumor is needed before any conclusions can be drawn about your particular tumor.</x:v>
@@ -1875,7 +1887,7 @@
         <x:v>Bankers are nice people, and since my neighbor is a banker, he must be a nice guy.</x:v>
       </x:c>
       <x:c r="L38" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M38" t="str"/>
       <x:c r="N38" t="str"/>
@@ -1949,25 +1961,25 @@
       <x:c r="H40" t="str"/>
       <x:c r="I40" t="str"/>
       <x:c r="J40" t="str">
-        <x:v>Pointing out individual cases or data that seem to confirm a particular position, while ignoring cases or data that may contradict that position.</x:v>
+        <x:v>Occurs when someone selects only the evidence that supports a conclusion and ignores a wider body of evidence that weakens, qualifies, or reverses it.</x:v>
       </x:c>
       <x:c r="K40" t="str">
-        <x:v>I found 2 statistical studies that conclude violent video games do not actually increase violence among children. That's proof enough for me!</x:v>
+        <x:v>A commentator cites one favorable month of inflation data as proof that the economy has fully recovered while ignoring the broader trend, wages, and household costs.</x:v>
       </x:c>
       <x:c r="L40" t="str">
-        <x:v>How many studies on violent video games have been conducted, and why are the others not included for a balanced assessment? This fallacy is similar to the &lt;a href="http://logfall.wordpress.com/sharpshooter-fallacy/"&gt;sharpshooter fallacy&lt;/a&gt;.</x:v>
+        <x:v>Cherry picking can involve hand-picked dates, unusual baselines, isolated anecdotes, or a single study taken out of a larger research picture. The defect is not using examples, but using a biased sample as if it were representative.</x:v>
       </x:c>
       <x:c r="M40" t="str">
-        <x:v>It is often claimed that the troubles someone experiences in life are due to some god's response to their ungodliness. These claims are made while ignoring the troubles of "godly" people. Pat Robertson claimed that the earthquake in Haiti was due to the Haitians making a pact with the devil years earlier.</x:v>
+        <x:v>After the September 10, 2024 Harris-Trump debate, both campaigns highlighted only the slices of jobs and manufacturing statistics that favored their own record while skipping the broader timeline.</x:v>
       </x:c>
       <x:c r="N40" t="str">
-        <x:v>When examining the the 10 years between 1998 and 2007 a 0.3-degree cooling trend in the average global temperature can be inferred. However, if we instead shift the decade to encompass the years 1997 to 2006, we see a 0.6-degree warming trend. Picking either span of 10 years to defend your position on global warming is fallacious.</x:v>
+        <x:v>Climate arguments often choose a starting year with an unusually hot or cool baseline so that a short graph looks flat or dramatic even when the longer record points elsewhere.</x:v>
       </x:c>
       <x:c r="O40" t="str"/>
       <x:c r="P40" t="str"/>
       <x:c r="Q40" t="str"/>
       <x:c r="R40" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2001,7 +2013,7 @@
         <x:v>Why must we accept medieval art as having any value when it emerged from the same period in which people burned witches and believed in fairies?</x:v>
       </x:c>
       <x:c r="L41" t="str">
-        <x:v>This is a type of faulty generalization since the error is over-generalizing from a period of several wrong concepts to concluding that all concepts within that period were wrong. A more detailed treatment of faulty generalizations can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+        <x:v>This is a type of faulty generalization since the error is over-generalizing from a period of several wrong concepts to concluding that all concepts within that period were wrong. A more detailed treatment of faulty generalizations can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M41" t="str">
         <x:v>Many early doctors held superstitions that would make us wary of visiting their office were they alive and holding the same beliefs today. This does not mean their practice of medicine was worthless for those alive in their day..</x:v>
@@ -2091,7 +2103,7 @@
         <x:v>Paper money can be exchanged. An economy is composed of paper money, so an economy can be exchanged.</x:v>
       </x:c>
       <x:c r="L43" t="str">
-        <x:v>This is the converse of the &lt;a href="http://logfall.wordpress.com/division-fallacy/"&gt;division fallacy&lt;/a&gt;.</x:v>
+        <x:v>This is the converse of the division fallacy.</x:v>
       </x:c>
       <x:c r="M43" t="str">
         <x:v>Were someone to argue "The average Canadian makes only 90% of what the average American makes, so Canada's GDP is 90% of the GDP of the U.S.", they would be committing the composition fallacy.</x:v>
@@ -2134,7 +2146,8 @@
         <x:v>This fallacy results from esteeming certainty as an objective validation of a proposition rather than as an emotion that could be misguided. Sometimes it is an emotional certainty that prevents the emotional pain that might result from following the evidence into disbelief, and other times it is triggered by a legitimate intuition that results in an emotional snowball of certainty that does not assess the possible evidential clues hidden in the intuition for validity.</x:v>
       </x:c>
       <x:c r="M44" t="str">
-        <x:v>Theists often conflate the emotional confidence derived from other emotions such as peace and love with evidence for the existence of their god. This essentially makes belief circular; "I know what I know".&lt;br /&gt;[&lt;a href="http://speeches.byu.edu/reader/reader.php?id=10547"&gt;Example&lt;/a&gt;].</x:v>
+        <x:v>Theists often conflate the emotional confidence derived from other emotions such as peace and love with evidence for the existence of their god. This essentially makes belief circular; "I know what I know".
+[Example].</x:v>
       </x:c>
       <x:c r="N44" t="str"/>
       <x:c r="O44" t="str"/>
@@ -2218,13 +2231,18 @@
         <x:v>Those with faith in some form of holy scriptures often accuse each other of contextomy. This is probably more a function of the vagueness of the context which allows for multiple interpretations.</x:v>
       </x:c>
       <x:c r="M46" t="str">
-        <x:v>The commander of British forces in Afghanistan, Mark Carleton-Smith said the following.&lt;blockquote&gt;"We're not going to win this war. It's about reducing it to a manageable level of insurgency that's not a strategic threat and can be managed by the Afghan army."&lt;/blockquote&gt;Only the first line was quoted by some media outlets, distorting the true intention of the commander.</x:v>
+        <x:v>The commander of British forces in Afghanistan, Mark Carleton-Smith said the following."We're not going to win this war. It's about reducing it to a manageable level of insurgency that's not a strategic threat and can be managed by the Afghan army."
+Only the first line was quoted by some media outlets, distorting the true intention of the commander.</x:v>
       </x:c>
       <x:c r="N46" t="str">
-        <x:v>The following is a quote by Charles Darwin.&lt;blockquote&gt;"Why then is not every geological formation and every stratum full of such intermediate links? Geology assuredly does not reveal any such finely-graduated organic chain; and this, perhaps, is the most obvious and serious objection which can be urged against the theory. "&lt;/blockquote&gt;Taken out of context, this quote is easily perceived to be Darwin doubting his own theory. However, Darwin continued...&lt;blockquote&gt;"The explanation lies, as I believe, in the extreme imperfection of the geological record. In the first place, it should always be borne in mind what sort of intermediate forms must, on the theory, have formerly existed... "&lt;/blockquote&gt;.</x:v>
+        <x:v>The following is a quote by Charles Darwin."Why then is not every geological formation and every stratum full of such intermediate links? Geology assuredly does not reveal any such finely-graduated organic chain; and this, perhaps, is the most obvious and serious objection which can be urged against the theory. "
+Taken out of context, this quote is easily perceived to be Darwin doubting his own theory. However, Darwin continued..."The explanation lies, as I believe, in the extreme imperfection of the geological record. In the first place, it should always be borne in mind what sort of intermediate forms must, on the theory, have formerly existed... ".</x:v>
       </x:c>
       <x:c r="O46" t="str">
-        <x:v>Consider this bible verse.&lt;blockquote&gt; Hosea 11:1 "When Israel was a child, I loved him, and out of Egypt I called my son."&lt;/blockquote&gt;Now note how Matthew later unequivocally denotes this verse in Hosea as a messianic prophecy. He is refering to Jesus' time in Egypt when he writes...&lt;blockquote&gt; Matthew 2:15 "And was there until the death of Herod: that it might be fulfilled which was spoken of the Lord by the prophet, saying, Out of Egypt have I called my son.'"&lt;/blockquote&gt;But now let's return to the very next verse in Hosea.&lt;blockquote&gt; Hosea 11:2 "But the more I called Israel, the further they went from me. They sacrificed to the Baals and they burned incense to images."&lt;/blockquote&gt;Unless you want to say Jesus sacrificed to the Baals, you've got to say Matthew took this verse out of context.</x:v>
+        <x:v>Consider this bible verse. Hosea 11:1 "When Israel was a child, I loved him, and out of Egypt I called my son."
+Now note how Matthew later unequivocally denotes this verse in Hosea as a messianic prophecy. He is refering to Jesus' time in Egypt when he writes... Matthew 2:15 "And was there until the death of Herod: that it might be fulfilled which was spoken of the Lord by the prophet, saying, Out of Egypt have I called my son.'"
+But now let's return to the very next verse in Hosea. Hosea 11:2 "But the more I called Israel, the further they went from me. They sacrificed to the Baals and they burned incense to images."
+Unless you want to say Jesus sacrificed to the Baals, you've got to say Matthew took this verse out of context.</x:v>
       </x:c>
       <x:c r="P46" t="str"/>
       <x:c r="Q46" t="str"/>
@@ -2260,7 +2278,7 @@
         <x:v>Rejecting an argument on the grounds that one of it's concepts cannot be defined discretely into a precise category.</x:v>
       </x:c>
       <x:c r="K47" t="str">
-        <x:v>You can't claim that your backpack is heavy until you give me a precise definition of "heavy.".</x:v>
+        <x:v>You can't claim that your backpack is heavy until you give me a precise definition of "heavy."</x:v>
       </x:c>
       <x:c r="L47" t="str">
         <x:v>This fallacy highlights the need to employ terms that are as precise and quantified as possible. The fallacy is not always on the side of the person suggesting a proposition has no meaning until imprecise terms are defined. Sometime the burden of clarification is on the party who is making a claim. Claims can be so imprecise as to be impotent.</x:v>
@@ -2301,27 +2319,25 @@
         <x:v>cum hoc ergo propter hoc</x:v>
       </x:c>
       <x:c r="J48" t="str">
-        <x:v>Occurs when a correlation found between two variables is presumed to demonstrate a causal relationship.</x:v>
+        <x:v>Occurs when someone treats a correlation, coincidence, or time pattern as if it already established that one factor caused the other.</x:v>
       </x:c>
       <x:c r="K48" t="str">
-        <x:v>Children who eat breakfast have higher grades, so eating breakfast causes higher grades.</x:v>
+        <x:v>A school adds an AI tutoring tool and test scores rise the next semester, so the district concludes that the tool caused the improvement without ruling out teacher changes, cohort differences, or extra tutoring time.</x:v>
       </x:c>
       <x:c r="L48" t="str">
-        <x:v>It may be that there is a 3rd factor causing both higher grades and eating breakfast such as more responsible parents who help children with homework as well as make sure they eat breakfast. While correlation is evidence for causation, especially when other factors have been controlled for, moving from correlation to causation demands a rigorous scientific protocol.</x:v>
+        <x:v>Correlations matter because they can reveal patterns worth investigating. The fallacy is jumping straight from 'these moved together' to 'this caused that' without checking mechanisms, timing, controls, or alternative explanations.</x:v>
       </x:c>
       <x:c r="M48" t="str">
-        <x:v>It has been argued that religious belief is what has made America economically strong, and, conversely, that a lack of religious belief is what keeps crime rates so low in Japan. Neither claim is warranted if merely based on the coexistence of the 2 variables cited.</x:v>
+        <x:v>Claims about teen mental health and social media often move too quickly from parallel trend lines to a settled single-cause story, even though researchers still debate the size, direction, and mechanisms of the effect.</x:v>
       </x:c>
       <x:c r="N48" t="str">
-        <x:v>It seems quite clear that people who eat diet food are heavier than those who don't. What can we say about any possible arrow of causation between diet food and heavier people? Is there causation? Which direction is the causation? Is it necessarily uni-directional?</x:v>
-      </x:c>
-      <x:c r="O48" t="str">
-        <x:v>It has been claimed that people with red cars drive faster than people with blue cars. What is it about the color red that causes faster driving. Or is it that more aggressive personalities like both red and speed. Or is possible that the data used to conclude that drivers of red cars drive faster than blue cars is taken from a biased source? Do police target red cars more than they do blue cars, thereby skewing the data?</x:v>
-      </x:c>
+        <x:v>Political messaging about crime, immigration, inflation, or schooling frequently points to two trends moving together and treats that alone as proof of causation.</x:v>
+      </x:c>
+      <x:c r="O48" t="str"/>
       <x:c r="P48" t="str"/>
       <x:c r="Q48" t="str"/>
       <x:c r="R48" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2431,7 +2447,7 @@
         <x:v>Can you prove I'm not wearing an invisible hat?</x:v>
       </x:c>
       <x:c r="L51" t="str">
-        <x:v>Similar to "negative proof fallacy.".</x:v>
+        <x:v>Similar to "negative proof fallacy."</x:v>
       </x:c>
       <x:c r="M51" t="str"/>
       <x:c r="N51" t="str"/>
@@ -2551,10 +2567,12 @@
         <x:v>If I were a movie star, I'd be popular. But I'm not a movie star, so I'm not popular.</x:v>
       </x:c>
       <x:c r="L54" t="str">
-        <x:v>&lt;br /&gt;&amp;nbsp;&lt;br /&gt;&lt;blockquote&gt;If P, then Q &lt;br /&gt;Not Q &lt;br /&gt;Therefore, not P&lt;/blockquote&gt;.</x:v>
+        <x:v>If P, then Q
+Not Q
+Therefore, not P.</x:v>
       </x:c>
       <x:c r="M54" t="str">
-        <x:v>Some might deny the antecedent by arguing "If you work hard, you will get a good job. Therefore, if you do not work hard you will not get a good job.".</x:v>
+        <x:v>Some might deny the antecedent by arguing "If you work hard, you will get a good job. Therefore, if you do not work hard you will not get a good job."</x:v>
       </x:c>
       <x:c r="N54" t="str"/>
       <x:c r="O54" t="str"/>
@@ -2593,7 +2611,7 @@
         <x:v>My girlfriend wanted to know whether I had cheated on her. I told her that perhaps it was impossible to have cheated on her since if I had cheated, it would mean we never really had a relationship to cheat on.</x:v>
       </x:c>
       <x:c r="L55" t="str">
-        <x:v>This fallacy is the converse of the &lt;a href="http://logfall.wordpress.com/false-dilemma/"&gt;false dilemma&lt;/a&gt;.</x:v>
+        <x:v>This fallacy is the converse of the false dilemma.</x:v>
       </x:c>
       <x:c r="M55" t="str">
         <x:v>Theists commonly claim their particular god becomes so angry over the very first offense a human commits, that he immediately condemns that human to eternal torment. They then also claim that same god is "patient" and "loving" towards humans. If you have a god invariably and continuously committing impatient acts, you don't have a patient god.</x:v>
@@ -2639,7 +2657,7 @@
         <x:v>Because a brain possesses thoughts, and a brain is composed of neurons, therefore these neurons pass thoughts back and forth.</x:v>
       </x:c>
       <x:c r="L56" t="str">
-        <x:v>This is the converse of the &lt;a href="http://logfall.wordpress.com/composition-fallacy/"&gt;composition fallacy&lt;/a&gt;.</x:v>
+        <x:v>This is the converse of the composition fallacy.</x:v>
       </x:c>
       <x:c r="M56" t="str">
         <x:v>Were someone to argue "Canada's GDP is 10% of the GDP of the U.S., so the average Canadian makes only 10% of what the average American makes", they would be committing the division fallacy.</x:v>
@@ -2929,10 +2947,12 @@
         <x:v>No humans are birds. Some birds are not lawyers. Therefore some lawyers are not humans.</x:v>
       </x:c>
       <x:c r="L63" t="str">
-        <x:v>&lt;br /&gt;&amp;nbsp;&lt;br /&gt;&lt;blockquote&gt;Some/all As are not Bs. &lt;br /&gt;Some/all Bs are not Cs.&lt;br /&gt;Therefore, no A is C.&lt;/blockquote&gt;.</x:v>
+        <x:v>Some/all As are not Bs.
+Some/all Bs are not Cs.
+Therefore, no A is C.</x:v>
       </x:c>
       <x:c r="M63" t="str">
-        <x:v>Another example might be "Since no republicans are democrats and some democrats are not farmers, it follows that some farmers are not republicans.".</x:v>
+        <x:v>Another example might be "Since no republicans are democrats and some democrats are not farmers, it follows that some farmers are not republicans."</x:v>
       </x:c>
       <x:c r="N63" t="str"/>
       <x:c r="O63" t="str"/>
@@ -3097,13 +3117,15 @@
         <x:v>Because physicists say mass equals energy, therefore mass can travel the speed of light.</x:v>
       </x:c>
       <x:c r="L67" t="str">
-        <x:v>If some system &lt;i&gt;A&lt;/i&gt; has both function &lt;i&gt;X&lt;/i&gt; and function &lt;i&gt;Y&lt;/i&gt;, and some system &lt;i&gt;B&lt;/i&gt; has a function &lt;i&gt;X′&lt;/i&gt; corresponding to &lt;i&gt;A&lt;/i&gt;'s function &lt;i&gt;X&lt;/i&gt;, then the system &lt;i&gt;B&lt;/i&gt; should also have a function &lt;i&gt;Y′&lt;/i&gt; that is analogous to &lt;i&gt;A&lt;/i&gt;'s function &lt;i&gt;Y&lt;/i&gt; for the analogy to succeed.</x:v>
+        <x:v>If some system A has both function X and function Y, and some system B has a function X′ corresponding to A's function X, then the system B should also have a function Y′ that is analogous to A's function Y for the analogy to succeed.</x:v>
       </x:c>
       <x:c r="M67" t="str">
-        <x:v>Consider the following argument. &lt;blockquote&gt;Teaching teenagers how to succeed in marriage prior to being married is like trying to teach someone how to ride a bicycle prior to placing them on a bicycle. &lt;/blockquote&gt;This is a false analogy in that it assumes the same type of learning mechanism used for the muscular memory of cycling is also used for grasping the dynamics of marriage.</x:v>
+        <x:v>Consider the following argument. Teaching teenagers how to succeed in marriage prior to being married is like trying to teach someone how to ride a bicycle prior to placing them on a bicycle.
+This is a false analogy in that it assumes the same type of learning mechanism used for the muscular memory of cycling is also used for grasping the dynamics of marriage.</x:v>
       </x:c>
       <x:c r="N67" t="str">
-        <x:v>Consider the following argument. &lt;blockquote&gt;Dating is like gambling. You'll win a few, and lose a few.&lt;/blockquote&gt;This is a false analogy in that it ignores the non-randon aspects of selecting a date.</x:v>
+        <x:v>Consider the following argument. Dating is like gambling. You'll win a few, and lose a few.
+This is a false analogy in that it ignores the non-randon aspects of selecting a date.</x:v>
       </x:c>
       <x:c r="O67" t="str"/>
       <x:c r="P67" t="str"/>
@@ -3213,28 +3235,25 @@
         <x:v>false dichotomy, middle ground</x:v>
       </x:c>
       <x:c r="J70" t="str">
-        <x:v>Occurs when two alternative positions or choices are wrongly assumed to be the only ones possible.</x:v>
+        <x:v>Occurs when someone presents a limited set of options as if they were the only live possibilities, while reasonable alternatives are ignored or suppressed.</x:v>
       </x:c>
       <x:c r="K70" t="str">
-        <x:v>If you are not with us, you're against us!</x:v>
+        <x:v>Either we pass this surveillance bill exactly as written, or we are choosing chaos and lawlessness.</x:v>
       </x:c>
       <x:c r="L70" t="str">
-        <x:v>One informative example is the statement "&lt;i&gt;Either this rock is alive or dead.&lt;/i&gt;". This completely ignores the option that the rock is "lifeless", which does not carry the misleading connotation that "dead" carries. "Dead" implies having previously lived, while "lifeless" does not.
-&lt;hr /&gt;A false dilemma is the inverse of the fallacy of &lt;a href="http://logfall.wordpress.com/denying-the-correlative/"&gt;denying the correlative&lt;/a&gt;. The &lt;a href="http://logfall.wordpress.com/single-cause-fallacy/"&gt;single cause fallacy&lt;/a&gt; is one type of false dilemma.</x:v>
+        <x:v>The pressure comes from pretending that a complex decision has only two doors. Sometimes the omitted alternatives are compromises, phased approaches, or the option of rejecting the framing altogether.</x:v>
       </x:c>
       <x:c r="M70" t="str">
-        <x:v>One common false dilemma frequently heard during any war is as follows. &lt;blockquote&gt;Are you in favor of this war? If not, you can't call yourself a patriot.&lt;/blockquote&gt;.</x:v>
+        <x:v>In 2024 immigration debates, many campaign messages reduced the issue to a choice between mass deportation and open borders, leaving out enforcement, asylum reform, and legal migration policy.</x:v>
       </x:c>
       <x:c r="N70" t="str">
-        <x:v>Theists often argue "&lt;i&gt;You don't worship my god? Why do you hate him so much?&lt;/i&gt;" This completely ignores the possibility that someone does not worship a god because they don't believe in that particular god or don't believe in any god.</x:v>
-      </x:c>
-      <x:c r="O70" t="str">
-        <x:v>Often, two ideologies that are in conflict such as big pharmaceutical companies and alternative medicine are framed as a dilemma; the drugs of one side work, and the drugs of the other do not. This is a false dilemma since the claims of both sides could be correct...or incorrect. The improprieties or failures of neither side validate the claims of the other side, nor does the demonstration of efficacy on one side invalidate the claims of efficacy of the other side.</x:v>
-      </x:c>
+        <x:v>School discussions about generative AI are often framed as either banning it completely or surrendering all meaningful learning, even though classrooms can set narrower rules for citation, drafting, and acceptable assistance.</x:v>
+      </x:c>
+      <x:c r="O70" t="str"/>
       <x:c r="P70" t="str"/>
       <x:c r="Q70" t="str"/>
       <x:c r="R70" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -3316,7 +3335,7 @@
         <x:v>He and his 4 brothers are bald, so his mother must also be bald.</x:v>
       </x:c>
       <x:c r="L72" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M72" t="str"/>
       <x:c r="N72" t="str"/>
@@ -3352,7 +3371,7 @@
         <x:v>Your argument that Santa is not real because he would need to fly his sleigh at impossible speeds on Christmas Eve is not valid since you don't even believe in Santa.</x:v>
       </x:c>
       <x:c r="L73" t="str">
-        <x:v>This fallacy is often used in response to an "&lt;i&gt;argumentum ad absurdum&lt;/i&gt;" in which assumptions are granted for the sake of argument to demonstrate that they lead to an incoherency. To plug an assumption into a argument to show the illogicality of that argument does not require an epistemic commitment to the assumption.</x:v>
+        <x:v>This fallacy is often used in response to an "argumentum ad absurdum" in which assumptions are granted for the sake of argument to demonstrate that they lead to an incoherency. To plug an assumption into a argument to show the illogicality of that argument does not require an epistemic commitment to the assumption.</x:v>
       </x:c>
       <x:c r="M73" t="str">
         <x:v>Some atheists argue that "any god that is both omnipotent and omniscient would not allow evil into the world." When theists dismiss this or a similar argument by saying "you don't believe in god, so you can't use the notion of god in your assumptions", they commit the fallacy of denying a hypothetical.</x:v>
@@ -3397,9 +3416,9 @@
         <x:v>While we understand that all girls are also children, this fact needs to be included as an assumption for the argument to be valid.</x:v>
       </x:c>
       <x:c r="M74" t="str">
-        <x:v>&lt;blockquote&gt;Power corrupts.&lt;br /&gt;
-Knowledge is power.&lt;br /&gt;
-Therefore knowledge corrupts.&lt;/blockquote&gt;
+        <x:v>Power corrupts.
+Knowledge is power.
+Therefore knowledge corrupts.
 This fallacy actually 4 terms since the term "power" as 2 different meanings.</x:v>
       </x:c>
       <x:c r="N74" t="str"/>
@@ -3538,7 +3557,7 @@
       </x:c>
       <x:c r="L77" t="str">
         <x:v>A hasty generalization might be a result of an insufficient sample size, imprecise measurements, or subjective reporting.
-This is a type of faulty generalization. A more detailed treatment of faulty generalizations can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+This is a type of faulty generalization. A more detailed treatment of faulty generalizations can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M77" t="str">
         <x:v>A foreign journalist who wanted to report on New York fashion might jump to a hasty generalization if visiting New York on October 31st.</x:v>
@@ -3748,7 +3767,9 @@
         <x:v>Because all pigs like mud, and no birds are pigs, therefore no birds like mud.</x:v>
       </x:c>
       <x:c r="L82" t="str">
-        <x:v>&lt;br /&gt;&amp;nbsp;&lt;br /&gt;&lt;blockquote&gt;All As are Cs. &lt;br /&gt;No Bs are As.&lt;br /&gt;Therefore, no Bs are Cs.&lt;/blockquote&gt;.</x:v>
+        <x:v>All As are Cs.
+No Bs are As.
+Therefore, no Bs are Cs.</x:v>
       </x:c>
       <x:c r="M82" t="str">
         <x:v>Conservapedia once had an article devoted to showing a relationship between atheism and obesity. The general idea was that most atheists are obese, and no theists are atheists, and therefore few theists are obese.</x:v>
@@ -3786,7 +3807,7 @@
         <x:v>We have only blurry photo evidence for the existence of alien space ships, but that's only because the aliens have technology that prevent our cameras from functioning properly.</x:v>
       </x:c>
       <x:c r="L83" t="str">
-        <x:v>This fallacy is similar to the &lt;a href="logfall.wordpress.com/suppressed-correlative/"&gt;suppressed correlative&lt;/a&gt;.</x:v>
+        <x:v>This fallacy is similar to the suppressed correlative.</x:v>
       </x:c>
       <x:c r="M83" t="str">
         <x:v>Some theists claim that their particular god answers prayer, but there is no possible outcome that does not fall within their definition of answered prayer. This makes their god equivalent to material cause and effect at best, but more probably non-existent.</x:v>
@@ -3958,8 +3979,9 @@
         <x:v>Nearly all humans wear clothing in public, so it is immoral not to.</x:v>
       </x:c>
       <x:c r="L87" t="str">
-        <x:v>Any "ought" ought to be accompanied by an "if" if it is to have any meaning. For example, you can tell your friend he ought to hurry if he wants to catch the bus, but an "ought" isolated from an "if" carries no meaning. Even a statement such as "You ought to listen to your parents" carries an implicit "if". If you do as they say, you'll avoid undesirable consequences. Another example is in the context of a game of chess. You ought not cheat in chess because it is socially unacceptable; i.e., if you want to maintain social respect. Even religious-based moral "oughts" contain implicit "if"s as in "You ought not lie if you want to please God and avoid eternal torment." "Ought"s cannot be divorced from "if"s.&lt;br /&gt;&amp;nbsp;&lt;br /&gt;
-&lt;blockquote&gt;"&lt;i&gt;In every system of morality, which I have hitherto met with, I have always remark'd, that the author proceeds for some time in the ordinary ways of reasoning, and establishes the being of a God, or makes observations concerning human affairs; when all of a sudden I am surpriz'd to find, that instead of the usual copulations of propositions, is, and is not, I meet with no proposition that is not connected with an ought, or an ought not. This change is imperceptible; but is however, of the last consequence. For as this ought, or ought not, expresses some new relation or affirmation, 'tis necessary that it shou'd be observ'd and explain'd; and at the same time that a reason should be given; for what seems altogether inconceivable, how this new relation can be a deduction from others, which are entirely different from it.&lt;/i&gt;"&lt;br /&gt;David Hume in &lt;i&gt;Treatise of Human Nature&lt;/i&gt; &lt;/blockquote&gt;.</x:v>
+        <x:v>Any "ought" ought to be accompanied by an "if" if it is to have any meaning. For example, you can tell your friend he ought to hurry if he wants to catch the bus, but an "ought" isolated from an "if" carries no meaning. Even a statement such as "You ought to listen to your parents" carries an implicit "if". If you do as they say, you'll avoid undesirable consequences. Another example is in the context of a game of chess. You ought not cheat in chess because it is socially unacceptable; i.e., if you want to maintain social respect. Even religious-based moral "oughts" contain implicit "if"s as in "You ought not lie if you want to please God and avoid eternal torment." "Ought"s cannot be divorced from "if"s.
+"In every system of morality, which I have hitherto met with, I have always remark'd, that the author proceeds for some time in the ordinary ways of reasoning, and establishes the being of a God, or makes observations concerning human affairs; when all of a sudden I am surpriz'd to find, that instead of the usual copulations of propositions, is, and is not, I meet with no proposition that is not connected with an ought, or an ought not. This change is imperceptible; but is however, of the last consequence. For as this ought, or ought not, expresses some new relation or affirmation, 'tis necessary that it shou'd be observ'd and explain'd; and at the same time that a reason should be given; for what seems altogether inconceivable, how this new relation can be a deduction from others, which are entirely different from it."
+David Hume in Treatise of Human Nature.</x:v>
       </x:c>
       <x:c r="M87" t="str">
         <x:v>Ayn Rand argued that one ought to act in a way consistent with one's own rational self-interests. The implicit "if" is presumably "if you want to live a long and happy life." Yet it is never explained why a life of altruism cannot also lead to a long and happy life, and why it ought to be replaced by a more egoistic existence.</x:v>
@@ -4204,7 +4226,8 @@
         <x:v>With many of the moon landing conspiracy theorists, as each of their claims is rebutted, they will move on to the next claim saying "But what about..." There appears to be no set degree of evidence that will convince them.</x:v>
       </x:c>
       <x:c r="O93" t="str">
-        <x:v>Consider the following popular internet post.&lt;blockquote&gt;Boy writes God a letter, "Dear God, why do you let bad things happen in our schools?" God replies,"Dear son, I'm not allowed in your schools."&lt;/blockquote&gt;If this particular god is giving his banishment from schools as the sole reason why bad things happen in those schools, then schools in which this particular god is allowed should not experience bad things. When presented with this corollary, those defending the quote often move the goalpost back to a more sensible and defensible position that makes the presence of bad people in schools the reason for bad things happening in those schools.</x:v>
+        <x:v>Consider the following popular internet post.Boy writes God a letter, "Dear God, why do you let bad things happen in our schools?" God replies,"Dear son, I'm not allowed in your schools."
+If this particular god is giving his banishment from schools as the sole reason why bad things happen in those schools, then schools in which this particular god is allowed should not experience bad things. When presented with this corollary, those defending the quote often move the goalpost back to a more sensible and defensible position that makes the presence of bad people in schools the reason for bad things happening in those schools.</x:v>
       </x:c>
       <x:c r="P93" t="str"/>
       <x:c r="Q93" t="str"/>
@@ -4287,7 +4310,7 @@
         <x:v>If someone claims that global warming is due to human activity, then justifies their position by saying "You can't prove human activity is not the cause of global warming", they have committed this fallacy.</x:v>
       </x:c>
       <x:c r="N95" t="str">
-        <x:v>In the U.S., until someone accused of a crime has been found guilty based on sufficient evidence, they are presumed innocent. This does not mean they &lt;strong&gt;are&lt;/strong&gt; innocent of the crime. It is just that we start with the assumption that they are innocent until (if ever) sufficient evidence warrants our deeming them guilty.</x:v>
+        <x:v>In the U.S., until someone accused of a crime has been found guilty based on sufficient evidence, they are presumed innocent. This does not mean they are innocent of the crime. It is just that we start with the assumption that they are innocent until (if ever) sufficient evidence warrants our deeming them guilty.</x:v>
       </x:c>
       <x:c r="O95" t="str"/>
       <x:c r="P95" t="str"/>
@@ -4367,13 +4390,13 @@
         <x:v>How can you call yourself a patriot when you are against this war!</x:v>
       </x:c>
       <x:c r="L97" t="str">
-        <x:v>Those who employ this fallacy will often interject &lt;i&gt;ad hoc&lt;/i&gt; or arbitrary criteria to maintain an artificial delineation.</x:v>
+        <x:v>Those who employ this fallacy will often interject ad hoc or arbitrary criteria to maintain an artificial delineation.</x:v>
       </x:c>
       <x:c r="M97" t="str">
-        <x:v>If a theist informs an atheist that his position is indefensible since Stalin was an atheist, it would be a &lt;i&gt;no true Scotsman&lt;/i&gt; fallacy for the atheist to suggest that Stalin was not a &lt;i&gt;real&lt;/i&gt; atheist. And it would be forfeiting the chance to point out the theist's own fallacy of &lt;a href="http://logfall.wordpress.com/top-down-condemnation/"&gt;top-down condemnation&lt;/a&gt;.</x:v>
+        <x:v>If a theist informs an atheist that his position is indefensible since Stalin was an atheist, it would be a no true Scotsman fallacy for the atheist to suggest that Stalin was not a real atheist. And it would be forfeiting the chance to point out the theist's own fallacy of top-down condemnation.</x:v>
       </x:c>
       <x:c r="N97" t="str">
-        <x:v>If an atheist informs a Christian that his position is indefensible since Hitler was an Christian, it would be a &lt;i&gt;no true Scotsman&lt;/i&gt; fallacy for the theist to suggest that Hitler was not a &lt;i&gt;real&lt;/i&gt; Christian. And it would be forfeiting the chance to point out the atheist's own fallacy of &lt;a href="http://logfall.wordpress.com/top-down-condemnation/"&gt;top-down condemnation&lt;/a&gt;.</x:v>
+        <x:v>If an atheist informs a Christian that his position is indefensible since Hitler was an Christian, it would be a no true Scotsman fallacy for the theist to suggest that Hitler was not a real Christian. And it would be forfeiting the chance to point out the atheist's own fallacy of top-down condemnation.</x:v>
       </x:c>
       <x:c r="O97" t="str"/>
       <x:c r="P97" t="str"/>
@@ -4457,7 +4480,7 @@
         <x:v>She's likes bowling, so she certainly drinks beer as do most other bowlers.</x:v>
       </x:c>
       <x:c r="L99" t="str">
-        <x:v>This fallacy is measured in degrees. For example, you might be warranted in saying "John will probably like this book since the last book he enjoyed was also science fiction.".</x:v>
+        <x:v>This fallacy is measured in degrees. For example, you might be warranted in saying "John will probably like this book since the last book he enjoyed was also science fiction."</x:v>
       </x:c>
       <x:c r="M99" t="str">
         <x:v>Because Judge John E. Jones III was appointed by George W. Bush, it was assumed by many that he would favor the right-leaning anti-evolutionists in the Dover trial over intelligent design. This turned out to not be the case.</x:v>
@@ -4543,7 +4566,7 @@
         <x:v>But, Dad! Your $20 is not going to replace the car I crashed! Keep your money!</x:v>
       </x:c>
       <x:c r="L101" t="str">
-        <x:v>&lt;br /&gt;&amp;nbsp;&lt;br /&gt;&lt;blockquote&gt;"&lt;i&gt;The perfect is the enemy of the good.&lt;/i&gt;" ~Voltaire&lt;/blockquote&gt;.</x:v>
+        <x:v>"The perfect is the enemy of the good." ~Voltaire.</x:v>
       </x:c>
       <x:c r="M101" t="str">
         <x:v>Some in the US claim that tighter border controls are "not the solution" to the problem of illegal immigration, and ignore the fact that tighter borders might make a significant difference.</x:v>
@@ -4581,7 +4604,7 @@
         <x:v>I remember you once shouted in anger at your brother. You are essentially an angry person.</x:v>
       </x:c>
       <x:c r="L102" t="str">
-        <x:v>Those employing this fallacy are removing semantic resolution from the issue, and are demanding others to categorize quite disparate degrees of phenomena into only 2 categories. This is similar to &lt;a href="logfall.wordpress.com/semantic-pixelization/"&gt;semantic pixelization&lt;/a&gt;.</x:v>
+        <x:v>Those employing this fallacy are removing semantic resolution from the issue, and are demanding others to categorize quite disparate degrees of phenomena into only 2 categories. This is similar to semantic pixelization.</x:v>
       </x:c>
       <x:c r="M102" t="str">
         <x:v>It has been questioned why, when blind-folded, people cannot walk in a straight line. It would actually be highly unusual for a person to maintain a straight line, and there is a wide range of possible degrees of accuracy between straight and highly curved. To ignore this continuum is to forfeit useful semantic resolution.</x:v>
@@ -4632,10 +4655,10 @@
         <x:v>This is a type of straw-man fallacy.</x:v>
       </x:c>
       <x:c r="M103" t="str">
-        <x:v>If person &lt;i&gt;A&lt;/i&gt; claims their "loving" god will eternally torture the humans he created if they disobey him, and person &lt;i&gt;B&lt;/i&gt; claims this is analogous to a "loving" human father eternally torturing his children if they disobey, for person &lt;i&gt;A&lt;/i&gt; would unjustifiably pervert the analogy if they were to claim that the analogy does hold for irrelevant reasons such as "the human father is not righteous" or "human fathers don't live eternally".</x:v>
+        <x:v>If person A claims their "loving" god will eternally torture the humans he created if they disobey him, and person B claims this is analogous to a "loving" human father eternally torturing his children if they disobey, for person A would unjustifiably pervert the analogy if they were to claim that the analogy does hold for irrelevant reasons such as "the human father is not righteous" or "human fathers don't live eternally".</x:v>
       </x:c>
       <x:c r="N103" t="str">
-        <x:v>If person &lt;i&gt;A&lt;/i&gt; claims religious faith gives people joy that hides and prevents other possible joys in life in the same way that cocaine gives junkies joy at the expense of other possible joys in life, person &lt;i&gt;B&lt;/i&gt; would unjustifiably pervert the analogy if they were to claim that the analogy does hold for irrelevant reasons such as "cocaine is not legal" or "people with faith serve God.".</x:v>
+        <x:v>If person A claims religious faith gives people joy that hides and prevents other possible joys in life in the same way that cocaine gives junkies joy at the expense of other possible joys in life, person B would unjustifiably pervert the analogy if they were to claim that the analogy does hold for irrelevant reasons such as "cocaine is not legal" or "people with faith serve God."</x:v>
       </x:c>
       <x:c r="O103" t="str"/>
       <x:c r="P103" t="str"/>
@@ -4673,7 +4696,7 @@
         <x:v>Some theists suggest that archeological evidence of biblical sites is evidence for the biblical miracles mentioned in the same passage as is the site. Uncovering historical evidence for the existence of St. Nicolas does not lend credibilty to flying reindeer.</x:v>
       </x:c>
       <x:c r="N104" t="str">
-        <x:v>Some people argue that evidence for government impropriety on issue &lt;i&gt;X&lt;/i&gt; implies that there is also impropriety on issue &lt;i&gt;Y&lt;/i&gt;. While inductive evidence derived from assessing habitual behavior warrants a measured degree of speculation, it does not warrant confidence incommensurate to that evidence.</x:v>
+        <x:v>Some people argue that evidence for government impropriety on issue X implies that there is also impropriety on issue Y. While inductive evidence derived from assessing habitual behavior warrants a measured degree of speculation, it does not warrant confidence incommensurate to that evidence.</x:v>
       </x:c>
       <x:c r="O104" t="str"/>
       <x:c r="P104" t="str"/>
@@ -4755,7 +4778,7 @@
         <x:v>After I started wearing a copper bracelet, my health improved! It worked!</x:v>
       </x:c>
       <x:c r="L106" t="str">
-        <x:v>Causation must be rigorously demonstrated. Phenomena that occur in sequence do not necessarily have a causal link. This fallacy is related to the &lt;a href="http://logfall.wordpress.com/correlation-is-not-causation/"&gt;correlation is not causation&lt;/a&gt; fallacy.</x:v>
+        <x:v>Causation must be rigorously demonstrated. Phenomena that occur in sequence do not necessarily have a causal link. This fallacy is related to the correlation is not causation fallacy.</x:v>
       </x:c>
       <x:c r="M106" t="str">
         <x:v>Most people feel a period of elation every time they voluntarily change jobs. Many are tempted to cite the conditions of the new job as the reason for their better mood. Is it the new job that is causing the elation, or merely the change?</x:v>
@@ -4797,7 +4820,7 @@
         <x:v>This apple is red, so all apples must be red.</x:v>
       </x:c>
       <x:c r="L107" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M107" t="str"/>
       <x:c r="N107" t="str"/>
@@ -4842,7 +4865,7 @@
         <x:v>This is often a tactic used in formal speeches. If not all the many minor points introduced are not addressed by the opponent, the verbose contender will claim victory.</x:v>
       </x:c>
       <x:c r="M108" t="str">
-        <x:v>Donald Rumsfeld once said...&lt;blockquote&gt;There are known knowns. These are things we know that we know. There are known unknowns. That is to say, there are things that we know we don't know. But there are also unknown unknowns. There are things we don't know we don't know.&lt;/blockquote&gt;.</x:v>
+        <x:v>Donald Rumsfeld once said...There are known knowns. These are things we know that we know. There are known unknowns. That is to say, there are things that we know we don't know. But there are also unknown unknowns. There are things we don't know we don't know.</x:v>
       </x:c>
       <x:c r="N108" t="str"/>
       <x:c r="O108" t="str"/>
@@ -4993,7 +5016,8 @@
         <x:v>I have a golden square triangle instead of a heart in my chest, and I have the lab analysis to prove it.</x:v>
       </x:c>
       <x:c r="L112" t="str">
-        <x:v>If someone claims to have a golden square triangle in their chest, and provides gold flakes or a lab analysis as evidence, you don't have to test the gold flakes or scrutinize the lab analysis for authenticity before you dismiss the notion that they have a golden square triangle in their chest. If a concept has been demonstrated to be illogical, no amount of evidence will salvage that concept.&lt;br /&gt;To a lesser degree, what we define as physical impossibilities can be dismissed in the same way we can dismiss logical impossibilities. However, we must be careful since what is physical laws have been abstracted from nature by humans, and may not be absolute. However, this caveat does not mean we are wrong to dismiss with a high degree of confidence any concept that science considers a physical impossibility.</x:v>
+        <x:v>If someone claims to have a golden square triangle in their chest, and provides gold flakes or a lab analysis as evidence, you don't have to test the gold flakes or scrutinize the lab analysis for authenticity before you dismiss the notion that they have a golden square triangle in their chest. If a concept has been demonstrated to be illogical, no amount of evidence will salvage that concept.
+To a lesser degree, what we define as physical impossibilities can be dismissed in the same way we can dismiss logical impossibilities. However, we must be careful since what is physical laws have been abstracted from nature by humans, and may not be absolute. However, this caveat does not mean we are wrong to dismiss with a high degree of confidence any concept that science considers a physical impossibility.</x:v>
       </x:c>
       <x:c r="M112" t="str">
         <x:v>Some theists define their god as both infinitely "loving" and infinitely "hateful" to humans. We need not scrutinize their holy book or nature for evidence of their incoherent god. If there is evidence for a god in nature, their god has already been eliminated as a candidate due to the absurdity of his definition.</x:v>
@@ -5035,7 +5059,7 @@
         <x:v>Last year we had 12 car accidents on main street, double the previous year's figures! The frequency of accidents on Main Street fell to only 6 again after a speed camera was installed early this year. Therefore, the speed camera has improved road safety.</x:v>
       </x:c>
       <x:c r="L113" t="str">
-        <x:v>This is similar to the &lt;a href="http://logfall.wordpress.com/post-hoc-ergo-propter-hoc/"&gt;post hoc ergo propter hoc&lt;/a&gt; fallacy, but is based on the "regression to the mean" principle in which certain phenomena naturally fluctuate in volume or intensity. This statistical "noise" in the data is natural and expected.</x:v>
+        <x:v>This is similar to the post hoc ergo propter hoc fallacy, but is based on the "regression to the mean" principle in which certain phenomena naturally fluctuate in volume or intensity. This statistical "noise" in the data is natural and expected.</x:v>
       </x:c>
       <x:c r="M113" t="str">
         <x:v>In 1999 the Department of Education in Massachusetts gave it's school improvement goals, then subsequently tested those districts for any detectable improvement. Unsurprisingly, the bottom 50% of the schools made notable improvement. What was not so heavily emphasized was that the top 50% of their schools fell about the same degree as the bottom 50% gained. The apparent improvement of the bottom half and the apparent drop of the top half of any single phenomena is what is statistically expected and does not necessarily show the efficacy of any policy in effect at the time.</x:v>
@@ -5165,7 +5189,7 @@
         <x:v>You say you tend to believe you'll not die before you're 50. If you don't believe you'll die before you're 50, why did you buy a life insurance policy when you were 30?</x:v>
       </x:c>
       <x:c r="L116" t="str">
-        <x:v>In the example, the person making the argument is attempting to make his opponents belief binary so it can be more easily criticized. The belief most individuals have that they will live past 50 is not some binary and absolute belief, but rather is a degree of belief that emerges from an actuarial assessment of the probabilities. This fallacy is similar to the &lt;a href="logfall.wordpress.com/perfect-standard/"&gt;perfect standard&lt;/a&gt; fallacy.</x:v>
+        <x:v>In the example, the person making the argument is attempting to make his opponents belief binary so it can be more easily criticized. The belief most individuals have that they will live past 50 is not some binary and absolute belief, but rather is a degree of belief that emerges from an actuarial assessment of the probabilities. This fallacy is similar to the perfect standard fallacy.</x:v>
       </x:c>
       <x:c r="M116" t="str">
         <x:v>The media often make statements such as "the murder rate increased by 50% last year" instead of more clearly stating "there were 3 murders committed this year, one more than last year." This unnecessarily diminishes the semantic resolution.</x:v>
@@ -5215,7 +5239,7 @@
         <x:v>It would be great if we could reduce the national debt without raising taxes or reducing spending. Therefore there must be a way we can accomplish this.</x:v>
       </x:c>
       <x:c r="L117" t="str">
-        <x:v>This fallacy is similar to &lt;a href="http://logfall.wordpress.com/wishful-thinking/"&gt;wishful thinking&lt;/a&gt;.</x:v>
+        <x:v>This fallacy is similar to wishful thinking.</x:v>
       </x:c>
       <x:c r="M117" t="str">
         <x:v>If, in response to painful demographic gaps in health care coverage, it is argued that having a national health care bill would be a wonderful thing, and is therefore necessary, this would be committing the sentimental fallacy. The desire for something does not warrant its realization. Other factors such as long-term consequences must be considered. Emotion does not carry an imperative.</x:v>
@@ -5259,7 +5283,7 @@
         <x:v>Last year, the governor promised to stimulate the economy during his term, and you will note that this year there has been an increase of 2,000 jobs in the service industry.</x:v>
       </x:c>
       <x:c r="L118" t="str">
-        <x:v>The governor in the example may be ignoring other less-favorable data to paint a picture of success. This fallacy is similar to &lt;a href="http://logfall.wordpress.com/cherry-picking/"&gt;cherry-picking&lt;/a&gt;. It is subjectively and arbitrarily (though perhaps subconsciously) selecting data that will bolster your position while ignoring data inconsistent with your position. For this reason, scientists attempt to reduce subjectivity by starting with a hypothesis, then attempt to falsify that hypothesis by every imaginable means. This increases the objectivity basic to scientific success and respectability.</x:v>
+        <x:v>The governor in the example may be ignoring other less-favorable data to paint a picture of success. This fallacy is similar to cherry-picking. It is subjectively and arbitrarily (though perhaps subconsciously) selecting data that will bolster your position while ignoring data inconsistent with your position. For this reason, scientists attempt to reduce subjectivity by starting with a hypothesis, then attempt to falsify that hypothesis by every imaginable means. This increases the objectivity basic to scientific success and respectability.</x:v>
       </x:c>
       <x:c r="M118" t="str">
         <x:v>Consider someone who claims he can accurately and consistently predict the outcome of coin flips. After 5 flips he has only guessed 2 flips correctly (40%), and wants to continue the experiment. Finally after 20 flips, he has guessed 13 correctly, and wants to stop, making his accuracy appear to be 65%. However, because he was able to choose when to quit, the results are subjectively biased, and do not meet the standards of experimentation set by science.</x:v>
@@ -5305,7 +5329,7 @@
         <x:v>The drop in crime in our neighborhood is due to better policing.</x:v>
       </x:c>
       <x:c r="L119" t="str">
-        <x:v>The actual cause of a local drop in crime may actually be a collection of causes such as the installation of surveillance cameras, a better local economy that has given would-be criminals jobs and money, improved forensics, new home entertainment hardware and software that keep would-be criminals preoccupied, better role models, and tougher laws that have locked up the most frequent offenders. This fallacy is a type of &lt;a href="http://logfall.wordpress.com/false-dilemma/"&gt;false dilemma&lt;/a&gt;.</x:v>
+        <x:v>The actual cause of a local drop in crime may actually be a collection of causes such as the installation of surveillance cameras, a better local economy that has given would-be criminals jobs and money, improved forensics, new home entertainment hardware and software that keep would-be criminals preoccupied, better role models, and tougher laws that have locked up the most frequent offenders. This fallacy is a type of false dilemma.</x:v>
       </x:c>
       <x:c r="M119" t="str">
         <x:v>Nearly every country that has become prosperous throughout history has had some of its citizens claiming that their greatness was entirely due to the superiority of their nationality or their particular god.</x:v>
@@ -5345,25 +5369,25 @@
         <x:v>fallacy of the beard</x:v>
       </x:c>
       <x:c r="J120" t="str">
-        <x:v>The argument that a small first step will inevitably leads to a chain of related events culminating in some significant undesirable impact.</x:v>
+        <x:v>Occurs when someone claims that a relatively small first step will trigger a chain of worsening outcomes without showing why that chain is likely, stable, or hard to stop.</x:v>
       </x:c>
       <x:c r="K120" t="str">
-        <x:v>If we allow alcohol use on campus, we will eventually be forced to allow illicit drug use.</x:v>
+        <x:v>If we let students use AI for brainstorming, next year nobody will learn to write and universities will stop caring whether humans produced any work at all.</x:v>
       </x:c>
       <x:c r="L120" t="str">
-        <x:v>This is a fallacy only where there is certainty in the conclusion and an absence of evidence that similar contexts have produced or would produce degenerating standards. There may very well be a snowball effect possible for the given phenomenon, but the evidence for such must accompany the argument. This is related to the &lt;a href="http://logfall.wordpress.com/continuum-fallacy/"&gt;continuum fallacy&lt;/a&gt;.</x:v>
+        <x:v>Some slopes are real, especially when incentives, precedent, or institutional weakness make escalation predictable. The fallacy appears when the chain is asserted rather than argued for.</x:v>
       </x:c>
       <x:c r="M120" t="str">
-        <x:v>Some social conservatives have argued that, if we accept gay marriage, there is nothing stopping us from allowing polygamy, adult/child marriage, or marriage between species. Unless this argument is accompanied by evidence or argumentation that the legalization of gay marriage removes all constraints upon the other forms of marriage cited, this is a slippery slope fallacy.</x:v>
+        <x:v>In 2024 arguments over classroom AI, both enthusiasts and critics often predicted inevitable futures - either total educational collapse or total educational liberation - without showing why intermediate guardrails would fail.</x:v>
       </x:c>
       <x:c r="N120" t="str">
-        <x:v>On the second day of the Scopes Trial, Clarence Darrow argued... &lt;blockquote&gt;If today you can take a thing like evolution and make it a crime to teach it in the public school, tomorrow you can make it a crime to teach it in the private schools, and the next year you can make it a crime to teach it to the hustings or in the church. At the next session you may ban books and the newspapers. Soon you may set Catholic against Protestant and Protestant against Protestant, and try to foist your own religion upon the minds of men. If you can do one you can do the other. Ignorance and fanaticism is ever busy and needs feeding. Always it is feeding and gloating for more. Today it is the public school teachers, tomorrow the private. The next day the preachers and the lectures, the magazines, the books, the newspapers. After [a]while, your honor, it is the setting of man against man and creed against creed until with flying banners and beating drums we are marching backward to the glorious ages of the sixteenth century when bigots lighted fagots to burn the men who dared to bring any intelligence and enlightenment and culture to the human mind.&lt;br /&gt;&lt;sup&gt;&lt;a herf="http://www.law.umkc.edu/faculty/projects/ftrials/scopes/day2.htm"&gt;source&lt;/a&gt;&lt;/sup&gt;&lt;/blockquote&gt;.</x:v>
+        <x:v>Election rhetoric about mail voting, early voting, or routine administrative changes often predicts the total breakdown of legitimacy from one policy shift without evidence for the full cascade.</x:v>
       </x:c>
       <x:c r="O120" t="str"/>
       <x:c r="P120" t="str"/>
       <x:c r="Q120" t="str"/>
       <x:c r="R120" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -5401,7 +5425,7 @@
         <x:v>Some communities have proposed that police officers and their families be exempt from citations for traffic offenses. But it would seem that the reasons given for establishing speed limits would hold also for the families of police officers.</x:v>
       </x:c>
       <x:c r="N121" t="str">
-        <x:v>Many religions hold that forgiveness should be granted without bloodshed or payment of any sort, yet exempt their own god by offering irrelevant excuses such as "God is holy" or "God's ways are not our ways.".</x:v>
+        <x:v>Many religions hold that forgiveness should be granted without bloodshed or payment of any sort, yet exempt their own god by offering irrelevant excuses such as "God is holy" or "God's ways are not our ways."</x:v>
       </x:c>
       <x:c r="O121" t="str"/>
       <x:c r="P121" t="str"/>
@@ -5439,7 +5463,7 @@
         <x:v>All the Hispanics I've seen interviewed on television are not the least bit shy, so your neighbor Felipe surely can't be shy!</x:v>
       </x:c>
       <x:c r="L122" t="str">
-        <x:v>This is a type of faulty generalization. A more detailed treatment of faulty generalizations can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+        <x:v>This is a type of faulty generalization. A more detailed treatment of faulty generalizations can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M122" t="str">
         <x:v>Because of the salient drama surrounding abortion clinic bombings, it became easy to erroneously view all abortion opponents as gun-wielding lunatics.</x:v>
@@ -5521,29 +5545,25 @@
       <x:c r="H124" t="str"/>
       <x:c r="I124" t="str"/>
       <x:c r="J124" t="str">
-        <x:v>Providing a misrepresentation of an opponent's position that can then be more easily attacked.</x:v>
+        <x:v>Occurs when someone replaces an opponent's actual position with a weaker, more extreme, or simplified version and then refutes that easier target.</x:v>
       </x:c>
       <x:c r="K124" t="str">
-        <x:v>Evolutionists believe life came from nothing. Nothing can come from nothing, so their position is absurd!</x:v>
+        <x:v>A proposal to require disclosure labels on AI-generated campaign ads is attacked as 'wanting the government to ban political speech.'</x:v>
       </x:c>
       <x:c r="L124" t="str">
-        <x:v>This fallacy is a result of either poor research or deliberate distortion of the opponent's argument.</x:v>
+        <x:v>A straw man can be created by exaggeration, selective quotation, or by ignoring the qualifying parts of the original claim. It is not enough that a reply is critical; the key problem is that the reply no longer addresses the real position.</x:v>
       </x:c>
       <x:c r="M124" t="str">
-        <x:v>&lt;blockquote&gt;"&lt;i&gt;Gradually by the course of evolution, [green slime] developed into animals and plants and at last into MAN. Man, so the theologians assure us, is so splendid a Being that he may well be regarded as the culmination to which the long ages of nebula and slime were a prelude. I think the theologians must have been fortunate in their human contacts. They do not seem to me to have given due weight to Hitler..&lt;/i&gt;."&lt;sup&gt;&lt;br /&gt;
-Bertrand Russell, "Is There a God?" (1952), in The Collected Papers of Bertrand Russell, Volume 11: Last Philosophical Testament, 1943-68, ed. John G. Slater and Peter Köllner (London: Routledge, 1997), pp. 545.&lt;/sup&gt; &lt;/blockquote&gt;
-Russell completely ignores the Christian doctrine of the &lt;i&gt;fall of man&lt;/i&gt;, and is therefore addressing a straw man here.</x:v>
+        <x:v>During the September 10, 2024 Harris-Trump debate, claims about abortion rights were repeatedly recast into the far more extreme charge that Democrats support killing babies after birth, which is not the position being defended.</x:v>
       </x:c>
       <x:c r="N124" t="str">
-        <x:v>Some argue that those committed to science think science is infallible or worthy of worship.</x:v>
-      </x:c>
-      <x:c r="O124" t="str">
-        <x:v>Some argue that all Christians become Christians only because they fear the consequences of not believing.</x:v>
-      </x:c>
+        <x:v>Debates over campus speech and content moderation often turn a narrower argument about rules, incentives, or disclosure into the cartoon claim that one side 'wants censorship' or 'wants total chaos.'</x:v>
+      </x:c>
+      <x:c r="O124" t="str"/>
       <x:c r="P124" t="str"/>
       <x:c r="Q124" t="str"/>
       <x:c r="R124" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -5615,8 +5635,8 @@
         <x:v>You can't claim to be intelligent since there is someone always more intelligent than you are.</x:v>
       </x:c>
       <x:c r="L126" t="str">
-        <x:v>The consequence of this fallacy is that the term in question is made impotent by removing any contrasting concept.&lt;br /&gt;
-This fallacy is similar to the &lt;a href="http://logfall.wordpress.com/continuum-fallacy/"&gt;continuum fallacy&lt;/a&gt;.</x:v>
+        <x:v>The consequence of this fallacy is that the term in question is made impotent by removing any contrasting concept.
+This fallacy is similar to the continuum fallacy.</x:v>
       </x:c>
       <x:c r="M126" t="str">
         <x:v>The god of some theists becomes so wrathful over a human's very 1st offense that he deems that offender worthy of eternal torment. This very same god is defined as "loving" and "patient" by these theists, and this definition is justified by suggesting that their wrathful god usually waits a while before sending the offender to eternal torment. The absurdity of this is clear when considering a neighbor who, after claiming to love his children, eternally beats them upon their first offense, but only after they've had dinner.</x:v>
@@ -5756,7 +5776,7 @@
         <x:v>Christians often quote the verse "The fool has said in his heart, 'there is no God'" sometimes as if this is a justification for belief in God, and sometimes simply as a thought-terminator.</x:v>
       </x:c>
       <x:c r="P129" t="str">
-        <x:v>When having their expectations questioned, older people often, due to either having no real answer or having no interest in giving an answer, say "When you're my age, you'll understand.".</x:v>
+        <x:v>When having their expectations questioned, older people often, due to either having no real answer or having no interest in giving an answer, say "When you're my age, you'll understand."</x:v>
       </x:c>
       <x:c r="Q129" t="str"/>
       <x:c r="R129" t="str">
@@ -5790,7 +5810,7 @@
         <x:v>My neighbor is a banker, and is a jerk. Therefore, bankers are jerks.</x:v>
       </x:c>
       <x:c r="L130" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M130" t="str">
         <x:v>If you break your leg the first time on the ski slopes, this is not evidence that skiing is any more dangerous than other sports. Actual statistical significance derived from a sufficiently large data set is necessary before such a conclusion can be made, in spite of your disinclination to get back on the slopes anytime soon.</x:v>
@@ -5876,7 +5896,7 @@
         <x:v>My neighbor is a banker, and a really nice guy. Therefore, bankers are nice guys.</x:v>
       </x:c>
       <x:c r="L132" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary &lt;a href="http://logfall.wordpress.com/inductive-errors/"&gt;Inductive Errors&lt;/a&gt; page.</x:v>
+        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
       </x:c>
       <x:c r="M132" t="str">
         <x:v>If a convenience store clerk successfully disarms a would-be robber, this is not evidence that confronting robbers is the best policy. A much larger sample of cases would be necessary before any inductive conclusion can be made.</x:v>
@@ -6051,7 +6071,7 @@
         <x:v>In the example, the conclusion does not follow since it is 2-leggedness that is the larger more general category, encompassing both humans and birds, without either one of the smaller more specific categories encompassing the other. If one of the premises instead stated that all 2-legged things are birds, then the argument would be valid (but not sound).</x:v>
       </x:c>
       <x:c r="M136" t="str">
-        <x:v>Young people needing social acceptance often argue to themselves in a way that might be stated "The cool wear sunglasses, and I'm wearing sunglasses. Therefore I'm one of the cool.".</x:v>
+        <x:v>Young people needing social acceptance often argue to themselves in a way that might be stated "The cool wear sunglasses, and I'm wearing sunglasses. Therefore I'm one of the cool."</x:v>
       </x:c>
       <x:c r="N136" t="str"/>
       <x:c r="O136" t="str"/>
@@ -6087,7 +6107,9 @@
         <x:v>In the example, "energy", "force", "balances" and "essences" are all too vague to submit to scientific scrutiny.</x:v>
       </x:c>
       <x:c r="M137" t="str">
-        <x:v>&lt;blockquote&gt;&lt;i&gt;There are only three sports: bullfighting, motor racing, and mountaineering; all the rest are merely games.&lt;/i&gt;&lt;br /&gt;~Ernest Hemmingway&lt;/blockquote&gt;The definitions of "sports" and " games" are vague, and make a refutation difficult.</x:v>
+        <x:v>There are only three sports: bullfighting, motor racing, and mountaineering; all the rest are merely games.
+~Ernest Hemmingway
+The definitions of "sports" and " games" are vague, and make a refutation difficult.</x:v>
       </x:c>
       <x:c r="N137" t="str">
         <x:v>Theists often introduce words such as "faith" and "sin" that have definitions that are contested even within their own sect.</x:v>
@@ -6175,11 +6197,14 @@
         <x:v>The claim of an accessible witness to an event that there are inaccessible additional witnesses to that event carries no evidential weight for that event.</x:v>
       </x:c>
       <x:c r="M139" t="str">
-        <x:v>&lt;blockquote&gt;"I have personally witnessed irrefutable miracle healings (i.e. stunted limb growing out to full length spontaneously in a matter of seconds,) in response to prayer in the name of Jesus. I would guess there were close to 40 witnesses to this miracle healing, many of whom, including myself, were standing only 2 or 3 feet away from the man who was healed; some of whom I still know by first and/or last name."&lt;/blockquote&gt;
-[&lt;a href="http://www.physorg.com/news165555744.html"&gt;Source&lt;/a&gt;].</x:v>
+        <x:v>"I have personally witnessed irrefutable miracle healings (i.e. stunted limb growing out to full length spontaneously in a matter of seconds,) in response to prayer in the name of Jesus. I would guess there were close to 40 witnesses to this miracle healing, many of whom, including myself, were standing only 2 or 3 feet away from the man who was healed; some of whom I still know by first and/or last name."
+[Source].</x:v>
       </x:c>
       <x:c r="N139" t="str">
-        <x:v>&lt;blockquote&gt;&lt;i&gt;After that, he [Jesus, after his alleged resurrection] appeared to more than five hundred of the brothers at the same time, most of whom are still living, though some have fallen asleep.&lt;/i&gt;&lt;br /&gt;1 Corinthians 15:6&lt;/blockquote&gt;This verse is often cited by Christians as evidence for the resurrection.&lt;br /&gt;[&lt;a href="http://www.leaderu.com/everystudent/easter/articles/josh2.html"&gt;Example&lt;/a&gt;].</x:v>
+        <x:v>After that, he [Jesus, after his alleged resurrection] appeared to more than five hundred of the brothers at the same time, most of whom are still living, though some have fallen asleep.
+1 Corinthians 15:6
+This verse is often cited by Christians as evidence for the resurrection.
+[Example].</x:v>
       </x:c>
       <x:c r="O139" t="str"/>
       <x:c r="P139" t="str"/>

</xml_diff>

<commit_message>
Expand LogFall editorial rewrites
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbb06db31815a441b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R37f93d70b5094a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R348c512875f343ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R72869a05766e45b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rcc7d7bbd5192405d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R5f3831ef85bb4749"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -315,28 +315,25 @@
       <x:c r="H2" t="str"/>
       <x:c r="I2" t="str"/>
       <x:c r="J2" t="str">
-        <x:v>Invoking the popular but wrong notion that finding no evidence for something is no evidence for the absence of that thing.</x:v>
+        <x:v>Occurs when someone treats a failure to find expected evidence as if it counted for nothing against the claim, even in a context where the claim should leave detectable traces.</x:v>
       </x:c>
       <x:c r="K2" t="str">
-        <x:v>The fact that you did not see me at your birthday party does not mean I was not there!</x:v>
+        <x:v>Multiple audits found no trace of the vote-flipping scheme, but that proves nothing; if the conspiracy were real, of course it would leave no evidence.</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>The absence of evidence it not evidence of absence.
-This argument, attributed to Carl Sagan, is often invoked when claims of a god comes under scrutiny. While the absence of evidence is not proof of absence, it is, to varying degrees, evidence of absence. The degree of evidence an absence of evidence is for the absence of anything will depend on the context. If there is no evidence of thing X in a location Y, the degree that will constitute evidence for the absence of that thing depends upon how we substantiate the variables. Is X a molecule, mouse or monster? Is Y a cup, couch or continent?</x:v>
+        <x:v>Sometimes absence of evidence really is weak evidence, especially when the search tools are poor or the target is hard to detect. But when repeated investigation under the right conditions turns up nothing, that absence is itself evidence.</x:v>
       </x:c>
       <x:c r="M2" t="str">
-        <x:v>After a Harvard Medical School study on the effects of prayer on heart surgery patients showed no statistical advantage of prayer, it was argued that "the absence of evidence is not evidence of absence".</x:v>
+        <x:v>After officials in Springfield, Ohio said there were no credible reports supporting the September 2024 rumor that Haitian immigrants were abducting and eating pets, some defenders treated the lack of evidence as irrelevant or as proof of a cover-up rather than as evidence against the rumor.</x:v>
       </x:c>
       <x:c r="N2" t="str">
-        <x:v>Those who claim they have the biblical holy spirit helping them to make predictions or avoid logical fallacies in discussion, when confronted with evidence that they are, at best, only on par with those who do not claim to have a holy spirit, they often invoke this absence of evidence fallacy. They then often claim the burden of proof falls on those denying the existence of their holy spirit.</x:v>
-      </x:c>
-      <x:c r="O2" t="str">
-        <x:v>Donald Rumsfeld invoked the "absence of evidence" fallacy in reference to possible weapons of mass destruction in Iraq.</x:v>
-      </x:c>
+        <x:v>Claims of widespread noncitizen voting in 2024 often survived repeated audits and official reviews by insisting that the absence of supporting evidence was exactly what one should expect from a hidden scheme.</x:v>
+      </x:c>
+      <x:c r="O2" t="str"/>
       <x:c r="P2" t="str"/>
       <x:c r="Q2" t="str"/>
       <x:c r="R2" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -805,21 +802,25 @@
       <x:c r="H13" t="str"/>
       <x:c r="I13" t="str"/>
       <x:c r="J13" t="str">
-        <x:v>Occurs when a position is promoted through the manipulation of emotions, rather than through the presentation of an actual argument.</x:v>
+        <x:v>Occurs when a conclusion is pushed mainly by triggering fear, pity, outrage, pride, or hope rather than by showing that the conclusion follows from the evidence.</x:v>
       </x:c>
       <x:c r="K13" t="str">
-        <x:v>It would be awesome to know that we were not alone in the universe. I can't help but believe space aliens exist out there somewhere.</x:v>
+        <x:v>If you vote against this bill, remember the faces of the children who will suffer, and ask yourself how you will sleep at night.</x:v>
       </x:c>
       <x:c r="L13" t="str">
-        <x:v>This fallacy has itself been categorized as a tactical fallacy, but is a parent category for specific appeals to emotion that are not listed among the primary fallacies. - All appeal to emotion fallacies.</x:v>
-      </x:c>
-      <x:c r="M13" t="str"/>
-      <x:c r="N13" t="str"/>
+        <x:v>Emotion is not irrational by itself. The fallacy appears when emotion substitutes for the reasoning that still needs to be supplied.</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>In 2024 campaign advertising, immigration, crime, and abortion messages often relied on fear-laden images and worst-case anecdotes whose emotional force far exceeded the actual argument being made.</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>The spread of AI-generated political ads and deepfakes in 2024 showed how cheaply campaigns can trigger outrage or panic before voters have time to inspect the evidence.</x:v>
+      </x:c>
       <x:c r="O13" t="str"/>
       <x:c r="P13" t="str"/>
       <x:c r="Q13" t="str"/>
       <x:c r="R13" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1404,26 +1405,25 @@
         <x:v>appeal to ignorance</x:v>
       </x:c>
       <x:c r="J27" t="str">
-        <x:v>Assuming that something is true because it has not been proven false, or false because it has not been proven to be true.</x:v>
+        <x:v>Occurs when someone concludes that a claim is true because it has not been disproved, or false because it has not been proved.</x:v>
       </x:c>
       <x:c r="K27" t="str">
-        <x:v>Fairies must exist since we've seen no evidence falsifying their existence.</x:v>
+        <x:v>No one has proved that the leaked memo is fake, so it is probably genuine.</x:v>
       </x:c>
       <x:c r="L27" t="str">
-        <x:v>Phrases that often accompany this fallacy include "What are the odds!" and "Explain that!" The inability of the (or a particular) human brain to grasp the stochastic or conceptual complexities of a particular concept do not warrant the introduction of magic or a god or luck as an explanation.
-Note that there is warrant to dismiss out-of-hand claims that are logically or physically impossible. If I claim I possess a square triangle, or a flying reindeer, you are warranted in stating unequivocally that I am wrong.</x:v>
+        <x:v>The burden is not met by pointing to a gap in refutation. A claim needs positive support of its own. Lack of an explanation is not the same thing as evidence for a preferred explanation.</x:v>
       </x:c>
       <x:c r="M27" t="str">
-        <x:v>Some say we are warranted in believing that the Loch Ness Monster exists since there is no evidence to the contrary.</x:v>
+        <x:v>After an anonymous affidavit circulated online in September 2024 alleging that ABC had secretly rigged the Harris-Trump debate, many posts treated the absence of immediate disproof as if it were evidence that the allegation was real.</x:v>
       </x:c>
       <x:c r="N27" t="str">
-        <x:v>Some who do not accept a particular scientific theory often point to a single node in the matrix of converging lines of evidence for the theory, point out its short-comings, then claim the theory is wrong. If you've lived next to Betty and Bob for 20 years who are presumably married, and happen to see Betty with an unidentified man one afternoon, you are not warranted in believing that Betty and Bob are not married.</x:v>
+        <x:v>UAP discussions often jump from 'we do not yet know what caused this' to 'therefore it was extraterrestrial technology,' which treats unexplained as if it meant explained by the favored hypothesis.</x:v>
       </x:c>
       <x:c r="O27" t="str"/>
       <x:c r="P27" t="str"/>
       <x:c r="Q27" t="str"/>
       <x:c r="R27" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1757,21 +1757,25 @@
       <x:c r="H35" t="str"/>
       <x:c r="I35" t="str"/>
       <x:c r="J35" t="str">
-        <x:v>Making a probability judgment without taking into account known empirical statistics about the probability.</x:v>
+        <x:v>Occurs when someone judges how likely a case is by focusing on vivid case-specific evidence while ignoring the underlying frequency of the thing in question.</x:v>
       </x:c>
       <x:c r="K35" t="str">
-        <x:v>The rare disease detection device is 99% accurate, and it detected that I have a rare disease. Therefore I almost certainly do have a rare disease.</x:v>
+        <x:v>This fraud filter is 98% accurate and flagged my transaction, so there is almost no chance the alert is wrong.</x:v>
       </x:c>
       <x:c r="L35" t="str">
-        <x:v>If there are 10 terrorists in a city of 1,000,000, and you have a device on the subway that detects terrorists with a seemingly very high accuracy rate of 99.9%, you are going to experience 100 false positives of innocent citizens for every terrorist you correctly identify.</x:v>
-      </x:c>
-      <x:c r="M35" t="str"/>
-      <x:c r="N35" t="str"/>
+        <x:v>For rare conditions or rare events, even very accurate tests can generate more false positives than true positives. The missing question is not just 'How accurate is the test?' but 'How common is the condition before the test is applied?'</x:v>
+      </x:c>
+      <x:c r="M35" t="str">
+        <x:v>Discussion of noncitizen voting in the 2024 election often highlighted a handful of cases while skipping the base rate: tens of millions of lawful ballots were cast, so isolated cases do not by themselves show a widespread system-level problem.</x:v>
+      </x:c>
+      <x:c r="N35" t="str">
+        <x:v>Fraud detection, medical screening, and predictive-policing tools can sound highly reliable in percentage terms while still misclassifying large numbers of people when the targeted event is rare.</x:v>
+      </x:c>
       <x:c r="O35" t="str"/>
       <x:c r="P35" t="str"/>
       <x:c r="Q35" t="str"/>
       <x:c r="R35" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2815,29 +2819,25 @@
       <x:c r="H60" t="str"/>
       <x:c r="I60" t="str"/>
       <x:c r="J60" t="str">
-        <x:v>The misleading use of a term that has more than one meaning.</x:v>
+        <x:v>Occurs when a key word or phrase slides between different meanings inside the same argument, creating the illusion of support.</x:v>
       </x:c>
       <x:c r="K60" t="str">
-        <x:v>The strange man told me he wanted to take me out. I had him arrested for making a death threat.</x:v>
+        <x:v>The AI model can 'learn,' and students learn, so the model must understand lessons in the same way students do.</x:v>
       </x:c>
       <x:c r="L60" t="str">
-        <x:v>This example equivocates between the meaning of "take out" as an romantic activity, and "take out" as a murder.</x:v>
+        <x:v>Equivocation often works because the same word is doing two jobs at once. The surface grammar stays stable while the meaning shifts underneath.</x:v>
       </x:c>
       <x:c r="M60" t="str">
-        <x:v>You've probably heard the argument that "scientists can't even predict tomorrow's weather! What makes them thing they can predict the weather a decade from now?" This equivocates between daily weather predictions and yearly weather predictions. Daily weather predictions for 10 years from now are no better than they are for 10 days from now, but that does not mean climate scientists cannot accurately predict general trends in weather.</x:v>
+        <x:v>Debates over content moderation regularly equivocate between censorship by the state and moderation decisions by private platforms, as if both were the same kind of speech restriction.</x:v>
       </x:c>
       <x:c r="N60" t="str">
-        <x:v>Some people argue that, since humans wrote a holy book, a god did not write that particular holy book. This is an equivocation on the word "write" since it sometimes means "to pen" and other times "to author".</x:v>
-      </x:c>
-      <x:c r="O60" t="str">
-        <x:v>The word "faith" has recently been a word with diverse denotations that enable unproductive equivocation in dialog. Some will say "where the evidence ends, there faith begins", while in another context suggest that our belief that the sun will rise tomorrow is also "faith" though based on inductive reason and an understanding of the mechanism.</x:v>
-      </x:c>
-      <x:c r="P60" t="str">
-        <x:v>The term "theory" has 2 distinct meanings that are often conflated in equivocation when someone wishes to diminish the standing of a scientific theory. They simply replace the noble connotations associated with a scientific theory with the less-than-noble connotation of the vernacular use of "theory".</x:v>
-      </x:c>
+        <x:v>Public discussion of AI often slides between thin technical meanings of words such as 'reasoning,' 'understanding,' or 'hallucination' and thicker human meanings, which makes claims sound stronger than the evidence warrants.</x:v>
+      </x:c>
+      <x:c r="O60" t="str"/>
+      <x:c r="P60" t="str"/>
       <x:c r="Q60" t="str"/>
       <x:c r="R60" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -3550,24 +3550,25 @@
         <x:v>fallacy of insufficient statistics, fallacy of insufficient sample, fallacy of the lonely fact, leaping to a conclusion, hasty induction, secundum quid</x:v>
       </x:c>
       <x:c r="J77" t="str">
-        <x:v>Leaping to a conclusion with insufficient statistics or a insufficient sample size.</x:v>
+        <x:v>Occurs when someone draws a broad conclusion from too little evidence, too small a sample, or a badly skewed sample.</x:v>
       </x:c>
       <x:c r="K77" t="str">
-        <x:v>I drove through the town and counted 20 residents, all of them women. The town has only female residents.</x:v>
+        <x:v>I interviewed four students about AI and two admitted cheating, so generative AI is ruining education.</x:v>
       </x:c>
       <x:c r="L77" t="str">
-        <x:v>A hasty generalization might be a result of an insufficient sample size, imprecise measurements, or subjective reporting.
-This is a type of faulty generalization. A more detailed treatment of faulty generalizations can be found on the supplementary Inductive Errors page.</x:v>
+        <x:v>The problem is not moving from sample to population; all induction does that. The problem is pretending a weak or unrepresentative sample carries more weight than it does.</x:v>
       </x:c>
       <x:c r="M77" t="str">
-        <x:v>A foreign journalist who wanted to report on New York fashion might jump to a hasty generalization if visiting New York on October 31st.</x:v>
-      </x:c>
-      <x:c r="N77" t="str"/>
+        <x:v>A single viral video of a fight, theft, or protest is often used online as if it reveals what a whole city, campus, or demographic group is like.</x:v>
+      </x:c>
+      <x:c r="N77" t="str">
+        <x:v>Election commentary frequently treats one poll, one county, or one diner focus group as proof of a national shift, even when the broader polling picture is mixed.</x:v>
+      </x:c>
       <x:c r="O77" t="str"/>
       <x:c r="P77" t="str"/>
       <x:c r="Q77" t="str"/>
       <x:c r="R77" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -4211,28 +4212,25 @@
       </x:c>
       <x:c r="I93" t="str"/>
       <x:c r="J93" t="str">
-        <x:v>Occurs when the evidence presented to meet an initial standard of evidence is dismissed, and some greater standard of evidence is then imposed.</x:v>
+        <x:v>Occurs when evidence that was supposed to satisfy a stated standard is dismissed and a new, harder standard is introduced so the conclusion never has to be reconsidered.</x:v>
       </x:c>
       <x:c r="K93" t="str">
-        <x:v>I bet you can't lift this box! ... All right, I see you can lift that box, but I bet you can't lift this one over here!</x:v>
+        <x:v>If the model can pass the bar exam, I'll admit it is useful. It passes, and the reply becomes: useful doesn't count unless it can run an entire law firm without errors.</x:v>
       </x:c>
       <x:c r="L93" t="str">
-        <x:v>It is often difficult for both sides of an issue to agree upon what would constitute sufficient evidence. However, such an agreement is foundational to any real progress in an honest discussion.</x:v>
+        <x:v>Standards can be refined in good faith, especially when both sides notice a weak test. The fallacy appears when the revision functions mainly to avoid conceding that the earlier standard was met.</x:v>
       </x:c>
       <x:c r="M93" t="str">
-        <x:v>There have been many claims throughout recent years made by dualists about the limits of brain science to explain mental processes with the implication that belief in dualism is therefore warranted. When new studies falsify these claims, new claims are introduced.</x:v>
+        <x:v>Public AI debates in 2024 often moved from benchmark scores to some new test the moment a model cleared the previous bar, making 'proof' of competence permanently out of reach.</x:v>
       </x:c>
       <x:c r="N93" t="str">
-        <x:v>With many of the moon landing conspiracy theorists, as each of their claims is rebutted, they will move on to the next claim saying "But what about..." There appears to be no set degree of evidence that will convince them.</x:v>
-      </x:c>
-      <x:c r="O93" t="str">
-        <x:v>Consider the following popular internet post.Boy writes God a letter, "Dear God, why do you let bad things happen in our schools?" God replies,"Dear son, I'm not allowed in your schools."
-If this particular god is giving his banishment from schools as the sole reason why bad things happen in those schools, then schools in which this particular god is allowed should not experience bad things. When presented with this corollary, those defending the quote often move the goalpost back to a more sensible and defensible position that makes the presence of bad people in schools the reason for bad things happening in those schools.</x:v>
-      </x:c>
+        <x:v>Election-conspiracy arguments often work this way: once courts, audits, and recounts address one claim, the standard shifts to a different alleged irregularity without any willingness to concede what the earlier evidence settled.</x:v>
+      </x:c>
+      <x:c r="O93" t="str"/>
       <x:c r="P93" t="str"/>
       <x:c r="Q93" t="str"/>
       <x:c r="R93" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -4384,25 +4382,25 @@
       </x:c>
       <x:c r="I97" t="str"/>
       <x:c r="J97" t="str">
-        <x:v>Occurs when a conventional categorization is denied based on unconventional or arbitrary criteria.</x:v>
+        <x:v>Occurs when someone protects a generalization from counterexamples by redefining the group with an ad hoc 'real' or 'true' membership test.</x:v>
       </x:c>
       <x:c r="K97" t="str">
-        <x:v>How can you call yourself a patriot when you are against this war!</x:v>
+        <x:v>No real conservative would support that immigration bill.</x:v>
       </x:c>
       <x:c r="L97" t="str">
-        <x:v>Those who employ this fallacy will often interject ad hoc or arbitrary criteria to maintain an artificial delineation.</x:v>
+        <x:v>Sometimes categories do have genuine criteria. The fallacy arises when the criteria are improvised only after a counterexample appears, so the definition changes to save the claim.</x:v>
       </x:c>
       <x:c r="M97" t="str">
-        <x:v>If a theist informs an atheist that his position is indefensible since Stalin was an atheist, it would be a no true Scotsman fallacy for the atheist to suggest that Stalin was not a real atheist. And it would be forfeiting the chance to point out the theist's own fallacy of top-down condemnation.</x:v>
+        <x:v>In 2024 intraparty fights, Republicans who backed Ukraine aid or accepted the 2020 certification were often dismissed as 'not real conservatives' instead of being treated as counterexamples within conservatism.</x:v>
       </x:c>
       <x:c r="N97" t="str">
-        <x:v>If an atheist informs a Christian that his position is indefensible since Hitler was an Christian, it would be a no true Scotsman fallacy for the theist to suggest that Hitler was not a real Christian. And it would be forfeiting the chance to point out the atheist's own fallacy of top-down condemnation.</x:v>
+        <x:v>Religious and ideological arguments frequently insist that anyone whose behavior embarrasses the group was never a 'true' believer in the first place, which preserves group purity by redefinition.</x:v>
       </x:c>
       <x:c r="O97" t="str"/>
       <x:c r="P97" t="str"/>
       <x:c r="Q97" t="str"/>
       <x:c r="R97" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -4772,23 +4770,25 @@
         <x:v>false cause, coincidental correlation, correlation not causation</x:v>
       </x:c>
       <x:c r="J106" t="str">
-        <x:v>Occurs when a cause of a phenomenon is attributed to a prior phenomenon without providing evidence of causation.</x:v>
+        <x:v>Occurs when someone infers that because one event happened before another, the earlier event caused the later one.</x:v>
       </x:c>
       <x:c r="K106" t="str">
-        <x:v>After I started wearing a copper bracelet, my health improved! It worked!</x:v>
+        <x:v>I started a new supplement on Monday and my headaches eased by Friday, so the supplement must have fixed the problem.</x:v>
       </x:c>
       <x:c r="L106" t="str">
-        <x:v>Causation must be rigorously demonstrated. Phenomena that occur in sequence do not necessarily have a causal link. This fallacy is related to the correlation is not causation fallacy.</x:v>
+        <x:v>Temporal order matters for causation, but it is only one ingredient. The improvement might be coincidence, regression to the mean, other background changes, or a different cause entirely.</x:v>
       </x:c>
       <x:c r="M106" t="str">
-        <x:v>Most people feel a period of elation every time they voluntarily change jobs. Many are tempted to cite the conditions of the new job as the reason for their better mood. Is it the new job that is causing the elation, or merely the change?</x:v>
-      </x:c>
-      <x:c r="N106" t="str"/>
+        <x:v>Wellness and self-optimization discourse in 2024 routinely credited cold plunges, supplements, or glucose hacks for improvements that followed several simultaneous lifestyle changes.</x:v>
+      </x:c>
+      <x:c r="N106" t="str">
+        <x:v>Politicians often claim that a policy worked because a good trend appeared soon after the policy was announced, even when the trend began earlier or other explanations remain stronger.</x:v>
+      </x:c>
       <x:c r="O106" t="str"/>
       <x:c r="P106" t="str"/>
       <x:c r="Q106" t="str"/>
       <x:c r="R106" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
@@ -5980,25 +5980,25 @@
         <x:v>two wrongs make a right</x:v>
       </x:c>
       <x:c r="J134" t="str">
-        <x:v>Occurs when it is assumed that, if one wrong has been committed, another wrong will remove its culpability.</x:v>
+        <x:v>Occurs when criticism is answered not by engaging the issue, but by pointing to similar hypocrisy or wrongdoing elsewhere.</x:v>
       </x:c>
       <x:c r="K134" t="str">
-        <x:v>I admit to stretching the truth a bit, but you and everyone else tells a white lie from time to time. You can't judge me.</x:v>
+        <x:v>You cannot criticize my fabricated quote because your side spreads misinformation too.</x:v>
       </x:c>
       <x:c r="L134" t="str">
-        <x:v>No degree of hypocrisy will invalidate the hypocrite's argument.</x:v>
+        <x:v>Hypocrisy can matter for trust, but it does not by itself answer whether the original claim, act, or argument was wrong.</x:v>
       </x:c>
       <x:c r="M134" t="str">
-        <x:v>There are very few countries that have not been called "terrorist states". Whenever hostilities escalate, there is commonly an exchange of such accusations.</x:v>
+        <x:v>In the June 27, 2024 Biden-Trump debate and the September 10, 2024 Harris-Trump debate, many charges were met with 'your side did it too' responses that redirected blame without addressing the original allegation.</x:v>
       </x:c>
       <x:c r="N134" t="str">
-        <x:v>Whenever skeptics disparage faith as a failed approach to truth, theists often retort "But you have faith in science!" This is to ignore the warranted inductively-derived confidence skeptics place in the superior reputation of success that science enjoys over faith. Only where the degree of belief is not commensurate to the degree of evidence is belief unwarranted, and the degree of inductive evidence of science's success is quite high.</x:v>
+        <x:v>Arguments about misinformation, climate, religion, and media bias often slide into scorekeeping about who is worse rather than whether the specific criticized claim is true or justified.</x:v>
       </x:c>
       <x:c r="O134" t="str"/>
       <x:c r="P134" t="str"/>
       <x:c r="Q134" t="str"/>
       <x:c r="R134" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="135">

</xml_diff>

<commit_message>
Modernize additional classic fallacies
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R72869a05766e45b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rcc7d7bbd5192405d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R5f3831ef85bb4749"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re922b3b1e6d44545"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R9afeaebffa634e78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R287248fcd40a4654"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -754,27 +754,25 @@
       </x:c>
       <x:c r="I12" t="str"/>
       <x:c r="J12" t="str">
-        <x:v>An argument that assumes the consequences of an idea, to some degree, reflect the veracity of the idea.</x:v>
+        <x:v>Occurs when someone treats the desirability or undesirability of a conclusion as if it were evidence that the conclusion is true or false.</x:v>
       </x:c>
       <x:c r="K12" t="str">
-        <x:v>If a virus erased my hard-drive, I'd loose all my work documents. It can't possibly happen.</x:v>
+        <x:v>If climate change were really this serious, it would mean expensive changes to how we live and work, so the science must be exaggerated.</x:v>
       </x:c>
       <x:c r="L12" t="str">
-        <x:v>This is usually an argument that plays on vested interests.</x:v>
+        <x:v>Consequences matter for what we should do, but they do not by themselves determine what is true. A painful implication does not refute a claim, and a comforting implication does not confirm one.</x:v>
       </x:c>
       <x:c r="M12" t="str">
-        <x:v>It has been frequently argued that there can't possibly be a god since it would mean he has allowed evil and suffering in the world. The mere negative consequences do not deny the possibility of a god. You must also explain why a god would necessarily not permit evil and suffering in the world.</x:v>
+        <x:v>Some climate arguments treat the economic and political inconvenience of decarbonization as if it counted against the underlying science itself.</x:v>
       </x:c>
       <x:c r="N12" t="str">
-        <x:v>A common argument heard is that, because Hitler based his genocide on evolution, this is an indication that evolution is wrong.</x:v>
-      </x:c>
-      <x:c r="O12" t="str">
-        <x:v>A very common argument for an eternal soul is "If we do not have a soul, then we would be without an objective purpose!" The argument usually ends here with the implication that such a conclusion is unthinkable and unacceptable. An honest thinker dismisses no conclusion due to the emotional discomfort that accompanies it.</x:v>
-      </x:c>
+        <x:v>In debates about AI consciousness, animal cognition, or moral status, people sometimes argue that the conclusion cannot be right because accepting it would create uncomfortable obligations.</x:v>
+      </x:c>
+      <x:c r="O12" t="str"/>
       <x:c r="P12" t="str"/>
       <x:c r="Q12" t="str"/>
       <x:c r="R12" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -978,28 +976,25 @@
       <x:c r="H17" t="str"/>
       <x:c r="I17" t="str"/>
       <x:c r="J17" t="str">
-        <x:v>An argument in which something is deemed correct or good if it is natural, and is deemed incorrect or bad if it is unnatural.</x:v>
+        <x:v>Occurs when something is praised as good, safe, or right merely because it is called natural, or condemned as bad merely because it is called unnatural.</x:v>
       </x:c>
       <x:c r="K17" t="str">
-        <x:v>Birds are monogamous. Therefore, humans should also be monogamous.</x:v>
+        <x:v>This remedy must be safer than prescription medicine because it is completely natural.</x:v>
       </x:c>
       <x:c r="L17" t="str">
-        <x:v>It does not take much exploration of nature to realize that it is not a very coherent or desirable standard for human conduct. Nor is nature, as is, very amenable to human survival. This is why medicine perennially combats the influenza virus, and would eradicate it if possible. Interestingly, the most "natural" of all actions inherent to life is the striving for survival. This puts humans at odds with the rest of nature and what is "natural". This is why we ingest neither natural hemlock nor synthetic poisons.
-In many cases, once the act that is deemed "unnatural" is scrutinized, it is discovered that the act is merely emotionally unpalatable to the person making the categorization.</x:v>
+        <x:v>Natural things can heal, but they can also poison, infect, and kill. The fallacy treats a vague origin label as if it already settled the medical, moral, or practical question.</x:v>
       </x:c>
       <x:c r="M17" t="str">
-        <x:v>Some claim that genetically modified crops are "wrong" for the sole reason that they are not what nature has naturally produced. There may be good reason for caution in growing genetically-modified crops, but the fact that they are merely "unnatural" is not good reason.</x:v>
+        <x:v>Wellness marketing for raw milk, supplements, and 'clean' products often treats natural as if it automatically meant safer, healthier, or morally superior.</x:v>
       </x:c>
       <x:c r="N17" t="str">
-        <x:v>While there are sects that eschew medical intervention, most humans seek medical attention when they are injured rather than allowing nature to run its course.</x:v>
-      </x:c>
-      <x:c r="O17" t="str">
-        <x:v>Cocaine was once touted as a "natural" remedy for many ailments. Today, not many consider the use of cocaine to be a very wise treatment due to its addictive effects.</x:v>
-      </x:c>
+        <x:v>Arguments about sex, family, and medicine often smuggle a moral conclusion into the descriptive claim that one pattern is simply 'what nature intended.'</x:v>
+      </x:c>
+      <x:c r="O17" t="str"/>
       <x:c r="P17" t="str"/>
       <x:c r="Q17" t="str"/>
       <x:c r="R17" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1151,23 +1146,25 @@
       <x:c r="H21" t="str"/>
       <x:c r="I21" t="str"/>
       <x:c r="J21" t="str">
-        <x:v>Assuming that, because something could happen, it is inevitable that it will happen.</x:v>
+        <x:v>Occurs when someone assumes that because something could happen, it is therefore likely or inevitable that it will happen.</x:v>
       </x:c>
       <x:c r="K21" t="str">
-        <x:v>I'm bound to win the lottery if I just keep buying tickets.</x:v>
+        <x:v>If I keep backing enough meme stocks, one of them is bound to make me rich.</x:v>
       </x:c>
       <x:c r="L21" t="str">
-        <x:v>A remote possibility does not equate to an inevitability for a finite life.</x:v>
+        <x:v>Possibility is a very weak starting point. Many things are possible without being probable, and many probable things still fail to happen in any given case.</x:v>
       </x:c>
       <x:c r="M21" t="str">
-        <x:v>The real possibility that a meteor will strike your house while you sleep does not warrant your concern.</x:v>
-      </x:c>
-      <x:c r="N21" t="str"/>
+        <x:v>Crypto, lottery, and sports-betting talk often slides from 'this could happen' to 'this is bound to happen,' especially after a short streak of wins.</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>Election and catastrophe commentary often treats a legally or physically possible scenario as if it were destined simply because people can imagine it vividly.</x:v>
+      </x:c>
       <x:c r="O21" t="str"/>
       <x:c r="P21" t="str"/>
       <x:c r="Q21" t="str"/>
       <x:c r="R21" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1279,23 +1276,25 @@
       <x:c r="H24" t="str"/>
       <x:c r="I24" t="str"/>
       <x:c r="J24" t="str">
-        <x:v>Occurs when a claim is deemed correct on the basis that it has a long-standing tradition behind it.</x:v>
+        <x:v>Occurs when a claim or practice is defended mainly because it has a long history, customary status, or familiar place in a community.</x:v>
       </x:c>
       <x:c r="K24" t="str">
-        <x:v>Polygamy is wrong because marriage here in our country has long been only between one man and one women.</x:v>
+        <x:v>We have always opened school ceremonies this way, so that must be the right way to do it.</x:v>
       </x:c>
       <x:c r="L24" t="str">
-        <x:v>All traditional practices were at one time new. The age of a practice neither validates or invalidates the practice. Patricide, child sacrifice and self-immolation were all well-established traditions at one time, yet are now generally abhorred.</x:v>
+        <x:v>Traditions can embody wisdom, but age alone does not prove justice, truth, or usefulness. A tradition still has to survive present scrutiny.</x:v>
       </x:c>
       <x:c r="M24" t="str">
-        <x:v>Both extremes on the issue of public nudity have invoked this fallacy to justify their position.</x:v>
-      </x:c>
-      <x:c r="N24" t="str"/>
+        <x:v>In 2024 arguments that the United States is a 'Christian nation,' long practice and selective founding-era precedent were often treated as if they settled the constitutional question.</x:v>
+      </x:c>
+      <x:c r="N24" t="str">
+        <x:v>Arguments about schooling, marriage, and gender roles often rely on 'we have always done it this way' instead of showing why the tradition remains just or effective.</x:v>
+      </x:c>
       <x:c r="O24" t="str"/>
       <x:c r="P24" t="str"/>
       <x:c r="Q24" t="str"/>
       <x:c r="R24" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1363,23 +1362,25 @@
       <x:c r="H26" t="str"/>
       <x:c r="I26" t="str"/>
       <x:c r="J26" t="str">
-        <x:v>Assuming that, if an argument for some conclusion is fallacious, then the conclusion is false.</x:v>
+        <x:v>Occurs when someone infers that because a particular argument for a conclusion is weak or fallacious, the conclusion itself must therefore be false.</x:v>
       </x:c>
       <x:c r="K26" t="str">
-        <x:v>Tom told me that, because all Cubans are human, and I am a human, therefore I am a Cuban. His argument is invalid, and therefore I am not a Cuban.</x:v>
+        <x:v>That activist exaggerated one statistic about housing, so the housing shortage itself must be a myth.</x:v>
       </x:c>
       <x:c r="L26" t="str">
-        <x:v>The fact that someone commits a fallacy when defending a claim does not make their claim false.</x:v>
+        <x:v>A bad argument can defend a true claim, and a strong claim can be defended poorly. Refuting the reasoning offered is not the same thing as refuting the conclusion.</x:v>
       </x:c>
       <x:c r="M26" t="str">
-        <x:v>This fallacy is common in heated discussions in which ad hominem attacks are frequent. Often the person attacked will point to the ad hominem, then declare their own position validated.</x:v>
-      </x:c>
-      <x:c r="N26" t="str"/>
+        <x:v>When a candidate exaggerates one statistic, opponents often jump from 'that argument was flawed' to 'the broader policy position must therefore be false.'</x:v>
+      </x:c>
+      <x:c r="N26" t="str">
+        <x:v>Online 'gotcha' culture frequently treats catching a fallacious defense as if it automatically disproved whatever the speaker was trying to defend.</x:v>
+      </x:c>
       <x:c r="O26" t="str"/>
       <x:c r="P26" t="str"/>
       <x:c r="Q26" t="str"/>
       <x:c r="R26" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -3111,27 +3112,25 @@
       <x:c r="H67" t="str"/>
       <x:c r="I67" t="str"/>
       <x:c r="J67" t="str">
-        <x:v>A case in which the analogy fails to coherently maintain a parallel to the original concept on the point in question.</x:v>
+        <x:v>Occurs when one thing is treated as sufficiently like another even though the comparison breaks down at the point the argument depends on.</x:v>
       </x:c>
       <x:c r="K67" t="str">
-        <x:v>Because physicists say mass equals energy, therefore mass can travel the speed of light.</x:v>
+        <x:v>A chatbot writes essays a bit like a student, so teaching with chatbots must be basically the same as hiring a tutor.</x:v>
       </x:c>
       <x:c r="L67" t="str">
-        <x:v>If some system A has both function X and function Y, and some system B has a function X′ corresponding to A's function X, then the system B should also have a function Y′ that is analogous to A's function Y for the analogy to succeed.</x:v>
+        <x:v>Analogies can clarify unfamiliar ideas, but they prove very little unless the shared features are actually relevant to the conclusion being drawn.</x:v>
       </x:c>
       <x:c r="M67" t="str">
-        <x:v>Consider the following argument. Teaching teenagers how to succeed in marriage prior to being married is like trying to teach someone how to ride a bicycle prior to placing them on a bicycle.
-This is a false analogy in that it assumes the same type of learning mechanism used for the muscular memory of cycling is also used for grasping the dynamics of marriage.</x:v>
+        <x:v>Debates about AI frequently compare models to children, interns, parrots, or brains, then carry over conclusions from the analogy that the underlying system may not support.</x:v>
       </x:c>
       <x:c r="N67" t="str">
-        <x:v>Consider the following argument. Dating is like gambling. You'll win a few, and lose a few.
-This is a false analogy in that it ignores the non-randon aspects of selecting a date.</x:v>
+        <x:v>Fiscal debates often compare a national budget to a household budget; the analogy can illuminate some constraints but breaks down when it is treated as a full map of macroeconomics.</x:v>
       </x:c>
       <x:c r="O67" t="str"/>
       <x:c r="P67" t="str"/>
       <x:c r="Q67" t="str"/>
       <x:c r="R67" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -3500,27 +3499,25 @@
       <x:c r="H76" t="str"/>
       <x:c r="I76" t="str"/>
       <x:c r="J76" t="str">
-        <x:v>Occurs when a conclusion is suggested based solely on something or someone's origin rather than its current meaning or context.</x:v>
+        <x:v>Occurs when a claim, practice, or idea is judged mainly by its origin rather than by its present content, evidence, or merits.</x:v>
       </x:c>
       <x:c r="K76" t="str">
-        <x:v>Australia will never become a great nation considering it arose from penal colonies of mere criminals.</x:v>
+        <x:v>That proposal started on TikTok, so it must be nonsense.</x:v>
       </x:c>
       <x:c r="L76" t="str">
-        <x:v>The value of ideas and strength of arguments can be assessed wholly independently of the conditions of their engendering.</x:v>
+        <x:v>Origins can matter when they reveal bias, incentives, or reliability concerns. The fallacy appears when origin is treated as enough to settle the issue without examining the claim itself.</x:v>
       </x:c>
       <x:c r="M76" t="str">
-        <x:v>Some suggest that the cruel human experiments Nazi conducted cannot be scientifically reliable. The conditions surrounding the the data collection does not invalidate the reliability of that data.</x:v>
+        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported.</x:v>
       </x:c>
       <x:c r="N76" t="str">
-        <x:v>Claiming that Christmas trees are somehow evil since they originated in pagan tradition would be a genetic fallacy.</x:v>
-      </x:c>
-      <x:c r="O76" t="str">
-        <x:v>Refusing to celebrate Halloween since it had its origin in superstition and myth would be a genetic fallacy.</x:v>
-      </x:c>
+        <x:v>In cultural and religious arguments, a practice or symbol is often condemned solely because of its historical roots, even when the live question is what it means or does now.</x:v>
+      </x:c>
+      <x:c r="O76" t="str"/>
       <x:c r="P76" t="str"/>
       <x:c r="Q76" t="str"/>
       <x:c r="R76" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -4726,25 +4723,25 @@
       <x:c r="H105" t="str"/>
       <x:c r="I105" t="str"/>
       <x:c r="J105" t="str">
-        <x:v>Where negative claims are preemptively made against a position with the intention of discrediting whatever person is about to say.</x:v>
+        <x:v>Occurs when negative framing is introduced in advance so that whatever a person says next will be dismissed before it is fairly heard.</x:v>
       </x:c>
       <x:c r="K105" t="str">
-        <x:v>Before my opponent speaks, let me remind you that he is a college dropout and has never held a job longer than a year.</x:v>
+        <x:v>Before this researcher speaks, remember that she once worked in Washington, so you already know what kind of agenda she has.</x:v>
       </x:c>
       <x:c r="L105" t="str">
-        <x:v>This fallacy is often found in public forums where the audience includes those who lack critical thinking skills and who are prone to emotional arguments.</x:v>
+        <x:v>Source criticism can be relevant, but poisoning the well tries to make the audience stop listening before the argument or evidence is even on the table.</x:v>
       </x:c>
       <x:c r="M105" t="str">
-        <x:v>Sarah Palin's crowning as a beauty pageant queen in 1984 is often introduced by those who wish to bring into question her competency. Beauty pageant contestants are often considered less intelligent than what is needed for public office.</x:v>
+        <x:v>In political and media fights, audiences are often primed to treat a judge, journalist, scientist, or witness as corrupt before that person's specific evidence is even heard.</x:v>
       </x:c>
       <x:c r="N105" t="str">
-        <x:v>Barack Obama's Muslim father is often brought up in political dialogue in an attempt to poison the well. Many Americans have a fear of a Muslim agenda in Washington. His middle name "Hussein" is also emphsized to heightened this fear.</x:v>
+        <x:v>After the September 2024 Harris-Trump debate, repeated claims that moderators and outlets were inherently rigged encouraged supporters to dismiss later fact-checks in advance rather than assess them on the merits.</x:v>
       </x:c>
       <x:c r="O105" t="str"/>
       <x:c r="P105" t="str"/>
       <x:c r="Q105" t="str"/>
       <x:c r="R105" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
@@ -4976,21 +4973,25 @@
       <x:c r="H111" t="str"/>
       <x:c r="I111" t="str"/>
       <x:c r="J111" t="str">
-        <x:v>Occurs when a speaker attempts to distract the audience from an unresolved topic by introducing a new topic the speaker feels more comfortable with.</x:v>
+        <x:v>Occurs when someone diverts attention from the unresolved issue by switching to a different issue that is easier, safer, or more emotionally useful.</x:v>
       </x:c>
       <x:c r="K111" t="str">
-        <x:v>I don't have evidence with me that home-schooling best prepares students for university, but, anyway, if we don't home-school our children, they will end up with few morals.</x:v>
+        <x:v>Asked whether the housing plan would lower rents, the candidate pivots to the failures of the other party's immigration policy.</x:v>
       </x:c>
       <x:c r="L111" t="str">
-        <x:v>Most of the tactical and emotional fallacies fall into this general category.</x:v>
-      </x:c>
-      <x:c r="M111" t="str"/>
-      <x:c r="N111" t="str"/>
+        <x:v>Not every detour is fallacious; context can matter. The fallacy appears when the diversion substitutes for addressing the question that was actually on the table.</x:v>
+      </x:c>
+      <x:c r="M111" t="str">
+        <x:v>In the June 27, 2024 Biden-Trump debate, answers about the economy, abortion, and January 6 often veered into immigration, personal fitness, or unrelated grievances instead of the question asked.</x:v>
+      </x:c>
+      <x:c r="N111" t="str">
+        <x:v>Online arguments about institutional abuse, policing, or bias often slide away from the specific allegation and into some other controversy the speaker would rather discuss.</x:v>
+      </x:c>
       <x:c r="O111" t="str"/>
       <x:c r="P111" t="str"/>
       <x:c r="Q111" t="str"/>
       <x:c r="R111" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="112">

</xml_diff>

<commit_message>
Modernize emotional and tactical fallacies
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re922b3b1e6d44545"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R9afeaebffa634e78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R287248fcd40a4654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9c2fccc48bc4418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R11b4ceae84534631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rb52d371b11034e7b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -846,25 +846,25 @@
       </x:c>
       <x:c r="I14" t="str"/>
       <x:c r="J14" t="str">
-        <x:v>An appeal to emotion where an argument is made by increasing fear and prejudice towards the opposing side.</x:v>
+        <x:v>Occurs when someone tries to secure agreement mainly by amplifying danger, threat, or panic rather than by showing that the conclusion is supported.</x:v>
       </x:c>
       <x:c r="K14" t="str">
-        <x:v>If you don't vote her into office, terrorism will accelerate, and our great nation will fall.</x:v>
+        <x:v>If we do not pass this surveillance bill tonight, the next attack will be on our hands.</x:v>
       </x:c>
       <x:c r="L14" t="str">
-        <x:v>Appealing to fear works. You won't find many atheists in countries where atheism warrants the death penalty. Fear has long been co-opted to initiate wars and oppressive laws.</x:v>
+        <x:v>Fear can be rational when the threat is real and well evidenced. The fallacy appears when fear does the persuasive work that evidence and reasoning have not done.</x:v>
       </x:c>
       <x:c r="M14" t="str">
-        <x:v>Many religions claim that if you don't believe their "loving" god is the true god, you will be tortured forever.</x:v>
+        <x:v>Campaign messaging about immigrants, crime, and cultural decline often relies on catastrophic imagery that outruns the actual evidence offered for the policy being sold.</x:v>
       </x:c>
       <x:c r="N14" t="str">
-        <x:v>Fear of death is what compels many cancer patients to accept the mendacious claims of snake-oil salesmen.</x:v>
+        <x:v>Scams involving miracle cures, emergency investments, or account security often push people to act before they can think by making delay feel dangerous.</x:v>
       </x:c>
       <x:c r="O14" t="str"/>
       <x:c r="P14" t="str"/>
       <x:c r="Q14" t="str"/>
       <x:c r="R14" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -934,21 +934,25 @@
       <x:c r="H16" t="str"/>
       <x:c r="I16" t="str"/>
       <x:c r="J16" t="str">
-        <x:v>Occurs when a premise is dismissed, by calling into question the motives of its sponsor.</x:v>
+        <x:v>Occurs when a claim is dismissed by speculating about the speaker's motives instead of addressing the claim itself.</x:v>
       </x:c>
       <x:c r="K16" t="str">
-        <x:v>The director gave her the leading role only because he wanted to date her.</x:v>
+        <x:v>Of course the researcher says rent control backfires; landlords fund her institute.</x:v>
       </x:c>
       <x:c r="L16" t="str">
-        <x:v>While a questionable motive might allow us to expect a particular bias within the argument, it is the argument itself that must be assessed.</x:v>
-      </x:c>
-      <x:c r="M16" t="str"/>
-      <x:c r="N16" t="str"/>
+        <x:v>Motives can be relevant to bias and credibility, but they do not automatically settle whether the argument or evidence is sound.</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>After the September 2024 ABC debate, accusations about moderator bias were often used not just to question fairness, but to pre-dismiss later fact-checks without engaging their substance.</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>In debates about climate, vaccines, and AI policy, critics are often waved away as 'funded,' 'bought,' or 'performing for clicks' instead of being answered.</x:v>
+      </x:c>
       <x:c r="O16" t="str"/>
       <x:c r="P16" t="str"/>
       <x:c r="Q16" t="str"/>
       <x:c r="R16" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1022,21 +1026,25 @@
       <x:c r="H18" t="str"/>
       <x:c r="I18" t="str"/>
       <x:c r="J18" t="str">
-        <x:v>Occurs when a proposal is claimed to be superior or better solely based on it being new or modern.</x:v>
+        <x:v>Occurs when something is treated as better mainly because it is new, cutting-edge, or marketed as the future.</x:v>
       </x:c>
       <x:c r="K18" t="str">
-        <x:v>This brilliant strategy that the management has introduced is revolutionary and will change the way we do business!</x:v>
+        <x:v>This AI-first classroom platform is obviously better than the old method because it is the future of learning.</x:v>
       </x:c>
       <x:c r="L18" t="str">
-        <x:v>This fallacy often results from the human tendency for change and new stimuli.</x:v>
-      </x:c>
-      <x:c r="M18" t="str"/>
-      <x:c r="N18" t="str"/>
+        <x:v>New tools and ideas can be improvements, but novelty itself is not proof. The relevant questions are performance, tradeoffs, and evidence, not freshness.</x:v>
+      </x:c>
+      <x:c r="M18" t="str">
+        <x:v>In the 2024 rush to adopt generative AI, many products were pitched as inherently superior because they were new, even when reliability, labor impact, and safety were still unsettled.</x:v>
+      </x:c>
+      <x:c r="N18" t="str">
+        <x:v>Political and management rhetoric often treats 'innovation' as a reason to trust a strategy before any serious test of whether it solves the underlying problem.</x:v>
+      </x:c>
       <x:c r="O18" t="str"/>
       <x:c r="P18" t="str"/>
       <x:c r="Q18" t="str"/>
       <x:c r="R18" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1064,21 +1072,25 @@
       </x:c>
       <x:c r="I19" t="str"/>
       <x:c r="J19" t="str">
-        <x:v>An argument in which the evoking of sympathy is used in an attempt to validate the argument.</x:v>
+        <x:v>Occurs when sympathy for a person or group is used as if it were evidence that a claim is true or a conclusion follows.</x:v>
       </x:c>
       <x:c r="K19" t="str">
-        <x:v>If there is no after-life, then the lives of tens of millions suffering in poverty have no meaning.</x:v>
+        <x:v>You have to pass me, professor. If I fail, I lose my scholarship and disappoint my family.</x:v>
       </x:c>
       <x:c r="L19" t="str">
-        <x:v>This is only a fallacy when it serves as a foundation for a belief in a particular claim.</x:v>
-      </x:c>
-      <x:c r="M19" t="str"/>
-      <x:c r="N19" t="str"/>
+        <x:v>Compassion can matter for what response is humane, but it does not determine whether the underlying claim has been proved.</x:v>
+      </x:c>
+      <x:c r="M19" t="str">
+        <x:v>Fundraising and advocacy campaigns sometimes imply that questioning a factual claim is itself heartless, shifting the pressure from evidence to emotional identification.</x:v>
+      </x:c>
+      <x:c r="N19" t="str">
+        <x:v>Public figures under scrutiny sometimes ask to be believed or excused because they are suffering, overwhelmed, or facing intense pressure, even when those facts do not establish the truth of what they are saying.</x:v>
+      </x:c>
       <x:c r="O19" t="str"/>
       <x:c r="P19" t="str"/>
       <x:c r="Q19" t="str"/>
       <x:c r="R19" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1192,21 +1204,25 @@
       </x:c>
       <x:c r="I22" t="str"/>
       <x:c r="J22" t="str">
-        <x:v>An argument in which the use of ridicule or shame is introduced in an attempt to invalidate the opposing position.</x:v>
+        <x:v>Occurs when mockery, embarrassment, or derision is used in place of showing why a view is false.</x:v>
       </x:c>
       <x:c r="K22" t="str">
-        <x:v>So, since you believe in evolution, you have to believe your grandfather was an ape! Hilarious!</x:v>
+        <x:v>You care about online privacy? What are you, hiding in a tinfoil bunker?</x:v>
       </x:c>
       <x:c r="L22" t="str">
-        <x:v>Ridicule is a fallacy only when it is used to persuade others to hold a certain belief.</x:v>
-      </x:c>
-      <x:c r="M22" t="str"/>
-      <x:c r="N22" t="str"/>
+        <x:v>Ridicule can make a position look silly without ever testing whether it is wrong. Laughter is not an argument.</x:v>
+      </x:c>
+      <x:c r="M22" t="str">
+        <x:v>Debates about religion, feminism, climate, and AI are often reduced to memes whose purpose is to make one side look ridiculous rather than to assess the actual claim.</x:v>
+      </x:c>
+      <x:c r="N22" t="str">
+        <x:v>Online discourse frequently treats a sarcastic dunk or quote-tweet pile-on as if public humiliation itself were refutation.</x:v>
+      </x:c>
       <x:c r="O22" t="str"/>
       <x:c r="P22" t="str"/>
       <x:c r="Q22" t="str"/>
       <x:c r="R22" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1234,21 +1250,25 @@
       </x:c>
       <x:c r="I23" t="str"/>
       <x:c r="J23" t="str">
-        <x:v>An appeal to emotion in which an argument is made through exploiting bitterness towards the proponents of an opposing position.</x:v>
+        <x:v>Occurs when resentment, bitterness, or hostility toward another group is used to drive support for a conclusion.</x:v>
       </x:c>
       <x:c r="K23" t="str">
-        <x:v>If you think we should bailout that bank, consider that the incompetent traders who created this financial fiasco will be celebrating with champagne while we, the common folk, will be paying even higher taxes.</x:v>
+        <x:v>Do not support student debt relief; think of the smug graduates who will celebrate while you keep paying.</x:v>
       </x:c>
       <x:c r="L23" t="str">
-        <x:v>What some might call an appeal to spite others might call an appeal to justice, so this fallacy can be quite fuzzy.</x:v>
-      </x:c>
-      <x:c r="M23" t="str"/>
-      <x:c r="N23" t="str"/>
+        <x:v>Anger at the people who might benefit from a policy does not settle whether the policy is wise, fair, or effective.</x:v>
+      </x:c>
+      <x:c r="M23" t="str">
+        <x:v>Campaign messages often invite voters to reject a proposal because hated elites, immigrants, bankers, or academics might benefit, even when that says nothing about the proposal's merits.</x:v>
+      </x:c>
+      <x:c r="N23" t="str">
+        <x:v>Social-media outrage often works by making the audience feel that supporting a view would somehow reward people they already dislike.</x:v>
+      </x:c>
       <x:c r="O23" t="str"/>
       <x:c r="P23" t="str"/>
       <x:c r="Q23" t="str"/>
       <x:c r="R23" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -3192,23 +3212,25 @@
       <x:c r="H69" t="str"/>
       <x:c r="I69" t="str"/>
       <x:c r="J69" t="str">
-        <x:v>Is the assertion that a compromise near the middle of two positions is correct.</x:v>
+        <x:v>Occurs when the midpoint between two positions is treated as correct simply because it lies between them.</x:v>
       </x:c>
       <x:c r="K69" t="str">
-        <x:v>If the cyclist had been wearing a helmet as he ought to have, my drunk driving would not have killed him. The court should reduce my prison sentence from 10 to 5 years.</x:v>
+        <x:v>One side says the election was secure and another says it was stolen, so the honest answer is probably that it was a little stolen.</x:v>
       </x:c>
       <x:c r="L69" t="str">
-        <x:v>Note that not all compromises to a middle position are faulty as in price negotiations for a new car.</x:v>
+        <x:v>Disagreement does not imply that the truth is halfway between the parties. One side may simply be much more right than the other.</x:v>
       </x:c>
       <x:c r="M69" t="str">
-        <x:v>If your spouse wants to spend the weekend in Las Vegas, and you would like to stay home in Los Angeles, offering the compromise of spending the weekend in the desert between the 2 cities would probably be a bad idea.</x:v>
-      </x:c>
-      <x:c r="N69" t="str"/>
+        <x:v>Coverage of climate, public health, and election integrity can slide into 'both sides' framing that treats consensus and fringe denial as if splitting the difference were balanced or fair.</x:v>
+      </x:c>
+      <x:c r="N69" t="str">
+        <x:v>In personal and workplace disputes, people often assume each side must be equally at fault, even when the evidence is lopsided.</x:v>
+      </x:c>
       <x:c r="O69" t="str"/>
       <x:c r="P69" t="str"/>
       <x:c r="Q69" t="str"/>
       <x:c r="R69" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -4555,25 +4577,25 @@
         <x:v>nirvana fallacy</x:v>
       </x:c>
       <x:c r="J101" t="str">
-        <x:v>Occurs when an argument assumes that a perfect solution must exist and/or that a solution should be rejected because some part of the problem would still exist after it has been implemented.</x:v>
+        <x:v>Occurs when a useful solution is dismissed because it does not fully solve the problem or because some flaws would remain afterward.</x:v>
       </x:c>
       <x:c r="K101" t="str">
-        <x:v>But, Dad! Your $20 is not going to replace the car I crashed! Keep your money!</x:v>
+        <x:v>There is no point building more housing if rents will still be too high afterward.</x:v>
       </x:c>
       <x:c r="L101" t="str">
-        <x:v>"The perfect is the enemy of the good." ~Voltaire.</x:v>
+        <x:v>A partial improvement can still be worthwhile. The mistake is demanding perfection from one proposal when no realistic policy can eliminate the problem entirely.</x:v>
       </x:c>
       <x:c r="M101" t="str">
-        <x:v>Some in the US claim that tighter border controls are "not the solution" to the problem of illegal immigration, and ignore the fact that tighter borders might make a significant difference.</x:v>
+        <x:v>Climate and transit proposals are often rejected because they will not solve emissions or congestion completely, as if incomplete progress counted as no progress.</x:v>
       </x:c>
       <x:c r="N101" t="str">
-        <x:v>Some argue "You can't stop illicit drug use, so there is no sense in having laws against illicit drugs." Changing the referent from illicit drugs to murder highlights the fallacy.</x:v>
+        <x:v>Arguments about AI safety, gun policy, and public health often dismiss guardrails for failing to eliminate every bad case, rather than asking whether they would reduce harm.</x:v>
       </x:c>
       <x:c r="O101" t="str"/>
       <x:c r="P101" t="str"/>
       <x:c r="Q101" t="str"/>
       <x:c r="R101" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -5414,25 +5436,25 @@
       <x:c r="H121" t="str"/>
       <x:c r="I121" t="str"/>
       <x:c r="J121" t="str">
-        <x:v>Occurs when a proponent of a position attempts to introduce an exemption to a generally accepted rule or principle without justifying the exemption.</x:v>
+        <x:v>Occurs when someone asks for an exception to a rule or standard but does not provide a relevant reason for why the favored case should be exempt.</x:v>
       </x:c>
       <x:c r="K121" t="str">
-        <x:v>Prayer works, but it's just that you can't subject it's claims to the tools of science.</x:v>
+        <x:v>Data privacy matters for everyone else's app, but our app is different because our mission is important.</x:v>
       </x:c>
       <x:c r="L121" t="str">
-        <x:v>In the example, why would claims of material effects from spiritual causes be off-limits to scientific scrutiny when the effects of all other causes can be assessed by science?</x:v>
+        <x:v>Exceptions can be justified, but they need a principled reason. Mere attachment to the favored case is not enough.</x:v>
       </x:c>
       <x:c r="M121" t="str">
-        <x:v>Some communities have proposed that police officers and their families be exempt from citations for traffic offenses. But it would seem that the reasons given for establishing speed limits would hold also for the families of police officers.</x:v>
+        <x:v>Political actors often demand strict accountability, civility, or transparency for opponents while inventing excuses for why their own side should be judged differently.</x:v>
       </x:c>
       <x:c r="N121" t="str">
-        <x:v>Many religions hold that forgiveness should be granted without bloodshed or payment of any sort, yet exempt their own god by offering irrelevant excuses such as "God is holy" or "God's ways are not our ways."</x:v>
+        <x:v>Religious and ideological arguments often exempt cherished claims from the evidence standards applied to ordinary claims.</x:v>
       </x:c>
       <x:c r="O121" t="str"/>
       <x:c r="P121" t="str"/>
       <x:c r="Q121" t="str"/>
       <x:c r="R121" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -6151,23 +6173,25 @@
       </x:c>
       <x:c r="I138" t="str"/>
       <x:c r="J138" t="str">
-        <x:v>In which a decision is encouraged based on what might be pleasing to imagine, rather than based on evidence or reason.</x:v>
+        <x:v>Occurs when a belief or decision is driven mainly by what would be pleasing, hopeful, or comforting if true rather than by what the evidence supports.</x:v>
       </x:c>
       <x:c r="K138" t="str">
-        <x:v>If there were no life after death, then this life would be rather meaningless, and so I choose to believe we have an eternal soul.</x:v>
+        <x:v>This stock is too exciting to fail, so I am sure it will recover.</x:v>
       </x:c>
       <x:c r="L138" t="str">
-        <x:v>This fallacy is probably the most human of all fallacies. It is almost to suggest, that if you want or believe something strongly enough, that something must be or become true.</x:v>
+        <x:v>Hope can sustain action, but it does not convert possibility into evidence. The stronger the desire, the easier it is to mistake wanting for warrant.</x:v>
       </x:c>
       <x:c r="M138" t="str">
-        <x:v>If it were argued that the desire of the majority of citizens for universal health care coverage makes it imperative that we pass a universal health care coverage bill, this would be committing the wishful thinking fallacy. There may be no objective way for some countries to pay for the plan given their resources. The fact that something would make us happy does not mean we deserve or can realize that something.</x:v>
-      </x:c>
-      <x:c r="N138" t="str"/>
+        <x:v>Speculative markets, miracle-cure promises, and election-night narratives often run on the thought that a hoped-for outcome is somehow more likely because people badly want it.</x:v>
+      </x:c>
+      <x:c r="N138" t="str">
+        <x:v>Beliefs about the afterlife, destiny, or technological salvation are often defended by saying life would feel bleak without them, which speaks to desire rather than truth.</x:v>
+      </x:c>
       <x:c r="O138" t="str"/>
       <x:c r="P138" t="str"/>
       <x:c r="Q138" t="str"/>
       <x:c r="R138" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="139">

</xml_diff>

<commit_message>
Expand LogFall causal and rhetorical rewrites
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9c2fccc48bc4418f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R11b4ceae84534631"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rb52d371b11034e7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R489a20f6307842bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rb6b4f73b303e44e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R89dd8c3ff0604458"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1470,25 +1470,25 @@
         <x:v>argumentum ad nauseam</x:v>
       </x:c>
       <x:c r="J28" t="str">
-        <x:v>Assuming that, because no one cares to discuss your position with you any longer, that your position is correct.</x:v>
+        <x:v>Occurs when repetition is treated as if it adds evidence, wearing down doubt or making a claim seem true through familiarity.</x:v>
       </x:c>
       <x:c r="K28" t="str">
-        <x:v>I've been arguing with my wife for 20 years about my gambling habit. She finally stopped arguing with me, demonstrating that I've been right all these years.</x:v>
+        <x:v>People have been saying for months that the election was stolen, so there has to be something to it.</x:v>
       </x:c>
       <x:c r="L28" t="str">
-        <x:v>The unfortunate thing about this fallacy is that it often works. The mere repetition of a fallacious argument will often lead to its entrenchment in a society.</x:v>
+        <x:v>A claim does not become better supported because it is repeated by the same speaker, echoed by many speakers, or circulated for a long time. Repetition changes familiarity, not the underlying evidence.</x:v>
       </x:c>
       <x:c r="M28" t="str">
-        <x:v>The tobacco companies persistently spread disinformation for years, and, in so doing, successfully converted many young people to the smoking that eventually killed them.</x:v>
+        <x:v>The Springfield, Ohio pet-eating rumor in September 2024 moved from rumor to national talking point largely through repetition across social media, cable segments, and campaign rhetoric even though local officials said there was no credible evidence.</x:v>
       </x:c>
       <x:c r="N28" t="str">
-        <x:v>The dictators of many countries set up propaganda campaigns that simply repeat the largely mythical achievements of the "glorious leader".</x:v>
+        <x:v>Claims of widespread noncitizen voting often survive audit after audit because the same allegation is repeated so often that persistence itself gets mistaken for proof.</x:v>
       </x:c>
       <x:c r="O28" t="str"/>
       <x:c r="P28" t="str"/>
       <x:c r="Q28" t="str"/>
       <x:c r="R28" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1612,23 +1612,25 @@
         <x:v>appeal to belief, appeal to the majority, appeal to the people</x:v>
       </x:c>
       <x:c r="J31" t="str">
-        <x:v>Occurs when a conclusion is claimed to be true solely because many people believe it to be true.</x:v>
+        <x:v>Occurs when a claim is treated as true, reasonable, or justified mainly because many people believe it, share it, or act on it.</x:v>
       </x:c>
       <x:c r="K31" t="str">
-        <x:v>Nearly everyone believes there are moral rules we must live by, so for you to claim these moral rules do not exist is ridiculous!</x:v>
+        <x:v>Millions of people are using this detox protocol online, so it cannot be pseudoscience.</x:v>
       </x:c>
       <x:c r="L31" t="str">
-        <x:v>This fallacy is usually committed by those who start with the assumption that belief in something is evidence for the existence of that something. In other words, an epistemic commitment is indicative of ontological fact. they place much confidence in the reliability of the human mind to arrive at true beliefs. This assumption, however, must be tested. An easy test of this assumption would be to consider how many humans hold beliefs that are incomparable with the beliefs of most of the world. Given the many incompatible religious and political beliefs, it seems quite clear that our basic ability to formulate true beliefs is not very reliable, and therefore convention is not a very good measure of correctness. This unreliability becomes even more salient when we consider the many erroneous beliefs our own ancestors held but a few decades ago.</x:v>
+        <x:v>Popularity can reveal what people want, fear, or have been persuaded by, but it does not settle what is true. Crowds can be informed, confused, manipulated, or all three at once.</x:v>
       </x:c>
       <x:c r="M31" t="str">
-        <x:v>Nearly everyone speeds while driving, but invoking this fact will probably not convine the police officer standing at your window. Nor should it convice him. Laws are often made based on the fact that too many people believe and do the very same thing.</x:v>
-      </x:c>
-      <x:c r="N31" t="str"/>
+        <x:v>Advocates of raw milk and other 'natural' wellness products often point to growing enthusiasm, celebrity uptake, or huge followings as if social momentum itself established safety or effectiveness.</x:v>
+      </x:c>
+      <x:c r="N31" t="str">
+        <x:v>Viral political claims are often defended with phrases like 'everyone is talking about it' or 'it has millions of views,' which confuses reach with reliability.</x:v>
+      </x:c>
       <x:c r="O31" t="str"/>
       <x:c r="P31" t="str"/>
       <x:c r="Q31" t="str"/>
       <x:c r="R31" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -1737,24 +1739,25 @@
         <x:v>ipse-dixitism</x:v>
       </x:c>
       <x:c r="J34" t="str">
-        <x:v>Occurs when a controversial premise is introduced without substantiation.</x:v>
+        <x:v>Occurs when a contested claim is simply asserted, often confidently, without the evidence needed to justify it.</x:v>
       </x:c>
       <x:c r="K34" t="str">
-        <x:v>My father Is 3 meters tall. Your father is only 1 meter tall. Therefore my father is taller than your father.</x:v>
+        <x:v>The jobs report was obviously manipulated. Everyone knows that.</x:v>
       </x:c>
       <x:c r="L34" t="str">
-        <x:v>This fallacy is often accompanies by a phrase such as "Trust me." It might be considered a self-referential appeal to authority. A more rigorous and constrained discussion might allow you to ask "What is you evidence for that claim?" However, when bare assertions are constantly thrown out as red herrings, it may be best to abandon any hope of real dialog. "When I use a word" Humpty Dumpty said, "...it means just what I choose it to mean-neither more nor less."
-Lewis Carroll, Through the Looking Glass.</x:v>
+        <x:v>Confidence, volume, and repetition can make a bare assertion sound weighty, but they do not do the evidential work. When the core support is missing, the proper question is still: What is the evidence?</x:v>
       </x:c>
       <x:c r="M34" t="str">
-        <x:v>Many economic or political arguments begin with bare assertions such as "The economy can't grow without tax breaks, so we need to..."</x:v>
-      </x:c>
-      <x:c r="N34" t="str"/>
+        <x:v>The anonymous affidavit circulated after the September 2024 ABC debate was treated by many users as explosive proof of moderator collusion even though the central accusations were not substantiated.</x:v>
+      </x:c>
+      <x:c r="N34" t="str">
+        <x:v>Public arguments about crime, immigration, vaccines, and election administration often begin with unsupported declarations that function rhetorically as if they were already established facts.</x:v>
+      </x:c>
       <x:c r="O34" t="str"/>
       <x:c r="P34" t="str"/>
       <x:c r="Q34" t="str"/>
       <x:c r="R34" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -1946,19 +1949,25 @@
       <x:c r="H39" t="str"/>
       <x:c r="I39" t="str"/>
       <x:c r="J39" t="str">
-        <x:v>An argument which disregards lost opportunity costs (typically non-obvious, difficult to determine or otherwise hidden) associated with destroying property of others, or other ways of externalizing costs onto others.</x:v>
+        <x:v>Occurs when destruction or forced replacement is treated as an economic gain because the visible spending is counted while the unseen losses and forgone alternatives are ignored.</x:v>
       </x:c>
       <x:c r="K39" t="str">
-        <x:v>After downtown vandalism, a mayor praises the damage for 'creating jobs' for glaziers while ignoring the shops, wages, and purchases that would have existed if the windows had never been broken.</x:v>
-      </x:c>
-      <x:c r="L39" t="str"/>
-      <x:c r="M39" t="str"/>
-      <x:c r="N39" t="str"/>
+        <x:v>The storm wrecked half the boardwalk, but at least all the rebuilding will be great for the local economy.</x:v>
+      </x:c>
+      <x:c r="L39" t="str">
+        <x:v>Repair work creates visible activity, but it mainly restores value that was lost. The missing comparison is what households, firms, insurers, and governments could have done with those same resources if the damage had not occurred.</x:v>
+      </x:c>
+      <x:c r="M39" t="str">
+        <x:v>After Hurricanes Helene and Milton in October 2024, some commentary emphasized reconstruction jobs and spending while downplaying the destroyed homes, shuttered businesses, and other uses those resources would have supported.</x:v>
+      </x:c>
+      <x:c r="N39" t="str">
+        <x:v>Cyberattacks, vandalism, and infrastructure failures are sometimes framed as hidden economic stimulus because repairs employ people, even though the spending mainly compensates for an avoidable loss.</x:v>
+      </x:c>
       <x:c r="O39" t="str"/>
       <x:c r="P39" t="str"/>
       <x:c r="Q39" t="str"/>
       <x:c r="R39" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -3863,25 +3872,25 @@
       <x:c r="H84" t="str"/>
       <x:c r="I84" t="str"/>
       <x:c r="J84" t="str">
-        <x:v>Occurs when not enough information is provided to make a complete comparison.</x:v>
+        <x:v>Occurs when one option is called better, worse, cheaper, safer, or more effective without specifying the relevant comparison class or the other factors that matter.</x:v>
       </x:c>
       <x:c r="K84" t="str">
-        <x:v>This watch is more accurate than that watch, so it's better to buy this one.</x:v>
+        <x:v>This city has lower rent than New York, so it is a more affordable place to live.</x:v>
       </x:c>
       <x:c r="L84" t="str">
-        <x:v>When buying a new watch, many factor such as price, functionality and style need to be taken into consideration.</x:v>
+        <x:v>A comparison can be true in one narrow respect while misleading overall. The missing pieces might include quality, risk, wages, inflation, time horizon, tradeoffs, or alternative baselines.</x:v>
       </x:c>
       <x:c r="M84" t="str">
-        <x:v>If a national health care package is deemed the only response to demographic gaps in health care coverage without proper consideration of long-term financial and social consequences, this is an incomplete comparison.</x:v>
+        <x:v>Campaign arguments about the economy often isolate one metric such as gas prices, job totals, or stock indexes and treat that single comparison as if it captured the whole condition of household life.</x:v>
       </x:c>
       <x:c r="N84" t="str">
-        <x:v>If you claim that young people today are wealthier than their parents had at the same age, you would be committing an incomplete comparison fallacy. You'll have to take into account monetary inflation, plus the changing perceived value placed on items and services such as health care, transportation, and computers.</x:v>
+        <x:v>Technology marketing frequently calls a new tool 'more productive' without clarifying productive for whom, under what workflow, at what error rate, and at what human cost.</x:v>
       </x:c>
       <x:c r="O84" t="str"/>
       <x:c r="P84" t="str"/>
       <x:c r="Q84" t="str"/>
       <x:c r="R84" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -4117,19 +4126,25 @@
       <x:c r="H90" t="str"/>
       <x:c r="I90" t="str"/>
       <x:c r="J90" t="str">
-        <x:v>Related to the belief that labour-saving technologies increase unemployment by reducing demand for labour.</x:v>
+        <x:v>Occurs when labor-saving technology is treated as if it must reduce total employment or human usefulness simply because it automates some existing tasks.</x:v>
       </x:c>
       <x:c r="K90" t="str">
-        <x:v>A city blocks warehouse automation on the ground that any labor-saving technology must reduce total employment, without considering how demand and new roles can shift elsewhere.</x:v>
-      </x:c>
-      <x:c r="L90" t="str"/>
-      <x:c r="M90" t="str"/>
-      <x:c r="N90" t="str"/>
+        <x:v>If the company adopts AI support tools, there will be nothing left for people to do.</x:v>
+      </x:c>
+      <x:c r="L90" t="str">
+        <x:v>New technology can displace real jobs and create painful transitions. The fallacy is the stronger claim that automation as such can only destroy work, rather than reorganize it, lower costs, create new roles, or shift labor elsewhere.</x:v>
+      </x:c>
+      <x:c r="M90" t="str">
+        <x:v>Debates over generative AI in 2024 often jumped straight from 'this automates part of my job' to 'therefore it will inevitably make people broadly unemployable,' skipping the more complicated evidence about substitution, augmentation, and new roles.</x:v>
+      </x:c>
+      <x:c r="N90" t="str">
+        <x:v>The U.S. dockworker fight over port automation in October 2024 showed why the issue is serious, but it also illustrated the need to distinguish real bargaining and transition questions from the blanket claim that productivity-enhancing technology is always socially worse.</x:v>
+      </x:c>
       <x:c r="O90" t="str"/>
       <x:c r="P90" t="str"/>
       <x:c r="Q90" t="str"/>
       <x:c r="R90" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -4275,23 +4290,25 @@
       <x:c r="H94" t="str"/>
       <x:c r="I94" t="str"/>
       <x:c r="J94" t="str">
-        <x:v>The claim that if something is natural, pleasant, or popular, then it is good or right.</x:v>
+        <x:v>Occurs when something is treated as good, safe, or morally preferable mainly because it is called natural, traditional, or closer to nature.</x:v>
       </x:c>
       <x:c r="K94" t="str">
-        <x:v>I know I'm in love with a bank robber. But how could could it be wrong if it feels so right?</x:v>
-      </x:c>
-      <x:c r="L94" t="str"/>
+        <x:v>Raw milk must be healthier because it is the way milk comes from the cow.</x:v>
+      </x:c>
+      <x:c r="L94" t="str">
+        <x:v>Natural things can be wonderful, harmful, neutral, or context-dependent. Arsenic, viruses, and earthquakes are natural too. The relevant questions are evidence, outcomes, and tradeoffs, not whether something sounds untouched.</x:v>
+      </x:c>
       <x:c r="M94" t="str">
-        <x:v>It has been argued that, the poverty of the uneducated is deserved because they choose not to further their education. This ignores the arguably vicious circular causation between a low education level and the inability to earn enough money to get an education. Conversely, there is nothing inherent to the status of the affluent that makes them "worthy" or "deserving" of their fate.</x:v>
+        <x:v>The 2026 push to expand raw milk access often leaned on the idea that unprocessed equals healthier, despite repeated warnings from public-health officials that the safety risks are real and the claimed benefits remain unproven.</x:v>
       </x:c>
       <x:c r="N94" t="str">
-        <x:v>Some proponents of Social Darwinism suggested that, because evolution operates on the survival of the fittest, that we ought to extend this notion of survival of the fittest to social policies. There is no coherent reason why humans need to adopt nature's agenda as their own agenda.</x:v>
+        <x:v>Wellness marketing routinely sells herbs, supplements, detoxes, and hormone routines by invoking nature itself as if natural origin settled the medical question.</x:v>
       </x:c>
       <x:c r="O94" t="str"/>
       <x:c r="P94" t="str"/>
       <x:c r="Q94" t="str"/>
       <x:c r="R94" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4357,21 +4374,25 @@
       <x:c r="H96" t="str"/>
       <x:c r="I96" t="str"/>
       <x:c r="J96" t="str">
-        <x:v>Occurs when a solution to a problem is said to have no value because it is not perfect.</x:v>
+        <x:v>Occurs when a realistic option is rejected because it does not solve a problem perfectly or because an imagined ideal is used as the standard of comparison.</x:v>
       </x:c>
       <x:c r="K96" t="str">
-        <x:v>They shouldn't get married since they often have arguments.</x:v>
+        <x:v>If carbon labels will not eliminate greenwashing entirely, there is no point requiring them.</x:v>
       </x:c>
       <x:c r="L96" t="str">
-        <x:v>This is very similar to the "perfect solution fallacy." "The perfect is the enemy of the good." ~Voltaire.</x:v>
-      </x:c>
-      <x:c r="M96" t="str"/>
-      <x:c r="N96" t="str"/>
+        <x:v>Most policies, tools, and institutions are partial fixes. The right question is often whether an option improves matters relative to feasible alternatives, not whether it achieves a flawless end state.</x:v>
+      </x:c>
+      <x:c r="M96" t="str">
+        <x:v>Critics of content moderation, election safeguards, AI guardrails, and climate policy often reject incremental measures on the grounds that bad cases will still exist, as if imperfection erased all value.</x:v>
+      </x:c>
+      <x:c r="N96" t="str">
+        <x:v>Debates about public-health interventions frequently collapse into 'if it does not stop every case, it failed,' which compares reality to fantasy rather than to the available alternatives.</x:v>
+      </x:c>
       <x:c r="O96" t="str"/>
       <x:c r="P96" t="str"/>
       <x:c r="Q96" t="str"/>
       <x:c r="R96" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -5300,25 +5321,25 @@
       <x:c r="H118" t="str"/>
       <x:c r="I118" t="str"/>
       <x:c r="J118" t="str">
-        <x:v>Picking your target after you make your prediction or speculation to ensure that you are right.</x:v>
+        <x:v>Occurs when someone highlights the data cluster that supports a favored story only after looking at the results, then treats that hand-picked pattern as if it had been the tested target all along.</x:v>
       </x:c>
       <x:c r="K118" t="str">
-        <x:v>Last year, the governor promised to stimulate the economy during his term, and you will note that this year there has been an increase of 2,000 jobs in the service industry.</x:v>
+        <x:v>I examined dozens of neighborhoods, found the one where crime fell after my program launched, and declared the program a proven success.</x:v>
       </x:c>
       <x:c r="L118" t="str">
-        <x:v>The governor in the example may be ignoring other less-favorable data to paint a picture of success. This fallacy is similar to cherry-picking. It is subjectively and arbitrarily (though perhaps subconsciously) selecting data that will bolster your position while ignoring data inconsistent with your position. For this reason, scientists attempt to reduce subjectivity by starting with a hypothesis, then attempt to falsify that hypothesis by every imaginable means. This increases the objectivity basic to scientific success and respectability.</x:v>
+        <x:v>This is close to cherry picking, but the emphasis is on drawing the target around the bullet holes after the shots land. Post hoc pattern-hunting can make randomness, noise, or mixed data look like confirmation.</x:v>
       </x:c>
       <x:c r="M118" t="str">
-        <x:v>Consider someone who claims he can accurately and consistently predict the outcome of coin flips. After 5 flips he has only guessed 2 flips correctly (40%), and wants to continue the experiment. Finally after 20 flips, he has guessed 13 correctly, and wants to stop, making his accuracy appear to be 65%. However, because he was able to choose when to quit, the results are subjectively biased, and do not meet the standards of experimentation set by science.</x:v>
+        <x:v>Economic and election commentary often selects the time window, county, or subgroup that flatters the preferred narrative after the fact, then presents that slice as the decisive measure.</x:v>
       </x:c>
       <x:c r="N118" t="str">
-        <x:v>Cherry picking data on global warming has been one area of recent abuse. "If you look at the data and sort of cherry-pick a micro-trend within a bigger trend, that technique is particularly suspect," says John Grego, a professor of statistics at the University of South Carolina.</x:v>
+        <x:v>AI benchmarking and startup marketing sometimes advertise the few tasks where a model shines while leaving out the wider distribution of tasks where the results are weaker or unstable.</x:v>
       </x:c>
       <x:c r="O118" t="str"/>
       <x:c r="P118" t="str"/>
       <x:c r="Q118" t="str"/>
       <x:c r="R118" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
@@ -5346,25 +5367,25 @@
         <x:v>joint effect, causal oversimplification</x:v>
       </x:c>
       <x:c r="J119" t="str">
-        <x:v>Occurs when it is assumed that there is merely one cause of a phenomenon while other possibly contributing causes go undetected, are ignored or are illegitimately minimized.</x:v>
+        <x:v>Occurs when a complex outcome is explained as if one cause alone did the work, while other relevant causes are ignored or illegitimately minimized.</x:v>
       </x:c>
       <x:c r="K119" t="str">
-        <x:v>The drop in crime in our neighborhood is due to better policing.</x:v>
+        <x:v>Inflation happened because of one policy decision.</x:v>
       </x:c>
       <x:c r="L119" t="str">
-        <x:v>The actual cause of a local drop in crime may actually be a collection of causes such as the installation of surveillance cameras, a better local economy that has given would-be criminals jobs and money, improved forensics, new home entertainment hardware and software that keep would-be criminals preoccupied, better role models, and tougher laws that have locked up the most frequent offenders. This fallacy is a type of false dilemma.</x:v>
+        <x:v>Some causes are more important than others, and sometimes one factor really is dominant. The fallacy appears when a multi-causal phenomenon is flattened into a one-variable story without enough evidence.</x:v>
       </x:c>
       <x:c r="M119" t="str">
-        <x:v>Nearly every country that has become prosperous throughout history has had some of its citizens claiming that their greatness was entirely due to the superiority of their nationality or their particular god.</x:v>
+        <x:v>Arguments about inflation, crime, housing costs, and educational decline often blame one villain such as immigrants, regulation, presidents, or social media, even when the outcome reflects multiple interacting causes.</x:v>
       </x:c>
       <x:c r="N119" t="str">
-        <x:v>Whenever there is a school shooting, there emerge dozens of speculative opinions, each fingering a single cause such as poor parenting, violent video games, secular education, or the availability of guns. A responsible opinion would attempt cite evidence for the weight of each possible cause.</x:v>
+        <x:v>After school shootings or viral episodes of unrest, public commentary regularly rushes to one master explanation instead of asking how incentives, access, institutions, culture, and personal history combine.</x:v>
       </x:c>
       <x:c r="O119" t="str"/>
       <x:c r="P119" t="str"/>
       <x:c r="Q119" t="str"/>
       <x:c r="R119" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -5612,21 +5633,25 @@
       <x:c r="H125" t="str"/>
       <x:c r="I125" t="str"/>
       <x:c r="J125" t="str">
-        <x:v>Occurs when the style of the argument's presentation is emphasized, while marginalizing the actual content of the argument.</x:v>
+        <x:v>Occurs when the polish, confidence, charisma, or dramatic force of a presentation is treated as if it established the quality of the argument itself.</x:v>
       </x:c>
       <x:c r="K125" t="str">
-        <x:v>The audience's applause for my points during the debate this evening demonstrates the veracity of my arguments.</x:v>
+        <x:v>She demolished the debate because the crowd cheered and her one-liners landed.</x:v>
       </x:c>
       <x:c r="L125" t="str">
-        <x:v>This seems to be the prevailing fallacy in politics. However, a beautiful delivery does not necessarily mean there is no real content.</x:v>
-      </x:c>
-      <x:c r="M125" t="str"/>
-      <x:c r="N125" t="str"/>
+        <x:v>Strong delivery can make good arguments easier to hear, but it can also camouflage weak ones. Audiences often remember certainty, rhythm, and applause longer than the actual reasoning.</x:v>
+      </x:c>
+      <x:c r="M125" t="str">
+        <x:v>Coverage of the September 10, 2024 Harris-Trump debate often focused on who seemed stronger, calmer, or more in command, which matters politically but does not by itself settle whether the claims on stage were accurate.</x:v>
+      </x:c>
+      <x:c r="N125" t="str">
+        <x:v>Short-form video and podcast culture reward confidence, pace, and rhetorical dominance, making it easy for a slick performance to outperform a careful but less theatrical argument.</x:v>
+      </x:c>
       <x:c r="O125" t="str"/>
       <x:c r="P125" t="str"/>
       <x:c r="Q125" t="str"/>
       <x:c r="R125" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="126">

</xml_diff>

<commit_message>
Modernize social and rhetorical fallacies
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R489a20f6307842bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rb6b4f73b303e44e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R89dd8c3ff0604458"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Raef4d65edded4b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R698b59db294e4512"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R5e4a55ccdd36485c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -612,23 +612,25 @@
       <x:c r="H9" t="str"/>
       <x:c r="I9" t="str"/>
       <x:c r="J9" t="str">
-        <x:v>Occurs when it is implied that one must believe all or nothing of a particular set of beliefs.</x:v>
+        <x:v>Occurs when support for part of a view, or problems with part of a view, are treated as if they force total acceptance or total rejection of the whole package.</x:v>
       </x:c>
       <x:c r="K9" t="str">
-        <x:v>There are many historical documents that substantiate the notion that Saint Nicolas gave gifts to children. So to say he doesn't descend chimneys on Christmas Eve is against the historical facts.</x:v>
-      </x:c>
-      <x:c r="L9" t="str"/>
+        <x:v>One error in this report means the entire investigation is worthless.</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>Many systems of belief, institutions, and documents are mixed. Partial support or partial failure rarely justifies an everything-or-nothing verdict.</x:v>
+      </x:c>
       <x:c r="M9" t="str">
-        <x:v>Some theists cite evidence that some of the historical references in the bible are collaborated with extra-biblical sources, then imply that everything found within the bible, including the miracles, are also true.</x:v>
+        <x:v>In 2024 media battles, a single correction or mistaken detail was often used to dismiss an outlet's entire reporting on elections, immigration, or public health.</x:v>
       </x:c>
       <x:c r="N9" t="str">
-        <x:v>Some atheists confront theists with arguments against the notion of eternal torment, though many theists do not believe in an actual burning hell.</x:v>
+        <x:v>Religious, ideological, and policy debates often act as though rejecting one doctrine, statistic, or mechanism commits you to rejecting the entire worldview.</x:v>
       </x:c>
       <x:c r="O9" t="str"/>
       <x:c r="P9" t="str"/>
       <x:c r="Q9" t="str"/>
       <x:c r="R9" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -892,21 +894,25 @@
       </x:c>
       <x:c r="I15" t="str"/>
       <x:c r="J15" t="str">
-        <x:v>An appeal to emotion in which the use of flattery is used to attract support for the argument.</x:v>
+        <x:v>Occurs when someone tries to win agreement by flattering the audience's intelligence, courage, independence, or special insight instead of supplying the missing evidence.</x:v>
       </x:c>
       <x:c r="K15" t="str">
-        <x:v>Your intelligence prevents you from rejecting the truth of my claim.</x:v>
+        <x:v>You are too perceptive to fall for the official story, so you can already see why my theory must be right.</x:v>
       </x:c>
       <x:c r="L15" t="str">
-        <x:v>There is a fine line between flattery and honest kindness. Ignoring truth a bit to accommodate kindness is perhaps the most forgivable fallacy.</x:v>
-      </x:c>
-      <x:c r="M15" t="str"/>
-      <x:c r="N15" t="str"/>
+        <x:v>Compliments can be sincere and harmless. The fallacy appears when praise does the persuasive work by making agreement feel like a badge of intelligence or independence.</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>Wellness, crypto, and conspiracy marketing often tells followers they are 'awake,' 'elite,' or 'smart enough to see through the lie,' turning assent into a test of self-image.</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>Political fundraising and influencer media frequently flatter supporters as the few people brave or intelligent enough to 'see what is really happening' before asking them to accept weakly supported claims.</x:v>
+      </x:c>
       <x:c r="O15" t="str"/>
       <x:c r="P15" t="str"/>
       <x:c r="Q15" t="str"/>
       <x:c r="R15" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1118,23 +1124,25 @@
         <x:v>argumentum ad lazarum</x:v>
       </x:c>
       <x:c r="J20" t="str">
-        <x:v>Suggesting the truth of a conclusion necessarily negatively correlates to it's proponent's financial situation.</x:v>
+        <x:v>Occurs when a claim is treated as more trustworthy, virtuous, or true mainly because its proponent is poor, ordinary, or from humble circumstances.</x:v>
       </x:c>
       <x:c r="K20" t="str">
-        <x:v>He can be trusted due to his humble upbringing in a one-room cabin deep in the mountains.</x:v>
+        <x:v>He grew up with nothing, so his economic diagnosis must be more reliable than the experts'.</x:v>
       </x:c>
       <x:c r="L20" t="str">
-        <x:v>The converse of this fallacy is the appeal to wealth fallacy.</x:v>
+        <x:v>Background can illuminate perspective, but hardship is not a truth detector. A difficult life story may earn sympathy or respect without settling the claim being made.</x:v>
       </x:c>
       <x:c r="M20" t="str">
-        <x:v>The humble beginnings of many political candidates are often emphasized in an attempt to get the common citizen to identify with the candidate.</x:v>
-      </x:c>
-      <x:c r="N20" t="str"/>
+        <x:v>Campaign biographies in 2024 often leaned heavily on working-class roots and hardship stories, which may matter politically but do not by themselves verify a candidate's policy claims.</x:v>
+      </x:c>
+      <x:c r="N20" t="str">
+        <x:v>Populist media often imply that 'ordinary people' are automatically more honest than credentialed critics, as if social position alone settled the argument.</x:v>
+      </x:c>
       <x:c r="O20" t="str"/>
       <x:c r="P20" t="str"/>
       <x:c r="Q20" t="str"/>
       <x:c r="R20" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1342,23 +1350,25 @@
         <x:v>argumentum ad crumenam</x:v>
       </x:c>
       <x:c r="J25" t="str">
-        <x:v>Suggesting the truth of a conclusion necessarily positively correlates to it's proponent's financial situation.</x:v>
+        <x:v>Occurs when a claim is treated as more credible or correct mainly because it comes from a rich, famous, or financially successful person.</x:v>
       </x:c>
       <x:c r="K25" t="str">
-        <x:v>If your ideas had any real merit, you'd be rich by now.</x:v>
+        <x:v>He built a billion-dollar company, so his views on health policy must be right.</x:v>
       </x:c>
       <x:c r="L25" t="str">
-        <x:v>The converse of this fallacy is the appeal to poverty fallacy.</x:v>
+        <x:v>Success can indicate skill in a particular domain, but money is not a universal credential. Wealth may buy attention, not truth.</x:v>
       </x:c>
       <x:c r="M25" t="str">
-        <x:v>The financial success of an individual is often cited as evidence for their competency to take the helm of additional ventures, some of which may require skills other than what a successful business person can offer.</x:v>
-      </x:c>
-      <x:c r="N25" t="str"/>
+        <x:v>In 2024 and 2025, fans and investors often treated billionaire founders' views on AI, politics, or medicine as self-validating because of their wealth rather than because the evidence was strong.</x:v>
+      </x:c>
+      <x:c r="N25" t="str">
+        <x:v>The unverified ABC debate affidavit gained extra credibility online after high-profile wealthy amplifiers helped circulate it, as though status itself made the claim more trustworthy.</x:v>
+      </x:c>
       <x:c r="O25" t="str"/>
       <x:c r="P25" t="str"/>
       <x:c r="Q25" t="str"/>
       <x:c r="R25" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1516,25 +1526,25 @@
         <x:v>argumentum ex silentio</x:v>
       </x:c>
       <x:c r="J29" t="str">
-        <x:v>A conclusion deemed true based on the lack of opposition.</x:v>
+        <x:v>Occurs when a claim is treated as validated because opponents, authorities, or witnesses did not deny it, respond to it, or mention it.</x:v>
       </x:c>
       <x:c r="K29" t="str">
-        <x:v>Because my opponent failed to address my point, my point is validated.</x:v>
+        <x:v>The agency never answered my thread, so my accusation must be true.</x:v>
       </x:c>
       <x:c r="L29" t="str">
-        <x:v>If a point is not addressed, rarely does it become anything other than an unaddressed point. However, this is context-dependent. If you see a vampire sitting across from you on the subway, and none of the other passengers seem interested, you might first consider what medication you might have taken that morning before wielding your wooden stake since the silence of the other passengers in such a setting would be unusual. The key question to ask is "How unusual is this silence?"</x:v>
+        <x:v>Silence can matter when a response would clearly be expected and feasible. Outside that setting, it often tells us little.</x:v>
       </x:c>
       <x:c r="M29" t="str">
-        <x:v>The disinterest and subsequent silence of doctors on the claims of dubious medial remedies is often spun to imply their tacit support, or at minimum, their lack of opposition.</x:v>
+        <x:v>The absence of public confirmation for many election-fraud and migrant-voting rumors was often spun as suspicious silence rather than as a sign that the underlying evidence was weak or nonexistent.</x:v>
       </x:c>
       <x:c r="N29" t="str">
-        <x:v>The phrase "no comment", which can be uttered for a wide variety of reasons, is often spun by the media to evoke suspicion of a secret or mystery.</x:v>
+        <x:v>A 'no comment' from campaigns, police, or institutions is regularly treated as if it were a tacit admission, even though legal, strategic, or practical reasons may explain the silence.</x:v>
       </x:c>
       <x:c r="O29" t="str"/>
       <x:c r="P29" t="str"/>
       <x:c r="Q29" t="str"/>
       <x:c r="R29" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1564,25 +1574,25 @@
         <x:v>appeal to the stick, appeal to force</x:v>
       </x:c>
       <x:c r="J30" t="str">
-        <x:v>Occurs when an argument is made through coercion or threats of force towards an opposing party.</x:v>
+        <x:v>Occurs when agreement is extracted by threat, intimidation, or coercive pressure rather than by showing that the claim is true.</x:v>
       </x:c>
       <x:c r="K30" t="str">
-        <x:v>You've been a good employee up to this point, John. And I think you'll agree that shining my shoes is not at all as humiliating as losing your job.</x:v>
+        <x:v>Support this initiative, or do not expect your contract to be renewed.</x:v>
       </x:c>
       <x:c r="L30" t="str">
-        <x:v>This fallacy works superficially. You may gain the cooperation of many through the Machiavellian use of force, but historically, those who lived by the sword often died by the sword. And the sword never changed the truth of the matter.</x:v>
+        <x:v>Threats can force compliance, but they do not transform a bad argument into a good one. Fear may explain why someone goes along; it does not show that the view is correct.</x:v>
       </x:c>
       <x:c r="M30" t="str">
-        <x:v>There are millions of people who believe that, if you do not also believe in their particular version of god, that you will be eternally tortured.</x:v>
+        <x:v>In countries where blasphemy, apostasy, or political dissent can trigger severe punishment, outward conformity is often mistaken for genuine persuasion when it may simply reflect fear.</x:v>
       </x:c>
       <x:c r="N30" t="str">
-        <x:v>In some countries, apostasy from a particular religion is deemed worthy of death. To what degree does belief subconsciously conform to threats such as these?</x:v>
+        <x:v>Online campaigns that threaten doxxing, blacklisting, or mass harassment often aim to secure silence or agreement by making disagreement personally costly.</x:v>
       </x:c>
       <x:c r="O30" t="str"/>
       <x:c r="P30" t="str"/>
       <x:c r="Q30" t="str"/>
       <x:c r="R30" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2041,23 +2051,25 @@
       <x:c r="H41" t="str"/>
       <x:c r="I41" t="str"/>
       <x:c r="J41" t="str">
-        <x:v>Occurs when a conclusion is deemed incorrect because it was commonly held when something else that was clearly false was also commonly held.</x:v>
+        <x:v>Occurs when an idea is dismissed mainly because it is old, premodern, or associated with a period that also held many false beliefs.</x:v>
       </x:c>
       <x:c r="K41" t="str">
-        <x:v>Why must we accept medieval art as having any value when it emerged from the same period in which people burned witches and believed in fairies?</x:v>
+        <x:v>That argument comes from ancient philosophy, so modern people can ignore it.</x:v>
       </x:c>
       <x:c r="L41" t="str">
-        <x:v>This is a type of faulty generalization since the error is over-generalizing from a period of several wrong concepts to concluding that all concepts within that period were wrong. A more detailed treatment of faulty generalizations can be found on the supplementary Inductive Errors page.</x:v>
+        <x:v>Older views can be wrong, but age alone neither refutes nor confirms them. The real question is whether the reasoning survives scrutiny.</x:v>
       </x:c>
       <x:c r="M41" t="str">
-        <x:v>Many early doctors held superstitions that would make us wary of visiting their office were they alive and holding the same beliefs today. This does not mean their practice of medicine was worthless for those alive in their day..</x:v>
-      </x:c>
-      <x:c r="N41" t="str"/>
+        <x:v>Social-media arguments often dismiss older religious, philosophical, or literary texts as worthless simply because they come from a less enlightened era, skipping the actual argument.</x:v>
+      </x:c>
+      <x:c r="N41" t="str">
+        <x:v>People also dismiss pre-digital scholarship wholesale as outdated while still relying on concepts, institutions, and moral categories that earlier thinkers helped shape.</x:v>
+      </x:c>
       <x:c r="O41" t="str"/>
       <x:c r="P41" t="str"/>
       <x:c r="Q41" t="str"/>
       <x:c r="R41" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2171,24 +2183,25 @@
       <x:c r="H44" t="str"/>
       <x:c r="I44" t="str"/>
       <x:c r="J44" t="str">
-        <x:v>Occurs when the certainty one feels in respect to a claim is submitted as evidence for the veracity of that claim.</x:v>
+        <x:v>Occurs when a speaker's certainty, intensity, or felt conviction is treated as if it were evidence that the claim is true.</x:v>
       </x:c>
       <x:c r="K44" t="str">
-        <x:v>I've never swayed from my confidence that Santa is real, and there is no degree of evidence that can counter the way I feel.</x:v>
+        <x:v>I know it in my gut with total certainty, and that certainty is all the proof I need.</x:v>
       </x:c>
       <x:c r="L44" t="str">
-        <x:v>This fallacy results from esteeming certainty as an objective validation of a proposition rather than as an emotion that could be misguided. Sometimes it is an emotional certainty that prevents the emotional pain that might result from following the evidence into disbelief, and other times it is triggered by a legitimate intuition that results in an emotional snowball of certainty that does not assess the possible evidential clues hidden in the intuition for validity.</x:v>
+        <x:v>Confidence can track expertise, but it can also track charisma, identity, adrenaline, fear, or repeated exposure to a claim. Certainty is a psychological state, not a built-in proof.</x:v>
       </x:c>
       <x:c r="M44" t="str">
-        <x:v>Theists often conflate the emotional confidence derived from other emotions such as peace and love with evidence for the existence of their god. This essentially makes belief circular; "I know what I know".
-[Example].</x:v>
-      </x:c>
-      <x:c r="N44" t="str"/>
+        <x:v>The anonymous ABC debate affidavit spread partly because influential accounts amplified it with extraordinary certainty before any reliable verification had appeared.</x:v>
+      </x:c>
+      <x:c r="N44" t="str">
+        <x:v>In arguments about AI consciousness, election fraud, religion, and wellness, people often present their felt certainty as if it were itself a kind of evidence rather than something that also needs checking.</x:v>
+      </x:c>
       <x:c r="O44" t="str"/>
       <x:c r="P44" t="str"/>
       <x:c r="Q44" t="str"/>
       <x:c r="R44" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2256,32 +2269,25 @@
         <x:v>quoting out of context</x:v>
       </x:c>
       <x:c r="J46" t="str">
-        <x:v>The selective excerpting of words from their original linguistic context in a way that distorts the intended meaning.</x:v>
+        <x:v>Occurs when words are selectively excerpted from their original context in a way that changes or distorts what the speaker meant.</x:v>
       </x:c>
       <x:c r="K46" t="str">
-        <x:v>My wife told me she needed me to take out the garbage. When she was moving out a week later, I told her she was a liar for having said she "needed me".</x:v>
+        <x:v>The scientist said the result was 'uncertain,' so he admitted the theory was collapsing.</x:v>
       </x:c>
       <x:c r="L46" t="str">
-        <x:v>Those with faith in some form of holy scriptures often accuse each other of contextomy. This is probably more a function of the vagueness of the context which allows for multiple interpretations.</x:v>
+        <x:v>Shortening a quote is not automatically deceptive. The fallacy appears when the omitted context would materially change how a fair reader understands the statement.</x:v>
       </x:c>
       <x:c r="M46" t="str">
-        <x:v>The commander of British forces in Afghanistan, Mark Carleton-Smith said the following."We're not going to win this war. It's about reducing it to a manageable level of insurgency that's not a strategic threat and can be managed by the Afghan army."
-Only the first line was quoted by some media outlets, distorting the true intention of the commander.</x:v>
+        <x:v>Edited debate clips, viral subtitled videos, and quote-card politics in 2024 regularly removed the surrounding setup, qualifier, or punchline that made the original meaning very different.</x:v>
       </x:c>
       <x:c r="N46" t="str">
-        <x:v>The following is a quote by Charles Darwin."Why then is not every geological formation and every stratum full of such intermediate links? Geology assuredly does not reveal any such finely-graduated organic chain; and this, perhaps, is the most obvious and serious objection which can be urged against the theory. "
-Taken out of context, this quote is easily perceived to be Darwin doubting his own theory. However, Darwin continued..."The explanation lies, as I believe, in the extreme imperfection of the geological record. In the first place, it should always be borne in mind what sort of intermediate forms must, on the theory, have formerly existed... ".</x:v>
-      </x:c>
-      <x:c r="O46" t="str">
-        <x:v>Consider this bible verse. Hosea 11:1 "When Israel was a child, I loved him, and out of Egypt I called my son."
-Now note how Matthew later unequivocally denotes this verse in Hosea as a messianic prophecy. He is refering to Jesus' time in Egypt when he writes... Matthew 2:15 "And was there until the death of Herod: that it might be fulfilled which was spoken of the Lord by the prophet, saying, Out of Egypt have I called my son.'"
-But now let's return to the very next verse in Hosea. Hosea 11:2 "But the more I called Israel, the further they went from me. They sacrificed to the Baals and they burned incense to images."
-Unless you want to say Jesus sacrificed to the Baals, you've got to say Matthew took this verse out of context.</x:v>
-      </x:c>
+        <x:v>Public figures and partisans often quote one alarming sentence from a report, study, or speech while cutting the lines that immediately limit, explain, or even reverse the apparent claim.</x:v>
+      </x:c>
+      <x:c r="O46" t="str"/>
       <x:c r="P46" t="str"/>
       <x:c r="Q46" t="str"/>
       <x:c r="R46" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -4206,19 +4212,25 @@
       <x:c r="H92" t="str"/>
       <x:c r="I92" t="str"/>
       <x:c r="J92" t="str">
-        <x:v>Involves describing an occurrence, often exceptional, in vivid detail, to distort the actual severity of the problem.</x:v>
+        <x:v>Occurs when a striking anecdote or emotionally intense case is used to make a problem seem more common, clear, or representative than the broader evidence allows.</x:v>
       </x:c>
       <x:c r="K92" t="str">
-        <x:v>You should never date a Texas girl. My friend dated one, and she slashed the tires on his car and killed his dog.</x:v>
-      </x:c>
-      <x:c r="L92" t="str"/>
-      <x:c r="M92" t="str"/>
-      <x:c r="N92" t="str"/>
+        <x:v>One terrifying subway assault proves the whole city is descending into chaos.</x:v>
+      </x:c>
+      <x:c r="L92" t="str">
+        <x:v>Vivid cases matter, especially when they reveal harms abstract statistics can hide. The fallacy arises when memorable exceptions are used as if they were the normal pattern.</x:v>
+      </x:c>
+      <x:c r="M92" t="str">
+        <x:v>The Springfield rumor gained traction partly because lurid, memorable imagery traveled faster than the dull but crucial fact that authorities found no supporting evidence.</x:v>
+      </x:c>
+      <x:c r="N92" t="str">
+        <x:v>Viral clips of shoplifting, airplane incidents, or isolated crimes are often used to imply a general trend without the comparative data needed to show that the example is typical.</x:v>
+      </x:c>
       <x:c r="O92" t="str"/>
       <x:c r="P92" t="str"/>
       <x:c r="Q92" t="str"/>
       <x:c r="R92" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -5806,29 +5818,25 @@
       <x:c r="H129" t="str"/>
       <x:c r="I129" t="str"/>
       <x:c r="J129" t="str">
-        <x:v>Occurs when a commonly heard and accepted phrase is rhetorically introduced as a substitute for an actual argument.</x:v>
+        <x:v>Occurs when a familiar slogan or stock phrase is used to stop inquiry, deflect scrutiny, or create the feeling that an issue has already been settled.</x:v>
       </x:c>
       <x:c r="K129" t="str">
-        <x:v>The more things change, the more they stay the same. Humans will never overcome their violent nature in spite of recent claims of progress.</x:v>
+        <x:v>It is what it is, so there is nothing more to discuss.</x:v>
       </x:c>
       <x:c r="L129" t="str">
-        <x:v>Some aphorisms fall into the category of faulty generalizations. It is usually difficult to find a pithy phrase that captures the nuances of the concept.</x:v>
+        <x:v>Aphorisms can be wise shortcuts, but they become fallacious when they replace the reasoning that the situation still requires.</x:v>
       </x:c>
       <x:c r="M129" t="str">
-        <x:v>The phrase "Only God knows" is often interjected at the end of a discussion to imply that no one is justified in taking a position on the issue, or to assume the evidence is balanced on both sides.</x:v>
+        <x:v>Phrases such as 'Do your own research,' 'common sense,' or 'if you know, you know' are often used online not to open inquiry but to make further questions look unnecessary or naive.</x:v>
       </x:c>
       <x:c r="N129" t="str">
-        <x:v>Sometime the phrase "Freedom is not free" is used to infer a clear justification for entering a war.</x:v>
-      </x:c>
-      <x:c r="O129" t="str">
-        <x:v>Christians often quote the verse "The fool has said in his heart, 'there is no God'" sometimes as if this is a justification for belief in God, and sometimes simply as a thought-terminator.</x:v>
-      </x:c>
-      <x:c r="P129" t="str">
-        <x:v>When having their expectations questioned, older people often, due to either having no real answer or having no interest in giving an answer, say "When you're my age, you'll understand."</x:v>
-      </x:c>
+        <x:v>Political and religious arguments frequently end with slogans like 'Freedom is not free' or 'Only God knows,' which can be meaningful in some contexts but often function as conversation-stoppers.</x:v>
+      </x:c>
+      <x:c r="O129" t="str"/>
+      <x:c r="P129" t="str"/>
       <x:c r="Q129" t="str"/>
       <x:c r="R129" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -6074,19 +6082,25 @@
       <x:c r="H135" t="str"/>
       <x:c r="I135" t="str"/>
       <x:c r="J135" t="str">
-        <x:v>Occurs when it is assumed that, if one wrong has been committed, another wrong will remove its culpability.</x:v>
+        <x:v>Occurs when someone treats one wrong act as justified because it responds to, retaliates against, or balances out another wrong.</x:v>
       </x:c>
       <x:c r="K135" t="str">
-        <x:v>My opponent maliciously attacked my character, and I am therefore justified in pointing out a few of his improprieties.</x:v>
-      </x:c>
-      <x:c r="L135" t="str"/>
-      <x:c r="M135" t="str"/>
-      <x:c r="N135" t="str"/>
+        <x:v>Their side spread fake clips about us, so we are justified in spreading a few about them.</x:v>
+      </x:c>
+      <x:c r="L135" t="str">
+        <x:v>Exposing hypocrisy can matter, but retaliation does not erase the original wrong or magically sanitize a copy of it.</x:v>
+      </x:c>
+      <x:c r="M135" t="str">
+        <x:v>In 2024 election discourse, misinformation was often excused with the claim that the other side lies too, as if symmetry or revenge transformed falsehood into fairness.</x:v>
+      </x:c>
+      <x:c r="N135" t="str">
+        <x:v>Debates about censorship, doxxing, and dirty campaign tactics often slide from condemnation into imitation, with each side treating the other's bad behavior as a license to do the same.</x:v>
+      </x:c>
       <x:c r="O135" t="str"/>
       <x:c r="P135" t="str"/>
       <x:c r="Q135" t="str"/>
       <x:c r="R135" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="136">

</xml_diff>

<commit_message>
Add favicon and expand LogFall rewrites
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Raef4d65edded4b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R698b59db294e4512"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R5e4a55ccdd36485c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R17e1dd59dc08462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Racd1cbb768704858"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Ra05835a798084c54"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -660,25 +660,25 @@
       </x:c>
       <x:c r="I10" t="str"/>
       <x:c r="J10" t="str">
-        <x:v>Occurs when an claim is deemed true based on the accomplishments of its sponsor.</x:v>
+        <x:v>Occurs when a claim is treated as true or weighty mainly because the person promoting it has impressive accomplishments in some other domain.</x:v>
       </x:c>
       <x:c r="K10" t="str">
-        <x:v>Isaac Newton had such an impact on science, so there must have been some value in his later work in alchemy.</x:v>
+        <x:v>She built a famous tech company, so her views on nutrition and aging must be scientifically trustworthy.</x:v>
       </x:c>
       <x:c r="L10" t="str">
-        <x:v>Arguments are independent of the source. Intelligent people can have poor arguments, and unintelligent can produce strong arguments. Though it is human nature to over-emphasize the virtues or vices of the voice behind the argument, neither shoot nor celebrate the messenger. Worthy arguments stand on their own.</x:v>
+        <x:v>Real accomplishment can justify attention, but it does not automatically transfer expertise across domains. The relevant question is still whether the claim is supported.</x:v>
       </x:c>
       <x:c r="M10" t="str">
-        <x:v>The use of celebrities to sell products is based on this fallacy. The public grants a spokesperson with highly-visible accomplishments high credibility, even when endorsing products and ideas unrelated to their accomplishments.</x:v>
+        <x:v>Celebrity founders, athletes, and actors often lend credibility to products and causes far outside their expertise, from supplements to financial schemes to political narratives.</x:v>
       </x:c>
       <x:c r="N10" t="str">
-        <x:v>Sir Arthur Conan Doyle, the brilliant creator of the very logical Sherlock Holmes series promoted belief in fairies.</x:v>
+        <x:v>Public arguments about AI frequently treat the prestige of well-known founders as if it settled disputes that still require technical evidence, replication, and broader expert scrutiny.</x:v>
       </x:c>
       <x:c r="O10" t="str"/>
       <x:c r="P10" t="str"/>
       <x:c r="Q10" t="str"/>
       <x:c r="R10" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1708,24 +1708,25 @@
         <x:v>guilt by association</x:v>
       </x:c>
       <x:c r="J33" t="str">
-        <x:v>Occurs when a claim is deemed true or untrue based on an association with some irrelevant element.</x:v>
+        <x:v>Occurs when a claim is accepted or dismissed because of some irrelevant association rather than because of the merits of the claim itself.</x:v>
       </x:c>
       <x:c r="K33" t="str">
-        <x:v>Jane is an exceptional pianist, and also pretty. Therefore, all pianists are pretty.</x:v>
+        <x:v>That housing proposal is backed by Silicon Valley donors, so it must be corrupt.</x:v>
       </x:c>
       <x:c r="L33" t="str">
-        <x:v>There may, however, be a relevant association between two qualities. If, for example, you note that pianists have long fingers, there may be a causal relationship between long fingers and pianists, though this needs to be substantiated with evidence and argumentation.
-This is a type of proof by example fallacy. A more detailed treatment of proof by example fallacies can be found on the supplementary Inductive Errors page.</x:v>
+        <x:v>Associations can sometimes matter when they reveal bias, incentives, or causal links. The fallacy appears when the link is treated as decisive even though it does not address the argument.</x:v>
       </x:c>
       <x:c r="M33" t="str">
-        <x:v>If you argue that, because Japanese are polite, they would never push each other, you have not seen a rush hour subway train in Tokyo. Pushing does not necessarily entail impoliteness..</x:v>
-      </x:c>
-      <x:c r="N33" t="str"/>
+        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported.</x:v>
+      </x:c>
+      <x:c r="N33" t="str">
+        <x:v>Political arguments routinely assume that if a bad person, rival group, or disliked movement touched an idea, the idea itself must be false or tainted.</x:v>
+      </x:c>
       <x:c r="O33" t="str"/>
       <x:c r="P33" t="str"/>
       <x:c r="Q33" t="str"/>
       <x:c r="R33" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -2777,21 +2778,25 @@
       <x:c r="H58" t="str"/>
       <x:c r="I58" t="str"/>
       <x:c r="J58" t="str">
-        <x:v>Occurs when an argument is said to be wrong, yet no information or explanation about what in the argument was wrong.</x:v>
+        <x:v>Occurs when someone declares an argument false, debunked, or dishonest without identifying the specific flaw that would actually show it is false.</x:v>
       </x:c>
       <x:c r="K58" t="str">
-        <x:v>You misrepresented my position in your argument, so your argument is clearly wrong.</x:v>
+        <x:v>That has been thoroughly debunked, obviously, so I do not need to explain anything further.</x:v>
       </x:c>
       <x:c r="L58" t="str">
-        <x:v>If you claim someone has misrepresented your argument, you'll need to rigorously substantiate that. If you identify a flaw in someone's argument, take the time to detail that flaw rather than simply telling them they are wrong.</x:v>
-      </x:c>
-      <x:c r="M58" t="str"/>
-      <x:c r="N58" t="str"/>
+        <x:v>Not every conversation requires a full essay, but a real refutation still has to point to some error in reasoning, evidence, or interpretation. Mere dismissal is not argument.</x:v>
+      </x:c>
+      <x:c r="M58" t="str">
+        <x:v>Online fights about elections, Israel and Gaza, climate, and AI often rely on 'debunked' as a performance word rather than as a pointer to the actual evidence.</x:v>
+      </x:c>
+      <x:c r="N58" t="str">
+        <x:v>In fast-moving social media disputes, people often treat tone, certainty, and pile-on consensus as if they were enough to count as refutation.</x:v>
+      </x:c>
       <x:c r="O58" t="str"/>
       <x:c r="P58" t="str"/>
       <x:c r="Q58" t="str"/>
       <x:c r="R58" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -3061,27 +3066,25 @@
         <x:v>complex question, fallacy of presupposition, loaded question, plurium interrogationum</x:v>
       </x:c>
       <x:c r="J65" t="str">
-        <x:v>Occurs when someone asks a question that presupposes something that has not been proven or accepted by all the people involved.</x:v>
+        <x:v>Occurs when a question smuggles in one or more assumptions that have not been established, then pressures the listener to answer as if those assumptions were already settled.</x:v>
       </x:c>
       <x:c r="K65" t="str">
-        <x:v>So Henry, have you stopped beating your wife?</x:v>
+        <x:v>When did your newsroom decide to coordinate its coverage with the campaign?</x:v>
       </x:c>
       <x:c r="L65" t="str">
-        <x:v>This fallacy combines several assumptions into a interrogative statement that erroneously demands a single binary answer.</x:v>
+        <x:v>A loaded question can force a false choice because any direct answer seems to concede what the question improperly assumed. The first task is often to challenge the hidden premise, not to answer on its terms.</x:v>
       </x:c>
       <x:c r="M65" t="str">
-        <x:v>Atheists are often asked a question similar to "So, if you don't believe in the afterlife, why don't you commit suicide since you have nothing to live for?" Not believing in the afterlife does not mean this life is not worth living.</x:v>
+        <x:v>Debates about religion, politics, and gender often turn on questions that quietly presuppose bad faith, delusion, or malicious intent before any of that has been shown.</x:v>
       </x:c>
       <x:c r="N65" t="str">
-        <x:v>Theists are sometimes asked by atheists "Would you be as delusional if you did not believe in God?" The word "delusional" inplies a mental illness that does not necessarily follow from belief in a god.</x:v>
-      </x:c>
-      <x:c r="O65" t="str">
-        <x:v>Theists sometimes ask atheists the more rhetorical question "You hate God since you want to continue in your sin, right?" This wrongly assumes it is possible to hate something you don't believe in, that you believe in the concept of sin, that you believe you are sinning, and that you hate god due to your choice of a sinful life.</x:v>
-      </x:c>
+        <x:v>Interviewers and posters sometimes frame questions so that merely engaging already concedes the accusation, especially in culture-war exchanges built for clipping and outrage.</x:v>
+      </x:c>
+      <x:c r="O65" t="str"/>
       <x:c r="P65" t="str"/>
       <x:c r="Q65" t="str"/>
       <x:c r="R65" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -3191,19 +3194,25 @@
       <x:c r="H68" t="str"/>
       <x:c r="I68" t="str"/>
       <x:c r="J68" t="str">
-        <x:v>Occurs when an advocate appeals to an irrelevant, unqualified, unidentified, biased or fabricated source in support of an argument.</x:v>
+        <x:v>Occurs when support for a claim is borrowed from a source that is fabricated, misquoted, unqualified, anonymous in the wrong way, or otherwise not what it is presented to be.</x:v>
       </x:c>
       <x:c r="K68" t="str">
-        <x:v>A viral post claims a Nobel Prize winner proved a miracle cure works, but the quote is misattributed and the researcher never made the claim.</x:v>
-      </x:c>
-      <x:c r="L68" t="str"/>
-      <x:c r="M68" t="str"/>
-      <x:c r="N68" t="str"/>
+        <x:v>A viral image says a Nobel Prize winner proved the treatment works, but the quote is fake and the expert never said it.</x:v>
+      </x:c>
+      <x:c r="L68" t="str">
+        <x:v>Source quality matters, but only if the source is real, relevant, and represented fairly. A false attribution can make weak claims feel borrowed from a stronger authority than they actually have.</x:v>
+      </x:c>
+      <x:c r="M68" t="str">
+        <x:v>The anonymous affidavit circulated after the September 2024 ABC debate was amplified as if it were a verified insider source even though the core allegations were not authenticated.</x:v>
+      </x:c>
+      <x:c r="N68" t="str">
+        <x:v>Viral quote cards and screenshot posts often attach dramatic claims to scientists, judges, or agencies who never said them, counting on readers to trust the label instead of checking the source.</x:v>
+      </x:c>
       <x:c r="O68" t="str"/>
       <x:c r="P68" t="str"/>
       <x:c r="Q68" t="str"/>
       <x:c r="R68" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -3319,25 +3328,25 @@
         <x:v>agree to disagree</x:v>
       </x:c>
       <x:c r="J71" t="str">
-        <x:v>Offering an unwarranted or premature truce on a point of contention in order to misrepresent opponent's position as unprovable or inconclusive.</x:v>
+        <x:v>Occurs when someone calls for a truce, balance, or 'agree to disagree' posture not because the evidence is genuinely inconclusive, but because their position is under pressure and they want to freeze the score.</x:v>
       </x:c>
       <x:c r="K71" t="str">
-        <x:v>My belief that all swans are white isn't necessarily falsified by your photo of a black swan. We'll just have to agree to disagree.</x:v>
+        <x:v>Your black-swan photo does not settle anything. Let's just agree that both of us may be right.</x:v>
       </x:c>
       <x:c r="L71" t="str">
-        <x:v>This tactic is often employed by the side with the weakest argument.</x:v>
+        <x:v>Real uncertainty exists, and sometimes compromise is appropriate. The fallacy appears when manufactured neutrality is used to protect a losing claim from the consequences of the evidence.</x:v>
       </x:c>
       <x:c r="M71" t="str">
-        <x:v>Culture X may concede that culture Y has the prerogative to continue with practices that culture X considers immoral, as long as culture Y makes the same concession for culture X. The ethical arguments for each practice are ignored.</x:v>
+        <x:v>Public arguments about evolution, election claims, and medical misinformation sometimes ask audiences to treat both sides as equally plausible even after the evidential balance is lopsided.</x:v>
       </x:c>
       <x:c r="N71" t="str">
-        <x:v>Evolution opponents will often concede that both evolution and intelligent design are valid viewpoints, implying that neither can be falsified or demonstrated, and that they have equal evidential support.</x:v>
+        <x:v>In online debate culture, a retreat into 'everyone has their own truth' often appears right after a concrete factual claim has gone badly for one side.</x:v>
       </x:c>
       <x:c r="O71" t="str"/>
       <x:c r="P71" t="str"/>
       <x:c r="Q71" t="str"/>
       <x:c r="R71" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3760,19 +3769,25 @@
       <x:c r="H81" t="str"/>
       <x:c r="I81" t="str"/>
       <x:c r="J81" t="str">
-        <x:v>An argument that appears to support both sides of an issue by employing terms that diminish the actual incompatability between the positions.</x:v>
+        <x:v>Occurs when someone uses strategically shifting language that seems to support both sides by quietly changing the meaning of the key term to suit the audience.</x:v>
       </x:c>
       <x:c r="K81" t="str">
-        <x:v>If by "affair" you mean the hurtful action of cheating on your spouse, then I'm much against it. But if by "affair" you mean the inevitable outcome of an adventurous spirit, then I'm all for it.</x:v>
-      </x:c>
-      <x:c r="L81" t="str"/>
-      <x:c r="M81" t="str"/>
-      <x:c r="N81" t="str"/>
+        <x:v>If by 'AI regulation' you mean stopping abuse, I support it. But if by 'AI regulation' you mean slowing innovation, I oppose it.</x:v>
+      </x:c>
+      <x:c r="L81" t="str">
+        <x:v>This is not mere nuance. The problem is rhetorical double-speaking that blurs real disagreement by sliding between incompatible senses of the same label.</x:v>
+      </x:c>
+      <x:c r="M81" t="str">
+        <x:v>Politicians often define contested terms like 'freedom,' 'censorship,' 'riot,' 'peaceful,' or 'family values' one way for sympathetic listeners and another way when challenged by critics.</x:v>
+      </x:c>
+      <x:c r="N81" t="str">
+        <x:v>Debates about AI, speech, and policing frequently proceed as if both camps agree until someone notices that the central term has been doing two very different jobs.</x:v>
+      </x:c>
       <x:c r="O81" t="str"/>
       <x:c r="P81" t="str"/>
       <x:c r="Q81" t="str"/>
       <x:c r="R81" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -4052,19 +4067,25 @@
       <x:c r="H88" t="str"/>
       <x:c r="I88" t="str"/>
       <x:c r="J88" t="str">
-        <x:v>Insulting or pejorative language to influence the recipient's judgment.</x:v>
+        <x:v>Occurs when pejorative, loaded, or insulting language is used to steer judgment in place of actual support for the conclusion.</x:v>
       </x:c>
       <x:c r="K88" t="str">
-        <x:v>Your position on free community health checks is accepted only by prostitutes! Only whores would accept such a concept!</x:v>
-      </x:c>
-      <x:c r="L88" t="str"/>
-      <x:c r="M88" t="str"/>
-      <x:c r="N88" t="str"/>
+        <x:v>Only a coward would oppose this bill.</x:v>
+      </x:c>
+      <x:c r="L88" t="str">
+        <x:v>Some labels are fair descriptions, but the fallacy appears when the emotional sting of the label is doing the work that evidence and argument have not done.</x:v>
+      </x:c>
+      <x:c r="M88" t="str">
+        <x:v>Words like 'groomer,' 'traitor,' 'fascist,' 'woke,' 'cultist,' and 'denier' are often deployed less to clarify than to trigger a moral reaction before the argument can be examined.</x:v>
+      </x:c>
+      <x:c r="N88" t="str">
+        <x:v>Political and religious arguments frequently pre-load the conclusion by choosing terms that make disagreement sound shameful or corrupt from the start.</x:v>
+      </x:c>
       <x:c r="O88" t="str"/>
       <x:c r="P88" t="str"/>
       <x:c r="Q88" t="str"/>
       <x:c r="R88" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -4734,25 +4755,25 @@
       <x:c r="H104" t="str"/>
       <x:c r="I104" t="str"/>
       <x:c r="J104" t="str">
-        <x:v>Occurs when one is connected to a second assumption in a non-contingent way, then the 1st assumption is deemed justified by evidence for the 2nd assumption.</x:v>
+        <x:v>Occurs when evidence for one claim is illegitimately used as if it also confirmed a second claim that merely travels alongside it.</x:v>
       </x:c>
       <x:c r="K104" t="str">
-        <x:v>I've told you that I'm a CIA agent from Boston. Here's my driver's license showing a Boston address. That should make it clear that I work for the CIA.</x:v>
+        <x:v>The affidavit got one stage detail right, so its larger conspiracy claims must be credible too.</x:v>
       </x:c>
       <x:c r="L104" t="str">
-        <x:v>This fallacy is true only where there is a non-contingent relationship. However, if you were to claim you had been married and produced an official document of your divorce, that constitutes evidence for both the divorce and a necessary prior marriage. To a softer degree, claiming that you met the president, then producing a photo of you together with the president's wife would constitute evidence for your claim you met the president.</x:v>
+        <x:v>A true or well-supported detail can increase trust only where the claims are genuinely linked. Often the extra conclusion is just hitching a ride on evidence that belongs to something narrower.</x:v>
       </x:c>
       <x:c r="M104" t="str">
-        <x:v>Some theists suggest that archeological evidence of biblical sites is evidence for the biblical miracles mentioned in the same passage as is the site. Uncovering historical evidence for the existence of St. Nicolas does not lend credibilty to flying reindeer.</x:v>
+        <x:v>After the September 2024 ABC debate, the fact that the lecterns differed in height was treated by some users as if it supported much broader unverified claims about secret coordination and leaked questions.</x:v>
       </x:c>
       <x:c r="N104" t="str">
-        <x:v>Some people argue that evidence for government impropriety on issue X implies that there is also impropriety on issue Y. While inductive evidence derived from assessing habitual behavior warrants a measured degree of speculation, it does not warrant confidence incommensurate to that evidence.</x:v>
+        <x:v>Conspiracy arguments often point to one authentic photo, real location, or correct minor fact and then use that narrow success to smuggle in much larger unsupported conclusions.</x:v>
       </x:c>
       <x:c r="O104" t="str"/>
       <x:c r="P104" t="str"/>
       <x:c r="Q104" t="str"/>
       <x:c r="R104" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -4908,23 +4929,25 @@
         <x:v>argumentum verbosium, proof by intimidation</x:v>
       </x:c>
       <x:c r="J108" t="str">
-        <x:v>Submitting an argument too complex, obtuse or verbose to reasonably deal with.</x:v>
+        <x:v>Occurs when a claim is protected by an avalanche of words, side points, jargon, or branching assertions that overwhelm reasonable scrutiny and create the illusion of depth.</x:v>
       </x:c>
       <x:c r="K108" t="str">
-        <x:v>Insomuch as it remains within our agency, it behooves us to eschew obfuscation, and espouse elucidation.</x:v>
+        <x:v>The theory must be right because nobody has time to answer all 87 points in my thread.</x:v>
       </x:c>
       <x:c r="L108" t="str">
-        <x:v>This is often a tactic used in formal speeches. If not all the many minor points introduced are not addressed by the opponent, the verbose contender will claim victory.</x:v>
+        <x:v>Complexity is not itself a fallacy. The problem is using sprawl as a shield, making it costly to respond point by point and then treating any unanswered fragment as proof of victory.</x:v>
       </x:c>
       <x:c r="M108" t="str">
-        <x:v>Donald Rumsfeld once said...There are known knowns. These are things we know that we know. There are known unknowns. That is to say, there are things that we know we don't know. But there are also unknown unknowns. There are things we don't know we don't know.</x:v>
-      </x:c>
-      <x:c r="N108" t="str"/>
+        <x:v>Podcast debates, marathon livestreams, and mega-threads often bury the central claim beneath so many tangents that audiences mistake exhaustion for concession.</x:v>
+      </x:c>
+      <x:c r="N108" t="str">
+        <x:v>AI-generated text makes this tactic cheaper by allowing people to produce long, confident, fast-moving argument dumps that sound comprehensive while remaining poorly grounded.</x:v>
+      </x:c>
       <x:c r="O108" t="str"/>
       <x:c r="P108" t="str"/>
       <x:c r="Q108" t="str"/>
       <x:c r="R108" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
@@ -5988,25 +6011,25 @@
       <x:c r="H133" t="str"/>
       <x:c r="I133" t="str"/>
       <x:c r="J133" t="str">
-        <x:v>When, for every new question, the inductive evidence from relevant past experience is ignored.</x:v>
+        <x:v>Occurs when each new claim is treated as if the relevant history of prior failures, hoaxes, or false alarms did not exist and should confer no default expectation at all.</x:v>
       </x:c>
       <x:c r="K133" t="str">
-        <x:v>Wake up, Dear! Something's banging on the trash cans again. I know that for the hundreds of other times you've checked, it's only been cats, but could you please go out and make sure it isn't zombies this time?</x:v>
+        <x:v>Yes, the last hundred miracle predictions failed, but this new one starts with a perfectly clean slate.</x:v>
       </x:c>
       <x:c r="L133" t="str">
-        <x:v>After thousands of investigations into claims of ghost hauntings, researchers have discovered many material causes, but no ghosts. Therefore, the next time someone claims to have seen a ghost, we are warranted in defaulting to the expectation of a material explanation.</x:v>
+        <x:v>A track record does not make contrary outcomes impossible, but it does affect rational priors. Ignoring repeated past failure forces every new case to borrow more credibility than it has earned.</x:v>
       </x:c>
       <x:c r="M133" t="str">
-        <x:v>After thousands of investigations into claims of ghost hauntings, researchers have discovered many material causes, but no ghosts. Therefore, the next time someone claims to have seen a ghost, we are warranted in defaulting to the expectation of a material explanation.</x:v>
+        <x:v>Baseless claims about widespread noncitizen voting keep getting relaunched as if decades of rarity, audits, and failed alarms provide no reason for initial skepticism.</x:v>
       </x:c>
       <x:c r="N133" t="str">
-        <x:v>For each new alleged miracle, many theists demand skeptics to demonstrate it was not a miracle, supposing that, until such negative proof is provided, they are warranted in believing it was an actual miracle. This ignores centuries of claims of miracles being shown to either fall well within the parameters of natural phenomena and statistics, or being too inaccessible to the scrutiny of science. This track record not only permits, but demands a default to a methodological naturalism in which we expect a material explanation, and in which the burden of proof rests entirely on those proposing something contrary to the successful track-record of material causes.</x:v>
+        <x:v>Every new blurry UFO clip, miracle cure, or ghost story is often pitched as if the long record of ordinary explanations should have zero effect on our starting expectations.</x:v>
       </x:c>
       <x:c r="O133" t="str"/>
       <x:c r="P133" t="str"/>
       <x:c r="Q133" t="str"/>
       <x:c r="R133" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -6160,29 +6183,25 @@
       <x:c r="H137" t="str"/>
       <x:c r="I137" t="str"/>
       <x:c r="J137" t="str">
-        <x:v>Occurs when terms are intentionally chosen for their vagueness in an attempt to make a position unassailable.</x:v>
+        <x:v>Occurs when vague, elastic, or undefined terms are chosen so that a position sounds meaningful while resisting clear testing or criticism.</x:v>
       </x:c>
       <x:c r="K137" t="str">
-        <x:v>The energy in these pills creates a force that balances the body's essences.</x:v>
+        <x:v>These capsules restore your body's subtle energies and harmonize your inner system.</x:v>
       </x:c>
       <x:c r="L137" t="str">
-        <x:v>In the example, "energy", "force", "balances" and "essences" are all too vague to submit to scientific scrutiny.</x:v>
+        <x:v>Vagueness can be useful early in exploration, but it becomes fallacious when the fog is preserved to prevent serious evaluation. If key terms cannot be pinned down, the claim can keep slipping away from critique.</x:v>
       </x:c>
       <x:c r="M137" t="str">
-        <x:v>There are only three sports: bullfighting, motor racing, and mountaineering; all the rest are merely games.
-~Ernest Hemmingway
-The definitions of "sports" and " games" are vague, and make a refutation difficult.</x:v>
+        <x:v>Alternative-health and wellness marketing often leans on words like 'toxins,' 'energy,' 'balance,' and 'boost' precisely because they sound scientific while remaining hard to falsify.</x:v>
       </x:c>
       <x:c r="N137" t="str">
-        <x:v>Theists often introduce words such as "faith" and "sin" that have definitions that are contested even within their own sect.</x:v>
-      </x:c>
-      <x:c r="O137" t="str">
-        <x:v>Those promoting alternative medicines often invoke vague terms such as "energy" and "essence" that seem to have no real referent that can be assessed and critiqued.</x:v>
-      </x:c>
+        <x:v>In arguments about spirituality, self-help, and even AI, flexible phrases can be stretched to fit almost any outcome, which makes the view feel resilient without making it well supported.</x:v>
+      </x:c>
+      <x:c r="O137" t="str"/>
       <x:c r="P137" t="str"/>
       <x:c r="Q137" t="str"/>
       <x:c r="R137" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="138">

</xml_diff>

<commit_message>
Expand evidential and epistemic rewrites
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R17e1dd59dc08462f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Racd1cbb768704858"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Ra05835a798084c54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6d85295873c840d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R27570ab94ec64491"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rcd9de94395f042fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1662,23 +1662,25 @@
       <x:c r="H32" t="str"/>
       <x:c r="I32" t="str"/>
       <x:c r="J32" t="str">
-        <x:v>The syntactic use of negation to wrongly imply an affirmative epistemic commitment.</x:v>
+        <x:v>Occurs when the wording of a negative position is manipulated so that mere non-belief is treated as if it were the same thing as a strong positive denial.</x:v>
       </x:c>
       <x:c r="K32" t="str">
-        <x:v>Where's your evidence for your belief that there are no unicorns? Your faith in the lack of unicorns is no different from my faith in the existence of unicorns.</x:v>
+        <x:v>If you say you are not convinced ghosts exist, then you are really making the positive claim that ghosts do not exist and now you owe proof.</x:v>
       </x:c>
       <x:c r="L32" t="str">
-        <x:v>A positive belief that there are no unicorns is not equivalent to no belief in unicorns. Having no belief in unicorns may be a result of never having heard of the concept of unicorns, or never having had sufficient evidence to believe they exist.</x:v>
+        <x:v>There is an important difference between suspending belief, doubting a claim, and asserting the opposite claim. Collapsing those positions is often a way of shifting burdens that have not been earned.</x:v>
       </x:c>
       <x:c r="M32" t="str">
-        <x:v>Some suggest that the suspension of belief in a particular god-claim is itself an affirmative belief. The arguments goes "It's not that you merely have no belief in my version of god; you believe that my god does not exist!" This claim is then employed in an attempt to demonstrate that "we both have faith" or "you have to provide evidence for your no-god belief." Believing that there is not enough evidence to believe a particular claim is not an affirmative belief; it is a negative belief, and does not require faith or possess the burden of proof.</x:v>
-      </x:c>
-      <x:c r="N32" t="str"/>
+        <x:v>Religious and paranormal debates often insist that skepticism itself is just another faith commitment, as if withholding belief carried the same evidential burden as proposing the phenomenon.</x:v>
+      </x:c>
+      <x:c r="N32" t="str">
+        <x:v>Arguments about election fraud and miracle claims sometimes recast 'I have not seen enough evidence' into 'you are certain it never happened' so the original claimant can dodge the burden of proof.</x:v>
+      </x:c>
       <x:c r="O32" t="str"/>
       <x:c r="P32" t="str"/>
       <x:c r="Q32" t="str"/>
       <x:c r="R32" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2436,27 +2438,25 @@
       <x:c r="H50" t="str"/>
       <x:c r="I50" t="str"/>
       <x:c r="J50" t="str">
-        <x:v>Occurs when overwhelming evidence for a phenomenon is rejected on the grounds that the causal mechanism is not known or understood.</x:v>
+        <x:v>Occurs when strong evidence for a phenomenon is rejected solely because the underlying mechanism is still incomplete, disputed, or not yet fully understood.</x:v>
       </x:c>
       <x:c r="K50" t="str">
-        <x:v>Scientists still can't explain how and why lightning occurs. Therefore, I am not obligated to assume that the cause is electromagnetic.</x:v>
+        <x:v>Until scientists can explain exactly how this pattern arises, we should not accept that the pattern is real.</x:v>
       </x:c>
       <x:c r="L50" t="str">
-        <x:v>Though the existence of a coherent and predictive mechanism is significant evidence for belief in a particular phenomenon, very often, there are other forms of evidence that are sufficient to warrant belief, even when a mechanism is missing from the theory. Consider a scenario in which an individual claims to be able to predict the outcome of coin-flips on a fair coin. Your skepticism is warranted for perhaps the first 10-20 correctly predicted flips, but at some point, you will be compelled to concede that, even though you don't know the mechanism, the individual's claim warrants your belief.</x:v>
+        <x:v>Mechanisms matter, but evidence can justify belief before the full causal story is finished. Observation often outruns explanation.</x:v>
       </x:c>
       <x:c r="M50" t="str">
-        <x:v>For many years, people were attributing the flight of the bumblebee to something miraculous since there was, at that time, no credible material mechanism available to explain how so small a wing surface could successfully levitate the relatively large mass of the bumblebee.</x:v>
+        <x:v>Public disputes about climate, evolution, and health regularly treat unresolved details in the mechanism as if they erased the larger evidential picture.</x:v>
       </x:c>
       <x:c r="N50" t="str">
-        <x:v>Some claim evolution cannot be accepted as fact until the mechanism is fully teased out, in spite of much converging evidence for evolution from many domains of research.</x:v>
-      </x:c>
-      <x:c r="O50" t="str">
-        <x:v>It is sometimes claimed that dualism, the belief that mind and brain are separate entities, warrants no credibility until a mechanism that explains how the immaterial can interface with the material is discovered and explained. However, if there was clear evidence of ESP in which the mind exhibited an independence of physical location, then that would possible constitute sufficient evidence for belief in dualism, even in the absence of a known mechanism.</x:v>
-      </x:c>
+        <x:v>Research on AI transcription errors in 2024 showed that systems were inventing statements people never said; even before every technical cause was nailed down, the pattern itself was already evidence of a real reliability problem.</x:v>
+      </x:c>
+      <x:c r="O50" t="str"/>
       <x:c r="P50" t="str"/>
       <x:c r="Q50" t="str"/>
       <x:c r="R50" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -2482,21 +2482,25 @@
       <x:c r="H51" t="str"/>
       <x:c r="I51" t="str"/>
       <x:c r="J51" t="str">
-        <x:v>Attempting to avoid the burden of proof for some claim by demanding proof of the contrary from whoever questions that claim.</x:v>
+        <x:v>Occurs when someone tries to protect a claim by insisting that critics must prove the claim false instead of the claimant first supplying adequate support.</x:v>
       </x:c>
       <x:c r="K51" t="str">
-        <x:v>Can you prove I'm not wearing an invisible hat?</x:v>
+        <x:v>You cannot say the vote-rigging plot is false unless you can prove every suspicious clip has an innocent explanation.</x:v>
       </x:c>
       <x:c r="L51" t="str">
-        <x:v>Similar to "negative proof fallacy."</x:v>
-      </x:c>
-      <x:c r="M51" t="str"/>
-      <x:c r="N51" t="str"/>
+        <x:v>Sometimes counterevidence matters, but the default burden still sits with the person making the substantive claim. Lack of disproof is not the same as proof.</x:v>
+      </x:c>
+      <x:c r="M51" t="str">
+        <x:v>Conspiracy claims about noncitizen voting, ballot destruction, or machine tampering often survive by demanding that every rumor be individually disproved rather than by presenting strong evidence that the conspiracy exists.</x:v>
+      </x:c>
+      <x:c r="N51" t="str">
+        <x:v>Miracle, UFO, and paranormal arguments frequently say skeptics must show exactly what happened in each case, as though the claimant had no burden until that impossible task is finished.</x:v>
+      </x:c>
       <x:c r="O51" t="str"/>
       <x:c r="P51" t="str"/>
       <x:c r="Q51" t="str"/>
       <x:c r="R51" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -2518,23 +2522,25 @@
       <x:c r="H52" t="str"/>
       <x:c r="I52" t="str"/>
       <x:c r="J52" t="str">
-        <x:v>Diminishing semantic resolution by creating artificially discrete epistemic categories.</x:v>
+        <x:v>Occurs when belief is forced into crude either-or boxes even though the evidence supports a range of confidence levels rather than a single sharp threshold.</x:v>
       </x:c>
       <x:c r="K52" t="str">
-        <x:v>Either you believe in space aliens or you don't! Tell me whether you believe in space aliens!</x:v>
+        <x:v>Stop hedging. Either you believe AI systems are conscious or you do not.</x:v>
       </x:c>
       <x:c r="L52" t="str">
-        <x:v>Evidence commonly arrives in degrees. If belief is to be warranted, it must map to the evidence. Therefore, belief is necessarily non-discrete.</x:v>
+        <x:v>Responsible belief often comes in degrees. Treating confidence as all-or-nothing hides uncertainty, nuance, and the actual strength of the evidence.</x:v>
       </x:c>
       <x:c r="M52" t="str">
-        <x:v>Both theists and atheists often over-categorize the position of others by suggesting one must either belief or disbelieve in a god. However, unless you belief the evidence for a particular god arrives in discrete packets, it must be admitted that belief in that god will fall somewhere on a continuum.</x:v>
-      </x:c>
-      <x:c r="N52" t="str"/>
+        <x:v>Debates about God, UFOs, AI consciousness, and election fraud often demand yes-or-no declarations even when the intellectually honest position is conditional, partial, or still under revision.</x:v>
+      </x:c>
+      <x:c r="N52" t="str">
+        <x:v>Culture-war exchanges frequently treat probabilistic language such as 'unlikely,' 'not yet shown,' or 'some evidence but not enough' as weakness rather than as proper calibration.</x:v>
+      </x:c>
       <x:c r="O52" t="str"/>
       <x:c r="P52" t="str"/>
       <x:c r="Q52" t="str"/>
       <x:c r="R52" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -2556,27 +2562,25 @@
       <x:c r="H53" t="str"/>
       <x:c r="I53" t="str"/>
       <x:c r="J53" t="str">
-        <x:v>Occurs when a worthy hypothetical is rejected on grounds it is rare or improbable.</x:v>
+        <x:v>Occurs when a hypothetical test case is dismissed as irrelevant merely because it is rare, extreme, or unlikely, even though the principle under debate is supposed to be universal.</x:v>
       </x:c>
       <x:c r="K53" t="str">
-        <x:v>Your scenario of having to choose between killing your child or your father or letting them both starve does is not applicable to my moral code since such a dilemma has probably never actually occurred in real life.</x:v>
+        <x:v>That edge case does not matter because it almost never happens.</x:v>
       </x:c>
       <x:c r="L53" t="str">
-        <x:v>If someone suggests they are in possession of a universal moral law, then even the most improbable scenarios is fair game to test that universal moral law. If you say killing another human is always wrong, then you'll need to address any conceivable scenario in which one human is faced with the choice of killing another.</x:v>
+        <x:v>A remote hypothetical can still be useful when the issue is whether a rule really holds without exception. Improbable cases often expose hidden limits in principles that sounded absolute.</x:v>
       </x:c>
       <x:c r="M53" t="str">
-        <x:v>One remote scenario and moral dilemma is a situation in which you have the opportunity to save several lives on a trail by pushing a single person onto the tracks, thus killing him. The fact that the scenario is improbable does not mean that it cannot be used to test the validity and consistency of a moral principle.</x:v>
+        <x:v>Arguments about free speech, self-defense, abortion, lying, and triage often reject hard edge cases simply because they are uncomfortable, even though those cases are precisely what test universal rules.</x:v>
       </x:c>
       <x:c r="N53" t="str">
-        <x:v>Another scenario and moral dilemma is a situation in which there are 10 persons of various ages, sizes, intelligences, talents and genders on a lifeboat with only enough food for 20 meals. How do you allot the food? This remote scenario is a legitimate test of a moral code.</x:v>
-      </x:c>
-      <x:c r="O53" t="str">
-        <x:v>Another remote scenario is a situation in which a mother, hiding with her child and 20 other innocent people from men with guns, must decide to smother her crying child in order to save herself and the 20 others.</x:v>
-      </x:c>
+        <x:v>Policy debates about AI safety and biosecurity sometimes wave away low-probability scenarios too quickly, even when the whole argument concerns whether a system is robust under stress.</x:v>
+      </x:c>
+      <x:c r="O53" t="str"/>
       <x:c r="P53" t="str"/>
       <x:c r="Q53" t="str"/>
       <x:c r="R53" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -2818,25 +2822,25 @@
       <x:c r="H59" t="str"/>
       <x:c r="I59" t="str"/>
       <x:c r="J59" t="str">
-        <x:v>Occurs when the effects of a belief in a thing are assumed to be evidence for the existence of that thing.</x:v>
+        <x:v>Occurs when the psychological or social effects of believing something are treated as evidence that the thing believed in actually exists or is true.</x:v>
       </x:c>
       <x:c r="K59" t="str">
-        <x:v>Those who believe they are intelligent, out-perform those who think they are not intelligent on IQ tests. Therefore they are more intelligent.</x:v>
+        <x:v>People who trust this ritual feel calmer and more purposeful, so that shows the invisible force behind it is real.</x:v>
       </x:c>
       <x:c r="L59" t="str">
-        <x:v>This fallacy is essentially that of ignoring the placebo effect or other mental effects of belief.</x:v>
+        <x:v>Beliefs can change mood, confidence, behavior, pain perception, and group cohesion regardless of whether their object exists. The benefits of belief do not by themselves settle the ontology.</x:v>
       </x:c>
       <x:c r="M59" t="str">
-        <x:v>Many of those who believe in homeopathy are usually heal after taking homeopathy medicine. It's supporters often claim this is proof for the efficacy of the medicine, and ignore possible placebo effects.</x:v>
+        <x:v>Raw milk, supplement, and alternative-health advocates often point to the felt benefits reported by believers while skipping the role of expectation, placebo effects, and other background changes.</x:v>
       </x:c>
       <x:c r="N59" t="str">
-        <x:v>Some studies that allegedly show that theists are happier than atheists are extended as evidence for the power of god, rather than the power of belief in god.</x:v>
+        <x:v>Arguments that religion must be true because believers report comfort, purpose, or improved well-being often confuse the power of belief with evidence for the reality of the object believed in.</x:v>
       </x:c>
       <x:c r="O59" t="str"/>
       <x:c r="P59" t="str"/>
       <x:c r="Q59" t="str"/>
       <x:c r="R59" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -3374,21 +3378,25 @@
       <x:c r="H72" t="str"/>
       <x:c r="I72" t="str"/>
       <x:c r="J72" t="str">
-        <x:v>Occurs when an inductive conclusion is unwarranted by the degree of evidence or ignores information that warrants an exception.</x:v>
+        <x:v>Occurs when an inductive conclusion reaches further than the available evidence can reasonably support, or ignores information that should limit the generalization.</x:v>
       </x:c>
       <x:c r="K72" t="str">
-        <x:v>He and his 4 brothers are bald, so his mother must also be bald.</x:v>
+        <x:v>Two chatbots hallucinated legal citations, so large language models are useless for every serious task.</x:v>
       </x:c>
       <x:c r="L72" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
-      </x:c>
-      <x:c r="M72" t="str"/>
-      <x:c r="N72" t="str"/>
+        <x:v>Generalization is unavoidable, but it has to be scaled to the quality, size, and representativeness of the evidence. The problem is not generalizing at all; it is generalizing too aggressively.</x:v>
+      </x:c>
+      <x:c r="M72" t="str">
+        <x:v>Viral anecdotes about migrants, students, police, or AI tools often get inflated into sweeping claims about entire groups or systems after only a handful of cases.</x:v>
+      </x:c>
+      <x:c r="N72" t="str">
+        <x:v>Election and media arguments routinely take one error, one clip, or one scandal as proof that the whole institution always behaves the same way.</x:v>
+      </x:c>
       <x:c r="O72" t="str"/>
       <x:c r="P72" t="str"/>
       <x:c r="Q72" t="str"/>
       <x:c r="R72" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -4887,21 +4895,25 @@
       <x:c r="H107" t="str"/>
       <x:c r="I107" t="str"/>
       <x:c r="J107" t="str">
-        <x:v>Occurs when examples are offered as inductive proof for a universal proposition.</x:v>
+        <x:v>Occurs when one or a few examples are offered as if they were enough to establish a universal claim.</x:v>
       </x:c>
       <x:c r="K107" t="str">
-        <x:v>This apple is red, so all apples must be red.</x:v>
+        <x:v>My friend used a chatbot to draft a great memo, so AI is clearly ready to replace analysts.</x:v>
       </x:c>
       <x:c r="L107" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
-      </x:c>
-      <x:c r="M107" t="str"/>
-      <x:c r="N107" t="str"/>
+        <x:v>Examples can illustrate a claim, but they do not by themselves prove a universal proposition. The missing question is whether the example is representative.</x:v>
+      </x:c>
+      <x:c r="M107" t="str">
+        <x:v>A single accurate prediction, one striking conversion story, or one dramatic crime clip is often treated as if it proved a broad thesis about markets, religion, or social decline.</x:v>
+      </x:c>
+      <x:c r="N107" t="str">
+        <x:v>Debates about AI often jump from one impressive demo or one embarrassing failure to a total conclusion about the technology as a whole.</x:v>
+      </x:c>
       <x:c r="O107" t="str"/>
       <x:c r="P107" t="str"/>
       <x:c r="Q107" t="str"/>
       <x:c r="R107" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -5089,24 +5101,25 @@
       <x:c r="H112" t="str"/>
       <x:c r="I112" t="str"/>
       <x:c r="J112" t="str">
-        <x:v>Occurs when a proponent of an illogical concept demands evidence before dismissing the illogical concept.</x:v>
+        <x:v>Occurs when someone demands empirical evidence before rejecting a concept that is already incoherent, self-contradictory, or logically impossible on its own terms.</x:v>
       </x:c>
       <x:c r="K112" t="str">
-        <x:v>I have a golden square triangle instead of a heart in my chest, and I have the lab analysis to prove it.</x:v>
+        <x:v>You cannot dismiss my square triangle theory until you check all the data.</x:v>
       </x:c>
       <x:c r="L112" t="str">
-        <x:v>If someone claims to have a golden square triangle in their chest, and provides gold flakes or a lab analysis as evidence, you don't have to test the gold flakes or scrutinize the lab analysis for authenticity before you dismiss the notion that they have a golden square triangle in their chest. If a concept has been demonstrated to be illogical, no amount of evidence will salvage that concept.
-To a lesser degree, what we define as physical impossibilities can be dismissed in the same way we can dismiss logical impossibilities. However, we must be careful since what is physical laws have been abstracted from nature by humans, and may not be absolute. However, this caveat does not mean we are wrong to dismiss with a high degree of confidence any concept that science considers a physical impossibility.</x:v>
+        <x:v>Evidence matters for empirical claims, but it cannot rescue a contradiction. If the concept itself does not make sense, more observations do not repair it.</x:v>
       </x:c>
       <x:c r="M112" t="str">
-        <x:v>Some theists define their god as both infinitely "loving" and infinitely "hateful" to humans. We need not scrutinize their holy book or nature for evidence of their incoherent god. If there is evidence for a god in nature, their god has already been eliminated as a candidate due to the absurdity of his definition.</x:v>
-      </x:c>
-      <x:c r="N112" t="str"/>
+        <x:v>Some arguments define a being, force, or property in mutually incompatible ways and then insist critics still need field evidence before calling the view incoherent.</x:v>
+      </x:c>
+      <x:c r="N112" t="str">
+        <x:v>Online debate often treats every claim as if it deserved purely empirical testing, even when the real defect appears earlier at the level of definition or logical consistency.</x:v>
+      </x:c>
       <x:c r="O112" t="str"/>
       <x:c r="P112" t="str"/>
       <x:c r="Q112" t="str"/>
       <x:c r="R112" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -5312,23 +5325,25 @@
       <x:c r="H117" t="str"/>
       <x:c r="I117" t="str"/>
       <x:c r="J117" t="str">
-        <x:v>An argument that wrongly assumes that what is most pleasant is most true.</x:v>
+        <x:v>Occurs when the desirability, comfort, or emotional appeal of an outcome is treated as if that were evidence that the outcome is true, feasible, or justified.</x:v>
       </x:c>
       <x:c r="K117" t="str">
-        <x:v>It would be great if we could reduce the national debt without raising taxes or reducing spending. Therefore there must be a way we can accomplish this.</x:v>
+        <x:v>It would be beautiful if this treatment worked for everyone, so there must be a way to make that story true.</x:v>
       </x:c>
       <x:c r="L117" t="str">
-        <x:v>This fallacy is similar to wishful thinking.</x:v>
+        <x:v>Emotional attraction can explain why we want a conclusion, but not whether the conclusion is supported. A heartwarming possibility can still be false or impractical.</x:v>
       </x:c>
       <x:c r="M117" t="str">
-        <x:v>If, in response to painful demographic gaps in health care coverage, it is argued that having a national health care bill would be a wonderful thing, and is therefore necessary, this would be committing the sentimental fallacy. The desire for something does not warrant its realization. Other factors such as long-term consequences must be considered. Emotion does not carry an imperative.</x:v>
-      </x:c>
-      <x:c r="N117" t="str"/>
+        <x:v>Fundraising pitches, miracle-cure stories, and uplifting viral posts often rely on the emotional payoff of the conclusion to make scrutiny feel mean or unnecessary.</x:v>
+      </x:c>
+      <x:c r="N117" t="str">
+        <x:v>Public debate about policy sometimes slides from 'this would be compassionate' to 'therefore it must be workable and correct,' skipping the harder evidential and tradeoff questions.</x:v>
+      </x:c>
       <x:c r="O117" t="str"/>
       <x:c r="P117" t="str"/>
       <x:c r="Q117" t="str"/>
       <x:c r="R117" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -6271,29 +6286,25 @@
       <x:c r="H139" t="str"/>
       <x:c r="I139" t="str"/>
       <x:c r="J139" t="str">
-        <x:v>Occurs when a witness attempts to bolster their own testimony by claiming, with no independent substantiation, that there were other witnesses.</x:v>
+        <x:v>Occurs when testimony is padded by unverifiable references to other alleged witnesses, creating the illusion of corroboration without actually providing independent support.</x:v>
       </x:c>
       <x:c r="K139" t="str">
-        <x:v>I saw a ghost 5 years ago, and my uncle who died last year told me he also saw it!</x:v>
+        <x:v>I saw the miracle myself, and dozens of others saw it too, though none of them are available to check.</x:v>
       </x:c>
       <x:c r="L139" t="str">
-        <x:v>The claim of an accessible witness to an event that there are inaccessible additional witnesses to that event carries no evidential weight for that event.</x:v>
+        <x:v>Real corroboration requires accessible, independent testimony or records. Simply claiming that more witnesses exist adds almost nothing if the chain cannot be examined.</x:v>
       </x:c>
       <x:c r="M139" t="str">
-        <x:v>"I have personally witnessed irrefutable miracle healings (i.e. stunted limb growing out to full length spontaneously in a matter of seconds,) in response to prayer in the name of Jesus. I would guess there were close to 40 witnesses to this miracle healing, many of whom, including myself, were standing only 2 or 3 feet away from the man who was healed; some of whom I still know by first and/or last name."
-[Source].</x:v>
+        <x:v>Paranormal, religious, and conspiracy stories often swell in authority by invoking unnamed doctors, secret insiders, or hundreds of silent observers who never become independently available.</x:v>
       </x:c>
       <x:c r="N139" t="str">
-        <x:v>After that, he [Jesus, after his alleged resurrection] appeared to more than five hundred of the brothers at the same time, most of whom are still living, though some have fallen asleep.
-1 Corinthians 15:6
-This verse is often cited by Christians as evidence for the resurrection.
-[Example].</x:v>
+        <x:v>Historical arguments sometimes treat a late report that 'many people saw it' as if that were the same thing as actually having many separate testimonies.</x:v>
       </x:c>
       <x:c r="O139" t="str"/>
       <x:c r="P139" t="str"/>
       <x:c r="Q139" t="str"/>
       <x:c r="R139" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -6317,25 +6328,25 @@
       <x:c r="H140" t="str"/>
       <x:c r="I140" t="str"/>
       <x:c r="J140" t="str">
-        <x:v>Occurs when actual cause and effect are mistakenly reversed.</x:v>
+        <x:v>Occurs when a real association is noticed but the direction of causation is reversed.</x:v>
       </x:c>
       <x:c r="K140" t="str">
-        <x:v>I've noticed that people with psychological disorders tend to use recreational drugs. They must be taking drugs to relieve the trauma of their disorders.</x:v>
+        <x:v>People who are already struggling concentrate more on self-help content, so the content must be what created the struggle.</x:v>
       </x:c>
       <x:c r="L140" t="str">
-        <x:v>Without evidence to indicate causation and the direction of that causation, the coincidence of two phenomena is at best correlation.</x:v>
+        <x:v>Correlations can be real while still pointing the wrong way. Without evidence about timing, mechanism, and alternatives, reversing cause and effect is easy.</x:v>
       </x:c>
       <x:c r="M140" t="str">
-        <x:v>The increase of handguns has often been cited as the cause of increasing crime. Before this claim can be rigorously substantiated, the degree that crime has had on the increase in handguns purchased for increased personal security in the area of increased crime will have to be teased out.</x:v>
+        <x:v>Arguments about social media and teen mental health often assume a one-way causal story even though distress can also increase the tendency to seek certain kinds of online engagement.</x:v>
       </x:c>
       <x:c r="N140" t="str">
-        <x:v>In the middle ages, Europeans noticed that people who got sick had fewer fleas on their bodies, leading them to conclude that fleas prevent illness. The actual mechanism was that an illness was usually accompanied by a fever, which then forced the heat-sensitive fleas to look for another host.</x:v>
+        <x:v>Crime, policing, and economic debates frequently treat a response variable as if it were the cause, such as assuming security purchases create fear rather than fear driving security purchases.</x:v>
       </x:c>
       <x:c r="O140" t="str"/>
       <x:c r="P140" t="str"/>
       <x:c r="Q140" t="str"/>
       <x:c r="R140" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Modernize conceptual and linguistic fallacies
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6d85295873c840d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R27570ab94ec64491"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rcd9de94395f042fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R33c940c6b5af40b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R2519e6195e644bb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R2c9b867674c44805"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -353,25 +353,25 @@
       <x:c r="H3" t="str"/>
       <x:c r="I3" t="str"/>
       <x:c r="J3" t="str">
-        <x:v>Occurs when an abstraction is denied existence or agency by claiming the substrate is the actual theater of agency.</x:v>
+        <x:v>Occurs when someone denies the reality or causal relevance of a higher-level pattern just because the pattern is realized through lower-level parts.</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>You can't claim that computers "work" since it is, in fact, merely transistors that are doing the actual processing.</x:v>
+        <x:v>There is no such thing as inflation hurting families; there are only individual transactions between buyers and sellers.</x:v>
       </x:c>
       <x:c r="L3" t="str">
-        <x:v>In most cases, any individual who denies the emergent properties of any abstracted concept can be shown to be inconsistent by asking whether they believe in other emergent properties such as economic recessions, bird migrations, fashion trends, and insect swarming.</x:v>
+        <x:v>Abstract patterns can still be real and explanatory even when they depend on smaller physical or social components. Economies, institutions, languages, and ecosystems do not stop being real because they are made of people, words, or organisms.</x:v>
       </x:c>
       <x:c r="M3" t="str">
-        <x:v>Some have argued that it is wrong to say "science works" since it takes an actual scientist to do science. This is to deny the ability (and goal) of science as an institution to minimize subjective error in the quest for truth by taking the process out of the hands of its constituents (subjective scientists) and to place it in the hands of a method that includes peer review that maximizes objectivity.</x:v>
+        <x:v>People sometimes say 'science does not discover anything, only scientists do,' as if that erased the reality of science as a method and institution with stable norms and effects.</x:v>
       </x:c>
       <x:c r="N3" t="str">
-        <x:v>One related issue is linguistic meaning. Some erroneously suggest that words themselves possess meaning rather the linguistic community in which those words are employed. Linguistic meaning is a product of convention, and is not immutably contained in the word itself. This causes individuals to irrationally demand others to adopt their own understanding of a term rather than simply seeking a common term that facilitates the communication of the concept.</x:v>
+        <x:v>Debates about algorithms, markets, and social platforms often pretend there is no system-level behavior because only users or lines of code act at the micro level.</x:v>
       </x:c>
       <x:c r="O3" t="str"/>
       <x:c r="P3" t="str"/>
       <x:c r="Q3" t="str"/>
       <x:c r="R3" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -391,27 +391,25 @@
       <x:c r="H4" t="str"/>
       <x:c r="I4" t="str"/>
       <x:c r="J4" t="str">
-        <x:v>Occurs when a law abstracted from observation is considered to be logically necessary.</x:v>
+        <x:v>Occurs when a model, law, or abstraction drawn from experience is treated as if it were a logically necessary rule that reality cannot ever depart from.</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>The law of gravity says that two objects of mass attract each other, so when physicists say gravity can repel, they don't know what they're talking about.</x:v>
+        <x:v>Moore's Law says computing power keeps doubling, so any slowdown would be impossible.</x:v>
       </x:c>
       <x:c r="L4" t="str">
-        <x:v>In the gravity example, the very physicist who christened the "law of gravity" also believe it repels in some cases. Each law is only reliable to the extent of its predictive success, and may come with stipulations. This is a type of faulty generalization that arises when induction justifiably categorizes an event or state extremely improbable. The fallacy arises when we say something that is physically improbable is logically impossible. A more detailed treatment of faulty generalizations can be found on the supplementary Inductive Errors page.</x:v>
+        <x:v>Useful abstractions describe patterns with varying scope and durability. They are not automatically eternal, exceptionless constraints on what can happen.</x:v>
       </x:c>
       <x:c r="M4" t="str">
-        <x:v>Consider the Law of Reciprocity. This law describes how healthy societies find cohesion when a critical level of altruism is reached among its constituents. However, its descriptive power does not in any way imply that societies will actualize cohesion based on altruism.</x:v>
+        <x:v>People often treat economic or technological 'laws' as if they guaranteed the future rather than summarizing a contingent historical pattern that may bend, pause, or fail.</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>The Law of Diminishing Returns is another good example. This law is an inductive generalization from our economic interactions. This law does not constrain economics, nor is prior to it, but rather economic phenomena restrict our formulation of economic laws.</x:v>
-      </x:c>
-      <x:c r="O4" t="str">
-        <x:v>Moore's Law which states that the number of transistors that can be inexpensively placed on a circuit board doubles about every 2 years is another example. Due to physical constraints, this law is expected to fail at some point. This is also a type of human standard fallacy in which an artifact of human abstraction is given more authority than is warranted.</x:v>
-      </x:c>
+        <x:v>In AI discourse, scaling trends are sometimes talked about as destiny, as though past curves logically force a particular future rather than merely suggesting one.</x:v>
+      </x:c>
+      <x:c r="O4" t="str"/>
       <x:c r="P4" t="str"/>
       <x:c r="Q4" t="str"/>
       <x:c r="R4" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2146,25 +2144,25 @@
         <x:v>distribution fallacy</x:v>
       </x:c>
       <x:c r="J43" t="str">
-        <x:v>The misconception that something true of the constituents of a whole must also necessarily be true of the whole.</x:v>
+        <x:v>Occurs when something true of the parts is assumed to be true of the whole they compose.</x:v>
       </x:c>
       <x:c r="K43" t="str">
-        <x:v>Paper money can be exchanged. An economy is composed of paper money, so an economy can be exchanged.</x:v>
+        <x:v>Each feature we added tested well in isolation, so the full product must be excellent.</x:v>
       </x:c>
       <x:c r="L43" t="str">
-        <x:v>This is the converse of the division fallacy.</x:v>
+        <x:v>Parts can interact in ways that change the result at the larger scale. What is beneficial, efficient, or true locally may not stay that way globally.</x:v>
       </x:c>
       <x:c r="M43" t="str">
-        <x:v>Were someone to argue "The average Canadian makes only 90% of what the average American makes, so Canada's GDP is 90% of the GDP of the U.S.", they would be committing the composition fallacy.</x:v>
+        <x:v>A company may assume that because every team is cutting costs responsibly, the organization as a whole will thrive, even though simultaneous cuts can gut the shared systems the teams depend on.</x:v>
       </x:c>
       <x:c r="N43" t="str">
-        <x:v>If you were to suggest that, because the average Japanese is 90% certain that ghosts exist, 90% of Japanese believe in ghosts, you would be committing the composition fallacy.</x:v>
+        <x:v>In policy debates, people often assume that what is prudent for one household, firm, or voter must be prudent for the entire economy or democracy at once.</x:v>
       </x:c>
       <x:c r="O43" t="str"/>
       <x:c r="P43" t="str"/>
       <x:c r="Q43" t="str"/>
       <x:c r="R43" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2318,25 +2316,25 @@
         <x:v>fallacy of the beard</x:v>
       </x:c>
       <x:c r="J47" t="str">
-        <x:v>Rejecting an argument on the grounds that one of it's concepts cannot be defined discretely into a precise category.</x:v>
+        <x:v>Occurs when a claim is rejected simply because the concept involved has blurry boundaries rather than a perfectly sharp cutoff.</x:v>
       </x:c>
       <x:c r="K47" t="str">
-        <x:v>You can't claim that your backpack is heavy until you give me a precise definition of "heavy."</x:v>
+        <x:v>You cannot call this ad misleading unless you can identify the exact word where persuasion becomes deception.</x:v>
       </x:c>
       <x:c r="L47" t="str">
-        <x:v>This fallacy highlights the need to employ terms that are as precise and quantified as possible. The fallacy is not always on the side of the person suggesting a proposition has no meaning until imprecise terms are defined. Sometime the burden of clarification is on the party who is making a claim. Claims can be so imprecise as to be impotent.</x:v>
+        <x:v>Many real concepts come in degrees. Vagueness at the boundary does not make the broader concept meaningless or unusable.</x:v>
       </x:c>
       <x:c r="M47" t="str">
-        <x:v>One common example of the continuum fallacy is in a scenario in which one must determine what constitutes "evidence" and "proof"for a given proposition. If someone claims to be able to accurately predict coin flips, for example, just how many consecutive correctly predicted flips would constitute evidence (beyond statistical noise) for the claim? And how many flips would constitute proof of this ability? The take-away caveat is that we need to define our terms as rigorously as possible, and not try to constrain concepts that inherently fall on a continuum to discrete categories.</x:v>
+        <x:v>Arguments about misinformation, bias, wealth, addiction, and consciousness often demand an impossible razor-sharp line and then pretend the lack of that line defeats the concept altogether.</x:v>
       </x:c>
       <x:c r="N47" t="str">
-        <x:v>Imagine a client claims you took "too long" to deliver a product, and refuses to pay for the product. Claiming that "too long" is an incorrect term since other companies take longer to deliver is an instantiation of the continuum fallacy. It is best to clearly stipulate your terms of delivery to your clients prior to their ordering.</x:v>
+        <x:v>In everyday disputes, someone may deny that a delay was 'too long' or a fee was 'too high' simply because no exact threshold was announced in advance.</x:v>
       </x:c>
       <x:c r="O47" t="str"/>
       <x:c r="P47" t="str"/>
       <x:c r="Q47" t="str"/>
       <x:c r="R47" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2406,19 +2404,25 @@
       <x:c r="H49" t="str"/>
       <x:c r="I49" t="str"/>
       <x:c r="J49" t="str">
-        <x:v>Involves the confusion between two notions by defining one in terms of the other.</x:v>
+        <x:v>Occurs when a substantive question is illegitimately 'solved' by defining one contested concept into another.</x:v>
       </x:c>
       <x:c r="K49" t="str">
-        <x:v>Justice is simply whatever the law permits, so once a policy is legal it is automatically just.</x:v>
-      </x:c>
-      <x:c r="L49" t="str"/>
-      <x:c r="M49" t="str"/>
-      <x:c r="N49" t="str"/>
+        <x:v>Justice just means whatever the law permits, so once a policy is legal it is automatically just.</x:v>
+      </x:c>
+      <x:c r="L49" t="str">
+        <x:v>Definitions can clarify usage, but they do not settle the underlying issue by fiat. Rewording a problem is not the same as answering it.</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>Culture-war debates often define words like 'freedom,' 'woman,' 'democracy,' or 'terrorism' in ways that quietly smuggle the desired conclusion into the starting point.</x:v>
+      </x:c>
+      <x:c r="N49" t="str">
+        <x:v>Moral and political disputes frequently collapse into dictionary wars where one side pretends that owning the label settles the argument.</x:v>
+      </x:c>
       <x:c r="O49" t="str"/>
       <x:c r="P49" t="str"/>
       <x:c r="Q49" t="str"/>
       <x:c r="R49" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -2696,25 +2700,25 @@
         <x:v>distribution fallacy</x:v>
       </x:c>
       <x:c r="J56" t="str">
-        <x:v>Occurs when one reasons logically that something true of an entire thing must also be true of all or some of its parts.</x:v>
+        <x:v>Occurs when something true of a whole is assumed to be true of each part or member of that whole.</x:v>
       </x:c>
       <x:c r="K56" t="str">
-        <x:v>Because a brain possesses thoughts, and a brain is composed of neurons, therefore these neurons pass thoughts back and forth.</x:v>
+        <x:v>The university is wealthy, so every department there must be flush with cash.</x:v>
       </x:c>
       <x:c r="L56" t="str">
-        <x:v>This is the converse of the composition fallacy.</x:v>
+        <x:v>A whole can have properties its parts do not share equally. Group-level success, size, reputation, or wealth does not automatically distribute itself down to each component.</x:v>
       </x:c>
       <x:c r="M56" t="str">
-        <x:v>Were someone to argue "Canada's GDP is 10% of the GDP of the U.S., so the average Canadian makes only 10% of what the average American makes", they would be committing the division fallacy.</x:v>
+        <x:v>People often infer that because a country is rich, any given citizen must be comfortable, skipping inequality, regional gaps, and individual circumstance.</x:v>
       </x:c>
       <x:c r="N56" t="str">
-        <x:v>If you were to suggest that, because 50% of Japanese believe in ghosts, the average Japanese is only half-certain that ghosts exist, you would be committing the division fallacy.</x:v>
+        <x:v>A popular movement, successful company, or prestigious institution can still contain weak teams, poor ideas, or underfunded units.</x:v>
       </x:c>
       <x:c r="O56" t="str"/>
       <x:c r="P56" t="str"/>
       <x:c r="Q56" t="str"/>
       <x:c r="R56" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -2744,25 +2748,25 @@
         <x:v>distribution fallacy</x:v>
       </x:c>
       <x:c r="J57" t="str">
-        <x:v>Inferences about the nature of specific individuals are based solely upon aggregate statistics collected for the group to which those individuals belong.</x:v>
+        <x:v>Occurs when statistics about a group are used to draw conclusions about particular individuals in that group.</x:v>
       </x:c>
       <x:c r="K57" t="str">
-        <x:v>Because the average German is taller than me, you won't find a German who is shorter than me.</x:v>
+        <x:v>This district has high average test scores, so the student from that district must be academically strong.</x:v>
       </x:c>
       <x:c r="L57" t="str">
-        <x:v>Averages are useful when a higher resolution of the context would be cumbersome. However, there may be some contexts where an understanding of the actual distribution is required.</x:v>
+        <x:v>Aggregate data can be useful, but it does not tell you where any one individual falls within the distribution. Group averages do not erase overlap, variation, or outliers.</x:v>
       </x:c>
       <x:c r="M57" t="str">
-        <x:v>In a part of town with many nursing homes and nursery schools, the average age may be 35. It would be a mistake, however, to then expect to see many middle-age individuals in that part of town.</x:v>
+        <x:v>Zip-code analytics, polling blocs, and demographic summaries are often treated as if they gave a direct reading of the motives or traits of each person inside the category.</x:v>
       </x:c>
       <x:c r="N57" t="str">
-        <x:v>The average income of many countries is largely uninformative since there exists a large gulf between the rich and poor.</x:v>
+        <x:v>Political commentary frequently talks as if 'suburban women,' 'young men,' or 'college voters' were internally uniform rather than broad, heterogeneous groups.</x:v>
       </x:c>
       <x:c r="O57" t="str"/>
       <x:c r="P57" t="str"/>
       <x:c r="Q57" t="str"/>
       <x:c r="R57" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -3114,21 +3118,25 @@
       <x:c r="H66" t="str"/>
       <x:c r="I66" t="str"/>
       <x:c r="J66" t="str">
-        <x:v>A degree of unwarranted necessity is placed in the conclusion based on the necessity of one or more of its premises.</x:v>
+        <x:v>Occurs when a condition that is necessary given someone's current description is treated as if it were permanently or universally necessary in the real world.</x:v>
       </x:c>
       <x:c r="K66" t="str">
-        <x:v>I'm a bachelor, and being a bachelor is necessarily being unmarried, therefore I can never marry since I need to be single.</x:v>
+        <x:v>He is unemployed now, and being unemployed means not having a job, so he cannot possibly be employed next month.</x:v>
       </x:c>
       <x:c r="L66" t="str">
-        <x:v>Something may be logically necessary due to a definition, but this necessity does not carry over into the actual world in which one can choose to change their marital status.</x:v>
-      </x:c>
-      <x:c r="M66" t="str"/>
-      <x:c r="N66" t="str"/>
+        <x:v>Some predicates are necessary only relative to a present state or definition. That necessity does not magically extend across time, possibility, or changed conditions.</x:v>
+      </x:c>
+      <x:c r="M66" t="str">
+        <x:v>People sometimes move from 'this rule currently defines the category' to 'therefore the category could never be revised or altered,' confusing present convention with fixed necessity.</x:v>
+      </x:c>
+      <x:c r="N66" t="str">
+        <x:v>In institutional debates, a temporary legal or procedural status is often spoken of as if it were an immutable fact about what can never happen.</x:v>
+      </x:c>
       <x:c r="O66" t="str"/>
       <x:c r="P66" t="str"/>
       <x:c r="Q66" t="str"/>
       <x:c r="R66" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -4553,25 +4561,25 @@
       <x:c r="H99" t="str"/>
       <x:c r="I99" t="str"/>
       <x:c r="J99" t="str">
-        <x:v>Consists of assuming that things often grouped together by tradition or culture must always be grouped that way.</x:v>
+        <x:v>Occurs when traits that are often bundled together by stereotype, tradition, or habit are treated as if they must always come as a package.</x:v>
       </x:c>
       <x:c r="K99" t="str">
-        <x:v>She's likes bowling, so she certainly drinks beer as do most other bowlers.</x:v>
+        <x:v>He is a gamer, so he must be antisocial and male.</x:v>
       </x:c>
       <x:c r="L99" t="str">
-        <x:v>This fallacy is measured in degrees. For example, you might be warranted in saying "John will probably like this book since the last book he enjoyed was also science fiction."</x:v>
+        <x:v>Some traits do cluster more often than chance would predict, but the cluster is not a logical necessity. A familiar package can make us overread what belongs together.</x:v>
       </x:c>
       <x:c r="M99" t="str">
-        <x:v>Because Judge John E. Jones III was appointed by George W. Bush, it was assumed by many that he would favor the right-leaning anti-evolutionists in the Dover trial over intelligent design. This turned out to not be the case.</x:v>
+        <x:v>Campaign and media narratives often assume that working-class, rural, religious, or college-educated identities come with one full political bundle attached.</x:v>
       </x:c>
       <x:c r="N99" t="str">
-        <x:v>Tiger Woods was a surprised to many who assumed that black golfers could never attain the skill-level of white golfers.</x:v>
+        <x:v>People frequently expect hobbies, musical taste, fashion, or ethnicity to drag a whole associated worldview behind them even when the individual breaks the pattern.</x:v>
       </x:c>
       <x:c r="O99" t="str"/>
       <x:c r="P99" t="str"/>
       <x:c r="Q99" t="str"/>
       <x:c r="R99" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -4677,25 +4685,25 @@
       <x:c r="H102" t="str"/>
       <x:c r="I102" t="str"/>
       <x:c r="J102" t="str">
-        <x:v>Occurs when an ideal of perfection is placed in contrast to a gradient of many imperfect states, implying that there are only 2 discrete categories.</x:v>
+        <x:v>Occurs when a messy range of better and worse cases is collapsed into a rigid perfect-or-failed binary.</x:v>
       </x:c>
       <x:c r="K102" t="str">
-        <x:v>I remember you once shouted in anger at your brother. You are essentially an angry person.</x:v>
+        <x:v>One factual slip means this journalist is a liar rather than merely mistaken on that point.</x:v>
       </x:c>
       <x:c r="L102" t="str">
-        <x:v>Those employing this fallacy are removing semantic resolution from the issue, and are demanding others to categorize quite disparate degrees of phenomena into only 2 categories. This is similar to semantic pixelization.</x:v>
+        <x:v>Many human traits and performances come in degrees. Treating any deviation from an ideal as proof of total failure destroys the resolution needed for fair judgment.</x:v>
       </x:c>
       <x:c r="M102" t="str">
-        <x:v>It has been questioned why, when blind-folded, people cannot walk in a straight line. It would actually be highly unusual for a person to maintain a straight line, and there is a wide range of possible degrees of accuracy between straight and highly curved. To ignore this continuum is to forfeit useful semantic resolution.</x:v>
+        <x:v>Debates about media bias, moral character, and institutional trust often assume that if a person or outlet is not perfectly objective, then it is simply propaganda.</x:v>
       </x:c>
       <x:c r="N102" t="str">
-        <x:v>Some pessimistically point to the fact that, at any given moment, there is a violent conflict somewhere in the world. They set up a artificial violent/non-violent dichotomy, then extrapolate from the existence of violence that humanity is inherently violent, ignoring the many functional and largely altruistic societies at peace around the world that world paint a more nuanced picture of humanity.</x:v>
+        <x:v>Public discussion of peace, tolerance, and fairness often ignores large improvements because some imperfection remains somewhere.</x:v>
       </x:c>
       <x:c r="O102" t="str"/>
       <x:c r="P102" t="str"/>
       <x:c r="Q102" t="str"/>
       <x:c r="R102" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -5191,25 +5199,25 @@
         <x:v>hypostatization, concretism</x:v>
       </x:c>
       <x:c r="J114" t="str">
-        <x:v>Occurs when an abstraction is treated as if it were a real event or physical entity.</x:v>
+        <x:v>Occurs when an abstraction is spoken of as if it were a concrete agent or thing in a way that misleads rather than merely using harmless metaphor.</x:v>
       </x:c>
       <x:c r="K114" t="str">
-        <x:v>The falling tree chose to flatten my new truck. So I hacked it into firewood and punished it in my wood stove.</x:v>
+        <x:v>The market decided to punish us because it was angry.</x:v>
       </x:c>
       <x:c r="L114" t="str">
-        <x:v>In the example of a falling tree "choosing" a route, intention and guilt is wrongly ascribed to the non-conscious and amoral tree. Reification is usually only a problem where linguistic rigor is required. To draw someone's attention to the "angry" clouds is no fallacy, but a perfectly good linguistic device that effectively conveys real meaning.</x:v>
+        <x:v>Metaphor can be useful shorthand, but the fallacy appears when agency, intention, or moral responsibility is attributed to an abstraction as though it literally possessed a mind of its own.</x:v>
       </x:c>
       <x:c r="M114" t="str">
-        <x:v>If you were to suggest that religion is immoral since it scares humans into behaving well, you would have committed the fallacy of reification since religion is neither a moral agent that can act immorally, nor can it have the intention to scare someone since it is not a cognitive entity.</x:v>
+        <x:v>People talk as if capitalism, democracy, the algorithm, or history itself wants, fears, rewards, or punishes, which can hide the actual network of human choices and incentives underneath.</x:v>
       </x:c>
       <x:c r="N114" t="str">
-        <x:v>If you were to claim capitalism is "evil", you would be reifying capitalism by equating it to a moral agent.</x:v>
+        <x:v>AI discussions sometimes slide from 'the model produced this output' to 'the AI wants this outcome,' smuggling in a stronger picture of agency than the evidence supports.</x:v>
       </x:c>
       <x:c r="O114" t="str"/>
       <x:c r="P114" t="str"/>
       <x:c r="Q114" t="str"/>
       <x:c r="R114" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -5810,27 +5818,25 @@
       <x:c r="H128" t="str"/>
       <x:c r="I128" t="str"/>
       <x:c r="J128" t="str">
-        <x:v>The claim that some object or idea has a purpose or necessary end point in the absence of evidence for that end point.</x:v>
+        <x:v>Occurs when a purpose, goal, or final destination is attributed to something without adequate evidence that such an end point was built into it.</x:v>
       </x:c>
       <x:c r="K128" t="str">
-        <x:v>Why would God have given us noses if he hadn't planned that we should wear glasses?</x:v>
+        <x:v>Evolution created human intelligence because nature was trying to produce minds like ours.</x:v>
       </x:c>
       <x:c r="L128" t="str">
-        <x:v>Only after the existence of an end point has been evidentially established can it serve as a foundation for other dependent concepts.</x:v>
+        <x:v>Some things really are designed for purposes, but purpose should not be assumed where it has not been shown. Processes can produce outcomes without aiming at them.</x:v>
       </x:c>
       <x:c r="M128" t="str">
-        <x:v>According to Bertrand Russell, it was once claimed that rabbits were created with white tails so they would be easy for hunters to shoot.</x:v>
+        <x:v>People often speak as if history is automatically bending toward justice, collapse, nationalism, or liberation, as though social change carried its own guaranteed destination.</x:v>
       </x:c>
       <x:c r="N128" t="str">
-        <x:v>Evolution is often misunderstood as teleological as evidenced by suggestions that there is some end-goal of evolution such as homo sapiens. Evolution might be better understood as the genetic movement of a species to better align its genetic composition to the environmental context, rather than striving towards some genetic goal independent of a environmental context.</x:v>
-      </x:c>
-      <x:c r="O128" t="str">
-        <x:v>One creationist infamously created a video purporting that the hand-shaped banana was evidence of a designer. Modern bananas have been bred by agriculturists to have the shape they do.</x:v>
-      </x:c>
+        <x:v>In technology debates, AI progress is sometimes framed as if it were inherently marching toward a single destined endpoint such as AGI rather than following contingent technical and social paths.</x:v>
+      </x:c>
+      <x:c r="O128" t="str"/>
       <x:c r="P128" t="str"/>
       <x:c r="Q128" t="str"/>
       <x:c r="R128" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="129">

</xml_diff>

<commit_message>
Modernize formal fallacy entries
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R33c940c6b5af40b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R2519e6195e644bb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R2c9b867674c44805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rca3924e12fb04b2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R0e538384e81f42a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R1800f0b848f44e66"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -479,26 +479,25 @@
       <x:c r="H6" t="str"/>
       <x:c r="I6" t="str"/>
       <x:c r="J6" t="str">
-        <x:v>Occurs when a categorical syllogism has a positive conclusion, but at least one negative premise.</x:v>
+        <x:v>Occurs when a syllogism tries to draw a positive conclusion even though one of the premises is negative in a way that cannot support that conclusion.</x:v>
       </x:c>
       <x:c r="K6" t="str">
-        <x:v>I don't eat meat. People who eat meat have no compassion. Therefore, I have compassion.</x:v>
+        <x:v>This source is not anonymous. Anonymous sources are unreliable. Therefore this source is reliable.</x:v>
       </x:c>
       <x:c r="L6" t="str">
-        <x:v>If A ⊄ B and B ⊄ C then A ⊂ C.
-This fallacy is made clear when we follow this same form and say "If I'm not a goose, and geese don't play bingo, therefore I play bingo."</x:v>
+        <x:v>Ruling something out does not automatically place it into the positive category you want. 'Not bad' does not by itself mean 'good,' and 'not that' does not by itself mean 'this.'</x:v>
       </x:c>
       <x:c r="M6" t="str">
-        <x:v>This fallacy is often a part of tribalism in which the following type of argument is implicitly made.We don't do that.
-People who do that are bad.
-Therefore, we are good.</x:v>
-      </x:c>
-      <x:c r="N6" t="str"/>
+        <x:v>Tribal arguments often move from 'we are not them' and 'they are bad' to 'therefore we are trustworthy,' even though the conclusion has not been earned.</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>Media and politics frequently treat the failure of one rival source as if it directly validated a different source that still needs its own support.</x:v>
+      </x:c>
       <x:c r="O6" t="str"/>
       <x:c r="P6" t="str"/>
       <x:c r="Q6" t="str"/>
       <x:c r="R6" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -524,27 +523,25 @@
       <x:c r="H7" t="str"/>
       <x:c r="I7" t="str"/>
       <x:c r="J7" t="str">
-        <x:v>Concluding that one logical disjunction must be false because the other disjunct is true; A or B; A; therefore not B.</x:v>
+        <x:v>Occurs when someone treats an ordinary 'or' as if it were exclusive and concludes that one option must be false because the other is true.</x:v>
       </x:c>
       <x:c r="K7" t="str">
-        <x:v>My new neighbor looked so happy, I knew he had either a girlfriend or a wife. He told me he has a wife, so I know he does not have a girlfriend.</x:v>
+        <x:v>This video is either edited or misleading. It is edited, so it cannot also be misleading.</x:v>
       </x:c>
       <x:c r="L7" t="str">
-        <x:v>P or Q
-P
-Therefore, not Q
-This fallacy is made clear when when follow this same form and say "To have a girlfriend like Tom's, you have to be either rich or famous. He's rich, so he can't be famous."
-Note that this fallacy does not hold for exclusive disjunctions where P and Q cannot both be true.</x:v>
+        <x:v>Some disjunctions are genuinely exclusive, but many are not. Two options can coexist unless the statement or context really rules that out.</x:v>
       </x:c>
       <x:c r="M7" t="str">
-        <x:v>Some politicians might argue that, to lower the deficit, we'll need to either cut programs or raise taxes, then suggest that, since they've already cut taxes, cutting programs wouldn't also contribute to alleviating the problem.</x:v>
-      </x:c>
-      <x:c r="N7" t="str"/>
+        <x:v>Budget rhetoric often suggests that because one policy tool is on the table, another cannot also matter, as if tradeoffs always come in only one-at-a-time form.</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>Public debate regularly acts as though a claim must be either emotional or strategic, either true or persuasive, either mistaken or manipulative, when in reality both descriptions may apply.</x:v>
+      </x:c>
       <x:c r="O7" t="str"/>
       <x:c r="P7" t="str"/>
       <x:c r="Q7" t="str"/>
       <x:c r="R7" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -570,25 +567,25 @@
       <x:c r="H8" t="str"/>
       <x:c r="I8" t="str"/>
       <x:c r="J8" t="str">
-        <x:v>The antecedent in a conditional is claimed to be true because the consequent is true; if A, then B; B, therefore A.</x:v>
+        <x:v>Occurs when someone reasons from 'if A, then B' and then wrongly infers A merely because B is observed.</x:v>
       </x:c>
       <x:c r="K8" t="str">
-        <x:v>Whenever it rains, people carry umbrellas. People are carrying umbrellas, so it must be raining.</x:v>
+        <x:v>If a clip is AI-generated, it may show warped hands. This clip shows warped hands, so it must be AI-generated.</x:v>
       </x:c>
       <x:c r="L8" t="str">
-        <x:v>If P, then Q
-Q
-Therefore, P.</x:v>
+        <x:v>A consequence can have many causes. Observing the result does not tell you which sufficient condition produced it.</x:v>
       </x:c>
       <x:c r="M8" t="str">
-        <x:v>If Tom says "All ducks can fly", and Bob responds "Not true. Bats can fly and they're not ducks", Bob has fallaciously affirmed the consequent of Tom's statement as if Tom had said "This animal can fly and is therefore a duck."</x:v>
-      </x:c>
-      <x:c r="N8" t="str"/>
+        <x:v>Political misinformation often treats one suspicious-looking detail as proof of a favored cause, even though many other explanations remain live.</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>Arguments about fraud, manipulation, and AI generation frequently jump from a telltale symptom to a confident diagnosis without ruling out alternatives.</x:v>
+      </x:c>
       <x:c r="O8" t="str"/>
       <x:c r="P8" t="str"/>
       <x:c r="Q8" t="str"/>
       <x:c r="R8" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2610,25 +2607,25 @@
       <x:c r="H54" t="str"/>
       <x:c r="I54" t="str"/>
       <x:c r="J54" t="str">
-        <x:v>Occurs when the consequent in an indicative conditional is claimed to be false because the antecedent is false; if A, then B; not A, therefore not B.</x:v>
+        <x:v>Occurs when someone reasons from 'if A, then B' and then wrongly infers 'not B' merely because A is absent.</x:v>
       </x:c>
       <x:c r="K54" t="str">
-        <x:v>If I were a movie star, I'd be popular. But I'm not a movie star, so I'm not popular.</x:v>
+        <x:v>If a study is peer-reviewed, it is worth taking seriously. This report is not peer-reviewed, so it is worthless.</x:v>
       </x:c>
       <x:c r="L54" t="str">
-        <x:v>If P, then Q
-Not Q
-Therefore, not P.</x:v>
+        <x:v>One route to a conclusion does not have to be the only route. The absence of one sufficient condition does not automatically remove every other possible basis.</x:v>
       </x:c>
       <x:c r="M54" t="str">
-        <x:v>Some might deny the antecedent by arguing "If you work hard, you will get a good job. Therefore, if you do not work hard you will not get a good job."</x:v>
-      </x:c>
-      <x:c r="N54" t="str"/>
+        <x:v>Debates about expertise often assume that if a source lacks one credential or prestige marker, there can be no meaningful evidence at all in what it says.</x:v>
+      </x:c>
+      <x:c r="N54" t="str">
+        <x:v>In everyday arguments, people often assume that if the ideal cause is absent, the observed effect cannot still arise through another path.</x:v>
+      </x:c>
       <x:c r="O54" t="str"/>
       <x:c r="P54" t="str"/>
       <x:c r="Q54" t="str"/>
       <x:c r="R54" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -2990,25 +2987,25 @@
       <x:c r="H63" t="str"/>
       <x:c r="I63" t="str"/>
       <x:c r="J63" t="str">
-        <x:v>Occurs when a categorical syllogism that is invalid because both of its premises are negative.</x:v>
+        <x:v>Occurs when two negative premises are used in a syllogism even though they fail to establish the positive link the conclusion requires.</x:v>
       </x:c>
       <x:c r="K63" t="str">
-        <x:v>No humans are birds. Some birds are not lawyers. Therefore some lawyers are not humans.</x:v>
+        <x:v>No journalists are judges. Some judges are not activists. Therefore some activists are not journalists.</x:v>
       </x:c>
       <x:c r="L63" t="str">
-        <x:v>Some/all As are not Bs.
-Some/all Bs are not Cs.
-Therefore, no A is C.</x:v>
+        <x:v>Two exclusions do not by themselves tell you how the remaining categories relate. Keeping groups apart is not the same as establishing a valid connection among them.</x:v>
       </x:c>
       <x:c r="M63" t="str">
-        <x:v>Another example might be "Since no republicans are democrats and some democrats are not farmers, it follows that some farmers are not republicans."</x:v>
-      </x:c>
-      <x:c r="N63" t="str"/>
+        <x:v>Identity arguments sometimes pile up statements about what two groups are not and then pretend that the missing positive relation has somehow been proved.</x:v>
+      </x:c>
+      <x:c r="N63" t="str">
+        <x:v>This form often hides inside rhetorical contrasts where speakers rely on the sound of elimination rather than a genuine logical bridge.</x:v>
+      </x:c>
       <x:c r="O63" t="str"/>
       <x:c r="P63" t="str"/>
       <x:c r="Q63" t="str"/>
       <x:c r="R63" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -3032,23 +3029,25 @@
       <x:c r="H64" t="str"/>
       <x:c r="I64" t="str"/>
       <x:c r="J64" t="str">
-        <x:v>Argues to a conclusion that implies that a class has at least one member, but without such an implication in the premises.</x:v>
+        <x:v>Occurs when a conclusion assumes that something exists even though the premises never established that any such thing exists.</x:v>
       </x:c>
       <x:c r="K64" t="str">
-        <x:v>Creatures who hide in the woods are not aggressive. Bigfoot hides in the woods. Therefore Bigfoot is not aggressive.</x:v>
+        <x:v>Every unicorn in this forest is shy. Therefore at least one unicorn in this forest is shy.</x:v>
       </x:c>
       <x:c r="L64" t="str">
-        <x:v>This fallacy can be remedied by converting the assertions to conditionals with "If ___ were ___, ...".</x:v>
+        <x:v>Universal statements can be true even when the class is empty. Talking about all members of a category does not guarantee that there are any members to begin with.</x:v>
       </x:c>
       <x:c r="M64" t="str">
-        <x:v>To post a sign saying shoplifters.</x:v>
-      </x:c>
-      <x:c r="N64" t="str"/>
+        <x:v>Arguments about 'the average user,' 'the typical elite,' or 'the real moderate voter' sometimes slip from a hypothetical category into the assumption that a concrete instance must exist.</x:v>
+      </x:c>
+      <x:c r="N64" t="str">
+        <x:v>Formal and theological debates alike often move too quickly from what would be true if something existed to the claim that it therefore does exist.</x:v>
+      </x:c>
       <x:c r="O64" t="str"/>
       <x:c r="P64" t="str"/>
       <x:c r="Q64" t="str"/>
       <x:c r="R64" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -3468,26 +3467,25 @@
       <x:c r="H74" t="str"/>
       <x:c r="I74" t="str"/>
       <x:c r="J74" t="str">
-        <x:v>A categorical syllogism that has four terms.</x:v>
+        <x:v>Occurs when a syllogism seems to use three terms but actually uses four because one term shifts meaning halfway through the argument.</x:v>
       </x:c>
       <x:c r="K74" t="str">
-        <x:v>All children like candy, and all boys are children. So, all girls like candy.</x:v>
+        <x:v>Nothing is better than open debate. A sandwich is better than nothing. Therefore a sandwich is better than open debate.</x:v>
       </x:c>
       <x:c r="L74" t="str">
-        <x:v>While we understand that all girls are also children, this fact needs to be included as an assumption for the argument to be valid.</x:v>
+        <x:v>The surface wording can make the argument sound tidy, but the hidden term shift breaks the structure. A reused word is not enough; it has to keep the same meaning.</x:v>
       </x:c>
       <x:c r="M74" t="str">
-        <x:v>Power corrupts.
-Knowledge is power.
-Therefore knowledge corrupts.
-This fallacy actually 4 terms since the term "power" as 2 different meanings.</x:v>
-      </x:c>
-      <x:c r="N74" t="str"/>
+        <x:v>Public arguments often slide between technical and ordinary meanings of words like 'theory,' 'freedom,' 'bias,' or 'intelligence,' then pretend the resulting syllogism is valid.</x:v>
+      </x:c>
+      <x:c r="N74" t="str">
+        <x:v>Because the same label can carry prestige in one context and a thinner meaning in another, term shifts often smuggle in conclusions the premises did not support.</x:v>
+      </x:c>
       <x:c r="O74" t="str"/>
       <x:c r="P74" t="str"/>
       <x:c r="Q74" t="str"/>
       <x:c r="R74" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -3827,25 +3825,25 @@
       <x:c r="H82" t="str"/>
       <x:c r="I82" t="str"/>
       <x:c r="J82" t="str">
-        <x:v>Occurs when a categorical syllogism is invalid because its major term is undistributed in the major premise but distributed in the conclusion.</x:v>
+        <x:v>Occurs when a syllogism distributes the major term in the conclusion even though the major premise never distributed it there.</x:v>
       </x:c>
       <x:c r="K82" t="str">
-        <x:v>Because all pigs like mud, and no birds are pigs, therefore no birds like mud.</x:v>
+        <x:v>All billionaires are famous. No teachers are billionaires. Therefore no teachers are famous.</x:v>
       </x:c>
       <x:c r="L82" t="str">
-        <x:v>All As are Cs.
-No Bs are As.
-Therefore, no Bs are Cs.</x:v>
+        <x:v>Excluding one group from a subset does not exclude it from the wider property attached to that subset. The conclusion reaches further than the premises license.</x:v>
       </x:c>
       <x:c r="M82" t="str">
-        <x:v>Conservapedia once had an article devoted to showing a relationship between atheism and obesity. The general idea was that most atheists are obese, and no theists are atheists, and therefore few theists are obese.</x:v>
-      </x:c>
-      <x:c r="N82" t="str"/>
+        <x:v>Stereotype arguments often move from 'all members of group A have trait B' and 'group C is not group A' to 'therefore group C lacks trait B,' which does not follow.</x:v>
+      </x:c>
+      <x:c r="N82" t="str">
+        <x:v>This pattern appears when people treat one pathway to fame, corruption, risk, or success as if it were the only pathway.</x:v>
+      </x:c>
       <x:c r="O82" t="str"/>
       <x:c r="P82" t="str"/>
       <x:c r="Q82" t="str"/>
       <x:c r="R82" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -4211,19 +4209,25 @@
       <x:c r="H91" t="str"/>
       <x:c r="I91" t="str"/>
       <x:c r="J91" t="str">
-        <x:v>Occurs when the substitution of identical designators in a true statement leads to a potentially false one.</x:v>
+        <x:v>Occurs when two names or descriptions refer to the same thing, but a belief or knowledge context blocks simple substitution and the argument ignores that.</x:v>
       </x:c>
       <x:c r="K91" t="str">
-        <x:v>Since I know who my girlfriend is, but don't know who ate all the ice cream, my girlfriend is not the person who ate the ice cream.</x:v>
-      </x:c>
-      <x:c r="L91" t="str"/>
-      <x:c r="M91" t="str"/>
-      <x:c r="N91" t="str"/>
+        <x:v>I know who my senator is, but I do not know who wrote this anonymous op-ed, so my senator could not have written it.</x:v>
+      </x:c>
+      <x:c r="L91" t="str">
+        <x:v>In ordinary factual contexts, identical referents can be substituted safely. In belief, knowledge, or perception contexts, that move can fail because the speaker's information is incomplete.</x:v>
+      </x:c>
+      <x:c r="M91" t="str">
+        <x:v>This fallacy shows up whenever people infer identity or non-identity from what someone knows, recognizes, or can name rather than from the underlying facts.</x:v>
+      </x:c>
+      <x:c r="N91" t="str">
+        <x:v>Mystery, anonymity, and pseudonym debates often slide into this mistake by assuming that not knowing a description means the object cannot be the same one known under another description.</x:v>
+      </x:c>
       <x:c r="O91" t="str"/>
       <x:c r="P91" t="str"/>
       <x:c r="Q91" t="str"/>
       <x:c r="R91" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -4381,25 +4385,25 @@
       <x:c r="H95" t="str"/>
       <x:c r="I95" t="str"/>
       <x:c r="J95" t="str">
-        <x:v>Assuming that, because a premise cannot be proven false, the premise must be true; or that, because a premise cannot be proven true, the premise must be false.</x:v>
+        <x:v>Occurs when a claim is treated as true because it has not been disproved, or false because it has not been proved.</x:v>
       </x:c>
       <x:c r="K95" t="str">
-        <x:v>Can you prove I'm not wearing an invisible hat? If you can't, I'm justified in believing I am.</x:v>
+        <x:v>No one has disproved the hidden vote-switching software, so it is reasonable to believe it exists.</x:v>
       </x:c>
       <x:c r="L95" t="str">
-        <x:v>The degree of warrant for a given proposition is the degree of evidence that favors that proposition, not the absence of evidence that would falsify the proposition. The ability to say "You can't prove I'm not right" does not mean you are warranted in believing you are right.</x:v>
+        <x:v>The rational status of a claim depends on the evidence for it, not on whether someone has managed to close every imaginable contrary possibility.</x:v>
       </x:c>
       <x:c r="M95" t="str">
-        <x:v>If someone claims that global warming is due to human activity, then justifies their position by saying "You can't prove human activity is not the cause of global warming", they have committed this fallacy.</x:v>
+        <x:v>Election, paranormal, and conspiracy claims often survive by saying 'you cannot prove it did not happen,' as if that absence of disproof supplied positive warrant.</x:v>
       </x:c>
       <x:c r="N95" t="str">
-        <x:v>In the U.S., until someone accused of a crime has been found guilty based on sufficient evidence, they are presumed innocent. This does not mean they are innocent of the crime. It is just that we start with the assumption that they are innocent until (if ever) sufficient evidence warrants our deeming them guilty.</x:v>
+        <x:v>Skeptics can also commit the reverse mistake when they treat an unproved claim as definitively false rather than merely unestablished.</x:v>
       </x:c>
       <x:c r="O95" t="str"/>
       <x:c r="P95" t="str"/>
       <x:c r="Q95" t="str"/>
       <x:c r="R95" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -5603,25 +5607,25 @@
       <x:c r="H123" t="str"/>
       <x:c r="I123" t="str"/>
       <x:c r="J123" t="str">
-        <x:v>A complex argument which loses logical cohesion somewhere in the complexity.</x:v>
+        <x:v>Occurs when an argument becomes so internally tangled that its pieces no longer form a coherent chain from premise to conclusion even though it sounds intricate.</x:v>
       </x:c>
       <x:c r="K123" t="str">
-        <x:v>If you only asked me, I would tell you the truth. But you didn't ask, so if I told you a lie you wouldn't believe it was a lie since the truth is not what you asked for.</x:v>
+        <x:v>If the story were false, fact-checkers would deny it. Because they denied it, they proved it was true, since they only deny dangerous truths.</x:v>
       </x:c>
       <x:c r="L123" t="str">
-        <x:v>This fallacy is often a composite collection of several fallacies within one argument, and is primarily limited to 1) those intentionally complicating an argument to inoculate it from criticism, and 2) those who sincerely have difficulty formulating coherent arguments with valid causal relations.</x:v>
+        <x:v>Sometimes the problem is deliberate obscurity; other times it is sincere confusion. Either way, complexity should not be mistaken for structure.</x:v>
       </x:c>
       <x:c r="M123" t="str">
-        <x:v>Immediately after my birth in 1961, both cancer rates and the nationalization of Cuban tourism increased. Because some of these cancer patients were Cuban tourists, I am obligated to build a hospital in Havana.</x:v>
+        <x:v>Conspiracy reasoning often spirals into self-sealing loops where every attempted refutation becomes fresh confirmation through an increasingly baroque chain of premises.</x:v>
       </x:c>
       <x:c r="N123" t="str">
-        <x:v>Because no one would be reading this unless they had a remote interest in logical fallacies, those on the remote island of Fiji have no interest in logical fallacies and therefore cannot read.</x:v>
+        <x:v>AI-generated argument dumps can produce this effect by chaining plausible-sounding clauses that never quite add up to a valid line of reasoning.</x:v>
       </x:c>
       <x:c r="O123" t="str"/>
       <x:c r="P123" t="str"/>
       <x:c r="Q123" t="str"/>
       <x:c r="R123" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -6168,23 +6172,25 @@
       <x:c r="H136" t="str"/>
       <x:c r="I136" t="str"/>
       <x:c r="J136" t="str">
-        <x:v>Occurs when the middle general term in a categorical syllogism is not distributed to more specific terms of the same category.</x:v>
+        <x:v>Occurs when two things are linked to the same broader category and the argument wrongly infers that one of them must therefore be the other.</x:v>
       </x:c>
       <x:c r="K136" t="str">
-        <x:v>All humans are 2-legged, and all birds are 2-legged. Therefore all humans are birds.</x:v>
+        <x:v>All conspiracy theorists distrust institutions. I distrust institutions. Therefore I am a conspiracy theorist.</x:v>
       </x:c>
       <x:c r="L136" t="str">
-        <x:v>In the example, the conclusion does not follow since it is 2-leggedness that is the larger more general category, encompassing both humans and birds, without either one of the smaller more specific categories encompassing the other. If one of the premises instead stated that all 2-legged things are birds, then the argument would be valid (but not sound).</x:v>
+        <x:v>Sharing a feature does not establish identity or class inclusion unless the shared feature actually covers the whole relevant group. A middle term can connect without unifying.</x:v>
       </x:c>
       <x:c r="M136" t="str">
-        <x:v>Young people needing social acceptance often argue to themselves in a way that might be stated "The cool wear sunglasses, and I'm wearing sunglasses. Therefore I'm one of the cool."</x:v>
-      </x:c>
-      <x:c r="N136" t="str"/>
+        <x:v>Lifestyle and identity marketing often says 'the cool do X' and 'I do X,' then slides to 'therefore I am one of the cool,' even though the shared feature is too broad.</x:v>
+      </x:c>
+      <x:c r="N136" t="str">
+        <x:v>Political commentary frequently infers that because two camps are skeptical of the same institution or support the same policy, they must belong to the same underlying movement.</x:v>
+      </x:c>
       <x:c r="O136" t="str"/>
       <x:c r="P136" t="str"/>
       <x:c r="Q136" t="str"/>
       <x:c r="R136" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="137">

</xml_diff>

<commit_message>
Complete first-pass fallacy modernization
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rca3924e12fb04b2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R0e538384e81f42a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R1800f0b848f44e66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re8e7462bef4c452b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Ra55f7425f32c4160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rca65faafd2eb41b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1875,25 +1875,25 @@
         <x:v>a dicto simpliciter ad dictum secundum quid, faulty generalization</x:v>
       </x:c>
       <x:c r="J37" t="str">
-        <x:v>An argument of the following form. Group "A" has the negative quality "x" and "a" belongs to group "A". Therefore "a" has "x".</x:v>
+        <x:v>Occurs when a negative generalization about a group is used as if it settled the character or behavior of a specific member of that group.</x:v>
       </x:c>
       <x:c r="K37" t="str">
-        <x:v>Bankers are jerks, and because my neighbor is a banker, he must be a jerk.</x:v>
+        <x:v>People in private equity only care about money, so the new board member from that industry is obviously going to gut the program.</x:v>
       </x:c>
       <x:c r="L37" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
+        <x:v>Even if a group tendency were real, it would not eliminate the need for evidence about the particular person under discussion.</x:v>
       </x:c>
       <x:c r="M37" t="str">
-        <x:v>If you learn that you have a tumor, the fact that many tumors are malignant, inoperable and fatal does not mean that you should despair since many tumors can be successfully treated. More information about the type and stage of the tumor is needed before any conclusions can be drawn about your particular tumor.</x:v>
+        <x:v>After scandals in policing, finance, or clergy, critics sometimes assume any individual in the profession personally shares the worst traits of the institution.</x:v>
       </x:c>
       <x:c r="N37" t="str">
-        <x:v>If you have been bitten by the last 3 dogs you've approached, you are warranted in being cautious about the next dog you approach in a similar context. However, 3 data points is a rather small sample size to draw any general conclusions. The fact that you have been bitten 3 times in a row many not much reflect on the general disposition of dogs, but more on the context in which you encounter them such as while you are climbing through a window to rob someone.</x:v>
+        <x:v>Online discourse often treats party label, employer, or religious affiliation as if it were enough to prove what a specific person believes or will do.</x:v>
       </x:c>
       <x:c r="O37" t="str"/>
       <x:c r="P37" t="str"/>
       <x:c r="Q37" t="str"/>
       <x:c r="R37" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -1917,21 +1917,25 @@
         <x:v>a dicto simpliciter ad dictum secundum quid, faulty generalization</x:v>
       </x:c>
       <x:c r="J38" t="str">
-        <x:v>An argument of the following form. Group "A" has the positive quality "x" and "a" belongs to group "A". Therefore "a" has "x".</x:v>
+        <x:v>Occurs when a positive generalization about a group is used as if it established the virtue or competence of a specific member of that group.</x:v>
       </x:c>
       <x:c r="K38" t="str">
-        <x:v>Bankers are nice people, and since my neighbor is a banker, he must be a nice guy.</x:v>
+        <x:v>She works for a medical charity, so she must be careful with the facts and impossible to corrupt.</x:v>
       </x:c>
       <x:c r="L38" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
-      </x:c>
-      <x:c r="M38" t="str"/>
-      <x:c r="N38" t="str"/>
+        <x:v>A flattering stereotype is still a stereotype. Group membership can create a first impression, but it does not establish the individual's actual record.</x:v>
+      </x:c>
+      <x:c r="M38" t="str">
+        <x:v>Prestige effects often lead audiences to assume that anyone from a famous university or respected nonprofit is trustworthy even outside their area of expertise.</x:v>
+      </x:c>
+      <x:c r="N38" t="str">
+        <x:v>Voters sometimes infer that a candidate from a reform organization must be personally honest before examining the candidate's own conduct.</x:v>
+      </x:c>
       <x:c r="O38" t="str"/>
       <x:c r="P38" t="str"/>
       <x:c r="Q38" t="str"/>
       <x:c r="R38" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2095,25 +2099,25 @@
         <x:v>chicken, the egg problem</x:v>
       </x:c>
       <x:c r="J42" t="str">
-        <x:v>Occurs when the consequence of the phenomenon is said to be an inescapable cause of the phenomenon when the truth may be otherwise.</x:v>
+        <x:v>Occurs when a feedback loop is treated as if it fully explains, proves, or justifies a result, even though the loop may be contingent, breakable, or not sufficient for the claimed conclusion.</x:v>
       </x:c>
       <x:c r="K42" t="str">
-        <x:v>My music CD is not popular because people are not listening to it. And people are not listening to it because it is not popular. If they would only listen to it, it would become popular.</x:v>
+        <x:v>The app is not popular because nobody uses it, and nobody uses it because it is not popular, so if people would just use it once it would obviously become a hit.</x:v>
       </x:c>
       <x:c r="L42" t="str">
-        <x:v>Note that the fallacy is not in identifying actual causal circularity, but in claiming that the circularity is unavoidable when it is not, or in claiming that the circularity validates the truthfulness of one of the premises. It may not be the case that your music CD would become popular even were there some way possible to get people to listen to it. Actual evidence will have to be introduced to show that the circularity is indeed vicious, and that the removal of the circularity would actually result in what the assumption claims.</x:v>
+        <x:v>Circular dynamics can be real, but identifying a loop does not show that the loop is unstoppable or that breaking one link would guarantee the hoped-for outcome. Further evidence is still needed.</x:v>
       </x:c>
       <x:c r="M42" t="str">
-        <x:v>The nuclear arms race of the 20th century was based in part on the assumption that the other side would actually use their weapons should they ever gain a significant advantage in the race, an assumption that may not have been accurate.</x:v>
+        <x:v>Job markets sometimes create genuine experience loops, but it is still a mistake to assume that every applicant locked out by the loop would necessarily succeed if only one employer made an exception.</x:v>
       </x:c>
       <x:c r="N42" t="str">
-        <x:v>An argument against evolution has been the proverbial chicken-or-the-egg problem in which it is suggested that the chicken is dependent on a prior egg, and an egg is dependent on a prior chicken. Evolutionary biologists believed both evolved jointly just as an embryo jointly develops its interdependent heart and brain.</x:v>
+        <x:v>Commentators often say a platform is influential because everyone talks about it and everyone talks about it because it is influential, using the loop itself as if it settled the argument.</x:v>
       </x:c>
       <x:c r="O42" t="str"/>
       <x:c r="P42" t="str"/>
       <x:c r="Q42" t="str"/>
       <x:c r="R42" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2225,19 +2229,25 @@
       <x:c r="H45" t="str"/>
       <x:c r="I45" t="str"/>
       <x:c r="J45" t="str">
-        <x:v>The assumption that an outcome simultaneously satisfying multiple conditions is more probable than an outcome satisfying fewer of those same conditions.</x:v>
+        <x:v>Occurs when a more detailed scenario is treated as more probable than a less detailed scenario that already contains it.</x:v>
       </x:c>
       <x:c r="K45" t="str">
-        <x:v>Because Susan is young, it is more probable that she is both a student and unmarried than that she is merely a student.</x:v>
-      </x:c>
-      <x:c r="L45" t="str"/>
-      <x:c r="M45" t="str"/>
-      <x:c r="N45" t="str"/>
+        <x:v>Because the candidate is young and progressive, it is more likely that she is both a climate activist and a vegan than that she is simply a climate activist.</x:v>
+      </x:c>
+      <x:c r="L45" t="str">
+        <x:v>Adding conditions never makes a claim more probable than a broader version of that same claim. Extra detail can make a story feel more representative while making it statistically less likely.</x:v>
+      </x:c>
+      <x:c r="M45" t="str">
+        <x:v>Political profiling often mistakes a vivid stereotype for probability, assuming that a person matching one trait is more likely to match an even narrower bundle of traits as well.</x:v>
+      </x:c>
+      <x:c r="N45" t="str">
+        <x:v>AI narratives sometimes suggest that because a model appears articulate, it is more likely to be both highly capable and aligned than merely capable, even though the conjunction is narrower.</x:v>
+      </x:c>
       <x:c r="O45" t="str"/>
       <x:c r="P45" t="str"/>
       <x:c r="Q45" t="str"/>
       <x:c r="R45" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -2651,25 +2661,25 @@
       </x:c>
       <x:c r="I55" t="str"/>
       <x:c r="J55" t="str">
-        <x:v>Occurs when attempts are made at introducing alternatives where none exist.</x:v>
+        <x:v>Occurs when one side of a genuine contrast is denied or redefined so the opposing term has no place to apply.</x:v>
       </x:c>
       <x:c r="K55" t="str">
-        <x:v>My girlfriend wanted to know whether I had cheated on her. I told her that perhaps it was impossible to have cheated on her since if I had cheated, it would mean we never really had a relationship to cheat on.</x:v>
+        <x:v>If the relationship was strong enough to survive it, then it was not really cheating, because real cheating would have ended the relationship.</x:v>
       </x:c>
       <x:c r="L55" t="str">
-        <x:v>This fallacy is the converse of the false dilemma.</x:v>
+        <x:v>Some concepts only make sense against their correlative opposite. Erasing the contrast does not answer the accusation; it changes the meaning of the term.</x:v>
       </x:c>
       <x:c r="M55" t="str">
-        <x:v>Theists commonly claim their particular god becomes so angry over the very first offense a human commits, that he immediately condemns that human to eternal torment. They then also claim that same god is "patient" and "loving" towards humans. If you have a god invariably and continuously committing impatient acts, you don't have a patient god.</x:v>
+        <x:v>Public arguments sometimes say a decision cannot count as censorship unless it was total state control, effectively denying any middle range where the term usefully applies.</x:v>
       </x:c>
       <x:c r="N55" t="str">
-        <x:v>Telling your date "I'm in a complicated relationship" is not an answer to their question "Are you married?" and is denying the correlative.</x:v>
+        <x:v>Debates about betrayal, fraud, or coercion often narrow the term so drastically that almost no real case can qualify.</x:v>
       </x:c>
       <x:c r="O55" t="str"/>
       <x:c r="P55" t="str"/>
       <x:c r="Q55" t="str"/>
       <x:c r="R55" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2907,21 +2917,25 @@
       <x:c r="H61" t="str"/>
       <x:c r="I61" t="str"/>
       <x:c r="J61" t="str">
-        <x:v>In which a speaker will use a general definition of a term to denote a specific insinuation.</x:v>
+        <x:v>Occurs when a broad or harmless sense of a word is used to insinuate a narrower, stronger, or more loaded sense of the same word.</x:v>
       </x:c>
       <x:c r="K61" t="str">
-        <x:v>My mother said that ice cream was good, but it maliciously fell on my shoe.</x:v>
+        <x:v>The chatbot says it 'understands' the question, so it must understand it in the full human sense.</x:v>
       </x:c>
       <x:c r="L61" t="str">
-        <x:v>This example equivocates between "good" meaning "of positive value" and "good" meaning "morally upright".</x:v>
-      </x:c>
-      <x:c r="M61" t="str"/>
-      <x:c r="N61" t="str"/>
+        <x:v>The argument trades on the prestige or emotional force of the stronger meaning while relying on the thinner meaning when challenged.</x:v>
+      </x:c>
+      <x:c r="M61" t="str">
+        <x:v>Public arguments about censorship often slide from the general fact that content was moderated to the much stronger charge that it was censored in the same sense as state suppression.</x:v>
+      </x:c>
+      <x:c r="N61" t="str">
+        <x:v>AI marketing repeatedly benefits from equivocation between technical terms such as 'learn,' 'reason,' or 'understand' and their thicker human meanings.</x:v>
+      </x:c>
       <x:c r="O61" t="str"/>
       <x:c r="P61" t="str"/>
       <x:c r="Q61" t="str"/>
       <x:c r="R61" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -2945,25 +2959,25 @@
       <x:c r="H62" t="str"/>
       <x:c r="I62" t="str"/>
       <x:c r="J62" t="str">
-        <x:v>Occurs when it is argued that the original or historical meaning of a word or phrase is necessarily similar to its actual present-day meaning.</x:v>
+        <x:v>Occurs when a word's original or historical meaning is treated as if it controlled the word's present meaning.</x:v>
       </x:c>
       <x:c r="K62" t="str">
-        <x:v>Because "gay" meant "happy" in the past, you can't call homosexuals "gay" unless they are happy.</x:v>
+        <x:v>Because 'literally' once had a narrower sense, any modern emphatic use must be simply wrong.</x:v>
       </x:c>
       <x:c r="L62" t="str">
-        <x:v>Language inevitably changes. To be understood, a participant in the game of communication in any language will need to employ the language in the way it is currently conventionally used. Words are merely tools to convey concepts. When certain terms fail due to the speaker deviating from their conventional usage, the speaker, instead of demanding the denotation associated with the origin of the term, ought to either choose other terms that more clearly convey their ideas to the language community, or stipulate a provisional definition of the term. Words themselves contain no meaning other than what the language community has granted them.</x:v>
+        <x:v>Words change through use. Present meaning is set by current linguistic convention, not by the oldest recoverable ancestor of the term.</x:v>
       </x:c>
       <x:c r="M62" t="str">
-        <x:v>In recent years, there has been much wrangling over what the meaning of "theist", "deist", "atheist" and "agnostic" actually mean. The answer is, when terms become as hotly debated as these are, they have lost their meaning. It is difficult for concepts as nuanced as these are, to find a single term that accurately captures its full meaning. Instead of demanding others accept your own understanding or the historical meaning of a particular term, give a longer more nuanced explanation of your position. The convenience of a shorter term does not count for much if meaning is sacrificed.</x:v>
+        <x:v>Culture-war and identity debates often turn into fights over what labels 'really mean' based on older usage rather than on how the community currently uses them.</x:v>
       </x:c>
       <x:c r="N62" t="str">
-        <x:v>Some have argued that the "n" word originally came from the Latin "niger", meaning "black", and therefore is not an offensive term. This completely ignores the conventional meaning it has today, and it is within convention that meaning is created. On the other side of this issue you have people attempting to remove the "n" word from Mark Twain books, perhaps not understanding that the term was not used disparagingly by all in that era. Negatively connoted terms can be salvaged by a linguistic community as was the term "queer" through the efforts of the gay community.</x:v>
+        <x:v>People sometimes defend or condemn a term by appealing to its root language while ignoring the fact that social meaning has moved far beyond the origin.</x:v>
       </x:c>
       <x:c r="O62" t="str"/>
       <x:c r="P62" t="str"/>
       <x:c r="Q62" t="str"/>
       <x:c r="R62" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -3425,25 +3439,25 @@
       <x:c r="H73" t="str"/>
       <x:c r="I73" t="str"/>
       <x:c r="J73" t="str">
-        <x:v>An attempt to disallow an assumption introduced for the sake of argument because it is not actually believed.</x:v>
+        <x:v>Occurs when a hypothetical premise is rejected simply because the speaker does not actually believe it.</x:v>
       </x:c>
       <x:c r="K73" t="str">
-        <x:v>Your argument that Santa is not real because he would need to fly his sleigh at impossible speeds on Christmas Eve is not valid since you don't even believe in Santa.</x:v>
+        <x:v>You say that even if the policy achieved its stated goal it would still be too costly, but that objection fails because you do not really believe the policy would work.</x:v>
       </x:c>
       <x:c r="L73" t="str">
-        <x:v>This fallacy is often used in response to an "argumentum ad absurdum" in which assumptions are granted for the sake of argument to demonstrate that they lead to an incoherency. To plug an assumption into a argument to show the illogicality of that argument does not require an epistemic commitment to the assumption.</x:v>
+        <x:v>Reasoning from an assumption to test its implications is not the same as endorsing the assumption.</x:v>
       </x:c>
       <x:c r="M73" t="str">
-        <x:v>Some atheists argue that "any god that is both omnipotent and omniscient would not allow evil into the world." When theists dismiss this or a similar argument by saying "you don't believe in god, so you can't use the notion of god in your assumptions", they commit the fallacy of denying a hypothetical.</x:v>
+        <x:v>Reductio arguments in theology, AI, and politics are often misread as confessions rather than as tests of what would follow if the other side's claim were granted.</x:v>
       </x:c>
       <x:c r="N73" t="str">
-        <x:v>To argue "If Bigfoot were real, physical evidence would have turned up by now" carries no epistemic commitment to the existence of Bigfoot.</x:v>
+        <x:v>Debates stall when a conditional claim such as 'even if you are right, the consequence would still be unacceptable' is treated as if it were a statement of belief.</x:v>
       </x:c>
       <x:c r="O73" t="str"/>
       <x:c r="P73" t="str"/>
       <x:c r="Q73" t="str"/>
       <x:c r="R73" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -3513,25 +3527,25 @@
         <x:v>monte carlo fallacy, hot hand fallacy</x:v>
       </x:c>
       <x:c r="J75" t="str">
-        <x:v>The incorrect belief that the likelihood of a random event can be affected by or predicted from other, independent events.</x:v>
+        <x:v>Occurs when someone thinks past outcomes of independent events make a future independent outcome more or less likely than it really is.</x:v>
       </x:c>
       <x:c r="K75" t="str">
-        <x:v>The coin flip has resulted in 5 "heads" in a row. I'm overdue for a "tails".</x:v>
+        <x:v>The coin has landed heads five times in a row, so tails is due next.</x:v>
       </x:c>
       <x:c r="L75" t="str">
-        <x:v>True randomness will contain patches of what looks like uniformity to minds highly prone to extract patterns. The converse of the gambler's fallacy is the hot hand fallacy in which a winning steak is irrationally expected to continue.</x:v>
+        <x:v>Random sequences naturally contain streaks. When the events are truly independent, the next event does not remember the last one.</x:v>
       </x:c>
       <x:c r="M75" t="str">
-        <x:v>People often irrationally suppose that their 50th international flight is much more likely to end in tragedy than their 1st international flight. All things being equal, the risk is the same for every international flight.</x:v>
+        <x:v>People sometimes feel that after many routine flights or medical screenings in a row, a disaster or diagnosis is somehow 'due,' even though independent risks do not balance themselves that way.</x:v>
       </x:c>
       <x:c r="N75" t="str">
-        <x:v>For most gambling games, the chances of winning or losing the same amount remains constant with each game played. However, if coins are accumulating in a machine that must eventually pay out, there is an increased chance of winning with each play.</x:v>
+        <x:v>In gambling and investing language, talk of a roulette table or slot machine being 'ready to pay out' often confuses a streaky pattern with a real shift in odds.</x:v>
       </x:c>
       <x:c r="O75" t="str"/>
       <x:c r="P75" t="str"/>
       <x:c r="Q75" t="str"/>
       <x:c r="R75" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -3649,23 +3663,25 @@
       <x:c r="H78" t="str"/>
       <x:c r="I78" t="str"/>
       <x:c r="J78" t="str">
-        <x:v>Assuming that decision makers of the past viewed events from the same perspective and had the same information as those subsequently analyzing the decision.</x:v>
+        <x:v>Occurs when people in the past are judged as if they had the same information, background assumptions, and hindsight available to later observers.</x:v>
       </x:c>
       <x:c r="K78" t="str">
-        <x:v>If I had lived in medieval times, I would certainly not have thought the sun circled the earth as did all the other fools!</x:v>
+        <x:v>Anyone living in 2007 should have seen the financial crash coming exactly as we see it now.</x:v>
       </x:c>
       <x:c r="L78" t="str">
-        <x:v>We often do not appreciate the strength of societal influence on our belief systems.</x:v>
+        <x:v>Hindsight compresses uncertainty and highlights the clues that mattered. Real historical agents were working inside a noisier, more limited information environment.</x:v>
       </x:c>
       <x:c r="M78" t="str">
-        <x:v>Most people would like to think they would have not accepted slavery and other common practices we now consider barbaric had they lived a thousand years ago.</x:v>
-      </x:c>
-      <x:c r="N78" t="str"/>
+        <x:v>People often imagine they would easily have rejected past medical myths, empires, or moral blind spots, underestimating how strongly institutions and available evidence shape belief.</x:v>
+      </x:c>
+      <x:c r="N78" t="str">
+        <x:v>Post-crisis commentary regularly rewrites messy contingencies into obvious warning signs that were supposedly plain to everyone at the time.</x:v>
+      </x:c>
       <x:c r="O78" t="str"/>
       <x:c r="P78" t="str"/>
       <x:c r="Q78" t="str"/>
       <x:c r="R78" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -3691,23 +3707,25 @@
       <x:c r="H79" t="str"/>
       <x:c r="I79" t="str"/>
       <x:c r="J79" t="str">
-        <x:v>Occurs when a lower level of perception is introduced to explain perception at a higher level, then explains the lower level by invoking the very terms of perception in question.</x:v>
+        <x:v>Occurs when a mind-like inner observer is smuggled in to explain mind-like abilities, thereby postponing rather than solving the explanation.</x:v>
       </x:c>
       <x:c r="K79" t="str">
-        <x:v>Our brains see a face when light from that face enters our eyes, is passed to our neurons, and the face is finally recognized by our neurons.</x:v>
+        <x:v>Vision works because the brain forms an internal picture and then an inner observer looks at that picture.</x:v>
       </x:c>
       <x:c r="L79" t="str">
-        <x:v>To explain sight by saying our neurons "see" is to only add another seeing entity which must itself have a deeper brain that "sees", thus leading to an infinite regress.</x:v>
+        <x:v>If the inner observer can already do the job, the original explanatory problem just reappears one level down.</x:v>
       </x:c>
       <x:c r="M79" t="str">
-        <x:v>If someone were to argue that our brains make moral decisions by passing the relevant data to our soul which, in turn, makes the decision for the brain, then this simply defers the explanation of the concept of moral decision-making from the brain to the soul, demanding yet another explanation; how the soul makes moral decisions.</x:v>
-      </x:c>
-      <x:c r="N79" t="str"/>
+        <x:v>Popular neuroscience writing sometimes says that the brain 'decides' or a memory center 'knows' in ways that merely rename the puzzle rather than explain it.</x:v>
+      </x:c>
+      <x:c r="N79" t="str">
+        <x:v>Criticism of AI can do something similar when it assumes a hidden module inside the system literally understands the output in the same way a person would.</x:v>
+      </x:c>
       <x:c r="O79" t="str"/>
       <x:c r="P79" t="str"/>
       <x:c r="Q79" t="str"/>
       <x:c r="R79" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -3735,31 +3753,25 @@
         <x:v>appeal to law</x:v>
       </x:c>
       <x:c r="J80" t="str">
-        <x:v>Occurs when a human law, categorization, definition or judgment is assumed to supersede objective fact.</x:v>
+        <x:v>Occurs when a human classification, rule, or label is treated as if it automatically determined the underlying fact or moral status.</x:v>
       </x:c>
       <x:c r="K80" t="str">
-        <x:v>Because there is a law against chewing gum on Wednesdays, it is immoral to chew gum on Wednesdays.</x:v>
+        <x:v>The platform's policy now defines this claim as misinformation, so it became false the moment the label was applied.</x:v>
       </x:c>
       <x:c r="L80" t="str">
-        <x:v>A law against chewing gum on Wednesdays does not suddenly make the act immoral. If it was not immoral prior to a law forbidding it, why would a human law make it so?</x:v>
+        <x:v>Institutional labels can matter legally or practically, but they do not by themselves create truth, value, or natural kinds.</x:v>
       </x:c>
       <x:c r="M80" t="str">
-        <x:v>Some argue that the use of recreational drugs is immoral by virtue of there existing a human-authored law forbidding their usage.</x:v>
+        <x:v>Markets and media often confuse approved, certified, or official with true, safe, or just.</x:v>
       </x:c>
       <x:c r="N80" t="str">
-        <x:v>Quite regularly, a coroner mistakenly declares someone dead, only to have them revive. In these cases, you'll often have family members claiming that it was a miracle that the patient did the impossible and rose from the "dead". As medicine advances, we can expect the current human definition of "death" pushed back to reflect the ever-increasing period within which resuscitation is possible.</x:v>
-      </x:c>
-      <x:c r="O80" t="str">
-        <x:v>Frequently, the dictionary definition of a term is invoked as the final authority on the way that term should be used. Clearly the writers of dictionaries assessed the conventional usage of words to formulate their entries. It is convention, not a human-made dictionary, that is the final authority on the denotation of a particular term. The only other option is to agree upon a stipulated definition of a term before engaging in dialog.</x:v>
-      </x:c>
-      <x:c r="P80" t="str">
-        <x:v>Prior to the word "deconversion" becoming mainstream, there were arguments by some theists that, because the word was not found in a dictionary, the concept it denoted was illegitimate.</x:v>
-      </x:c>
-      <x:c r="Q80" t="str">
-        <x:v>When identifying a flaw in your opponent's thinking, there is often the tendency to invoke the "official" name of that fallacy, and hurl the name at your opponent and/or the audience hoping the poison you deem that fallacy to possess will invalidate your opponent's position. At times this is valid; if the fallacy is a formal fallacy, and your opponent's position is fully contingent upon the argument with the fallacy, then you have indeed defeated their position. However, fallacies are collected and named by humans, and many fallacies are not discretely fallacious; they fall on a continuum between rationality and error. It is, therefore, usually much more productive to spend the necessary time explaining why their argument is fallacious rather than calling it by name and looking with mock surprise at your "irrational" opponent (though there may be times where this may accomplish your agenda). This site is not the ultimate authority on logical fallacies, but is merely a tool.</x:v>
-      </x:c>
+        <x:v>Political rhetoric often treats whatever a legislature recognizes or forbids as automatically morally right or wrong.</x:v>
+      </x:c>
+      <x:c r="O80" t="str"/>
+      <x:c r="P80" t="str"/>
+      <x:c r="Q80" t="str"/>
       <x:c r="R80" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -3865,25 +3877,25 @@
       <x:c r="H83" t="str"/>
       <x:c r="I83" t="str"/>
       <x:c r="J83" t="str">
-        <x:v>Occurs when every possible outcome is predicted by a theory, thereby rendering it either redundant to what is materially expected or non-existent.</x:v>
+        <x:v>Occurs when a view is framed so every possible outcome fits it equally well, leaving no meaningful room for the claim to fail.</x:v>
       </x:c>
       <x:c r="K83" t="str">
-        <x:v>We have only blurry photo evidence for the existence of alien space ships, but that's only because the aliens have technology that prevent our cameras from functioning properly.</x:v>
+        <x:v>If the forecast comes true, the psychic was right; if it fails, the warning changed the future, which also proves the psychic was right.</x:v>
       </x:c>
       <x:c r="L83" t="str">
-        <x:v>This fallacy is similar to the suppressed correlative.</x:v>
+        <x:v>A claim that survives every observation unchanged may be emotionally resilient, but it has surrendered explanatory power.</x:v>
       </x:c>
       <x:c r="M83" t="str">
-        <x:v>Some theists claim that their particular god answers prayer, but there is no possible outcome that does not fall within their definition of answered prayer. This makes their god equivalent to material cause and effect at best, but more probably non-existent.</x:v>
+        <x:v>Conspiracy systems often explain both the presence and the absence of evidence as confirmation.</x:v>
       </x:c>
       <x:c r="N83" t="str">
-        <x:v>Some atheists claim that," either you're an atheist or you're not. Make up your mind." This implies that absolute evidence is available for an absolute decision one way or the other. There is a smooth gradient of evidence on the question of a god, and therefore a justified belief will often necessarily fall somewhere on that gradient rather than on a discrete pole of belief or disbelief. This does not, of course, hold true for disbelief in gods that are logically impossible.</x:v>
+        <x:v>Some technology hype frames both success and failure as proof that general intelligence is just around the corner.</x:v>
       </x:c>
       <x:c r="O83" t="str"/>
       <x:c r="P83" t="str"/>
       <x:c r="Q83" t="str"/>
       <x:c r="R83" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -3951,23 +3963,25 @@
       <x:c r="H85" t="str"/>
       <x:c r="I85" t="str"/>
       <x:c r="J85" t="str">
-        <x:v>Occurs when complex nodes of comparison are used that make it falsely appear as if a complete comparison has been made.</x:v>
+        <x:v>Occurs when different comparison targets are used across different dimensions to create the illusion of one all-around winner.</x:v>
       </x:c>
       <x:c r="K85" t="str">
-        <x:v>My son Arthur runs faster than Thomas, gets higher grades than George, and plays piano better than William. He's definitely the most talented boy.</x:v>
+        <x:v>This laptop is cheaper than Brand A, lighter than Brand B, and faster than Brand C, so it is plainly the best laptop on the market.</x:v>
       </x:c>
       <x:c r="L85" t="str">
-        <x:v>This is a common fallacy employed by advertizers who compare their product against the least attractive competing product for each particular feature.</x:v>
+        <x:v>A complete comparison needs a consistent baseline or a transparent weighting of tradeoffs, not a collage of unrelated best cases.</x:v>
       </x:c>
       <x:c r="M85" t="str">
-        <x:v>If you claim your English skills are better than those of Tom and Andrew since Tom can't spell and and Andrew has a low vocabulary, you are committing the inconsistent comparison fallacy since you are simply cherry-picking those skills that favor you in a complex matrix of skills, and there may be other possible relevant measures of English for which you may be weaker than both Tom and Andrew.</x:v>
-      </x:c>
-      <x:c r="N85" t="str"/>
+        <x:v>Consumer ads often compare each feature against whichever rival looks weakest on that feature, then announce overall superiority.</x:v>
+      </x:c>
+      <x:c r="N85" t="str">
+        <x:v>Campaign brag sheets sometimes do the same by mixing job growth, crime, housing, and graduation metrics against different jurisdictions and different years.</x:v>
+      </x:c>
       <x:c r="O85" t="str"/>
       <x:c r="P85" t="str"/>
       <x:c r="Q85" t="str"/>
       <x:c r="R85" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -3993,25 +4007,25 @@
       <x:c r="H86" t="str"/>
       <x:c r="I86" t="str"/>
       <x:c r="J86" t="str">
-        <x:v>The assumption that the meaning intended by an author of a concept is not relevant to the understanding of that concept.</x:v>
+        <x:v>Occurs when the creator's intended meaning is treated as irrelevant in contexts where that intention is actually important to understanding the work or statement.</x:v>
       </x:c>
       <x:c r="K86" t="str">
-        <x:v>We ought to interpret "right to bear arms" within the context of our own time, and ignore the intent of the authors of the phrase.</x:v>
+        <x:v>The author says the essay was satirical, but we should ignore that completely and read it only through our own current assumptions.</x:v>
       </x:c>
       <x:c r="L86" t="str">
-        <x:v>Sometimes the evidence for the author's intentions is not in the actual literature, but must be extracted from other sources such as personal letters and notes.</x:v>
+        <x:v>Authorial intent is not always the only thing that matters, but it is often part of the evidence. Declaring it irrelevant by default can flatten interpretation into projection.</x:v>
       </x:c>
       <x:c r="M86" t="str">
-        <x:v>Some claim that Einstein was a theist based on some of his statements referring to "God". A more careful examination of his personal correspondence seems to suggest that he was, at most, a deist.</x:v>
+        <x:v>Debates over constitutional language, literature, and political slogans often swing too far toward present-day interpretation while discarding what the author or framers were trying to do.</x:v>
       </x:c>
       <x:c r="N86" t="str">
-        <x:v>Some might suggest that Mark Twain's use of the "n" word belies the author's racism, not taking into consideration the more benign use of the term in that era, nor any literary device Twain might have been employing.</x:v>
+        <x:v>Online arguments about memes, jokes, and clips frequently ignore context and stated intent altogether, then treat the most inflammatory possible reading as the only serious one.</x:v>
       </x:c>
       <x:c r="O86" t="str"/>
       <x:c r="P86" t="str"/>
       <x:c r="Q86" t="str"/>
       <x:c r="R86" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -4037,25 +4051,25 @@
         <x:v>isolated ought</x:v>
       </x:c>
       <x:c r="J87" t="str">
-        <x:v>The inappropriate inference that, because something is a particular way, it ought to be that way.</x:v>
+        <x:v>Occurs when a descriptive claim about what is common, natural, or actual is treated as if it directly established what ought to be done.</x:v>
       </x:c>
       <x:c r="K87" t="str">
-        <x:v>Nearly all humans wear clothing in public, so it is immoral not to.</x:v>
+        <x:v>Most companies monitor workers in some form now, so employees ought to accept constant tracking as normal.</x:v>
       </x:c>
       <x:c r="L87" t="str">
-        <x:v>Any "ought" ought to be accompanied by an "if" if it is to have any meaning. For example, you can tell your friend he ought to hurry if he wants to catch the bus, but an "ought" isolated from an "if" carries no meaning. Even a statement such as "You ought to listen to your parents" carries an implicit "if". If you do as they say, you'll avoid undesirable consequences. Another example is in the context of a game of chess. You ought not cheat in chess because it is socially unacceptable; i.e., if you want to maintain social respect. Even religious-based moral "oughts" contain implicit "if"s as in "You ought not lie if you want to please God and avoid eternal torment." "Ought"s cannot be divorced from "if"s.
-"In every system of morality, which I have hitherto met with, I have always remark'd, that the author proceeds for some time in the ordinary ways of reasoning, and establishes the being of a God, or makes observations concerning human affairs; when all of a sudden I am surpriz'd to find, that instead of the usual copulations of propositions, is, and is not, I meet with no proposition that is not connected with an ought, or an ought not. This change is imperceptible; but is however, of the last consequence. For as this ought, or ought not, expresses some new relation or affirmation, 'tis necessary that it shou'd be observ'd and explain'd; and at the same time that a reason should be given; for what seems altogether inconceivable, how this new relation can be a deduction from others, which are entirely different from it."
-David Hume in Treatise of Human Nature.</x:v>
+        <x:v>An ought needs a normative premise about goals, duties, or values. Facts alone do not generate that extra step.</x:v>
       </x:c>
       <x:c r="M87" t="str">
-        <x:v>Ayn Rand argued that one ought to act in a way consistent with one's own rational self-interests. The implicit "if" is presumably "if you want to live a long and happy life." Yet it is never explained why a life of altruism cannot also lead to a long and happy life, and why it ought to be replaced by a more egoistic existence.</x:v>
-      </x:c>
-      <x:c r="N87" t="str"/>
+        <x:v>Arguments about gender, family, and competition often slide from claims about what is common in nature to claims about what is therefore morally required.</x:v>
+      </x:c>
+      <x:c r="N87" t="str">
+        <x:v>Workplace norms are regularly defended by saying they are simply how the market works, even when the moral question is precisely whether the market should work that way.</x:v>
+      </x:c>
       <x:c r="O87" t="str"/>
       <x:c r="P87" t="str"/>
       <x:c r="Q87" t="str"/>
       <x:c r="R87" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -4121,29 +4135,25 @@
       <x:c r="H89" t="str"/>
       <x:c r="I89" t="str"/>
       <x:c r="J89" t="str">
-        <x:v>The assumption that a phenomenon functions linearly, overlooking important factors that produce non-linearity.</x:v>
+        <x:v>Occurs when someone assumes that doubling the input will double the output even though the system has thresholds, saturation, feedback loops, or diminishing returns.</x:v>
       </x:c>
       <x:c r="K89" t="str">
-        <x:v>The mortality rate of cats falling 20 stories will be double that of cats falling 10 stories.</x:v>
+        <x:v>One dose gave a modest result, so taking twice as much should produce twice the benefit.</x:v>
       </x:c>
       <x:c r="L89" t="str">
-        <x:v>The mortality rate for cats falling from 10 stories may be lower than for those falling from 20 due to several non-linear factors including non-linear acceleration and terminal velocity, and the non-linear time for a cat to turn itself upright and relax.</x:v>
+        <x:v>Many real systems change slowly at first, then rapidly, then plateau, or even reverse after a threshold.</x:v>
       </x:c>
       <x:c r="M89" t="str">
-        <x:v>To suggest that a person drinking 10 alcoholic drinks will be half as impaired as a person who has had 5 alcoholic drinks is to fail to understand many possible non-linear factors.</x:v>
+        <x:v>Growth forecasts for social platforms often assume audience reach will keep scaling smoothly even after attention markets saturate.</x:v>
       </x:c>
       <x:c r="N89" t="str">
-        <x:v>Spending twice the current budget on education will probably not double the test scores of students.</x:v>
-      </x:c>
-      <x:c r="O89" t="str">
-        <x:v>Having twice the income of your neighbor will probably not make you twice as happy.</x:v>
-      </x:c>
-      <x:c r="P89" t="str">
-        <x:v>It's very seldom that drinking a $200 bottle of wine results in 10 times the pleasure of drinking a $20 bottle of wine due to the law of diminishing returns.</x:v>
-      </x:c>
+        <x:v>Policy debates about climate, housing, and healthcare frequently ignore the non-linear effects of bottlenecks, incentives, and behavioral feedback.</x:v>
+      </x:c>
+      <x:c r="O89" t="str"/>
+      <x:c r="P89" t="str"/>
       <x:c r="Q89" t="str"/>
       <x:c r="R89" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -4523,25 +4533,25 @@
         <x:v>hasty generalization</x:v>
       </x:c>
       <x:c r="J98" t="str">
-        <x:v>A generalization that is coupled with qualifications so restrictive that the generalization is essentially impotent.</x:v>
+        <x:v>Occurs when a general principle is padded with so many exceptions that it no longer guides action or says much of substance.</x:v>
       </x:c>
       <x:c r="K98" t="str">
-        <x:v>I'm the type of man who always pays for my date's dinner...except in the case where she want to go somewhere other than KFC.</x:v>
+        <x:v>I believe in free expression, except when the speech is offensive, politically costly, factually shaky, socially awkward, or risky to my side.</x:v>
       </x:c>
       <x:c r="L98" t="str">
-        <x:v>An overwhelming exception is based on an accurate generalization, but is coupled with so many qualifications or such extreme qualifications that the generalization is rendered anemic and meaningless.</x:v>
+        <x:v>A principle can have limits, but if the exceptions swallow the rule, the apparent commitment becomes mostly decorative.</x:v>
       </x:c>
       <x:c r="M98" t="str">
-        <x:v>Some theists argue that their god is patient...except for whenever someone sins...at which point the offender is deemed worthy of eternal torture by a now wrathful god...and everyone regularly sins.</x:v>
+        <x:v>Public commitments to transparency, merit, or local control often vanish once they threaten a favored outcome.</x:v>
       </x:c>
       <x:c r="N98" t="str">
-        <x:v>Many citizens argue that their country is a peaceful country...except whenever it is provoked. The definition of "provoke" is then liberally defined to encompass any trivial offense of another country.</x:v>
+        <x:v>Organizations sometimes advertise simple values statements that become practically meaningless once the long list of carve-outs is revealed.</x:v>
       </x:c>
       <x:c r="O98" t="str"/>
       <x:c r="P98" t="str"/>
       <x:c r="Q98" t="str"/>
       <x:c r="R98" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -4611,19 +4621,25 @@
       <x:c r="H100" t="str"/>
       <x:c r="I100" t="str"/>
       <x:c r="J100" t="str">
-        <x:v>Occurs when an inanimate object is wrongly treated as if it has the characteristics of animate objects.</x:v>
+        <x:v>Occurs when human feelings, intentions, or judgments are projected onto impersonal things and then treated as if the projection explained reality.</x:v>
       </x:c>
       <x:c r="K100" t="str">
-        <x:v>Look at the flowers lean towards the sun. You're cruel to sit in their sunlight!</x:v>
-      </x:c>
-      <x:c r="L100" t="str"/>
-      <x:c r="M100" t="str"/>
-      <x:c r="N100" t="str"/>
+        <x:v>The market is punishing voters today because it is afraid of reform.</x:v>
+      </x:c>
+      <x:c r="L100" t="str">
+        <x:v>Personifying weather, markets, or algorithms can be a vivid metaphor, but it becomes fallacious when the metaphor is used as literal evidence.</x:v>
+      </x:c>
+      <x:c r="M100" t="str">
+        <x:v>People often say the algorithm hates them, loves outrage, or wants to silence them when the actual explanation is a mix of optimization rules and incentives.</x:v>
+      </x:c>
+      <x:c r="N100" t="str">
+        <x:v>News coverage sometimes treats storms, markets, or viruses as if they were moral agents taking revenge, sending messages, or rewarding virtue.</x:v>
+      </x:c>
       <x:c r="O100" t="str"/>
       <x:c r="P100" t="str"/>
       <x:c r="Q100" t="str"/>
       <x:c r="R100" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -4737,25 +4753,25 @@
       </x:c>
       <x:c r="I103" t="str"/>
       <x:c r="J103" t="str">
-        <x:v>Twisting an opponent's analogy to mean something broader than intended.</x:v>
+        <x:v>Occurs when an analogy is deliberately stretched past its intended point so it can be mocked or refuted.</x:v>
       </x:c>
       <x:c r="K103" t="str">
-        <x:v>Tom said life is like a river in that those who spend the energy to maneuver their boats to the middle of the river will see more during their lifetime. This is ridiculous since he can not explained where the boats come from.</x:v>
+        <x:v>Calling public-health reserves an insurance policy is silly, because insurance companies do not hire epidemiologists.</x:v>
       </x:c>
       <x:c r="L103" t="str">
-        <x:v>This is a type of straw-man fallacy.</x:v>
+        <x:v>An analogy usually highlights one structural similarity, not a one-to-one mapping of every detail.</x:v>
       </x:c>
       <x:c r="M103" t="str">
-        <x:v>If person A claims their "loving" god will eternally torture the humans he created if they disobey him, and person B claims this is analogous to a "loving" human father eternally torturing his children if they disobey, for person A would unjustifiably pervert the analogy if they were to claim that the analogy does hold for irrelevant reasons such as "the human father is not righteous" or "human fathers don't live eternally".</x:v>
+        <x:v>Infrastructure analogies about bridges, firewalls, or guardrails are often attacked by demanding that every literal feature transfer over exactly.</x:v>
       </x:c>
       <x:c r="N103" t="str">
-        <x:v>If person A claims religious faith gives people joy that hides and prevents other possible joys in life in the same way that cocaine gives junkies joy at the expense of other possible joys in life, person B would unjustifiably pervert the analogy if they were to claim that the analogy does hold for irrelevant reasons such as "cocaine is not legal" or "people with faith serve God."</x:v>
+        <x:v>Debaters sometimes turn an opponent's limited comparison into a cartoon version so they can say the analogy obviously fails.</x:v>
       </x:c>
       <x:c r="O103" t="str"/>
       <x:c r="P103" t="str"/>
       <x:c r="Q103" t="str"/>
       <x:c r="R103" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -4995,19 +5011,25 @@
       <x:c r="H109" t="str"/>
       <x:c r="I109" t="str"/>
       <x:c r="J109" t="str">
-        <x:v>Assuming that a low probability of false matches means an improbable false match will not be found.</x:v>
+        <x:v>Occurs when a low probability of a false match is confused with a low probability that a matched person is innocent.</x:v>
       </x:c>
       <x:c r="K109" t="str">
-        <x:v>The probability of winning the lottery without cheating is a million to one, so the winner must have cheated.</x:v>
-      </x:c>
-      <x:c r="L109" t="str"/>
-      <x:c r="M109" t="str"/>
-      <x:c r="N109" t="str"/>
+        <x:v>The facial-recognition system is 99.9% accurate, so the person it flagged must almost certainly be the suspect.</x:v>
+      </x:c>
+      <x:c r="L109" t="str">
+        <x:v>The missing piece is the base rate. Even a very accurate test can generate many false matches when the target condition is rare.</x:v>
+      </x:c>
+      <x:c r="M109" t="str">
+        <x:v>Crime and security debates often overstate the force of DNA, face-recognition, or screening matches by ignoring how many non-matching people were also in the pool.</x:v>
+      </x:c>
+      <x:c r="N109" t="str">
+        <x:v>A similar mistake appears whenever a diagnostic tool's false-positive rate is treated as if it directly gave the chance that any one flagged person is guilty, sick, or dangerous.</x:v>
+      </x:c>
       <x:c r="O109" t="str"/>
       <x:c r="P109" t="str"/>
       <x:c r="Q109" t="str"/>
       <x:c r="R109" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -5031,25 +5053,25 @@
       <x:c r="H110" t="str"/>
       <x:c r="I110" t="str"/>
       <x:c r="J110" t="str">
-        <x:v>Occurs when an observer presupposes the objectivity of his own perspective when analyzing a behavioral event.</x:v>
+        <x:v>Occurs when someone projects their own motives, fears, or mental structure onto others and treats that projection as insight into those other people.</x:v>
       </x:c>
       <x:c r="K110" t="str">
-        <x:v>My buddies probably wish they were not married just as I do.</x:v>
+        <x:v>I need religion to keep my impulses in check, so atheists must secretly want religion for the same reason.</x:v>
       </x:c>
       <x:c r="L110" t="str">
-        <x:v>This fallacy is usually committed evermore infrequently as people age and explore the opinions and experiences of others outside their own community.</x:v>
+        <x:v>Self-knowledge can be useful, but it is not a universal template. Other people may share some motives while differing sharply on others.</x:v>
       </x:c>
       <x:c r="M110" t="str">
-        <x:v>Many theists who feel protected from their own impulses within the stricture of their religion's moral code accuse those who live without a moral code of having nothing that would prevent them from rape or murder. They subjectively assume that others share the same impulses they possess.</x:v>
+        <x:v>People often assume that because they would lie, panic, or seek status in a situation, anyone else in that situation must be driven by the same motive.</x:v>
       </x:c>
       <x:c r="N110" t="str">
-        <x:v>Many life-long atheists presume that theists are less than truthful when those theists claim they have experienced god speaking to them.</x:v>
+        <x:v>Political and religious debate is full of claims about what opponents 'really know' or 'really fear' that reflect the speaker's own psychology more than the target's.</x:v>
       </x:c>
       <x:c r="O110" t="str"/>
       <x:c r="P110" t="str"/>
       <x:c r="Q110" t="str"/>
       <x:c r="R110" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -5157,25 +5179,25 @@
       <x:c r="H113" t="str"/>
       <x:c r="I113" t="str"/>
       <x:c r="J113" t="str">
-        <x:v>Ascribes the cause of some phenomenon to some non-statistical factor, when natural and expected statistical fluctuations may account for the apparent phenomenon.</x:v>
+        <x:v>Occurs when movement back toward a normal range after an extreme result is credited to some intervention that may have had little or nothing to do with it.</x:v>
       </x:c>
       <x:c r="K113" t="str">
-        <x:v>Last year we had 12 car accidents on main street, double the previous year's figures! The frequency of accidents on Main Street fell to only 6 again after a speed camera was installed early this year. Therefore, the speed camera has improved road safety.</x:v>
+        <x:v>The student had an unusually bad test, got lectured by the teacher, and then scored closer to normal on the next test, so the lecture must have caused the improvement.</x:v>
       </x:c>
       <x:c r="L113" t="str">
-        <x:v>This is similar to the post hoc ergo propter hoc fallacy, but is based on the "regression to the mean" principle in which certain phenomena naturally fluctuate in volume or intensity. This statistical "noise" in the data is natural and expected.</x:v>
+        <x:v>After unusually high or low outcomes, partial reversion toward the average is often expected even without special causal forces.</x:v>
       </x:c>
       <x:c r="M113" t="str">
-        <x:v>In 1999 the Department of Education in Massachusetts gave it's school improvement goals, then subsequently tested those districts for any detectable improvement. Unsurprisingly, the bottom 50% of the schools made notable improvement. What was not so heavily emphasized was that the top 50% of their schools fell about the same degree as the bottom 50% gained. The apparent improvement of the bottom half and the apparent drop of the top half of any single phenomena is what is statistically expected and does not necessarily show the efficacy of any policy in effect at the time.</x:v>
+        <x:v>Sports commentators routinely over-credit halftime speeches or rituals for rebounds that would be unsurprising after an extreme first-half performance.</x:v>
       </x:c>
       <x:c r="N113" t="str">
-        <x:v>Two very tall parents will most likely have children who are taller than the average child. However, due to the natural regression to the mean, the children will also likely be shorter than the average height of their parents. To attribute the shortness of the child relative to their parents to anything other than a statistical expectation without accompanying evidence would be a regression fallacy.</x:v>
+        <x:v>Investors and managers often mistake a natural bounce after a terrible quarter for proof that a new slogan, consultant, or memo fixed the underlying problem.</x:v>
       </x:c>
       <x:c r="O113" t="str"/>
       <x:c r="P113" t="str"/>
       <x:c r="Q113" t="str"/>
       <x:c r="R113" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -5249,23 +5271,25 @@
         <x:v>retrodiction, post-diction</x:v>
       </x:c>
       <x:c r="J115" t="str">
-        <x:v>Arguing that, because some event has occurred, its occurrence was inevitable and should have been clear from the "obvious" causes.</x:v>
+        <x:v>Occurs when, after an outcome happens, people claim it was inevitable or obvious all along even though the uncertainty beforehand was real.</x:v>
       </x:c>
       <x:c r="K115" t="str">
-        <x:v>From the time the young Wayne Gretzky first put on skates, it was obvious from his natural ability and determinism that he was destined for greatness.</x:v>
+        <x:v>Once the startup collapsed, everyone said its failure had been obvious from day one.</x:v>
       </x:c>
       <x:c r="L115" t="str">
-        <x:v>The Wayne Gretzky example of "retrodiction" ignores all the forgotten children of parents who would now also be retrodicting had their children, who may have exhibited the same potential and determination as young Wayne, not failed to live up to the aspirations of their parents for some reason or other.</x:v>
+        <x:v>An outcome can make a story feel inevitable in retrospect without ever having been inevitable in advance. Hindsight strips away the branching paths that were live at the time.</x:v>
       </x:c>
       <x:c r="M115" t="str">
-        <x:v>Subsequent to the stock market crash of 2008-2009, many financial pundits who had failed to offer prospective deterministic predictions prior to the crash began to make retrospective deterministic retrospection, implying that the dynamics that lead to the crash were obvious to them.</x:v>
-      </x:c>
-      <x:c r="N115" t="str"/>
+        <x:v>After elections, market crashes, and celebrity scandals, commentators often speak as if the final result had been written into the evidence from the start rather than emerging from many uncertain factors.</x:v>
+      </x:c>
+      <x:c r="N115" t="str">
+        <x:v>This fallacy regularly follows close races and volatile technologies, where later narratives overstate how clear the winning path supposedly was.</x:v>
+      </x:c>
       <x:c r="O115" t="str"/>
       <x:c r="P115" t="str"/>
       <x:c r="Q115" t="str"/>
       <x:c r="R115" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -5287,29 +5311,25 @@
         <x:v>reductive semantic resolution</x:v>
       </x:c>
       <x:c r="J116" t="str">
-        <x:v>Occurs when a term or concept with low semantic precision is chosen over an available more precise term or concept in a way that distorts the opponent's stance.</x:v>
+        <x:v>Occurs when a fuzzy, graded, or probabilistic position is forced into unnaturally sharp categories so it becomes easier to attack.</x:v>
       </x:c>
       <x:c r="K116" t="str">
-        <x:v>You say you tend to believe you'll not die before you're 50. If you don't believe you'll die before you're 50, why did you buy a life insurance policy when you were 30?</x:v>
+        <x:v>If you say the rollout is probably safe, are you claiming it is perfectly safe with zero chance of failure?</x:v>
       </x:c>
       <x:c r="L116" t="str">
-        <x:v>In the example, the person making the argument is attempting to make his opponents belief binary so it can be more easily criticized. The belief most individuals have that they will live past 50 is not some binary and absolute belief, but rather is a degree of belief that emerges from an actuarial assessment of the probabilities. This fallacy is similar to the perfect standard fallacy.</x:v>
+        <x:v>Many concepts such as belief, risk, identity, and influence work by degree. Treating them as all-or-nothing can falsify the speaker's actual position.</x:v>
       </x:c>
       <x:c r="M116" t="str">
-        <x:v>The media often make statements such as "the murder rate increased by 50% last year" instead of more clearly stating "there were 3 murders committed this year, one more than last year." This unnecessarily diminishes the semantic resolution.</x:v>
+        <x:v>Election, public-health, and AI debates often force nuanced confidence claims into binary boxes such as certain or uncertain, safe or unsafe, real or fake.</x:v>
       </x:c>
       <x:c r="N116" t="str">
-        <x:v>You'll often hear statement such as "Just give me a straight answer! Do you or do you not enjoy taking drugs? Stop being evasive!" To answer "yes" or "no" would be to unnecessarily remove semantic resolution since enjoyment is a concept of degrees, and "drugs" is a term of multiple meanings.</x:v>
-      </x:c>
-      <x:c r="O116" t="str">
-        <x:v>When reporting crimes, the media often unnecessarily reduces semantic resolution by referring to an 18-year-old perpetrator or victim as a "man" or "woman" while referring to a 17-year-old as a "child".</x:v>
-      </x:c>
-      <x:c r="P116" t="str">
-        <x:v>Official titles of company officials are often vague and meaningless due to an attempt to heighten the prestige of the official. You may find yourself speaking to a "vice president" who is only one of 200 vice presidents in a company of 250 staff. The resolution that would allow you to better assess the real authority of the individual has been intentionally removed.</x:v>
-      </x:c>
+        <x:v>Arguments about what someone believes frequently replace a spectrum of confidence with a yes-or-no label that the original speaker never endorsed.</x:v>
+      </x:c>
+      <x:c r="O116" t="str"/>
+      <x:c r="P116" t="str"/>
       <x:c r="Q116" t="str"/>
       <x:c r="R116" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -5563,27 +5583,25 @@
       <x:c r="H122" t="str"/>
       <x:c r="I122" t="str"/>
       <x:c r="J122" t="str">
-        <x:v>Occurs when a person uncritically assumes that every member within a certain porous category is like those that receive the most coverage in the media.</x:v>
+        <x:v>Occurs when the most visible or most covered cases in a category are treated as if they represent the category as a whole.</x:v>
       </x:c>
       <x:c r="K122" t="str">
-        <x:v>All the Hispanics I've seen interviewed on television are not the least bit shy, so your neighbor Felipe surely can't be shy!</x:v>
+        <x:v>Every protester must be violent because the clips that reached my feed were violent.</x:v>
       </x:c>
       <x:c r="L122" t="str">
-        <x:v>This is a type of faulty generalization. A more detailed treatment of faulty generalizations can be found on the supplementary Inductive Errors page.</x:v>
+        <x:v>Attention is selective. Media, algorithms, and memory amplify the dramatic cases, not the ordinary distribution.</x:v>
       </x:c>
       <x:c r="M122" t="str">
-        <x:v>Because of the salient drama surrounding abortion clinic bombings, it became easy to erroneously view all abortion opponents as gun-wielding lunatics.</x:v>
+        <x:v>Crime clips, campus incidents, and viral protest footage often dominate public perception far beyond their representativeness, making whole groups look more extreme than they are.</x:v>
       </x:c>
       <x:c r="N122" t="str">
-        <x:v>Some could argue, based on television interviews, that Americans are not at all shy. This wold be a erroneous assumption since those to shy to be interviewed are never seen. This is the same type of error that leads to a selection bias in statistical studies.</x:v>
-      </x:c>
-      <x:c r="O122" t="str">
-        <x:v>While most Japanese who watch their pessimistic media assumed the 1,000 murders in 2010 in Japan was much higher than in what seemed to be a more peaceful past, the number was nearly 3 times lower than the murder rate in the 1950s, and remains one of the lowest per captita murder rates in the world.</x:v>
-      </x:c>
+        <x:v>People watching political interviews can easily conclude that a population is loud, combative, or theatrical without noticing that quieter members of the same population rarely become visible.</x:v>
+      </x:c>
+      <x:c r="O122" t="str"/>
       <x:c r="P122" t="str"/>
       <x:c r="Q122" t="str"/>
       <x:c r="R122" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -5739,26 +5757,25 @@
       <x:c r="H126" t="str"/>
       <x:c r="I126" t="str"/>
       <x:c r="J126" t="str">
-        <x:v>An argument which tries to redefine one mutually exclusive option so that it encompasses the other option.</x:v>
+        <x:v>Occurs when one term in a meaningful contrast is redefined so broadly or so narrowly that its opposing term can no longer do any work.</x:v>
       </x:c>
       <x:c r="K126" t="str">
-        <x:v>You can't claim to be intelligent since there is someone always more intelligent than you are.</x:v>
+        <x:v>No one is really healthy, because there is always someone healthier.</x:v>
       </x:c>
       <x:c r="L126" t="str">
-        <x:v>The consequence of this fallacy is that the term in question is made impotent by removing any contrasting concept.
-This fallacy is similar to the continuum fallacy.</x:v>
+        <x:v>Correlative terms such as healthy and unhealthy, free and restricted, informed and uninformed, or biased and impartial depend on contrasts that can be weakened without disappearing.</x:v>
       </x:c>
       <x:c r="M126" t="str">
-        <x:v>The god of some theists becomes so wrathful over a human's very 1st offense that he deems that offender worthy of eternal torment. This very same god is defined as "loving" and "patient" by these theists, and this definition is justified by suggesting that their wrathful god usually waits a while before sending the offender to eternal torment. The absurdity of this is clear when considering a neighbor who, after claiming to love his children, eternally beats them upon their first offense, but only after they've had dinner.</x:v>
+        <x:v>Critics sometimes argue that because everyone has some bias, calling a report biased says nothing, as if degrees of distortion and unfairness were impossible.</x:v>
       </x:c>
       <x:c r="N126" t="str">
-        <x:v>Some atheists claim that, to be a god-believer, you have to be "deluded". This definition of "deluded" would encompass most humans, rendering the word "deluded" much less meaningful as it did when it defined a much smaller set of humans.</x:v>
+        <x:v>Debates about freedom and censorship often set the positive term to an impossible ideal so that ordinary, useful distinctions collapse.</x:v>
       </x:c>
       <x:c r="O126" t="str"/>
       <x:c r="P126" t="str"/>
       <x:c r="Q126" t="str"/>
       <x:c r="R126" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -5786,19 +5803,25 @@
       </x:c>
       <x:c r="I127" t="str"/>
       <x:c r="J127" t="str">
-        <x:v>Occurs when a correlative is redefined so that one alternative is made impossible.</x:v>
+        <x:v>Occurs when a contrast term is emptied by redefining its counterpart so the distinction collapses.</x:v>
       </x:c>
       <x:c r="K127" t="str">
-        <x:v>Everyone expresses some emotion every day, so to say I'm being emotional has no basis!</x:v>
-      </x:c>
-      <x:c r="L127" t="str"/>
-      <x:c r="M127" t="str"/>
-      <x:c r="N127" t="str"/>
+        <x:v>Everyone has some bias, so calling this report biased tells us nothing.</x:v>
+      </x:c>
+      <x:c r="L127" t="str">
+        <x:v>The fact that a property comes in degrees does not erase the usefulness of the distinction. This duplicate record is kept in sync so both site entries carry a modernized explanation.</x:v>
+      </x:c>
+      <x:c r="M127" t="str">
+        <x:v>Public arguments often pretend that if no one is perfectly objective, then objectivity and bias can never be discussed in meaningful comparative terms.</x:v>
+      </x:c>
+      <x:c r="N127" t="str">
+        <x:v>A similar move appears when people say every restriction limits freedom somehow, therefore no restriction can be singled out as unusually coercive.</x:v>
+      </x:c>
       <x:c r="O127" t="str"/>
       <x:c r="P127" t="str"/>
       <x:c r="Q127" t="str"/>
       <x:c r="R127" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -5908,25 +5931,25 @@
         <x:v>a dicto secundum quid ad dictum simpliciter, proof by example</x:v>
       </x:c>
       <x:c r="J130" t="str">
-        <x:v>An argument of the following form. "a" has the negative quality "x" and belongs to the group "A". Therefore "A"s have "x".</x:v>
+        <x:v>Occurs when a negative trait found in one member of a group is used to condemn the group as a whole.</x:v>
       </x:c>
       <x:c r="K130" t="str">
-        <x:v>My neighbor is a banker, and is a jerk. Therefore, bankers are jerks.</x:v>
+        <x:v>One rideshare driver ran a scam on me, so rideshare drivers are crooks.</x:v>
       </x:c>
       <x:c r="L130" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
+        <x:v>A vivid case can motivate investigation, but it does not by itself justify a population-level conclusion.</x:v>
       </x:c>
       <x:c r="M130" t="str">
-        <x:v>If you break your leg the first time on the ski slopes, this is not evidence that skiing is any more dangerous than other sports. Actual statistical significance derived from a sufficiently large data set is necessary before such a conclusion can be made, in spite of your disinclination to get back on the slopes anytime soon.</x:v>
+        <x:v>Isolated crime stories are often turned into sweeping claims about immigrants, professions, age groups, or political movements.</x:v>
       </x:c>
       <x:c r="N130" t="str">
-        <x:v>When confronted with statistical evidence that a university degree improves your chances of securing a satisfying job, citing your unemployed Ph.D. neighbor does not invalidate the statistical evidence, and is a top-down condemnation fallacy.</x:v>
+        <x:v>A single corporate scandal can quickly become a claim that the entire industry is rotten in exactly the same way.</x:v>
       </x:c>
       <x:c r="O130" t="str"/>
       <x:c r="P130" t="str"/>
       <x:c r="Q130" t="str"/>
       <x:c r="R130" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -5958,19 +5981,25 @@
         <x:v>a dicto simpliciter quid ad dictium secundum</x:v>
       </x:c>
       <x:c r="J131" t="str">
-        <x:v>Occurs when an exception to a generalization is wrongly called for.</x:v>
+        <x:v>Occurs when a reasonable generalization is attacked by demanding that it hold without relevant scope conditions or exceptions.</x:v>
       </x:c>
       <x:c r="K131" t="str">
-        <x:v>Since cutting someone with a knife is a crime, surgeons are criminals.</x:v>
-      </x:c>
-      <x:c r="L131" t="str"/>
-      <x:c r="M131" t="str"/>
-      <x:c r="N131" t="str"/>
+        <x:v>You say processed sugar is unhealthy, but endurance athletes use sugar during races, so your generalization collapses.</x:v>
+      </x:c>
+      <x:c r="L131" t="str">
+        <x:v>Generalizations are often default-pattern claims, not exceptionless universal laws.</x:v>
+      </x:c>
+      <x:c r="M131" t="str">
+        <x:v>Public-health advice is often dismissed by pointing to unusual edge cases even when the advice was clearly aimed at ordinary conditions.</x:v>
+      </x:c>
+      <x:c r="N131" t="str">
+        <x:v>Safety rules and economic patterns are frequently challenged by exceptions that do not actually undermine the broader tendency being described.</x:v>
+      </x:c>
       <x:c r="O131" t="str"/>
       <x:c r="P131" t="str"/>
       <x:c r="Q131" t="str"/>
       <x:c r="R131" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -5994,29 +6023,25 @@
         <x:v>a dicto secundum quid ad dictum simpliciter, proof by example</x:v>
       </x:c>
       <x:c r="J132" t="str">
-        <x:v>An argument of the following form. "a" has the positive quality "x" and belongs to the group "A". Therefore "A"s have "x".</x:v>
+        <x:v>Occurs when a positive trait found in one member of a group is used to justify a positive conclusion about the group as a whole.</x:v>
       </x:c>
       <x:c r="K132" t="str">
-        <x:v>My neighbor is a banker, and a really nice guy. Therefore, bankers are nice guys.</x:v>
+        <x:v>My landlord fixed things promptly, so landlords get an unfairly bad reputation.</x:v>
       </x:c>
       <x:c r="L132" t="str">
-        <x:v>A more detailed treatment of this fallacy can be found on the supplementary Inductive Errors page.</x:v>
+        <x:v>A favorable anecdote can remind us not to overgeneralize negatively, but it cannot prove that the larger class is generally positive.</x:v>
       </x:c>
       <x:c r="M132" t="str">
-        <x:v>If a convenience store clerk successfully disarms a would-be robber, this is not evidence that confronting robbers is the best policy. A much larger sample of cases would be necessary before any inductive conclusion can be made.</x:v>
+        <x:v>One transparent politician or one ethical corporation is often used to imply that the surrounding system is healthier than the broader evidence suggests.</x:v>
       </x:c>
       <x:c r="N132" t="str">
-        <x:v>If your friend wins the lottery after entering a number based on his birthday and weight, this is not evidence that combining a participant's birthday and weight will yield a number that is in any way connected to a winning lottery number.</x:v>
-      </x:c>
-      <x:c r="O132" t="str">
-        <x:v>When confronted with statistical data that smoking is harmful, claiming that your smoking 105-year-old uncle disproves the statistics is a top-down justification fallacy.</x:v>
-      </x:c>
-      <x:c r="P132" t="str">
-        <x:v>If, when shown statistical evidence that acquiring a university degree increases your chances of acquiring a satisfying carreer, you invoke successful college drop-out Bill Gates in an attempt to invalidate the statistics, you have committed the top-down justification fallacy.</x:v>
-      </x:c>
+        <x:v>People frequently infer that an institution is trustworthy because they personally encountered one helpful employee inside it.</x:v>
+      </x:c>
+      <x:c r="O132" t="str"/>
+      <x:c r="P132" t="str"/>
       <x:c r="Q132" t="str"/>
       <x:c r="R132" t="str">
-        <x:v>cleaned-from-root</x:v>
+        <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
     <x:row r="133">

</xml_diff>

<commit_message>
Remove home spreadsheet nav link
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re8e7462bef4c452b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Ra55f7425f32c4160"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rca65faafd2eb41b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Red598a78fd4e4add"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R57c2eecee5644e0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Re51af8ed4aa84a7c"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Remove duplicate entry and add SEO metadata
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Red598a78fd4e4add"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R57c2eecee5644e0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Re51af8ed4aa84a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb8aa4757824a4409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R75383f7ddee64eba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Ra3677d9f163f453b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -206,7 +206,7 @@
         <x:v>Record count</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>139</x:v>
+        <x:v>138</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -5780,42 +5780,38 @@
     </x:row>
     <x:row r="127">
       <x:c r="A127" t="str">
-        <x:v>Suppressed correlative (DUPLICATE)</x:v>
+        <x:v>Teleological fallacy</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>suppressed-correlative-duplicate</x:v>
+        <x:v>teleological-fallacy</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>Linguistic</x:v>
-      </x:c>
-      <x:c r="D127" t="str">
         <x:v>Conceptual</x:v>
       </x:c>
+      <x:c r="D127" t="str"/>
       <x:c r="E127" t="str">
-        <x:v>9</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F127" t="str">
         <x:v>Formal Fallacy</x:v>
       </x:c>
       <x:c r="G127" t="str"/>
-      <x:c r="H127" t="str">
-        <x:v>Correlative based fallacy</x:v>
-      </x:c>
+      <x:c r="H127" t="str"/>
       <x:c r="I127" t="str"/>
       <x:c r="J127" t="str">
-        <x:v>Occurs when a contrast term is emptied by redefining its counterpart so the distinction collapses.</x:v>
+        <x:v>Occurs when a purpose, goal, or final destination is attributed to something without adequate evidence that such an end point was built into it.</x:v>
       </x:c>
       <x:c r="K127" t="str">
-        <x:v>Everyone has some bias, so calling this report biased tells us nothing.</x:v>
+        <x:v>Evolution created human intelligence because nature was trying to produce minds like ours.</x:v>
       </x:c>
       <x:c r="L127" t="str">
-        <x:v>The fact that a property comes in degrees does not erase the usefulness of the distinction. This duplicate record is kept in sync so both site entries carry a modernized explanation.</x:v>
+        <x:v>Some things really are designed for purposes, but purpose should not be assumed where it has not been shown. Processes can produce outcomes without aiming at them.</x:v>
       </x:c>
       <x:c r="M127" t="str">
-        <x:v>Public arguments often pretend that if no one is perfectly objective, then objectivity and bias can never be discussed in meaningful comparative terms.</x:v>
+        <x:v>People often speak as if history is automatically bending toward justice, collapse, nationalism, or liberation, as though social change carried its own guaranteed destination.</x:v>
       </x:c>
       <x:c r="N127" t="str">
-        <x:v>A similar move appears when people say every restriction limits freedom somehow, therefore no restriction can be singled out as unusually coercive.</x:v>
+        <x:v>In technology debates, AI progress is sometimes framed as if it were inherently marching toward a single destined endpoint such as AGI rather than following contingent technical and social paths.</x:v>
       </x:c>
       <x:c r="O127" t="str"/>
       <x:c r="P127" t="str"/>
@@ -5826,38 +5822,40 @@
     </x:row>
     <x:row r="128">
       <x:c r="A128" t="str">
-        <x:v>Teleological fallacy</x:v>
+        <x:v>Thought-terminating cliché</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>teleological-fallacy</x:v>
+        <x:v>thought-terminating-clich</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>Conceptual</x:v>
+        <x:v>Tactical</x:v>
       </x:c>
       <x:c r="D128" t="str"/>
       <x:c r="E128" t="str">
-        <x:v>19</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="F128" t="str">
-        <x:v>Formal Fallacy</x:v>
-      </x:c>
-      <x:c r="G128" t="str"/>
+        <x:v>Informal Fallacy</x:v>
+      </x:c>
+      <x:c r="G128" t="str">
+        <x:v>Faulty Generalization</x:v>
+      </x:c>
       <x:c r="H128" t="str"/>
       <x:c r="I128" t="str"/>
       <x:c r="J128" t="str">
-        <x:v>Occurs when a purpose, goal, or final destination is attributed to something without adequate evidence that such an end point was built into it.</x:v>
+        <x:v>Occurs when a familiar slogan or stock phrase is used to stop inquiry, deflect scrutiny, or create the feeling that an issue has already been settled.</x:v>
       </x:c>
       <x:c r="K128" t="str">
-        <x:v>Evolution created human intelligence because nature was trying to produce minds like ours.</x:v>
+        <x:v>It is what it is, so there is nothing more to discuss.</x:v>
       </x:c>
       <x:c r="L128" t="str">
-        <x:v>Some things really are designed for purposes, but purpose should not be assumed where it has not been shown. Processes can produce outcomes without aiming at them.</x:v>
+        <x:v>Aphorisms can be wise shortcuts, but they become fallacious when they replace the reasoning that the situation still requires.</x:v>
       </x:c>
       <x:c r="M128" t="str">
-        <x:v>People often speak as if history is automatically bending toward justice, collapse, nationalism, or liberation, as though social change carried its own guaranteed destination.</x:v>
+        <x:v>Phrases such as 'Do your own research,' 'common sense,' or 'if you know, you know' are often used online not to open inquiry but to make further questions look unnecessary or naive.</x:v>
       </x:c>
       <x:c r="N128" t="str">
-        <x:v>In technology debates, AI progress is sometimes framed as if it were inherently marching toward a single destined endpoint such as AGI rather than following contingent technical and social paths.</x:v>
+        <x:v>Political and religious arguments frequently end with slogans like 'Freedom is not free' or 'Only God knows,' which can be meaningful in some contexts but often function as conversation-stoppers.</x:v>
       </x:c>
       <x:c r="O128" t="str"/>
       <x:c r="P128" t="str"/>
@@ -5868,40 +5866,38 @@
     </x:row>
     <x:row r="129">
       <x:c r="A129" t="str">
-        <x:v>Thought-terminating cliché</x:v>
+        <x:v>Top-down condemnation</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>thought-terminating-clich</x:v>
+        <x:v>top-down-condemnation</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>Tactical</x:v>
-      </x:c>
-      <x:c r="D129" t="str"/>
-      <x:c r="E129" t="str">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="F129" t="str">
-        <x:v>Informal Fallacy</x:v>
-      </x:c>
-      <x:c r="G129" t="str">
-        <x:v>Faulty Generalization</x:v>
-      </x:c>
+        <x:v>Conceptual</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>Evidential</x:v>
+      </x:c>
+      <x:c r="E129" t="str"/>
+      <x:c r="F129" t="str"/>
+      <x:c r="G129" t="str"/>
       <x:c r="H129" t="str"/>
-      <x:c r="I129" t="str"/>
+      <x:c r="I129" t="str">
+        <x:v>a dicto secundum quid ad dictum simpliciter, proof by example</x:v>
+      </x:c>
       <x:c r="J129" t="str">
-        <x:v>Occurs when a familiar slogan or stock phrase is used to stop inquiry, deflect scrutiny, or create the feeling that an issue has already been settled.</x:v>
+        <x:v>Occurs when a negative trait found in one member of a group is used to condemn the group as a whole.</x:v>
       </x:c>
       <x:c r="K129" t="str">
-        <x:v>It is what it is, so there is nothing more to discuss.</x:v>
+        <x:v>One rideshare driver ran a scam on me, so rideshare drivers are crooks.</x:v>
       </x:c>
       <x:c r="L129" t="str">
-        <x:v>Aphorisms can be wise shortcuts, but they become fallacious when they replace the reasoning that the situation still requires.</x:v>
+        <x:v>A vivid case can motivate investigation, but it does not by itself justify a population-level conclusion.</x:v>
       </x:c>
       <x:c r="M129" t="str">
-        <x:v>Phrases such as 'Do your own research,' 'common sense,' or 'if you know, you know' are often used online not to open inquiry but to make further questions look unnecessary or naive.</x:v>
+        <x:v>Isolated crime stories are often turned into sweeping claims about immigrants, professions, age groups, or political movements.</x:v>
       </x:c>
       <x:c r="N129" t="str">
-        <x:v>Political and religious arguments frequently end with slogans like 'Freedom is not free' or 'Only God knows,' which can be meaningful in some contexts but often function as conversation-stoppers.</x:v>
+        <x:v>A single corporate scandal can quickly become a claim that the entire industry is rotten in exactly the same way.</x:v>
       </x:c>
       <x:c r="O129" t="str"/>
       <x:c r="P129" t="str"/>
@@ -5912,10 +5908,10 @@
     </x:row>
     <x:row r="130">
       <x:c r="A130" t="str">
-        <x:v>Top-down condemnation</x:v>
+        <x:v>Top-down faulty generalization</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>top-down-condemnation</x:v>
+        <x:v>top-down-faulty-generalization</x:v>
       </x:c>
       <x:c r="C130" t="str">
         <x:v>Conceptual</x:v>
@@ -5923,27 +5919,35 @@
       <x:c r="D130" t="str">
         <x:v>Evidential</x:v>
       </x:c>
-      <x:c r="E130" t="str"/>
-      <x:c r="F130" t="str"/>
-      <x:c r="G130" t="str"/>
-      <x:c r="H130" t="str"/>
+      <x:c r="E130" t="str">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F130" t="str">
+        <x:v>Informal Fallacy</x:v>
+      </x:c>
+      <x:c r="G130" t="str">
+        <x:v>A dicto simpliciter quid ad dictium secundum</x:v>
+      </x:c>
+      <x:c r="H130" t="str">
+        <x:v>Dicto simpliciter</x:v>
+      </x:c>
       <x:c r="I130" t="str">
-        <x:v>a dicto secundum quid ad dictum simpliciter, proof by example</x:v>
+        <x:v>a dicto simpliciter quid ad dictium secundum</x:v>
       </x:c>
       <x:c r="J130" t="str">
-        <x:v>Occurs when a negative trait found in one member of a group is used to condemn the group as a whole.</x:v>
+        <x:v>Occurs when a reasonable generalization is attacked by demanding that it hold without relevant scope conditions or exceptions.</x:v>
       </x:c>
       <x:c r="K130" t="str">
-        <x:v>One rideshare driver ran a scam on me, so rideshare drivers are crooks.</x:v>
+        <x:v>You say processed sugar is unhealthy, but endurance athletes use sugar during races, so your generalization collapses.</x:v>
       </x:c>
       <x:c r="L130" t="str">
-        <x:v>A vivid case can motivate investigation, but it does not by itself justify a population-level conclusion.</x:v>
+        <x:v>Generalizations are often default-pattern claims, not exceptionless universal laws.</x:v>
       </x:c>
       <x:c r="M130" t="str">
-        <x:v>Isolated crime stories are often turned into sweeping claims about immigrants, professions, age groups, or political movements.</x:v>
+        <x:v>Public-health advice is often dismissed by pointing to unusual edge cases even when the advice was clearly aimed at ordinary conditions.</x:v>
       </x:c>
       <x:c r="N130" t="str">
-        <x:v>A single corporate scandal can quickly become a claim that the entire industry is rotten in exactly the same way.</x:v>
+        <x:v>Safety rules and economic patterns are frequently challenged by exceptions that do not actually undermine the broader tendency being described.</x:v>
       </x:c>
       <x:c r="O130" t="str"/>
       <x:c r="P130" t="str"/>
@@ -5954,10 +5958,10 @@
     </x:row>
     <x:row r="131">
       <x:c r="A131" t="str">
-        <x:v>Top-down faulty generalization</x:v>
+        <x:v>Top-down justification</x:v>
       </x:c>
       <x:c r="B131" t="str">
-        <x:v>top-down-faulty-generalization</x:v>
+        <x:v>top-down-justification</x:v>
       </x:c>
       <x:c r="C131" t="str">
         <x:v>Conceptual</x:v>
@@ -5965,35 +5969,27 @@
       <x:c r="D131" t="str">
         <x:v>Evidential</x:v>
       </x:c>
-      <x:c r="E131" t="str">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="F131" t="str">
-        <x:v>Informal Fallacy</x:v>
-      </x:c>
-      <x:c r="G131" t="str">
-        <x:v>A dicto simpliciter quid ad dictium secundum</x:v>
-      </x:c>
-      <x:c r="H131" t="str">
-        <x:v>Dicto simpliciter</x:v>
-      </x:c>
+      <x:c r="E131" t="str"/>
+      <x:c r="F131" t="str"/>
+      <x:c r="G131" t="str"/>
+      <x:c r="H131" t="str"/>
       <x:c r="I131" t="str">
-        <x:v>a dicto simpliciter quid ad dictium secundum</x:v>
+        <x:v>a dicto secundum quid ad dictum simpliciter, proof by example</x:v>
       </x:c>
       <x:c r="J131" t="str">
-        <x:v>Occurs when a reasonable generalization is attacked by demanding that it hold without relevant scope conditions or exceptions.</x:v>
+        <x:v>Occurs when a positive trait found in one member of a group is used to justify a positive conclusion about the group as a whole.</x:v>
       </x:c>
       <x:c r="K131" t="str">
-        <x:v>You say processed sugar is unhealthy, but endurance athletes use sugar during races, so your generalization collapses.</x:v>
+        <x:v>My landlord fixed things promptly, so landlords get an unfairly bad reputation.</x:v>
       </x:c>
       <x:c r="L131" t="str">
-        <x:v>Generalizations are often default-pattern claims, not exceptionless universal laws.</x:v>
+        <x:v>A favorable anecdote can remind us not to overgeneralize negatively, but it cannot prove that the larger class is generally positive.</x:v>
       </x:c>
       <x:c r="M131" t="str">
-        <x:v>Public-health advice is often dismissed by pointing to unusual edge cases even when the advice was clearly aimed at ordinary conditions.</x:v>
+        <x:v>One transparent politician or one ethical corporation is often used to imply that the surrounding system is healthier than the broader evidence suggests.</x:v>
       </x:c>
       <x:c r="N131" t="str">
-        <x:v>Safety rules and economic patterns are frequently challenged by exceptions that do not actually undermine the broader tendency being described.</x:v>
+        <x:v>People frequently infer that an institution is trustworthy because they personally encountered one helpful employee inside it.</x:v>
       </x:c>
       <x:c r="O131" t="str"/>
       <x:c r="P131" t="str"/>
@@ -6004,38 +6000,34 @@
     </x:row>
     <x:row r="132">
       <x:c r="A132" t="str">
-        <x:v>Top-down justification</x:v>
+        <x:v>Track-record reset</x:v>
       </x:c>
       <x:c r="B132" t="str">
-        <x:v>top-down-justification</x:v>
+        <x:v>track-record-reset</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>Conceptual</x:v>
-      </x:c>
-      <x:c r="D132" t="str">
         <x:v>Evidential</x:v>
       </x:c>
+      <x:c r="D132" t="str"/>
       <x:c r="E132" t="str"/>
       <x:c r="F132" t="str"/>
       <x:c r="G132" t="str"/>
       <x:c r="H132" t="str"/>
-      <x:c r="I132" t="str">
-        <x:v>a dicto secundum quid ad dictum simpliciter, proof by example</x:v>
-      </x:c>
+      <x:c r="I132" t="str"/>
       <x:c r="J132" t="str">
-        <x:v>Occurs when a positive trait found in one member of a group is used to justify a positive conclusion about the group as a whole.</x:v>
+        <x:v>Occurs when each new claim is treated as if the relevant history of prior failures, hoaxes, or false alarms did not exist and should confer no default expectation at all.</x:v>
       </x:c>
       <x:c r="K132" t="str">
-        <x:v>My landlord fixed things promptly, so landlords get an unfairly bad reputation.</x:v>
+        <x:v>Yes, the last hundred miracle predictions failed, but this new one starts with a perfectly clean slate.</x:v>
       </x:c>
       <x:c r="L132" t="str">
-        <x:v>A favorable anecdote can remind us not to overgeneralize negatively, but it cannot prove that the larger class is generally positive.</x:v>
+        <x:v>A track record does not make contrary outcomes impossible, but it does affect rational priors. Ignoring repeated past failure forces every new case to borrow more credibility than it has earned.</x:v>
       </x:c>
       <x:c r="M132" t="str">
-        <x:v>One transparent politician or one ethical corporation is often used to imply that the surrounding system is healthier than the broader evidence suggests.</x:v>
+        <x:v>Baseless claims about widespread noncitizen voting keep getting relaunched as if decades of rarity, audits, and failed alarms provide no reason for initial skepticism.</x:v>
       </x:c>
       <x:c r="N132" t="str">
-        <x:v>People frequently infer that an institution is trustworthy because they personally encountered one helpful employee inside it.</x:v>
+        <x:v>Every new blurry UFO clip, miracle cure, or ghost story is often pitched as if the long record of ordinary explanations should have zero effect on our starting expectations.</x:v>
       </x:c>
       <x:c r="O132" t="str"/>
       <x:c r="P132" t="str"/>
@@ -6046,34 +6038,44 @@
     </x:row>
     <x:row r="133">
       <x:c r="A133" t="str">
-        <x:v>Track-record reset</x:v>
+        <x:v>Tu quoque</x:v>
       </x:c>
       <x:c r="B133" t="str">
-        <x:v>track-record-reset</x:v>
+        <x:v>tu-quoque</x:v>
       </x:c>
       <x:c r="C133" t="str">
         <x:v>Evidential</x:v>
       </x:c>
-      <x:c r="D133" t="str"/>
-      <x:c r="E133" t="str"/>
-      <x:c r="F133" t="str"/>
-      <x:c r="G133" t="str"/>
+      <x:c r="D133" t="str">
+        <x:v>Tactical</x:v>
+      </x:c>
+      <x:c r="E133" t="str">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F133" t="str">
+        <x:v>Informal Fallacy</x:v>
+      </x:c>
+      <x:c r="G133" t="str">
+        <x:v>Red Herring</x:v>
+      </x:c>
       <x:c r="H133" t="str"/>
-      <x:c r="I133" t="str"/>
+      <x:c r="I133" t="str">
+        <x:v>two wrongs make a right</x:v>
+      </x:c>
       <x:c r="J133" t="str">
-        <x:v>Occurs when each new claim is treated as if the relevant history of prior failures, hoaxes, or false alarms did not exist and should confer no default expectation at all.</x:v>
+        <x:v>Occurs when criticism is answered not by engaging the issue, but by pointing to similar hypocrisy or wrongdoing elsewhere.</x:v>
       </x:c>
       <x:c r="K133" t="str">
-        <x:v>Yes, the last hundred miracle predictions failed, but this new one starts with a perfectly clean slate.</x:v>
+        <x:v>You cannot criticize my fabricated quote because your side spreads misinformation too.</x:v>
       </x:c>
       <x:c r="L133" t="str">
-        <x:v>A track record does not make contrary outcomes impossible, but it does affect rational priors. Ignoring repeated past failure forces every new case to borrow more credibility than it has earned.</x:v>
+        <x:v>Hypocrisy can matter for trust, but it does not by itself answer whether the original claim, act, or argument was wrong.</x:v>
       </x:c>
       <x:c r="M133" t="str">
-        <x:v>Baseless claims about widespread noncitizen voting keep getting relaunched as if decades of rarity, audits, and failed alarms provide no reason for initial skepticism.</x:v>
+        <x:v>In the June 27, 2024 Biden-Trump debate and the September 10, 2024 Harris-Trump debate, many charges were met with 'your side did it too' responses that redirected blame without addressing the original allegation.</x:v>
       </x:c>
       <x:c r="N133" t="str">
-        <x:v>Every new blurry UFO clip, miracle cure, or ghost story is often pitched as if the long record of ordinary explanations should have zero effect on our starting expectations.</x:v>
+        <x:v>Arguments about misinformation, climate, religion, and media bias often slide into scorekeeping about who is worse rather than whether the specific criticized claim is true or justified.</x:v>
       </x:c>
       <x:c r="O133" t="str"/>
       <x:c r="P133" t="str"/>
@@ -6084,10 +6086,10 @@
     </x:row>
     <x:row r="134">
       <x:c r="A134" t="str">
-        <x:v>Tu quoque</x:v>
+        <x:v>Two wrongs make a right</x:v>
       </x:c>
       <x:c r="B134" t="str">
-        <x:v>tu-quoque</x:v>
+        <x:v>two-wrongs-make-a-right</x:v>
       </x:c>
       <x:c r="C134" t="str">
         <x:v>Evidential</x:v>
@@ -6096,7 +6098,7 @@
         <x:v>Tactical</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="F134" t="str">
         <x:v>Informal Fallacy</x:v>
@@ -6105,23 +6107,21 @@
         <x:v>Red Herring</x:v>
       </x:c>
       <x:c r="H134" t="str"/>
-      <x:c r="I134" t="str">
-        <x:v>two wrongs make a right</x:v>
-      </x:c>
+      <x:c r="I134" t="str"/>
       <x:c r="J134" t="str">
-        <x:v>Occurs when criticism is answered not by engaging the issue, but by pointing to similar hypocrisy or wrongdoing elsewhere.</x:v>
+        <x:v>Occurs when someone treats one wrong act as justified because it responds to, retaliates against, or balances out another wrong.</x:v>
       </x:c>
       <x:c r="K134" t="str">
-        <x:v>You cannot criticize my fabricated quote because your side spreads misinformation too.</x:v>
+        <x:v>Their side spread fake clips about us, so we are justified in spreading a few about them.</x:v>
       </x:c>
       <x:c r="L134" t="str">
-        <x:v>Hypocrisy can matter for trust, but it does not by itself answer whether the original claim, act, or argument was wrong.</x:v>
+        <x:v>Exposing hypocrisy can matter, but retaliation does not erase the original wrong or magically sanitize a copy of it.</x:v>
       </x:c>
       <x:c r="M134" t="str">
-        <x:v>In the June 27, 2024 Biden-Trump debate and the September 10, 2024 Harris-Trump debate, many charges were met with 'your side did it too' responses that redirected blame without addressing the original allegation.</x:v>
+        <x:v>In 2024 election discourse, misinformation was often excused with the claim that the other side lies too, as if symmetry or revenge transformed falsehood into fairness.</x:v>
       </x:c>
       <x:c r="N134" t="str">
-        <x:v>Arguments about misinformation, climate, religion, and media bias often slide into scorekeeping about who is worse rather than whether the specific criticized claim is true or justified.</x:v>
+        <x:v>Debates about censorship, doxxing, and dirty campaign tactics often slide from condemnation into imitation, with each side treating the other's bad behavior as a license to do the same.</x:v>
       </x:c>
       <x:c r="O134" t="str"/>
       <x:c r="P134" t="str"/>
@@ -6132,42 +6132,38 @@
     </x:row>
     <x:row r="135">
       <x:c r="A135" t="str">
-        <x:v>Two wrongs make a right</x:v>
+        <x:v>Undistributed middle</x:v>
       </x:c>
       <x:c r="B135" t="str">
-        <x:v>two-wrongs-make-a-right</x:v>
+        <x:v>undistributed-middle</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>Evidential</x:v>
-      </x:c>
-      <x:c r="D135" t="str">
-        <x:v>Tactical</x:v>
-      </x:c>
+        <x:v>Formal</x:v>
+      </x:c>
+      <x:c r="D135" t="str"/>
       <x:c r="E135" t="str">
-        <x:v>121</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F135" t="str">
-        <x:v>Informal Fallacy</x:v>
-      </x:c>
-      <x:c r="G135" t="str">
-        <x:v>Red Herring</x:v>
-      </x:c>
+        <x:v>Formal Fallacy</x:v>
+      </x:c>
+      <x:c r="G135" t="str"/>
       <x:c r="H135" t="str"/>
       <x:c r="I135" t="str"/>
       <x:c r="J135" t="str">
-        <x:v>Occurs when someone treats one wrong act as justified because it responds to, retaliates against, or balances out another wrong.</x:v>
+        <x:v>Occurs when two things are linked to the same broader category and the argument wrongly infers that one of them must therefore be the other.</x:v>
       </x:c>
       <x:c r="K135" t="str">
-        <x:v>Their side spread fake clips about us, so we are justified in spreading a few about them.</x:v>
+        <x:v>All conspiracy theorists distrust institutions. I distrust institutions. Therefore I am a conspiracy theorist.</x:v>
       </x:c>
       <x:c r="L135" t="str">
-        <x:v>Exposing hypocrisy can matter, but retaliation does not erase the original wrong or magically sanitize a copy of it.</x:v>
+        <x:v>Sharing a feature does not establish identity or class inclusion unless the shared feature actually covers the whole relevant group. A middle term can connect without unifying.</x:v>
       </x:c>
       <x:c r="M135" t="str">
-        <x:v>In 2024 election discourse, misinformation was often excused with the claim that the other side lies too, as if symmetry or revenge transformed falsehood into fairness.</x:v>
+        <x:v>Lifestyle and identity marketing often says 'the cool do X' and 'I do X,' then slides to 'therefore I am one of the cool,' even though the shared feature is too broad.</x:v>
       </x:c>
       <x:c r="N135" t="str">
-        <x:v>Debates about censorship, doxxing, and dirty campaign tactics often slide from condemnation into imitation, with each side treating the other's bad behavior as a license to do the same.</x:v>
+        <x:v>Political commentary frequently infers that because two camps are skeptical of the same institution or support the same policy, they must belong to the same underlying movement.</x:v>
       </x:c>
       <x:c r="O135" t="str"/>
       <x:c r="P135" t="str"/>
@@ -6178,38 +6174,34 @@
     </x:row>
     <x:row r="136">
       <x:c r="A136" t="str">
-        <x:v>Undistributed middle</x:v>
+        <x:v>Vague insulators</x:v>
       </x:c>
       <x:c r="B136" t="str">
-        <x:v>undistributed-middle</x:v>
+        <x:v>vague-insulators</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>Formal</x:v>
+        <x:v>Tactical</x:v>
       </x:c>
       <x:c r="D136" t="str"/>
-      <x:c r="E136" t="str">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="F136" t="str">
-        <x:v>Formal Fallacy</x:v>
-      </x:c>
+      <x:c r="E136" t="str"/>
+      <x:c r="F136" t="str"/>
       <x:c r="G136" t="str"/>
       <x:c r="H136" t="str"/>
       <x:c r="I136" t="str"/>
       <x:c r="J136" t="str">
-        <x:v>Occurs when two things are linked to the same broader category and the argument wrongly infers that one of them must therefore be the other.</x:v>
+        <x:v>Occurs when vague, elastic, or undefined terms are chosen so that a position sounds meaningful while resisting clear testing or criticism.</x:v>
       </x:c>
       <x:c r="K136" t="str">
-        <x:v>All conspiracy theorists distrust institutions. I distrust institutions. Therefore I am a conspiracy theorist.</x:v>
+        <x:v>These capsules restore your body's subtle energies and harmonize your inner system.</x:v>
       </x:c>
       <x:c r="L136" t="str">
-        <x:v>Sharing a feature does not establish identity or class inclusion unless the shared feature actually covers the whole relevant group. A middle term can connect without unifying.</x:v>
+        <x:v>Vagueness can be useful early in exploration, but it becomes fallacious when the fog is preserved to prevent serious evaluation. If key terms cannot be pinned down, the claim can keep slipping away from critique.</x:v>
       </x:c>
       <x:c r="M136" t="str">
-        <x:v>Lifestyle and identity marketing often says 'the cool do X' and 'I do X,' then slides to 'therefore I am one of the cool,' even though the shared feature is too broad.</x:v>
+        <x:v>Alternative-health and wellness marketing often leans on words like 'toxins,' 'energy,' 'balance,' and 'boost' precisely because they sound scientific while remaining hard to falsify.</x:v>
       </x:c>
       <x:c r="N136" t="str">
-        <x:v>Political commentary frequently infers that because two camps are skeptical of the same institution or support the same policy, they must belong to the same underlying movement.</x:v>
+        <x:v>In arguments about spirituality, self-help, and even AI, flexible phrases can be stretched to fit almost any outcome, which makes the view feel resilient without making it well supported.</x:v>
       </x:c>
       <x:c r="O136" t="str"/>
       <x:c r="P136" t="str"/>
@@ -6220,34 +6212,44 @@
     </x:row>
     <x:row r="137">
       <x:c r="A137" t="str">
-        <x:v>Vague insulators</x:v>
+        <x:v>Wishful thinking</x:v>
       </x:c>
       <x:c r="B137" t="str">
-        <x:v>vague-insulators</x:v>
+        <x:v>wishful-thinking</x:v>
       </x:c>
       <x:c r="C137" t="str">
-        <x:v>Tactical</x:v>
-      </x:c>
-      <x:c r="D137" t="str"/>
-      <x:c r="E137" t="str"/>
-      <x:c r="F137" t="str"/>
-      <x:c r="G137" t="str"/>
-      <x:c r="H137" t="str"/>
+        <x:v>Evidential</x:v>
+      </x:c>
+      <x:c r="D137" t="str">
+        <x:v>Epistemic, Emotional</x:v>
+      </x:c>
+      <x:c r="E137" t="str">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="F137" t="str">
+        <x:v>Informal Fallacy</x:v>
+      </x:c>
+      <x:c r="G137" t="str">
+        <x:v>Red Herring</x:v>
+      </x:c>
+      <x:c r="H137" t="str">
+        <x:v>Appeal to consequences</x:v>
+      </x:c>
       <x:c r="I137" t="str"/>
       <x:c r="J137" t="str">
-        <x:v>Occurs when vague, elastic, or undefined terms are chosen so that a position sounds meaningful while resisting clear testing or criticism.</x:v>
+        <x:v>Occurs when a belief or decision is driven mainly by what would be pleasing, hopeful, or comforting if true rather than by what the evidence supports.</x:v>
       </x:c>
       <x:c r="K137" t="str">
-        <x:v>These capsules restore your body's subtle energies and harmonize your inner system.</x:v>
+        <x:v>This stock is too exciting to fail, so I am sure it will recover.</x:v>
       </x:c>
       <x:c r="L137" t="str">
-        <x:v>Vagueness can be useful early in exploration, but it becomes fallacious when the fog is preserved to prevent serious evaluation. If key terms cannot be pinned down, the claim can keep slipping away from critique.</x:v>
+        <x:v>Hope can sustain action, but it does not convert possibility into evidence. The stronger the desire, the easier it is to mistake wanting for warrant.</x:v>
       </x:c>
       <x:c r="M137" t="str">
-        <x:v>Alternative-health and wellness marketing often leans on words like 'toxins,' 'energy,' 'balance,' and 'boost' precisely because they sound scientific while remaining hard to falsify.</x:v>
+        <x:v>Speculative markets, miracle-cure promises, and election-night narratives often run on the thought that a hoped-for outcome is somehow more likely because people badly want it.</x:v>
       </x:c>
       <x:c r="N137" t="str">
-        <x:v>In arguments about spirituality, self-help, and even AI, flexible phrases can be stretched to fit almost any outcome, which makes the view feel resilient without making it well supported.</x:v>
+        <x:v>Beliefs about the afterlife, destiny, or technological salvation are often defended by saying life would feel bleak without them, which speaks to desire rather than truth.</x:v>
       </x:c>
       <x:c r="O137" t="str"/>
       <x:c r="P137" t="str"/>
@@ -6258,44 +6260,36 @@
     </x:row>
     <x:row r="138">
       <x:c r="A138" t="str">
-        <x:v>Wishful thinking</x:v>
+        <x:v>Witness chain</x:v>
       </x:c>
       <x:c r="B138" t="str">
-        <x:v>wishful-thinking</x:v>
+        <x:v>witness-chain</x:v>
       </x:c>
       <x:c r="C138" t="str">
+        <x:v>Conceptual</x:v>
+      </x:c>
+      <x:c r="D138" t="str">
         <x:v>Evidential</x:v>
       </x:c>
-      <x:c r="D138" t="str">
-        <x:v>Epistemic, Emotional</x:v>
-      </x:c>
-      <x:c r="E138" t="str">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="F138" t="str">
-        <x:v>Informal Fallacy</x:v>
-      </x:c>
-      <x:c r="G138" t="str">
-        <x:v>Red Herring</x:v>
-      </x:c>
-      <x:c r="H138" t="str">
-        <x:v>Appeal to consequences</x:v>
-      </x:c>
+      <x:c r="E138" t="str"/>
+      <x:c r="F138" t="str"/>
+      <x:c r="G138" t="str"/>
+      <x:c r="H138" t="str"/>
       <x:c r="I138" t="str"/>
       <x:c r="J138" t="str">
-        <x:v>Occurs when a belief or decision is driven mainly by what would be pleasing, hopeful, or comforting if true rather than by what the evidence supports.</x:v>
+        <x:v>Occurs when testimony is padded by unverifiable references to other alleged witnesses, creating the illusion of corroboration without actually providing independent support.</x:v>
       </x:c>
       <x:c r="K138" t="str">
-        <x:v>This stock is too exciting to fail, so I am sure it will recover.</x:v>
+        <x:v>I saw the miracle myself, and dozens of others saw it too, though none of them are available to check.</x:v>
       </x:c>
       <x:c r="L138" t="str">
-        <x:v>Hope can sustain action, but it does not convert possibility into evidence. The stronger the desire, the easier it is to mistake wanting for warrant.</x:v>
+        <x:v>Real corroboration requires accessible, independent testimony or records. Simply claiming that more witnesses exist adds almost nothing if the chain cannot be examined.</x:v>
       </x:c>
       <x:c r="M138" t="str">
-        <x:v>Speculative markets, miracle-cure promises, and election-night narratives often run on the thought that a hoped-for outcome is somehow more likely because people badly want it.</x:v>
+        <x:v>Paranormal, religious, and conspiracy stories often swell in authority by invoking unnamed doctors, secret insiders, or hundreds of silent observers who never become independently available.</x:v>
       </x:c>
       <x:c r="N138" t="str">
-        <x:v>Beliefs about the afterlife, destiny, or technological salvation are often defended by saying life would feel bleak without them, which speaks to desire rather than truth.</x:v>
+        <x:v>Historical arguments sometimes treat a late report that 'many people saw it' as if that were the same thing as actually having many separate testimonies.</x:v>
       </x:c>
       <x:c r="O138" t="str"/>
       <x:c r="P138" t="str"/>
@@ -6306,83 +6300,43 @@
     </x:row>
     <x:row r="139">
       <x:c r="A139" t="str">
-        <x:v>Witness chain</x:v>
+        <x:v>Wrong causal direction</x:v>
       </x:c>
       <x:c r="B139" t="str">
-        <x:v>witness-chain</x:v>
+        <x:v>wrong-causal-direction</x:v>
       </x:c>
       <x:c r="C139" t="str">
-        <x:v>Conceptual</x:v>
-      </x:c>
-      <x:c r="D139" t="str">
-        <x:v>Evidential</x:v>
-      </x:c>
-      <x:c r="E139" t="str"/>
-      <x:c r="F139" t="str"/>
+        <x:v>Causal</x:v>
+      </x:c>
+      <x:c r="D139" t="str"/>
+      <x:c r="E139" t="str">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="F139" t="str">
+        <x:v>Informal Fallacy</x:v>
+      </x:c>
       <x:c r="G139" t="str"/>
       <x:c r="H139" t="str"/>
       <x:c r="I139" t="str"/>
       <x:c r="J139" t="str">
-        <x:v>Occurs when testimony is padded by unverifiable references to other alleged witnesses, creating the illusion of corroboration without actually providing independent support.</x:v>
+        <x:v>Occurs when a real association is noticed but the direction of causation is reversed.</x:v>
       </x:c>
       <x:c r="K139" t="str">
-        <x:v>I saw the miracle myself, and dozens of others saw it too, though none of them are available to check.</x:v>
+        <x:v>People who are already struggling concentrate more on self-help content, so the content must be what created the struggle.</x:v>
       </x:c>
       <x:c r="L139" t="str">
-        <x:v>Real corroboration requires accessible, independent testimony or records. Simply claiming that more witnesses exist adds almost nothing if the chain cannot be examined.</x:v>
+        <x:v>Correlations can be real while still pointing the wrong way. Without evidence about timing, mechanism, and alternatives, reversing cause and effect is easy.</x:v>
       </x:c>
       <x:c r="M139" t="str">
-        <x:v>Paranormal, religious, and conspiracy stories often swell in authority by invoking unnamed doctors, secret insiders, or hundreds of silent observers who never become independently available.</x:v>
+        <x:v>Arguments about social media and teen mental health often assume a one-way causal story even though distress can also increase the tendency to seek certain kinds of online engagement.</x:v>
       </x:c>
       <x:c r="N139" t="str">
-        <x:v>Historical arguments sometimes treat a late report that 'many people saw it' as if that were the same thing as actually having many separate testimonies.</x:v>
+        <x:v>Crime, policing, and economic debates frequently treat a response variable as if it were the cause, such as assuming security purchases create fear rather than fear driving security purchases.</x:v>
       </x:c>
       <x:c r="O139" t="str"/>
       <x:c r="P139" t="str"/>
       <x:c r="Q139" t="str"/>
       <x:c r="R139" t="str">
-        <x:v>modernized-2026-pass</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="140">
-      <x:c r="A140" t="str">
-        <x:v>Wrong causal direction</x:v>
-      </x:c>
-      <x:c r="B140" t="str">
-        <x:v>wrong-causal-direction</x:v>
-      </x:c>
-      <x:c r="C140" t="str">
-        <x:v>Causal</x:v>
-      </x:c>
-      <x:c r="D140" t="str"/>
-      <x:c r="E140" t="str">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="F140" t="str">
-        <x:v>Informal Fallacy</x:v>
-      </x:c>
-      <x:c r="G140" t="str"/>
-      <x:c r="H140" t="str"/>
-      <x:c r="I140" t="str"/>
-      <x:c r="J140" t="str">
-        <x:v>Occurs when a real association is noticed but the direction of causation is reversed.</x:v>
-      </x:c>
-      <x:c r="K140" t="str">
-        <x:v>People who are already struggling concentrate more on self-help content, so the content must be what created the struggle.</x:v>
-      </x:c>
-      <x:c r="L140" t="str">
-        <x:v>Correlations can be real while still pointing the wrong way. Without evidence about timing, mechanism, and alternatives, reversing cause and effect is easy.</x:v>
-      </x:c>
-      <x:c r="M140" t="str">
-        <x:v>Arguments about social media and teen mental health often assume a one-way causal story even though distress can also increase the tendency to seek certain kinds of online engagement.</x:v>
-      </x:c>
-      <x:c r="N140" t="str">
-        <x:v>Crime, policing, and economic debates frequently treat a response variable as if it were the cause, such as assuming security purchases create fear rather than fear driving security purchases.</x:v>
-      </x:c>
-      <x:c r="O140" t="str"/>
-      <x:c r="P140" t="str"/>
-      <x:c r="Q140" t="str"/>
-      <x:c r="R140" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
     </x:row>
@@ -6444,7 +6398,7 @@
         <x:v>Linguistic</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>Confusion created by wording, ambiguity, framing, or unstable definitions.</x:v>
@@ -6455,7 +6409,7 @@
         <x:v>Conceptual</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C6" t="str">
         <x:v>Errors caused by bad categories, weak distinctions, or distorted conceptual boundaries.</x:v>

</xml_diff>

<commit_message>
Save Cloudflare analytics tag for fallacy pages
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb8aa4757824a4409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R75383f7ddee64eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Ra3677d9f163f453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R70bf3d7c6eb449df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R9c93f40d2bc84f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R4794e28ed06844de"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Switch canonical site URL to logfall.com
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R70bf3d7c6eb449df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R9c93f40d2bc84f98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R4794e28ed06844de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1cdb3a6a4d8746a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R3cbbafb5ce0142a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R0dce9c02aaf54ea5"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Refresh fallacy pages with neutral palette
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R5600d42ac7dd4c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rdaee1a5e246c4f26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rcdaa0c9666ea4f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R52146d3dded64a71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rb517fdad91124970"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R43dcae04be8b46d9"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Audit alias coverage and hide empty alias cards
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R52146d3dded64a71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rb517fdad91124970"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R43dcae04be8b46d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R41b6ea0ddf53443e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R81fd489ce71140ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R9fb82353edc24c67"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2176,7 +2176,7 @@
       <x:c r="H42" t="str"/>
       <x:c r="I42" t="str"/>
       <x:c r="J42" t="str">
-        <x:v>chicken, the egg problem</x:v>
+        <x:v>chicken or the egg problem</x:v>
       </x:c>
       <x:c r="K42" t="str">
         <x:v>Occurs when a feedback loop is treated as if it fully explains, proves, or justifies a result, even though the loop may be contingent, breakable, or not sufficient for the claimed conclusion.</x:v>

</xml_diff>

<commit_message>
Add attributed case studies across fallacy pages
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4926f70ebbfa4510"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rf21d6e3cace749b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Ra6cf48e6d6574219"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R316bf591757f49b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R54067ec4d5be495d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R074be61854bc4376"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -356,14 +356,20 @@
         <x:v>Sometimes absence of evidence really is weak evidence, especially when the search tools are poor or the target is hard to detect. But when repeated investigation under the right conditions turns up nothing, that absence is itself evidence.</x:v>
       </x:c>
       <x:c r="N2" t="str">
-        <x:v>After officials in Springfield, Ohio said there were no credible reports supporting the September 2024 rumor that Haitian immigrants were abducting and eating pets, some defenders treated the lack of evidence as irrelevant or as proof of a cover-up rather than as evidence against the rumor.</x:v>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O2" t="str">
-        <x:v>Claims of widespread noncitizen voting in 2024 often survived repeated audits and official reviews by insisting that the absence of supporting evidence was exactly what one should expect from a hidden scheme.</x:v>
-      </x:c>
-      <x:c r="P2" t="str"/>
-      <x:c r="Q2" t="str"/>
-      <x:c r="R2" t="str"/>
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q2" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="R2" t="str">
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+      </x:c>
       <x:c r="S2" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -395,14 +401,20 @@
         <x:v>Abstract patterns can still be real and explanatory even when they depend on smaller physical or social components. Economies, institutions, languages, and ecosystems do not stop being real because they are made of people, words, or organisms.</x:v>
       </x:c>
       <x:c r="N3" t="str">
-        <x:v>People sometimes say 'science does not discover anything, only scientists do,' as if that erased the reality of science as a method and institution with stable norms and effects.</x:v>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="O3" t="str">
-        <x:v>Debates about algorithms, markets, and social platforms often pretend there is no system-level behavior because only users or lines of code act at the micro level.</x:v>
-      </x:c>
-      <x:c r="P3" t="str"/>
-      <x:c r="Q3" t="str"/>
-      <x:c r="R3" t="str"/>
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q3" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R3" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S3" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -434,14 +446,20 @@
         <x:v>Useful abstractions describe patterns with varying scope and durability. They are not automatically eternal, exceptionless constraints on what can happen.</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>People often treat economic or technological 'laws' as if they guaranteed the future rather than summarizing a contingent historical pattern that may bend, pause, or fail.</x:v>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>In AI discourse, scaling trends are sometimes talked about as destiny, as though past curves logically force a particular future rather than merely suggesting one.</x:v>
-      </x:c>
-      <x:c r="P4" t="str"/>
-      <x:c r="Q4" t="str"/>
-      <x:c r="R4" t="str"/>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q4" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R4" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
       <x:c r="S4" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -481,14 +499,20 @@
         <x:v>Character can matter when credibility itself is at issue, such as fraud, conflicts of interest, or proven dishonesty. The fallacy appears when those personal facts are used instead of answering the actual reasons or evidence.</x:v>
       </x:c>
       <x:c r="N5" t="str">
-        <x:v>In the June 27, 2024 Biden-Trump debate, policy exchanges repeatedly slid into attacks on each candidate's age, criminal exposure, or family rather than sustained engagement with the argument on the table.</x:v>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="O5" t="str">
-        <x:v>Online discussion of climate, vaccines, and AI policy often substitutes labels such as 'shill,' 'grifter,' or 'elitist' for any serious response to the evidence.</x:v>
-      </x:c>
-      <x:c r="P5" t="str"/>
-      <x:c r="Q5" t="str"/>
-      <x:c r="R5" t="str"/>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="P5" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="Q5" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
+      <x:c r="R5" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
       <x:c r="S5" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -524,14 +548,20 @@
         <x:v>Ruling something out does not automatically place it into the positive category you want. 'Not bad' does not by itself mean 'good,' and 'not that' does not by itself mean 'this.'</x:v>
       </x:c>
       <x:c r="N6" t="str">
-        <x:v>Tribal arguments often move from 'we are not them' and 'they are bad' to 'therefore we are trustworthy,' even though the conclusion has not been earned.</x:v>
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O6" t="str">
-        <x:v>Media and politics frequently treat the failure of one rival source as if it directly validated a different source that still needs its own support.</x:v>
-      </x:c>
-      <x:c r="P6" t="str"/>
-      <x:c r="Q6" t="str"/>
-      <x:c r="R6" t="str"/>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="Q6" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R6" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
       <x:c r="S6" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -569,14 +599,20 @@
         <x:v>Some disjunctions are genuinely exclusive, but many are not. Two options can coexist unless the statement or context really rules that out.</x:v>
       </x:c>
       <x:c r="N7" t="str">
-        <x:v>Budget rhetoric often suggests that because one policy tool is on the table, another cannot also matter, as if tradeoffs always come in only one-at-a-time form.</x:v>
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O7" t="str">
-        <x:v>Public debate regularly acts as though a claim must be either emotional or strategic, either true or persuasive, either mistaken or manipulative, when in reality both descriptions may apply.</x:v>
-      </x:c>
-      <x:c r="P7" t="str"/>
-      <x:c r="Q7" t="str"/>
-      <x:c r="R7" t="str"/>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P7" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="Q7" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R7" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S7" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -614,14 +650,20 @@
         <x:v>A consequence can have many causes. Observing the result does not tell you which sufficient condition produced it.</x:v>
       </x:c>
       <x:c r="N8" t="str">
-        <x:v>Political misinformation often treats one suspicious-looking detail as proof of a favored cause, even though many other explanations remain live.</x:v>
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O8" t="str">
-        <x:v>Arguments about fraud, manipulation, and AI generation frequently jump from a telltale symptom to a confident diagnosis without ruling out alternatives.</x:v>
-      </x:c>
-      <x:c r="P8" t="str"/>
-      <x:c r="Q8" t="str"/>
-      <x:c r="R8" t="str"/>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="Q8" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R8" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S8" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -655,14 +697,20 @@
         <x:v>Many systems of belief, institutions, and documents are mixed. Partial support or partial failure rarely justifies an everything-or-nothing verdict.</x:v>
       </x:c>
       <x:c r="N9" t="str">
-        <x:v>In 2024 media battles, a single correction or mistaken detail was often used to dismiss an outlet's entire reporting on elections, immigration, or public health.</x:v>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>Religious, ideological, and policy debates often act as though rejecting one doctrine, statistic, or mechanism commits you to rejecting the entire worldview.</x:v>
-      </x:c>
-      <x:c r="P9" t="str"/>
-      <x:c r="Q9" t="str"/>
-      <x:c r="R9" t="str"/>
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+      </x:c>
+      <x:c r="P9" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q9" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R9" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S9" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -700,14 +748,20 @@
         <x:v>Anecdotes can be useful for illustration, hypothesis generation, or showing that something can happen. The fallacy appears when one memorable case is used to outweigh stronger evidence about what usually happens or what the larger data set shows.</x:v>
       </x:c>
       <x:c r="N10" t="str">
-        <x:v>Arguments about vaccines, supplements, and raw milk often lean on a neighbor's success story or a family anecdote as if that settled what the best studies show.</x:v>
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
       </x:c>
       <x:c r="O10" t="str">
-        <x:v>Debates about AI productivity and remote work often treat one manager's striking success or failure story as if it established the general rule for everyone.</x:v>
-      </x:c>
-      <x:c r="P10" t="str"/>
-      <x:c r="Q10" t="str"/>
-      <x:c r="R10" t="str"/>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="P10" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="Q10" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="R10" t="str">
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+      </x:c>
       <x:c r="S10" t="str">
         <x:v>added-2026-completeness-pass</x:v>
       </x:c>
@@ -749,14 +803,20 @@
         <x:v>Real accomplishment can justify attention, but it does not automatically transfer expertise across domains. The relevant question is still whether the claim is supported.</x:v>
       </x:c>
       <x:c r="N11" t="str">
-        <x:v>Celebrity founders, athletes, and actors often lend credibility to products and causes far outside their expertise, from supplements to financial schemes to political narratives.</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>Public arguments about AI frequently treat the prestige of well-known founders as if it settled disputes that still require technical evidence, replication, and broader expert scrutiny.</x:v>
-      </x:c>
-      <x:c r="P11" t="str"/>
-      <x:c r="Q11" t="str"/>
-      <x:c r="R11" t="str"/>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
+      <x:c r="Q11" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="R11" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
       <x:c r="S11" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -798,14 +858,20 @@
         <x:v>Expert testimony can be good evidence when the authority is relevant, the expertise is genuine, and the claim fits the expert consensus. The fallacy appears when prestige replaces argument.</x:v>
       </x:c>
       <x:c r="N12" t="str">
-        <x:v>Debates about nutrition, vaccines, crypto, and AI frequently lean on celebrity experts or founders speaking outside their strongest field, while the underlying studies and uncertainties get little attention.</x:v>
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="O12" t="str">
-        <x:v>In public discussion of AI safety and capability, people often present a famous CEO's confidence level as if it were itself a substitute for technical evidence or broad expert agreement.</x:v>
-      </x:c>
-      <x:c r="P12" t="str"/>
-      <x:c r="Q12" t="str"/>
-      <x:c r="R12" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P12" t="str">
+        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+      </x:c>
+      <x:c r="Q12" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="R12" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S12" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -847,14 +913,20 @@
         <x:v>Consequences matter for what we should do, but they do not by themselves determine what is true. A painful implication does not refute a claim, and a comforting implication does not confirm one.</x:v>
       </x:c>
       <x:c r="N13" t="str">
-        <x:v>Some climate arguments treat the economic and political inconvenience of decarbonization as if it counted against the underlying science itself.</x:v>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="O13" t="str">
-        <x:v>In debates about AI consciousness, animal cognition, or moral status, people sometimes argue that the conclusion cannot be right because accepting it would create uncomfortable obligations.</x:v>
-      </x:c>
-      <x:c r="P13" t="str"/>
-      <x:c r="Q13" t="str"/>
-      <x:c r="R13" t="str"/>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P13" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="Q13" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="R13" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
       <x:c r="S13" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -896,14 +968,20 @@
         <x:v>Emotion is not irrational by itself. The fallacy appears when emotion substitutes for the reasoning that still needs to be supplied.</x:v>
       </x:c>
       <x:c r="N14" t="str">
-        <x:v>In 2024 campaign advertising, immigration, crime, and abortion messages often relied on fear-laden images and worst-case anecdotes whose emotional force far exceeded the actual argument being made.</x:v>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O14" t="str">
-        <x:v>The spread of AI-generated political ads and deepfakes in 2024 showed how cheaply campaigns can trigger outrage or panic before voters have time to inspect the evidence.</x:v>
-      </x:c>
-      <x:c r="P14" t="str"/>
-      <x:c r="Q14" t="str"/>
-      <x:c r="R14" t="str"/>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="P14" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="Q14" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R14" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
       <x:c r="S14" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -943,14 +1021,20 @@
         <x:v>Fear can be rational when the threat is real and well evidenced. The fallacy appears when fear does the persuasive work that evidence and reasoning have not done.</x:v>
       </x:c>
       <x:c r="N15" t="str">
-        <x:v>Campaign messaging about immigrants, crime, and cultural decline often relies on catastrophic imagery that outruns the actual evidence offered for the policy being sold.</x:v>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="O15" t="str">
-        <x:v>Scams involving miracle cures, emergency investments, or account security often push people to act before they can think by making delay feel dangerous.</x:v>
-      </x:c>
-      <x:c r="P15" t="str"/>
-      <x:c r="Q15" t="str"/>
-      <x:c r="R15" t="str"/>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P15" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="Q15" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R15" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
       <x:c r="S15" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -990,14 +1074,20 @@
         <x:v>Compliments can be sincere and harmless. The fallacy appears when praise does the persuasive work by making agreement feel like a badge of intelligence or independence.</x:v>
       </x:c>
       <x:c r="N16" t="str">
-        <x:v>Wellness, crypto, and conspiracy marketing often tells followers they are 'awake,' 'elite,' or 'smart enough to see through the lie,' turning assent into a test of self-image.</x:v>
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="O16" t="str">
-        <x:v>Political fundraising and influencer media frequently flatter supporters as the few people brave or intelligent enough to 'see what is really happening' before asking them to accept weakly supported claims.</x:v>
-      </x:c>
-      <x:c r="P16" t="str"/>
-      <x:c r="Q16" t="str"/>
-      <x:c r="R16" t="str"/>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="P16" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="Q16" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="R16" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
       <x:c r="S16" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1037,14 +1127,20 @@
         <x:v>Motives can be relevant to bias and credibility, but they do not automatically settle whether the argument or evidence is sound.</x:v>
       </x:c>
       <x:c r="N17" t="str">
-        <x:v>After the September 2024 ABC debate, accusations about moderator bias were often used not just to question fairness, but to pre-dismiss later fact-checks without engaging their substance.</x:v>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O17" t="str">
-        <x:v>In debates about climate, vaccines, and AI policy, critics are often waved away as 'funded,' 'bought,' or 'performing for clicks' instead of being answered.</x:v>
-      </x:c>
-      <x:c r="P17" t="str"/>
-      <x:c r="Q17" t="str"/>
-      <x:c r="R17" t="str"/>
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="P17" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="Q17" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
+      <x:c r="R17" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
       <x:c r="S17" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1084,14 +1180,20 @@
         <x:v>Natural things can heal, but they can also poison, infect, and kill. The fallacy treats a vague origin label as if it already settled the medical, moral, or practical question.</x:v>
       </x:c>
       <x:c r="N18" t="str">
-        <x:v>Wellness marketing for raw milk, supplements, and 'clean' products often treats natural as if it automatically meant safer, healthier, or morally superior.</x:v>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O18" t="str">
-        <x:v>Arguments about sex, family, and medicine often smuggle a moral conclusion into the descriptive claim that one pattern is simply 'what nature intended.'</x:v>
-      </x:c>
-      <x:c r="P18" t="str"/>
-      <x:c r="Q18" t="str"/>
-      <x:c r="R18" t="str"/>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="P18" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="Q18" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="R18" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
       <x:c r="S18" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1133,14 +1235,20 @@
         <x:v>New tools and ideas can be improvements, but novelty itself is not proof. The relevant questions are performance, tradeoffs, and evidence, not freshness.</x:v>
       </x:c>
       <x:c r="N19" t="str">
-        <x:v>In the 2024 rush to adopt generative AI, many products were pitched as inherently superior because they were new, even when reliability, labor impact, and safety were still unsettled.</x:v>
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="O19" t="str">
-        <x:v>Political and management rhetoric often treats 'innovation' as a reason to trust a strategy before any serious test of whether it solves the underlying problem.</x:v>
-      </x:c>
-      <x:c r="P19" t="str"/>
-      <x:c r="Q19" t="str"/>
-      <x:c r="R19" t="str"/>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="P19" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="Q19" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="R19" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S19" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1180,14 +1288,20 @@
         <x:v>Compassion can matter for what response is humane, but it does not determine whether the underlying claim has been proved.</x:v>
       </x:c>
       <x:c r="N20" t="str">
-        <x:v>Fundraising and advocacy campaigns sometimes imply that questioning a factual claim is itself heartless, shifting the pressure from evidence to emotional identification.</x:v>
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="O20" t="str">
-        <x:v>Public figures under scrutiny sometimes ask to be believed or excused because they are suffering, overwhelmed, or facing intense pressure, even when those facts do not establish the truth of what they are saying.</x:v>
-      </x:c>
-      <x:c r="P20" t="str"/>
-      <x:c r="Q20" t="str"/>
-      <x:c r="R20" t="str"/>
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
+      <x:c r="P20" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="Q20" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="R20" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S20" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1227,14 +1341,20 @@
         <x:v>Background can illuminate perspective, but hardship is not a truth detector. A difficult life story may earn sympathy or respect without settling the claim being made.</x:v>
       </x:c>
       <x:c r="N21" t="str">
-        <x:v>Campaign biographies in 2024 often leaned heavily on working-class roots and hardship stories, which may matter politically but do not by themselves verify a candidate's policy claims.</x:v>
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="O21" t="str">
-        <x:v>Populist media often imply that 'ordinary people' are automatically more honest than credentialed critics, as if social position alone settled the argument.</x:v>
-      </x:c>
-      <x:c r="P21" t="str"/>
-      <x:c r="Q21" t="str"/>
-      <x:c r="R21" t="str"/>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="P21" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="Q21" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="R21" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
       <x:c r="S21" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1270,14 +1390,20 @@
         <x:v>Possibility is a very weak starting point. Many things are possible without being probable, and many probable things still fail to happen in any given case.</x:v>
       </x:c>
       <x:c r="N22" t="str">
-        <x:v>Crypto, lottery, and sports-betting talk often slides from 'this could happen' to 'this is bound to happen,' especially after a short streak of wins.</x:v>
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O22" t="str">
-        <x:v>Election and catastrophe commentary often treats a legally or physically possible scenario as if it were destined simply because people can imagine it vividly.</x:v>
-      </x:c>
-      <x:c r="P22" t="str"/>
-      <x:c r="Q22" t="str"/>
-      <x:c r="R22" t="str"/>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P22" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q22" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="R22" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
       <x:c r="S22" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1317,14 +1443,20 @@
         <x:v>Ridicule can make a position look silly without ever testing whether it is wrong. Laughter is not an argument.</x:v>
       </x:c>
       <x:c r="N23" t="str">
-        <x:v>Debates about religion, feminism, climate, and AI are often reduced to memes whose purpose is to make one side look ridiculous rather than to assess the actual claim.</x:v>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O23" t="str">
-        <x:v>Online discourse frequently treats a sarcastic dunk or quote-tweet pile-on as if public humiliation itself were refutation.</x:v>
-      </x:c>
-      <x:c r="P23" t="str"/>
-      <x:c r="Q23" t="str"/>
-      <x:c r="R23" t="str"/>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="P23" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
+      <x:c r="Q23" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="R23" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S23" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1364,14 +1496,20 @@
         <x:v>Anger at the people who might benefit from a policy does not settle whether the policy is wise, fair, or effective.</x:v>
       </x:c>
       <x:c r="N24" t="str">
-        <x:v>Campaign messages often invite voters to reject a proposal because hated elites, immigrants, bankers, or academics might benefit, even when that says nothing about the proposal's merits.</x:v>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O24" t="str">
-        <x:v>Social-media outrage often works by making the audience feel that supporting a view would somehow reward people they already dislike.</x:v>
-      </x:c>
-      <x:c r="P24" t="str"/>
-      <x:c r="Q24" t="str"/>
-      <x:c r="R24" t="str"/>
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="P24" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="Q24" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R24" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
       <x:c r="S24" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1413,14 +1551,20 @@
         <x:v>Traditions can embody wisdom, but age alone does not prove justice, truth, or usefulness. A tradition still has to survive present scrutiny.</x:v>
       </x:c>
       <x:c r="N25" t="str">
-        <x:v>In 2024 arguments that the United States is a 'Christian nation,' long practice and selective founding-era precedent were often treated as if they settled the constitutional question.</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O25" t="str">
-        <x:v>Arguments about schooling, marriage, and gender roles often rely on 'we have always done it this way' instead of showing why the tradition remains just or effective.</x:v>
-      </x:c>
-      <x:c r="P25" t="str"/>
-      <x:c r="Q25" t="str"/>
-      <x:c r="R25" t="str"/>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P25" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="Q25" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="R25" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
       <x:c r="S25" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1460,14 +1604,20 @@
         <x:v>Success can indicate skill in a particular domain, but money is not a universal credential. Wealth may buy attention, not truth.</x:v>
       </x:c>
       <x:c r="N26" t="str">
-        <x:v>In 2024 and 2025, fans and investors often treated billionaire founders' views on AI, politics, or medicine as self-validating because of their wealth rather than because the evidence was strong.</x:v>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="O26" t="str">
-        <x:v>The unverified ABC debate affidavit gained extra credibility online after high-profile wealthy amplifiers helped circulate it, as though status itself made the claim more trustworthy.</x:v>
-      </x:c>
-      <x:c r="P26" t="str"/>
-      <x:c r="Q26" t="str"/>
-      <x:c r="R26" t="str"/>
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
+      <x:c r="P26" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="Q26" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="R26" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
       <x:c r="S26" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1503,14 +1653,20 @@
         <x:v>A bad argument can defend a true claim, and a strong claim can be defended poorly. Refuting the reasoning offered is not the same thing as refuting the conclusion.</x:v>
       </x:c>
       <x:c r="N27" t="str">
-        <x:v>When a candidate exaggerates one statistic, opponents often jump from 'that argument was flawed' to 'the broader policy position must therefore be false.'</x:v>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O27" t="str">
-        <x:v>Online 'gotcha' culture frequently treats catching a fallacious defense as if it automatically disproved whatever the speaker was trying to defend.</x:v>
-      </x:c>
-      <x:c r="P27" t="str"/>
-      <x:c r="Q27" t="str"/>
-      <x:c r="R27" t="str"/>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P27" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="Q27" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R27" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
       <x:c r="S27" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1548,14 +1704,20 @@
         <x:v>The burden is not met by pointing to a gap in refutation. A claim needs positive support of its own. Lack of an explanation is not the same thing as evidence for a preferred explanation.</x:v>
       </x:c>
       <x:c r="N28" t="str">
-        <x:v>After an anonymous affidavit circulated online in September 2024 alleging that ABC had secretly rigged the Harris-Trump debate, many posts treated the absence of immediate disproof as if it were evidence that the allegation was real.</x:v>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O28" t="str">
-        <x:v>UAP discussions often jump from 'we do not yet know what caused this' to 'therefore it was extraterrestrial technology,' which treats unexplained as if it meant explained by the favored hypothesis.</x:v>
-      </x:c>
-      <x:c r="P28" t="str"/>
-      <x:c r="Q28" t="str"/>
-      <x:c r="R28" t="str"/>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="P28" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="Q28" t="str">
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="R28" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
       <x:c r="S28" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1593,14 +1755,20 @@
         <x:v>Our imagination is not a reliable measure of what reality permits. Difficulty understanding a mechanism may justify caution or further inquiry, but it does not by itself establish that a preferred alternative is true.</x:v>
       </x:c>
       <x:c r="N29" t="str">
-        <x:v>Discussions of evolution, climate systems, and AI often slide from 'I do not see how that could work' to 'therefore it cannot be right.'</x:v>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O29" t="str">
-        <x:v>Paranormal and conspiracy arguments often rely on the mirror image of the same move: 'I cannot imagine another explanation, so my favored explanation must be true.'</x:v>
-      </x:c>
-      <x:c r="P29" t="str"/>
-      <x:c r="Q29" t="str"/>
-      <x:c r="R29" t="str"/>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="P29" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="Q29" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R29" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
       <x:c r="S29" t="str">
         <x:v>added-2026-completeness-pass</x:v>
       </x:c>
@@ -1638,14 +1806,20 @@
         <x:v>A claim does not become better supported because it is repeated by the same speaker, echoed by many speakers, or circulated for a long time. Repetition changes familiarity, not the underlying evidence.</x:v>
       </x:c>
       <x:c r="N30" t="str">
-        <x:v>The Springfield, Ohio pet-eating rumor in September 2024 moved from rumor to national talking point largely through repetition across social media, cable segments, and campaign rhetoric even though local officials said there was no credible evidence.</x:v>
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
       </x:c>
       <x:c r="O30" t="str">
-        <x:v>Claims of widespread noncitizen voting often survive audit after audit because the same allegation is repeated so often that persistence itself gets mistaken for proof.</x:v>
-      </x:c>
-      <x:c r="P30" t="str"/>
-      <x:c r="Q30" t="str"/>
-      <x:c r="R30" t="str"/>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="P30" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="Q30" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
+      <x:c r="R30" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
       <x:c r="S30" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1685,14 +1859,20 @@
         <x:v>Silence can matter when a response would clearly be expected and feasible. Outside that setting, it often tells us little.</x:v>
       </x:c>
       <x:c r="N31" t="str">
-        <x:v>The absence of public confirmation for many election-fraud and migrant-voting rumors was often spun as suspicious silence rather than as a sign that the underlying evidence was weak or nonexistent.</x:v>
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
       <x:c r="O31" t="str">
-        <x:v>A 'no comment' from campaigns, police, or institutions is regularly treated as if it were a tacit admission, even though legal, strategic, or practical reasons may explain the silence.</x:v>
-      </x:c>
-      <x:c r="P31" t="str"/>
-      <x:c r="Q31" t="str"/>
-      <x:c r="R31" t="str"/>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="P31" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q31" t="str">
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="R31" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
       <x:c r="S31" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1734,14 +1914,20 @@
         <x:v>Threats can force compliance, but they do not transform a bad argument into a good one. Fear may explain why someone goes along; it does not show that the view is correct.</x:v>
       </x:c>
       <x:c r="N32" t="str">
-        <x:v>In countries where blasphemy, apostasy, or political dissent can trigger severe punishment, outward conformity is often mistaken for genuine persuasion when it may simply reflect fear.</x:v>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="O32" t="str">
-        <x:v>Online campaigns that threaten doxxing, blacklisting, or mass harassment often aim to secure silence or agreement by making disagreement personally costly.</x:v>
-      </x:c>
-      <x:c r="P32" t="str"/>
-      <x:c r="Q32" t="str"/>
-      <x:c r="R32" t="str"/>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="P32" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="Q32" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="R32" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S32" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1785,14 +1971,20 @@
         <x:v>Popularity can reveal what people want, fear, or have been persuaded by, but it does not settle what is true. Crowds can be informed, confused, manipulated, or all three at once.</x:v>
       </x:c>
       <x:c r="N33" t="str">
-        <x:v>Advocates of raw milk and other 'natural' wellness products often point to growing enthusiasm, celebrity uptake, or huge followings as if social momentum itself established safety or effectiveness.</x:v>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="O33" t="str">
-        <x:v>Viral political claims are often defended with phrases like 'everyone is talking about it' or 'it has millions of views,' which confuses reach with reliability.</x:v>
-      </x:c>
-      <x:c r="P33" t="str"/>
-      <x:c r="Q33" t="str"/>
-      <x:c r="R33" t="str"/>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="P33" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="Q33" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R33" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
       <x:c r="S33" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1826,14 +2018,20 @@
         <x:v>There is an important difference between suspending belief, doubting a claim, and asserting the opposite claim. Collapsing those positions is often a way of shifting burdens that have not been earned.</x:v>
       </x:c>
       <x:c r="N34" t="str">
-        <x:v>Religious and paranormal debates often insist that skepticism itself is just another faith commitment, as if withholding belief carried the same evidential burden as proposing the phenomenon.</x:v>
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O34" t="str">
-        <x:v>Arguments about election fraud and miracle claims sometimes recast 'I have not seen enough evidence' into 'you are certain it never happened' so the original claimant can dodge the burden of proof.</x:v>
-      </x:c>
-      <x:c r="P34" t="str"/>
-      <x:c r="Q34" t="str"/>
-      <x:c r="R34" t="str"/>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="P34" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="Q34" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="R34" t="str">
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
       <x:c r="S34" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1875,14 +2073,20 @@
         <x:v>Associations can sometimes matter when they reveal bias, incentives, or causal links. The fallacy appears when the link is treated as decisive even though it does not address the argument.</x:v>
       </x:c>
       <x:c r="N35" t="str">
-        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported.</x:v>
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="O35" t="str">
-        <x:v>Political arguments routinely assume that if a bad person, rival group, or disliked movement touched an idea, the idea itself must be false or tainted.</x:v>
-      </x:c>
-      <x:c r="P35" t="str"/>
-      <x:c r="Q35" t="str"/>
-      <x:c r="R35" t="str"/>
+        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+      </x:c>
+      <x:c r="P35" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="Q35" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="R35" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
       <x:c r="S35" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1918,14 +2122,20 @@
         <x:v>Confidence, volume, and repetition can make a bare assertion sound weighty, but they do not do the evidential work. When the core support is missing, the proper question is still: What is the evidence?</x:v>
       </x:c>
       <x:c r="N36" t="str">
-        <x:v>The anonymous affidavit circulated after the September 2024 ABC debate was treated by many users as explosive proof of moderator collusion even though the central accusations were not substantiated.</x:v>
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
       </x:c>
       <x:c r="O36" t="str">
-        <x:v>Public arguments about crime, immigration, vaccines, and election administration often begin with unsupported declarations that function rhetorically as if they were already established facts.</x:v>
-      </x:c>
-      <x:c r="P36" t="str"/>
-      <x:c r="Q36" t="str"/>
-      <x:c r="R36" t="str"/>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P36" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="Q36" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
+      <x:c r="R36" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
       <x:c r="S36" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1961,14 +2171,20 @@
         <x:v>For rare conditions or rare events, even very accurate tests can generate more false positives than true positives. The missing question is not just 'How accurate is the test?' but 'How common is the condition before the test is applied?'</x:v>
       </x:c>
       <x:c r="N37" t="str">
-        <x:v>Discussion of noncitizen voting in the 2024 election often highlighted a handful of cases while skipping the base rate: tens of millions of lawful ballots were cast, so isolated cases do not by themselves show a widespread system-level problem.</x:v>
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
       <x:c r="O37" t="str">
-        <x:v>Fraud detection, medical screening, and predictive-policing tools can sound highly reliable in percentage terms while still misclassifying large numbers of people when the targeted event is rare.</x:v>
-      </x:c>
-      <x:c r="P37" t="str"/>
-      <x:c r="Q37" t="str"/>
-      <x:c r="R37" t="str"/>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="P37" t="str">
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="Q37" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R37" t="str">
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
       <x:c r="S37" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2006,14 +2222,20 @@
         <x:v>Circularity can be obvious, but it is often hidden behind rewording, loaded descriptions, or a chain of claims that loops back to the start. The argument feels like support has been offered when the conclusion has only been restated.</x:v>
       </x:c>
       <x:c r="N38" t="str">
-        <x:v>Conspiracy-style reasoning often treats the absence of confirming evidence as proof that the conspiracy is powerful enough to hide the evidence, which assumes the conclusion inside the explanation.</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O38" t="str">
-        <x:v>Debates about 'real journalism' or 'real science' sometimes define the trustworthy outlet or institution as whichever one already agrees with the speaker's preferred view.</x:v>
-      </x:c>
-      <x:c r="P38" t="str"/>
-      <x:c r="Q38" t="str"/>
-      <x:c r="R38" t="str"/>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P38" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q38" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R38" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S38" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2049,14 +2271,20 @@
         <x:v>Even if a group tendency were real, it would not eliminate the need for evidence about the particular person under discussion.</x:v>
       </x:c>
       <x:c r="N39" t="str">
-        <x:v>After scandals in policing, finance, or clergy, critics sometimes assume any individual in the profession personally shares the worst traits of the institution.</x:v>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="O39" t="str">
-        <x:v>Online discourse often treats party label, employer, or religious affiliation as if it were enough to prove what a specific person believes or will do.</x:v>
-      </x:c>
-      <x:c r="P39" t="str"/>
-      <x:c r="Q39" t="str"/>
-      <x:c r="R39" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P39" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="Q39" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="R39" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S39" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2092,14 +2320,20 @@
         <x:v>A flattering stereotype is still a stereotype. Group membership can create a first impression, but it does not establish the individual's actual record.</x:v>
       </x:c>
       <x:c r="N40" t="str">
-        <x:v>Prestige effects often lead audiences to assume that anyone from a famous university or respected nonprofit is trustworthy even outside their area of expertise.</x:v>
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="O40" t="str">
-        <x:v>Voters sometimes infer that a candidate from a reform organization must be personally honest before examining the candidate's own conduct.</x:v>
-      </x:c>
-      <x:c r="P40" t="str"/>
-      <x:c r="Q40" t="str"/>
-      <x:c r="R40" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P40" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="Q40" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R40" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S40" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2137,14 +2371,20 @@
         <x:v>Repair work creates visible activity, but it mainly restores value that was lost. The missing comparison is what households, firms, insurers, and governments could have done with those same resources if the damage had not occurred.</x:v>
       </x:c>
       <x:c r="N41" t="str">
-        <x:v>After Hurricanes Helene and Milton in October 2024, some commentary emphasized reconstruction jobs and spending while downplaying the destroyed homes, shuttered businesses, and other uses those resources would have supported.</x:v>
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
       </x:c>
       <x:c r="O41" t="str">
-        <x:v>Cyberattacks, vandalism, and infrastructure failures are sometimes framed as hidden economic stimulus because repairs employ people, even though the spending mainly compensates for an avoidable loss.</x:v>
-      </x:c>
-      <x:c r="P41" t="str"/>
-      <x:c r="Q41" t="str"/>
-      <x:c r="R41" t="str"/>
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+      </x:c>
+      <x:c r="P41" t="str">
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
+      <x:c r="Q41" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R41" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
       <x:c r="S41" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2184,14 +2424,20 @@
         <x:v>Cherry picking can involve hand-picked dates, unusual baselines, isolated anecdotes, or a single study taken out of a larger research picture. The defect is not using examples, but using a biased sample as if it were representative.</x:v>
       </x:c>
       <x:c r="N42" t="str">
-        <x:v>After the September 10, 2024 Harris-Trump debate, both campaigns highlighted only the slices of jobs and manufacturing statistics that favored their own record while skipping the broader timeline.</x:v>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="O42" t="str">
-        <x:v>Climate arguments often choose a starting year with an unusually hot or cool baseline so that a short graph looks flat or dramatic even when the longer record points elsewhere.</x:v>
-      </x:c>
-      <x:c r="P42" t="str"/>
-      <x:c r="Q42" t="str"/>
-      <x:c r="R42" t="str"/>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="P42" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
+      <x:c r="Q42" t="str">
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+      </x:c>
+      <x:c r="R42" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
       <x:c r="S42" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2231,14 +2477,20 @@
         <x:v>Older views can be wrong, but age alone neither refutes nor confirms them. The real question is whether the reasoning survives scrutiny.</x:v>
       </x:c>
       <x:c r="N43" t="str">
-        <x:v>Social-media arguments often dismiss older religious, philosophical, or literary texts as worthless simply because they come from a less enlightened era, skipping the actual argument.</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O43" t="str">
-        <x:v>People also dismiss pre-digital scholarship wholesale as outdated while still relying on concepts, institutions, and moral categories that earlier thinkers helped shape.</x:v>
-      </x:c>
-      <x:c r="P43" t="str"/>
-      <x:c r="Q43" t="str"/>
-      <x:c r="R43" t="str"/>
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="P43" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="Q43" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="R43" t="str">
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+      </x:c>
       <x:c r="S43" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2278,14 +2530,20 @@
         <x:v>Circular dynamics can be real, but identifying a loop does not show that the loop is unstoppable or that breaking one link would guarantee the hoped-for outcome. Further evidence is still needed.</x:v>
       </x:c>
       <x:c r="N44" t="str">
-        <x:v>Job markets sometimes create genuine experience loops, but it is still a mistake to assume that every applicant locked out by the loop would necessarily succeed if only one employer made an exception.</x:v>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O44" t="str">
-        <x:v>Commentators often say a platform is influential because everyone talks about it and everyone talks about it because it is influential, using the loop itself as if it settled the argument.</x:v>
-      </x:c>
-      <x:c r="P44" t="str"/>
-      <x:c r="Q44" t="str"/>
-      <x:c r="R44" t="str"/>
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="P44" t="str">
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="Q44" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="R44" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
       <x:c r="S44" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2325,14 +2583,20 @@
         <x:v>Parts can interact in ways that change the result at the larger scale. What is beneficial, efficient, or true locally may not stay that way globally.</x:v>
       </x:c>
       <x:c r="N45" t="str">
-        <x:v>A company may assume that because every team is cutting costs responsibly, the organization as a whole will thrive, even though simultaneous cuts can gut the shared systems the teams depend on.</x:v>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O45" t="str">
-        <x:v>In policy debates, people often assume that what is prudent for one household, firm, or voter must be prudent for the entire economy or democracy at once.</x:v>
-      </x:c>
-      <x:c r="P45" t="str"/>
-      <x:c r="Q45" t="str"/>
-      <x:c r="R45" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P45" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q45" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="R45" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S45" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2368,14 +2632,20 @@
         <x:v>Confidence can track expertise, but it can also track charisma, identity, adrenaline, fear, or repeated exposure to a claim. Certainty is a psychological state, not a built-in proof.</x:v>
       </x:c>
       <x:c r="N46" t="str">
-        <x:v>The anonymous ABC debate affidavit spread partly because influential accounts amplified it with extraordinary certainty before any reliable verification had appeared.</x:v>
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="O46" t="str">
-        <x:v>In arguments about AI consciousness, election fraud, religion, and wellness, people often present their felt certainty as if it were itself a kind of evidence rather than something that also needs checking.</x:v>
-      </x:c>
-      <x:c r="P46" t="str"/>
-      <x:c r="Q46" t="str"/>
-      <x:c r="R46" t="str"/>
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="P46" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="Q46" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="R46" t="str">
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
       <x:c r="S46" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2413,14 +2683,20 @@
         <x:v>Adding conditions never makes a claim more probable than a broader version of that same claim. Extra detail can make a story feel more representative while making it statistically less likely.</x:v>
       </x:c>
       <x:c r="N47" t="str">
-        <x:v>Political profiling often mistakes a vivid stereotype for probability, assuming that a person matching one trait is more likely to match an even narrower bundle of traits as well.</x:v>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="O47" t="str">
-        <x:v>AI narratives sometimes suggest that because a model appears articulate, it is more likely to be both highly capable and aligned than merely capable, even though the conjunction is narrower.</x:v>
-      </x:c>
-      <x:c r="P47" t="str"/>
-      <x:c r="Q47" t="str"/>
-      <x:c r="R47" t="str"/>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P47" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="Q47" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R47" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
       <x:c r="S47" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2462,14 +2738,20 @@
         <x:v>Shortening a quote is not automatically deceptive. The fallacy appears when the omitted context would materially change how a fair reader understands the statement.</x:v>
       </x:c>
       <x:c r="N48" t="str">
-        <x:v>Edited debate clips, viral subtitled videos, and quote-card politics in 2024 regularly removed the surrounding setup, qualifier, or punchline that made the original meaning very different.</x:v>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="O48" t="str">
-        <x:v>Public figures and partisans often quote one alarming sentence from a report, study, or speech while cutting the lines that immediately limit, explain, or even reverse the apparent claim.</x:v>
-      </x:c>
-      <x:c r="P48" t="str"/>
-      <x:c r="Q48" t="str"/>
-      <x:c r="R48" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P48" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="Q48" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="R48" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
       <x:c r="S48" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2509,14 +2791,20 @@
         <x:v>Many real concepts come in degrees. Vagueness at the boundary does not make the broader concept meaningless or unusable.</x:v>
       </x:c>
       <x:c r="N49" t="str">
-        <x:v>Arguments about misinformation, bias, wealth, addiction, and consciousness often demand an impossible razor-sharp line and then pretend the lack of that line defeats the concept altogether.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O49" t="str">
-        <x:v>In everyday disputes, someone may deny that a delay was 'too long' or a fee was 'too high' simply because no exact threshold was announced in advance.</x:v>
-      </x:c>
-      <x:c r="P49" t="str"/>
-      <x:c r="Q49" t="str"/>
-      <x:c r="R49" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P49" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="Q49" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="R49" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
       <x:c r="S49" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2554,14 +2842,20 @@
         <x:v>Correlations matter because they can reveal patterns worth investigating. The fallacy is jumping straight from 'these moved together' to 'this caused that' without checking mechanisms, timing, controls, or alternative explanations.</x:v>
       </x:c>
       <x:c r="N50" t="str">
-        <x:v>Claims about teen mental health and social media often move too quickly from parallel trend lines to a settled single-cause story, even though researchers still debate the size, direction, and mechanisms of the effect.</x:v>
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="O50" t="str">
-        <x:v>Political messaging about crime, immigration, inflation, or schooling frequently points to two trends moving together and treats that alone as proof of causation.</x:v>
-      </x:c>
-      <x:c r="P50" t="str"/>
-      <x:c r="Q50" t="str"/>
-      <x:c r="R50" t="str"/>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="P50" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="Q50" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="R50" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
       <x:c r="S50" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2599,14 +2893,20 @@
         <x:v>Definitions can clarify usage, but they do not settle the underlying issue by fiat. Rewording a problem is not the same as answering it.</x:v>
       </x:c>
       <x:c r="N51" t="str">
-        <x:v>Culture-war debates often define words like 'freedom,' 'woman,' 'democracy,' or 'terrorism' in ways that quietly smuggle the desired conclusion into the starting point.</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O51" t="str">
-        <x:v>Moral and political disputes frequently collapse into dictionary wars where one side pretends that owning the label settles the argument.</x:v>
-      </x:c>
-      <x:c r="P51" t="str"/>
-      <x:c r="Q51" t="str"/>
-      <x:c r="R51" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P51" t="str">
+        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+      </x:c>
+      <x:c r="Q51" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R51" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
       <x:c r="S51" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2638,14 +2938,20 @@
         <x:v>Mechanisms matter, but evidence can justify belief before the full causal story is finished. Observation often outruns explanation.</x:v>
       </x:c>
       <x:c r="N52" t="str">
-        <x:v>Public disputes about climate, evolution, and health regularly treat unresolved details in the mechanism as if they erased the larger evidential picture.</x:v>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O52" t="str">
-        <x:v>Research on AI transcription errors in 2024 showed that systems were inventing statements people never said; even before every technical cause was nailed down, the pattern itself was already evidence of a real reliability problem.</x:v>
-      </x:c>
-      <x:c r="P52" t="str"/>
-      <x:c r="Q52" t="str"/>
-      <x:c r="R52" t="str"/>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="P52" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="Q52" t="str">
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
+      <x:c r="R52" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S52" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2685,14 +2991,20 @@
         <x:v>Sometimes counterevidence matters, but the default burden still sits with the person making the substantive claim. Lack of disproof is not the same as proof.</x:v>
       </x:c>
       <x:c r="N53" t="str">
-        <x:v>Conspiracy claims about noncitizen voting, ballot destruction, or machine tampering often survive by demanding that every rumor be individually disproved rather than by presenting strong evidence that the conspiracy exists.</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O53" t="str">
-        <x:v>Miracle, UFO, and paranormal arguments frequently say skeptics must show exactly what happened in each case, as though the claimant had no burden until that impossible task is finished.</x:v>
-      </x:c>
-      <x:c r="P53" t="str"/>
-      <x:c r="Q53" t="str"/>
-      <x:c r="R53" t="str"/>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P53" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
+      <x:c r="Q53" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="R53" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S53" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2726,14 +3038,20 @@
         <x:v>Responsible belief often comes in degrees. Treating confidence as all-or-nothing hides uncertainty, nuance, and the actual strength of the evidence.</x:v>
       </x:c>
       <x:c r="N54" t="str">
-        <x:v>Debates about God, UFOs, AI consciousness, and election fraud often demand yes-or-no declarations even when the intellectually honest position is conditional, partial, or still under revision.</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O54" t="str">
-        <x:v>Culture-war exchanges frequently treat probabilistic language such as 'unlikely,' 'not yet shown,' or 'some evidence but not enough' as weakness rather than as proper calibration.</x:v>
-      </x:c>
-      <x:c r="P54" t="str"/>
-      <x:c r="Q54" t="str"/>
-      <x:c r="R54" t="str"/>
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
+      <x:c r="P54" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q54" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="R54" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
       <x:c r="S54" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2767,14 +3085,20 @@
         <x:v>A remote hypothetical can still be useful when the issue is whether a rule really holds without exception. Improbable cases often expose hidden limits in principles that sounded absolute.</x:v>
       </x:c>
       <x:c r="N55" t="str">
-        <x:v>Arguments about free speech, self-defense, abortion, lying, and triage often reject hard edge cases simply because they are uncomfortable, even though those cases are precisely what test universal rules.</x:v>
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="O55" t="str">
-        <x:v>Policy debates about AI safety and biosecurity sometimes wave away low-probability scenarios too quickly, even when the whole argument concerns whether a system is robust under stress.</x:v>
-      </x:c>
-      <x:c r="P55" t="str"/>
-      <x:c r="Q55" t="str"/>
-      <x:c r="R55" t="str"/>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="P55" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="Q55" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R55" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S55" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2812,14 +3136,20 @@
         <x:v>One route to a conclusion does not have to be the only route. The absence of one sufficient condition does not automatically remove every other possible basis.</x:v>
       </x:c>
       <x:c r="N56" t="str">
-        <x:v>Debates about expertise often assume that if a source lacks one credential or prestige marker, there can be no meaningful evidence at all in what it says.</x:v>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O56" t="str">
-        <x:v>In everyday arguments, people often assume that if the ideal cause is absent, the observed effect cannot still arise through another path.</x:v>
-      </x:c>
-      <x:c r="P56" t="str"/>
-      <x:c r="Q56" t="str"/>
-      <x:c r="R56" t="str"/>
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P56" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q56" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="R56" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
       <x:c r="S56" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2857,14 +3187,20 @@
         <x:v>Some concepts only make sense against their correlative opposite. Erasing the contrast does not answer the accusation; it changes the meaning of the term.</x:v>
       </x:c>
       <x:c r="N57" t="str">
-        <x:v>Public arguments sometimes say a decision cannot count as censorship unless it was total state control, effectively denying any middle range where the term usefully applies.</x:v>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O57" t="str">
-        <x:v>Debates about betrayal, fraud, or coercion often narrow the term so drastically that almost no real case can qualify.</x:v>
-      </x:c>
-      <x:c r="P57" t="str"/>
-      <x:c r="Q57" t="str"/>
-      <x:c r="R57" t="str"/>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P57" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q57" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R57" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S57" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2904,14 +3240,20 @@
         <x:v>A whole can have properties its parts do not share equally. Group-level success, size, reputation, or wealth does not automatically distribute itself down to each component.</x:v>
       </x:c>
       <x:c r="N58" t="str">
-        <x:v>People often infer that because a country is rich, any given citizen must be comfortable, skipping inequality, regional gaps, and individual circumstance.</x:v>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O58" t="str">
-        <x:v>A popular movement, successful company, or prestigious institution can still contain weak teams, poor ideas, or underfunded units.</x:v>
-      </x:c>
-      <x:c r="P58" t="str"/>
-      <x:c r="Q58" t="str"/>
-      <x:c r="R58" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P58" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q58" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R58" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S58" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2953,14 +3295,20 @@
         <x:v>Aggregate data can be useful, but it does not tell you where any one individual falls within the distribution. Group averages do not erase overlap, variation, or outliers.</x:v>
       </x:c>
       <x:c r="N59" t="str">
-        <x:v>Zip-code analytics, polling blocs, and demographic summaries are often treated as if they gave a direct reading of the motives or traits of each person inside the category.</x:v>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="O59" t="str">
-        <x:v>Political commentary frequently talks as if 'suburban women,' 'young men,' or 'college voters' were internally uniform rather than broad, heterogeneous groups.</x:v>
-      </x:c>
-      <x:c r="P59" t="str"/>
-      <x:c r="Q59" t="str"/>
-      <x:c r="R59" t="str"/>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P59" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="Q59" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="R59" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S59" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2992,14 +3340,20 @@
         <x:v>Not every conversation requires a full essay, but a real refutation still has to point to some error in reasoning, evidence, or interpretation. Mere dismissal is not argument.</x:v>
       </x:c>
       <x:c r="N60" t="str">
-        <x:v>Online fights about elections, Israel and Gaza, climate, and AI often rely on 'debunked' as a performance word rather than as a pointer to the actual evidence.</x:v>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="O60" t="str">
-        <x:v>In fast-moving social media disputes, people often treat tone, certainty, and pile-on consensus as if they were enough to count as refutation.</x:v>
-      </x:c>
-      <x:c r="P60" t="str"/>
-      <x:c r="Q60" t="str"/>
-      <x:c r="R60" t="str"/>
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
+      <x:c r="P60" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="Q60" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="R60" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S60" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3035,14 +3389,20 @@
         <x:v>Beliefs can change mood, confidence, behavior, pain perception, and group cohesion regardless of whether their object exists. The benefits of belief do not by themselves settle the ontology.</x:v>
       </x:c>
       <x:c r="N61" t="str">
-        <x:v>Raw milk, supplement, and alternative-health advocates often point to the felt benefits reported by believers while skipping the role of expectation, placebo effects, and other background changes.</x:v>
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="O61" t="str">
-        <x:v>Arguments that religion must be true because believers report comfort, purpose, or improved well-being often confuse the power of belief with evidence for the reality of the object believed in.</x:v>
-      </x:c>
-      <x:c r="P61" t="str"/>
-      <x:c r="Q61" t="str"/>
-      <x:c r="R61" t="str"/>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="P61" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q61" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="R61" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S61" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3078,14 +3438,20 @@
         <x:v>Equivocation often works because the same word is doing two jobs at once. The surface grammar stays stable while the meaning shifts underneath.</x:v>
       </x:c>
       <x:c r="N62" t="str">
-        <x:v>Debates over content moderation regularly equivocate between censorship by the state and moderation decisions by private platforms, as if both were the same kind of speech restriction.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O62" t="str">
-        <x:v>Public discussion of AI often slides between thin technical meanings of words such as 'reasoning,' 'understanding,' or 'hallucination' and thicker human meanings, which makes claims sound stronger than the evidence warrants.</x:v>
-      </x:c>
-      <x:c r="P62" t="str"/>
-      <x:c r="Q62" t="str"/>
-      <x:c r="R62" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P62" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="Q62" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R62" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
       <x:c r="S62" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3121,14 +3487,20 @@
         <x:v>The argument trades on the prestige or emotional force of the stronger meaning while relying on the thinner meaning when challenged.</x:v>
       </x:c>
       <x:c r="N63" t="str">
-        <x:v>Public arguments about censorship often slide from the general fact that content was moderated to the much stronger charge that it was censored in the same sense as state suppression.</x:v>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O63" t="str">
-        <x:v>AI marketing repeatedly benefits from equivocation between technical terms such as 'learn,' 'reason,' or 'understand' and their thicker human meanings.</x:v>
-      </x:c>
-      <x:c r="P63" t="str"/>
-      <x:c r="Q63" t="str"/>
-      <x:c r="R63" t="str"/>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P63" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q63" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="R63" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S63" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3164,14 +3536,20 @@
         <x:v>Words change through use. Present meaning is set by current linguistic convention, not by the oldest recoverable ancestor of the term.</x:v>
       </x:c>
       <x:c r="N64" t="str">
-        <x:v>Culture-war and identity debates often turn into fights over what labels 'really mean' based on older usage rather than on how the community currently uses them.</x:v>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O64" t="str">
-        <x:v>People sometimes defend or condemn a term by appealing to its root language while ignoring the fact that social meaning has moved far beyond the origin.</x:v>
-      </x:c>
-      <x:c r="P64" t="str"/>
-      <x:c r="Q64" t="str"/>
-      <x:c r="R64" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P64" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="Q64" t="str">
+        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+      </x:c>
+      <x:c r="R64" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
       <x:c r="S64" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3207,14 +3585,20 @@
         <x:v>Two exclusions do not by themselves tell you how the remaining categories relate. Keeping groups apart is not the same as establishing a valid connection among them.</x:v>
       </x:c>
       <x:c r="N65" t="str">
-        <x:v>Identity arguments sometimes pile up statements about what two groups are not and then pretend that the missing positive relation has somehow been proved.</x:v>
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O65" t="str">
-        <x:v>This form often hides inside rhetorical contrasts where speakers rely on the sound of elimination rather than a genuine logical bridge.</x:v>
-      </x:c>
-      <x:c r="P65" t="str"/>
-      <x:c r="Q65" t="str"/>
-      <x:c r="R65" t="str"/>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P65" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q65" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R65" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
       <x:c r="S65" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3250,14 +3634,20 @@
         <x:v>Universal statements can be true even when the class is empty. Talking about all members of a category does not guarantee that there are any members to begin with.</x:v>
       </x:c>
       <x:c r="N66" t="str">
-        <x:v>Arguments about 'the average user,' 'the typical elite,' or 'the real moderate voter' sometimes slip from a hypothetical category into the assumption that a concrete instance must exist.</x:v>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="O66" t="str">
-        <x:v>Formal and theological debates alike often move too quickly from what would be true if something existed to the claim that it therefore does exist.</x:v>
-      </x:c>
-      <x:c r="P66" t="str"/>
-      <x:c r="Q66" t="str"/>
-      <x:c r="R66" t="str"/>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P66" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="Q66" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R66" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S66" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3295,14 +3685,20 @@
         <x:v>A loaded question can force a false choice because any direct answer seems to concede what the question improperly assumed. The first task is often to challenge the hidden premise, not to answer on its terms.</x:v>
       </x:c>
       <x:c r="N67" t="str">
-        <x:v>Debates about religion, politics, and gender often turn on questions that quietly presuppose bad faith, delusion, or malicious intent before any of that has been shown.</x:v>
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="O67" t="str">
-        <x:v>Interviewers and posters sometimes frame questions so that merely engaging already concedes the accusation, especially in culture-war exchanges built for clipping and outrage.</x:v>
-      </x:c>
-      <x:c r="P67" t="str"/>
-      <x:c r="Q67" t="str"/>
-      <x:c r="R67" t="str"/>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="P67" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="Q67" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="R67" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
       <x:c r="S67" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3340,14 +3736,20 @@
         <x:v>Some predicates are necessary only relative to a present state or definition. That necessity does not magically extend across time, possibility, or changed conditions.</x:v>
       </x:c>
       <x:c r="N68" t="str">
-        <x:v>People sometimes move from 'this rule currently defines the category' to 'therefore the category could never be revised or altered,' confusing present convention with fixed necessity.</x:v>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O68" t="str">
-        <x:v>In institutional debates, a temporary legal or procedural status is often spoken of as if it were an immutable fact about what can never happen.</x:v>
-      </x:c>
-      <x:c r="P68" t="str"/>
-      <x:c r="Q68" t="str"/>
-      <x:c r="R68" t="str"/>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P68" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q68" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R68" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S68" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3385,14 +3787,20 @@
         <x:v>Analogies can clarify unfamiliar ideas, but they prove very little unless the shared features are actually relevant to the conclusion being drawn.</x:v>
       </x:c>
       <x:c r="N69" t="str">
-        <x:v>Debates about AI frequently compare models to children, interns, parrots, or brains, then carry over conclusions from the analogy that the underlying system may not support.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O69" t="str">
-        <x:v>Fiscal debates often compare a national budget to a household budget; the analogy can illuminate some constraints but breaks down when it is treated as a full map of macroeconomics.</x:v>
-      </x:c>
-      <x:c r="P69" t="str"/>
-      <x:c r="Q69" t="str"/>
-      <x:c r="R69" t="str"/>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="P69" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="Q69" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R69" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
       <x:c r="S69" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3430,14 +3838,20 @@
         <x:v>Source quality matters, but only if the source is real, relevant, and represented fairly. A false attribution can make weak claims feel borrowed from a stronger authority than they actually have.</x:v>
       </x:c>
       <x:c r="N70" t="str">
-        <x:v>The anonymous affidavit circulated after the September 2024 ABC debate was amplified as if it were a verified insider source even though the core allegations were not authenticated.</x:v>
+        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
       </x:c>
       <x:c r="O70" t="str">
-        <x:v>Viral quote cards and screenshot posts often attach dramatic claims to scientists, judges, or agencies who never said them, counting on readers to trust the label instead of checking the source.</x:v>
-      </x:c>
-      <x:c r="P70" t="str"/>
-      <x:c r="Q70" t="str"/>
-      <x:c r="R70" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P70" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="Q70" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R70" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
       <x:c r="S70" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3475,14 +3889,20 @@
         <x:v>Fairness does not always require symmetry. When one side is supported by overwhelming evidence and the other is weak, fringe, or fabricated, equal presentation can mislead an audience about the actual state of the issue.</x:v>
       </x:c>
       <x:c r="N71" t="str">
-        <x:v>Coverage of climate change, vaccine safety, and election administration often becomes misleading when fringe claims are presented as if they stand on equal footing with the evidential consensus.</x:v>
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
       <x:c r="O71" t="str">
-        <x:v>Public moderators sometimes treat a polished unsupported claim and a well-supported cautious claim as equivalent contributions simply because both parties are speaking confidently.</x:v>
-      </x:c>
-      <x:c r="P71" t="str"/>
-      <x:c r="Q71" t="str"/>
-      <x:c r="R71" t="str"/>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="P71" t="str">
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
+      <x:c r="Q71" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="R71" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
       <x:c r="S71" t="str">
         <x:v>added-2026-completeness-pass</x:v>
       </x:c>
@@ -3520,14 +3940,20 @@
         <x:v>Disagreement does not imply that the truth is halfway between the parties. One side may simply be much more right than the other.</x:v>
       </x:c>
       <x:c r="N72" t="str">
-        <x:v>Coverage of climate, public health, and election integrity can slide into 'both sides' framing that treats consensus and fringe denial as if splitting the difference were balanced or fair.</x:v>
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="O72" t="str">
-        <x:v>In personal and workplace disputes, people often assume each side must be equally at fault, even when the evidence is lopsided.</x:v>
-      </x:c>
-      <x:c r="P72" t="str"/>
-      <x:c r="Q72" t="str"/>
-      <x:c r="R72" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P72" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q72" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="R72" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
       <x:c r="S72" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3565,14 +3991,20 @@
         <x:v>The pressure comes from pretending that a complex decision has only two doors. Sometimes the omitted alternatives are compromises, phased approaches, or the option of rejecting the framing altogether.</x:v>
       </x:c>
       <x:c r="N73" t="str">
-        <x:v>In 2024 immigration debates, many campaign messages reduced the issue to a choice between mass deportation and open borders, leaving out enforcement, asylum reform, and legal migration policy.</x:v>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="O73" t="str">
-        <x:v>School discussions about generative AI are often framed as either banning it completely or surrendering all meaningful learning, even though classrooms can set narrower rules for citation, drafting, and acceptable assistance.</x:v>
-      </x:c>
-      <x:c r="P73" t="str"/>
-      <x:c r="Q73" t="str"/>
-      <x:c r="R73" t="str"/>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="P73" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="Q73" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="R73" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S73" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3610,14 +4042,20 @@
         <x:v>Two things can share some features without being equal in scale, intent, risk, or moral significance. The fallacy appears when a superficial resemblance is used to flatten those differences into sameness.</x:v>
       </x:c>
       <x:c r="N74" t="str">
-        <x:v>Political debate often treats an ordinary gaffe and a deliberate disinformation effort as if both were just the same kind of 'spin.'</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O74" t="str">
-        <x:v>Arguments about war, protest, and public ethics often compare acts that differ radically in magnitude or purpose while speaking as if the moral ledger is now even.</x:v>
-      </x:c>
-      <x:c r="P74" t="str"/>
-      <x:c r="Q74" t="str"/>
-      <x:c r="R74" t="str"/>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P74" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="Q74" t="str">
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+      </x:c>
+      <x:c r="R74" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S74" t="str">
         <x:v>added-2026-completeness-pass</x:v>
       </x:c>
@@ -3659,14 +4097,20 @@
         <x:v>Real uncertainty exists, and sometimes compromise is appropriate. The fallacy appears when manufactured neutrality is used to protect a losing claim from the consequences of the evidence.</x:v>
       </x:c>
       <x:c r="N75" t="str">
-        <x:v>Public arguments about evolution, election claims, and medical misinformation sometimes ask audiences to treat both sides as equally plausible even after the evidential balance is lopsided.</x:v>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="O75" t="str">
-        <x:v>In online debate culture, a retreat into 'everyone has their own truth' often appears right after a concrete factual claim has gone badly for one side.</x:v>
-      </x:c>
-      <x:c r="P75" t="str"/>
-      <x:c r="Q75" t="str"/>
-      <x:c r="R75" t="str"/>
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
+      <x:c r="P75" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
+      <x:c r="Q75" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="R75" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
       <x:c r="S75" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3706,14 +4150,20 @@
         <x:v>Generalization is unavoidable, but it has to be scaled to the quality, size, and representativeness of the evidence. The problem is not generalizing at all; it is generalizing too aggressively.</x:v>
       </x:c>
       <x:c r="N76" t="str">
-        <x:v>Viral anecdotes about migrants, students, police, or AI tools often get inflated into sweeping claims about entire groups or systems after only a handful of cases.</x:v>
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
       <x:c r="O76" t="str">
-        <x:v>Election and media arguments routinely take one error, one clip, or one scandal as proof that the whole institution always behaves the same way.</x:v>
-      </x:c>
-      <x:c r="P76" t="str"/>
-      <x:c r="Q76" t="str"/>
-      <x:c r="R76" t="str"/>
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+      </x:c>
+      <x:c r="P76" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="Q76" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R76" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
       <x:c r="S76" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3747,14 +4197,20 @@
         <x:v>Reasoning from an assumption to test its implications is not the same as endorsing the assumption.</x:v>
       </x:c>
       <x:c r="N77" t="str">
-        <x:v>Reductio arguments in theology, AI, and politics are often misread as confessions rather than as tests of what would follow if the other side's claim were granted.</x:v>
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="O77" t="str">
-        <x:v>Debates stall when a conditional claim such as 'even if you are right, the consequence would still be unacceptable' is treated as if it were a statement of belief.</x:v>
-      </x:c>
-      <x:c r="P77" t="str"/>
-      <x:c r="Q77" t="str"/>
-      <x:c r="R77" t="str"/>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="P77" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q77" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="R77" t="str">
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+      </x:c>
       <x:c r="S77" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3790,14 +4246,20 @@
         <x:v>The surface wording can make the argument sound tidy, but the hidden term shift breaks the structure. A reused word is not enough; it has to keep the same meaning.</x:v>
       </x:c>
       <x:c r="N78" t="str">
-        <x:v>Public arguments often slide between technical and ordinary meanings of words like 'theory,' 'freedom,' 'bias,' or 'intelligence,' then pretend the resulting syllogism is valid.</x:v>
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O78" t="str">
-        <x:v>Because the same label can carry prestige in one context and a thinner meaning in another, term shifts often smuggle in conclusions the premises did not support.</x:v>
-      </x:c>
-      <x:c r="P78" t="str"/>
-      <x:c r="Q78" t="str"/>
-      <x:c r="R78" t="str"/>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P78" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="Q78" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R78" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S78" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3837,14 +4299,20 @@
         <x:v>Random sequences naturally contain streaks. When the events are truly independent, the next event does not remember the last one.</x:v>
       </x:c>
       <x:c r="N79" t="str">
-        <x:v>People sometimes feel that after many routine flights or medical screenings in a row, a disaster or diagnosis is somehow 'due,' even though independent risks do not balance themselves that way.</x:v>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="O79" t="str">
-        <x:v>In gambling and investing language, talk of a roulette table or slot machine being 'ready to pay out' often confuses a streaky pattern with a real shift in odds.</x:v>
-      </x:c>
-      <x:c r="P79" t="str"/>
-      <x:c r="Q79" t="str"/>
-      <x:c r="R79" t="str"/>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="P79" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="Q79" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R79" t="str">
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+      </x:c>
       <x:c r="S79" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3884,14 +4352,20 @@
         <x:v>Origins can matter when they reveal bias, incentives, or reliability concerns. The fallacy appears when origin is treated as enough to settle the issue without examining the claim itself.</x:v>
       </x:c>
       <x:c r="N80" t="str">
-        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O80" t="str">
-        <x:v>In cultural and religious arguments, a practice or symbol is often condemned solely because of its historical roots, even when the live question is what it means or does now.</x:v>
-      </x:c>
-      <x:c r="P80" t="str"/>
-      <x:c r="Q80" t="str"/>
-      <x:c r="R80" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P80" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="Q80" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R80" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
       <x:c r="S80" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3933,14 +4407,20 @@
         <x:v>The problem is not moving from sample to population; all induction does that. The problem is pretending a weak or unrepresentative sample carries more weight than it does.</x:v>
       </x:c>
       <x:c r="N81" t="str">
-        <x:v>A single viral video of a fight, theft, or protest is often used online as if it reveals what a whole city, campus, or demographic group is like.</x:v>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="O81" t="str">
-        <x:v>Election commentary frequently treats one poll, one county, or one diner focus group as proof of a national shift, even when the broader polling picture is mixed.</x:v>
-      </x:c>
-      <x:c r="P81" t="str"/>
-      <x:c r="Q81" t="str"/>
-      <x:c r="R81" t="str"/>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="P81" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="Q81" t="str">
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+      </x:c>
+      <x:c r="R81" t="str">
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
       <x:c r="S81" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3976,14 +4456,20 @@
         <x:v>Hindsight compresses uncertainty and highlights the clues that mattered. Real historical agents were working inside a noisier, more limited information environment.</x:v>
       </x:c>
       <x:c r="N82" t="str">
-        <x:v>People often imagine they would easily have rejected past medical myths, empires, or moral blind spots, underestimating how strongly institutions and available evidence shape belief.</x:v>
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
       <x:c r="O82" t="str">
-        <x:v>Post-crisis commentary regularly rewrites messy contingencies into obvious warning signs that were supposedly plain to everyone at the time.</x:v>
-      </x:c>
-      <x:c r="P82" t="str"/>
-      <x:c r="Q82" t="str"/>
-      <x:c r="R82" t="str"/>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="P82" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="Q82" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="R82" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
       <x:c r="S82" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4021,14 +4507,20 @@
         <x:v>If the inner observer can already do the job, the original explanatory problem just reappears one level down.</x:v>
       </x:c>
       <x:c r="N83" t="str">
-        <x:v>Popular neuroscience writing sometimes says that the brain 'decides' or a memory center 'knows' in ways that merely rename the puzzle rather than explain it.</x:v>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O83" t="str">
-        <x:v>Criticism of AI can do something similar when it assumes a hidden module inside the system literally understands the output in the same way a person would.</x:v>
-      </x:c>
-      <x:c r="P83" t="str"/>
-      <x:c r="Q83" t="str"/>
-      <x:c r="R83" t="str"/>
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P83" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="Q83" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R83" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
       <x:c r="S83" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4068,14 +4560,20 @@
         <x:v>Institutional labels can matter legally or practically, but they do not by themselves create truth, value, or natural kinds.</x:v>
       </x:c>
       <x:c r="N84" t="str">
-        <x:v>Markets and media often confuse approved, certified, or official with true, safe, or just.</x:v>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O84" t="str">
-        <x:v>Political rhetoric often treats whatever a legislature recognizes or forbids as automatically morally right or wrong.</x:v>
-      </x:c>
-      <x:c r="P84" t="str"/>
-      <x:c r="Q84" t="str"/>
-      <x:c r="R84" t="str"/>
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P84" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q84" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="R84" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
       <x:c r="S84" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4111,14 +4609,20 @@
         <x:v>This is not mere nuance. The problem is rhetorical double-speaking that blurs real disagreement by sliding between incompatible senses of the same label.</x:v>
       </x:c>
       <x:c r="N85" t="str">
-        <x:v>Politicians often define contested terms like 'freedom,' 'censorship,' 'riot,' 'peaceful,' or 'family values' one way for sympathetic listeners and another way when challenged by critics.</x:v>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="O85" t="str">
-        <x:v>Debates about AI, speech, and policing frequently proceed as if both camps agree until someone notices that the central term has been doing two very different jobs.</x:v>
-      </x:c>
-      <x:c r="P85" t="str"/>
-      <x:c r="Q85" t="str"/>
-      <x:c r="R85" t="str"/>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P85" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
+      <x:c r="Q85" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R85" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
       <x:c r="S85" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4154,14 +4658,20 @@
         <x:v>Excluding one group from a subset does not exclude it from the wider property attached to that subset. The conclusion reaches further than the premises license.</x:v>
       </x:c>
       <x:c r="N86" t="str">
-        <x:v>Stereotype arguments often move from 'all members of group A have trait B' and 'group C is not group A' to 'therefore group C lacks trait B,' which does not follow.</x:v>
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O86" t="str">
-        <x:v>This pattern appears when people treat one pathway to fame, corruption, risk, or success as if it were the only pathway.</x:v>
-      </x:c>
-      <x:c r="P86" t="str"/>
-      <x:c r="Q86" t="str"/>
-      <x:c r="R86" t="str"/>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P86" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="Q86" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="R86" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
       <x:c r="S86" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4195,14 +4705,20 @@
         <x:v>A claim that survives every observation unchanged may be emotionally resilient, but it has surrendered explanatory power.</x:v>
       </x:c>
       <x:c r="N87" t="str">
-        <x:v>Conspiracy systems often explain both the presence and the absence of evidence as confirmation.</x:v>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O87" t="str">
-        <x:v>Some technology hype frames both success and failure as proof that general intelligence is just around the corner.</x:v>
-      </x:c>
-      <x:c r="P87" t="str"/>
-      <x:c r="Q87" t="str"/>
-      <x:c r="R87" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P87" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="Q87" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="R87" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S87" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4238,14 +4754,20 @@
         <x:v>A comparison can be true in one narrow respect while misleading overall. The missing pieces might include quality, risk, wages, inflation, time horizon, tradeoffs, or alternative baselines.</x:v>
       </x:c>
       <x:c r="N88" t="str">
-        <x:v>Campaign arguments about the economy often isolate one metric such as gas prices, job totals, or stock indexes and treat that single comparison as if it captured the whole condition of household life.</x:v>
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
       </x:c>
       <x:c r="O88" t="str">
-        <x:v>Technology marketing frequently calls a new tool 'more productive' without clarifying productive for whom, under what workflow, at what error rate, and at what human cost.</x:v>
-      </x:c>
-      <x:c r="P88" t="str"/>
-      <x:c r="Q88" t="str"/>
-      <x:c r="R88" t="str"/>
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="P88" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q88" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R88" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
       <x:c r="S88" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4283,14 +4805,20 @@
         <x:v>A complete comparison needs a consistent baseline or a transparent weighting of tradeoffs, not a collage of unrelated best cases.</x:v>
       </x:c>
       <x:c r="N89" t="str">
-        <x:v>Consumer ads often compare each feature against whichever rival looks weakest on that feature, then announce overall superiority.</x:v>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O89" t="str">
-        <x:v>Campaign brag sheets sometimes do the same by mixing job growth, crime, housing, and graduation metrics against different jurisdictions and different years.</x:v>
-      </x:c>
-      <x:c r="P89" t="str"/>
-      <x:c r="Q89" t="str"/>
-      <x:c r="R89" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P89" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q89" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R89" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
       <x:c r="S89" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4328,14 +4856,20 @@
         <x:v>Authorial intent is not always the only thing that matters, but it is often part of the evidence. Declaring it irrelevant by default can flatten interpretation into projection.</x:v>
       </x:c>
       <x:c r="N90" t="str">
-        <x:v>Debates over constitutional language, literature, and political slogans often swing too far toward present-day interpretation while discarding what the author or framers were trying to do.</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O90" t="str">
-        <x:v>Online arguments about memes, jokes, and clips frequently ignore context and stated intent altogether, then treat the most inflammatory possible reading as the only serious one.</x:v>
-      </x:c>
-      <x:c r="P90" t="str"/>
-      <x:c r="Q90" t="str"/>
-      <x:c r="R90" t="str"/>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="P90" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="Q90" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="R90" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
       <x:c r="S90" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4373,14 +4907,20 @@
         <x:v>An ought needs a normative premise about goals, duties, or values. Facts alone do not generate that extra step.</x:v>
       </x:c>
       <x:c r="N91" t="str">
-        <x:v>Arguments about gender, family, and competition often slide from claims about what is common in nature to claims about what is therefore morally required.</x:v>
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O91" t="str">
-        <x:v>Workplace norms are regularly defended by saying they are simply how the market works, even when the moral question is precisely whether the market should work that way.</x:v>
-      </x:c>
-      <x:c r="P91" t="str"/>
-      <x:c r="Q91" t="str"/>
-      <x:c r="R91" t="str"/>
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="P91" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="Q91" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R91" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S91" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4418,14 +4958,20 @@
         <x:v>Some labels are fair descriptions, but the fallacy appears when the emotional sting of the label is doing the work that evidence and argument have not done.</x:v>
       </x:c>
       <x:c r="N92" t="str">
-        <x:v>Words like 'groomer,' 'traitor,' 'fascist,' 'woke,' 'cultist,' and 'denier' are often deployed less to clarify than to trigger a moral reaction before the argument can be examined.</x:v>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="O92" t="str">
-        <x:v>Political and religious arguments frequently pre-load the conclusion by choosing terms that make disagreement sound shameful or corrupt from the start.</x:v>
-      </x:c>
-      <x:c r="P92" t="str"/>
-      <x:c r="Q92" t="str"/>
-      <x:c r="R92" t="str"/>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P92" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="Q92" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
+      <x:c r="R92" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
       <x:c r="S92" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4459,14 +5005,20 @@
         <x:v>Many real systems change slowly at first, then rapidly, then plateau, or even reverse after a threshold.</x:v>
       </x:c>
       <x:c r="N93" t="str">
-        <x:v>Growth forecasts for social platforms often assume audience reach will keep scaling smoothly even after attention markets saturate.</x:v>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="O93" t="str">
-        <x:v>Policy debates about climate, housing, and healthcare frequently ignore the non-linear effects of bottlenecks, incentives, and behavioral feedback.</x:v>
-      </x:c>
-      <x:c r="P93" t="str"/>
-      <x:c r="Q93" t="str"/>
-      <x:c r="R93" t="str"/>
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
+      <x:c r="P93" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q93" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="R93" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
       <x:c r="S93" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4502,14 +5054,20 @@
         <x:v>New technology can displace real jobs and create painful transitions. The fallacy is the stronger claim that automation as such can only destroy work, rather than reorganize it, lower costs, create new roles, or shift labor elsewhere.</x:v>
       </x:c>
       <x:c r="N94" t="str">
-        <x:v>Debates over generative AI in 2024 often jumped straight from 'this automates part of my job' to 'therefore it will inevitably make people broadly unemployable,' skipping the more complicated evidence about substitution, augmentation, and new roles.</x:v>
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="O94" t="str">
-        <x:v>The U.S. dockworker fight over port automation in October 2024 showed why the issue is serious, but it also illustrated the need to distinguish real bargaining and transition questions from the blanket claim that productivity-enhancing technology is always socially worse.</x:v>
-      </x:c>
-      <x:c r="P94" t="str"/>
-      <x:c r="Q94" t="str"/>
-      <x:c r="R94" t="str"/>
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="P94" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
+      <x:c r="Q94" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="R94" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
       <x:c r="S94" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4545,14 +5103,20 @@
         <x:v>In ordinary factual contexts, identical referents can be substituted safely. In belief, knowledge, or perception contexts, that move can fail because the speaker's information is incomplete.</x:v>
       </x:c>
       <x:c r="N95" t="str">
-        <x:v>This fallacy shows up whenever people infer identity or non-identity from what someone knows, recognizes, or can name rather than from the underlying facts.</x:v>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="O95" t="str">
-        <x:v>Mystery, anonymity, and pseudonym debates often slide into this mistake by assuming that not knowing a description means the object cannot be the same one known under another description.</x:v>
-      </x:c>
-      <x:c r="P95" t="str"/>
-      <x:c r="Q95" t="str"/>
-      <x:c r="R95" t="str"/>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P95" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q95" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R95" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
       <x:c r="S95" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4594,14 +5158,20 @@
         <x:v>Vivid cases matter, especially when they reveal harms abstract statistics can hide. The fallacy arises when memorable exceptions are used as if they were the normal pattern.</x:v>
       </x:c>
       <x:c r="N96" t="str">
-        <x:v>The Springfield rumor gained traction partly because lurid, memorable imagery traveled faster than the dull but crucial fact that authorities found no supporting evidence.</x:v>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="O96" t="str">
-        <x:v>Viral clips of shoplifting, airplane incidents, or isolated crimes are often used to imply a general trend without the comparative data needed to show that the example is typical.</x:v>
-      </x:c>
-      <x:c r="P96" t="str"/>
-      <x:c r="Q96" t="str"/>
-      <x:c r="R96" t="str"/>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P96" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="Q96" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R96" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S96" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4641,14 +5211,20 @@
         <x:v>Standards can be refined in good faith, especially when both sides notice a weak test. The fallacy appears when the revision functions mainly to avoid conceding that the earlier standard was met.</x:v>
       </x:c>
       <x:c r="N97" t="str">
-        <x:v>Public AI debates in 2024 often moved from benchmark scores to some new test the moment a model cleared the previous bar, making 'proof' of competence permanently out of reach.</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O97" t="str">
-        <x:v>Election-conspiracy arguments often work this way: once courts, audits, and recounts address one claim, the standard shifts to a different alleged irregularity without any willingness to concede what the earlier evidence settled.</x:v>
-      </x:c>
-      <x:c r="P97" t="str"/>
-      <x:c r="Q97" t="str"/>
-      <x:c r="R97" t="str"/>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="P97" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="Q97" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="R97" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
       <x:c r="S97" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4686,14 +5262,20 @@
         <x:v>Natural things can be wonderful, harmful, neutral, or context-dependent. Arsenic, viruses, and earthquakes are natural too. The relevant questions are evidence, outcomes, and tradeoffs, not whether something sounds untouched.</x:v>
       </x:c>
       <x:c r="N98" t="str">
-        <x:v>The 2026 push to expand raw milk access often leaned on the idea that unprocessed equals healthier, despite repeated warnings from public-health officials that the safety risks are real and the claimed benefits remain unproven.</x:v>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O98" t="str">
-        <x:v>Wellness marketing routinely sells herbs, supplements, detoxes, and hormone routines by invoking nature itself as if natural origin settled the medical question.</x:v>
-      </x:c>
-      <x:c r="P98" t="str"/>
-      <x:c r="Q98" t="str"/>
-      <x:c r="R98" t="str"/>
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="P98" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="Q98" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R98" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S98" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4729,14 +5311,20 @@
         <x:v>The rational status of a claim depends on the evidence for it, not on whether someone has managed to close every imaginable contrary possibility.</x:v>
       </x:c>
       <x:c r="N99" t="str">
-        <x:v>Election, paranormal, and conspiracy claims often survive by saying 'you cannot prove it did not happen,' as if that absence of disproof supplied positive warrant.</x:v>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="O99" t="str">
-        <x:v>Skeptics can also commit the reverse mistake when they treat an unproved claim as definitively false rather than merely unestablished.</x:v>
-      </x:c>
-      <x:c r="P99" t="str"/>
-      <x:c r="Q99" t="str"/>
-      <x:c r="R99" t="str"/>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P99" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q99" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R99" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S99" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4772,14 +5360,20 @@
         <x:v>Most policies, tools, and institutions are partial fixes. The right question is often whether an option improves matters relative to feasible alternatives, not whether it achieves a flawless end state.</x:v>
       </x:c>
       <x:c r="N100" t="str">
-        <x:v>Critics of content moderation, election safeguards, AI guardrails, and climate policy often reject incremental measures on the grounds that bad cases will still exist, as if imperfection erased all value.</x:v>
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O100" t="str">
-        <x:v>Debates about public-health interventions frequently collapse into 'if it does not stop every case, it failed,' which compares reality to fantasy rather than to the available alternatives.</x:v>
-      </x:c>
-      <x:c r="P100" t="str"/>
-      <x:c r="Q100" t="str"/>
-      <x:c r="R100" t="str"/>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P100" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="Q100" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R100" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
       <x:c r="S100" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4823,14 +5417,20 @@
         <x:v>Sometimes categories do have genuine criteria. The fallacy arises when the criteria are improvised only after a counterexample appears, so the definition changes to save the claim.</x:v>
       </x:c>
       <x:c r="N101" t="str">
-        <x:v>In 2024 intraparty fights, Republicans who backed Ukraine aid or accepted the 2020 certification were often dismissed as 'not real conservatives' instead of being treated as counterexamples within conservatism.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O101" t="str">
-        <x:v>Religious and ideological arguments frequently insist that anyone whose behavior embarrasses the group was never a 'true' believer in the first place, which preserves group purity by redefinition.</x:v>
-      </x:c>
-      <x:c r="P101" t="str"/>
-      <x:c r="Q101" t="str"/>
-      <x:c r="R101" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P101" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="Q101" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="R101" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
       <x:c r="S101" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4870,14 +5470,20 @@
         <x:v>A principle can have limits, but if the exceptions swallow the rule, the apparent commitment becomes mostly decorative.</x:v>
       </x:c>
       <x:c r="N102" t="str">
-        <x:v>Public commitments to transparency, merit, or local control often vanish once they threaten a favored outcome.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O102" t="str">
-        <x:v>Organizations sometimes advertise simple values statements that become practically meaningless once the long list of carve-outs is revealed.</x:v>
-      </x:c>
-      <x:c r="P102" t="str"/>
-      <x:c r="Q102" t="str"/>
-      <x:c r="R102" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P102" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="Q102" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="R102" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
       <x:c r="S102" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4913,14 +5519,20 @@
         <x:v>Some traits do cluster more often than chance would predict, but the cluster is not a logical necessity. A familiar package can make us overread what belongs together.</x:v>
       </x:c>
       <x:c r="N103" t="str">
-        <x:v>Campaign and media narratives often assume that working-class, rural, religious, or college-educated identities come with one full political bundle attached.</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O103" t="str">
-        <x:v>People frequently expect hobbies, musical taste, fashion, or ethnicity to drag a whole associated worldview behind them even when the individual breaks the pattern.</x:v>
-      </x:c>
-      <x:c r="P103" t="str"/>
-      <x:c r="Q103" t="str"/>
-      <x:c r="R103" t="str"/>
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="P103" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="Q103" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="R103" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S103" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4960,14 +5572,20 @@
         <x:v>Personifying weather, markets, or algorithms can be a vivid metaphor, but it becomes fallacious when the metaphor is used as literal evidence.</x:v>
       </x:c>
       <x:c r="N104" t="str">
-        <x:v>People often say the algorithm hates them, loves outrage, or wants to silence them when the actual explanation is a mix of optimization rules and incentives.</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O104" t="str">
-        <x:v>News coverage sometimes treats storms, markets, or viruses as if they were moral agents taking revenge, sending messages, or rewarding virtue.</x:v>
-      </x:c>
-      <x:c r="P104" t="str"/>
-      <x:c r="Q104" t="str"/>
-      <x:c r="R104" t="str"/>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="P104" t="str">
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+      </x:c>
+      <x:c r="Q104" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="R104" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
       <x:c r="S104" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5005,14 +5623,20 @@
         <x:v>A partial improvement can still be worthwhile. The mistake is demanding perfection from one proposal when no realistic policy can eliminate the problem entirely.</x:v>
       </x:c>
       <x:c r="N105" t="str">
-        <x:v>Climate and transit proposals are often rejected because they will not solve emissions or congestion completely, as if incomplete progress counted as no progress.</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O105" t="str">
-        <x:v>Arguments about AI safety, gun policy, and public health often dismiss guardrails for failing to eliminate every bad case, rather than asking whether they would reduce harm.</x:v>
-      </x:c>
-      <x:c r="P105" t="str"/>
-      <x:c r="Q105" t="str"/>
-      <x:c r="R105" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P105" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="Q105" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R105" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
       <x:c r="S105" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5044,14 +5668,20 @@
         <x:v>Many human traits and performances come in degrees. Treating any deviation from an ideal as proof of total failure destroys the resolution needed for fair judgment.</x:v>
       </x:c>
       <x:c r="N106" t="str">
-        <x:v>Debates about media bias, moral character, and institutional trust often assume that if a person or outlet is not perfectly objective, then it is simply propaganda.</x:v>
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
       </x:c>
       <x:c r="O106" t="str">
-        <x:v>Public discussion of peace, tolerance, and fairness often ignores large improvements because some imperfection remains somewhere.</x:v>
-      </x:c>
-      <x:c r="P106" t="str"/>
-      <x:c r="Q106" t="str"/>
-      <x:c r="R106" t="str"/>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="P106" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="Q106" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="R106" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
       <x:c r="S106" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5093,14 +5723,20 @@
         <x:v>An analogy usually highlights one structural similarity, not a one-to-one mapping of every detail.</x:v>
       </x:c>
       <x:c r="N107" t="str">
-        <x:v>Infrastructure analogies about bridges, firewalls, or guardrails are often attacked by demanding that every literal feature transfer over exactly.</x:v>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="O107" t="str">
-        <x:v>Debaters sometimes turn an opponent's limited comparison into a cartoon version so they can say the analogy obviously fails.</x:v>
-      </x:c>
-      <x:c r="P107" t="str"/>
-      <x:c r="Q107" t="str"/>
-      <x:c r="R107" t="str"/>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P107" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="Q107" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R107" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S107" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5132,14 +5768,20 @@
         <x:v>A true or well-supported detail can increase trust only where the claims are genuinely linked. Often the extra conclusion is just hitching a ride on evidence that belongs to something narrower.</x:v>
       </x:c>
       <x:c r="N108" t="str">
-        <x:v>After the September 2024 ABC debate, the fact that the lecterns differed in height was treated by some users as if it supported much broader unverified claims about secret coordination and leaked questions.</x:v>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="O108" t="str">
-        <x:v>Conspiracy arguments often point to one authentic photo, real location, or correct minor fact and then use that narrow success to smuggle in much larger unsupported conclusions.</x:v>
-      </x:c>
-      <x:c r="P108" t="str"/>
-      <x:c r="Q108" t="str"/>
-      <x:c r="R108" t="str"/>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="P108" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="Q108" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R108" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S108" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5177,14 +5819,20 @@
         <x:v>Source criticism can be relevant, but poisoning the well tries to make the audience stop listening before the argument or evidence is even on the table.</x:v>
       </x:c>
       <x:c r="N109" t="str">
-        <x:v>In political and media fights, audiences are often primed to treat a judge, journalist, scientist, or witness as corrupt before that person's specific evidence is even heard.</x:v>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="O109" t="str">
-        <x:v>After the September 2024 Harris-Trump debate, repeated claims that moderators and outlets were inherently rigged encouraged supporters to dismiss later fact-checks in advance rather than assess them on the merits.</x:v>
-      </x:c>
-      <x:c r="P109" t="str"/>
-      <x:c r="Q109" t="str"/>
-      <x:c r="R109" t="str"/>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P109" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="Q109" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
+      <x:c r="R109" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
       <x:c r="S109" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5222,14 +5870,20 @@
         <x:v>Temporal order matters for causation, but it is only one ingredient. The improvement might be coincidence, regression to the mean, other background changes, or a different cause entirely.</x:v>
       </x:c>
       <x:c r="N110" t="str">
-        <x:v>Wellness and self-optimization discourse in 2024 routinely credited cold plunges, supplements, or glucose hacks for improvements that followed several simultaneous lifestyle changes.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O110" t="str">
-        <x:v>Politicians often claim that a policy worked because a good trend appeared soon after the policy was announced, even when the trend began earlier or other explanations remain stronger.</x:v>
-      </x:c>
-      <x:c r="P110" t="str"/>
-      <x:c r="Q110" t="str"/>
-      <x:c r="R110" t="str"/>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="P110" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="Q110" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R110" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
       <x:c r="S110" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5267,14 +5921,20 @@
         <x:v>Examples can illustrate a claim, but they do not by themselves prove a universal proposition. The missing question is whether the example is representative.</x:v>
       </x:c>
       <x:c r="N111" t="str">
-        <x:v>A single accurate prediction, one striking conversion story, or one dramatic crime clip is often treated as if it proved a broad thesis about markets, religion, or social decline.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O111" t="str">
-        <x:v>Debates about AI often jump from one impressive demo or one embarrassing failure to a total conclusion about the technology as a whole.</x:v>
-      </x:c>
-      <x:c r="P111" t="str"/>
-      <x:c r="Q111" t="str"/>
-      <x:c r="R111" t="str"/>
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="P111" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q111" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R111" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S111" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5314,14 +5974,20 @@
         <x:v>Complexity is not itself a fallacy. The problem is using sprawl as a shield, making it costly to respond point by point and then treating any unanswered fragment as proof of victory.</x:v>
       </x:c>
       <x:c r="N112" t="str">
-        <x:v>Podcast debates, marathon livestreams, and mega-threads often bury the central claim beneath so many tangents that audiences mistake exhaustion for concession.</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O112" t="str">
-        <x:v>AI-generated text makes this tactic cheaper by allowing people to produce long, confident, fast-moving argument dumps that sound comprehensive while remaining poorly grounded.</x:v>
-      </x:c>
-      <x:c r="P112" t="str"/>
-      <x:c r="Q112" t="str"/>
-      <x:c r="R112" t="str"/>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="P112" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="Q112" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="R112" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S112" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5357,14 +6023,20 @@
         <x:v>The missing piece is the base rate. Even a very accurate test can generate many false matches when the target condition is rare.</x:v>
       </x:c>
       <x:c r="N113" t="str">
-        <x:v>Crime and security debates often overstate the force of DNA, face-recognition, or screening matches by ignoring how many non-matching people were also in the pool.</x:v>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="O113" t="str">
-        <x:v>A similar mistake appears whenever a diagnostic tool's false-positive rate is treated as if it directly gave the chance that any one flagged person is guilty, sick, or dangerous.</x:v>
-      </x:c>
-      <x:c r="P113" t="str"/>
-      <x:c r="Q113" t="str"/>
-      <x:c r="R113" t="str"/>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="P113" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q113" t="str">
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
+      <x:c r="R113" t="str">
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+      </x:c>
       <x:c r="S113" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5400,14 +6072,20 @@
         <x:v>Self-knowledge can be useful, but it is not a universal template. Other people may share some motives while differing sharply on others.</x:v>
       </x:c>
       <x:c r="N114" t="str">
-        <x:v>People often assume that because they would lie, panic, or seek status in a situation, anyone else in that situation must be driven by the same motive.</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O114" t="str">
-        <x:v>Political and religious debate is full of claims about what opponents 'really know' or 'really fear' that reflect the speaker's own psychology more than the target's.</x:v>
-      </x:c>
-      <x:c r="P114" t="str"/>
-      <x:c r="Q114" t="str"/>
-      <x:c r="R114" t="str"/>
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="P114" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="Q114" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R114" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
       <x:c r="S114" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5445,14 +6123,20 @@
         <x:v>Not every detour is fallacious; context can matter. The fallacy appears when the diversion substitutes for addressing the question that was actually on the table.</x:v>
       </x:c>
       <x:c r="N115" t="str">
-        <x:v>In the June 27, 2024 Biden-Trump debate, answers about the economy, abortion, and January 6 often veered into immigration, personal fitness, or unrelated grievances instead of the question asked.</x:v>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="O115" t="str">
-        <x:v>Online arguments about institutional abuse, policing, or bias often slide away from the specific allegation and into some other controversy the speaker would rather discuss.</x:v>
-      </x:c>
-      <x:c r="P115" t="str"/>
-      <x:c r="Q115" t="str"/>
-      <x:c r="R115" t="str"/>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="P115" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="Q115" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="R115" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
       <x:c r="S115" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5484,14 +6168,20 @@
         <x:v>Evidence matters for empirical claims, but it cannot rescue a contradiction. If the concept itself does not make sense, more observations do not repair it.</x:v>
       </x:c>
       <x:c r="N116" t="str">
-        <x:v>Some arguments define a being, force, or property in mutually incompatible ways and then insist critics still need field evidence before calling the view incoherent.</x:v>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="O116" t="str">
-        <x:v>Online debate often treats every claim as if it deserved purely empirical testing, even when the real defect appears earlier at the level of definition or logical consistency.</x:v>
-      </x:c>
-      <x:c r="P116" t="str"/>
-      <x:c r="Q116" t="str"/>
-      <x:c r="R116" t="str"/>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="P116" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q116" t="str">
+        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+      </x:c>
+      <x:c r="R116" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S116" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5529,14 +6219,20 @@
         <x:v>After unusually high or low outcomes, partial reversion toward the average is often expected even without special causal forces.</x:v>
       </x:c>
       <x:c r="N117" t="str">
-        <x:v>Sports commentators routinely over-credit halftime speeches or rituals for rebounds that would be unsurprising after an extreme first-half performance.</x:v>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="O117" t="str">
-        <x:v>Investors and managers often mistake a natural bounce after a terrible quarter for proof that a new slogan, consultant, or memo fixed the underlying problem.</x:v>
-      </x:c>
-      <x:c r="P117" t="str"/>
-      <x:c r="Q117" t="str"/>
-      <x:c r="R117" t="str"/>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P117" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="Q117" t="str">
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+      </x:c>
+      <x:c r="R117" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S117" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5578,14 +6274,20 @@
         <x:v>Metaphor can be useful shorthand, but the fallacy appears when agency, intention, or moral responsibility is attributed to an abstraction as though it literally possessed a mind of its own.</x:v>
       </x:c>
       <x:c r="N118" t="str">
-        <x:v>People talk as if capitalism, democracy, the algorithm, or history itself wants, fears, rewards, or punishes, which can hide the actual network of human choices and incentives underneath.</x:v>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O118" t="str">
-        <x:v>AI discussions sometimes slide from 'the model produced this output' to 'the AI wants this outcome,' smuggling in a stronger picture of agency than the evidence supports.</x:v>
-      </x:c>
-      <x:c r="P118" t="str"/>
-      <x:c r="Q118" t="str"/>
-      <x:c r="R118" t="str"/>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="P118" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="Q118" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="R118" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
       <x:c r="S118" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5625,14 +6327,20 @@
         <x:v>An outcome can make a story feel inevitable in retrospect without ever having been inevitable in advance. Hindsight strips away the branching paths that were live at the time.</x:v>
       </x:c>
       <x:c r="N119" t="str">
-        <x:v>After elections, market crashes, and celebrity scandals, commentators often speak as if the final result had been written into the evidence from the start rather than emerging from many uncertain factors.</x:v>
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="O119" t="str">
-        <x:v>This fallacy regularly follows close races and volatile technologies, where later narratives overstate how clear the winning path supposedly was.</x:v>
-      </x:c>
-      <x:c r="P119" t="str"/>
-      <x:c r="Q119" t="str"/>
-      <x:c r="R119" t="str"/>
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="P119" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="Q119" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R119" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
       <x:c r="S119" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5666,14 +6374,20 @@
         <x:v>Many concepts such as belief, risk, identity, and influence work by degree. Treating them as all-or-nothing can falsify the speaker's actual position.</x:v>
       </x:c>
       <x:c r="N120" t="str">
-        <x:v>Election, public-health, and AI debates often force nuanced confidence claims into binary boxes such as certain or uncertain, safe or unsafe, real or fake.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O120" t="str">
-        <x:v>Arguments about what someone believes frequently replace a spectrum of confidence with a yes-or-no label that the original speaker never endorsed.</x:v>
-      </x:c>
-      <x:c r="P120" t="str"/>
-      <x:c r="Q120" t="str"/>
-      <x:c r="R120" t="str"/>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="P120" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q120" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R120" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
       <x:c r="S120" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5713,14 +6427,20 @@
         <x:v>Emotional attraction can explain why we want a conclusion, but not whether the conclusion is supported. A heartwarming possibility can still be false or impractical.</x:v>
       </x:c>
       <x:c r="N121" t="str">
-        <x:v>Fundraising pitches, miracle-cure stories, and uplifting viral posts often rely on the emotional payoff of the conclusion to make scrutiny feel mean or unnecessary.</x:v>
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="O121" t="str">
-        <x:v>Public debate about policy sometimes slides from 'this would be compassionate' to 'therefore it must be workable and correct,' skipping the harder evidential and tradeoff questions.</x:v>
-      </x:c>
-      <x:c r="P121" t="str"/>
-      <x:c r="Q121" t="str"/>
-      <x:c r="R121" t="str"/>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P121" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="Q121" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
+      <x:c r="R121" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
       <x:c r="S121" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5760,14 +6480,20 @@
         <x:v>This is close to cherry picking, but the emphasis is on drawing the target around the bullet holes after the shots land. Post hoc pattern-hunting can make randomness, noise, or mixed data look like confirmation.</x:v>
       </x:c>
       <x:c r="N122" t="str">
-        <x:v>Economic and election commentary often selects the time window, county, or subgroup that flatters the preferred narrative after the fact, then presents that slice as the decisive measure.</x:v>
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
       <x:c r="O122" t="str">
-        <x:v>AI benchmarking and startup marketing sometimes advertise the few tasks where a model shines while leaving out the wider distribution of tasks where the results are weaker or unstable.</x:v>
-      </x:c>
-      <x:c r="P122" t="str"/>
-      <x:c r="Q122" t="str"/>
-      <x:c r="R122" t="str"/>
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P122" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q122" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="R122" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
       <x:c r="S122" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5807,14 +6533,20 @@
         <x:v>Some causes are more important than others, and sometimes one factor really is dominant. The fallacy appears when a multi-causal phenomenon is flattened into a one-variable story without enough evidence.</x:v>
       </x:c>
       <x:c r="N123" t="str">
-        <x:v>Arguments about inflation, crime, housing costs, and educational decline often blame one villain such as immigrants, regulation, presidents, or social media, even when the outcome reflects multiple interacting causes.</x:v>
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="O123" t="str">
-        <x:v>After school shootings or viral episodes of unrest, public commentary regularly rushes to one master explanation instead of asking how incentives, access, institutions, culture, and personal history combine.</x:v>
-      </x:c>
-      <x:c r="P123" t="str"/>
-      <x:c r="Q123" t="str"/>
-      <x:c r="R123" t="str"/>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="P123" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="Q123" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="R123" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S123" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5854,14 +6586,20 @@
         <x:v>Some slopes are real, especially when incentives, precedent, or institutional weakness make escalation predictable. The fallacy appears when the chain is asserted rather than argued for.</x:v>
       </x:c>
       <x:c r="N124" t="str">
-        <x:v>In 2024 arguments over classroom AI, both enthusiasts and critics often predicted inevitable futures - either total educational collapse or total educational liberation - without showing why intermediate guardrails would fail.</x:v>
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="O124" t="str">
-        <x:v>Election rhetoric about mail voting, early voting, or routine administrative changes often predicts the total breakdown of legitimacy from one policy shift without evidence for the full cascade.</x:v>
-      </x:c>
-      <x:c r="P124" t="str"/>
-      <x:c r="Q124" t="str"/>
-      <x:c r="R124" t="str"/>
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="P124" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="Q124" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R124" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
       <x:c r="S124" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5899,14 +6637,20 @@
         <x:v>Exceptions can be justified, but they need a principled reason. Mere attachment to the favored case is not enough.</x:v>
       </x:c>
       <x:c r="N125" t="str">
-        <x:v>Political actors often demand strict accountability, civility, or transparency for opponents while inventing excuses for why their own side should be judged differently.</x:v>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O125" t="str">
-        <x:v>Religious and ideological arguments often exempt cherished claims from the evidence standards applied to ordinary claims.</x:v>
-      </x:c>
-      <x:c r="P125" t="str"/>
-      <x:c r="Q125" t="str"/>
-      <x:c r="R125" t="str"/>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P125" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q125" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="R125" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S125" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5944,14 +6688,20 @@
         <x:v>Attention is selective. Media, algorithms, and memory amplify the dramatic cases, not the ordinary distribution.</x:v>
       </x:c>
       <x:c r="N126" t="str">
-        <x:v>Crime clips, campus incidents, and viral protest footage often dominate public perception far beyond their representativeness, making whole groups look more extreme than they are.</x:v>
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="O126" t="str">
-        <x:v>People watching political interviews can easily conclude that a population is loud, combative, or theatrical without noticing that quieter members of the same population rarely become visible.</x:v>
-      </x:c>
-      <x:c r="P126" t="str"/>
-      <x:c r="Q126" t="str"/>
-      <x:c r="R126" t="str"/>
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+      </x:c>
+      <x:c r="P126" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q126" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="R126" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
       <x:c r="S126" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5987,14 +6737,20 @@
         <x:v>Sometimes the problem is deliberate obscurity; other times it is sincere confusion. Either way, complexity should not be mistaken for structure.</x:v>
       </x:c>
       <x:c r="N127" t="str">
-        <x:v>Conspiracy reasoning often spirals into self-sealing loops where every attempted refutation becomes fresh confirmation through an increasingly baroque chain of premises.</x:v>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O127" t="str">
-        <x:v>AI-generated argument dumps can produce this effect by chaining plausible-sounding clauses that never quite add up to a valid line of reasoning.</x:v>
-      </x:c>
-      <x:c r="P127" t="str"/>
-      <x:c r="Q127" t="str"/>
-      <x:c r="R127" t="str"/>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P127" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="Q127" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R127" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S127" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6032,14 +6788,20 @@
         <x:v>A straw man can be created by exaggeration, selective quotation, or by ignoring the qualifying parts of the original claim. It is not enough that a reply is critical; the key problem is that the reply no longer addresses the real position.</x:v>
       </x:c>
       <x:c r="N128" t="str">
-        <x:v>During the September 10, 2024 Harris-Trump debate, claims about abortion rights were repeatedly recast into the far more extreme charge that Democrats support killing babies after birth, which is not the position being defended.</x:v>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="O128" t="str">
-        <x:v>Debates over campus speech and content moderation often turn a narrower argument about rules, incentives, or disclosure into the cartoon claim that one side 'wants censorship' or 'wants total chaos.'</x:v>
-      </x:c>
-      <x:c r="P128" t="str"/>
-      <x:c r="Q128" t="str"/>
-      <x:c r="R128" t="str"/>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="P128" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="Q128" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
+      <x:c r="R128" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
       <x:c r="S128" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6079,14 +6841,20 @@
         <x:v>Strong delivery can make good arguments easier to hear, but it can also camouflage weak ones. Audiences often remember certainty, rhythm, and applause longer than the actual reasoning.</x:v>
       </x:c>
       <x:c r="N129" t="str">
-        <x:v>Coverage of the September 10, 2024 Harris-Trump debate often focused on who seemed stronger, calmer, or more in command, which matters politically but does not by itself settle whether the claims on stage were accurate.</x:v>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O129" t="str">
-        <x:v>Short-form video and podcast culture reward confidence, pace, and rhetorical dominance, making it easy for a slick performance to outperform a careful but less theatrical argument.</x:v>
-      </x:c>
-      <x:c r="P129" t="str"/>
-      <x:c r="Q129" t="str"/>
-      <x:c r="R129" t="str"/>
+        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+      </x:c>
+      <x:c r="P129" t="str">
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
+      <x:c r="Q129" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="R129" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
       <x:c r="S129" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6124,14 +6892,20 @@
         <x:v>Correlative terms such as healthy and unhealthy, free and restricted, informed and uninformed, or biased and impartial depend on contrasts that can be weakened without disappearing.</x:v>
       </x:c>
       <x:c r="N130" t="str">
-        <x:v>Critics sometimes argue that because everyone has some bias, calling a report biased says nothing, as if degrees of distortion and unfairness were impossible.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O130" t="str">
-        <x:v>Debates about freedom and censorship often set the positive term to an impossible ideal so that ordinary, useful distinctions collapse.</x:v>
-      </x:c>
-      <x:c r="P130" t="str"/>
-      <x:c r="Q130" t="str"/>
-      <x:c r="R130" t="str"/>
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="P130" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="Q130" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R130" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
       <x:c r="S130" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6169,14 +6943,20 @@
         <x:v>The visible winners are often the easiest cases to notice, but they are not the whole sample. Ignoring the many failed or filtered-out cases makes strategies look safer, smarter, or more effective than they really are.</x:v>
       </x:c>
       <x:c r="N131" t="str">
-        <x:v>Startup and creator advice often highlights spectacular winners while the much larger number of people who copied the same strategy and failed remain largely invisible.</x:v>
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
       <x:c r="O131" t="str">
-        <x:v>Investment talk routinely showcases the funds, traders, and backtests that survived long enough to look impressive while the dead funds and broken strategies quietly disappear.</x:v>
-      </x:c>
-      <x:c r="P131" t="str"/>
-      <x:c r="Q131" t="str"/>
-      <x:c r="R131" t="str"/>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P131" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
+      <x:c r="Q131" t="str">
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="R131" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S131" t="str">
         <x:v>added-2026-completeness-pass</x:v>
       </x:c>
@@ -6212,14 +6992,20 @@
         <x:v>Some things really are designed for purposes, but purpose should not be assumed where it has not been shown. Processes can produce outcomes without aiming at them.</x:v>
       </x:c>
       <x:c r="N132" t="str">
-        <x:v>People often speak as if history is automatically bending toward justice, collapse, nationalism, or liberation, as though social change carried its own guaranteed destination.</x:v>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O132" t="str">
-        <x:v>In technology debates, AI progress is sometimes framed as if it were inherently marching toward a single destined endpoint such as AGI rather than following contingent technical and social paths.</x:v>
-      </x:c>
-      <x:c r="P132" t="str"/>
-      <x:c r="Q132" t="str"/>
-      <x:c r="R132" t="str"/>
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P132" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="Q132" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="R132" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
       <x:c r="S132" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6257,14 +7043,20 @@
         <x:v>Aphorisms can be wise shortcuts, but they become fallacious when they replace the reasoning that the situation still requires.</x:v>
       </x:c>
       <x:c r="N133" t="str">
-        <x:v>Phrases such as 'Do your own research,' 'common sense,' or 'if you know, you know' are often used online not to open inquiry but to make further questions look unnecessary or naive.</x:v>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O133" t="str">
-        <x:v>Political and religious arguments frequently end with slogans like 'Freedom is not free' or 'Only God knows,' which can be meaningful in some contexts but often function as conversation-stoppers.</x:v>
-      </x:c>
-      <x:c r="P133" t="str"/>
-      <x:c r="Q133" t="str"/>
-      <x:c r="R133" t="str"/>
+        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+      </x:c>
+      <x:c r="P133" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="Q133" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="R133" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S133" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6300,14 +7092,20 @@
         <x:v>A vivid case can motivate investigation, but it does not by itself justify a population-level conclusion.</x:v>
       </x:c>
       <x:c r="N134" t="str">
-        <x:v>Isolated crime stories are often turned into sweeping claims about immigrants, professions, age groups, or political movements.</x:v>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O134" t="str">
-        <x:v>A single corporate scandal can quickly become a claim that the entire industry is rotten in exactly the same way.</x:v>
-      </x:c>
-      <x:c r="P134" t="str"/>
-      <x:c r="Q134" t="str"/>
-      <x:c r="R134" t="str"/>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P134" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q134" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="R134" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S134" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6351,14 +7149,20 @@
         <x:v>Generalizations are often default-pattern claims, not exceptionless universal laws.</x:v>
       </x:c>
       <x:c r="N135" t="str">
-        <x:v>Public-health advice is often dismissed by pointing to unusual edge cases even when the advice was clearly aimed at ordinary conditions.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O135" t="str">
-        <x:v>Safety rules and economic patterns are frequently challenged by exceptions that do not actually undermine the broader tendency being described.</x:v>
-      </x:c>
-      <x:c r="P135" t="str"/>
-      <x:c r="Q135" t="str"/>
-      <x:c r="R135" t="str"/>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="P135" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="Q135" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R135" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
       <x:c r="S135" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6394,14 +7198,20 @@
         <x:v>A favorable anecdote can remind us not to overgeneralize negatively, but it cannot prove that the larger class is generally positive.</x:v>
       </x:c>
       <x:c r="N136" t="str">
-        <x:v>One transparent politician or one ethical corporation is often used to imply that the surrounding system is healthier than the broader evidence suggests.</x:v>
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="O136" t="str">
-        <x:v>People frequently infer that an institution is trustworthy because they personally encountered one helpful employee inside it.</x:v>
-      </x:c>
-      <x:c r="P136" t="str"/>
-      <x:c r="Q136" t="str"/>
-      <x:c r="R136" t="str"/>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P136" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="Q136" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="R136" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
       <x:c r="S136" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6433,14 +7243,20 @@
         <x:v>A track record does not make contrary outcomes impossible, but it does affect rational priors. Ignoring repeated past failure forces every new case to borrow more credibility than it has earned.</x:v>
       </x:c>
       <x:c r="N137" t="str">
-        <x:v>Baseless claims about widespread noncitizen voting keep getting relaunched as if decades of rarity, audits, and failed alarms provide no reason for initial skepticism.</x:v>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="O137" t="str">
-        <x:v>Every new blurry UFO clip, miracle cure, or ghost story is often pitched as if the long record of ordinary explanations should have zero effect on our starting expectations.</x:v>
-      </x:c>
-      <x:c r="P137" t="str"/>
-      <x:c r="Q137" t="str"/>
-      <x:c r="R137" t="str"/>
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+      </x:c>
+      <x:c r="P137" t="str">
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
+      <x:c r="Q137" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="R137" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
       <x:c r="S137" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6482,14 +7298,20 @@
         <x:v>Hypocrisy can matter for trust, but it does not by itself answer whether the original claim, act, or argument was wrong.</x:v>
       </x:c>
       <x:c r="N138" t="str">
-        <x:v>In the June 27, 2024 Biden-Trump debate and the September 10, 2024 Harris-Trump debate, many charges were met with 'your side did it too' responses that redirected blame without addressing the original allegation.</x:v>
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="O138" t="str">
-        <x:v>Arguments about misinformation, climate, religion, and media bias often slide into scorekeeping about who is worse rather than whether the specific criticized claim is true or justified.</x:v>
-      </x:c>
-      <x:c r="P138" t="str"/>
-      <x:c r="Q138" t="str"/>
-      <x:c r="R138" t="str"/>
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P138" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="Q138" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R138" t="str">
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
       <x:c r="S138" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6529,14 +7351,20 @@
         <x:v>Exposing hypocrisy can matter, but retaliation does not erase the original wrong or magically sanitize a copy of it.</x:v>
       </x:c>
       <x:c r="N139" t="str">
-        <x:v>In 2024 election discourse, misinformation was often excused with the claim that the other side lies too, as if symmetry or revenge transformed falsehood into fairness.</x:v>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="O139" t="str">
-        <x:v>Debates about censorship, doxxing, and dirty campaign tactics often slide from condemnation into imitation, with each side treating the other's bad behavior as a license to do the same.</x:v>
-      </x:c>
-      <x:c r="P139" t="str"/>
-      <x:c r="Q139" t="str"/>
-      <x:c r="R139" t="str"/>
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+      </x:c>
+      <x:c r="P139" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="Q139" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="R139" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
       <x:c r="S139" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6572,14 +7400,20 @@
         <x:v>Sharing a feature does not establish identity or class inclusion unless the shared feature actually covers the whole relevant group. A middle term can connect without unifying.</x:v>
       </x:c>
       <x:c r="N140" t="str">
-        <x:v>Lifestyle and identity marketing often says 'the cool do X' and 'I do X,' then slides to 'therefore I am one of the cool,' even though the shared feature is too broad.</x:v>
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="O140" t="str">
-        <x:v>Political commentary frequently infers that because two camps are skeptical of the same institution or support the same policy, they must belong to the same underlying movement.</x:v>
-      </x:c>
-      <x:c r="P140" t="str"/>
-      <x:c r="Q140" t="str"/>
-      <x:c r="R140" t="str"/>
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="P140" t="str">
+        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q140" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R140" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S140" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6611,14 +7445,20 @@
         <x:v>Vagueness can be useful early in exploration, but it becomes fallacious when the fog is preserved to prevent serious evaluation. If key terms cannot be pinned down, the claim can keep slipping away from critique.</x:v>
       </x:c>
       <x:c r="N141" t="str">
-        <x:v>Alternative-health and wellness marketing often leans on words like 'toxins,' 'energy,' 'balance,' and 'boost' precisely because they sound scientific while remaining hard to falsify.</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O141" t="str">
-        <x:v>In arguments about spirituality, self-help, and even AI, flexible phrases can be stretched to fit almost any outcome, which makes the view feel resilient without making it well supported.</x:v>
-      </x:c>
-      <x:c r="P141" t="str"/>
-      <x:c r="Q141" t="str"/>
-      <x:c r="R141" t="str"/>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="P141" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="Q141" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="R141" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
       <x:c r="S141" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6662,14 +7502,20 @@
         <x:v>Hope can sustain action, but it does not convert possibility into evidence. The stronger the desire, the easier it is to mistake wanting for warrant.</x:v>
       </x:c>
       <x:c r="N142" t="str">
-        <x:v>Speculative markets, miracle-cure promises, and election-night narratives often run on the thought that a hoped-for outcome is somehow more likely because people badly want it.</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O142" t="str">
-        <x:v>Beliefs about the afterlife, destiny, or technological salvation are often defended by saying life would feel bleak without them, which speaks to desire rather than truth.</x:v>
-      </x:c>
-      <x:c r="P142" t="str"/>
-      <x:c r="Q142" t="str"/>
-      <x:c r="R142" t="str"/>
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="P142" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="Q142" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="R142" t="str">
+        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+      </x:c>
       <x:c r="S142" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6703,14 +7549,20 @@
         <x:v>Real corroboration requires accessible, independent testimony or records. Simply claiming that more witnesses exist adds almost nothing if the chain cannot be examined.</x:v>
       </x:c>
       <x:c r="N143" t="str">
-        <x:v>Paranormal, religious, and conspiracy stories often swell in authority by invoking unnamed doctors, secret insiders, or hundreds of silent observers who never become independently available.</x:v>
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="O143" t="str">
-        <x:v>Historical arguments sometimes treat a late report that 'many people saw it' as if that were the same thing as actually having many separate testimonies.</x:v>
-      </x:c>
-      <x:c r="P143" t="str"/>
-      <x:c r="Q143" t="str"/>
-      <x:c r="R143" t="str"/>
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="P143" t="str">
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+      </x:c>
+      <x:c r="Q143" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="R143" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
       <x:c r="S143" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6746,14 +7598,20 @@
         <x:v>Correlations can be real while still pointing the wrong way. Without evidence about timing, mechanism, and alternatives, reversing cause and effect is easy.</x:v>
       </x:c>
       <x:c r="N144" t="str">
-        <x:v>Arguments about social media and teen mental health often assume a one-way causal story even though distress can also increase the tendency to seek certain kinds of online engagement.</x:v>
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="O144" t="str">
-        <x:v>Crime, policing, and economic debates frequently treat a response variable as if it were the cause, such as assuming security purchases create fear rather than fear driving security purchases.</x:v>
-      </x:c>
-      <x:c r="P144" t="str"/>
-      <x:c r="Q144" t="str"/>
-      <x:c r="R144" t="str"/>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+      </x:c>
+      <x:c r="P144" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="Q144" t="str">
+        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+      </x:c>
+      <x:c r="R144" t="str">
+        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
       <x:c r="S144" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>

</xml_diff>

<commit_message>
Tighten case study matching by fallacy
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R316bf591757f49b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R54067ec4d5be495d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R074be61854bc4376"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1b368b82c05244fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R2713cfdf029a432c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R58bef55075f0490f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -356,20 +356,14 @@
         <x:v>Sometimes absence of evidence really is weak evidence, especially when the search tools are poor or the target is hard to detect. But when repeated investigation under the right conditions turns up nothing, that absence is itself evidence.</x:v>
       </x:c>
       <x:c r="N2" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>After officials in Springfield, Ohio said there were no credible reports supporting the September 2024 rumor that Haitian immigrants were abducting and eating pets, some defenders treated the lack of evidence as irrelevant or as proof of a cover-up rather than as evidence against the rumor.</x:v>
       </x:c>
       <x:c r="O2" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="P2" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="Q2" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="R2" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
-      </x:c>
+        <x:v>Claims of widespread noncitizen voting in 2024 often survived repeated audits and official reviews by insisting that the absence of supporting evidence was exactly what one should expect from a hidden scheme.</x:v>
+      </x:c>
+      <x:c r="P2" t="str"/>
+      <x:c r="Q2" t="str"/>
+      <x:c r="R2" t="str"/>
       <x:c r="S2" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -401,20 +395,14 @@
         <x:v>Abstract patterns can still be real and explanatory even when they depend on smaller physical or social components. Economies, institutions, languages, and ecosystems do not stop being real because they are made of people, words, or organisms.</x:v>
       </x:c>
       <x:c r="N3" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>People sometimes say 'science does not discover anything, only scientists do,' as if that erased the reality of science as a method and institution with stable norms and effects.</x:v>
       </x:c>
       <x:c r="O3" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="P3" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="Q3" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R3" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>Debates about algorithms, markets, and social platforms often pretend there is no system-level behavior because only users or lines of code act at the micro level.</x:v>
+      </x:c>
+      <x:c r="P3" t="str"/>
+      <x:c r="Q3" t="str"/>
+      <x:c r="R3" t="str"/>
       <x:c r="S3" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -446,20 +434,14 @@
         <x:v>Useful abstractions describe patterns with varying scope and durability. They are not automatically eternal, exceptionless constraints on what can happen.</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>People often treat economic or technological 'laws' as if they guaranteed the future rather than summarizing a contingent historical pattern that may bend, pause, or fail.</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="P4" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="Q4" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="R4" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
+        <x:v>In AI discourse, scaling trends are sometimes talked about as destiny, as though past curves logically force a particular future rather than merely suggesting one.</x:v>
+      </x:c>
+      <x:c r="P4" t="str"/>
+      <x:c r="Q4" t="str"/>
+      <x:c r="R4" t="str"/>
       <x:c r="S4" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -499,19 +481,19 @@
         <x:v>Character can matter when credibility itself is at issue, such as fraud, conflicts of interest, or proven dishonesty. The fallacy appears when those personal facts are used instead of answering the actual reasons or evidence.</x:v>
       </x:c>
       <x:c r="N5" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
         <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
-      <x:c r="O5" t="str">
+      <x:c r="P5" t="str">
         <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
-      <x:c r="P5" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
       <x:c r="Q5" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+        <x:v>In the June 27, 2024 Biden-Trump debate, policy exchanges repeatedly slid into attacks on each candidate's age, criminal exposure, or family rather than sustained engagement with the argument on the table.</x:v>
       </x:c>
       <x:c r="R5" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+        <x:v>Online discussion of climate, vaccines, and AI policy often substitutes labels such as 'shill,' 'grifter,' or 'elitist' for any serious response to the evidence.</x:v>
       </x:c>
       <x:c r="S5" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -548,20 +530,14 @@
         <x:v>Ruling something out does not automatically place it into the positive category you want. 'Not bad' does not by itself mean 'good,' and 'not that' does not by itself mean 'this.'</x:v>
       </x:c>
       <x:c r="N6" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Tribal arguments often move from 'we are not them' and 'they are bad' to 'therefore we are trustworthy,' even though the conclusion has not been earned.</x:v>
       </x:c>
       <x:c r="O6" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="P6" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="Q6" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R6" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
+        <x:v>Media and politics frequently treat the failure of one rival source as if it directly validated a different source that still needs its own support.</x:v>
+      </x:c>
+      <x:c r="P6" t="str"/>
+      <x:c r="Q6" t="str"/>
+      <x:c r="R6" t="str"/>
       <x:c r="S6" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -599,20 +575,18 @@
         <x:v>Some disjunctions are genuinely exclusive, but many are not. Two options can coexist unless the statement or context really rules that out.</x:v>
       </x:c>
       <x:c r="N7" t="str">
+        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
         <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
-      <x:c r="O7" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
       <x:c r="P7" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>Budget rhetoric often suggests that because one policy tool is on the table, another cannot also matter, as if tradeoffs always come in only one-at-a-time form.</x:v>
       </x:c>
       <x:c r="Q7" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R7" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Public debate regularly acts as though a claim must be either emotional or strategic, either true or persuasive, either mistaken or manipulative, when in reality both descriptions may apply.</x:v>
+      </x:c>
+      <x:c r="R7" t="str"/>
       <x:c r="S7" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -650,19 +624,19 @@
         <x:v>A consequence can have many causes. Observing the result does not tell you which sufficient condition produced it.</x:v>
       </x:c>
       <x:c r="N8" t="str">
+        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
         <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
-      <x:c r="O8" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="P8" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
       <x:c r="Q8" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Political misinformation often treats one suspicious-looking detail as proof of a favored cause, even though many other explanations remain live.</x:v>
       </x:c>
       <x:c r="R8" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Arguments about fraud, manipulation, and AI generation frequently jump from a telltale symptom to a confident diagnosis without ruling out alternatives.</x:v>
       </x:c>
       <x:c r="S8" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -697,20 +671,14 @@
         <x:v>Many systems of belief, institutions, and documents are mixed. Partial support or partial failure rarely justifies an everything-or-nothing verdict.</x:v>
       </x:c>
       <x:c r="N9" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>In 2024 media battles, a single correction or mistaken detail was often used to dismiss an outlet's entire reporting on elections, immigration, or public health.</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
-      </x:c>
-      <x:c r="P9" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q9" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R9" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
+        <x:v>Religious, ideological, and policy debates often act as though rejecting one doctrine, statistic, or mechanism commits you to rejecting the entire worldview.</x:v>
+      </x:c>
+      <x:c r="P9" t="str"/>
+      <x:c r="Q9" t="str"/>
+      <x:c r="R9" t="str"/>
       <x:c r="S9" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -748,19 +716,19 @@
         <x:v>Anecdotes can be useful for illustration, hypothesis generation, or showing that something can happen. The fallacy appears when one memorable case is used to outweigh stronger evidence about what usually happens or what the larger data set shows.</x:v>
       </x:c>
       <x:c r="N10" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="O10" t="str">
         <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="P10" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
       </x:c>
       <x:c r="Q10" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>Arguments about vaccines, supplements, and raw milk often lean on a neighbor's success story or a family anecdote as if that settled what the best studies show.</x:v>
       </x:c>
       <x:c r="R10" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+        <x:v>Debates about AI productivity and remote work often treat one manager's striking success or failure story as if it established the general rule for everyone.</x:v>
       </x:c>
       <x:c r="S10" t="str">
         <x:v>added-2026-completeness-pass</x:v>
@@ -803,20 +771,14 @@
         <x:v>Real accomplishment can justify attention, but it does not automatically transfer expertise across domains. The relevant question is still whether the claim is supported.</x:v>
       </x:c>
       <x:c r="N11" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>Celebrity founders, athletes, and actors often lend credibility to products and causes far outside their expertise, from supplements to financial schemes to political narratives.</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="P11" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="Q11" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="R11" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
+        <x:v>Public arguments about AI frequently treat the prestige of well-known founders as if it settled disputes that still require technical evidence, replication, and broader expert scrutiny.</x:v>
+      </x:c>
+      <x:c r="P11" t="str"/>
+      <x:c r="Q11" t="str"/>
+      <x:c r="R11" t="str"/>
       <x:c r="S11" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -861,16 +823,16 @@
         <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="O12" t="str">
+        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+      </x:c>
+      <x:c r="P12" t="str">
         <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
-      <x:c r="P12" t="str">
-        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
-      </x:c>
       <x:c r="Q12" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Debates about nutrition, vaccines, crypto, and AI frequently lean on celebrity experts or founders speaking outside their strongest field, while the underlying studies and uncertainties get little attention.</x:v>
       </x:c>
       <x:c r="R12" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>In public discussion of AI safety and capability, people often present a famous CEO's confidence level as if it were itself a substitute for technical evidence or broad expert agreement.</x:v>
       </x:c>
       <x:c r="S12" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -913,20 +875,18 @@
         <x:v>Consequences matter for what we should do, but they do not by themselves determine what is true. A painful implication does not refute a claim, and a comforting implication does not confirm one.</x:v>
       </x:c>
       <x:c r="N13" t="str">
+        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+      </x:c>
+      <x:c r="O13" t="str">
         <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
-      <x:c r="O13" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
       <x:c r="P13" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+        <x:v>Some climate arguments treat the economic and political inconvenience of decarbonization as if it counted against the underlying science itself.</x:v>
       </x:c>
       <x:c r="Q13" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
-      <x:c r="R13" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
+        <x:v>In debates about AI consciousness, animal cognition, or moral status, people sometimes argue that the conclusion cannot be right because accepting it would create uncomfortable obligations.</x:v>
+      </x:c>
+      <x:c r="R13" t="str"/>
       <x:c r="S13" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -974,14 +934,12 @@
         <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>In 2024 campaign advertising, immigration, crime, and abortion messages often relied on fear-laden images and worst-case anecdotes whose emotional force far exceeded the actual argument being made.</x:v>
       </x:c>
       <x:c r="Q14" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R14" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
+        <x:v>The spread of AI-generated political ads and deepfakes in 2024 showed how cheaply campaigns can trigger outrage or panic before voters have time to inspect the evidence.</x:v>
+      </x:c>
+      <x:c r="R14" t="str"/>
       <x:c r="S14" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1021,19 +979,19 @@
         <x:v>Fear can be rational when the threat is real and well evidenced. The fallacy appears when fear does the persuasive work that evidence and reasoning have not done.</x:v>
       </x:c>
       <x:c r="N15" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
         <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
-      <x:c r="O15" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
       <x:c r="P15" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="Q15" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="R15" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="S15" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -1077,17 +1035,13 @@
         <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="O16" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>Wellness, crypto, and conspiracy marketing often tells followers they are 'awake,' 'elite,' or 'smart enough to see through the lie,' turning assent into a test of self-image.</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="Q16" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="R16" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
+        <x:v>Political fundraising and influencer media frequently flatter supporters as the few people brave or intelligent enough to 'see what is really happening' before asking them to accept weakly supported claims.</x:v>
+      </x:c>
+      <x:c r="Q16" t="str"/>
+      <x:c r="R16" t="str"/>
       <x:c r="S16" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1127,20 +1081,14 @@
         <x:v>Motives can be relevant to bias and credibility, but they do not automatically settle whether the argument or evidence is sound.</x:v>
       </x:c>
       <x:c r="N17" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>After the September 2024 ABC debate, accusations about moderator bias were often used not just to question fairness, but to pre-dismiss later fact-checks without engaging their substance.</x:v>
       </x:c>
       <x:c r="O17" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="P17" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
-      <x:c r="Q17" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
-      </x:c>
-      <x:c r="R17" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
+        <x:v>In debates about climate, vaccines, and AI policy, critics are often waved away as 'funded,' 'bought,' or 'performing for clicks' instead of being answered.</x:v>
+      </x:c>
+      <x:c r="P17" t="str"/>
+      <x:c r="Q17" t="str"/>
+      <x:c r="R17" t="str"/>
       <x:c r="S17" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1183,17 +1131,13 @@
         <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O18" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>Wellness marketing for raw milk, supplements, and 'clean' products often treats natural as if it automatically meant safer, healthier, or morally superior.</x:v>
       </x:c>
       <x:c r="P18" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="Q18" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="R18" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
+        <x:v>Arguments about sex, family, and medicine often smuggle a moral conclusion into the descriptive claim that one pattern is simply 'what nature intended.'</x:v>
+      </x:c>
+      <x:c r="Q18" t="str"/>
+      <x:c r="R18" t="str"/>
       <x:c r="S18" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1238,17 +1182,13 @@
         <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="O19" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>In the 2024 rush to adopt generative AI, many products were pitched as inherently superior because they were new, even when reliability, labor impact, and safety were still unsettled.</x:v>
       </x:c>
       <x:c r="P19" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="Q19" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
-      <x:c r="R19" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Political and management rhetoric often treats 'innovation' as a reason to trust a strategy before any serious test of whether it solves the underlying problem.</x:v>
+      </x:c>
+      <x:c r="Q19" t="str"/>
+      <x:c r="R19" t="str"/>
       <x:c r="S19" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1288,20 +1228,14 @@
         <x:v>Compassion can matter for what response is humane, but it does not determine whether the underlying claim has been proved.</x:v>
       </x:c>
       <x:c r="N20" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+        <x:v>Fundraising and advocacy campaigns sometimes imply that questioning a factual claim is itself heartless, shifting the pressure from evidence to emotional identification.</x:v>
       </x:c>
       <x:c r="O20" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="P20" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="Q20" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="R20" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Public figures under scrutiny sometimes ask to be believed or excused because they are suffering, overwhelmed, or facing intense pressure, even when those facts do not establish the truth of what they are saying.</x:v>
+      </x:c>
+      <x:c r="P20" t="str"/>
+      <x:c r="Q20" t="str"/>
+      <x:c r="R20" t="str"/>
       <x:c r="S20" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1344,17 +1278,13 @@
         <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="O21" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>Campaign biographies in 2024 often leaned heavily on working-class roots and hardship stories, which may matter politically but do not by themselves verify a candidate's policy claims.</x:v>
       </x:c>
       <x:c r="P21" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="Q21" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="R21" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
+        <x:v>Populist media often imply that 'ordinary people' are automatically more honest than credentialed critics, as if social position alone settled the argument.</x:v>
+      </x:c>
+      <x:c r="Q21" t="str"/>
+      <x:c r="R21" t="str"/>
       <x:c r="S21" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1390,19 +1320,19 @@
         <x:v>Possibility is a very weak starting point. Many things are possible without being probable, and many probable things still fail to happen in any given case.</x:v>
       </x:c>
       <x:c r="N22" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O22" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="P22" t="str">
+        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+      </x:c>
+      <x:c r="Q22" t="str">
         <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
-      <x:c r="P22" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q22" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
       <x:c r="R22" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Crypto, lottery, and sports-betting talk often slides from 'this could happen' to 'this is bound to happen,' especially after a short streak of wins.</x:v>
       </x:c>
       <x:c r="S22" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -1449,14 +1379,12 @@
         <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="P23" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>Debates about religion, feminism, climate, and AI are often reduced to memes whose purpose is to make one side look ridiculous rather than to assess the actual claim.</x:v>
       </x:c>
       <x:c r="Q23" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="R23" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Online discourse frequently treats a sarcastic dunk or quote-tweet pile-on as if public humiliation itself were refutation.</x:v>
+      </x:c>
+      <x:c r="R23" t="str"/>
       <x:c r="S23" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1496,20 +1424,14 @@
         <x:v>Anger at the people who might benefit from a policy does not settle whether the policy is wise, fair, or effective.</x:v>
       </x:c>
       <x:c r="N24" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>Campaign messages often invite voters to reject a proposal because hated elites, immigrants, bankers, or academics might benefit, even when that says nothing about the proposal's merits.</x:v>
       </x:c>
       <x:c r="O24" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
-      <x:c r="P24" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
-      <x:c r="Q24" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="R24" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
-      </x:c>
+        <x:v>Social-media outrage often works by making the audience feel that supporting a view would somehow reward people they already dislike.</x:v>
+      </x:c>
+      <x:c r="P24" t="str"/>
+      <x:c r="Q24" t="str"/>
+      <x:c r="R24" t="str"/>
       <x:c r="S24" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1557,14 +1479,12 @@
         <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="P25" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>In 2024 arguments that the United States is a 'Christian nation,' long practice and selective founding-era precedent were often treated as if they settled the constitutional question.</x:v>
       </x:c>
       <x:c r="Q25" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="R25" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
+        <x:v>Arguments about schooling, marriage, and gender roles often rely on 'we have always done it this way' instead of showing why the tradition remains just or effective.</x:v>
+      </x:c>
+      <x:c r="R25" t="str"/>
       <x:c r="S25" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1604,20 +1524,14 @@
         <x:v>Success can indicate skill in a particular domain, but money is not a universal credential. Wealth may buy attention, not truth.</x:v>
       </x:c>
       <x:c r="N26" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>In 2024 and 2025, fans and investors often treated billionaire founders' views on AI, politics, or medicine as self-validating because of their wealth rather than because the evidence was strong.</x:v>
       </x:c>
       <x:c r="O26" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
-      <x:c r="P26" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="Q26" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="R26" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
+        <x:v>The unverified ABC debate affidavit gained extra credibility online after high-profile wealthy amplifiers helped circulate it, as though status itself made the claim more trustworthy.</x:v>
+      </x:c>
+      <x:c r="P26" t="str"/>
+      <x:c r="Q26" t="str"/>
+      <x:c r="R26" t="str"/>
       <x:c r="S26" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1656,17 +1570,13 @@
         <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="O27" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>When a candidate exaggerates one statistic, opponents often jump from 'that argument was flawed' to 'the broader policy position must therefore be false.'</x:v>
       </x:c>
       <x:c r="P27" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="Q27" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R27" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
+        <x:v>Online 'gotcha' culture frequently treats catching a fallacious defense as if it automatically disproved whatever the speaker was trying to defend.</x:v>
+      </x:c>
+      <x:c r="Q27" t="str"/>
+      <x:c r="R27" t="str"/>
       <x:c r="S27" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1710,13 +1620,13 @@
         <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="P28" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="Q28" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>After an anonymous affidavit circulated online in September 2024 alleging that ABC had secretly rigged the Harris-Trump debate, many posts treated the absence of immediate disproof as if it were evidence that the allegation was real.</x:v>
       </x:c>
       <x:c r="R28" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>UAP discussions often jump from 'we do not yet know what caused this' to 'therefore it was extraterrestrial technology,' which treats unexplained as if it meant explained by the favored hypothesis.</x:v>
       </x:c>
       <x:c r="S28" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -1758,17 +1668,13 @@
         <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="O29" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>Discussions of evolution, climate systems, and AI often slide from 'I do not see how that could work' to 'therefore it cannot be right.'</x:v>
       </x:c>
       <x:c r="P29" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="Q29" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="R29" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
+        <x:v>Paranormal and conspiracy arguments often rely on the mirror image of the same move: 'I cannot imagine another explanation, so my favored explanation must be true.'</x:v>
+      </x:c>
+      <x:c r="Q29" t="str"/>
+      <x:c r="R29" t="str"/>
       <x:c r="S29" t="str">
         <x:v>added-2026-completeness-pass</x:v>
       </x:c>
@@ -1806,19 +1712,19 @@
         <x:v>A claim does not become better supported because it is repeated by the same speaker, echoed by many speakers, or circulated for a long time. Repetition changes familiarity, not the underlying evidence.</x:v>
       </x:c>
       <x:c r="N30" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="O30" t="str">
         <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="P30" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
       </x:c>
       <x:c r="Q30" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
       </x:c>
       <x:c r="R30" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>The Springfield, Ohio pet-eating rumor in September 2024 moved from rumor to national talking point largely through repetition across social media, cable segments, and campaign rhetoric even though local officials said there was no credible evidence.</x:v>
       </x:c>
       <x:c r="S30" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -1859,20 +1765,14 @@
         <x:v>Silence can matter when a response would clearly be expected and feasible. Outside that setting, it often tells us little.</x:v>
       </x:c>
       <x:c r="N31" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+        <x:v>The absence of public confirmation for many election-fraud and migrant-voting rumors was often spun as suspicious silence rather than as a sign that the underlying evidence was weak or nonexistent.</x:v>
       </x:c>
       <x:c r="O31" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="P31" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="Q31" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
-      </x:c>
-      <x:c r="R31" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
+        <x:v>A 'no comment' from campaigns, police, or institutions is regularly treated as if it were a tacit admission, even though legal, strategic, or practical reasons may explain the silence.</x:v>
+      </x:c>
+      <x:c r="P31" t="str"/>
+      <x:c r="Q31" t="str"/>
+      <x:c r="R31" t="str"/>
       <x:c r="S31" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1914,20 +1814,14 @@
         <x:v>Threats can force compliance, but they do not transform a bad argument into a good one. Fear may explain why someone goes along; it does not show that the view is correct.</x:v>
       </x:c>
       <x:c r="N32" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>In countries where blasphemy, apostasy, or political dissent can trigger severe punishment, outward conformity is often mistaken for genuine persuasion when it may simply reflect fear.</x:v>
       </x:c>
       <x:c r="O32" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="P32" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="Q32" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="R32" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Online campaigns that threaten doxxing, blacklisting, or mass harassment often aim to secure silence or agreement by making disagreement personally costly.</x:v>
+      </x:c>
+      <x:c r="P32" t="str"/>
+      <x:c r="Q32" t="str"/>
+      <x:c r="R32" t="str"/>
       <x:c r="S32" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -1971,20 +1865,14 @@
         <x:v>Popularity can reveal what people want, fear, or have been persuaded by, but it does not settle what is true. Crowds can be informed, confused, manipulated, or all three at once.</x:v>
       </x:c>
       <x:c r="N33" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>Advocates of raw milk and other 'natural' wellness products often point to growing enthusiasm, celebrity uptake, or huge followings as if social momentum itself established safety or effectiveness.</x:v>
       </x:c>
       <x:c r="O33" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="P33" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="Q33" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R33" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
+        <x:v>Viral political claims are often defended with phrases like 'everyone is talking about it' or 'it has millions of views,' which confuses reach with reliability.</x:v>
+      </x:c>
+      <x:c r="P33" t="str"/>
+      <x:c r="Q33" t="str"/>
+      <x:c r="R33" t="str"/>
       <x:c r="S33" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2018,20 +1906,14 @@
         <x:v>There is an important difference between suspending belief, doubting a claim, and asserting the opposite claim. Collapsing those positions is often a way of shifting burdens that have not been earned.</x:v>
       </x:c>
       <x:c r="N34" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Religious and paranormal debates often insist that skepticism itself is just another faith commitment, as if withholding belief carried the same evidential burden as proposing the phenomenon.</x:v>
       </x:c>
       <x:c r="O34" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
-      </x:c>
-      <x:c r="P34" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="Q34" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="R34" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
-      </x:c>
+        <x:v>Arguments about election fraud and miracle claims sometimes recast 'I have not seen enough evidence' into 'you are certain it never happened' so the original claimant can dodge the burden of proof.</x:v>
+      </x:c>
+      <x:c r="P34" t="str"/>
+      <x:c r="Q34" t="str"/>
+      <x:c r="R34" t="str"/>
       <x:c r="S34" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2073,20 +1955,18 @@
         <x:v>Associations can sometimes matter when they reveal bias, incentives, or causal links. The fallacy appears when the link is treated as decisive even though it does not address the argument.</x:v>
       </x:c>
       <x:c r="N35" t="str">
+        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+      </x:c>
+      <x:c r="O35" t="str">
         <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
-      <x:c r="O35" t="str">
-        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
-      </x:c>
       <x:c r="P35" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported.</x:v>
       </x:c>
       <x:c r="Q35" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="R35" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
+        <x:v>Political arguments routinely assume that if a bad person, rival group, or disliked movement touched an idea, the idea itself must be false or tainted.</x:v>
+      </x:c>
+      <x:c r="R35" t="str"/>
       <x:c r="S35" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2122,19 +2002,19 @@
         <x:v>Confidence, volume, and repetition can make a bare assertion sound weighty, but they do not do the evidential work. When the core support is missing, the proper question is still: What is the evidence?</x:v>
       </x:c>
       <x:c r="N36" t="str">
+        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+      </x:c>
+      <x:c r="O36" t="str">
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+      </x:c>
+      <x:c r="P36" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
+      <x:c r="Q36" t="str">
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+      </x:c>
+      <x:c r="R36" t="str">
         <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="O36" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="P36" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="Q36" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
-      </x:c>
-      <x:c r="R36" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="S36" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -2171,16 +2051,16 @@
         <x:v>For rare conditions or rare events, even very accurate tests can generate more false positives than true positives. The missing question is not just 'How accurate is the test?' but 'How common is the condition before the test is applied?'</x:v>
       </x:c>
       <x:c r="N37" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="O37" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P37" t="str">
         <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
-      <x:c r="O37" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="P37" t="str">
+      <x:c r="Q37" t="str">
         <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
-      </x:c>
-      <x:c r="Q37" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="R37" t="str">
         <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
@@ -2225,17 +2105,13 @@
         <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O38" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>Conspiracy-style reasoning often treats the absence of confirming evidence as proof that the conspiracy is powerful enough to hide the evidence, which assumes the conclusion inside the explanation.</x:v>
       </x:c>
       <x:c r="P38" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q38" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="R38" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Debates about 'real journalism' or 'real science' sometimes define the trustworthy outlet or institution as whichever one already agrees with the speaker's preferred view.</x:v>
+      </x:c>
+      <x:c r="Q38" t="str"/>
+      <x:c r="R38" t="str"/>
       <x:c r="S38" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2271,20 +2147,14 @@
         <x:v>Even if a group tendency were real, it would not eliminate the need for evidence about the particular person under discussion.</x:v>
       </x:c>
       <x:c r="N39" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>After scandals in policing, finance, or clergy, critics sometimes assume any individual in the profession personally shares the worst traits of the institution.</x:v>
       </x:c>
       <x:c r="O39" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="P39" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="Q39" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="R39" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Online discourse often treats party label, employer, or religious affiliation as if it were enough to prove what a specific person believes or will do.</x:v>
+      </x:c>
+      <x:c r="P39" t="str"/>
+      <x:c r="Q39" t="str"/>
+      <x:c r="R39" t="str"/>
       <x:c r="S39" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2320,20 +2190,14 @@
         <x:v>A flattering stereotype is still a stereotype. Group membership can create a first impression, but it does not establish the individual's actual record.</x:v>
       </x:c>
       <x:c r="N40" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>Prestige effects often lead audiences to assume that anyone from a famous university or respected nonprofit is trustworthy even outside their area of expertise.</x:v>
       </x:c>
       <x:c r="O40" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="P40" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="Q40" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R40" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>Voters sometimes infer that a candidate from a reform organization must be personally honest before examining the candidate's own conduct.</x:v>
+      </x:c>
+      <x:c r="P40" t="str"/>
+      <x:c r="Q40" t="str"/>
+      <x:c r="R40" t="str"/>
       <x:c r="S40" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2371,20 +2235,14 @@
         <x:v>Repair work creates visible activity, but it mainly restores value that was lost. The missing comparison is what households, firms, insurers, and governments could have done with those same resources if the damage had not occurred.</x:v>
       </x:c>
       <x:c r="N41" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>After Hurricanes Helene and Milton in October 2024, some commentary emphasized reconstruction jobs and spending while downplaying the destroyed homes, shuttered businesses, and other uses those resources would have supported.</x:v>
       </x:c>
       <x:c r="O41" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
-      </x:c>
-      <x:c r="P41" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
-      </x:c>
-      <x:c r="Q41" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="R41" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
+        <x:v>Cyberattacks, vandalism, and infrastructure failures are sometimes framed as hidden economic stimulus because repairs employ people, even though the spending mainly compensates for an avoidable loss.</x:v>
+      </x:c>
+      <x:c r="P41" t="str"/>
+      <x:c r="Q41" t="str"/>
+      <x:c r="R41" t="str"/>
       <x:c r="S41" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2424,19 +2282,19 @@
         <x:v>Cherry picking can involve hand-picked dates, unusual baselines, isolated anecdotes, or a single study taken out of a larger research picture. The defect is not using examples, but using a biased sample as if it were representative.</x:v>
       </x:c>
       <x:c r="N42" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="O42" t="str">
+        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+      </x:c>
+      <x:c r="P42" t="str">
+        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+      </x:c>
+      <x:c r="Q42" t="str">
         <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
-      <x:c r="O42" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="P42" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="Q42" t="str">
+      <x:c r="R42" t="str">
         <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
-      </x:c>
-      <x:c r="R42" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
       </x:c>
       <x:c r="S42" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -2480,17 +2338,13 @@
         <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O43" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>Social-media arguments often dismiss older religious, philosophical, or literary texts as worthless simply because they come from a less enlightened era, skipping the actual argument.</x:v>
       </x:c>
       <x:c r="P43" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
-      <x:c r="Q43" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="R43" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
-      </x:c>
+        <x:v>People also dismiss pre-digital scholarship wholesale as outdated while still relying on concepts, institutions, and moral categories that earlier thinkers helped shape.</x:v>
+      </x:c>
+      <x:c r="Q43" t="str"/>
+      <x:c r="R43" t="str"/>
       <x:c r="S43" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2530,20 +2384,14 @@
         <x:v>Circular dynamics can be real, but identifying a loop does not show that the loop is unstoppable or that breaking one link would guarantee the hoped-for outcome. Further evidence is still needed.</x:v>
       </x:c>
       <x:c r="N44" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Job markets sometimes create genuine experience loops, but it is still a mistake to assume that every applicant locked out by the loop would necessarily succeed if only one employer made an exception.</x:v>
       </x:c>
       <x:c r="O44" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="P44" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
-      </x:c>
-      <x:c r="Q44" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
-      <x:c r="R44" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
+        <x:v>Commentators often say a platform is influential because everyone talks about it and everyone talks about it because it is influential, using the loop itself as if it settled the argument.</x:v>
+      </x:c>
+      <x:c r="P44" t="str"/>
+      <x:c r="Q44" t="str"/>
+      <x:c r="R44" t="str"/>
       <x:c r="S44" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2583,20 +2431,14 @@
         <x:v>Parts can interact in ways that change the result at the larger scale. What is beneficial, efficient, or true locally may not stay that way globally.</x:v>
       </x:c>
       <x:c r="N45" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>A company may assume that because every team is cutting costs responsibly, the organization as a whole will thrive, even though simultaneous cuts can gut the shared systems the teams depend on.</x:v>
       </x:c>
       <x:c r="O45" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="P45" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q45" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="R45" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>In policy debates, people often assume that what is prudent for one household, firm, or voter must be prudent for the entire economy or democracy at once.</x:v>
+      </x:c>
+      <x:c r="P45" t="str"/>
+      <x:c r="Q45" t="str"/>
+      <x:c r="R45" t="str"/>
       <x:c r="S45" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2632,20 +2474,18 @@
         <x:v>Confidence can track expertise, but it can also track charisma, identity, adrenaline, fear, or repeated exposure to a claim. Certainty is a psychological state, not a built-in proof.</x:v>
       </x:c>
       <x:c r="N46" t="str">
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+      </x:c>
+      <x:c r="O46" t="str">
         <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
-      <x:c r="O46" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
       <x:c r="P46" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>The anonymous ABC debate affidavit spread partly because influential accounts amplified it with extraordinary certainty before any reliable verification had appeared.</x:v>
       </x:c>
       <x:c r="Q46" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="R46" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
-      </x:c>
+        <x:v>In arguments about AI consciousness, election fraud, religion, and wellness, people often present their felt certainty as if it were itself a kind of evidence rather than something that also needs checking.</x:v>
+      </x:c>
+      <x:c r="R46" t="str"/>
       <x:c r="S46" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2683,20 +2523,14 @@
         <x:v>Adding conditions never makes a claim more probable than a broader version of that same claim. Extra detail can make a story feel more representative while making it statistically less likely.</x:v>
       </x:c>
       <x:c r="N47" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Political profiling often mistakes a vivid stereotype for probability, assuming that a person matching one trait is more likely to match an even narrower bundle of traits as well.</x:v>
       </x:c>
       <x:c r="O47" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="P47" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="Q47" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R47" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
+        <x:v>AI narratives sometimes suggest that because a model appears articulate, it is more likely to be both highly capable and aligned than merely capable, even though the conjunction is narrower.</x:v>
+      </x:c>
+      <x:c r="P47" t="str"/>
+      <x:c r="Q47" t="str"/>
+      <x:c r="R47" t="str"/>
       <x:c r="S47" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2738,20 +2572,18 @@
         <x:v>Shortening a quote is not automatically deceptive. The fallacy appears when the omitted context would materially change how a fair reader understands the statement.</x:v>
       </x:c>
       <x:c r="N48" t="str">
+        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+      </x:c>
+      <x:c r="O48" t="str">
         <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
-      <x:c r="O48" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
       <x:c r="P48" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Edited debate clips, viral subtitled videos, and quote-card politics in 2024 regularly removed the surrounding setup, qualifier, or punchline that made the original meaning very different.</x:v>
       </x:c>
       <x:c r="Q48" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="R48" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
+        <x:v>Public figures and partisans often quote one alarming sentence from a report, study, or speech while cutting the lines that immediately limit, explain, or even reverse the apparent claim.</x:v>
+      </x:c>
+      <x:c r="R48" t="str"/>
       <x:c r="S48" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2791,20 +2623,14 @@
         <x:v>Many real concepts come in degrees. Vagueness at the boundary does not make the broader concept meaningless or unusable.</x:v>
       </x:c>
       <x:c r="N49" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Arguments about misinformation, bias, wealth, addiction, and consciousness often demand an impossible razor-sharp line and then pretend the lack of that line defeats the concept altogether.</x:v>
       </x:c>
       <x:c r="O49" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="P49" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="Q49" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="R49" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
+        <x:v>In everyday disputes, someone may deny that a delay was 'too long' or a fee was 'too high' simply because no exact threshold was announced in advance.</x:v>
+      </x:c>
+      <x:c r="P49" t="str"/>
+      <x:c r="Q49" t="str"/>
+      <x:c r="R49" t="str"/>
       <x:c r="S49" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2842,19 +2668,19 @@
         <x:v>Correlations matter because they can reveal patterns worth investigating. The fallacy is jumping straight from 'these moved together' to 'this caused that' without checking mechanisms, timing, controls, or alternative explanations.</x:v>
       </x:c>
       <x:c r="N50" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="O50" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P50" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="Q50" t="str">
         <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
-      <x:c r="O50" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="P50" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="Q50" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
       <x:c r="R50" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>Claims about teen mental health and social media often move too quickly from parallel trend lines to a settled single-cause story, even though researchers still debate the size, direction, and mechanisms of the effect.</x:v>
       </x:c>
       <x:c r="S50" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -2896,17 +2722,13 @@
         <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O51" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Culture-war debates often define words like 'freedom,' 'woman,' 'democracy,' or 'terrorism' in ways that quietly smuggle the desired conclusion into the starting point.</x:v>
       </x:c>
       <x:c r="P51" t="str">
-        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
-      </x:c>
-      <x:c r="Q51" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="R51" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
+        <x:v>Moral and political disputes frequently collapse into dictionary wars where one side pretends that owning the label settles the argument.</x:v>
+      </x:c>
+      <x:c r="Q51" t="str"/>
+      <x:c r="R51" t="str"/>
       <x:c r="S51" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2944,14 +2766,12 @@
         <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="P52" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+        <x:v>Public disputes about climate, evolution, and health regularly treat unresolved details in the mechanism as if they erased the larger evidential picture.</x:v>
       </x:c>
       <x:c r="Q52" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
-      </x:c>
-      <x:c r="R52" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Research on AI transcription errors in 2024 showed that systems were inventing statements people never said; even before every technical cause was nailed down, the pattern itself was already evidence of a real reliability problem.</x:v>
+      </x:c>
+      <x:c r="R52" t="str"/>
       <x:c r="S52" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -2994,17 +2814,13 @@
         <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O53" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>Conspiracy claims about noncitizen voting, ballot destruction, or machine tampering often survive by demanding that every rumor be individually disproved rather than by presenting strong evidence that the conspiracy exists.</x:v>
       </x:c>
       <x:c r="P53" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="Q53" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="R53" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
+        <x:v>Miracle, UFO, and paranormal arguments frequently say skeptics must show exactly what happened in each case, as though the claimant had no burden until that impossible task is finished.</x:v>
+      </x:c>
+      <x:c r="Q53" t="str"/>
+      <x:c r="R53" t="str"/>
       <x:c r="S53" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3038,20 +2854,14 @@
         <x:v>Responsible belief often comes in degrees. Treating confidence as all-or-nothing hides uncertainty, nuance, and the actual strength of the evidence.</x:v>
       </x:c>
       <x:c r="N54" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>Debates about God, UFOs, AI consciousness, and election fraud often demand yes-or-no declarations even when the intellectually honest position is conditional, partial, or still under revision.</x:v>
       </x:c>
       <x:c r="O54" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
-      </x:c>
-      <x:c r="P54" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q54" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="R54" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
+        <x:v>Culture-war exchanges frequently treat probabilistic language such as 'unlikely,' 'not yet shown,' or 'some evidence but not enough' as weakness rather than as proper calibration.</x:v>
+      </x:c>
+      <x:c r="P54" t="str"/>
+      <x:c r="Q54" t="str"/>
+      <x:c r="R54" t="str"/>
       <x:c r="S54" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3085,20 +2895,14 @@
         <x:v>A remote hypothetical can still be useful when the issue is whether a rule really holds without exception. Improbable cases often expose hidden limits in principles that sounded absolute.</x:v>
       </x:c>
       <x:c r="N55" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>Arguments about free speech, self-defense, abortion, lying, and triage often reject hard edge cases simply because they are uncomfortable, even though those cases are precisely what test universal rules.</x:v>
       </x:c>
       <x:c r="O55" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="P55" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="Q55" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="R55" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Policy debates about AI safety and biosecurity sometimes wave away low-probability scenarios too quickly, even when the whole argument concerns whether a system is robust under stress.</x:v>
+      </x:c>
+      <x:c r="P55" t="str"/>
+      <x:c r="Q55" t="str"/>
+      <x:c r="R55" t="str"/>
       <x:c r="S55" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3142,14 +2946,12 @@
         <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="P56" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Debates about expertise often assume that if a source lacks one credential or prestige marker, there can be no meaningful evidence at all in what it says.</x:v>
       </x:c>
       <x:c r="Q56" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="R56" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
+        <x:v>In everyday arguments, people often assume that if the ideal cause is absent, the observed effect cannot still arise through another path.</x:v>
+      </x:c>
+      <x:c r="R56" t="str"/>
       <x:c r="S56" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3187,20 +2989,14 @@
         <x:v>Some concepts only make sense against their correlative opposite. Erasing the contrast does not answer the accusation; it changes the meaning of the term.</x:v>
       </x:c>
       <x:c r="N57" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>Public arguments sometimes say a decision cannot count as censorship unless it was total state control, effectively denying any middle range where the term usefully applies.</x:v>
       </x:c>
       <x:c r="O57" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="P57" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q57" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R57" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Debates about betrayal, fraud, or coercion often narrow the term so drastically that almost no real case can qualify.</x:v>
+      </x:c>
+      <x:c r="P57" t="str"/>
+      <x:c r="Q57" t="str"/>
+      <x:c r="R57" t="str"/>
       <x:c r="S57" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3240,20 +3036,14 @@
         <x:v>A whole can have properties its parts do not share equally. Group-level success, size, reputation, or wealth does not automatically distribute itself down to each component.</x:v>
       </x:c>
       <x:c r="N58" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>People often infer that because a country is rich, any given citizen must be comfortable, skipping inequality, regional gaps, and individual circumstance.</x:v>
       </x:c>
       <x:c r="O58" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="P58" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q58" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R58" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>A popular movement, successful company, or prestigious institution can still contain weak teams, poor ideas, or underfunded units.</x:v>
+      </x:c>
+      <x:c r="P58" t="str"/>
+      <x:c r="Q58" t="str"/>
+      <x:c r="R58" t="str"/>
       <x:c r="S58" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3295,20 +3085,14 @@
         <x:v>Aggregate data can be useful, but it does not tell you where any one individual falls within the distribution. Group averages do not erase overlap, variation, or outliers.</x:v>
       </x:c>
       <x:c r="N59" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>Zip-code analytics, polling blocs, and demographic summaries are often treated as if they gave a direct reading of the motives or traits of each person inside the category.</x:v>
       </x:c>
       <x:c r="O59" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="P59" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="Q59" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="R59" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Political commentary frequently talks as if 'suburban women,' 'young men,' or 'college voters' were internally uniform rather than broad, heterogeneous groups.</x:v>
+      </x:c>
+      <x:c r="P59" t="str"/>
+      <x:c r="Q59" t="str"/>
+      <x:c r="R59" t="str"/>
       <x:c r="S59" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3340,20 +3124,14 @@
         <x:v>Not every conversation requires a full essay, but a real refutation still has to point to some error in reasoning, evidence, or interpretation. Mere dismissal is not argument.</x:v>
       </x:c>
       <x:c r="N60" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Online fights about elections, Israel and Gaza, climate, and AI often rely on 'debunked' as a performance word rather than as a pointer to the actual evidence.</x:v>
       </x:c>
       <x:c r="O60" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
-      <x:c r="P60" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="Q60" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="R60" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>In fast-moving social media disputes, people often treat tone, certainty, and pile-on consensus as if they were enough to count as refutation.</x:v>
+      </x:c>
+      <x:c r="P60" t="str"/>
+      <x:c r="Q60" t="str"/>
+      <x:c r="R60" t="str"/>
       <x:c r="S60" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3389,20 +3167,14 @@
         <x:v>Beliefs can change mood, confidence, behavior, pain perception, and group cohesion regardless of whether their object exists. The benefits of belief do not by themselves settle the ontology.</x:v>
       </x:c>
       <x:c r="N61" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>Raw milk, supplement, and alternative-health advocates often point to the felt benefits reported by believers while skipping the role of expectation, placebo effects, and other background changes.</x:v>
       </x:c>
       <x:c r="O61" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="P61" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q61" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="R61" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
+        <x:v>Arguments that religion must be true because believers report comfort, purpose, or improved well-being often confuse the power of belief with evidence for the reality of the object believed in.</x:v>
+      </x:c>
+      <x:c r="P61" t="str"/>
+      <x:c r="Q61" t="str"/>
+      <x:c r="R61" t="str"/>
       <x:c r="S61" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3444,14 +3216,12 @@
         <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="P62" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Debates over content moderation regularly equivocate between censorship by the state and moderation decisions by private platforms, as if both were the same kind of speech restriction.</x:v>
       </x:c>
       <x:c r="Q62" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R62" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
+        <x:v>Public discussion of AI often slides between thin technical meanings of words such as 'reasoning,' 'understanding,' or 'hallucination' and thicker human meanings, which makes claims sound stronger than the evidence warrants.</x:v>
+      </x:c>
+      <x:c r="R62" t="str"/>
       <x:c r="S62" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3487,20 +3257,14 @@
         <x:v>The argument trades on the prestige or emotional force of the stronger meaning while relying on the thinner meaning when challenged.</x:v>
       </x:c>
       <x:c r="N63" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>Public arguments about censorship often slide from the general fact that content was moderated to the much stronger charge that it was censored in the same sense as state suppression.</x:v>
       </x:c>
       <x:c r="O63" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="P63" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q63" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="R63" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>AI marketing repeatedly benefits from equivocation between technical terms such as 'learn,' 'reason,' or 'understand' and their thicker human meanings.</x:v>
+      </x:c>
+      <x:c r="P63" t="str"/>
+      <x:c r="Q63" t="str"/>
+      <x:c r="R63" t="str"/>
       <x:c r="S63" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3536,20 +3300,14 @@
         <x:v>Words change through use. Present meaning is set by current linguistic convention, not by the oldest recoverable ancestor of the term.</x:v>
       </x:c>
       <x:c r="N64" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>Culture-war and identity debates often turn into fights over what labels 'really mean' based on older usage rather than on how the community currently uses them.</x:v>
       </x:c>
       <x:c r="O64" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="P64" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="Q64" t="str">
-        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
-      </x:c>
-      <x:c r="R64" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
+        <x:v>People sometimes defend or condemn a term by appealing to its root language while ignoring the fact that social meaning has moved far beyond the origin.</x:v>
+      </x:c>
+      <x:c r="P64" t="str"/>
+      <x:c r="Q64" t="str"/>
+      <x:c r="R64" t="str"/>
       <x:c r="S64" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3588,17 +3346,13 @@
         <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O65" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>Identity arguments sometimes pile up statements about what two groups are not and then pretend that the missing positive relation has somehow been proved.</x:v>
       </x:c>
       <x:c r="P65" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q65" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R65" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
+        <x:v>This form often hides inside rhetorical contrasts where speakers rely on the sound of elimination rather than a genuine logical bridge.</x:v>
+      </x:c>
+      <x:c r="Q65" t="str"/>
+      <x:c r="R65" t="str"/>
       <x:c r="S65" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3637,17 +3391,13 @@
         <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="O66" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>Arguments about 'the average user,' 'the typical elite,' or 'the real moderate voter' sometimes slip from a hypothetical category into the assumption that a concrete instance must exist.</x:v>
       </x:c>
       <x:c r="P66" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="Q66" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R66" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Formal and theological debates alike often move too quickly from what would be true if something existed to the claim that it therefore does exist.</x:v>
+      </x:c>
+      <x:c r="Q66" t="str"/>
+      <x:c r="R66" t="str"/>
       <x:c r="S66" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3685,20 +3435,14 @@
         <x:v>A loaded question can force a false choice because any direct answer seems to concede what the question improperly assumed. The first task is often to challenge the hidden premise, not to answer on its terms.</x:v>
       </x:c>
       <x:c r="N67" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+        <x:v>Debates about religion, politics, and gender often turn on questions that quietly presuppose bad faith, delusion, or malicious intent before any of that has been shown.</x:v>
       </x:c>
       <x:c r="O67" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="P67" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="Q67" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="R67" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
+        <x:v>Interviewers and posters sometimes frame questions so that merely engaging already concedes the accusation, especially in culture-war exchanges built for clipping and outrage.</x:v>
+      </x:c>
+      <x:c r="P67" t="str"/>
+      <x:c r="Q67" t="str"/>
+      <x:c r="R67" t="str"/>
       <x:c r="S67" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3736,20 +3480,14 @@
         <x:v>Some predicates are necessary only relative to a present state or definition. That necessity does not magically extend across time, possibility, or changed conditions.</x:v>
       </x:c>
       <x:c r="N68" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>People sometimes move from 'this rule currently defines the category' to 'therefore the category could never be revised or altered,' confusing present convention with fixed necessity.</x:v>
       </x:c>
       <x:c r="O68" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="P68" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q68" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="R68" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>In institutional debates, a temporary legal or procedural status is often spoken of as if it were an immutable fact about what can never happen.</x:v>
+      </x:c>
+      <x:c r="P68" t="str"/>
+      <x:c r="Q68" t="str"/>
+      <x:c r="R68" t="str"/>
       <x:c r="S68" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3787,20 +3525,14 @@
         <x:v>Analogies can clarify unfamiliar ideas, but they prove very little unless the shared features are actually relevant to the conclusion being drawn.</x:v>
       </x:c>
       <x:c r="N69" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Debates about AI frequently compare models to children, interns, parrots, or brains, then carry over conclusions from the analogy that the underlying system may not support.</x:v>
       </x:c>
       <x:c r="O69" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="P69" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="Q69" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R69" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
+        <x:v>Fiscal debates often compare a national budget to a household budget; the analogy can illuminate some constraints but breaks down when it is treated as a full map of macroeconomics.</x:v>
+      </x:c>
+      <x:c r="P69" t="str"/>
+      <x:c r="Q69" t="str"/>
+      <x:c r="R69" t="str"/>
       <x:c r="S69" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3847,10 +3579,10 @@
         <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="Q70" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>The anonymous affidavit circulated after the September 2024 ABC debate was amplified as if it were a verified insider source even though the core allegations were not authenticated.</x:v>
       </x:c>
       <x:c r="R70" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Viral quote cards and screenshot posts often attach dramatic claims to scientists, judges, or agencies who never said them, counting on readers to trust the label instead of checking the source.</x:v>
       </x:c>
       <x:c r="S70" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -3898,10 +3630,10 @@
         <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
       </x:c>
       <x:c r="Q71" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Coverage of climate change, vaccine safety, and election administration often becomes misleading when fringe claims are presented as if they stand on equal footing with the evidential consensus.</x:v>
       </x:c>
       <x:c r="R71" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>Public moderators sometimes treat a polished unsupported claim and a well-supported cautious claim as equivalent contributions simply because both parties are speaking confidently.</x:v>
       </x:c>
       <x:c r="S71" t="str">
         <x:v>added-2026-completeness-pass</x:v>
@@ -3943,17 +3675,13 @@
         <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="O72" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Coverage of climate, public health, and election integrity can slide into 'both sides' framing that treats consensus and fringe denial as if splitting the difference were balanced or fair.</x:v>
       </x:c>
       <x:c r="P72" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q72" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="R72" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
+        <x:v>In personal and workplace disputes, people often assume each side must be equally at fault, even when the evidence is lopsided.</x:v>
+      </x:c>
+      <x:c r="Q72" t="str"/>
+      <x:c r="R72" t="str"/>
       <x:c r="S72" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -3991,19 +3719,19 @@
         <x:v>The pressure comes from pretending that a complex decision has only two doors. Sometimes the omitted alternatives are compromises, phased approaches, or the option of rejecting the framing altogether.</x:v>
       </x:c>
       <x:c r="N73" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="O73" t="str">
+        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+      </x:c>
+      <x:c r="P73" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="Q73" t="str">
         <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
-      <x:c r="O73" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="P73" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="Q73" t="str">
+      <x:c r="R73" t="str">
         <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
-      <x:c r="R73" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="S73" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -4042,19 +3770,19 @@
         <x:v>Two things can share some features without being equal in scale, intent, risk, or moral significance. The fallacy appears when a superficial resemblance is used to flatten those differences into sameness.</x:v>
       </x:c>
       <x:c r="N74" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="O74" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="P74" t="str">
+        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+      </x:c>
+      <x:c r="Q74" t="str">
         <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
-      <x:c r="O74" t="str">
+      <x:c r="R74" t="str">
         <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="P74" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="Q74" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
-      </x:c>
-      <x:c r="R74" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="S74" t="str">
         <x:v>added-2026-completeness-pass</x:v>
@@ -4097,20 +3825,14 @@
         <x:v>Real uncertainty exists, and sometimes compromise is appropriate. The fallacy appears when manufactured neutrality is used to protect a losing claim from the consequences of the evidence.</x:v>
       </x:c>
       <x:c r="N75" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+        <x:v>Public arguments about evolution, election claims, and medical misinformation sometimes ask audiences to treat both sides as equally plausible even after the evidential balance is lopsided.</x:v>
       </x:c>
       <x:c r="O75" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
-      <x:c r="P75" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="Q75" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="R75" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
+        <x:v>In online debate culture, a retreat into 'everyone has their own truth' often appears right after a concrete factual claim has gone badly for one side.</x:v>
+      </x:c>
+      <x:c r="P75" t="str"/>
+      <x:c r="Q75" t="str"/>
+      <x:c r="R75" t="str"/>
       <x:c r="S75" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4150,19 +3872,19 @@
         <x:v>Generalization is unavoidable, but it has to be scaled to the quality, size, and representativeness of the evidence. The problem is not generalizing at all; it is generalizing too aggressively.</x:v>
       </x:c>
       <x:c r="N76" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="O76" t="str">
         <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
       <x:c r="P76" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
       <x:c r="Q76" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>Viral anecdotes about migrants, students, police, or AI tools often get inflated into sweeping claims about entire groups or systems after only a handful of cases.</x:v>
       </x:c>
       <x:c r="R76" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>Election and media arguments routinely take one error, one clip, or one scandal as proof that the whole institution always behaves the same way.</x:v>
       </x:c>
       <x:c r="S76" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -4197,20 +3919,14 @@
         <x:v>Reasoning from an assumption to test its implications is not the same as endorsing the assumption.</x:v>
       </x:c>
       <x:c r="N77" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>Reductio arguments in theology, AI, and politics are often misread as confessions rather than as tests of what would follow if the other side's claim were granted.</x:v>
       </x:c>
       <x:c r="O77" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="P77" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q77" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="R77" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
-      </x:c>
+        <x:v>Debates stall when a conditional claim such as 'even if you are right, the consequence would still be unacceptable' is treated as if it were a statement of belief.</x:v>
+      </x:c>
+      <x:c r="P77" t="str"/>
+      <x:c r="Q77" t="str"/>
+      <x:c r="R77" t="str"/>
       <x:c r="S77" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4246,20 +3962,14 @@
         <x:v>The surface wording can make the argument sound tidy, but the hidden term shift breaks the structure. A reused word is not enough; it has to keep the same meaning.</x:v>
       </x:c>
       <x:c r="N78" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Public arguments often slide between technical and ordinary meanings of words like 'theory,' 'freedom,' 'bias,' or 'intelligence,' then pretend the resulting syllogism is valid.</x:v>
       </x:c>
       <x:c r="O78" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="P78" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="Q78" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R78" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Because the same label can carry prestige in one context and a thinner meaning in another, term shifts often smuggle in conclusions the premises did not support.</x:v>
+      </x:c>
+      <x:c r="P78" t="str"/>
+      <x:c r="Q78" t="str"/>
+      <x:c r="R78" t="str"/>
       <x:c r="S78" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4299,20 +4009,14 @@
         <x:v>Random sequences naturally contain streaks. When the events are truly independent, the next event does not remember the last one.</x:v>
       </x:c>
       <x:c r="N79" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>People sometimes feel that after many routine flights or medical screenings in a row, a disaster or diagnosis is somehow 'due,' even though independent risks do not balance themselves that way.</x:v>
       </x:c>
       <x:c r="O79" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="P79" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="Q79" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="R79" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
-      </x:c>
+        <x:v>In gambling and investing language, talk of a roulette table or slot machine being 'ready to pay out' often confuses a streaky pattern with a real shift in odds.</x:v>
+      </x:c>
+      <x:c r="P79" t="str"/>
+      <x:c r="Q79" t="str"/>
+      <x:c r="R79" t="str"/>
       <x:c r="S79" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4352,20 +4056,14 @@
         <x:v>Origins can matter when they reveal bias, incentives, or reliability concerns. The fallacy appears when origin is treated as enough to settle the issue without examining the claim itself.</x:v>
       </x:c>
       <x:c r="N80" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported.</x:v>
       </x:c>
       <x:c r="O80" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="P80" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="Q80" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R80" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
+        <x:v>In cultural and religious arguments, a practice or symbol is often condemned solely because of its historical roots, even when the live question is what it means or does now.</x:v>
+      </x:c>
+      <x:c r="P80" t="str"/>
+      <x:c r="Q80" t="str"/>
+      <x:c r="R80" t="str"/>
       <x:c r="S80" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4410,16 +4108,16 @@
         <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="O81" t="str">
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+      </x:c>
+      <x:c r="P81" t="str">
         <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
-      <x:c r="P81" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
       <x:c r="Q81" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+        <x:v>A single viral video of a fight, theft, or protest is often used online as if it reveals what a whole city, campus, or demographic group is like.</x:v>
       </x:c>
       <x:c r="R81" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>Election commentary frequently treats one poll, one county, or one diner focus group as proof of a national shift, even when the broader polling picture is mixed.</x:v>
       </x:c>
       <x:c r="S81" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -4456,20 +4154,14 @@
         <x:v>Hindsight compresses uncertainty and highlights the clues that mattered. Real historical agents were working inside a noisier, more limited information environment.</x:v>
       </x:c>
       <x:c r="N82" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+        <x:v>People often imagine they would easily have rejected past medical myths, empires, or moral blind spots, underestimating how strongly institutions and available evidence shape belief.</x:v>
       </x:c>
       <x:c r="O82" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="P82" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="Q82" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
-      <x:c r="R82" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
+        <x:v>Post-crisis commentary regularly rewrites messy contingencies into obvious warning signs that were supposedly plain to everyone at the time.</x:v>
+      </x:c>
+      <x:c r="P82" t="str"/>
+      <x:c r="Q82" t="str"/>
+      <x:c r="R82" t="str"/>
       <x:c r="S82" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4507,20 +4199,14 @@
         <x:v>If the inner observer can already do the job, the original explanatory problem just reappears one level down.</x:v>
       </x:c>
       <x:c r="N83" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>Popular neuroscience writing sometimes says that the brain 'decides' or a memory center 'knows' in ways that merely rename the puzzle rather than explain it.</x:v>
       </x:c>
       <x:c r="O83" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="P83" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="Q83" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R83" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
+        <x:v>Criticism of AI can do something similar when it assumes a hidden module inside the system literally understands the output in the same way a person would.</x:v>
+      </x:c>
+      <x:c r="P83" t="str"/>
+      <x:c r="Q83" t="str"/>
+      <x:c r="R83" t="str"/>
       <x:c r="S83" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4560,20 +4246,14 @@
         <x:v>Institutional labels can matter legally or practically, but they do not by themselves create truth, value, or natural kinds.</x:v>
       </x:c>
       <x:c r="N84" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>Markets and media often confuse approved, certified, or official with true, safe, or just.</x:v>
       </x:c>
       <x:c r="O84" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="P84" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q84" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="R84" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
+        <x:v>Political rhetoric often treats whatever a legislature recognizes or forbids as automatically morally right or wrong.</x:v>
+      </x:c>
+      <x:c r="P84" t="str"/>
+      <x:c r="Q84" t="str"/>
+      <x:c r="R84" t="str"/>
       <x:c r="S84" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4609,20 +4289,14 @@
         <x:v>This is not mere nuance. The problem is rhetorical double-speaking that blurs real disagreement by sliding between incompatible senses of the same label.</x:v>
       </x:c>
       <x:c r="N85" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Politicians often define contested terms like 'freedom,' 'censorship,' 'riot,' 'peaceful,' or 'family values' one way for sympathetic listeners and another way when challenged by critics.</x:v>
       </x:c>
       <x:c r="O85" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="P85" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
-      <x:c r="Q85" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R85" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
+        <x:v>Debates about AI, speech, and policing frequently proceed as if both camps agree until someone notices that the central term has been doing two very different jobs.</x:v>
+      </x:c>
+      <x:c r="P85" t="str"/>
+      <x:c r="Q85" t="str"/>
+      <x:c r="R85" t="str"/>
       <x:c r="S85" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4658,20 +4332,14 @@
         <x:v>Excluding one group from a subset does not exclude it from the wider property attached to that subset. The conclusion reaches further than the premises license.</x:v>
       </x:c>
       <x:c r="N86" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Stereotype arguments often move from 'all members of group A have trait B' and 'group C is not group A' to 'therefore group C lacks trait B,' which does not follow.</x:v>
       </x:c>
       <x:c r="O86" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="P86" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="Q86" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="R86" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
+        <x:v>This pattern appears when people treat one pathway to fame, corruption, risk, or success as if it were the only pathway.</x:v>
+      </x:c>
+      <x:c r="P86" t="str"/>
+      <x:c r="Q86" t="str"/>
+      <x:c r="R86" t="str"/>
       <x:c r="S86" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4705,20 +4373,14 @@
         <x:v>A claim that survives every observation unchanged may be emotionally resilient, but it has surrendered explanatory power.</x:v>
       </x:c>
       <x:c r="N87" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Conspiracy systems often explain both the presence and the absence of evidence as confirmation.</x:v>
       </x:c>
       <x:c r="O87" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="P87" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="Q87" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="R87" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>Some technology hype frames both success and failure as proof that general intelligence is just around the corner.</x:v>
+      </x:c>
+      <x:c r="P87" t="str"/>
+      <x:c r="Q87" t="str"/>
+      <x:c r="R87" t="str"/>
       <x:c r="S87" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4757,17 +4419,13 @@
         <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
       </x:c>
       <x:c r="O88" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>Campaign arguments about the economy often isolate one metric such as gas prices, job totals, or stock indexes and treat that single comparison as if it captured the whole condition of household life.</x:v>
       </x:c>
       <x:c r="P88" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q88" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R88" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
+        <x:v>Technology marketing frequently calls a new tool 'more productive' without clarifying productive for whom, under what workflow, at what error rate, and at what human cost.</x:v>
+      </x:c>
+      <x:c r="Q88" t="str"/>
+      <x:c r="R88" t="str"/>
       <x:c r="S88" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4805,20 +4463,14 @@
         <x:v>A complete comparison needs a consistent baseline or a transparent weighting of tradeoffs, not a collage of unrelated best cases.</x:v>
       </x:c>
       <x:c r="N89" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Consumer ads often compare each feature against whichever rival looks weakest on that feature, then announce overall superiority.</x:v>
       </x:c>
       <x:c r="O89" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="P89" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q89" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="R89" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
+        <x:v>Campaign brag sheets sometimes do the same by mixing job growth, crime, housing, and graduation metrics against different jurisdictions and different years.</x:v>
+      </x:c>
+      <x:c r="P89" t="str"/>
+      <x:c r="Q89" t="str"/>
+      <x:c r="R89" t="str"/>
       <x:c r="S89" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4856,20 +4508,14 @@
         <x:v>Authorial intent is not always the only thing that matters, but it is often part of the evidence. Declaring it irrelevant by default can flatten interpretation into projection.</x:v>
       </x:c>
       <x:c r="N90" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Debates over constitutional language, literature, and political slogans often swing too far toward present-day interpretation while discarding what the author or framers were trying to do.</x:v>
       </x:c>
       <x:c r="O90" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="P90" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="Q90" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="R90" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
+        <x:v>Online arguments about memes, jokes, and clips frequently ignore context and stated intent altogether, then treat the most inflammatory possible reading as the only serious one.</x:v>
+      </x:c>
+      <x:c r="P90" t="str"/>
+      <x:c r="Q90" t="str"/>
+      <x:c r="R90" t="str"/>
       <x:c r="S90" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4907,20 +4553,14 @@
         <x:v>An ought needs a normative premise about goals, duties, or values. Facts alone do not generate that extra step.</x:v>
       </x:c>
       <x:c r="N91" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Arguments about gender, family, and competition often slide from claims about what is common in nature to claims about what is therefore morally required.</x:v>
       </x:c>
       <x:c r="O91" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="P91" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="Q91" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="R91" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Workplace norms are regularly defended by saying they are simply how the market works, even when the moral question is precisely whether the market should work that way.</x:v>
+      </x:c>
+      <x:c r="P91" t="str"/>
+      <x:c r="Q91" t="str"/>
+      <x:c r="R91" t="str"/>
       <x:c r="S91" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -4958,20 +4598,14 @@
         <x:v>Some labels are fair descriptions, but the fallacy appears when the emotional sting of the label is doing the work that evidence and argument have not done.</x:v>
       </x:c>
       <x:c r="N92" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+        <x:v>Words like 'groomer,' 'traitor,' 'fascist,' 'woke,' 'cultist,' and 'denier' are often deployed less to clarify than to trigger a moral reaction before the argument can be examined.</x:v>
       </x:c>
       <x:c r="O92" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="P92" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="Q92" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
-      <x:c r="R92" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
+        <x:v>Political and religious arguments frequently pre-load the conclusion by choosing terms that make disagreement sound shameful or corrupt from the start.</x:v>
+      </x:c>
+      <x:c r="P92" t="str"/>
+      <x:c r="Q92" t="str"/>
+      <x:c r="R92" t="str"/>
       <x:c r="S92" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5005,20 +4639,14 @@
         <x:v>Many real systems change slowly at first, then rapidly, then plateau, or even reverse after a threshold.</x:v>
       </x:c>
       <x:c r="N93" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>Growth forecasts for social platforms often assume audience reach will keep scaling smoothly even after attention markets saturate.</x:v>
       </x:c>
       <x:c r="O93" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
-      </x:c>
-      <x:c r="P93" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="Q93" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="R93" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
-      </x:c>
+        <x:v>Policy debates about climate, housing, and healthcare frequently ignore the non-linear effects of bottlenecks, incentives, and behavioral feedback.</x:v>
+      </x:c>
+      <x:c r="P93" t="str"/>
+      <x:c r="Q93" t="str"/>
+      <x:c r="R93" t="str"/>
       <x:c r="S93" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5060,14 +4688,12 @@
         <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="P94" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>Debates over generative AI in 2024 often jumped straight from 'this automates part of my job' to 'therefore it will inevitably make people broadly unemployable,' skipping the more complicated evidence about substitution, augmentation, and new roles.</x:v>
       </x:c>
       <x:c r="Q94" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="R94" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
+        <x:v>The U.S. dockworker fight over port automation in October 2024 showed why the issue is serious, but it also illustrated the need to distinguish real bargaining and transition questions from the blanket claim that productivity-enhancing technology is always socially worse.</x:v>
+      </x:c>
+      <x:c r="R94" t="str"/>
       <x:c r="S94" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5103,20 +4729,14 @@
         <x:v>In ordinary factual contexts, identical referents can be substituted safely. In belief, knowledge, or perception contexts, that move can fail because the speaker's information is incomplete.</x:v>
       </x:c>
       <x:c r="N95" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>This fallacy shows up whenever people infer identity or non-identity from what someone knows, recognizes, or can name rather than from the underlying facts.</x:v>
       </x:c>
       <x:c r="O95" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="P95" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q95" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R95" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
+        <x:v>Mystery, anonymity, and pseudonym debates often slide into this mistake by assuming that not knowing a description means the object cannot be the same one known under another description.</x:v>
+      </x:c>
+      <x:c r="P95" t="str"/>
+      <x:c r="Q95" t="str"/>
+      <x:c r="R95" t="str"/>
       <x:c r="S95" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5158,19 +4778,19 @@
         <x:v>Vivid cases matter, especially when they reveal harms abstract statistics can hide. The fallacy arises when memorable exceptions are used as if they were the normal pattern.</x:v>
       </x:c>
       <x:c r="N96" t="str">
+        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+      </x:c>
+      <x:c r="O96" t="str">
+        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+      </x:c>
+      <x:c r="P96" t="str">
         <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="O96" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="P96" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="Q96" t="str">
         <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="R96" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>The Springfield rumor gained traction partly because lurid, memorable imagery traveled faster than the dull but crucial fact that authorities found no supporting evidence.</x:v>
       </x:c>
       <x:c r="S96" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -5214,17 +4834,13 @@
         <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O97" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Public AI debates in 2024 often moved from benchmark scores to some new test the moment a model cleared the previous bar, making 'proof' of competence permanently out of reach.</x:v>
       </x:c>
       <x:c r="P97" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="Q97" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="R97" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
+        <x:v>Election-conspiracy arguments often work this way: once courts, audits, and recounts address one claim, the standard shifts to a different alleged irregularity without any willingness to concede what the earlier evidence settled.</x:v>
+      </x:c>
+      <x:c r="Q97" t="str"/>
+      <x:c r="R97" t="str"/>
       <x:c r="S97" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5265,17 +4881,13 @@
         <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="O98" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>The 2026 push to expand raw milk access often leaned on the idea that unprocessed equals healthier, despite repeated warnings from public-health officials that the safety risks are real and the claimed benefits remain unproven.</x:v>
       </x:c>
       <x:c r="P98" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="Q98" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="R98" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Wellness marketing routinely sells herbs, supplements, detoxes, and hormone routines by invoking nature itself as if natural origin settled the medical question.</x:v>
+      </x:c>
+      <x:c r="Q98" t="str"/>
+      <x:c r="R98" t="str"/>
       <x:c r="S98" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5311,20 +4923,14 @@
         <x:v>The rational status of a claim depends on the evidence for it, not on whether someone has managed to close every imaginable contrary possibility.</x:v>
       </x:c>
       <x:c r="N99" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Election, paranormal, and conspiracy claims often survive by saying 'you cannot prove it did not happen,' as if that absence of disproof supplied positive warrant.</x:v>
       </x:c>
       <x:c r="O99" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="P99" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q99" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R99" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Skeptics can also commit the reverse mistake when they treat an unproved claim as definitively false rather than merely unestablished.</x:v>
+      </x:c>
+      <x:c r="P99" t="str"/>
+      <x:c r="Q99" t="str"/>
+      <x:c r="R99" t="str"/>
       <x:c r="S99" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5360,20 +4966,14 @@
         <x:v>Most policies, tools, and institutions are partial fixes. The right question is often whether an option improves matters relative to feasible alternatives, not whether it achieves a flawless end state.</x:v>
       </x:c>
       <x:c r="N100" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Critics of content moderation, election safeguards, AI guardrails, and climate policy often reject incremental measures on the grounds that bad cases will still exist, as if imperfection erased all value.</x:v>
       </x:c>
       <x:c r="O100" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="P100" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="Q100" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R100" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
+        <x:v>Debates about public-health interventions frequently collapse into 'if it does not stop every case, it failed,' which compares reality to fantasy rather than to the available alternatives.</x:v>
+      </x:c>
+      <x:c r="P100" t="str"/>
+      <x:c r="Q100" t="str"/>
+      <x:c r="R100" t="str"/>
       <x:c r="S100" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5417,20 +5017,14 @@
         <x:v>Sometimes categories do have genuine criteria. The fallacy arises when the criteria are improvised only after a counterexample appears, so the definition changes to save the claim.</x:v>
       </x:c>
       <x:c r="N101" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>In 2024 intraparty fights, Republicans who backed Ukraine aid or accepted the 2020 certification were often dismissed as 'not real conservatives' instead of being treated as counterexamples within conservatism.</x:v>
       </x:c>
       <x:c r="O101" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="P101" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="Q101" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="R101" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
+        <x:v>Religious and ideological arguments frequently insist that anyone whose behavior embarrasses the group was never a 'true' believer in the first place, which preserves group purity by redefinition.</x:v>
+      </x:c>
+      <x:c r="P101" t="str"/>
+      <x:c r="Q101" t="str"/>
+      <x:c r="R101" t="str"/>
       <x:c r="S101" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5470,20 +5064,14 @@
         <x:v>A principle can have limits, but if the exceptions swallow the rule, the apparent commitment becomes mostly decorative.</x:v>
       </x:c>
       <x:c r="N102" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Public commitments to transparency, merit, or local control often vanish once they threaten a favored outcome.</x:v>
       </x:c>
       <x:c r="O102" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="P102" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="Q102" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="R102" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
+        <x:v>Organizations sometimes advertise simple values statements that become practically meaningless once the long list of carve-outs is revealed.</x:v>
+      </x:c>
+      <x:c r="P102" t="str"/>
+      <x:c r="Q102" t="str"/>
+      <x:c r="R102" t="str"/>
       <x:c r="S102" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5522,17 +5110,13 @@
         <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="O103" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Campaign and media narratives often assume that working-class, rural, religious, or college-educated identities come with one full political bundle attached.</x:v>
       </x:c>
       <x:c r="P103" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="Q103" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="R103" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>People frequently expect hobbies, musical taste, fashion, or ethnicity to drag a whole associated worldview behind them even when the individual breaks the pattern.</x:v>
+      </x:c>
+      <x:c r="Q103" t="str"/>
+      <x:c r="R103" t="str"/>
       <x:c r="S103" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5572,20 +5156,14 @@
         <x:v>Personifying weather, markets, or algorithms can be a vivid metaphor, but it becomes fallacious when the metaphor is used as literal evidence.</x:v>
       </x:c>
       <x:c r="N104" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>People often say the algorithm hates them, loves outrage, or wants to silence them when the actual explanation is a mix of optimization rules and incentives.</x:v>
       </x:c>
       <x:c r="O104" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="P104" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
-      </x:c>
-      <x:c r="Q104" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
-      <x:c r="R104" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
+        <x:v>News coverage sometimes treats storms, markets, or viruses as if they were moral agents taking revenge, sending messages, or rewarding virtue.</x:v>
+      </x:c>
+      <x:c r="P104" t="str"/>
+      <x:c r="Q104" t="str"/>
+      <x:c r="R104" t="str"/>
       <x:c r="S104" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5623,20 +5201,14 @@
         <x:v>A partial improvement can still be worthwhile. The mistake is demanding perfection from one proposal when no realistic policy can eliminate the problem entirely.</x:v>
       </x:c>
       <x:c r="N105" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Climate and transit proposals are often rejected because they will not solve emissions or congestion completely, as if incomplete progress counted as no progress.</x:v>
       </x:c>
       <x:c r="O105" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="P105" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="Q105" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R105" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
+        <x:v>Arguments about AI safety, gun policy, and public health often dismiss guardrails for failing to eliminate every bad case, rather than asking whether they would reduce harm.</x:v>
+      </x:c>
+      <x:c r="P105" t="str"/>
+      <x:c r="Q105" t="str"/>
+      <x:c r="R105" t="str"/>
       <x:c r="S105" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5671,17 +5243,13 @@
         <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
       </x:c>
       <x:c r="O106" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>Debates about media bias, moral character, and institutional trust often assume that if a person or outlet is not perfectly objective, then it is simply propaganda.</x:v>
       </x:c>
       <x:c r="P106" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="Q106" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="R106" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
+        <x:v>Public discussion of peace, tolerance, and fairness often ignores large improvements because some imperfection remains somewhere.</x:v>
+      </x:c>
+      <x:c r="Q106" t="str"/>
+      <x:c r="R106" t="str"/>
       <x:c r="S106" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5723,20 +5291,14 @@
         <x:v>An analogy usually highlights one structural similarity, not a one-to-one mapping of every detail.</x:v>
       </x:c>
       <x:c r="N107" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>Infrastructure analogies about bridges, firewalls, or guardrails are often attacked by demanding that every literal feature transfer over exactly.</x:v>
       </x:c>
       <x:c r="O107" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="P107" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="Q107" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R107" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Debaters sometimes turn an opponent's limited comparison into a cartoon version so they can say the analogy obviously fails.</x:v>
+      </x:c>
+      <x:c r="P107" t="str"/>
+      <x:c r="Q107" t="str"/>
+      <x:c r="R107" t="str"/>
       <x:c r="S107" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5768,20 +5330,14 @@
         <x:v>A true or well-supported detail can increase trust only where the claims are genuinely linked. Often the extra conclusion is just hitching a ride on evidence that belongs to something narrower.</x:v>
       </x:c>
       <x:c r="N108" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>After the September 2024 ABC debate, the fact that the lecterns differed in height was treated by some users as if it supported much broader unverified claims about secret coordination and leaked questions.</x:v>
       </x:c>
       <x:c r="O108" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="P108" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="Q108" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R108" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>Conspiracy arguments often point to one authentic photo, real location, or correct minor fact and then use that narrow success to smuggle in much larger unsupported conclusions.</x:v>
+      </x:c>
+      <x:c r="P108" t="str"/>
+      <x:c r="Q108" t="str"/>
+      <x:c r="R108" t="str"/>
       <x:c r="S108" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5819,20 +5375,14 @@
         <x:v>Source criticism can be relevant, but poisoning the well tries to make the audience stop listening before the argument or evidence is even on the table.</x:v>
       </x:c>
       <x:c r="N109" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>In political and media fights, audiences are often primed to treat a judge, journalist, scientist, or witness as corrupt before that person's specific evidence is even heard.</x:v>
       </x:c>
       <x:c r="O109" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="P109" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="Q109" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="R109" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
+        <x:v>After the September 2024 Harris-Trump debate, repeated claims that moderators and outlets were inherently rigged encouraged supporters to dismiss later fact-checks in advance rather than assess them on the merits.</x:v>
+      </x:c>
+      <x:c r="P109" t="str"/>
+      <x:c r="Q109" t="str"/>
+      <x:c r="R109" t="str"/>
       <x:c r="S109" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5870,20 +5420,14 @@
         <x:v>Temporal order matters for causation, but it is only one ingredient. The improvement might be coincidence, regression to the mean, other background changes, or a different cause entirely.</x:v>
       </x:c>
       <x:c r="N110" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Wellness and self-optimization discourse in 2024 routinely credited cold plunges, supplements, or glucose hacks for improvements that followed several simultaneous lifestyle changes.</x:v>
       </x:c>
       <x:c r="O110" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
-      </x:c>
-      <x:c r="P110" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="Q110" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R110" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
+        <x:v>Politicians often claim that a policy worked because a good trend appeared soon after the policy was announced, even when the trend began earlier or other explanations remain stronger.</x:v>
+      </x:c>
+      <x:c r="P110" t="str"/>
+      <x:c r="Q110" t="str"/>
+      <x:c r="R110" t="str"/>
       <x:c r="S110" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5927,14 +5471,12 @@
         <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="P111" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>A single accurate prediction, one striking conversion story, or one dramatic crime clip is often treated as if it proved a broad thesis about markets, religion, or social decline.</x:v>
       </x:c>
       <x:c r="Q111" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R111" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>Debates about AI often jump from one impressive demo or one embarrassing failure to a total conclusion about the technology as a whole.</x:v>
+      </x:c>
+      <x:c r="R111" t="str"/>
       <x:c r="S111" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -5977,17 +5519,13 @@
         <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="O112" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Podcast debates, marathon livestreams, and mega-threads often bury the central claim beneath so many tangents that audiences mistake exhaustion for concession.</x:v>
       </x:c>
       <x:c r="P112" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="Q112" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="R112" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
+        <x:v>AI-generated text makes this tactic cheaper by allowing people to produce long, confident, fast-moving argument dumps that sound comprehensive while remaining poorly grounded.</x:v>
+      </x:c>
+      <x:c r="Q112" t="str"/>
+      <x:c r="R112" t="str"/>
       <x:c r="S112" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6023,20 +5561,14 @@
         <x:v>The missing piece is the base rate. Even a very accurate test can generate many false matches when the target condition is rare.</x:v>
       </x:c>
       <x:c r="N113" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Crime and security debates often overstate the force of DNA, face-recognition, or screening matches by ignoring how many non-matching people were also in the pool.</x:v>
       </x:c>
       <x:c r="O113" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
-      </x:c>
-      <x:c r="P113" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q113" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
-      </x:c>
-      <x:c r="R113" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
-      </x:c>
+        <x:v>A similar mistake appears whenever a diagnostic tool's false-positive rate is treated as if it directly gave the chance that any one flagged person is guilty, sick, or dangerous.</x:v>
+      </x:c>
+      <x:c r="P113" t="str"/>
+      <x:c r="Q113" t="str"/>
+      <x:c r="R113" t="str"/>
       <x:c r="S113" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6072,20 +5604,14 @@
         <x:v>Self-knowledge can be useful, but it is not a universal template. Other people may share some motives while differing sharply on others.</x:v>
       </x:c>
       <x:c r="N114" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>People often assume that because they would lie, panic, or seek status in a situation, anyone else in that situation must be driven by the same motive.</x:v>
       </x:c>
       <x:c r="O114" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
-      <x:c r="P114" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
-      <x:c r="Q114" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="R114" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
+        <x:v>Political and religious debate is full of claims about what opponents 'really know' or 'really fear' that reflect the speaker's own psychology more than the target's.</x:v>
+      </x:c>
+      <x:c r="P114" t="str"/>
+      <x:c r="Q114" t="str"/>
+      <x:c r="R114" t="str"/>
       <x:c r="S114" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6123,19 +5649,19 @@
         <x:v>Not every detour is fallacious; context can matter. The fallacy appears when the diversion substitutes for addressing the question that was actually on the table.</x:v>
       </x:c>
       <x:c r="N115" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="O115" t="str">
         <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="P115" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="Q115" t="str">
         <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="R115" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+        <x:v>In the June 27, 2024 Biden-Trump debate, answers about the economy, abortion, and January 6 often veered into immigration, personal fitness, or unrelated grievances instead of the question asked.</x:v>
       </x:c>
       <x:c r="S115" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -6168,20 +5694,14 @@
         <x:v>Evidence matters for empirical claims, but it cannot rescue a contradiction. If the concept itself does not make sense, more observations do not repair it.</x:v>
       </x:c>
       <x:c r="N116" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>Some arguments define a being, force, or property in mutually incompatible ways and then insist critics still need field evidence before calling the view incoherent.</x:v>
       </x:c>
       <x:c r="O116" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="P116" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q116" t="str">
-        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
-      </x:c>
-      <x:c r="R116" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>Online debate often treats every claim as if it deserved purely empirical testing, even when the real defect appears earlier at the level of definition or logical consistency.</x:v>
+      </x:c>
+      <x:c r="P116" t="str"/>
+      <x:c r="Q116" t="str"/>
+      <x:c r="R116" t="str"/>
       <x:c r="S116" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6219,20 +5739,14 @@
         <x:v>After unusually high or low outcomes, partial reversion toward the average is often expected even without special causal forces.</x:v>
       </x:c>
       <x:c r="N117" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>Sports commentators routinely over-credit halftime speeches or rituals for rebounds that would be unsurprising after an extreme first-half performance.</x:v>
       </x:c>
       <x:c r="O117" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="P117" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="Q117" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
-      </x:c>
-      <x:c r="R117" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Investors and managers often mistake a natural bounce after a terrible quarter for proof that a new slogan, consultant, or memo fixed the underlying problem.</x:v>
+      </x:c>
+      <x:c r="P117" t="str"/>
+      <x:c r="Q117" t="str"/>
+      <x:c r="R117" t="str"/>
       <x:c r="S117" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6274,20 +5788,14 @@
         <x:v>Metaphor can be useful shorthand, but the fallacy appears when agency, intention, or moral responsibility is attributed to an abstraction as though it literally possessed a mind of its own.</x:v>
       </x:c>
       <x:c r="N118" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>People talk as if capitalism, democracy, the algorithm, or history itself wants, fears, rewards, or punishes, which can hide the actual network of human choices and incentives underneath.</x:v>
       </x:c>
       <x:c r="O118" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="P118" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="Q118" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="R118" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
+        <x:v>AI discussions sometimes slide from 'the model produced this output' to 'the AI wants this outcome,' smuggling in a stronger picture of agency than the evidence supports.</x:v>
+      </x:c>
+      <x:c r="P118" t="str"/>
+      <x:c r="Q118" t="str"/>
+      <x:c r="R118" t="str"/>
       <x:c r="S118" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6327,20 +5835,14 @@
         <x:v>An outcome can make a story feel inevitable in retrospect without ever having been inevitable in advance. Hindsight strips away the branching paths that were live at the time.</x:v>
       </x:c>
       <x:c r="N119" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>After elections, market crashes, and celebrity scandals, commentators often speak as if the final result had been written into the evidence from the start rather than emerging from many uncertain factors.</x:v>
       </x:c>
       <x:c r="O119" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="P119" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
-      <x:c r="Q119" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R119" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
+        <x:v>This fallacy regularly follows close races and volatile technologies, where later narratives overstate how clear the winning path supposedly was.</x:v>
+      </x:c>
+      <x:c r="P119" t="str"/>
+      <x:c r="Q119" t="str"/>
+      <x:c r="R119" t="str"/>
       <x:c r="S119" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6374,20 +5876,14 @@
         <x:v>Many concepts such as belief, risk, identity, and influence work by degree. Treating them as all-or-nothing can falsify the speaker's actual position.</x:v>
       </x:c>
       <x:c r="N120" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Election, public-health, and AI debates often force nuanced confidence claims into binary boxes such as certain or uncertain, safe or unsafe, real or fake.</x:v>
       </x:c>
       <x:c r="O120" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="P120" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="Q120" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R120" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
+        <x:v>Arguments about what someone believes frequently replace a spectrum of confidence with a yes-or-no label that the original speaker never endorsed.</x:v>
+      </x:c>
+      <x:c r="P120" t="str"/>
+      <x:c r="Q120" t="str"/>
+      <x:c r="R120" t="str"/>
       <x:c r="S120" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6427,20 +5923,14 @@
         <x:v>Emotional attraction can explain why we want a conclusion, but not whether the conclusion is supported. A heartwarming possibility can still be false or impractical.</x:v>
       </x:c>
       <x:c r="N121" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>Fundraising pitches, miracle-cure stories, and uplifting viral posts often rely on the emotional payoff of the conclusion to make scrutiny feel mean or unnecessary.</x:v>
       </x:c>
       <x:c r="O121" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="P121" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
-      <x:c r="Q121" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="R121" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
+        <x:v>Public debate about policy sometimes slides from 'this would be compassionate' to 'therefore it must be workable and correct,' skipping the harder evidential and tradeoff questions.</x:v>
+      </x:c>
+      <x:c r="P121" t="str"/>
+      <x:c r="Q121" t="str"/>
+      <x:c r="R121" t="str"/>
       <x:c r="S121" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6480,20 +5970,18 @@
         <x:v>This is close to cherry picking, but the emphasis is on drawing the target around the bullet holes after the shots land. Post hoc pattern-hunting can make randomness, noise, or mixed data look like confirmation.</x:v>
       </x:c>
       <x:c r="N122" t="str">
+        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+      </x:c>
+      <x:c r="O122" t="str">
         <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
-      <x:c r="O122" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
       <x:c r="P122" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>Economic and election commentary often selects the time window, county, or subgroup that flatters the preferred narrative after the fact, then presents that slice as the decisive measure.</x:v>
       </x:c>
       <x:c r="Q122" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="R122" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
+        <x:v>AI benchmarking and startup marketing sometimes advertise the few tasks where a model shines while leaving out the wider distribution of tasks where the results are weaker or unstable.</x:v>
+      </x:c>
+      <x:c r="R122" t="str"/>
       <x:c r="S122" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6533,19 +6021,19 @@
         <x:v>Some causes are more important than others, and sometimes one factor really is dominant. The fallacy appears when a multi-causal phenomenon is flattened into a one-variable story without enough evidence.</x:v>
       </x:c>
       <x:c r="N123" t="str">
+        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+      </x:c>
+      <x:c r="O123" t="str">
         <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
-      </x:c>
-      <x:c r="O123" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="P123" t="str">
         <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="Q123" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Arguments about inflation, crime, housing costs, and educational decline often blame one villain such as immigrants, regulation, presidents, or social media, even when the outcome reflects multiple interacting causes.</x:v>
       </x:c>
       <x:c r="R123" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>After school shootings or viral episodes of unrest, public commentary regularly rushes to one master explanation instead of asking how incentives, access, institutions, culture, and personal history combine.</x:v>
       </x:c>
       <x:c r="S123" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -6586,19 +6074,19 @@
         <x:v>Some slopes are real, especially when incentives, precedent, or institutional weakness make escalation predictable. The fallacy appears when the chain is asserted rather than argued for.</x:v>
       </x:c>
       <x:c r="N124" t="str">
+        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+      </x:c>
+      <x:c r="O124" t="str">
         <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
-      <x:c r="O124" t="str">
+      <x:c r="P124" t="str">
         <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
-      <x:c r="P124" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
       <x:c r="Q124" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>In 2024 arguments over classroom AI, both enthusiasts and critics often predicted inevitable futures - either total educational collapse or total educational liberation - without showing why intermediate guardrails would fail.</x:v>
       </x:c>
       <x:c r="R124" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Election rhetoric about mail voting, early voting, or routine administrative changes often predicts the total breakdown of legitimacy from one policy shift without evidence for the full cascade.</x:v>
       </x:c>
       <x:c r="S124" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -6643,14 +6131,12 @@
         <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="P125" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Political actors often demand strict accountability, civility, or transparency for opponents while inventing excuses for why their own side should be judged differently.</x:v>
       </x:c>
       <x:c r="Q125" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="R125" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>Religious and ideological arguments often exempt cherished claims from the evidence standards applied to ordinary claims.</x:v>
+      </x:c>
+      <x:c r="R125" t="str"/>
       <x:c r="S125" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6688,20 +6174,14 @@
         <x:v>Attention is selective. Media, algorithms, and memory amplify the dramatic cases, not the ordinary distribution.</x:v>
       </x:c>
       <x:c r="N126" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+        <x:v>Crime clips, campus incidents, and viral protest footage often dominate public perception far beyond their representativeness, making whole groups look more extreme than they are.</x:v>
       </x:c>
       <x:c r="O126" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
-      </x:c>
-      <x:c r="P126" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="Q126" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
-      </x:c>
-      <x:c r="R126" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
+        <x:v>People watching political interviews can easily conclude that a population is loud, combative, or theatrical without noticing that quieter members of the same population rarely become visible.</x:v>
+      </x:c>
+      <x:c r="P126" t="str"/>
+      <x:c r="Q126" t="str"/>
+      <x:c r="R126" t="str"/>
       <x:c r="S126" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6737,20 +6217,14 @@
         <x:v>Sometimes the problem is deliberate obscurity; other times it is sincere confusion. Either way, complexity should not be mistaken for structure.</x:v>
       </x:c>
       <x:c r="N127" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>Conspiracy reasoning often spirals into self-sealing loops where every attempted refutation becomes fresh confirmation through an increasingly baroque chain of premises.</x:v>
       </x:c>
       <x:c r="O127" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
-      <x:c r="P127" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="Q127" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R127" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>AI-generated argument dumps can produce this effect by chaining plausible-sounding clauses that never quite add up to a valid line of reasoning.</x:v>
+      </x:c>
+      <x:c r="P127" t="str"/>
+      <x:c r="Q127" t="str"/>
+      <x:c r="R127" t="str"/>
       <x:c r="S127" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6791,17 +6265,13 @@
         <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="O128" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>During the September 10, 2024 Harris-Trump debate, claims about abortion rights were repeatedly recast into the far more extreme charge that Democrats support killing babies after birth, which is not the position being defended.</x:v>
       </x:c>
       <x:c r="P128" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="Q128" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="R128" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
+        <x:v>Debates over campus speech and content moderation often turn a narrower argument about rules, incentives, or disclosure into the cartoon claim that one side 'wants censorship' or 'wants total chaos.'</x:v>
+      </x:c>
+      <x:c r="Q128" t="str"/>
+      <x:c r="R128" t="str"/>
       <x:c r="S128" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6850,10 +6320,10 @@
         <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="Q129" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Coverage of the September 10, 2024 Harris-Trump debate often focused on who seemed stronger, calmer, or more in command, which matters politically but does not by itself settle whether the claims on stage were accurate.</x:v>
       </x:c>
       <x:c r="R129" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>Short-form video and podcast culture reward confidence, pace, and rhetorical dominance, making it easy for a slick performance to outperform a careful but less theatrical argument.</x:v>
       </x:c>
       <x:c r="S129" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -6892,20 +6362,14 @@
         <x:v>Correlative terms such as healthy and unhealthy, free and restricted, informed and uninformed, or biased and impartial depend on contrasts that can be weakened without disappearing.</x:v>
       </x:c>
       <x:c r="N130" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Critics sometimes argue that because everyone has some bias, calling a report biased says nothing, as if degrees of distortion and unfairness were impossible.</x:v>
       </x:c>
       <x:c r="O130" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="P130" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
-      <x:c r="Q130" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R130" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
+        <x:v>Debates about freedom and censorship often set the positive term to an impossible ideal so that ordinary, useful distinctions collapse.</x:v>
+      </x:c>
+      <x:c r="P130" t="str"/>
+      <x:c r="Q130" t="str"/>
+      <x:c r="R130" t="str"/>
       <x:c r="S130" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -6946,17 +6410,13 @@
         <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
       <x:c r="O131" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Startup and creator advice often highlights spectacular winners while the much larger number of people who copied the same strategy and failed remain largely invisible.</x:v>
       </x:c>
       <x:c r="P131" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
-      </x:c>
-      <x:c r="Q131" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
-      </x:c>
-      <x:c r="R131" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
+        <x:v>Investment talk routinely showcases the funds, traders, and backtests that survived long enough to look impressive while the dead funds and broken strategies quietly disappear.</x:v>
+      </x:c>
+      <x:c r="Q131" t="str"/>
+      <x:c r="R131" t="str"/>
       <x:c r="S131" t="str">
         <x:v>added-2026-completeness-pass</x:v>
       </x:c>
@@ -6992,20 +6452,14 @@
         <x:v>Some things really are designed for purposes, but purpose should not be assumed where it has not been shown. Processes can produce outcomes without aiming at them.</x:v>
       </x:c>
       <x:c r="N132" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>People often speak as if history is automatically bending toward justice, collapse, nationalism, or liberation, as though social change carried its own guaranteed destination.</x:v>
       </x:c>
       <x:c r="O132" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="P132" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="Q132" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="R132" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
-      </x:c>
+        <x:v>In technology debates, AI progress is sometimes framed as if it were inherently marching toward a single destined endpoint such as AGI rather than following contingent technical and social paths.</x:v>
+      </x:c>
+      <x:c r="P132" t="str"/>
+      <x:c r="Q132" t="str"/>
+      <x:c r="R132" t="str"/>
       <x:c r="S132" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7043,20 +6497,14 @@
         <x:v>Aphorisms can be wise shortcuts, but they become fallacious when they replace the reasoning that the situation still requires.</x:v>
       </x:c>
       <x:c r="N133" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>Phrases such as 'Do your own research,' 'common sense,' or 'if you know, you know' are often used online not to open inquiry but to make further questions look unnecessary or naive.</x:v>
       </x:c>
       <x:c r="O133" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
-      </x:c>
-      <x:c r="P133" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="Q133" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="R133" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
+        <x:v>Political and religious arguments frequently end with slogans like 'Freedom is not free' or 'Only God knows,' which can be meaningful in some contexts but often function as conversation-stoppers.</x:v>
+      </x:c>
+      <x:c r="P133" t="str"/>
+      <x:c r="Q133" t="str"/>
+      <x:c r="R133" t="str"/>
       <x:c r="S133" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7092,20 +6540,14 @@
         <x:v>A vivid case can motivate investigation, but it does not by itself justify a population-level conclusion.</x:v>
       </x:c>
       <x:c r="N134" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Isolated crime stories are often turned into sweeping claims about immigrants, professions, age groups, or political movements.</x:v>
       </x:c>
       <x:c r="O134" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="P134" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="Q134" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="R134" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>A single corporate scandal can quickly become a claim that the entire industry is rotten in exactly the same way.</x:v>
+      </x:c>
+      <x:c r="P134" t="str"/>
+      <x:c r="Q134" t="str"/>
+      <x:c r="R134" t="str"/>
       <x:c r="S134" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7149,20 +6591,14 @@
         <x:v>Generalizations are often default-pattern claims, not exceptionless universal laws.</x:v>
       </x:c>
       <x:c r="N135" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Public-health advice is often dismissed by pointing to unusual edge cases even when the advice was clearly aimed at ordinary conditions.</x:v>
       </x:c>
       <x:c r="O135" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="P135" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="Q135" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R135" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
-      </x:c>
+        <x:v>Safety rules and economic patterns are frequently challenged by exceptions that do not actually undermine the broader tendency being described.</x:v>
+      </x:c>
+      <x:c r="P135" t="str"/>
+      <x:c r="Q135" t="str"/>
+      <x:c r="R135" t="str"/>
       <x:c r="S135" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7198,20 +6634,14 @@
         <x:v>A favorable anecdote can remind us not to overgeneralize negatively, but it cannot prove that the larger class is generally positive.</x:v>
       </x:c>
       <x:c r="N136" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>One transparent politician or one ethical corporation is often used to imply that the surrounding system is healthier than the broader evidence suggests.</x:v>
       </x:c>
       <x:c r="O136" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="P136" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
-      </x:c>
-      <x:c r="Q136" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
-      <x:c r="R136" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
+        <x:v>People frequently infer that an institution is trustworthy because they personally encountered one helpful employee inside it.</x:v>
+      </x:c>
+      <x:c r="P136" t="str"/>
+      <x:c r="Q136" t="str"/>
+      <x:c r="R136" t="str"/>
       <x:c r="S136" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7243,20 +6673,14 @@
         <x:v>A track record does not make contrary outcomes impossible, but it does affect rational priors. Ignoring repeated past failure forces every new case to borrow more credibility than it has earned.</x:v>
       </x:c>
       <x:c r="N137" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Baseless claims about widespread noncitizen voting keep getting relaunched as if decades of rarity, audits, and failed alarms provide no reason for initial skepticism.</x:v>
       </x:c>
       <x:c r="O137" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
-      </x:c>
-      <x:c r="P137" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
-      </x:c>
-      <x:c r="Q137" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
-      <x:c r="R137" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
+        <x:v>Every new blurry UFO clip, miracle cure, or ghost story is often pitched as if the long record of ordinary explanations should have zero effect on our starting expectations.</x:v>
+      </x:c>
+      <x:c r="P137" t="str"/>
+      <x:c r="Q137" t="str"/>
+      <x:c r="R137" t="str"/>
       <x:c r="S137" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7301,17 +6725,13 @@
         <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="O138" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>In the June 27, 2024 Biden-Trump debate and the September 10, 2024 Harris-Trump debate, many charges were met with 'your side did it too' responses that redirected blame without addressing the original allegation.</x:v>
       </x:c>
       <x:c r="P138" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
-      </x:c>
-      <x:c r="Q138" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R138" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
+        <x:v>Arguments about misinformation, climate, religion, and media bias often slide into scorekeeping about who is worse rather than whether the specific criticized claim is true or justified.</x:v>
+      </x:c>
+      <x:c r="Q138" t="str"/>
+      <x:c r="R138" t="str"/>
       <x:c r="S138" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7351,20 +6771,14 @@
         <x:v>Exposing hypocrisy can matter, but retaliation does not erase the original wrong or magically sanitize a copy of it.</x:v>
       </x:c>
       <x:c r="N139" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>In 2024 election discourse, misinformation was often excused with the claim that the other side lies too, as if symmetry or revenge transformed falsehood into fairness.</x:v>
       </x:c>
       <x:c r="O139" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
-      </x:c>
-      <x:c r="P139" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="Q139" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
-      <x:c r="R139" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
+        <x:v>Debates about censorship, doxxing, and dirty campaign tactics often slide from condemnation into imitation, with each side treating the other's bad behavior as a license to do the same.</x:v>
+      </x:c>
+      <x:c r="P139" t="str"/>
+      <x:c r="Q139" t="str"/>
+      <x:c r="R139" t="str"/>
       <x:c r="S139" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7403,17 +6817,13 @@
         <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="O140" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>Lifestyle and identity marketing often says 'the cool do X' and 'I do X,' then slides to 'therefore I am one of the cool,' even though the shared feature is too broad.</x:v>
       </x:c>
       <x:c r="P140" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q140" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
-      </x:c>
-      <x:c r="R140" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Political commentary frequently infers that because two camps are skeptical of the same institution or support the same policy, they must belong to the same underlying movement.</x:v>
+      </x:c>
+      <x:c r="Q140" t="str"/>
+      <x:c r="R140" t="str"/>
       <x:c r="S140" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7445,20 +6855,14 @@
         <x:v>Vagueness can be useful early in exploration, but it becomes fallacious when the fog is preserved to prevent serious evaluation. If key terms cannot be pinned down, the claim can keep slipping away from critique.</x:v>
       </x:c>
       <x:c r="N141" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>Alternative-health and wellness marketing often leans on words like 'toxins,' 'energy,' 'balance,' and 'boost' precisely because they sound scientific while remaining hard to falsify.</x:v>
       </x:c>
       <x:c r="O141" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
-      </x:c>
-      <x:c r="P141" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
-      </x:c>
-      <x:c r="Q141" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
-      </x:c>
-      <x:c r="R141" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
-      </x:c>
+        <x:v>In arguments about spirituality, self-help, and even AI, flexible phrases can be stretched to fit almost any outcome, which makes the view feel resilient without making it well supported.</x:v>
+      </x:c>
+      <x:c r="P141" t="str"/>
+      <x:c r="Q141" t="str"/>
+      <x:c r="R141" t="str"/>
       <x:c r="S141" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7502,19 +6906,19 @@
         <x:v>Hope can sustain action, but it does not convert possibility into evidence. The stronger the desire, the easier it is to mistake wanting for warrant.</x:v>
       </x:c>
       <x:c r="N142" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="O142" t="str">
         <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="P142" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="Q142" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Speculative markets, miracle-cure promises, and election-night narratives often run on the thought that a hoped-for outcome is somehow more likely because people badly want it.</x:v>
       </x:c>
       <x:c r="R142" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+        <x:v>Beliefs about the afterlife, destiny, or technological salvation are often defended by saying life would feel bleak without them, which speaks to desire rather than truth.</x:v>
       </x:c>
       <x:c r="S142" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -7549,20 +6953,14 @@
         <x:v>Real corroboration requires accessible, independent testimony or records. Simply claiming that more witnesses exist adds almost nothing if the chain cannot be examined.</x:v>
       </x:c>
       <x:c r="N143" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>Paranormal, religious, and conspiracy stories often swell in authority by invoking unnamed doctors, secret insiders, or hundreds of silent observers who never become independently available.</x:v>
       </x:c>
       <x:c r="O143" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
-      </x:c>
-      <x:c r="P143" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
-      </x:c>
-      <x:c r="Q143" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
-      </x:c>
-      <x:c r="R143" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
-      </x:c>
+        <x:v>Historical arguments sometimes treat a late report that 'many people saw it' as if that were the same thing as actually having many separate testimonies.</x:v>
+      </x:c>
+      <x:c r="P143" t="str"/>
+      <x:c r="Q143" t="str"/>
+      <x:c r="R143" t="str"/>
       <x:c r="S143" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>
@@ -7604,14 +7002,12 @@
         <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="P144" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+        <x:v>Arguments about social media and teen mental health often assume a one-way causal story even though distress can also increase the tendency to seek certain kinds of online engagement.</x:v>
       </x:c>
       <x:c r="Q144" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
-      </x:c>
-      <x:c r="R144" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
-      </x:c>
+        <x:v>Crime, policing, and economic debates frequently treat a response variable as if it were the cause, such as assuming security purchases create fear rather than fear driving security purchases.</x:v>
+      </x:c>
+      <x:c r="R144" t="str"/>
       <x:c r="S144" t="str">
         <x:v>modernized-2026-pass</x:v>
       </x:c>

</xml_diff>

<commit_message>
Add Phil Stilwell copyright to site and workbook
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1b368b82c05244fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R2713cfdf029a432c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R58bef55075f0490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra047f5b1f04045b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R6efea382043d438d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R2f935fbe77064198"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -240,6 +240,14 @@
         <x:v>Use the Fallacies sheet for entry-by-entry editing and the Categories sheet for counts.</x:v>
       </x:c>
     </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Copyright</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Copyright © Phil Stilwell</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Clarify rationality lab navigation and wording
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R5d7706e700d14d26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rbb5d6d762dc04f29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R050135aeb15a45ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbb5df2cd152b4f8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R12c41fadf3fd4f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R7c531a57e07c4623"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -326,25 +326,25 @@
         <x:v>Notes</x:v>
       </x:c>
       <x:c r="N1" s="1" t="str">
-        <x:v>Rationality Danger</x:v>
+        <x:v>Why This Mistake Matters</x:v>
       </x:c>
       <x:c r="O1" s="1" t="str">
-        <x:v>Dynamics to Notice</x:v>
+        <x:v>What to Watch For</x:v>
       </x:c>
       <x:c r="P1" s="1" t="str">
         <x:v>Warning Signs</x:v>
       </x:c>
       <x:c r="Q1" s="1" t="str">
-        <x:v>Interactive Mechanic</x:v>
+        <x:v>Suggested Tool</x:v>
       </x:c>
       <x:c r="R1" s="1" t="str">
-        <x:v>User Action</x:v>
+        <x:v>What the Reader Does</x:v>
       </x:c>
       <x:c r="S1" s="1" t="str">
-        <x:v>Feedback Logic</x:v>
+        <x:v>What the Tool Shows</x:v>
       </x:c>
       <x:c r="T1" s="1" t="str">
-        <x:v>Repair Prompts</x:v>
+        <x:v>How to Fix It</x:v>
       </x:c>
       <x:c r="U1" s="1" t="str">
         <x:v>Case Study 1</x:v>
@@ -10081,19 +10081,19 @@
         <x:v>Description</x:v>
       </x:c>
       <x:c r="D1" s="1" t="str">
-        <x:v>Primary Distortion</x:v>
+        <x:v>Main Reasoning Problem</x:v>
       </x:c>
       <x:c r="E1" s="1" t="str">
-        <x:v>Category Danger</x:v>
+        <x:v>Why This Kind Matters</x:v>
       </x:c>
       <x:c r="F1" s="1" t="str">
-        <x:v>Default Mechanic</x:v>
+        <x:v>Suggested Tool</x:v>
       </x:c>
       <x:c r="G1" s="1" t="str">
-        <x:v>User Action</x:v>
+        <x:v>What the Reader Does</x:v>
       </x:c>
       <x:c r="H1" s="1" t="str">
-        <x:v>Feedback</x:v>
+        <x:v>What the Tool Shows</x:v>
       </x:c>
     </x:row>
     <x:row r="2">

</xml_diff>

<commit_message>
Add illustrated companion posters across fallacy pages
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R80720494719d41a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R7a71eb9e24bb414d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R20bd8f846e954a2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc67b5d51a7754107"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R2013e3b73bc04a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Ra13cde2842024a5b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -196,8 +196,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="75.45999908447266" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28.940000534057617" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="82.7699966430664" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -257,33 +257,33 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="31.290000915527344" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="26.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="21.469999313354492" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21.469999313354492" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="21.469999313354492" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="21.469999313354492" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="21.469999313354492" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="21.469999313354492" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="28.829999923706055" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="27" max="27" width="21.469999313354492" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34.31999969482422" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28.940000534057617" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15.479999542236328" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="31.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="23.549999237060547" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -10491,14 +10491,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="21.469999313354492" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="11.65999984741211" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="43.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="43.560001373291016" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.789999961853027" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="47.779998779296875" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">

</xml_diff>

<commit_message>
Add image explanations to fallacy posters
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc67b5d51a7754107"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R2013e3b73bc04a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Ra13cde2842024a5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc2fc703c945341d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R039e7e3df44a4483"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rbc95dbb6c6874f6a"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Replace generic slider with fallacy walkthrough tool
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc2fc703c945341d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R039e7e3df44a4483"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rbc95dbb6c6874f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf8eefd33fcb347ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R0ab3e1b9961c4ccf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R055370bbded5437f"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Align tool guidance with walkthrough stages
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf8eefd33fcb347ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="R0ab3e1b9961c4ccf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R055370bbded5437f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb912caf07dba4c91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Ra77dd235adef4897"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rae19180d76da4520"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Expand case studies and surface citations
</commit_message>
<xml_diff>
--- a/logfall-root-edition.xlsx
+++ b/logfall-root-edition.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb912caf07dba4c91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Ra77dd235adef4897"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="Rae19180d76da4520"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R386acba1aa6b47a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallacies" sheetId="2" r:id="Rd9451e9a55604a5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R99c4336c38ae4440"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -420,10 +420,10 @@
         <x:v>Sometimes absence of evidence really is weak evidence, especially when the search tools are poor or the target is hard to detect. But when repeated investigation under the right conditions turns up nothing, that absence is itself evidence.</x:v>
       </x:c>
       <x:c r="V2" t="str">
-        <x:v>After officials in Springfield, Ohio said there were no credible reports supporting the September 2024 rumor that Haitian immigrants were abducting and eating pets, some defenders treated the lack of evidence as irrelevant or as proof of a cover-up rather than as evidence against the rumor.</x:v>
+        <x:v>After officials in Springfield, Ohio said there were no credible reports supporting the September 2024 rumor that Haitian immigrants were abducting and eating pets, some defenders treated the lack of evidence as irrelevant or as proof of a cover-up rather than as evidence against the rumor. The fallacy here is Absence of evidence fallacy: someone treats a failure to find expected evidence as if it counted for nothing against the claim, even in a context where the claim should leave detectable traces. That matters here because sometimes absence of evidence really is weak evidence, especially when the search tools are poor or the target is hard to detect. A better analysis would remember that when repeated investigation under the right conditions turns up nothing, that absence is itself evidence.</x:v>
       </x:c>
       <x:c r="W2" t="str">
-        <x:v>Claims of widespread noncitizen voting in 2024 often survived repeated audits and official reviews by insisting that the absence of supporting evidence was exactly what one should expect from a hidden scheme.</x:v>
+        <x:v>Claims of widespread noncitizen voting in 2024 often survived repeated audits and official reviews by insisting that the absence of supporting evidence was exactly what one should expect from a hidden scheme. The fallacy here is Absence of evidence fallacy: someone treats a failure to find expected evidence as if it counted for nothing against the claim, even in a context where the claim should leave detectable traces. That matters here because sometimes absence of evidence really is weak evidence, especially when the search tools are poor or the target is hard to detect. A better analysis would remember that when repeated investigation under the right conditions turns up nothing, that absence is itself evidence.</x:v>
       </x:c>
       <x:c r="X2" t="str"/>
       <x:c r="Y2" t="str"/>
@@ -483,10 +483,10 @@
         <x:v>Abstract patterns can still be real and explanatory even when they depend on smaller physical or social components. Economies, institutions, languages, and ecosystems do not stop being real because they are made of people, words, or organisms.</x:v>
       </x:c>
       <x:c r="V3" t="str">
-        <x:v>People sometimes say 'science does not discover anything, only scientists do,' as if that erased the reality of science as a method and institution with stable norms and effects.</x:v>
+        <x:v>People sometimes say 'science does not discover anything, only scientists do,' as if that erased the reality of science as a method and institution with stable norms and effects. The fallacy here is Abstraction denial: someone denies the reality or causal relevance of a higher-level pattern just because the pattern is realized through lower-level parts. That matters here because abstract patterns can still be real and explanatory even when they depend on smaller physical or social components. A better analysis would remember that economies, institutions, languages, and ecosystems do not stop being real because they are made of people, words, or organisms.</x:v>
       </x:c>
       <x:c r="W3" t="str">
-        <x:v>Debates about algorithms, markets, and social platforms often pretend there is no system-level behavior because only users or lines of code act at the micro level.</x:v>
+        <x:v>Debates about algorithms, markets, and social platforms often pretend there is no system-level behavior because only users or lines of code act at the micro level. The fallacy here is Abstraction denial: someone denies the reality or causal relevance of a higher-level pattern just because the pattern is realized through lower-level parts. That matters here because abstract patterns can still be real and explanatory even when they depend on smaller physical or social components. A better analysis would remember that economies, institutions, languages, and ecosystems do not stop being real because they are made of people, words, or organisms.</x:v>
       </x:c>
       <x:c r="X3" t="str"/>
       <x:c r="Y3" t="str"/>
@@ -546,10 +546,10 @@
         <x:v>Useful abstractions describe patterns with varying scope and durability. They are not automatically eternal, exceptionless constraints on what can happen.</x:v>
       </x:c>
       <x:c r="V4" t="str">
-        <x:v>People often treat economic or technological 'laws' as if they guaranteed the future rather than summarizing a contingent historical pattern that may bend, pause, or fail.</x:v>
+        <x:v>People often treat economic or technological 'laws' as if they guaranteed the future rather than summarizing a contingent historical pattern that may bend, pause, or fail. The fallacy here is Abstraction fallacy: a model, law, or abstraction drawn from experience is treated as if it were a logically necessary rule that reality cannot ever depart from. That matters here because useful abstractions describe patterns with varying scope and durability. A better analysis would remember that they are not automatically eternal, exceptionless constraints on what can happen.</x:v>
       </x:c>
       <x:c r="W4" t="str">
-        <x:v>In AI discourse, scaling trends are sometimes talked about as destiny, as though past curves logically force a particular future rather than merely suggesting one.</x:v>
+        <x:v>In AI discourse, scaling trends are sometimes talked about as destiny, as though past curves logically force a particular future rather than merely suggesting one. The fallacy here is Abstraction fallacy: a model, law, or abstraction drawn from experience is treated as if it were a logically necessary rule that reality cannot ever depart from. That matters here because useful abstractions describe patterns with varying scope and durability. A better analysis would remember that they are not automatically eternal, exceptionless constraints on what can happen.</x:v>
       </x:c>
       <x:c r="X4" t="str"/>
       <x:c r="Y4" t="str"/>
@@ -617,19 +617,28 @@
         <x:v>Character can matter when credibility itself is at issue, such as fraud, conflicts of interest, or proven dishonesty. The fallacy appears when those personal facts are used instead of answering the actual reasons or evidence.</x:v>
       </x:c>
       <x:c r="V5" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>AI experimentation is high risk, high reward for low-profile political campaigns
+AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. The fallacy here is Ad hominem: someone treats an attack on a person's character, motives, class, or biography as if it were a refutation of that person's argument. That matters here because character can matter when credibility itself is at issue, such as fraud, conflicts of interest, or proven dishonesty. That is the exact slip in this case: those personal facts are used instead of answering the actual reasons or evidence.
+Source: Associated Press | 2024-06-17
+https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="W5" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+        <x:v>Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement
+AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. The fallacy here is Ad hominem: someone treats an attack on a person's character, motives, class, or biography as if it were a refutation of that person's argument. That matters here because character can matter when credibility itself is at issue, such as fraud, conflicts of interest, or proven dishonesty. That is the exact slip in this case: those personal facts are used instead of answering the actual reasons or evidence.
+Source: Associated Press | 2024-09-10
+https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="X5" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate
+AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. The fallacy here is Ad hominem: someone treats an attack on a person's character, motives, class, or biography as if it were a refutation of that person's argument. That matters here because character can matter when credibility itself is at issue, such as fraud, conflicts of interest, or proven dishonesty. That is the exact slip in this case: those personal facts are used instead of answering the actual reasons or evidence.
+Source: Associated Press | 2024-06-27
+https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="Y5" t="str">
-        <x:v>In the June 27, 2024 Biden-Trump debate, policy exchanges repeatedly slid into attacks on each candidate's age, criminal exposure, or family rather than sustained engagement with the argument on the table.</x:v>
+        <x:v>In the June 27, 2024 Biden-Trump debate, policy exchanges repeatedly slid into attacks on each candidate's age, criminal exposure, or family rather than sustained engagement with the argument on the table. The fallacy here is Ad hominem: someone treats an attack on a person's character, motives, class, or biography as if it were a refutation of that person's argument. That matters here because character can matter when credibility itself is at issue, such as fraud, conflicts of interest, or proven dishonesty. That is the exact slip in this case: those personal facts are used instead of answering the actual reasons or evidence.</x:v>
       </x:c>
       <x:c r="Z5" t="str">
-        <x:v>Online discussion of climate, vaccines, and AI policy often substitutes labels such as 'shill,' 'grifter,' or 'elitist' for any serious response to the evidence.</x:v>
+        <x:v>Online discussion of climate, vaccines, and AI policy often substitutes labels such as 'shill,' 'grifter,' or 'elitist' for any serious response to the evidence. The fallacy here is Ad hominem: someone treats an attack on a person's character, motives, class, or biography as if it were a refutation of that person's argument. That matters here because character can matter when credibility itself is at issue, such as fraud, conflicts of interest, or proven dishonesty. That is the exact slip in this case: those personal facts are used instead of answering the actual reasons or evidence.</x:v>
       </x:c>
       <x:c r="AA5" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -690,10 +699,10 @@
         <x:v>Ruling something out does not automatically place it into the positive category you want. 'Not bad' does not by itself mean 'good,' and 'not that' does not by itself mean 'this.'</x:v>
       </x:c>
       <x:c r="V6" t="str">
-        <x:v>Tribal arguments often move from 'we are not them' and 'they are bad' to 'therefore we are trustworthy,' even though the conclusion has not been earned.</x:v>
+        <x:v>Tribal arguments often move from 'we are not them' and 'they are bad' to 'therefore we are trustworthy,' even though the conclusion has not been earned. The fallacy here is Affirmative conclusion from a negative premise: a syllogism tries to draw a positive conclusion even though one of the premises is negative in a way that cannot support that conclusion. That matters here because ruling something out does not automatically place it into the positive category you want. A better analysis would remember that 'Not bad' does not by itself mean 'good,' and 'not that' does not by itself mean 'this.'</x:v>
       </x:c>
       <x:c r="W6" t="str">
-        <x:v>Media and politics frequently treat the failure of one rival source as if it directly validated a different source that still needs its own support.</x:v>
+        <x:v>Media and politics frequently treat the failure of one rival source as if it directly validated a different source that still needs its own support. The fallacy here is Affirmative conclusion from a negative premise: a syllogism tries to draw a positive conclusion even though one of the premises is negative in a way that cannot support that conclusion. That matters here because ruling something out does not automatically place it into the positive category you want. A better analysis would remember that 'Not bad' does not by itself mean 'good,' and 'not that' does not by itself mean 'this.'</x:v>
       </x:c>
       <x:c r="X6" t="str"/>
       <x:c r="Y6" t="str"/>
@@ -759,16 +768,22 @@
         <x:v>Some disjunctions are genuinely exclusive, but many are not. Two options can coexist unless the statement or context really rules that out.</x:v>
       </x:c>
       <x:c r="V7" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not
+AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. The fallacy here is Affirming a disjunct: someone treats an ordinary 'or' as if it were exclusive and concludes that one option must be false because the other is true. That matters here because some disjunctions are genuinely exclusive, but many are not. A better analysis would remember that two options can coexist unless the statement or context really rules that out.
+Source: NPR | 2024-10-12
+https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="W7" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. The fallacy here is Affirming a disjunct: someone treats an ordinary 'or' as if it were exclusive and concludes that one option must be false because the other is true. That matters here because some disjunctions are genuinely exclusive, but many are not. A better analysis would remember that two options can coexist unless the statement or context really rules that out.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="X7" t="str">
-        <x:v>Budget rhetoric often suggests that because one policy tool is on the table, another cannot also matter, as if tradeoffs always come in only one-at-a-time form.</x:v>
+        <x:v>Budget rhetoric often suggests that because one policy tool is on the table, another cannot also matter, as if tradeoffs always come in only one-at-a-time form. The fallacy here is Affirming a disjunct: someone treats an ordinary 'or' as if it were exclusive and concludes that one option must be false because the other is true. That matters here because some disjunctions are genuinely exclusive, but many are not. A better analysis would remember that two options can coexist unless the statement or context really rules that out.</x:v>
       </x:c>
       <x:c r="Y7" t="str">
-        <x:v>Public debate regularly acts as though a claim must be either emotional or strategic, either true or persuasive, either mistaken or manipulative, when in reality both descriptions may apply.</x:v>
+        <x:v>Public debate regularly acts as though a claim must be either emotional or strategic, either true or persuasive, either mistaken or manipulative, when in reality both descriptions may apply. The fallacy here is Affirming a disjunct: someone treats an ordinary 'or' as if it were exclusive and concludes that one option must be false because the other is true. That matters here because some disjunctions are genuinely exclusive, but many are not. A better analysis would remember that two options can coexist unless the statement or context really rules that out.</x:v>
       </x:c>
       <x:c r="Z7" t="str"/>
       <x:c r="AA7" t="str">
@@ -832,19 +847,28 @@
         <x:v>A consequence can have many causes. Observing the result does not tell you which sufficient condition produced it.</x:v>
       </x:c>
       <x:c r="V8" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>AI experimentation is high risk, high reward for low-profile political campaigns
+AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. The fallacy here is Affirming the consequent: someone reasons from 'if A, then B' and then wrongly infers A merely because B is observed. That matters here because a consequence can have many causes. A better analysis would remember that observing the result does not tell you which sufficient condition produced it.
+Source: Associated Press | 2024-06-17
+https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="W8" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. The fallacy here is Affirming the consequent: someone reasons from 'if A, then B' and then wrongly infers A merely because B is observed. That matters here because a consequence can have many causes. A better analysis would remember that observing the result does not tell you which sufficient condition produced it.
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="X8" t="str">
-        <x:v>Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Pentagon study finds no sign of alien life in reported UFO sightings going back decades
+Across AP's UFO coverage in 2024, a recurring public inference was that whatever remains unexplained after initial review must therefore point to aliens or a cover-up. That is a vivid real-world case of treating open explanatory space as if it settled the conclusion. The fallacy here is Affirming the consequent: someone reasons from 'if A, then B' and then wrongly infers A merely because B is observed. That matters here because a consequence can have many causes. A better analysis would remember that observing the result does not tell you which sufficient condition produced it.
+Source: Associated Press | 2024-03-08
+https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="Y8" t="str">
-        <x:v>Political misinformation often treats one suspicious-looking detail as proof of a favored cause, even though many other explanations remain live.</x:v>
+        <x:v>Political misinformation often treats one suspicious-looking detail as proof of a favored cause, even though many other explanations remain live. The fallacy here is Affirming the consequent: someone reasons from 'if A, then B' and then wrongly infers A merely because B is observed. That matters here because a consequence can have many causes. A better analysis would remember that observing the result does not tell you which sufficient condition produced it.</x:v>
       </x:c>
       <x:c r="Z8" t="str">
-        <x:v>Arguments about fraud, manipulation, and AI generation frequently jump from a telltale symptom to a confident diagnosis without ruling out alternatives.</x:v>
+        <x:v>Arguments about fraud, manipulation, and AI generation frequently jump from a telltale symptom to a confident diagnosis without ruling out alternatives. The fallacy here is Affirming the consequent: someone reasons from 'if A, then B' and then wrongly infers A merely because B is observed. That matters here because a consequence can have many causes. A better analysis would remember that observing the result does not tell you which sufficient condition produced it.</x:v>
       </x:c>
       <x:c r="AA8" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -903,10 +927,10 @@
         <x:v>Many systems of belief, institutions, and documents are mixed. Partial support or partial failure rarely justifies an everything-or-nothing verdict.</x:v>
       </x:c>
       <x:c r="V9" t="str">
-        <x:v>In 2024 media battles, a single correction or mistaken detail was often used to dismiss an outlet's entire reporting on elections, immigration, or public health.</x:v>
+        <x:v>In 2024 media battles, a single correction or mistaken detail was often used to dismiss an outlet's entire reporting on elections, immigration, or public health. The fallacy here is All or nothing fallacy: support for part of a view, or problems with part of a view, are treated as if they force total acceptance or total rejection of the whole package. That matters here because many systems of belief, institutions, and documents are mixed. A better analysis would remember that partial support or partial failure rarely justifies an everything-or-nothing verdict.</x:v>
       </x:c>
       <x:c r="W9" t="str">
-        <x:v>Religious, ideological, and policy debates often act as though rejecting one doctrine, statistic, or mechanism commits you to rejecting the entire worldview.</x:v>
+        <x:v>Religious, ideological, and policy debates often act as though rejecting one doctrine, statistic, or mechanism commits you to rejecting the entire worldview. The fallacy here is All or nothing fallacy: support for part of a view, or problems with part of a view, are treated as if they force total acceptance or total rejection of the whole package. That matters here because many systems of belief, institutions, and documents are mixed. A better analysis would remember that partial support or partial failure rarely justifies an everything-or-nothing verdict.</x:v>
       </x:c>
       <x:c r="X9" t="str"/>
       <x:c r="Y9" t="str"/>
@@ -972,19 +996,28 @@
         <x:v>Anecdotes can be useful for illustration, hypothesis generation, or showing that something can happen. The fallacy appears when one memorable case is used to outweigh stronger evidence about what usually happens or what the larger data set shows.</x:v>
       </x:c>
       <x:c r="V10" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not
+NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. The fallacy here is Anecdotal fallacy: a vivid personal story, testimonial, or isolated case is treated as stronger evidence than broader, better, or more representative evidence. That matters here because anecdotes can be useful for illustration, hypothesis generation, or showing that something can happen. That is the exact slip in this case: one memorable case is used to outweigh stronger evidence about what usually happens or what the larger data set shows.
+Source: NPR | 2024-10-12
+https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="W10" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens
+AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. The fallacy here is Anecdotal fallacy: a vivid personal story, testimonial, or isolated case is treated as stronger evidence than broader, better, or more representative evidence. That matters here because anecdotes can be useful for illustration, hypothesis generation, or showing that something can happen. That is the exact slip in this case: one memorable case is used to outweigh stronger evidence about what usually happens or what the larger data set shows.
+Source: Associated Press | 2024-11-14
+https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="X10" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town
+PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. The fallacy here is Anecdotal fallacy: a vivid personal story, testimonial, or isolated case is treated as stronger evidence than broader, better, or more representative evidence. That matters here because anecdotes can be useful for illustration, hypothesis generation, or showing that something can happen. That is the exact slip in this case: one memorable case is used to outweigh stronger evidence about what usually happens or what the larger data set shows.
+Source: PolitiFact | 2024-09-09
+https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
       </x:c>
       <x:c r="Y10" t="str">
-        <x:v>Arguments about vaccines, supplements, and raw milk often lean on a neighbor's success story or a family anecdote as if that settled what the best studies show.</x:v>
+        <x:v>Arguments about vaccines, supplements, and raw milk often lean on a neighbor's success story or a family anecdote as if that settled what the best studies show. The fallacy here is Anecdotal fallacy: a vivid personal story, testimonial, or isolated case is treated as stronger evidence than broader, better, or more representative evidence. That matters here because anecdotes can be useful for illustration, hypothesis generation, or showing that something can happen. That is the exact slip in this case: one memorable case is used to outweigh stronger evidence about what usually happens or what the larger data set shows.</x:v>
       </x:c>
       <x:c r="Z10" t="str">
-        <x:v>Debates about AI productivity and remote work often treat one manager's striking success or failure story as if it established the general rule for everyone.</x:v>
+        <x:v>Debates about AI productivity and remote work often treat one manager's striking success or failure story as if it established the general rule for everyone. The fallacy here is Anecdotal fallacy: a vivid personal story, testimonial, or isolated case is treated as stronger evidence than broader, better, or more representative evidence. That matters here because anecdotes can be useful for illustration, hypothesis generation, or showing that something can happen. That is the exact slip in this case: one memorable case is used to outweigh stronger evidence about what usually happens or what the larger data set shows.</x:v>
       </x:c>
       <x:c r="AA10" t="str">
         <x:v>added-2026-completeness-pass</x:v>
@@ -1051,10 +1084,10 @@
         <x:v>Real accomplishment can justify attention, but it does not automatically transfer expertise across domains. The relevant question is still whether the claim is supported.</x:v>
       </x:c>
       <x:c r="V11" t="str">
-        <x:v>Celebrity founders, athletes, and actors often lend credibility to products and causes far outside their expertise, from supplements to financial schemes to political narratives.</x:v>
+        <x:v>Celebrity founders, athletes, and actors often lend credibility to products and causes far outside their expertise, from supplements to financial schemes to political narratives. The fallacy here is Appeal to accomplishment: a claim is treated as true or weighty mainly because the person promoting it has impressive accomplishments in some other domain. That matters here because real accomplishment can justify attention, but it does not automatically transfer expertise across domains. A better analysis would remember that the relevant question is still whether the claim is supported.</x:v>
       </x:c>
       <x:c r="W11" t="str">
-        <x:v>Public arguments about AI frequently treat the prestige of well-known founders as if it settled disputes that still require technical evidence, replication, and broader expert scrutiny.</x:v>
+        <x:v>Public arguments about AI frequently treat the prestige of well-known founders as if it settled disputes that still require technical evidence, replication, and broader expert scrutiny. The fallacy here is Appeal to accomplishment: a claim is treated as true or weighty mainly because the person promoting it has impressive accomplishments in some other domain. That matters here because real accomplishment can justify attention, but it does not automatically transfer expertise across domains. A better analysis would remember that the relevant question is still whether the claim is supported.</x:v>
       </x:c>
       <x:c r="X11" t="str"/>
       <x:c r="Y11" t="str"/>
@@ -1124,19 +1157,28 @@
         <x:v>Expert testimony can be good evidence when the authority is relevant, the expertise is genuine, and the claim fits the expert consensus. The fallacy appears when prestige replaces argument.</x:v>
       </x:c>
       <x:c r="V12" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+        <x:v>Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist
+In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. The fallacy here is Appeal to authority: someone treats an authority's endorsement as if it settled the issue, even when the authority is unqualified, the field is divided, or the claim still requires evidence. That matters here because expert testimony can be good evidence when the authority is relevant, the expertise is genuine, and the claim fits the expert consensus. That is the exact slip in this case: prestige replaces argument.
+Source: Associated Press | 2024-05-06
+https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="W12" t="str">
-        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+        <x:v>To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery
+AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. The fallacy here is Appeal to authority: someone treats an authority's endorsement as if it settled the issue, even when the authority is unqualified, the field is divided, or the claim still requires evidence. That matters here because expert testimony can be good evidence when the authority is relevant, the expertise is genuine, and the claim fits the expert consensus. That is the exact slip in this case: prestige replaces argument.
+Source: Associated Press | 2023-11-08
+https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
       </x:c>
       <x:c r="X12" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent
+AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. The fallacy here is Appeal to authority: someone treats an authority's endorsement as if it settled the issue, even when the authority is unqualified, the field is divided, or the claim still requires evidence. That matters here because expert testimony can be good evidence when the authority is relevant, the expertise is genuine, and the claim fits the expert consensus. That is the exact slip in this case: prestige replaces argument.
+Source: Associated Press | 2024-02-17
+https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="Y12" t="str">
-        <x:v>Debates about nutrition, vaccines, crypto, and AI frequently lean on celebrity experts or founders speaking outside their strongest field, while the underlying studies and uncertainties get little attention.</x:v>
+        <x:v>Debates about nutrition, vaccines, crypto, and AI frequently lean on celebrity experts or founders speaking outside their strongest field, while the underlying studies and uncertainties get little attention. The fallacy here is Appeal to authority: someone treats an authority's endorsement as if it settled the issue, even when the authority is unqualified, the field is divided, or the claim still requires evidence. That matters here because expert testimony can be good evidence when the authority is relevant, the expertise is genuine, and the claim fits the expert consensus. That is the exact slip in this case: prestige replaces argument.</x:v>
       </x:c>
       <x:c r="Z12" t="str">
-        <x:v>In public discussion of AI safety and capability, people often present a famous CEO's confidence level as if it were itself a substitute for technical evidence or broad expert agreement.</x:v>
+        <x:v>In public discussion of AI safety and capability, people often present a famous CEO's confidence level as if it were itself a substitute for technical evidence or broad expert agreement. The fallacy here is Appeal to authority: someone treats an authority's endorsement as if it settled the issue, even when the authority is unqualified, the field is divided, or the claim still requires evidence. That matters here because expert testimony can be good evidence when the authority is relevant, the expertise is genuine, and the claim fits the expert consensus. That is the exact slip in this case: prestige replaces argument.</x:v>
       </x:c>
       <x:c r="AA12" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -1203,16 +1245,22 @@
         <x:v>Consequences matter for what we should do, but they do not by themselves determine what is true. A painful implication does not refute a claim, and a comforting implication does not confirm one.</x:v>
       </x:c>
       <x:c r="V13" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. The fallacy here is Appeal to consequences: someone treats the desirability or undesirability of a conclusion as if it were evidence that the conclusion is true or false. That matters here because consequences matter for what we should do, but they do not by themselves determine what is true. A better analysis would remember that a painful implication does not refute a claim, and a comforting implication does not confirm one.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="W13" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate
+AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. The fallacy here is Appeal to consequences: someone treats the desirability or undesirability of a conclusion as if it were evidence that the conclusion is true or false. That matters here because consequences matter for what we should do, but they do not by themselves determine what is true. A better analysis would remember that a painful implication does not refute a claim, and a comforting implication does not confirm one.
+Source: Associated Press | 2024-06-27
+https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="X13" t="str">
-        <x:v>Some climate arguments treat the economic and political inconvenience of decarbonization as if it counted against the underlying science itself.</x:v>
+        <x:v>Some climate arguments treat the economic and political inconvenience of decarbonization as if it counted against the underlying science itself. The fallacy here is Appeal to consequences: someone treats the desirability or undesirability of a conclusion as if it were evidence that the conclusion is true or false. That matters here because consequences matter for what we should do, but they do not by themselves determine what is true. A better analysis would remember that a painful implication does not refute a claim, and a comforting implication does not confirm one.</x:v>
       </x:c>
       <x:c r="Y13" t="str">
-        <x:v>In debates about AI consciousness, animal cognition, or moral status, people sometimes argue that the conclusion cannot be right because accepting it would create uncomfortable obligations.</x:v>
+        <x:v>In debates about AI consciousness, animal cognition, or moral status, people sometimes argue that the conclusion cannot be right because accepting it would create uncomfortable obligations. The fallacy here is Appeal to consequences: someone treats the desirability or undesirability of a conclusion as if it were evidence that the conclusion is true or false. That matters here because consequences matter for what we should do, but they do not by themselves determine what is true. A better analysis would remember that a painful implication does not refute a claim, and a comforting implication does not confirm one.</x:v>
       </x:c>
       <x:c r="Z13" t="str"/>
       <x:c r="AA13" t="str">
@@ -1280,16 +1328,22 @@
         <x:v>Emotion is not irrational by itself. The fallacy appears when emotion substitutes for the reasoning that still needs to be supplied.</x:v>
       </x:c>
       <x:c r="V14" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>AI experimentation is high risk, high reward for low-profile political campaigns
+AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. The fallacy here is Appeal to emotion: a conclusion is pushed mainly by triggering fear, pity, outrage, pride, or hope rather than by showing that the conclusion follows from the evidence. That matters here because emotion is not irrational by itself. That is the exact slip in this case: emotion substitutes for the reasoning that still needs to be supplied.
+Source: Associated Press | 2024-06-17
+https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="W14" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate
+AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. The fallacy here is Appeal to emotion: a conclusion is pushed mainly by triggering fear, pity, outrage, pride, or hope rather than by showing that the conclusion follows from the evidence. That matters here because emotion is not irrational by itself. That is the exact slip in this case: emotion substitutes for the reasoning that still needs to be supplied.
+Source: Associated Press | 2024-06-27
+https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="X14" t="str">
-        <x:v>In 2024 campaign advertising, immigration, crime, and abortion messages often relied on fear-laden images and worst-case anecdotes whose emotional force far exceeded the actual argument being made.</x:v>
+        <x:v>In 2024 campaign advertising, immigration, crime, and abortion messages often relied on fear-laden images and worst-case anecdotes whose emotional force far exceeded the actual argument being made. The fallacy here is Appeal to emotion: a conclusion is pushed mainly by triggering fear, pity, outrage, pride, or hope rather than by showing that the conclusion follows from the evidence. That matters here because emotion is not irrational by itself. That is the exact slip in this case: emotion substitutes for the reasoning that still needs to be supplied.</x:v>
       </x:c>
       <x:c r="Y14" t="str">
-        <x:v>The spread of AI-generated political ads and deepfakes in 2024 showed how cheaply campaigns can trigger outrage or panic before voters have time to inspect the evidence.</x:v>
+        <x:v>The spread of AI-generated political ads and deepfakes in 2024 showed how cheaply campaigns can trigger outrage or panic before voters have time to inspect the evidence. The fallacy here is Appeal to emotion: a conclusion is pushed mainly by triggering fear, pity, outrage, pride, or hope rather than by showing that the conclusion follows from the evidence. That matters here because emotion is not irrational by itself. That is the exact slip in this case: emotion substitutes for the reasoning that still needs to be supplied.</x:v>
       </x:c>
       <x:c r="Z14" t="str"/>
       <x:c r="AA14" t="str">
@@ -1355,19 +1409,34 @@
         <x:v>Fear can be rational when the threat is real and well evidenced. The fallacy appears when fear does the persuasive work that evidence and reasoning have not done.</x:v>
       </x:c>
       <x:c r="V15" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>AI experimentation is high risk, high reward for low-profile political campaigns
+AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. The fallacy here is Appeal to fear: someone tries to secure agreement mainly by amplifying danger, threat, or panic rather than by showing that the conclusion is supported. That matters here because fear can be rational when the threat is real and well evidenced. That is the exact slip in this case: fear does the persuasive work that evidence and reasoning have not done.
+Source: Associated Press | 2024-06-17
+https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="W15" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging
+AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. The fallacy here is Appeal to fear: someone tries to secure agreement mainly by amplifying danger, threat, or panic rather than by showing that the conclusion is supported. That matters here because fear can be rational when the threat is real and well evidenced. That is the exact slip in this case: fear does the persuasive work that evidence and reasoning have not done.
+Source: Associated Press | 2024-05-18
+https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="X15" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>Q&amp;A on H5N1 Bird Flu
+FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. The fallacy here is Appeal to fear: someone tries to secure agreement mainly by amplifying danger, threat, or panic rather than by showing that the conclusion is supported. That matters here because fear can be rational when the threat is real and well evidenced. That is the exact slip in this case: fear does the persuasive work that evidence and reasoning have not done.
+Source: FactCheck.org | 2024-05-04
+https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="Y15" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets
+AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' The fallacy here is Appeal to fear: someone tries to secure agreement mainly by amplifying danger, threat, or panic rather than by showing that the conclusion is supported. That matters here because fear can be rational when the threat is real and well evidenced. That is the exact slip in this case: fear does the persuasive work that evidence and reasoning have not done.
+Source: Associated Press | 2024-09-26
+https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="Z15" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate
+AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. The fallacy here is Appeal to fear: someone tries to secure agreement mainly by amplifying danger, threat, or panic rather than by showing that the conclusion is supported. That matters here because fear can be rational when the threat is real and well evidenced. That is the exact slip in this case: fear does the persuasive work that evidence and reasoning have not done.
+Source: Associated Press | 2024-06-27
+https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="AA15" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -1432,13 +1501,16 @@
         <x:v>Compliments can be sincere and harmless. The fallacy appears when praise does the persuasive work by making agreement feel like a badge of intelligence or independence.</x:v>
       </x:c>
       <x:c r="V16" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+        <x:v>Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots
+AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. The fallacy here is Appeal to flattery: someone tries to win agreement by flattering the audience's intelligence, courage, independence, or special insight instead of supplying the missing evidence. That matters here because compliments can be sincere and harmless. That is the exact slip in this case: praise does the persuasive work by making agreement feel like a badge of intelligence or independence.
+Source: Associated Press | 2024-11-15
+https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="W16" t="str">
-        <x:v>Wellness, crypto, and conspiracy marketing often tells followers they are 'awake,' 'elite,' or 'smart enough to see through the lie,' turning assent into a test of self-image.</x:v>
+        <x:v>Wellness, crypto, and conspiracy marketing often tells followers they are 'awake,' 'elite,' or 'smart enough to see through the lie,' turning assent into a test of self-image. The fallacy here is Appeal to flattery: someone tries to win agreement by flattering the audience's intelligence, courage, independence, or special insight instead of supplying the missing evidence. That matters here because compliments can be sincere and harmless. That is the exact slip in this case: praise does the persuasive work by making agreement feel like a badge of intelligence or independence.</x:v>
       </x:c>
       <x:c r="X16" t="str">
-        <x:v>Political fundraising and influencer media frequently flatter supporters as the few people brave or intelligent enough to 'see what is really happening' before asking them to accept weakly supported claims.</x:v>
+        <x:v>Political fundraising and influencer media frequently flatter supporters as the few people brave or intelligent enough to 'see what is really happening' before asking them to accept weakly supported claims. The fallacy here is Appeal to flattery: someone tries to win agreement by flattering the audience's intelligence, courage, independence, or special insight instead of supplying the missing evidence. That matters here because compliments can be sincere and harmless. That is the exact slip in this case: praise does the persuasive work by making agreement feel like a badge of intelligence or independence.</x:v>
       </x:c>
       <x:c r="Y16" t="str"/>
       <x:c r="Z16" t="str"/>
@@ -1505,10 +1577,10 @@
         <x:v>Motives can be relevant to bias and credibility, but they do not automatically settle whether the argument or evidence is sound.</x:v>
       </x:c>
       <x:c r="V17" t="str">
-        <x:v>After the September 2024 ABC debate, accusations about moderator bias were often used not just to question fairness, but to pre-dismiss later fact-checks without engaging their substance.</x:v>
+        <x:v>After the September 2024 ABC debate, accusations about moderator bias were often used not just to question fairness, but to pre-dismiss later fact-checks without engaging their substance. The fallacy here is Appeal to motive: a claim is dismissed by speculating about the speaker's motives instead of addressing the claim itself. That matters here because motives can be relevant to bias and credibility, but they do not automatically settle whether the argument or evidence is sound. The better question is whether the emotional pull of the case is being mistaken for support.</x:v>
       </x:c>
       <x:c r="W17" t="str">
-        <x:v>In debates about climate, vaccines, and AI policy, critics are often waved away as 'funded,' 'bought,' or 'performing for clicks' instead of being answered.</x:v>
+        <x:v>In debates about climate, vaccines, and AI policy, critics are often waved away as 'funded,' 'bought,' or 'performing for clicks' instead of being answered. The fallacy here is Appeal to motive: a claim is dismissed by speculating about the speaker's motives instead of addressing the claim itself. That matters here because motives can be relevant to bias and credibility, but they do not automatically settle whether the argument or evidence is sound. The better question is whether the emotional pull of the case is being mistaken for support.</x:v>
       </x:c>
       <x:c r="X17" t="str"/>
       <x:c r="Y17" t="str"/>
@@ -1576,13 +1648,16 @@
         <x:v>Natural things can heal, but they can also poison, infect, and kill. The fallacy treats a vague origin label as if it already settled the medical, moral, or practical question.</x:v>
       </x:c>
       <x:c r="V18" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. The fallacy here is Appeal to nature: something is praised as good, safe, or right merely because it is called natural, or condemned as bad merely because it is called unnatural. That matters here because natural things can heal, but they can also poison, infect, and kill. A better analysis would remember that the fallacy treats a vague origin label as if it already settled the medical, moral, or practical question.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="W18" t="str">
-        <x:v>Wellness marketing for raw milk, supplements, and 'clean' products often treats natural as if it automatically meant safer, healthier, or morally superior.</x:v>
+        <x:v>Wellness marketing for raw milk, supplements, and 'clean' products often treats natural as if it automatically meant safer, healthier, or morally superior. The fallacy here is Appeal to nature: something is praised as good, safe, or right merely because it is called natural, or condemned as bad merely because it is called unnatural. That matters here because natural things can heal, but they can also poison, infect, and kill. A better analysis would remember that the fallacy treats a vague origin label as if it already settled the medical, moral, or practical question.</x:v>
       </x:c>
       <x:c r="X18" t="str">
-        <x:v>Arguments about sex, family, and medicine often smuggle a moral conclusion into the descriptive claim that one pattern is simply 'what nature intended.'</x:v>
+        <x:v>Arguments about sex, family, and medicine often smuggle a moral conclusion into the descriptive claim that one pattern is simply 'what nature intended.' The fallacy here is Appeal to nature: something is praised as good, safe, or right merely because it is called natural, or condemned as bad merely because it is called unnatural. That matters here because natural things can heal, but they can also poison, infect, and kill. A better analysis would remember that the fallacy treats a vague origin label as if it already settled the medical, moral, or practical question.</x:v>
       </x:c>
       <x:c r="Y18" t="str"/>
       <x:c r="Z18" t="str"/>
@@ -1651,13 +1726,16 @@
         <x:v>New tools and ideas can be improvements, but novelty itself is not proof. The relevant questions are performance, tradeoffs, and evidence, not freshness.</x:v>
       </x:c>
       <x:c r="V19" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+        <x:v>Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist
+In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. The fallacy here is Appeal to novelty: something is treated as better mainly because it is new, cutting-edge, or marketed as the future. That matters here because new tools and ideas can be improvements, but novelty itself is not proof. A better analysis would remember that the relevant questions are performance, tradeoffs, and evidence, not freshness.
+Source: Associated Press | 2024-05-06
+https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="W19" t="str">
-        <x:v>In the 2024 rush to adopt generative AI, many products were pitched as inherently superior because they were new, even when reliability, labor impact, and safety were still unsettled.</x:v>
+        <x:v>In the 2024 rush to adopt generative AI, many products were pitched as inherently superior because they were new, even when reliability, labor impact, and safety were still unsettled. The fallacy here is Appeal to novelty: something is treated as better mainly because it is new, cutting-edge, or marketed as the future. That matters here because new tools and ideas can be improvements, but novelty itself is not proof. A better analysis would remember that the relevant questions are performance, tradeoffs, and evidence, not freshness.</x:v>
       </x:c>
       <x:c r="X19" t="str">
-        <x:v>Political and management rhetoric often treats 'innovation' as a reason to trust a strategy before any serious test of whether it solves the underlying problem.</x:v>
+        <x:v>Political and management rhetoric often treats 'innovation' as a reason to trust a strategy before any serious test of whether it solves the underlying problem. The fallacy here is Appeal to novelty: something is treated as better mainly because it is new, cutting-edge, or marketed as the future. That matters here because new tools and ideas can be improvements, but novelty itself is not proof. A better analysis would remember that the relevant questions are performance, tradeoffs, and evidence, not freshness.</x:v>
       </x:c>
       <x:c r="Y19" t="str"/>
       <x:c r="Z19" t="str"/>
@@ -1724,10 +1802,10 @@
         <x:v>Compassion can matter for what response is humane, but it does not determine whether the underlying claim has been proved.</x:v>
       </x:c>
       <x:c r="V20" t="str">
-        <x:v>Fundraising and advocacy campaigns sometimes imply that questioning a factual claim is itself heartless, shifting the pressure from evidence to emotional identification.</x:v>
+        <x:v>Fundraising and advocacy campaigns sometimes imply that questioning a factual claim is itself heartless, shifting the pressure from evidence to emotional identification. The fallacy here is Appeal to pity: sympathy for a person or group is used as if it were evidence that a claim is true or a conclusion follows. That matters here because compassion can matter for what response is humane, but it does not determine whether the underlying claim has been proved. The better question is whether the emotional pull of the case is being mistaken for support.</x:v>
       </x:c>
       <x:c r="W20" t="str">
-        <x:v>Public figures under scrutiny sometimes ask to be believed or excused because they are suffering, overwhelmed, or facing intense pressure, even when those facts do not establish the truth of what they are saying.</x:v>
+        <x:v>Public figures under scrutiny sometimes ask to be believed or excused because they are suffering, overwhelmed, or facing intense pressure, even when those facts do not establish the truth of what they are saying. The fallacy here is Appeal to pity: sympathy for a person or group is used as if it were evidence that a claim is true or a conclusion follows. That matters here because compassion can matter for what response is humane, but it does not determine whether the underlying claim has been proved. The better question is whether the emotional pull of the case is being mistaken for support.</x:v>
       </x:c>
       <x:c r="X20" t="str"/>
       <x:c r="Y20" t="str"/>
@@ -1795,13 +1873,16 @@
         <x:v>Background can illuminate perspective, but hardship is not a truth detector. A difficult life story may earn sympathy or respect without settling the claim being made.</x:v>
       </x:c>
       <x:c r="V21" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+        <x:v>Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots
+AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. The fallacy here is Appeal to poverty: a claim is treated as more trustworthy, virtuous, or true mainly because its proponent is poor, ordinary, or from humble circumstances. That matters here because background can illuminate perspective, but hardship is not a truth detector. A better analysis would remember that a difficult life story may earn sympathy or respect without settling the claim being made.
+Source: Associated Press | 2024-11-15
+https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="W21" t="str">
-        <x:v>Campaign biographies in 2024 often leaned heavily on working-class roots and hardship stories, which may matter politically but do not by themselves verify a candidate's policy claims.</x:v>
+        <x:v>Campaign biographies in 2024 often leaned heavily on working-class roots and hardship stories, which may matter politically but do not by themselves verify a candidate's policy claims. The fallacy here is Appeal to poverty: a claim is treated as more trustworthy, virtuous, or true mainly because its proponent is poor, ordinary, or from humble circumstances. That matters here because background can illuminate perspective, but hardship is not a truth detector. A better analysis would remember that a difficult life story may earn sympathy or respect without settling the claim being made.</x:v>
       </x:c>
       <x:c r="X21" t="str">
-        <x:v>Populist media often imply that 'ordinary people' are automatically more honest than credentialed critics, as if social position alone settled the argument.</x:v>
+        <x:v>Populist media often imply that 'ordinary people' are automatically more honest than credentialed critics, as if social position alone settled the argument. The fallacy here is Appeal to poverty: a claim is treated as more trustworthy, virtuous, or true mainly because its proponent is poor, ordinary, or from humble circumstances. That matters here because background can illuminate perspective, but hardship is not a truth detector. A better analysis would remember that a difficult life story may earn sympathy or respect without settling the claim being made.</x:v>
       </x:c>
       <x:c r="Y21" t="str"/>
       <x:c r="Z21" t="str"/>
@@ -1864,19 +1945,31 @@
         <x:v>Possibility is a very weak starting point. Many things are possible without being probable, and many probable things still fail to happen in any given case.</x:v>
       </x:c>
       <x:c r="V22" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Pentagon study finds no sign of alien life in reported UFO sightings going back decades
+AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. The fallacy here is Appeal to probability: someone assumes that because something could happen, it is therefore likely or inevitable that it will happen. That matters here because possibility is a very weak starting point. A better analysis would remember that many things are possible without being probable, and many probable things still fail to happen in any given case.
+Source: Associated Press | 2024-03-08
+https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="W22" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens
+AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. The fallacy here is Appeal to probability: someone assumes that because something could happen, it is therefore likely or inevitable that it will happen. That matters here because possibility is a very weak starting point. A better analysis would remember that many things are possible without being probable, and many probable things still fail to happen in any given case.
+Source: Associated Press | 2024-11-14
+https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="X22" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+        <x:v>AI seen cutting worker numbers, survey by staffing company Adecco shows
+Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. The fallacy here is Appeal to probability: someone assumes that because something could happen, it is therefore likely or inevitable that it will happen. That matters here because possibility is a very weak starting point. A better analysis would remember that many things are possible without being probable, and many probable things still fail to happen in any given case.
+Source: Reuters | 2024-04-05
+https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="Y22" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>AI experimentation is high risk, high reward for low-profile political campaigns
+AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. The fallacy here is Appeal to probability: someone assumes that because something could happen, it is therefore likely or inevitable that it will happen. That matters here because possibility is a very weak starting point. A better analysis would remember that many things are possible without being probable, and many probable things still fail to happen in any given case.
+Source: Associated Press | 2024-06-17
+https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="Z22" t="str">
-        <x:v>Crypto, lottery, and sports-betting talk often slides from 'this could happen' to 'this is bound to happen,' especially after a short streak of wins.</x:v>
+        <x:v>Crypto, lottery, and sports-betting talk often slides from 'this could happen' to 'this is bound to happen,' especially after a short streak of wins. The fallacy here is Appeal to probability: someone assumes that because something could happen, it is therefore likely or inevitable that it will happen. That matters here because possibility is a very weak starting point. A better analysis would remember that many things are possible without being probable, and many probable things still fail to happen in any given case.</x:v>
       </x:c>
       <x:c r="AA22" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -1941,16 +2034,22 @@
         <x:v>Ridicule can make a position look silly without ever testing whether it is wrong. Laughter is not an argument.</x:v>
       </x:c>
       <x:c r="V23" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>AI experimentation is high risk, high reward for low-profile political campaigns
+AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. The fallacy here is Appeal to ridicule: mockery, embarrassment, or derision is used in place of showing why a view is false. That matters here because ridicule can make a position look silly without ever testing whether it is wrong. A better analysis would remember that laughter is not an argument.
+Source: Associated Press | 2024-06-17
+https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="W23" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+        <x:v>Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement
+AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. The fallacy here is Appeal to ridicule: mockery, embarrassment, or derision is used in place of showing why a view is false. That matters here because ridicule can make a position look silly without ever testing whether it is wrong. A better analysis would remember that laughter is not an argument.
+Source: Associated Press | 2024-09-10
+https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="X23" t="str">
-        <x:v>Debates about religion, feminism, climate, and AI are often reduced to memes whose purpose is to make one side look ridiculous rather than to assess the actual claim.</x:v>
+        <x:v>Debates about religion, feminism, climate, and AI are often reduced to memes whose purpose is to make one side look ridiculous rather than to assess the actual claim. The fallacy here is Appeal to ridicule: mockery, embarrassment, or derision is used in place of showing why a view is false. That matters here because ridicule can make a position look silly without ever testing whether it is wrong. A better analysis would remember that laughter is not an argument.</x:v>
       </x:c>
       <x:c r="Y23" t="str">
-        <x:v>Online discourse frequently treats a sarcastic dunk or quote-tweet pile-on as if public humiliation itself were refutation.</x:v>
+        <x:v>Online discourse frequently treats a sarcastic dunk or quote-tweet pile-on as if public humiliation itself were refutation. The fallacy here is Appeal to ridicule: mockery, embarrassment, or derision is used in place of showing why a view is false. That matters here because ridicule can make a position look silly without ever testing whether it is wrong. A better analysis would remember that laughter is not an argument.</x:v>
       </x:c>
       <x:c r="Z23" t="str"/>
       <x:c r="AA23" t="str">
@@ -2016,10 +2115,10 @@
         <x:v>Anger at the people who might benefit from a policy does not settle whether the policy is wise, fair, or effective.</x:v>
       </x:c>
       <x:c r="V24" t="str">
-        <x:v>Campaign messages often invite voters to reject a proposal because hated elites, immigrants, bankers, or academics might benefit, even when that says nothing about the proposal's merits.</x:v>
+        <x:v>Campaign messages often invite voters to reject a proposal because hated elites, immigrants, bankers, or academics might benefit, even when that says nothing about the proposal's merits. The fallacy here is Appeal to spite: resentment, bitterness, or hostility toward another group is used to drive support for a conclusion. That matters here because anger at the people who might benefit from a policy does not settle whether the policy is wise, fair, or effective. The better question is whether the emotional pull of the case is being mistaken for support.</x:v>
       </x:c>
       <x:c r="W24" t="str">
-        <x:v>Social-media outrage often works by making the audience feel that supporting a view would somehow reward people they already dislike.</x:v>
+        <x:v>Social-media outrage often works by making the audience feel that supporting a view would somehow reward people they already dislike. The fallacy here is Appeal to spite: resentment, bitterness, or hostility toward another group is used to drive support for a conclusion. That matters here because anger at the people who might benefit from a policy does not settle whether the policy is wise, fair, or effective. The better question is whether the emotional pull of the case is being mistaken for support.</x:v>
       </x:c>
       <x:c r="X24" t="str"/>
       <x:c r="Y24" t="str"/>
@@ -2089,16 +2188,22 @@
         <x:v>Traditions can embody wisdom, but age alone does not prove justice, truth, or usefulness. A tradition still has to survive present scrutiny.</x:v>
       </x:c>
       <x:c r="V25" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent
+AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. The fallacy here is Appeal to tradition: a claim or practice is defended mainly because it has a long history, customary status, or familiar place in a community. That matters here because traditions can embody wisdom, but age alone does not prove justice, truth, or usefulness. A better analysis would remember that a tradition still has to survive present scrutiny.
+Source: Associated Press | 2024-02-17
+https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="W25" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. The fallacy here is Appeal to tradition: a claim or practice is defended mainly because it has a long history, customary status, or familiar place in a community. That matters here because traditions can embody wisdom, but age alone does not prove justice, truth, or usefulness. A better analysis would remember that a tradition still has to survive present scrutiny.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="X25" t="str">
-        <x:v>In 2024 arguments that the United States is a 'Christian nation,' long practice and selective founding-era precedent were often treated as if they settled the constitutional question.</x:v>
+        <x:v>In 2024 arguments that the United States is a 'Christian nation,' long practice and selective founding-era precedent were often treated as if they settled the constitutional question. The fallacy here is Appeal to tradition: a claim or practice is defended mainly because it has a long history, customary status, or familiar place in a community. That matters here because traditions can embody wisdom, but age alone does not prove justice, truth, or usefulness. A better analysis would remember that a tradition still has to survive present scrutiny.</x:v>
       </x:c>
       <x:c r="Y25" t="str">
-        <x:v>Arguments about schooling, marriage, and gender roles often rely on 'we have always done it this way' instead of showing why the tradition remains just or effective.</x:v>
+        <x:v>Arguments about schooling, marriage, and gender roles often rely on 'we have always done it this way' instead of showing why the tradition remains just or effective. The fallacy here is Appeal to tradition: a claim or practice is defended mainly because it has a long history, customary status, or familiar place in a community. That matters here because traditions can embody wisdom, but age alone does not prove justice, truth, or usefulness. A better analysis would remember that a tradition still has to survive present scrutiny.</x:v>
       </x:c>
       <x:c r="Z25" t="str"/>
       <x:c r="AA25" t="str">
@@ -2164,10 +2269,10 @@
         <x:v>Success can indicate skill in a particular domain, but money is not a universal credential. Wealth may buy attention, not truth.</x:v>
       </x:c>
       <x:c r="V26" t="str">
-        <x:v>In 2024 and 2025, fans and investors often treated billionaire founders' views on AI, politics, or medicine as self-validating because of their wealth rather than because the evidence was strong.</x:v>
+        <x:v>In 2024 and 2025, fans and investors often treated billionaire founders' views on AI, politics, or medicine as self-validating because of their wealth rather than because the evidence was strong. The fallacy here is Appeal to wealth: a claim is treated as more credible or correct mainly because it comes from a rich, famous, or financially successful person. That matters here because success can indicate skill in a particular domain, but money is not a universal credential. A better analysis would remember that wealth may buy attention, not truth.</x:v>
       </x:c>
       <x:c r="W26" t="str">
-        <x:v>The unverified ABC debate affidavit gained extra credibility online after high-profile wealthy amplifiers helped circulate it, as though status itself made the claim more trustworthy.</x:v>
+        <x:v>The unverified ABC debate affidavit gained extra credibility online after high-profile wealthy amplifiers helped circulate it, as though status itself made the claim more trustworthy. The fallacy here is Appeal to wealth: a claim is treated as more credible or correct mainly because it comes from a rich, famous, or financially successful person. That matters here because success can indicate skill in a particular domain, but money is not a universal credential. A better analysis would remember that wealth may buy attention, not truth.</x:v>
       </x:c>
       <x:c r="X26" t="str"/>
       <x:c r="Y26" t="str"/>
@@ -2231,13 +2336,16 @@
         <x:v>A bad argument can defend a true claim, and a strong claim can be defended poorly. Refuting the reasoning offered is not the same thing as refuting the conclusion.</x:v>
       </x:c>
       <x:c r="V27" t="str">
-        <x:v>AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>AI experimentation is high risk, high reward for low-profile political campaigns
+AP's 2024 reporting on AI political content repeatedly showed how easy it is for people to move from 'this image has a common AI tell' to 'therefore this image must be AI-generated.' That conclusion can be tempting in practice, but the fact pattern only supports a possibility, not a guaranteed diagnosis. The fallacy here is Argument from fallacy: someone infers that because a particular argument for a conclusion is weak or fallacious, the conclusion itself must therefore be false. That matters here because a bad argument can defend a true claim, and a strong claim can be defended poorly. A better analysis would remember that refuting the reasoning offered is not the same thing as refuting the conclusion.
+Source: Associated Press | 2024-06-17
+https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="W27" t="str">
-        <x:v>When a candidate exaggerates one statistic, opponents often jump from 'that argument was flawed' to 'the broader policy position must therefore be false.'</x:v>
+        <x:v>When a candidate exaggerates one statistic, opponents often jump from 'that argument was flawed' to 'the broader policy position must therefore be false.' The fallacy here is Argument from fallacy: someone infers that because a particular argument for a conclusion is weak or fallacious, the conclusion itself must therefore be false. That matters here because a bad argument can defend a true claim, and a strong claim can be defended poorly. A better analysis would remember that refuting the reasoning offered is not the same thing as refuting the conclusion.</x:v>
       </x:c>
       <x:c r="X27" t="str">
-        <x:v>Online 'gotcha' culture frequently treats catching a fallacious defense as if it automatically disproved whatever the speaker was trying to defend.</x:v>
+        <x:v>Online 'gotcha' culture frequently treats catching a fallacious defense as if it automatically disproved whatever the speaker was trying to defend. The fallacy here is Argument from fallacy: someone infers that because a particular argument for a conclusion is weak or fallacious, the conclusion itself must therefore be false. That matters here because a bad argument can defend a true claim, and a strong claim can be defended poorly. A better analysis would remember that refuting the reasoning offered is not the same thing as refuting the conclusion.</x:v>
       </x:c>
       <x:c r="Y27" t="str"/>
       <x:c r="Z27" t="str"/>
@@ -2302,19 +2410,28 @@
         <x:v>The burden is not met by pointing to a gap in refutation. A claim needs positive support of its own. Lack of an explanation is not the same thing as evidence for a preferred explanation.</x:v>
       </x:c>
       <x:c r="V28" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Pentagon study finds no sign of alien life in reported UFO sightings going back decades
+AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. The fallacy here is Argument from ignorance: someone concludes that a claim is true because it has not been disproved, or false because it has not been proved. That matters here because the burden is not met by pointing to a gap in refutation. A better analysis would remember that a claim needs positive support of its own.
+Source: Associated Press | 2024-03-08
+https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="W28" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens
+AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. The fallacy here is Argument from ignorance: someone concludes that a claim is true because it has not been disproved, or false because it has not been proved. That matters here because the burden is not met by pointing to a gap in refutation. A better analysis would remember that a claim needs positive support of its own.
+Source: Associated Press | 2024-11-14
+https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="X28" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. The fallacy here is Argument from ignorance: someone concludes that a claim is true because it has not been disproved, or false because it has not been proved. That matters here because the burden is not met by pointing to a gap in refutation. A better analysis would remember that a claim needs positive support of its own.
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="Y28" t="str">
-        <x:v>After an anonymous affidavit circulated online in September 2024 alleging that ABC had secretly rigged the Harris-Trump debate, many posts treated the absence of immediate disproof as if it were evidence that the allegation was real.</x:v>
+        <x:v>After an anonymous affidavit circulated online in September 2024 alleging that ABC had secretly rigged the Harris-Trump debate, many posts treated the absence of immediate disproof as if it were evidence that the allegation was real. The fallacy here is Argument from ignorance: someone concludes that a claim is true because it has not been disproved, or false because it has not been proved. That matters here because the burden is not met by pointing to a gap in refutation. A better analysis would remember that a claim needs positive support of its own.</x:v>
       </x:c>
       <x:c r="Z28" t="str">
-        <x:v>UAP discussions often jump from 'we do not yet know what caused this' to 'therefore it was extraterrestrial technology,' which treats unexplained as if it meant explained by the favored hypothesis.</x:v>
+        <x:v>UAP discussions often jump from 'we do not yet know what caused this' to 'therefore it was extraterrestrial technology,' which treats unexplained as if it meant explained by the favored hypothesis. The fallacy here is Argument from ignorance: someone concludes that a claim is true because it has not been disproved, or false because it has not been proved. That matters here because the burden is not met by pointing to a gap in refutation. A better analysis would remember that a claim needs positive support of its own.</x:v>
       </x:c>
       <x:c r="AA28" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -2377,13 +2494,16 @@
         <x:v>Our imagination is not a reliable measure of what reality permits. Difficulty understanding a mechanism may justify caution or further inquiry, but it does not by itself establish that a preferred alternative is true.</x:v>
       </x:c>
       <x:c r="V29" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Pentagon study finds no sign of alien life in reported UFO sightings going back decades
+AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. The fallacy here is Argument from incredulity: someone treats their inability to imagine, explain, or believe a claim as evidence that the claim must be false, or conversely true. That matters here because our imagination is not a reliable measure of what reality permits. A better analysis would remember that difficulty understanding a mechanism may justify caution or further inquiry, but it does not by itself establish that a preferred alternative is true.
+Source: Associated Press | 2024-03-08
+https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="W29" t="str">
-        <x:v>Discussions of evolution, climate systems, and AI often slide from 'I do not see how that could work' to 'therefore it cannot be right.'</x:v>
+        <x:v>Discussions of evolution, climate systems, and AI often slide from 'I do not see how that could work' to 'therefore it cannot be right.' The fallacy here is Argument from incredulity: someone treats their inability to imagine, explain, or believe a claim as evidence that the claim must be false, or conversely true. That matters here because our imagination is not a reliable measure of what reality permits. A better analysis would remember that difficulty understanding a mechanism may justify caution or further inquiry, but it does not by itself establish that a preferred alternative is true.</x:v>
       </x:c>
       <x:c r="X29" t="str">
-        <x:v>Paranormal and conspiracy arguments often rely on the mirror image of the same move: 'I cannot imagine another explanation, so my favored explanation must be true.'</x:v>
+        <x:v>Paranormal and conspiracy arguments often rely on the mirror image of the same move: 'I cannot imagine another explanation, so my favored explanation must be true.' The fallacy here is Argument from incredulity: someone treats their inability to imagine, explain, or believe a claim as evidence that the claim must be false, or conversely true. That matters here because our imagination is not a reliable measure of what reality permits. A better analysis would remember that difficulty understanding a mechanism may justify caution or further inquiry, but it does not by itself establish that a preferred alternative is true.</x:v>
       </x:c>
       <x:c r="Y29" t="str"/>
       <x:c r="Z29" t="str"/>
@@ -2448,19 +2568,31 @@
         <x:v>A claim does not become better supported because it is repeated by the same speaker, echoed by many speakers, or circulated for a long time. Repetition changes familiarity, not the underlying evidence.</x:v>
       </x:c>
       <x:c r="V30" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging
+AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. The fallacy here is Argument from repetition: repetition is treated as if it adds evidence, wearing down doubt or making a claim seem true through familiarity. That matters here because a claim does not become better supported because it is repeated by the same speaker, echoed by many speakers, or circulated for a long time. A better analysis would remember that repetition changes familiarity, not the underlying evidence.
+Source: Associated Press | 2024-05-18
+https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="W30" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets
+AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' The fallacy here is Argument from repetition: repetition is treated as if it adds evidence, wearing down doubt or making a claim seem true through familiarity. That matters here because a claim does not become better supported because it is repeated by the same speaker, echoed by many speakers, or circulated for a long time. A better analysis would remember that repetition changes familiarity, not the underlying evidence.
+Source: Associated Press | 2024-09-26
+https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="X30" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town
+PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. The fallacy here is Argument from repetition: repetition is treated as if it adds evidence, wearing down doubt or making a claim seem true through familiarity. That matters here because a claim does not become better supported because it is repeated by the same speaker, echoed by many speakers, or circulated for a long time. A better analysis would remember that repetition changes familiarity, not the underlying evidence.
+Source: PolitiFact | 2024-09-09
+https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
       </x:c>
       <x:c r="Y30" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+        <x:v>Biden tells Trump to 'get a life, man' and stop storm misinformation
+AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. The fallacy here is Argument from repetition: repetition is treated as if it adds evidence, wearing down doubt or making a claim seem true through familiarity. That matters here because a claim does not become better supported because it is repeated by the same speaker, echoed by many speakers, or circulated for a long time. A better analysis would remember that repetition changes familiarity, not the underlying evidence.
+Source: Associated Press | 2024-10-10
+https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
       </x:c>
       <x:c r="Z30" t="str">
-        <x:v>The Springfield, Ohio pet-eating rumor in September 2024 moved from rumor to national talking point largely through repetition across social media, cable segments, and campaign rhetoric even though local officials said there was no credible evidence.</x:v>
+        <x:v>The Springfield, Ohio pet-eating rumor in September 2024 moved from rumor to national talking point largely through repetition across social media, cable segments, and campaign rhetoric even though local officials said there was no credible evidence. The fallacy here is Argument from repetition: repetition is treated as if it adds evidence, wearing down doubt or making a claim seem true through familiarity. That matters here because a claim does not become better supported because it is repeated by the same speaker, echoed by many speakers, or circulated for a long time. A better analysis would remember that repetition changes familiarity, not the underlying evidence.</x:v>
       </x:c>
       <x:c r="AA30" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -2525,10 +2657,10 @@
         <x:v>Silence can matter when a response would clearly be expected and feasible. Outside that setting, it often tells us little.</x:v>
       </x:c>
       <x:c r="V31" t="str">
-        <x:v>The absence of public confirmation for many election-fraud and migrant-voting rumors was often spun as suspicious silence rather than as a sign that the underlying evidence was weak or nonexistent.</x:v>
+        <x:v>The absence of public confirmation for many election-fraud and migrant-voting rumors was often spun as suspicious silence rather than as a sign that the underlying evidence was weak or nonexistent. The fallacy here is Argument from silence: a claim is treated as validated because opponents, authorities, or witnesses did not deny it, respond to it, or mention it. That matters here because silence can matter when a response would clearly be expected and feasible. A better analysis would remember that outside that setting, it often tells us little.</x:v>
       </x:c>
       <x:c r="W31" t="str">
-        <x:v>A 'no comment' from campaigns, police, or institutions is regularly treated as if it were a tacit admission, even though legal, strategic, or practical reasons may explain the silence.</x:v>
+        <x:v>A 'no comment' from campaigns, police, or institutions is regularly treated as if it were a tacit admission, even though legal, strategic, or practical reasons may explain the silence. The fallacy here is Argument from silence: a claim is treated as validated because opponents, authorities, or witnesses did not deny it, respond to it, or mention it. That matters here because silence can matter when a response would clearly be expected and feasible. A better analysis would remember that outside that setting, it often tells us little.</x:v>
       </x:c>
       <x:c r="X31" t="str"/>
       <x:c r="Y31" t="str"/>
@@ -2598,10 +2730,10 @@
         <x:v>Threats can force compliance, but they do not transform a bad argument into a good one. Fear may explain why someone goes along; it does not show that the view is correct.</x:v>
       </x:c>
       <x:c r="V32" t="str">
-        <x:v>In countries where blasphemy, apostasy, or political dissent can trigger severe punishment, outward conformity is often mistaken for genuine persuasion when it may simply reflect fear.</x:v>
+        <x:v>In countries where blasphemy, apostasy, or political dissent can trigger severe punishment, outward conformity is often mistaken for genuine persuasion when it may simply reflect fear. The fallacy here is Argumentum ad baculum: agreement is extracted by threat, intimidation, or coercive pressure rather than by showing that the claim is true. That matters here because threats can force compliance, but they do not transform a bad argument into a good one. A better analysis would remember that fear may explain why someone goes along; it does not show that the view is correct.</x:v>
       </x:c>
       <x:c r="W32" t="str">
-        <x:v>Online campaigns that threaten doxxing, blacklisting, or mass harassment often aim to secure silence or agreement by making disagreement personally costly.</x:v>
+        <x:v>Online campaigns that threaten doxxing, blacklisting, or mass harassment often aim to secure silence or agreement by making disagreement personally costly. The fallacy here is Argumentum ad baculum: agreement is extracted by threat, intimidation, or coercive pressure rather than by showing that the claim is true. That matters here because threats can force compliance, but they do not transform a bad argument into a good one. A better analysis would remember that fear may explain why someone goes along; it does not show that the view is correct.</x:v>
       </x:c>
       <x:c r="X32" t="str"/>
       <x:c r="Y32" t="str"/>
@@ -2673,10 +2805,10 @@
         <x:v>Popularity can reveal what people want, fear, or have been persuaded by, but it does not settle what is true. Crowds can be informed, confused, manipulated, or all three at once.</x:v>
       </x:c>
       <x:c r="V33" t="str">
-        <x:v>Advocates of raw milk and other 'natural' wellness products often point to growing enthusiasm, celebrity uptake, or huge followings as if social momentum itself established safety or effectiveness.</x:v>
+        <x:v>Advocates of raw milk and other 'natural' wellness products often point to growing enthusiasm, celebrity uptake, or huge followings as if social momentum itself established safety or effectiveness. The fallacy here is Argumentum ad populum: a claim is treated as true, reasonable, or justified mainly because many people believe it, share it, or act on it. That matters here because popularity can reveal what people want, fear, or have been persuaded by, but it does not settle what is true. A better analysis would remember that crowds can be informed, confused, manipulated, or all three at once.</x:v>
       </x:c>
       <x:c r="W33" t="str">
-        <x:v>Viral political claims are often defended with phrases like 'everyone is talking about it' or 'it has millions of views,' which confuses reach with reliability.</x:v>
+        <x:v>Viral political claims are often defended with phrases like 'everyone is talking about it' or 'it has millions of views,' which confuses reach with reliability. The fallacy here is Argumentum ad populum: a claim is treated as true, reasonable, or justified mainly because many people believe it, share it, or act on it. That matters here because popularity can reveal what people want, fear, or have been persuaded by, but it does not settle what is true. A better analysis would remember that crowds can be informed, confused, manipulated, or all three at once.</x:v>
       </x:c>
       <x:c r="X33" t="str"/>
       <x:c r="Y33" t="str"/>
@@ -2738,10 +2870,10 @@
         <x:v>There is an important difference between suspending belief, doubting a claim, and asserting the opposite claim. Collapsing those positions is often a way of shifting burdens that have not been earned.</x:v>
       </x:c>
       <x:c r="V34" t="str">
-        <x:v>Religious and paranormal debates often insist that skepticism itself is just another faith commitment, as if withholding belief carried the same evidential burden as proposing the phenomenon.</x:v>
+        <x:v>Religious and paranormal debates often insist that skepticism itself is just another faith commitment, as if withholding belief carried the same evidential burden as proposing the phenomenon. The fallacy here is Artificial negation: the wording of a negative position is manipulated so that mere non-belief is treated as if it were the same thing as a strong positive denial. That matters here because there is an important difference between suspending belief, doubting a claim, and asserting the opposite claim. A better analysis would remember that collapsing those positions is often a way of shifting burdens that have not been earned.</x:v>
       </x:c>
       <x:c r="W34" t="str">
-        <x:v>Arguments about election fraud and miracle claims sometimes recast 'I have not seen enough evidence' into 'you are certain it never happened' so the original claimant can dodge the burden of proof.</x:v>
+        <x:v>Arguments about election fraud and miracle claims sometimes recast 'I have not seen enough evidence' into 'you are certain it never happened' so the original claimant can dodge the burden of proof. The fallacy here is Artificial negation: the wording of a negative position is manipulated so that mere non-belief is treated as if it were the same thing as a strong positive denial. That matters here because there is an important difference between suspending belief, doubting a claim, and asserting the opposite claim. A better analysis would remember that collapsing those positions is often a way of shifting burdens that have not been earned.</x:v>
       </x:c>
       <x:c r="X34" t="str"/>
       <x:c r="Y34" t="str"/>
@@ -2811,16 +2943,22 @@
         <x:v>Associations can sometimes matter when they reveal bias, incentives, or causal links. The fallacy appears when the link is treated as decisive even though it does not address the argument.</x:v>
       </x:c>
       <x:c r="V35" t="str">
-        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+        <x:v>To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery
+AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. The fallacy here is Association fallacy: a claim is accepted or dismissed because of some irrelevant association rather than because of the merits of the claim itself. That matters here because associations can sometimes matter when they reveal bias, incentives, or causal links. That is the exact slip in this case: the link is treated as decisive even though it does not address the argument.
+Source: Associated Press | 2023-11-08
+https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
       </x:c>
       <x:c r="W35" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+        <x:v>Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots
+AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. The fallacy here is Association fallacy: a claim is accepted or dismissed because of some irrelevant association rather than because of the merits of the claim itself. That matters here because associations can sometimes matter when they reveal bias, incentives, or causal links. That is the exact slip in this case: the link is treated as decisive even though it does not address the argument.
+Source: Associated Press | 2024-11-15
+https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="X35" t="str">
-        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported.</x:v>
+        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported. The fallacy here is Association fallacy: a claim is accepted or dismissed because of some irrelevant association rather than because of the merits of the claim itself. That matters here because associations can sometimes matter when they reveal bias, incentives, or causal links. That is the exact slip in this case: the link is treated as decisive even though it does not address the argument.</x:v>
       </x:c>
       <x:c r="Y35" t="str">
-        <x:v>Political arguments routinely assume that if a bad person, rival group, or disliked movement touched an idea, the idea itself must be false or tainted.</x:v>
+        <x:v>Political arguments routinely assume that if a bad person, rival group, or disliked movement touched an idea, the idea itself must be false or tainted. The fallacy here is Association fallacy: a claim is accepted or dismissed because of some irrelevant association rather than because of the merits of the claim itself. That matters here because associations can sometimes matter when they reveal bias, incentives, or causal links. That is the exact slip in this case: the link is treated as decisive even though it does not address the argument.</x:v>
       </x:c>
       <x:c r="Z35" t="str"/>
       <x:c r="AA35" t="str">
@@ -2882,19 +3020,34 @@
         <x:v>Confidence, volume, and repetition can make a bare assertion sound weighty, but they do not do the evidential work. When the core support is missing, the proper question is still: What is the evidence?</x:v>
       </x:c>
       <x:c r="V36" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said
+AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. The fallacy here is Bare assertion fallacy: a contested claim is simply asserted, often confidently, without the evidence needed to justify it. That matters here because confidence, volume, and repetition can make a bare assertion sound weighty, but they do not do the evidential work. A better analysis would remember that when the core support is missing, the proper question is still: What is the evidence?
+Source: Associated Press | 2024-10-26
+https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="W36" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets
+AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' The fallacy here is Bare assertion fallacy: a contested claim is simply asserted, often confidently, without the evidence needed to justify it. That matters here because confidence, volume, and repetition can make a bare assertion sound weighty, but they do not do the evidential work. A better analysis would remember that when the core support is missing, the proper question is still: What is the evidence?
+Source: Associated Press | 2024-09-26
+https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="X36" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town
+PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. The fallacy here is Bare assertion fallacy: a contested claim is simply asserted, often confidently, without the evidence needed to justify it. That matters here because confidence, volume, and repetition can make a bare assertion sound weighty, but they do not do the evidential work. A better analysis would remember that when the core support is missing, the proper question is still: What is the evidence?
+Source: PolitiFact | 2024-09-09
+https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
       </x:c>
       <x:c r="Y36" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. The fallacy here is Bare assertion fallacy: a contested claim is simply asserted, often confidently, without the evidence needed to justify it. That matters here because confidence, volume, and repetition can make a bare assertion sound weighty, but they do not do the evidential work. A better analysis would remember that when the core support is missing, the proper question is still: What is the evidence?
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="Z36" t="str">
-        <x:v>AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. — Associated Press | Biden tells Trump to 'get a life, man' and stop storm misinformation | 2024-10-10 | https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
+        <x:v>Biden tells Trump to 'get a life, man' and stop storm misinformation
+AP's October 10, 2024 report on hurricane-response misinformation is a clean example of how disaster politics invites fear-based claims that spread faster than verification. The article is especially useful for showing how emotionally convenient numbers and slogans can be detached from what agencies actually said. The fallacy here is Bare assertion fallacy: a contested claim is simply asserted, often confidently, without the evidence needed to justify it. That matters here because confidence, volume, and repetition can make a bare assertion sound weighty, but they do not do the evidential work. A better analysis would remember that when the core support is missing, the proper question is still: What is the evidence?
+Source: Associated Press | 2024-10-10
+https://apnews.com/article/cb814f209e71481f078f20e569bc63d0</x:v>
       </x:c>
       <x:c r="AA36" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -2955,19 +3108,34 @@
         <x:v>For rare conditions or rare events, even very accurate tests can generate more false positives than true positives. The missing question is not just 'How accurate is the test?' but 'How common is the condition before the test is applied?'</x:v>
       </x:c>
       <x:c r="V37" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging
+AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. The fallacy here is Base rate fallacy: someone judges how likely a case is by focusing on vivid case-specific evidence while ignoring the underlying frequency of the thing in question. That matters here because for rare conditions or rare events, even very accurate tests can generate more false positives than true positives. A better analysis would remember that the missing question is not just 'How accurate is the test?' but 'How common is the condition before the test is applied?'
+Source: Associated Press | 2024-05-18
+https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="W37" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not
+NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. The fallacy here is Base rate fallacy: someone judges how likely a case is by focusing on vivid case-specific evidence while ignoring the underlying frequency of the thing in question. That matters here because for rare conditions or rare events, even very accurate tests can generate more false positives than true positives. A better analysis would remember that the missing question is not just 'How accurate is the test?' but 'How common is the condition before the test is applied?'
+Source: NPR | 2024-10-12
+https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="X37" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+        <x:v>Iowa finds several dozen instances of noncitizens voting in a past election
+AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. The fallacy here is Base rate fallacy: someone judges how likely a case is by focusing on vivid case-specific evidence while ignoring the underlying frequency of the thing in question. That matters here because for rare conditions or rare events, even very accurate tests can generate more false positives than true positives. A better analysis would remember that the missing question is not just 'How accurate is the test?' but 'How common is the condition before the test is applied?'
+Source: Associated Press | 2024-10-23
+https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
       <x:c r="Y37" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>Q&amp;A on H5N1 Bird Flu
+FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. The fallacy here is Base rate fallacy: someone judges how likely a case is by focusing on vivid case-specific evidence while ignoring the underlying frequency of the thing in question. That matters here because for rare conditions or rare events, even very accurate tests can generate more false positives than true positives. A better analysis would remember that the missing question is not just 'How accurate is the test?' but 'How common is the condition before the test is applied?'
+Source: FactCheck.org | 2024-05-04
+https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="Z37" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+        <x:v>Why AP called the Arizona Senate race for Ruben Gallego
+AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. The fallacy here is Base rate fallacy: someone judges how likely a case is by focusing on vivid case-specific evidence while ignoring the underlying frequency of the thing in question. That matters here because for rare conditions or rare events, even very accurate tests can generate more false positives than true positives. A better analysis would remember that the missing question is not just 'How accurate is the test?' but 'How common is the condition before the test is applied?'
+Source: Associated Press | 2024-11-12
+https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
       </x:c>
       <x:c r="AA37" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -3030,13 +3198,16 @@
         <x:v>Circularity can be obvious, but it is often hidden behind rewording, loaded descriptions, or a chain of claims that loops back to the start. The argument feels like support has been offered when the conclusion has only been restated.</x:v>
       </x:c>
       <x:c r="V38" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. The fallacy here is Begging the question: an argument quietly assumes the very point it is supposed to prove, so the conclusion is built into the premises. That matters here because circularity can be obvious, but it is often hidden behind rewording, loaded descriptions, or a chain of claims that loops back to the start. A better analysis would remember that the argument feels like support has been offered when the conclusion has only been restated.
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="W38" t="str">
-        <x:v>Conspiracy-style reasoning often treats the absence of confirming evidence as proof that the conspiracy is powerful enough to hide the evidence, which assumes the conclusion inside the explanation.</x:v>
+        <x:v>Conspiracy-style reasoning often treats the absence of confirming evidence as proof that the conspiracy is powerful enough to hide the evidence, which assumes the conclusion inside the explanation. The fallacy here is Begging the question: an argument quietly assumes the very point it is supposed to prove, so the conclusion is built into the premises. That matters here because circularity can be obvious, but it is often hidden behind rewording, loaded descriptions, or a chain of claims that loops back to the start. A better analysis would remember that the argument feels like support has been offered when the conclusion has only been restated.</x:v>
       </x:c>
       <x:c r="X38" t="str">
-        <x:v>Debates about 'real journalism' or 'real science' sometimes define the trustworthy outlet or institution as whichever one already agrees with the speaker's preferred view.</x:v>
+        <x:v>Debates about 'real journalism' or 'real science' sometimes define the trustworthy outlet or institution as whichever one already agrees with the speaker's preferred view. The fallacy here is Begging the question: an argument quietly assumes the very point it is supposed to prove, so the conclusion is built into the premises. That matters here because circularity can be obvious, but it is often hidden behind rewording, loaded descriptions, or a chain of claims that loops back to the start. A better analysis would remember that the argument feels like support has been offered when the conclusion has only been restated.</x:v>
       </x:c>
       <x:c r="Y38" t="str"/>
       <x:c r="Z38" t="str"/>
@@ -3099,10 +3270,10 @@
         <x:v>Even if a group tendency were real, it would not eliminate the need for evidence about the particular person under discussion.</x:v>
       </x:c>
       <x:c r="V39" t="str">
-        <x:v>After scandals in policing, finance, or clergy, critics sometimes assume any individual in the profession personally shares the worst traits of the institution.</x:v>
+        <x:v>After scandals in policing, finance, or clergy, critics sometimes assume any individual in the profession personally shares the worst traits of the institution. The fallacy here is Bottom-up condemnation: a negative generalization about a group is used as if it settled the character or behavior of a specific member of that group. That matters here because even if a group tendency were real, it would not eliminate the need for evidence about the particular person under discussion. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W39" t="str">
-        <x:v>Online discourse often treats party label, employer, or religious affiliation as if it were enough to prove what a specific person believes or will do.</x:v>
+        <x:v>Online discourse often treats party label, employer, or religious affiliation as if it were enough to prove what a specific person believes or will do. The fallacy here is Bottom-up condemnation: a negative generalization about a group is used as if it settled the character or behavior of a specific member of that group. That matters here because even if a group tendency were real, it would not eliminate the need for evidence about the particular person under discussion. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X39" t="str"/>
       <x:c r="Y39" t="str"/>
@@ -3166,10 +3337,10 @@
         <x:v>A flattering stereotype is still a stereotype. Group membership can create a first impression, but it does not establish the individual's actual record.</x:v>
       </x:c>
       <x:c r="V40" t="str">
-        <x:v>Prestige effects often lead audiences to assume that anyone from a famous university or respected nonprofit is trustworthy even outside their area of expertise.</x:v>
+        <x:v>Prestige effects often lead audiences to assume that anyone from a famous university or respected nonprofit is trustworthy even outside their area of expertise. The fallacy here is Bottom-up justification: a positive generalization about a group is used as if it established the virtue or competence of a specific member of that group. That matters here because a flattering stereotype is still a stereotype. A better analysis would remember that group membership can create a first impression, but it does not establish the individual's actual record.</x:v>
       </x:c>
       <x:c r="W40" t="str">
-        <x:v>Voters sometimes infer that a candidate from a reform organization must be personally honest before examining the candidate's own conduct.</x:v>
+        <x:v>Voters sometimes infer that a candidate from a reform organization must be personally honest before examining the candidate's own conduct. The fallacy here is Bottom-up justification: a positive generalization about a group is used as if it established the virtue or competence of a specific member of that group. That matters here because a flattering stereotype is still a stereotype. A better analysis would remember that group membership can create a first impression, but it does not establish the individual's actual record.</x:v>
       </x:c>
       <x:c r="X40" t="str"/>
       <x:c r="Y40" t="str"/>
@@ -3235,10 +3406,10 @@
         <x:v>Repair work creates visible activity, but it mainly restores value that was lost. The missing comparison is what households, firms, insurers, and governments could have done with those same resources if the damage had not occurred.</x:v>
       </x:c>
       <x:c r="V41" t="str">
-        <x:v>After Hurricanes Helene and Milton in October 2024, some commentary emphasized reconstruction jobs and spending while downplaying the destroyed homes, shuttered businesses, and other uses those resources would have supported.</x:v>
+        <x:v>After Hurricanes Helene and Milton in October 2024, some commentary emphasized reconstruction jobs and spending while downplaying the destroyed homes, shuttered businesses, and other uses those resources would have supported. The fallacy here is Broken window fallacy: destruction or forced replacement is treated as an economic gain because the visible spending is counted while the unseen losses and forgone alternatives are ignored. That matters here because repair work creates visible activity, but it mainly restores value that was lost. A better analysis would remember that the missing comparison is what households, firms, insurers, and governments could have done with those same resources if the damage had not occurred.</x:v>
       </x:c>
       <x:c r="W41" t="str">
-        <x:v>Cyberattacks, vandalism, and infrastructure failures are sometimes framed as hidden economic stimulus because repairs employ people, even though the spending mainly compensates for an avoidable loss.</x:v>
+        <x:v>Cyberattacks, vandalism, and infrastructure failures are sometimes framed as hidden economic stimulus because repairs employ people, even though the spending mainly compensates for an avoidable loss. The fallacy here is Broken window fallacy: destruction or forced replacement is treated as an economic gain because the visible spending is counted while the unseen losses and forgone alternatives are ignored. That matters here because repair work creates visible activity, but it mainly restores value that was lost. A better analysis would remember that the missing comparison is what households, firms, insurers, and governments could have done with those same resources if the damage had not occurred.</x:v>
       </x:c>
       <x:c r="X41" t="str"/>
       <x:c r="Y41" t="str"/>
@@ -3306,19 +3477,34 @@
         <x:v>Cherry picking can involve hand-picked dates, unusual baselines, isolated anecdotes, or a single study taken out of a larger research picture. The defect is not using examples, but using a biased sample as if it were representative.</x:v>
       </x:c>
       <x:c r="V42" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging
+AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. The fallacy here is Cherry picking: someone selects only the evidence that supports a conclusion and ignores a wider body of evidence that weakens, qualifies, or reverses it. That matters here because cherry picking can involve hand-picked dates, unusual baselines, isolated anecdotes, or a single study taken out of a larger research picture. A better analysis would remember that the defect is not using examples, but using a biased sample as if it were representative.
+Source: Associated Press | 2024-05-18
+https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="W42" t="str">
-        <x:v>AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. — Associated Press | New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens | 2024-11-14 | https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
+        <x:v>New Pentagon report on UFOs includes hundreds of new incidents but no evidence of aliens
+AP's November 14, 2024 story on hundreds of new UAP reports is a useful case because it mixes explained incidents, unexplained incidents, and limited data without pretending they all support the same conclusion. It is exactly the kind of evidence landscape that invites cherry-picking and premature certainty. The fallacy here is Cherry picking: someone selects only the evidence that supports a conclusion and ignores a wider body of evidence that weakens, qualifies, or reverses it. That matters here because cherry picking can involve hand-picked dates, unusual baselines, isolated anecdotes, or a single study taken out of a larger research picture. A better analysis would remember that the defect is not using examples, but using a biased sample as if it were representative.
+Source: Associated Press | 2024-11-14
+https://apnews.com/article/5638be273b753253713a478546849e46</x:v>
       </x:c>
       <x:c r="X42" t="str">
-        <x:v>PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. — PolitiFact | Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town | 2024-09-09 | https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
+        <x:v>Authorities rebut claims that Haitian immigrants are eating cats, waterfowl in Ohio town
+PolitiFact's September 9, 2024 Springfield fact check is a neat example of a rumor built out of anonymous posts, recycled images, and suggestive repetition rather than verifiable support. It shows how easily a story can feel established before it has actually been checked. The fallacy here is Cherry picking: someone selects only the evidence that supports a conclusion and ignores a wider body of evidence that weakens, qualifies, or reverses it. That matters here because cherry picking can involve hand-picked dates, unusual baselines, isolated anecdotes, or a single study taken out of a larger research picture. A better analysis would remember that the defect is not using examples, but using a biased sample as if it were representative.
+Source: PolitiFact | 2024-09-09
+https://www.politifact.com/factchecks/2024/sep/09/social-media/authorities-rebut-claims-that-haitian-immigrants-a/</x:v>
       </x:c>
       <x:c r="Y42" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate
+AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. The fallacy here is Cherry picking: someone selects only the evidence that supports a conclusion and ignores a wider body of evidence that weakens, qualifies, or reverses it. That matters here because cherry picking can involve hand-picked dates, unusual baselines, isolated anecdotes, or a single study taken out of a larger research picture. A better analysis would remember that the defect is not using examples, but using a biased sample as if it were representative.
+Source: Associated Press | 2024-06-27
+https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="Z42" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+        <x:v>Survivorship bias
+Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. The fallacy here is Cherry picking: someone selects only the evidence that supports a conclusion and ignores a wider body of evidence that weakens, qualifies, or reverses it. That matters here because cherry picking can involve hand-picked dates, unusual baselines, isolated anecdotes, or a single study taken out of a larger research picture. A better analysis would remember that the defect is not using examples, but using a biased sample as if it were representative.
+Source: Britannica | 2026-01-01
+https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
       <x:c r="AA42" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -3383,13 +3569,16 @@
         <x:v>Older views can be wrong, but age alone neither refutes nor confirms them. The real question is whether the reasoning survives scrutiny.</x:v>
       </x:c>
       <x:c r="V43" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent
+AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. The fallacy here is Chronological snobbery: an idea is dismissed mainly because it is old, premodern, or associated with a period that also held many false beliefs. That matters here because older views can be wrong, but age alone neither refutes nor confirms them. A better analysis would remember that the real question is whether the reasoning survives scrutiny.
+Source: Associated Press | 2024-02-17
+https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="W43" t="str">
-        <x:v>Social-media arguments often dismiss older religious, philosophical, or literary texts as worthless simply because they come from a less enlightened era, skipping the actual argument.</x:v>
+        <x:v>Social-media arguments often dismiss older religious, philosophical, or literary texts as worthless simply because they come from a less enlightened era, skipping the actual argument. The fallacy here is Chronological snobbery: an idea is dismissed mainly because it is old, premodern, or associated with a period that also held many false beliefs. That matters here because older views can be wrong, but age alone neither refutes nor confirms them. A better analysis would remember that the real question is whether the reasoning survives scrutiny.</x:v>
       </x:c>
       <x:c r="X43" t="str">
-        <x:v>People also dismiss pre-digital scholarship wholesale as outdated while still relying on concepts, institutions, and moral categories that earlier thinkers helped shape.</x:v>
+        <x:v>People also dismiss pre-digital scholarship wholesale as outdated while still relying on concepts, institutions, and moral categories that earlier thinkers helped shape. The fallacy here is Chronological snobbery: an idea is dismissed mainly because it is old, premodern, or associated with a period that also held many false beliefs. That matters here because older views can be wrong, but age alone neither refutes nor confirms them. A better analysis would remember that the real question is whether the reasoning survives scrutiny.</x:v>
       </x:c>
       <x:c r="Y43" t="str"/>
       <x:c r="Z43" t="str"/>
@@ -3456,10 +3645,10 @@
         <x:v>Circular dynamics can be real, but identifying a loop does not show that the loop is unstoppable or that breaking one link would guarantee the hoped-for outcome. Further evidence is still needed.</x:v>
       </x:c>
       <x:c r="V44" t="str">
-        <x:v>Job markets sometimes create genuine experience loops, but it is still a mistake to assume that every applicant locked out by the loop would necessarily succeed if only one employer made an exception.</x:v>
+        <x:v>Job markets sometimes create genuine experience loops, but it is still a mistake to assume that every applicant locked out by the loop would necessarily succeed if only one employer made an exception. The fallacy here is Circular cause and consequence: a feedback loop is treated as if it fully explains, proves, or justifies a result, even though the loop may be contingent, breakable, or not sufficient for the claimed conclusion. That matters here because circular dynamics can be real, but identifying a loop does not show that the loop is unstoppable or that breaking one link would guarantee the hoped-for outcome. A better analysis would remember that further evidence is still needed.</x:v>
       </x:c>
       <x:c r="W44" t="str">
-        <x:v>Commentators often say a platform is influential because everyone talks about it and everyone talks about it because it is influential, using the loop itself as if it settled the argument.</x:v>
+        <x:v>Commentators often say a platform is influential because everyone talks about it and everyone talks about it because it is influential, using the loop itself as if it settled the argument. The fallacy here is Circular cause and consequence: a feedback loop is treated as if it fully explains, proves, or justifies a result, even though the loop may be contingent, breakable, or not sufficient for the claimed conclusion. That matters here because circular dynamics can be real, but identifying a loop does not show that the loop is unstoppable or that breaking one link would guarantee the hoped-for outcome. A better analysis would remember that further evidence is still needed.</x:v>
       </x:c>
       <x:c r="X44" t="str"/>
       <x:c r="Y44" t="str"/>
@@ -3527,10 +3716,10 @@
         <x:v>Parts can interact in ways that change the result at the larger scale. What is beneficial, efficient, or true locally may not stay that way globally.</x:v>
       </x:c>
       <x:c r="V45" t="str">
-        <x:v>A company may assume that because every team is cutting costs responsibly, the organization as a whole will thrive, even though simultaneous cuts can gut the shared systems the teams depend on.</x:v>
+        <x:v>A company may assume that because every team is cutting costs responsibly, the organization as a whole will thrive, even though simultaneous cuts can gut the shared systems the teams depend on. The fallacy here is Composition fallacy: something true of the parts is assumed to be true of the whole they compose. That matters here because parts can interact in ways that change the result at the larger scale. A better analysis would remember that what is beneficial, efficient, or true locally may not stay that way globally.</x:v>
       </x:c>
       <x:c r="W45" t="str">
-        <x:v>In policy debates, people often assume that what is prudent for one household, firm, or voter must be prudent for the entire economy or democracy at once.</x:v>
+        <x:v>In policy debates, people often assume that what is prudent for one household, firm, or voter must be prudent for the entire economy or democracy at once. The fallacy here is Composition fallacy: something true of the parts is assumed to be true of the whole they compose. That matters here because parts can interact in ways that change the result at the larger scale. A better analysis would remember that what is beneficial, efficient, or true locally may not stay that way globally.</x:v>
       </x:c>
       <x:c r="X45" t="str"/>
       <x:c r="Y45" t="str"/>
@@ -3594,16 +3783,22 @@
         <x:v>Confidence can track expertise, but it can also track charisma, identity, adrenaline, fear, or repeated exposure to a claim. Certainty is a psychological state, not a built-in proof.</x:v>
       </x:c>
       <x:c r="V46" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+        <x:v>Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist
+In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. The fallacy here is Confidence as a validator: a speaker's certainty, intensity, or felt conviction is treated as if it were evidence that the claim is true. That matters here because confidence can track expertise, but it can also track charisma, identity, adrenaline, fear, or repeated exposure to a claim. A better analysis would remember that certainty is a psychological state, not a built-in proof.
+Source: Associated Press | 2024-05-06
+https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="W46" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said
+AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. The fallacy here is Confidence as a validator: a speaker's certainty, intensity, or felt conviction is treated as if it were evidence that the claim is true. That matters here because confidence can track expertise, but it can also track charisma, identity, adrenaline, fear, or repeated exposure to a claim. A better analysis would remember that certainty is a psychological state, not a built-in proof.
+Source: Associated Press | 2024-10-26
+https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="X46" t="str">
-        <x:v>The anonymous ABC debate affidavit spread partly because influential accounts amplified it with extraordinary certainty before any reliable verification had appeared.</x:v>
+        <x:v>The anonymous ABC debate affidavit spread partly because influential accounts amplified it with extraordinary certainty before any reliable verification had appeared. The fallacy here is Confidence as a validator: a speaker's certainty, intensity, or felt conviction is treated as if it were evidence that the claim is true. That matters here because confidence can track expertise, but it can also track charisma, identity, adrenaline, fear, or repeated exposure to a claim. A better analysis would remember that certainty is a psychological state, not a built-in proof.</x:v>
       </x:c>
       <x:c r="Y46" t="str">
-        <x:v>In arguments about AI consciousness, election fraud, religion, and wellness, people often present their felt certainty as if it were itself a kind of evidence rather than something that also needs checking.</x:v>
+        <x:v>In arguments about AI consciousness, election fraud, religion, and wellness, people often present their felt certainty as if it were itself a kind of evidence rather than something that also needs checking. The fallacy here is Confidence as a validator: a speaker's certainty, intensity, or felt conviction is treated as if it were evidence that the claim is true. That matters here because confidence can track expertise, but it can also track charisma, identity, adrenaline, fear, or repeated exposure to a claim. A better analysis would remember that certainty is a psychological state, not a built-in proof.</x:v>
       </x:c>
       <x:c r="Z46" t="str"/>
       <x:c r="AA46" t="str">
@@ -3667,10 +3862,10 @@
         <x:v>Adding conditions never makes a claim more probable than a broader version of that same claim. Extra detail can make a story feel more representative while making it statistically less likely.</x:v>
       </x:c>
       <x:c r="V47" t="str">
-        <x:v>Political profiling often mistakes a vivid stereotype for probability, assuming that a person matching one trait is more likely to match an even narrower bundle of traits as well.</x:v>
+        <x:v>Political profiling often mistakes a vivid stereotype for probability, assuming that a person matching one trait is more likely to match an even narrower bundle of traits as well. The fallacy here is Conjunction fallacy: a more detailed scenario is treated as more probable than a less detailed scenario that already contains it. That matters here because adding conditions never makes a claim more probable than a broader version of that same claim. A better analysis would remember that extra detail can make a story feel more representative while making it statistically less likely.</x:v>
       </x:c>
       <x:c r="W47" t="str">
-        <x:v>AI narratives sometimes suggest that because a model appears articulate, it is more likely to be both highly capable and aligned than merely capable, even though the conjunction is narrower.</x:v>
+        <x:v>AI narratives sometimes suggest that because a model appears articulate, it is more likely to be both highly capable and aligned than merely capable, even though the conjunction is narrower. The fallacy here is Conjunction fallacy: a more detailed scenario is treated as more probable than a less detailed scenario that already contains it. That matters here because adding conditions never makes a claim more probable than a broader version of that same claim. A better analysis would remember that extra detail can make a story feel more representative while making it statistically less likely.</x:v>
       </x:c>
       <x:c r="X47" t="str"/>
       <x:c r="Y47" t="str"/>
@@ -3740,16 +3935,22 @@
         <x:v>Shortening a quote is not automatically deceptive. The fallacy appears when the omitted context would materially change how a fair reader understands the statement.</x:v>
       </x:c>
       <x:c r="V48" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent
+AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. The fallacy here is Contextomy: words are selectively excerpted from their original context in a way that changes or distorts what the speaker meant. That matters here because shortening a quote is not automatically deceptive. That is the exact slip in this case: the omitted context would materially change how a fair reader understands the statement.
+Source: Associated Press | 2024-02-17
+https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="W48" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+        <x:v>Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement
+AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. The fallacy here is Contextomy: words are selectively excerpted from their original context in a way that changes or distorts what the speaker meant. That matters here because shortening a quote is not automatically deceptive. That is the exact slip in this case: the omitted context would materially change how a fair reader understands the statement.
+Source: Associated Press | 2024-09-10
+https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="X48" t="str">
-        <x:v>Edited debate clips, viral subtitled videos, and quote-card politics in 2024 regularly removed the surrounding setup, qualifier, or punchline that made the original meaning very different.</x:v>
+        <x:v>Edited debate clips, viral subtitled videos, and quote-card politics in 2024 regularly removed the surrounding setup, qualifier, or punchline that made the original meaning very different. The fallacy here is Contextomy: words are selectively excerpted from their original context in a way that changes or distorts what the speaker meant. That matters here because shortening a quote is not automatically deceptive. That is the exact slip in this case: the omitted context would materially change how a fair reader understands the statement.</x:v>
       </x:c>
       <x:c r="Y48" t="str">
-        <x:v>Public figures and partisans often quote one alarming sentence from a report, study, or speech while cutting the lines that immediately limit, explain, or even reverse the apparent claim.</x:v>
+        <x:v>Public figures and partisans often quote one alarming sentence from a report, study, or speech while cutting the lines that immediately limit, explain, or even reverse the apparent claim. The fallacy here is Contextomy: words are selectively excerpted from their original context in a way that changes or distorts what the speaker meant. That matters here because shortening a quote is not automatically deceptive. That is the exact slip in this case: the omitted context would materially change how a fair reader understands the statement.</x:v>
       </x:c>
       <x:c r="Z48" t="str"/>
       <x:c r="AA48" t="str">
@@ -3815,10 +4016,10 @@
         <x:v>Many real concepts come in degrees. Vagueness at the boundary does not make the broader concept meaningless or unusable.</x:v>
       </x:c>
       <x:c r="V49" t="str">
-        <x:v>Arguments about misinformation, bias, wealth, addiction, and consciousness often demand an impossible razor-sharp line and then pretend the lack of that line defeats the concept altogether.</x:v>
+        <x:v>Arguments about misinformation, bias, wealth, addiction, and consciousness often demand an impossible razor-sharp line and then pretend the lack of that line defeats the concept altogether. The fallacy here is Continuum fallacy: a claim is rejected simply because the concept involved has blurry boundaries rather than a perfectly sharp cutoff. That matters here because many real concepts come in degrees. A better analysis would remember that vagueness at the boundary does not make the broader concept meaningless or unusable.</x:v>
       </x:c>
       <x:c r="W49" t="str">
-        <x:v>In everyday disputes, someone may deny that a delay was 'too long' or a fee was 'too high' simply because no exact threshold was announced in advance.</x:v>
+        <x:v>In everyday disputes, someone may deny that a delay was 'too long' or a fee was 'too high' simply because no exact threshold was announced in advance. The fallacy here is Continuum fallacy: a claim is rejected simply because the concept involved has blurry boundaries rather than a perfectly sharp cutoff. That matters here because many real concepts come in degrees. A better analysis would remember that vagueness at the boundary does not make the broader concept meaningless or unusable.</x:v>
       </x:c>
       <x:c r="X49" t="str"/>
       <x:c r="Y49" t="str"/>
@@ -3884,19 +4085,31 @@
         <x:v>Correlations matter because they can reveal patterns worth investigating. The fallacy is jumping straight from 'these moved together' to 'this caused that' without checking mechanisms, timing, controls, or alternative explanations.</x:v>
       </x:c>
       <x:c r="V50" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging
+AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. The fallacy here is Correlation is not causation: someone treats a correlation, coincidence, or time pattern as if it already established that one factor caused the other. That matters here because correlations matter because they can reveal patterns worth investigating. A better analysis would remember that the fallacy is jumping straight from 'these moved together' to 'this caused that' without checking mechanisms, timing, controls, or alternative explanations.
+Source: Associated Press | 2024-05-18
+https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="W50" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not
+NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. The fallacy here is Correlation is not causation: someone treats a correlation, coincidence, or time pattern as if it already established that one factor caused the other. That matters here because correlations matter because they can reveal patterns worth investigating. A better analysis would remember that the fallacy is jumping straight from 'these moved together' to 'this caused that' without checking mechanisms, timing, controls, or alternative explanations.
+Source: NPR | 2024-10-12
+https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="X50" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate
+AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. The fallacy here is Correlation is not causation: someone treats a correlation, coincidence, or time pattern as if it already established that one factor caused the other. That matters here because correlations matter because they can reveal patterns worth investigating. A better analysis would remember that the fallacy is jumping straight from 'these moved together' to 'this caused that' without checking mechanisms, timing, controls, or alternative explanations.
+Source: Associated Press | 2024-06-27
+https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="Y50" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+        <x:v>AI seen cutting worker numbers, survey by staffing company Adecco shows
+Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. The fallacy here is Correlation is not causation: someone treats a correlation, coincidence, or time pattern as if it already established that one factor caused the other. That matters here because correlations matter because they can reveal patterns worth investigating. A better analysis would remember that the fallacy is jumping straight from 'these moved together' to 'this caused that' without checking mechanisms, timing, controls, or alternative explanations.
+Source: Reuters | 2024-04-05
+https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="Z50" t="str">
-        <x:v>Claims about teen mental health and social media often move too quickly from parallel trend lines to a settled single-cause story, even though researchers still debate the size, direction, and mechanisms of the effect.</x:v>
+        <x:v>Claims about teen mental health and social media often move too quickly from parallel trend lines to a settled single-cause story, even though researchers still debate the size, direction, and mechanisms of the effect. The fallacy here is Correlation is not causation: someone treats a correlation, coincidence, or time pattern as if it already established that one factor caused the other. That matters here because correlations matter because they can reveal patterns worth investigating. A better analysis would remember that the fallacy is jumping straight from 'these moved together' to 'this caused that' without checking mechanisms, timing, controls, or alternative explanations.</x:v>
       </x:c>
       <x:c r="AA50" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -3959,13 +4172,16 @@
         <x:v>Definitions can clarify usage, but they do not settle the underlying issue by fiat. Rewording a problem is not the same as answering it.</x:v>
       </x:c>
       <x:c r="V51" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent
+AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. The fallacy here is Definist fallacy: a substantive question is illegitimately 'solved' by defining one contested concept into another. That matters here because definitions can clarify usage, but they do not settle the underlying issue by fiat. A better analysis would remember that rewording a problem is not the same as answering it.
+Source: Associated Press | 2024-02-17
+https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="W51" t="str">
-        <x:v>Culture-war debates often define words like 'freedom,' 'woman,' 'democracy,' or 'terrorism' in ways that quietly smuggle the desired conclusion into the starting point.</x:v>
+        <x:v>Culture-war debates often define words like 'freedom,' 'woman,' 'democracy,' or 'terrorism' in ways that quietly smuggle the desired conclusion into the starting point. The fallacy here is Definist fallacy: a substantive question is illegitimately 'solved' by defining one contested concept into another. That matters here because definitions can clarify usage, but they do not settle the underlying issue by fiat. A better analysis would remember that rewording a problem is not the same as answering it.</x:v>
       </x:c>
       <x:c r="X51" t="str">
-        <x:v>Moral and political disputes frequently collapse into dictionary wars where one side pretends that owning the label settles the argument.</x:v>
+        <x:v>Moral and political disputes frequently collapse into dictionary wars where one side pretends that owning the label settles the argument. The fallacy here is Definist fallacy: a substantive question is illegitimately 'solved' by defining one contested concept into another. That matters here because definitions can clarify usage, but they do not settle the underlying issue by fiat. A better analysis would remember that rewording a problem is not the same as answering it.</x:v>
       </x:c>
       <x:c r="Y51" t="str"/>
       <x:c r="Z51" t="str"/>
@@ -4024,16 +4240,22 @@
         <x:v>Mechanisms matter, but evidence can justify belief before the full causal story is finished. Observation often outruns explanation.</x:v>
       </x:c>
       <x:c r="V52" t="str">
-        <x:v>AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. — Associated Press | Pentagon study finds no sign of alien life in reported UFO sightings going back decades | 2024-03-08 | https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
+        <x:v>Pentagon study finds no sign of alien life in reported UFO sightings going back decades
+AP's March 8, 2024 report on the Pentagon's UFO review is a textbook reminder that 'not fully explained' does not mean 'therefore alien' or 'therefore conspiracy.' The remaining uncertainty in the file is exactly what makes the episode useful for thinking about overconfident belief formation. The fallacy here is Demanding a mechanism: strong evidence for a phenomenon is rejected solely because the underlying mechanism is still incomplete, disputed, or not yet fully understood. That matters here because mechanisms matter, but evidence can justify belief before the full causal story is finished. A better analysis would remember that observation often outruns explanation.
+Source: Associated Press | 2024-03-08
+https://apnews.com/article/9a32aba88eb610cf16b2e9f0908704b3</x:v>
       </x:c>
       <x:c r="W52" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. — FactCheck.org | Q&amp;A on H5N1 Bird Flu | 2024-05-04 | https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
+        <x:v>Q&amp;A on H5N1 Bird Flu
+FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people need mechanisms, prevalence, and scope before drawing practical conclusions from a scary headline. It helps distinguish real uncertainty from reasoning that jumps too fast from fragments of evidence to a preferred story. The fallacy here is Demanding a mechanism: strong evidence for a phenomenon is rejected solely because the underlying mechanism is still incomplete, disputed, or not yet fully understood. That matters here because mechanisms matter, but evidence can justify belief before the full causal story is finished. A better analysis would remember that observation often outruns explanation.
+Source: FactCheck.org | 2024-05-04
+https://www.factcheck.org/2024/05/qa-on-h5n1-bird-flu/</x:v>
       </x:c>
       <x:c r="X52" t="str">
-        <x:v>Public disputes about climate, evolution, and health regularly treat unresolved details in the mechanism as if they erased the larger evidential picture.</x:v>
+        <x:v>Public disputes about climate, evolution, and health regularly treat unresolved details in the mechanism as if they erased the larger evidential picture. The fallacy here is Demanding a mechanism: strong evidence for a phenomenon is rejected solely because the underlying mechanism is still incomplete, disputed, or not yet fully understood. That matters here because mechanisms matter, but evidence can justify belief before the full causal story is finished. A better analysis would remember that observation often outruns explanation.</x:v>
       </x:c>
       <x:c r="Y52" t="str">
-        <x:v>Research on AI transcription errors in 2024 showed that systems were inventing statements people never said; even before every technical cause was nailed down, the pattern itself was already evidence of a real reliability problem.</x:v>
+        <x:v>Research on AI transcription errors in 2024 showed that systems were inventing statements people never said; even before every technical cause was nailed down, the pattern itself was already evidence of a real reliability problem. The fallacy here is Demanding a mechanism: strong evidence for a phenomenon is rejected solely because the underlying mechanism is still incomplete, disputed, or not yet fully understood. That matters here because mechanisms matter, but evidence can justify belief before the full causal story is finished. A better analysis would remember that observation often outruns explanation.</x:v>
       </x:c>
       <x:c r="Z52" t="str"/>
       <x:c r="AA52" t="str">
@@ -4099,13 +4321,16 @@
         <x:v>Sometimes counterevidence matters, but the default burden still sits with the person making the substantive claim. Lack of disproof is not the same as proof.</x:v>
       </x:c>
       <x:c r="V53" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. The fallacy here is Demanding negative proof: someone tries to protect a claim by insisting that critics must prove the claim false instead of the claimant first supplying adequate support. That matters here because sometimes counterevidence matters, but the default burden still sits with the person making the substantive claim. A better analysis would remember that lack of disproof is not the same as proof.
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="W53" t="str">
-        <x:v>Conspiracy claims about noncitizen voting, ballot destruction, or machine tampering often survive by demanding that every rumor be individually disproved rather than by presenting strong evidence that the conspiracy exists.</x:v>
+        <x:v>Conspiracy claims about noncitizen voting, ballot destruction, or machine tampering often survive by demanding that every rumor be individually disproved rather than by presenting strong evidence that the conspiracy exists. The fallacy here is Demanding negative proof: someone tries to protect a claim by insisting that critics must prove the claim false instead of the claimant first supplying adequate support. That matters here because sometimes counterevidence matters, but the default burden still sits with the person making the substantive claim. A better analysis would remember that lack of disproof is not the same as proof.</x:v>
       </x:c>
       <x:c r="X53" t="str">
-        <x:v>Miracle, UFO, and paranormal arguments frequently say skeptics must show exactly what happened in each case, as though the claimant had no burden until that impossible task is finished.</x:v>
+        <x:v>Miracle, UFO, and paranormal arguments frequently say skeptics must show exactly what happened in each case, as though the claimant had no burden until that impossible task is finished. The fallacy here is Demanding negative proof: someone tries to protect a claim by insisting that critics must prove the claim false instead of the claimant first supplying adequate support. That matters here because sometimes counterevidence matters, but the default burden still sits with the person making the substantive claim. A better analysis would remember that lack of disproof is not the same as proof.</x:v>
       </x:c>
       <x:c r="Y53" t="str"/>
       <x:c r="Z53" t="str"/>
@@ -4166,10 +4391,10 @@
         <x:v>Responsible belief often comes in degrees. Treating confidence as all-or-nothing hides uncertainty, nuance, and the actual strength of the evidence.</x:v>
       </x:c>
       <x:c r="V54" t="str">
-        <x:v>Debates about God, UFOs, AI consciousness, and election fraud often demand yes-or-no declarations even when the intellectually honest position is conditional, partial, or still under revision.</x:v>
+        <x:v>Debates about God, UFOs, AI consciousness, and election fraud often demand yes-or-no declarations even when the intellectually honest position is conditional, partial, or still under revision. The fallacy here is Denial of the epistemic gradient: belief is forced into crude either-or boxes even though the evidence supports a range of confidence levels rather than a single sharp threshold. That matters here because responsible belief often comes in degrees. A better analysis would remember that treating confidence as all-or-nothing hides uncertainty, nuance, and the actual strength of the evidence.</x:v>
       </x:c>
       <x:c r="W54" t="str">
-        <x:v>Culture-war exchanges frequently treat probabilistic language such as 'unlikely,' 'not yet shown,' or 'some evidence but not enough' as weakness rather than as proper calibration.</x:v>
+        <x:v>Culture-war exchanges frequently treat probabilistic language such as 'unlikely,' 'not yet shown,' or 'some evidence but not enough' as weakness rather than as proper calibration. The fallacy here is Denial of the epistemic gradient: belief is forced into crude either-or boxes even though the evidence supports a range of confidence levels rather than a single sharp threshold. That matters here because responsible belief often comes in degrees. A better analysis would remember that treating confidence as all-or-nothing hides uncertainty, nuance, and the actual strength of the evidence.</x:v>
       </x:c>
       <x:c r="X54" t="str"/>
       <x:c r="Y54" t="str"/>
@@ -4231,10 +4456,10 @@
         <x:v>A remote hypothetical can still be useful when the issue is whether a rule really holds without exception. Improbable cases often expose hidden limits in principles that sounded absolute.</x:v>
       </x:c>
       <x:c r="V55" t="str">
-        <x:v>Arguments about free speech, self-defense, abortion, lying, and triage often reject hard edge cases simply because they are uncomfortable, even though those cases are precisely what test universal rules.</x:v>
+        <x:v>Arguments about free speech, self-defense, abortion, lying, and triage often reject hard edge cases simply because they are uncomfortable, even though those cases are precisely what test universal rules. The fallacy here is Denying a remote hypothetical: a hypothetical test case is dismissed as irrelevant merely because it is rare, extreme, or unlikely, even though the principle under debate is supposed to be universal. That matters here because a remote hypothetical can still be useful when the issue is whether a rule really holds without exception. A better analysis would remember that improbable cases often expose hidden limits in principles that sounded absolute.</x:v>
       </x:c>
       <x:c r="W55" t="str">
-        <x:v>Policy debates about AI safety and biosecurity sometimes wave away low-probability scenarios too quickly, even when the whole argument concerns whether a system is robust under stress.</x:v>
+        <x:v>Policy debates about AI safety and biosecurity sometimes wave away low-probability scenarios too quickly, even when the whole argument concerns whether a system is robust under stress. The fallacy here is Denying a remote hypothetical: a hypothetical test case is dismissed as irrelevant merely because it is rare, extreme, or unlikely, even though the principle under debate is supposed to be universal. That matters here because a remote hypothetical can still be useful when the issue is whether a rule really holds without exception. A better analysis would remember that improbable cases often expose hidden limits in principles that sounded absolute.</x:v>
       </x:c>
       <x:c r="X55" t="str"/>
       <x:c r="Y55" t="str"/>
@@ -4300,16 +4525,22 @@
         <x:v>One route to a conclusion does not have to be the only route. The absence of one sufficient condition does not automatically remove every other possible basis.</x:v>
       </x:c>
       <x:c r="V56" t="str">
-        <x:v>PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's ABC-affidavit reconstruction is also a nice formal-inference case: because Trump was fact-checked more often, some commentators inferred that Harris must have received the questions in advance. Even if the premise were granted, the conclusion still did not logically follow. The fallacy here is Denying the antecedent: someone reasons from 'if A, then B' and then wrongly infers 'not B' merely because A is absent. That matters here because one route to a conclusion does not have to be the only route. A better analysis would remember that the absence of one sufficient condition does not automatically remove every other possible basis.
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="W56" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. The fallacy here is Denying the antecedent: someone reasons from 'if A, then B' and then wrongly infers 'not B' merely because A is absent. That matters here because one route to a conclusion does not have to be the only route. A better analysis would remember that the absence of one sufficient condition does not automatically remove every other possible basis.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="X56" t="str">
-        <x:v>Debates about expertise often assume that if a source lacks one credential or prestige marker, there can be no meaningful evidence at all in what it says.</x:v>
+        <x:v>Debates about expertise often assume that if a source lacks one credential or prestige marker, there can be no meaningful evidence at all in what it says. The fallacy here is Denying the antecedent: someone reasons from 'if A, then B' and then wrongly infers 'not B' merely because A is absent. That matters here because one route to a conclusion does not have to be the only route. A better analysis would remember that the absence of one sufficient condition does not automatically remove every other possible basis.</x:v>
       </x:c>
       <x:c r="Y56" t="str">
-        <x:v>In everyday arguments, people often assume that if the ideal cause is absent, the observed effect cannot still arise through another path.</x:v>
+        <x:v>In everyday arguments, people often assume that if the ideal cause is absent, the observed effect cannot still arise through another path. The fallacy here is Denying the antecedent: someone reasons from 'if A, then B' and then wrongly infers 'not B' merely because A is absent. That matters here because one route to a conclusion does not have to be the only route. A better analysis would remember that the absence of one sufficient condition does not automatically remove every other possible basis.</x:v>
       </x:c>
       <x:c r="Z56" t="str"/>
       <x:c r="AA56" t="str">
@@ -4373,10 +4604,10 @@
         <x:v>Some concepts only make sense against their correlative opposite. Erasing the contrast does not answer the accusation; it changes the meaning of the term.</x:v>
       </x:c>
       <x:c r="V57" t="str">
-        <x:v>Public arguments sometimes say a decision cannot count as censorship unless it was total state control, effectively denying any middle range where the term usefully applies.</x:v>
+        <x:v>Public arguments sometimes say a decision cannot count as censorship unless it was total state control, effectively denying any middle range where the term usefully applies. The fallacy here is Denying the correlative: one side of a genuine contrast is denied or redefined so the opposing term has no place to apply. That matters here because some concepts only make sense against their correlative opposite. A better analysis would remember that erasing the contrast does not answer the accusation; it changes the meaning of the term.</x:v>
       </x:c>
       <x:c r="W57" t="str">
-        <x:v>Debates about betrayal, fraud, or coercion often narrow the term so drastically that almost no real case can qualify.</x:v>
+        <x:v>Debates about betrayal, fraud, or coercion often narrow the term so drastically that almost no real case can qualify. The fallacy here is Denying the correlative: one side of a genuine contrast is denied or redefined so the opposing term has no place to apply. That matters here because some concepts only make sense against their correlative opposite. A better analysis would remember that erasing the contrast does not answer the accusation; it changes the meaning of the term.</x:v>
       </x:c>
       <x:c r="X57" t="str"/>
       <x:c r="Y57" t="str"/>
@@ -4444,10 +4675,10 @@
         <x:v>A whole can have properties its parts do not share equally. Group-level success, size, reputation, or wealth does not automatically distribute itself down to each component.</x:v>
       </x:c>
       <x:c r="V58" t="str">
-        <x:v>People often infer that because a country is rich, any given citizen must be comfortable, skipping inequality, regional gaps, and individual circumstance.</x:v>
+        <x:v>People often infer that because a country is rich, any given citizen must be comfortable, skipping inequality, regional gaps, and individual circumstance. The fallacy here is Division fallacy: something true of a whole is assumed to be true of each part or member of that whole. That matters here because a whole can have properties its parts do not share equally. A better analysis would remember that group-level success, size, reputation, or wealth does not automatically distribute itself down to each component.</x:v>
       </x:c>
       <x:c r="W58" t="str">
-        <x:v>A popular movement, successful company, or prestigious institution can still contain weak teams, poor ideas, or underfunded units.</x:v>
+        <x:v>A popular movement, successful company, or prestigious institution can still contain weak teams, poor ideas, or underfunded units. The fallacy here is Division fallacy: something true of a whole is assumed to be true of each part or member of that whole. That matters here because a whole can have properties its parts do not share equally. A better analysis would remember that group-level success, size, reputation, or wealth does not automatically distribute itself down to each component.</x:v>
       </x:c>
       <x:c r="X58" t="str"/>
       <x:c r="Y58" t="str"/>
@@ -4517,10 +4748,10 @@
         <x:v>Aggregate data can be useful, but it does not tell you where any one individual falls within the distribution. Group averages do not erase overlap, variation, or outliers.</x:v>
       </x:c>
       <x:c r="V59" t="str">
-        <x:v>Zip-code analytics, polling blocs, and demographic summaries are often treated as if they gave a direct reading of the motives or traits of each person inside the category.</x:v>
+        <x:v>Zip-code analytics, polling blocs, and demographic summaries are often treated as if they gave a direct reading of the motives or traits of each person inside the category. The fallacy here is Ecological fallacy: statistics about a group are used to draw conclusions about particular individuals in that group. That matters here because aggregate data can be useful, but it does not tell you where any one individual falls within the distribution. A better analysis would remember that group averages do not erase overlap, variation, or outliers.</x:v>
       </x:c>
       <x:c r="W59" t="str">
-        <x:v>Political commentary frequently talks as if 'suburban women,' 'young men,' or 'college voters' were internally uniform rather than broad, heterogeneous groups.</x:v>
+        <x:v>Political commentary frequently talks as if 'suburban women,' 'young men,' or 'college voters' were internally uniform rather than broad, heterogeneous groups. The fallacy here is Ecological fallacy: statistics about a group are used to draw conclusions about particular individuals in that group. That matters here because aggregate data can be useful, but it does not tell you where any one individual falls within the distribution. A better analysis would remember that group averages do not erase overlap, variation, or outliers.</x:v>
       </x:c>
       <x:c r="X59" t="str"/>
       <x:c r="Y59" t="str"/>
@@ -4580,10 +4811,10 @@
         <x:v>Not every conversation requires a full essay, but a real refutation still has to point to some error in reasoning, evidence, or interpretation. Mere dismissal is not argument.</x:v>
       </x:c>
       <x:c r="V60" t="str">
-        <x:v>Online fights about elections, Israel and Gaza, climate, and AI often rely on 'debunked' as a performance word rather than as a pointer to the actual evidence.</x:v>
+        <x:v>Online fights about elections, Israel and Gaza, climate, and AI often rely on 'debunked' as a performance word rather than as a pointer to the actual evidence. The fallacy here is Empty refutation: someone declares an argument false, debunked, or dishonest without identifying the specific flaw that would actually show it is false. That matters here because not every conversation requires a full essay, but a real refutation still has to point to some error in reasoning, evidence, or interpretation. A better analysis would remember that mere dismissal is not argument.</x:v>
       </x:c>
       <x:c r="W60" t="str">
-        <x:v>In fast-moving social media disputes, people often treat tone, certainty, and pile-on consensus as if they were enough to count as refutation.</x:v>
+        <x:v>In fast-moving social media disputes, people often treat tone, certainty, and pile-on consensus as if they were enough to count as refutation. The fallacy here is Empty refutation: someone declares an argument false, debunked, or dishonest without identifying the specific flaw that would actually show it is false. That matters here because not every conversation requires a full essay, but a real refutation still has to point to some error in reasoning, evidence, or interpretation. A better analysis would remember that mere dismissal is not argument.</x:v>
       </x:c>
       <x:c r="X60" t="str"/>
       <x:c r="Y60" t="str"/>
@@ -4647,10 +4878,10 @@
         <x:v>Beliefs can change mood, confidence, behavior, pain perception, and group cohesion regardless of whether their object exists. The benefits of belief do not by themselves settle the ontology.</x:v>
       </x:c>
       <x:c r="V61" t="str">
-        <x:v>Raw milk, supplement, and alternative-health advocates often point to the felt benefits reported by believers while skipping the role of expectation, placebo effects, and other background changes.</x:v>
+        <x:v>Raw milk, supplement, and alternative-health advocates often point to the felt benefits reported by believers while skipping the role of expectation, placebo effects, and other background changes. The fallacy here is Epistemic/ontological conflation: the psychological or social effects of believing something are treated as evidence that the thing believed in actually exists or is true. That matters here because beliefs can change mood, confidence, behavior, pain perception, and group cohesion regardless of whether their object exists. A better analysis would remember that the benefits of belief do not by themselves settle the ontology.</x:v>
       </x:c>
       <x:c r="W61" t="str">
-        <x:v>Arguments that religion must be true because believers report comfort, purpose, or improved well-being often confuse the power of belief with evidence for the reality of the object believed in.</x:v>
+        <x:v>Arguments that religion must be true because believers report comfort, purpose, or improved well-being often confuse the power of belief with evidence for the reality of the object believed in. The fallacy here is Epistemic/ontological conflation: the psychological or social effects of believing something are treated as evidence that the thing believed in actually exists or is true. That matters here because beliefs can change mood, confidence, behavior, pain perception, and group cohesion regardless of whether their object exists. A better analysis would remember that the benefits of belief do not by themselves settle the ontology.</x:v>
       </x:c>
       <x:c r="X61" t="str"/>
       <x:c r="Y61" t="str"/>
@@ -4714,16 +4945,22 @@
         <x:v>Equivocation often works because the same word is doing two jobs at once. The surface grammar stays stable while the meaning shifts underneath.</x:v>
       </x:c>
       <x:c r="V62" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Google makes fixes to AI-generated search summaries after outlandish answers went viral
+When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. The fallacy here is Equivocation: a key word or phrase slides between different meanings inside the same argument, creating the illusion of support. That matters here because equivocation often works because the same word is doing two jobs at once. A better analysis would remember that the surface grammar stays stable while the meaning shifts underneath.
+Source: Associated Press | 2024-05-31
+https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="W62" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent
+AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. The fallacy here is Equivocation: a key word or phrase slides between different meanings inside the same argument, creating the illusion of support. That matters here because equivocation often works because the same word is doing two jobs at once. A better analysis would remember that the surface grammar stays stable while the meaning shifts underneath.
+Source: Associated Press | 2024-02-17
+https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="X62" t="str">
-        <x:v>Debates over content moderation regularly equivocate between censorship by the state and moderation decisions by private platforms, as if both were the same kind of speech restriction.</x:v>
+        <x:v>Debates over content moderation regularly equivocate between censorship by the state and moderation decisions by private platforms, as if both were the same kind of speech restriction. The fallacy here is Equivocation: a key word or phrase slides between different meanings inside the same argument, creating the illusion of support. That matters here because equivocation often works because the same word is doing two jobs at once. A better analysis would remember that the surface grammar stays stable while the meaning shifts underneath.</x:v>
       </x:c>
       <x:c r="Y62" t="str">
-        <x:v>Public discussion of AI often slides between thin technical meanings of words such as 'reasoning,' 'understanding,' or 'hallucination' and thicker human meanings, which makes claims sound stronger than the evidence warrants.</x:v>
+        <x:v>Public discussion of AI often slides between thin technical meanings of words such as 'reasoning,' 'understanding,' or 'hallucination' and thicker human meanings, which makes claims sound stronger than the evidence warrants. The fallacy here is Equivocation: a key word or phrase slides between different meanings inside the same argument, creating the illusion of support. That matters here because equivocation often works because the same word is doing two jobs at once. A better analysis would remember that the surface grammar stays stable while the meaning shifts underneath.</x:v>
       </x:c>
       <x:c r="Z62" t="str"/>
       <x:c r="AA62" t="str">
@@ -4785,10 +5022,10 @@
         <x:v>The argument trades on the prestige or emotional force of the stronger meaning while relying on the thinner meaning when challenged.</x:v>
       </x:c>
       <x:c r="V63" t="str">
-        <x:v>Public arguments about censorship often slide from the general fact that content was moderated to the much stronger charge that it was censored in the same sense as state suppression.</x:v>
+        <x:v>Public arguments about censorship often slide from the general fact that content was moderated to the much stronger charge that it was censored in the same sense as state suppression. The fallacy here is Equivocation fallacy: a broad or harmless sense of a word is used to insinuate a narrower, stronger, or more loaded sense of the same word. That matters here because the argument trades on the prestige or emotional force of the stronger meaning while relying on the thinner meaning when challenged. The better question is whether the key term keeps the same meaning from one step of the argument to the next.</x:v>
       </x:c>
       <x:c r="W63" t="str">
-        <x:v>AI marketing repeatedly benefits from equivocation between technical terms such as 'learn,' 'reason,' or 'understand' and their thicker human meanings.</x:v>
+        <x:v>AI marketing repeatedly benefits from equivocation between technical terms such as 'learn,' 'reason,' or 'understand' and their thicker human meanings. The fallacy here is Equivocation fallacy: a broad or harmless sense of a word is used to insinuate a narrower, stronger, or more loaded sense of the same word. That matters here because the argument trades on the prestige or emotional force of the stronger meaning while relying on the thinner meaning when challenged. The better question is whether the key term keeps the same meaning from one step of the argument to the next.</x:v>
       </x:c>
       <x:c r="X63" t="str"/>
       <x:c r="Y63" t="str"/>
@@ -4852,10 +5089,10 @@
         <x:v>Words change through use. Present meaning is set by current linguistic convention, not by the oldest recoverable ancestor of the term.</x:v>
       </x:c>
       <x:c r="V64" t="str">
-        <x:v>Culture-war and identity debates often turn into fights over what labels 'really mean' based on older usage rather than on how the community currently uses them.</x:v>
+        <x:v>Culture-war and identity debates often turn into fights over what labels 'really mean' based on older usage rather than on how the community currently uses them. The fallacy here is Etymological fallacy: a word's original or historical meaning is treated as if it controlled the word's present meaning. That matters here because words change through use. A better analysis would remember that present meaning is set by current linguistic convention, not by the oldest recoverable ancestor of the term.</x:v>
       </x:c>
       <x:c r="W64" t="str">
-        <x:v>People sometimes defend or condemn a term by appealing to its root language while ignoring the fact that social meaning has moved far beyond the origin.</x:v>
+        <x:v>People sometimes defend or condemn a term by appealing to its root language while ignoring the fact that social meaning has moved far beyond the origin. The fallacy here is Etymological fallacy: a word's original or historical meaning is treated as if it controlled the word's present meaning. That matters here because words change through use. A better analysis would remember that present meaning is set by current linguistic convention, not by the oldest recoverable ancestor of the term.</x:v>
       </x:c>
       <x:c r="X64" t="str"/>
       <x:c r="Y64" t="str"/>
@@ -4919,13 +5156,16 @@
         <x:v>Two exclusions do not by themselves tell you how the remaining categories relate. Keeping groups apart is not the same as establishing a valid connection among them.</x:v>
       </x:c>
       <x:c r="V65" t="str">
-        <x:v>The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+The raw-milk and bird-flu stories from AP and FactCheck make another formal lesson plain: even if some processed products are risky or some official guidance has changed over time, it does not follow that unpasteurized milk is therefore safer. The inference trades on contrast, not valid implication. The fallacy here is Exclusive premises: two negative premises are used in a syllogism even though they fail to establish the positive link the conclusion requires. That matters here because two exclusions do not by themselves tell you how the remaining categories relate. A better analysis would remember that keeping groups apart is not the same as establishing a valid connection among them.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="W65" t="str">
-        <x:v>Identity arguments sometimes pile up statements about what two groups are not and then pretend that the missing positive relation has somehow been proved.</x:v>
+        <x:v>Identity arguments sometimes pile up statements about what two groups are not and then pretend that the missing positive relation has somehow been proved. The fallacy here is Exclusive premises: two negative premises are used in a syllogism even though they fail to establish the positive link the conclusion requires. That matters here because two exclusions do not by themselves tell you how the remaining categories relate. A better analysis would remember that keeping groups apart is not the same as establishing a valid connection among them.</x:v>
       </x:c>
       <x:c r="X65" t="str">
-        <x:v>This form often hides inside rhetorical contrasts where speakers rely on the sound of elimination rather than a genuine logical bridge.</x:v>
+        <x:v>This form often hides inside rhetorical contrasts where speakers rely on the sound of elimination rather than a genuine logical bridge. The fallacy here is Exclusive premises: two negative premises are used in a syllogism even though they fail to establish the positive link the conclusion requires. That matters here because two exclusions do not by themselves tell you how the remaining categories relate. A better analysis would remember that keeping groups apart is not the same as establishing a valid connection among them.</x:v>
       </x:c>
       <x:c r="Y65" t="str"/>
       <x:c r="Z65" t="str"/>
@@ -4988,13 +5228,16 @@
         <x:v>Universal statements can be true even when the class is empty. Talking about all members of a category does not guarantee that there are any members to begin with.</x:v>
       </x:c>
       <x:c r="V66" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not
+AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. The fallacy here is Existential fallacy: a conclusion assumes that something exists even though the premises never established that any such thing exists. That matters here because universal statements can be true even when the class is empty. A better analysis would remember that talking about all members of a category does not guarantee that there are any members to begin with.
+Source: NPR | 2024-10-12
+https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="W66" t="str">
-        <x:v>Arguments about 'the average user,' 'the typical elite,' or 'the real moderate voter' sometimes slip from a hypothetical category into the assumption that a concrete instance must exist.</x:v>
+        <x:v>Arguments about 'the average user,' 'the typical elite,' or 'the real moderate voter' sometimes slip from a hypothetical category into the assumption that a concrete instance must exist. The fallacy here is Existential fallacy: a conclusion assumes that something exists even though the premises never established that any such thing exists. That matters here because universal statements can be true even when the class is empty. A better analysis would remember that talking about all members of a category does not guarantee that there are any members to begin with.</x:v>
       </x:c>
       <x:c r="X66" t="str">
-        <x:v>Formal and theological debates alike often move too quickly from what would be true if something existed to the claim that it therefore does exist.</x:v>
+        <x:v>Formal and theological debates alike often move too quickly from what would be true if something existed to the claim that it therefore does exist. The fallacy here is Existential fallacy: a conclusion assumes that something exists even though the premises never established that any such thing exists. That matters here because universal statements can be true even when the class is empty. A better analysis would remember that talking about all members of a category does not guarantee that there are any members to begin with.</x:v>
       </x:c>
       <x:c r="Y66" t="str"/>
       <x:c r="Z66" t="str"/>
@@ -5059,10 +5302,10 @@
         <x:v>A loaded question can force a false choice because any direct answer seems to concede what the question improperly assumed. The first task is often to challenge the hidden premise, not to answer on its terms.</x:v>
       </x:c>
       <x:c r="V67" t="str">
-        <x:v>Debates about religion, politics, and gender often turn on questions that quietly presuppose bad faith, delusion, or malicious intent before any of that has been shown.</x:v>
+        <x:v>Debates about religion, politics, and gender often turn on questions that quietly presuppose bad faith, delusion, or malicious intent before any of that has been shown. The fallacy here is Fallacy of many questions: a question smuggles in one or more assumptions that have not been established, then pressures the listener to answer as if those assumptions were already settled. That matters here because a loaded question can force a false choice because any direct answer seems to concede what the question improperly assumed. A better analysis would remember that the first task is often to challenge the hidden premise, not to answer on its terms.</x:v>
       </x:c>
       <x:c r="W67" t="str">
-        <x:v>Interviewers and posters sometimes frame questions so that merely engaging already concedes the accusation, especially in culture-war exchanges built for clipping and outrage.</x:v>
+        <x:v>Interviewers and posters sometimes frame questions so that merely engaging already concedes the accusation, especially in culture-war exchanges built for clipping and outrage. The fallacy here is Fallacy of many questions: a question smuggles in one or more assumptions that have not been established, then pressures the listener to answer as if those assumptions were already settled. That matters here because a loaded question can force a false choice because any direct answer seems to concede what the question improperly assumed. A better analysis would remember that the first task is often to challenge the hidden premise, not to answer on its terms.</x:v>
       </x:c>
       <x:c r="X67" t="str"/>
       <x:c r="Y67" t="str"/>
@@ -5128,10 +5371,10 @@
         <x:v>Some predicates are necessary only relative to a present state or definition. That necessity does not magically extend across time, possibility, or changed conditions.</x:v>
       </x:c>
       <x:c r="V68" t="str">
-        <x:v>People sometimes move from 'this rule currently defines the category' to 'therefore the category could never be revised or altered,' confusing present convention with fixed necessity.</x:v>
+        <x:v>People sometimes move from 'this rule currently defines the category' to 'therefore the category could never be revised or altered,' confusing present convention with fixed necessity. The fallacy here is Fallacy of necessity: a condition that is necessary given someone's current description is treated as if it were permanently or universally necessary in the real world. That matters here because some predicates are necessary only relative to a present state or definition. A better analysis would remember that that necessity does not magically extend across time, possibility, or changed conditions.</x:v>
       </x:c>
       <x:c r="W68" t="str">
-        <x:v>In institutional debates, a temporary legal or procedural status is often spoken of as if it were an immutable fact about what can never happen.</x:v>
+        <x:v>In institutional debates, a temporary legal or procedural status is often spoken of as if it were an immutable fact about what can never happen. The fallacy here is Fallacy of necessity: a condition that is necessary given someone's current description is treated as if it were permanently or universally necessary in the real world. That matters here because some predicates are necessary only relative to a present state or definition. A better analysis would remember that that necessity does not magically extend across time, possibility, or changed conditions.</x:v>
       </x:c>
       <x:c r="X68" t="str"/>
       <x:c r="Y68" t="str"/>
@@ -5197,10 +5440,10 @@
         <x:v>Analogies can clarify unfamiliar ideas, but they prove very little unless the shared features are actually relevant to the conclusion being drawn.</x:v>
       </x:c>
       <x:c r="V69" t="str">
-        <x:v>Debates about AI frequently compare models to children, interns, parrots, or brains, then carry over conclusions from the analogy that the underlying system may not support.</x:v>
+        <x:v>Debates about AI frequently compare models to children, interns, parrots, or brains, then carry over conclusions from the analogy that the underlying system may not support. The fallacy here is False analogy: one thing is treated as sufficiently like another even though the comparison breaks down at the point the argument depends on. That matters here because analogies can clarify unfamiliar ideas, but they prove very little unless the shared features are actually relevant to the conclusion being drawn. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W69" t="str">
-        <x:v>Fiscal debates often compare a national budget to a household budget; the analogy can illuminate some constraints but breaks down when it is treated as a full map of macroeconomics.</x:v>
+        <x:v>Fiscal debates often compare a national budget to a household budget; the analogy can illuminate some constraints but breaks down when it is treated as a full map of macroeconomics. The fallacy here is False analogy: one thing is treated as sufficiently like another even though the comparison breaks down at the point the argument depends on. That matters here because analogies can clarify unfamiliar ideas, but they prove very little unless the shared features are actually relevant to the conclusion being drawn. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X69" t="str"/>
       <x:c r="Y69" t="str"/>
@@ -5266,19 +5509,28 @@
         <x:v>Source quality matters, but only if the source is real, relevant, and represented fairly. A false attribution can make weak claims feel borrowed from a stronger authority than they actually have.</x:v>
       </x:c>
       <x:c r="V70" t="str">
-        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+        <x:v>To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery
+AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. The fallacy here is False attribution: support for a claim is borrowed from a source that is fabricated, misquoted, unqualified, anonymous in the wrong way, or otherwise not what it is presented to be. That matters here because source quality matters, but only if the source is real, relevant, and represented fairly. A better analysis would remember that a false attribution can make weak claims feel borrowed from a stronger authority than they actually have.
+Source: Associated Press | 2023-11-08
+https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
       </x:c>
       <x:c r="W70" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Google makes fixes to AI-generated search summaries after outlandish answers went viral
+When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. The fallacy here is False attribution: support for a claim is borrowed from a source that is fabricated, misquoted, unqualified, anonymous in the wrong way, or otherwise not what it is presented to be. That matters here because source quality matters, but only if the source is real, relevant, and represented fairly. A better analysis would remember that a false attribution can make weak claims feel borrowed from a stronger authority than they actually have.
+Source: Associated Press | 2024-05-31
+https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="X70" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said
+AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. The fallacy here is False attribution: support for a claim is borrowed from a source that is fabricated, misquoted, unqualified, anonymous in the wrong way, or otherwise not what it is presented to be. That matters here because source quality matters, but only if the source is real, relevant, and represented fairly. A better analysis would remember that a false attribution can make weak claims feel borrowed from a stronger authority than they actually have.
+Source: Associated Press | 2024-10-26
+https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="Y70" t="str">
-        <x:v>The anonymous affidavit circulated after the September 2024 ABC debate was amplified as if it were a verified insider source even though the core allegations were not authenticated.</x:v>
+        <x:v>The anonymous affidavit circulated after the September 2024 ABC debate was amplified as if it were a verified insider source even though the core allegations were not authenticated. The fallacy here is False attribution: support for a claim is borrowed from a source that is fabricated, misquoted, unqualified, anonymous in the wrong way, or otherwise not what it is presented to be. That matters here because source quality matters, but only if the source is real, relevant, and represented fairly. A better analysis would remember that a false attribution can make weak claims feel borrowed from a stronger authority than they actually have.</x:v>
       </x:c>
       <x:c r="Z70" t="str">
-        <x:v>Viral quote cards and screenshot posts often attach dramatic claims to scientists, judges, or agencies who never said them, counting on readers to trust the label instead of checking the source.</x:v>
+        <x:v>Viral quote cards and screenshot posts often attach dramatic claims to scientists, judges, or agencies who never said them, counting on readers to trust the label instead of checking the source. The fallacy here is False attribution: support for a claim is borrowed from a source that is fabricated, misquoted, unqualified, anonymous in the wrong way, or otherwise not what it is presented to be. That matters here because source quality matters, but only if the source is real, relevant, and represented fairly. A better analysis would remember that a false attribution can make weak claims feel borrowed from a stronger authority than they actually have.</x:v>
       </x:c>
       <x:c r="AA70" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -5341,19 +5593,28 @@
         <x:v>Fairness does not always require symmetry. When one side is supported by overwhelming evidence and the other is weak, fringe, or fabricated, equal presentation can mislead an audience about the actual state of the issue.</x:v>
       </x:c>
       <x:c r="V71" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+        <x:v>Iowa finds several dozen instances of noncitizens voting in a past election
+AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. The fallacy here is False balance: a dispute is presented as if the competing sides were roughly equal in credibility or evidential support even though the evidence is not remotely balanced. That matters here because fairness does not always require symmetry. A better analysis would remember that when one side is supported by overwhelming evidence and the other is weak, fringe, or fabricated, equal presentation can mislead an audience about the actual state of the issue.
+Source: Associated Press | 2024-10-23
+https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
       <x:c r="W71" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>AP Explains: Migration is more complex than politics show
+AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. The fallacy here is False balance: a dispute is presented as if the competing sides were roughly equal in credibility or evidential support even though the evidence is not remotely balanced. That matters here because fairness does not always require symmetry. A better analysis would remember that when one side is supported by overwhelming evidence and the other is weak, fringe, or fabricated, equal presentation can mislead an audience about the actual state of the issue.
+Source: Associated Press | 2024-09-20
+https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="X71" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+        <x:v>Why AP called the Arizona Senate race for Ruben Gallego
+AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. The fallacy here is False balance: a dispute is presented as if the competing sides were roughly equal in credibility or evidential support even though the evidence is not remotely balanced. That matters here because fairness does not always require symmetry. A better analysis would remember that when one side is supported by overwhelming evidence and the other is weak, fringe, or fabricated, equal presentation can mislead an audience about the actual state of the issue.
+Source: Associated Press | 2024-11-12
+https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
       </x:c>
       <x:c r="Y71" t="str">
-        <x:v>Coverage of climate change, vaccine safety, and election administration often becomes misleading when fringe claims are presented as if they stand on equal footing with the evidential consensus.</x:v>
+        <x:v>Coverage of climate change, vaccine safety, and election administration often becomes misleading when fringe claims are presented as if they stand on equal footing with the evidential consensus. The fallacy here is False balance: a dispute is presented as if the competing sides were roughly equal in credibility or evidential support even though the evidence is not remotely balanced. That matters here because fairness does not always require symmetry. A better analysis would remember that when one side is supported by overwhelming evidence and the other is weak, fringe, or fabricated, equal presentation can mislead an audience about the actual state of the issue.</x:v>
       </x:c>
       <x:c r="Z71" t="str">
-        <x:v>Public moderators sometimes treat a polished unsupported claim and a well-supported cautious claim as equivalent contributions simply because both parties are speaking confidently.</x:v>
+        <x:v>Public moderators sometimes treat a polished unsupported claim and a well-supported cautious claim as equivalent contributions simply because both parties are speaking confidently. The fallacy here is False balance: a dispute is presented as if the competing sides were roughly equal in credibility or evidential support even though the evidence is not remotely balanced. That matters here because fairness does not always require symmetry. A better analysis would remember that when one side is supported by overwhelming evidence and the other is weak, fringe, or fabricated, equal presentation can mislead an audience about the actual state of the issue.</x:v>
       </x:c>
       <x:c r="AA71" t="str">
         <x:v>added-2026-completeness-pass</x:v>
@@ -5416,13 +5677,16 @@
         <x:v>Disagreement does not imply that the truth is halfway between the parties. One side may simply be much more right than the other.</x:v>
       </x:c>
       <x:c r="V72" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>Analysis-US port strike throws spotlight on big union foe: automation
+Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. The fallacy here is False compromise: the midpoint between two positions is treated as correct simply because it lies between them. That matters here because disagreement does not imply that the truth is halfway between the parties. A better analysis would remember that one side may simply be much more right than the other.
+Source: Reuters | 2024-10-04
+https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="W72" t="str">
-        <x:v>Coverage of climate, public health, and election integrity can slide into 'both sides' framing that treats consensus and fringe denial as if splitting the difference were balanced or fair.</x:v>
+        <x:v>Coverage of climate, public health, and election integrity can slide into 'both sides' framing that treats consensus and fringe denial as if splitting the difference were balanced or fair. The fallacy here is False compromise: the midpoint between two positions is treated as correct simply because it lies between them. That matters here because disagreement does not imply that the truth is halfway between the parties. A better analysis would remember that one side may simply be much more right than the other.</x:v>
       </x:c>
       <x:c r="X72" t="str">
-        <x:v>In personal and workplace disputes, people often assume each side must be equally at fault, even when the evidence is lopsided.</x:v>
+        <x:v>In personal and workplace disputes, people often assume each side must be equally at fault, even when the evidence is lopsided. The fallacy here is False compromise: the midpoint between two positions is treated as correct simply because it lies between them. That matters here because disagreement does not imply that the truth is halfway between the parties. A better analysis would remember that one side may simply be much more right than the other.</x:v>
       </x:c>
       <x:c r="Y72" t="str"/>
       <x:c r="Z72" t="str"/>
@@ -5487,19 +5751,34 @@
         <x:v>The pressure comes from pretending that a complex decision has only two doors. Sometimes the omitted alternatives are compromises, phased approaches, or the option of rejecting the framing altogether.</x:v>
       </x:c>
       <x:c r="V73" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging
+AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. The fallacy here is False dilemma: someone presents a limited set of options as if they were the only live possibilities, while reasonable alternatives are ignored or suppressed. That matters here because the pressure comes from pretending that a complex decision has only two doors. A better analysis would remember that sometimes the omitted alternatives are compromises, phased approaches, or the option of rejecting the framing altogether.
+Source: Associated Press | 2024-05-18
+https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="W73" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+        <x:v>Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement
+AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. The fallacy here is False dilemma: someone presents a limited set of options as if they were the only live possibilities, while reasonable alternatives are ignored or suppressed. That matters here because the pressure comes from pretending that a complex decision has only two doors. A better analysis would remember that sometimes the omitted alternatives are compromises, phased approaches, or the option of rejecting the framing altogether.
+Source: Associated Press | 2024-09-10
+https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="X73" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate
+AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. The fallacy here is False dilemma: someone presents a limited set of options as if they were the only live possibilities, while reasonable alternatives are ignored or suppressed. That matters here because the pressure comes from pretending that a complex decision has only two doors. A better analysis would remember that sometimes the omitted alternatives are compromises, phased approaches, or the option of rejecting the framing altogether.
+Source: Associated Press | 2024-06-27
+https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="Y73" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>AP Explains: Migration is more complex than politics show
+AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. The fallacy here is False dilemma: someone presents a limited set of options as if they were the only live possibilities, while reasonable alternatives are ignored or suppressed. That matters here because the pressure comes from pretending that a complex decision has only two doors. A better analysis would remember that sometimes the omitted alternatives are compromises, phased approaches, or the option of rejecting the framing altogether.
+Source: Associated Press | 2024-09-20
+https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="Z73" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>Analysis-US port strike throws spotlight on big union foe: automation
+Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. The fallacy here is False dilemma: someone presents a limited set of options as if they were the only live possibilities, while reasonable alternatives are ignored or suppressed. That matters here because the pressure comes from pretending that a complex decision has only two doors. A better analysis would remember that sometimes the omitted alternatives are compromises, phased approaches, or the option of rejecting the framing altogether.
+Source: Reuters | 2024-10-04
+https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="AA73" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -5562,19 +5841,34 @@
         <x:v>Two things can share some features without being equal in scale, intent, risk, or moral significance. The fallacy appears when a superficial resemblance is used to flatten those differences into sameness.</x:v>
       </x:c>
       <x:c r="V74" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging
+AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. The fallacy here is False equivalence: two things are treated as equivalent in seriousness, meaning, or explanatory weight despite relevant differences that make the comparison misleading. That matters here because two things can share some features without being equal in scale, intent, risk, or moral significance. That is the exact slip in this case: a superficial resemblance is used to flatten those differences into sameness.
+Source: Associated Press | 2024-05-18
+https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="W74" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not
+NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. The fallacy here is False equivalence: two things are treated as equivalent in seriousness, meaning, or explanatory weight despite relevant differences that make the comparison misleading. That matters here because two things can share some features without being equal in scale, intent, risk, or moral significance. That is the exact slip in this case: a superficial resemblance is used to flatten those differences into sameness.
+Source: NPR | 2024-10-12
+https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="X74" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+        <x:v>Iowa finds several dozen instances of noncitizens voting in a past election
+AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. The fallacy here is False equivalence: two things are treated as equivalent in seriousness, meaning, or explanatory weight despite relevant differences that make the comparison misleading. That matters here because two things can share some features without being equal in scale, intent, risk, or moral significance. That is the exact slip in this case: a superficial resemblance is used to flatten those differences into sameness.
+Source: Associated Press | 2024-10-23
+https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
       <x:c r="Y74" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent
+AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. The fallacy here is False equivalence: two things are treated as equivalent in seriousness, meaning, or explanatory weight despite relevant differences that make the comparison misleading. That matters here because two things can share some features without being equal in scale, intent, risk, or moral significance. That is the exact slip in this case: a superficial resemblance is used to flatten those differences into sameness.
+Source: Associated Press | 2024-02-17
+https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="Z74" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. The fallacy here is False equivalence: two things are treated as equivalent in seriousness, meaning, or explanatory weight despite relevant differences that make the comparison misleading. That matters here because two things can share some features without being equal in scale, intent, risk, or moral significance. That is the exact slip in this case: a superficial resemblance is used to flatten those differences into sameness.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="AA74" t="str">
         <x:v>added-2026-completeness-pass</x:v>
@@ -5641,10 +5935,10 @@
         <x:v>Real uncertainty exists, and sometimes compromise is appropriate. The fallacy appears when manufactured neutrality is used to protect a losing claim from the consequences of the evidence.</x:v>
       </x:c>
       <x:c r="V75" t="str">
-        <x:v>Public arguments about evolution, election claims, and medical misinformation sometimes ask audiences to treat both sides as equally plausible even after the evidential balance is lopsided.</x:v>
+        <x:v>Public arguments about evolution, election claims, and medical misinformation sometimes ask audiences to treat both sides as equally plausible even after the evidential balance is lopsided. The fallacy here is False surrender: someone calls for a truce, balance, or 'agree to disagree' posture not because the evidence is genuinely inconclusive, but because their position is under pressure and they want to freeze the score. That matters here because real uncertainty exists, and sometimes compromise is appropriate. That is the exact slip in this case: manufactured neutrality is used to protect a losing claim from the consequences of the evidence.</x:v>
       </x:c>
       <x:c r="W75" t="str">
-        <x:v>In online debate culture, a retreat into 'everyone has their own truth' often appears right after a concrete factual claim has gone badly for one side.</x:v>
+        <x:v>In online debate culture, a retreat into 'everyone has their own truth' often appears right after a concrete factual claim has gone badly for one side. The fallacy here is False surrender: someone calls for a truce, balance, or 'agree to disagree' posture not because the evidence is genuinely inconclusive, but because their position is under pressure and they want to freeze the score. That matters here because real uncertainty exists, and sometimes compromise is appropriate. That is the exact slip in this case: manufactured neutrality is used to protect a losing claim from the consequences of the evidence.</x:v>
       </x:c>
       <x:c r="X75" t="str"/>
       <x:c r="Y75" t="str"/>
@@ -5712,19 +6006,28 @@
         <x:v>Generalization is unavoidable, but it has to be scaled to the quality, size, and representativeness of the evidence. The problem is not generalizing at all; it is generalizing too aggressively.</x:v>
       </x:c>
       <x:c r="V76" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not
+NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. The fallacy here is Faulty generalization: an inductive conclusion reaches further than the available evidence can reasonably support, or ignores information that should limit the generalization. That matters here because generalization is unavoidable, but it has to be scaled to the quality, size, and representativeness of the evidence. A better analysis would remember that the problem is not generalizing at all; it is generalizing too aggressively.
+Source: NPR | 2024-10-12
+https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="W76" t="str">
-        <x:v>AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. — Associated Press | Iowa finds several dozen instances of noncitizens voting in a past election | 2024-10-23 | https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
+        <x:v>Iowa finds several dozen instances of noncitizens voting in a past election
+AP's coverage of Iowa finding dozens of noncitizen votes is useful precisely because it reports real violations without letting the count float free of scale. The story helps show the difference between acknowledging a genuine problem and inflating it into a sweeping narrative. The fallacy here is Faulty generalization: an inductive conclusion reaches further than the available evidence can reasonably support, or ignores information that should limit the generalization. That matters here because generalization is unavoidable, but it has to be scaled to the quality, size, and representativeness of the evidence. A better analysis would remember that the problem is not generalizing at all; it is generalizing too aggressively.
+Source: Associated Press | 2024-10-23
+https://apnews.com/article/622235f2771a372801a5e3c4d1a86343</x:v>
       </x:c>
       <x:c r="X76" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+        <x:v>Survivorship bias
+Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. The fallacy here is Faulty generalization: an inductive conclusion reaches further than the available evidence can reasonably support, or ignores information that should limit the generalization. That matters here because generalization is unavoidable, but it has to be scaled to the quality, size, and representativeness of the evidence. A better analysis would remember that the problem is not generalizing at all; it is generalizing too aggressively.
+Source: Britannica | 2026-01-01
+https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
       <x:c r="Y76" t="str">
-        <x:v>Viral anecdotes about migrants, students, police, or AI tools often get inflated into sweeping claims about entire groups or systems after only a handful of cases.</x:v>
+        <x:v>Viral anecdotes about migrants, students, police, or AI tools often get inflated into sweeping claims about entire groups or systems after only a handful of cases. The fallacy here is Faulty generalization: an inductive conclusion reaches further than the available evidence can reasonably support, or ignores information that should limit the generalization. That matters here because generalization is unavoidable, but it has to be scaled to the quality, size, and representativeness of the evidence. A better analysis would remember that the problem is not generalizing at all; it is generalizing too aggressively.</x:v>
       </x:c>
       <x:c r="Z76" t="str">
-        <x:v>Election and media arguments routinely take one error, one clip, or one scandal as proof that the whole institution always behaves the same way.</x:v>
+        <x:v>Election and media arguments routinely take one error, one clip, or one scandal as proof that the whole institution always behaves the same way. The fallacy here is Faulty generalization: an inductive conclusion reaches further than the available evidence can reasonably support, or ignores information that should limit the generalization. That matters here because generalization is unavoidable, but it has to be scaled to the quality, size, and representativeness of the evidence. A better analysis would remember that the problem is not generalizing at all; it is generalizing too aggressively.</x:v>
       </x:c>
       <x:c r="AA76" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -5783,10 +6086,10 @@
         <x:v>Reasoning from an assumption to test its implications is not the same as endorsing the assumption.</x:v>
       </x:c>
       <x:c r="V77" t="str">
-        <x:v>Reductio arguments in theology, AI, and politics are often misread as confessions rather than as tests of what would follow if the other side's claim were granted.</x:v>
+        <x:v>Reductio arguments in theology, AI, and politics are often misread as confessions rather than as tests of what would follow if the other side's claim were granted. The fallacy here is For the sake of argument denial: a hypothetical premise is rejected simply because the speaker does not actually believe it. That matters here because reasoning from an assumption to test its implications is not the same as endorsing the assumption. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W77" t="str">
-        <x:v>Debates stall when a conditional claim such as 'even if you are right, the consequence would still be unacceptable' is treated as if it were a statement of belief.</x:v>
+        <x:v>Debates stall when a conditional claim such as 'even if you are right, the consequence would still be unacceptable' is treated as if it were a statement of belief. The fallacy here is For the sake of argument denial: a hypothetical premise is rejected simply because the speaker does not actually believe it. That matters here because reasoning from an assumption to test its implications is not the same as endorsing the assumption. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X77" t="str"/>
       <x:c r="Y77" t="str"/>
@@ -5850,10 +6153,10 @@
         <x:v>The surface wording can make the argument sound tidy, but the hidden term shift breaks the structure. A reused word is not enough; it has to keep the same meaning.</x:v>
       </x:c>
       <x:c r="V78" t="str">
-        <x:v>Public arguments often slide between technical and ordinary meanings of words like 'theory,' 'freedom,' 'bias,' or 'intelligence,' then pretend the resulting syllogism is valid.</x:v>
+        <x:v>Public arguments often slide between technical and ordinary meanings of words like 'theory,' 'freedom,' 'bias,' or 'intelligence,' then pretend the resulting syllogism is valid. The fallacy here is Four terms fallacy: a syllogism seems to use three terms but actually uses four because one term shifts meaning halfway through the argument. That matters here because the surface wording can make the argument sound tidy, but the hidden term shift breaks the structure. A better analysis would remember that a reused word is not enough; it has to keep the same meaning.</x:v>
       </x:c>
       <x:c r="W78" t="str">
-        <x:v>Because the same label can carry prestige in one context and a thinner meaning in another, term shifts often smuggle in conclusions the premises did not support.</x:v>
+        <x:v>Because the same label can carry prestige in one context and a thinner meaning in another, term shifts often smuggle in conclusions the premises did not support. The fallacy here is Four terms fallacy: a syllogism seems to use three terms but actually uses four because one term shifts meaning halfway through the argument. That matters here because the surface wording can make the argument sound tidy, but the hidden term shift breaks the structure. A better analysis would remember that a reused word is not enough; it has to keep the same meaning.</x:v>
       </x:c>
       <x:c r="X78" t="str"/>
       <x:c r="Y78" t="str"/>
@@ -5921,10 +6224,10 @@
         <x:v>Random sequences naturally contain streaks. When the events are truly independent, the next event does not remember the last one.</x:v>
       </x:c>
       <x:c r="V79" t="str">
-        <x:v>People sometimes feel that after many routine flights or medical screenings in a row, a disaster or diagnosis is somehow 'due,' even though independent risks do not balance themselves that way.</x:v>
+        <x:v>People sometimes feel that after many routine flights or medical screenings in a row, a disaster or diagnosis is somehow 'due,' even though independent risks do not balance themselves that way. The fallacy here is Gambler's fallacy: someone thinks past outcomes of independent events make a future independent outcome more or less likely than it really is. That matters here because random sequences naturally contain streaks. A better analysis would remember that when the events are truly independent, the next event does not remember the last one.</x:v>
       </x:c>
       <x:c r="W79" t="str">
-        <x:v>In gambling and investing language, talk of a roulette table or slot machine being 'ready to pay out' often confuses a streaky pattern with a real shift in odds.</x:v>
+        <x:v>In gambling and investing language, talk of a roulette table or slot machine being 'ready to pay out' often confuses a streaky pattern with a real shift in odds. The fallacy here is Gambler's fallacy: someone thinks past outcomes of independent events make a future independent outcome more or less likely than it really is. That matters here because random sequences naturally contain streaks. A better analysis would remember that when the events are truly independent, the next event does not remember the last one.</x:v>
       </x:c>
       <x:c r="X79" t="str"/>
       <x:c r="Y79" t="str"/>
@@ -5992,10 +6295,10 @@
         <x:v>Origins can matter when they reveal bias, incentives, or reliability concerns. The fallacy appears when origin is treated as enough to settle the issue without examining the claim itself.</x:v>
       </x:c>
       <x:c r="V80" t="str">
-        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported.</x:v>
+        <x:v>People often dismiss an idea because it came from Silicon Valley, academia, Fox, MSNBC, Reddit, or X without asking whether the specific claim is supported. The fallacy here is Genetic fallacy: a claim, practice, or idea is judged mainly by its origin rather than by its present content, evidence, or merits. That matters here because origins can matter when they reveal bias, incentives, or reliability concerns. That is the exact slip in this case: origin is treated as enough to settle the issue without examining the claim itself.</x:v>
       </x:c>
       <x:c r="W80" t="str">
-        <x:v>In cultural and religious arguments, a practice or symbol is often condemned solely because of its historical roots, even when the live question is what it means or does now.</x:v>
+        <x:v>In cultural and religious arguments, a practice or symbol is often condemned solely because of its historical roots, even when the live question is what it means or does now. The fallacy here is Genetic fallacy: a claim, practice, or idea is judged mainly by its origin rather than by its present content, evidence, or merits. That matters here because origins can matter when they reveal bias, incentives, or reliability concerns. That is the exact slip in this case: origin is treated as enough to settle the issue without examining the claim itself.</x:v>
       </x:c>
       <x:c r="X80" t="str"/>
       <x:c r="Y80" t="str"/>
@@ -6065,19 +6368,28 @@
         <x:v>The problem is not moving from sample to population; all induction does that. The problem is pretending a weak or unrepresentative sample carries more weight than it does.</x:v>
       </x:c>
       <x:c r="V81" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging
+AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. The fallacy here is Hasty generalization: someone draws a broad conclusion from too little evidence, too small a sample, or a badly skewed sample. That matters here because the problem is not moving from sample to population; all induction does that. A better analysis would remember that the problem is pretending a weak or unrepresentative sample carries more weight than it does.
+Source: Associated Press | 2024-05-18
+https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="W81" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate
+AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. The fallacy here is Hasty generalization: someone draws a broad conclusion from too little evidence, too small a sample, or a badly skewed sample. That matters here because the problem is not moving from sample to population; all induction does that. A better analysis would remember that the problem is pretending a weak or unrepresentative sample carries more weight than it does.
+Source: Associated Press | 2024-06-27
+https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="X81" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>AP Explains: Migration is more complex than politics show
+AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. The fallacy here is Hasty generalization: someone draws a broad conclusion from too little evidence, too small a sample, or a badly skewed sample. That matters here because the problem is not moving from sample to population; all induction does that. A better analysis would remember that the problem is pretending a weak or unrepresentative sample carries more weight than it does.
+Source: Associated Press | 2024-09-20
+https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="Y81" t="str">
-        <x:v>A single viral video of a fight, theft, or protest is often used online as if it reveals what a whole city, campus, or demographic group is like.</x:v>
+        <x:v>A single viral video of a fight, theft, or protest is often used online as if it reveals what a whole city, campus, or demographic group is like. The fallacy here is Hasty generalization: someone draws a broad conclusion from too little evidence, too small a sample, or a badly skewed sample. That matters here because the problem is not moving from sample to population; all induction does that. A better analysis would remember that the problem is pretending a weak or unrepresentative sample carries more weight than it does.</x:v>
       </x:c>
       <x:c r="Z81" t="str">
-        <x:v>Election commentary frequently treats one poll, one county, or one diner focus group as proof of a national shift, even when the broader polling picture is mixed.</x:v>
+        <x:v>Election commentary frequently treats one poll, one county, or one diner focus group as proof of a national shift, even when the broader polling picture is mixed. The fallacy here is Hasty generalization: someone draws a broad conclusion from too little evidence, too small a sample, or a badly skewed sample. That matters here because the problem is not moving from sample to population; all induction does that. A better analysis would remember that the problem is pretending a weak or unrepresentative sample carries more weight than it does.</x:v>
       </x:c>
       <x:c r="AA81" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -6138,10 +6450,10 @@
         <x:v>Hindsight compresses uncertainty and highlights the clues that mattered. Real historical agents were working inside a noisier, more limited information environment.</x:v>
       </x:c>
       <x:c r="V82" t="str">
-        <x:v>People often imagine they would easily have rejected past medical myths, empires, or moral blind spots, underestimating how strongly institutions and available evidence shape belief.</x:v>
+        <x:v>People often imagine they would easily have rejected past medical myths, empires, or moral blind spots, underestimating how strongly institutions and available evidence shape belief. The fallacy here is Historian's fallacy: people in the past are judged as if they had the same information, background assumptions, and hindsight available to later observers. That matters here because hindsight compresses uncertainty and highlights the clues that mattered. A better analysis would remember that real historical agents were working inside a noisier, more limited information environment.</x:v>
       </x:c>
       <x:c r="W82" t="str">
-        <x:v>Post-crisis commentary regularly rewrites messy contingencies into obvious warning signs that were supposedly plain to everyone at the time.</x:v>
+        <x:v>Post-crisis commentary regularly rewrites messy contingencies into obvious warning signs that were supposedly plain to everyone at the time. The fallacy here is Historian's fallacy: people in the past are judged as if they had the same information, background assumptions, and hindsight available to later observers. That matters here because hindsight compresses uncertainty and highlights the clues that mattered. A better analysis would remember that real historical agents were working inside a noisier, more limited information environment.</x:v>
       </x:c>
       <x:c r="X82" t="str"/>
       <x:c r="Y82" t="str"/>
@@ -6207,10 +6519,10 @@
         <x:v>If the inner observer can already do the job, the original explanatory problem just reappears one level down.</x:v>
       </x:c>
       <x:c r="V83" t="str">
-        <x:v>Popular neuroscience writing sometimes says that the brain 'decides' or a memory center 'knows' in ways that merely rename the puzzle rather than explain it.</x:v>
+        <x:v>Popular neuroscience writing sometimes says that the brain 'decides' or a memory center 'knows' in ways that merely rename the puzzle rather than explain it. The fallacy here is Homunculus fallacy: a mind-like inner observer is smuggled in to explain mind-like abilities, thereby postponing rather than solving the explanation. That matters here because if the inner observer can already do the job, the original explanatory problem just reappears one level down. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W83" t="str">
-        <x:v>Criticism of AI can do something similar when it assumes a hidden module inside the system literally understands the output in the same way a person would.</x:v>
+        <x:v>Criticism of AI can do something similar when it assumes a hidden module inside the system literally understands the output in the same way a person would. The fallacy here is Homunculus fallacy: a mind-like inner observer is smuggled in to explain mind-like abilities, thereby postponing rather than solving the explanation. That matters here because if the inner observer can already do the job, the original explanatory problem just reappears one level down. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X83" t="str"/>
       <x:c r="Y83" t="str"/>
@@ -6278,10 +6590,10 @@
         <x:v>Institutional labels can matter legally or practically, but they do not by themselves create truth, value, or natural kinds.</x:v>
       </x:c>
       <x:c r="V84" t="str">
-        <x:v>Markets and media often confuse approved, certified, or official with true, safe, or just.</x:v>
+        <x:v>Markets and media often confuse approved, certified, or official with true, safe, or just. The fallacy here is Human standard fallacy: a human classification, rule, or label is treated as if it automatically determined the underlying fact or moral status. That matters here because institutional labels can matter legally or practically, but they do not by themselves create truth, value, or natural kinds. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W84" t="str">
-        <x:v>Political rhetoric often treats whatever a legislature recognizes or forbids as automatically morally right or wrong.</x:v>
+        <x:v>Political rhetoric often treats whatever a legislature recognizes or forbids as automatically morally right or wrong. The fallacy here is Human standard fallacy: a human classification, rule, or label is treated as if it automatically determined the underlying fact or moral status. That matters here because institutional labels can matter legally or practically, but they do not by themselves create truth, value, or natural kinds. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X84" t="str"/>
       <x:c r="Y84" t="str"/>
@@ -6345,10 +6657,10 @@
         <x:v>This is not mere nuance. The problem is rhetorical double-speaking that blurs real disagreement by sliding between incompatible senses of the same label.</x:v>
       </x:c>
       <x:c r="V85" t="str">
-        <x:v>Politicians often define contested terms like 'freedom,' 'censorship,' 'riot,' 'peaceful,' or 'family values' one way for sympathetic listeners and another way when challenged by critics.</x:v>
+        <x:v>Politicians often define contested terms like 'freedom,' 'censorship,' 'riot,' 'peaceful,' or 'family values' one way for sympathetic listeners and another way when challenged by critics. The fallacy here is If-by-whiskey: someone uses strategically shifting language that seems to support both sides by quietly changing the meaning of the key term to suit the audience. That matters here because this is not mere nuance. A better analysis would remember that the problem is rhetorical double-speaking that blurs real disagreement by sliding between incompatible senses of the same label.</x:v>
       </x:c>
       <x:c r="W85" t="str">
-        <x:v>Debates about AI, speech, and policing frequently proceed as if both camps agree until someone notices that the central term has been doing two very different jobs.</x:v>
+        <x:v>Debates about AI, speech, and policing frequently proceed as if both camps agree until someone notices that the central term has been doing two very different jobs. The fallacy here is If-by-whiskey: someone uses strategically shifting language that seems to support both sides by quietly changing the meaning of the key term to suit the audience. That matters here because this is not mere nuance. A better analysis would remember that the problem is rhetorical double-speaking that blurs real disagreement by sliding between incompatible senses of the same label.</x:v>
       </x:c>
       <x:c r="X85" t="str"/>
       <x:c r="Y85" t="str"/>
@@ -6412,10 +6724,10 @@
         <x:v>Excluding one group from a subset does not exclude it from the wider property attached to that subset. The conclusion reaches further than the premises license.</x:v>
       </x:c>
       <x:c r="V86" t="str">
-        <x:v>Stereotype arguments often move from 'all members of group A have trait B' and 'group C is not group A' to 'therefore group C lacks trait B,' which does not follow.</x:v>
+        <x:v>Stereotype arguments often move from 'all members of group A have trait B' and 'group C is not group A' to 'therefore group C lacks trait B,' which does not follow. The fallacy here is Illicit major: a syllogism distributes the major term in the conclusion even though the major premise never distributed it there. That matters here because excluding one group from a subset does not exclude it from the wider property attached to that subset. A better analysis would remember that the conclusion reaches further than the premises license.</x:v>
       </x:c>
       <x:c r="W86" t="str">
-        <x:v>This pattern appears when people treat one pathway to fame, corruption, risk, or success as if it were the only pathway.</x:v>
+        <x:v>This pattern appears when people treat one pathway to fame, corruption, risk, or success as if it were the only pathway. The fallacy here is Illicit major: a syllogism distributes the major term in the conclusion even though the major premise never distributed it there. That matters here because excluding one group from a subset does not exclude it from the wider property attached to that subset. A better analysis would remember that the conclusion reaches further than the premises license.</x:v>
       </x:c>
       <x:c r="X86" t="str"/>
       <x:c r="Y86" t="str"/>
@@ -6477,10 +6789,10 @@
         <x:v>A claim that survives every observation unchanged may be emotionally resilient, but it has surrendered explanatory power.</x:v>
       </x:c>
       <x:c r="V87" t="str">
-        <x:v>Conspiracy systems often explain both the presence and the absence of evidence as confirmation.</x:v>
+        <x:v>Conspiracy systems often explain both the presence and the absence of evidence as confirmation. The fallacy here is Impotent logical space: a view is framed so every possible outcome fits it equally well, leaving no meaningful room for the claim to fail. That matters here because a claim that survives every observation unchanged may be emotionally resilient, but it has surrendered explanatory power. The better question is whether the evidence has been weighed fairly before the conclusion is accepted.</x:v>
       </x:c>
       <x:c r="W87" t="str">
-        <x:v>Some technology hype frames both success and failure as proof that general intelligence is just around the corner.</x:v>
+        <x:v>Some technology hype frames both success and failure as proof that general intelligence is just around the corner. The fallacy here is Impotent logical space: a view is framed so every possible outcome fits it equally well, leaving no meaningful room for the claim to fail. That matters here because a claim that survives every observation unchanged may be emotionally resilient, but it has surrendered explanatory power. The better question is whether the evidence has been weighed fairly before the conclusion is accepted.</x:v>
       </x:c>
       <x:c r="X87" t="str"/>
       <x:c r="Y87" t="str"/>
@@ -6544,13 +6856,16 @@
         <x:v>A comparison can be true in one narrow respect while misleading overall. The missing pieces might include quality, risk, wages, inflation, time horizon, tradeoffs, or alternative baselines.</x:v>
       </x:c>
       <x:c r="V88" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+        <x:v>Why AP called the Arizona Senate race for Ruben Gallego
+AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. The fallacy here is Incomplete comparison: one option is called better, worse, cheaper, safer, or more effective without specifying the relevant comparison class or the other factors that matter. That matters here because a comparison can be true in one narrow respect while misleading overall. A better analysis would remember that the missing pieces might include quality, risk, wages, inflation, time horizon, tradeoffs, or alternative baselines.
+Source: Associated Press | 2024-11-12
+https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
       </x:c>
       <x:c r="W88" t="str">
-        <x:v>Campaign arguments about the economy often isolate one metric such as gas prices, job totals, or stock indexes and treat that single comparison as if it captured the whole condition of household life.</x:v>
+        <x:v>Campaign arguments about the economy often isolate one metric such as gas prices, job totals, or stock indexes and treat that single comparison as if it captured the whole condition of household life. The fallacy here is Incomplete comparison: one option is called better, worse, cheaper, safer, or more effective without specifying the relevant comparison class or the other factors that matter. That matters here because a comparison can be true in one narrow respect while misleading overall. A better analysis would remember that the missing pieces might include quality, risk, wages, inflation, time horizon, tradeoffs, or alternative baselines.</x:v>
       </x:c>
       <x:c r="X88" t="str">
-        <x:v>Technology marketing frequently calls a new tool 'more productive' without clarifying productive for whom, under what workflow, at what error rate, and at what human cost.</x:v>
+        <x:v>Technology marketing frequently calls a new tool 'more productive' without clarifying productive for whom, under what workflow, at what error rate, and at what human cost. The fallacy here is Incomplete comparison: one option is called better, worse, cheaper, safer, or more effective without specifying the relevant comparison class or the other factors that matter. That matters here because a comparison can be true in one narrow respect while misleading overall. A better analysis would remember that the missing pieces might include quality, risk, wages, inflation, time horizon, tradeoffs, or alternative baselines.</x:v>
       </x:c>
       <x:c r="Y88" t="str"/>
       <x:c r="Z88" t="str"/>
@@ -6615,10 +6930,10 @@
         <x:v>A complete comparison needs a consistent baseline or a transparent weighting of tradeoffs, not a collage of unrelated best cases.</x:v>
       </x:c>
       <x:c r="V89" t="str">
-        <x:v>Consumer ads often compare each feature against whichever rival looks weakest on that feature, then announce overall superiority.</x:v>
+        <x:v>Consumer ads often compare each feature against whichever rival looks weakest on that feature, then announce overall superiority. The fallacy here is Inconsistent comparison: different comparison targets are used across different dimensions to create the illusion of one all-around winner. That matters here because a complete comparison needs a consistent baseline or a transparent weighting of tradeoffs, not a collage of unrelated best cases. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W89" t="str">
-        <x:v>Campaign brag sheets sometimes do the same by mixing job growth, crime, housing, and graduation metrics against different jurisdictions and different years.</x:v>
+        <x:v>Campaign brag sheets sometimes do the same by mixing job growth, crime, housing, and graduation metrics against different jurisdictions and different years. The fallacy here is Inconsistent comparison: different comparison targets are used across different dimensions to create the illusion of one all-around winner. That matters here because a complete comparison needs a consistent baseline or a transparent weighting of tradeoffs, not a collage of unrelated best cases. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X89" t="str"/>
       <x:c r="Y89" t="str"/>
@@ -6684,10 +6999,10 @@
         <x:v>Authorial intent is not always the only thing that matters, but it is often part of the evidence. Declaring it irrelevant by default can flatten interpretation into projection.</x:v>
       </x:c>
       <x:c r="V90" t="str">
-        <x:v>Debates over constitutional language, literature, and political slogans often swing too far toward present-day interpretation while discarding what the author or framers were trying to do.</x:v>
+        <x:v>Debates over constitutional language, literature, and political slogans often swing too far toward present-day interpretation while discarding what the author or framers were trying to do. The fallacy here is Intentional fallacy: the creator's intended meaning is treated as irrelevant in contexts where that intention is actually important to understanding the work or statement. That matters here because authorial intent is not always the only thing that matters, but it is often part of the evidence. A better analysis would remember that declaring it irrelevant by default can flatten interpretation into projection.</x:v>
       </x:c>
       <x:c r="W90" t="str">
-        <x:v>Online arguments about memes, jokes, and clips frequently ignore context and stated intent altogether, then treat the most inflammatory possible reading as the only serious one.</x:v>
+        <x:v>Online arguments about memes, jokes, and clips frequently ignore context and stated intent altogether, then treat the most inflammatory possible reading as the only serious one. The fallacy here is Intentional fallacy: the creator's intended meaning is treated as irrelevant in contexts where that intention is actually important to understanding the work or statement. That matters here because authorial intent is not always the only thing that matters, but it is often part of the evidence. A better analysis would remember that declaring it irrelevant by default can flatten interpretation into projection.</x:v>
       </x:c>
       <x:c r="X90" t="str"/>
       <x:c r="Y90" t="str"/>
@@ -6753,10 +7068,10 @@
         <x:v>An ought needs a normative premise about goals, duties, or values. Facts alone do not generate that extra step.</x:v>
       </x:c>
       <x:c r="V91" t="str">
-        <x:v>Arguments about gender, family, and competition often slide from claims about what is common in nature to claims about what is therefore morally required.</x:v>
+        <x:v>Arguments about gender, family, and competition often slide from claims about what is common in nature to claims about what is therefore morally required. The fallacy here is Is-ought problem: a descriptive claim about what is common, natural, or actual is treated as if it directly established what ought to be done. That matters here because an ought needs a normative premise about goals, duties, or values. A better analysis would remember that facts alone do not generate that extra step.</x:v>
       </x:c>
       <x:c r="W91" t="str">
-        <x:v>Workplace norms are regularly defended by saying they are simply how the market works, even when the moral question is precisely whether the market should work that way.</x:v>
+        <x:v>Workplace norms are regularly defended by saying they are simply how the market works, even when the moral question is precisely whether the market should work that way. The fallacy here is Is-ought problem: a descriptive claim about what is common, natural, or actual is treated as if it directly established what ought to be done. That matters here because an ought needs a normative premise about goals, duties, or values. A better analysis would remember that facts alone do not generate that extra step.</x:v>
       </x:c>
       <x:c r="X91" t="str"/>
       <x:c r="Y91" t="str"/>
@@ -6822,10 +7137,10 @@
         <x:v>Some labels are fair descriptions, but the fallacy appears when the emotional sting of the label is doing the work that evidence and argument have not done.</x:v>
       </x:c>
       <x:c r="V92" t="str">
-        <x:v>Words like 'groomer,' 'traitor,' 'fascist,' 'woke,' 'cultist,' and 'denier' are often deployed less to clarify than to trigger a moral reaction before the argument can be examined.</x:v>
+        <x:v>Words like 'groomer,' 'traitor,' 'fascist,' 'woke,' 'cultist,' and 'denier' are often deployed less to clarify than to trigger a moral reaction before the argument can be examined. The fallacy here is Judgmental language: pejorative, loaded, or insulting language is used to steer judgment in place of actual support for the conclusion. That matters here because some labels are fair descriptions, but the fallacy appears when the emotional sting of the label is doing the work that evidence and argument have not done. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="W92" t="str">
-        <x:v>Political and religious arguments frequently pre-load the conclusion by choosing terms that make disagreement sound shameful or corrupt from the start.</x:v>
+        <x:v>Political and religious arguments frequently pre-load the conclusion by choosing terms that make disagreement sound shameful or corrupt from the start. The fallacy here is Judgmental language: pejorative, loaded, or insulting language is used to steer judgment in place of actual support for the conclusion. That matters here because some labels are fair descriptions, but the fallacy appears when the emotional sting of the label is doing the work that evidence and argument have not done. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="X92" t="str"/>
       <x:c r="Y92" t="str"/>
@@ -6887,10 +7202,10 @@
         <x:v>Many real systems change slowly at first, then rapidly, then plateau, or even reverse after a threshold.</x:v>
       </x:c>
       <x:c r="V93" t="str">
-        <x:v>Growth forecasts for social platforms often assume audience reach will keep scaling smoothly even after attention markets saturate.</x:v>
+        <x:v>Growth forecasts for social platforms often assume audience reach will keep scaling smoothly even after attention markets saturate. The fallacy here is Linearity fallacy: someone assumes that doubling the input will double the output even though the system has thresholds, saturation, feedback loops, or diminishing returns. That matters here because many real systems change slowly at first, then rapidly, then plateau, or even reverse after a threshold. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W93" t="str">
-        <x:v>Policy debates about climate, housing, and healthcare frequently ignore the non-linear effects of bottlenecks, incentives, and behavioral feedback.</x:v>
+        <x:v>Policy debates about climate, housing, and healthcare frequently ignore the non-linear effects of bottlenecks, incentives, and behavioral feedback. The fallacy here is Linearity fallacy: someone assumes that doubling the input will double the output even though the system has thresholds, saturation, feedback loops, or diminishing returns. That matters here because many real systems change slowly at first, then rapidly, then plateau, or even reverse after a threshold. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X93" t="str"/>
       <x:c r="Y93" t="str"/>
@@ -6954,16 +7269,22 @@
         <x:v>New technology can displace real jobs and create painful transitions. The fallacy is the stronger claim that automation as such can only destroy work, rather than reorganize it, lower costs, create new roles, or shift labor elsewhere.</x:v>
       </x:c>
       <x:c r="V94" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+        <x:v>AI seen cutting worker numbers, survey by staffing company Adecco shows
+Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. The fallacy here is Luddite fallacy: labor-saving technology is treated as if it must reduce total employment or human usefulness simply because it automates some existing tasks. That matters here because new technology can displace real jobs and create painful transitions. A better analysis would remember that the fallacy is the stronger claim that automation as such can only destroy work, rather than reorganize it, lower costs, create new roles, or shift labor elsewhere.
+Source: Reuters | 2024-04-05
+https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="W94" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>Analysis-US port strike throws spotlight on big union foe: automation
+Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. The fallacy here is Luddite fallacy: labor-saving technology is treated as if it must reduce total employment or human usefulness simply because it automates some existing tasks. That matters here because new technology can displace real jobs and create painful transitions. A better analysis would remember that the fallacy is the stronger claim that automation as such can only destroy work, rather than reorganize it, lower costs, create new roles, or shift labor elsewhere.
+Source: Reuters | 2024-10-04
+https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="X94" t="str">
-        <x:v>Debates over generative AI in 2024 often jumped straight from 'this automates part of my job' to 'therefore it will inevitably make people broadly unemployable,' skipping the more complicated evidence about substitution, augmentation, and new roles.</x:v>
+        <x:v>Debates over generative AI in 2024 often jumped straight from 'this automates part of my job' to 'therefore it will inevitably make people broadly unemployable,' skipping the more complicated evidence about substitution, augmentation, and new roles. The fallacy here is Luddite fallacy: labor-saving technology is treated as if it must reduce total employment or human usefulness simply because it automates some existing tasks. That matters here because new technology can displace real jobs and create painful transitions. A better analysis would remember that the fallacy is the stronger claim that automation as such can only destroy work, rather than reorganize it, lower costs, create new roles, or shift labor elsewhere.</x:v>
       </x:c>
       <x:c r="Y94" t="str">
-        <x:v>The U.S. dockworker fight over port automation in October 2024 showed why the issue is serious, but it also illustrated the need to distinguish real bargaining and transition questions from the blanket claim that productivity-enhancing technology is always socially worse.</x:v>
+        <x:v>The U.S. dockworker fight over port automation in October 2024 showed why the issue is serious, but it also illustrated the need to distinguish real bargaining and transition questions from the blanket claim that productivity-enhancing technology is always socially worse. The fallacy here is Luddite fallacy: labor-saving technology is treated as if it must reduce total employment or human usefulness simply because it automates some existing tasks. That matters here because new technology can displace real jobs and create painful transitions. A better analysis would remember that the fallacy is the stronger claim that automation as such can only destroy work, rather than reorganize it, lower costs, create new roles, or shift labor elsewhere.</x:v>
       </x:c>
       <x:c r="Z94" t="str"/>
       <x:c r="AA94" t="str">
@@ -7025,10 +7346,10 @@
         <x:v>In ordinary factual contexts, identical referents can be substituted safely. In belief, knowledge, or perception contexts, that move can fail because the speaker's information is incomplete.</x:v>
       </x:c>
       <x:c r="V95" t="str">
-        <x:v>This fallacy shows up whenever people infer identity or non-identity from what someone knows, recognizes, or can name rather than from the underlying facts.</x:v>
+        <x:v>This fallacy shows up whenever people infer identity or non-identity from what someone knows, recognizes, or can name rather than from the underlying facts. The fallacy here is Masked man fallacy: two names or descriptions refer to the same thing, but a belief or knowledge context blocks simple substitution and the argument ignores that. That matters here because in ordinary factual contexts, identical referents can be substituted safely. A better analysis would remember that in belief, knowledge, or perception contexts, that move can fail because the speaker's information is incomplete.</x:v>
       </x:c>
       <x:c r="W95" t="str">
-        <x:v>Mystery, anonymity, and pseudonym debates often slide into this mistake by assuming that not knowing a description means the object cannot be the same one known under another description.</x:v>
+        <x:v>Mystery, anonymity, and pseudonym debates often slide into this mistake by assuming that not knowing a description means the object cannot be the same one known under another description. The fallacy here is Masked man fallacy: two names or descriptions refer to the same thing, but a belief or knowledge context blocks simple substitution and the argument ignores that. That matters here because in ordinary factual contexts, identical referents can be substituted safely. A better analysis would remember that in belief, knowledge, or perception contexts, that move can fail because the speaker's information is incomplete.</x:v>
       </x:c>
       <x:c r="X95" t="str"/>
       <x:c r="Y95" t="str"/>
@@ -7098,19 +7419,31 @@
         <x:v>Vivid cases matter, especially when they reveal harms abstract statistics can hide. The fallacy arises when memorable exceptions are used as if they were the normal pattern.</x:v>
       </x:c>
       <x:c r="V96" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>AI experimentation is high risk, high reward for low-profile political campaigns
+AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. The fallacy here is Misleading vividness: a striking anecdote or emotionally intense case is used to make a problem seem more common, clear, or representative than the broader evidence allows. That matters here because vivid cases matter, especially when they reveal harms abstract statistics can hide. A better analysis would remember that the fallacy arises when memorable exceptions are used as if they were the normal pattern.
+Source: Associated Press | 2024-06-17
+https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="W96" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Google makes fixes to AI-generated search summaries after outlandish answers went viral
+When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. The fallacy here is Misleading vividness: a striking anecdote or emotionally intense case is used to make a problem seem more common, clear, or representative than the broader evidence allows. That matters here because vivid cases matter, especially when they reveal harms abstract statistics can hide. A better analysis would remember that the fallacy arises when memorable exceptions are used as if they were the normal pattern.
+Source: Associated Press | 2024-05-31
+https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="X96" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets
+AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' The fallacy here is Misleading vividness: a striking anecdote or emotionally intense case is used to make a problem seem more common, clear, or representative than the broader evidence allows. That matters here because vivid cases matter, especially when they reveal harms abstract statistics can hide. A better analysis would remember that the fallacy arises when memorable exceptions are used as if they were the normal pattern.
+Source: Associated Press | 2024-09-26
+https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="Y96" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>AP Explains: Migration is more complex than politics show
+AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. The fallacy here is Misleading vividness: a striking anecdote or emotionally intense case is used to make a problem seem more common, clear, or representative than the broader evidence allows. That matters here because vivid cases matter, especially when they reveal harms abstract statistics can hide. A better analysis would remember that the fallacy arises when memorable exceptions are used as if they were the normal pattern.
+Source: Associated Press | 2024-09-20
+https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="Z96" t="str">
-        <x:v>The Springfield rumor gained traction partly because lurid, memorable imagery traveled faster than the dull but crucial fact that authorities found no supporting evidence.</x:v>
+        <x:v>The Springfield rumor gained traction partly because lurid, memorable imagery traveled faster than the dull but crucial fact that authorities found no supporting evidence. The fallacy here is Misleading vividness: a striking anecdote or emotionally intense case is used to make a problem seem more common, clear, or representative than the broader evidence allows. That matters here because vivid cases matter, especially when they reveal harms abstract statistics can hide. A better analysis would remember that the fallacy arises when memorable exceptions are used as if they were the normal pattern.</x:v>
       </x:c>
       <x:c r="AA96" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -7175,13 +7508,16 @@
         <x:v>Standards can be refined in good faith, especially when both sides notice a weak test. The fallacy appears when the revision functions mainly to avoid conceding that the earlier standard was met.</x:v>
       </x:c>
       <x:c r="V97" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. The fallacy here is Moving the goalpost: evidence that was supposed to satisfy a stated standard is dismissed and a new, harder standard is introduced so the conclusion never has to be reconsidered. That matters here because standards can be refined in good faith, especially when both sides notice a weak test. That is the exact slip in this case: the revision functions mainly to avoid conceding that the earlier standard was met.
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="W97" t="str">
-        <x:v>Public AI debates in 2024 often moved from benchmark scores to some new test the moment a model cleared the previous bar, making 'proof' of competence permanently out of reach.</x:v>
+        <x:v>Public AI debates in 2024 often moved from benchmark scores to some new test the moment a model cleared the previous bar, making 'proof' of competence permanently out of reach. The fallacy here is Moving the goalpost: evidence that was supposed to satisfy a stated standard is dismissed and a new, harder standard is introduced so the conclusion never has to be reconsidered. That matters here because standards can be refined in good faith, especially when both sides notice a weak test. That is the exact slip in this case: the revision functions mainly to avoid conceding that the earlier standard was met.</x:v>
       </x:c>
       <x:c r="X97" t="str">
-        <x:v>Election-conspiracy arguments often work this way: once courts, audits, and recounts address one claim, the standard shifts to a different alleged irregularity without any willingness to concede what the earlier evidence settled.</x:v>
+        <x:v>Election-conspiracy arguments often work this way: once courts, audits, and recounts address one claim, the standard shifts to a different alleged irregularity without any willingness to concede what the earlier evidence settled. The fallacy here is Moving the goalpost: evidence that was supposed to satisfy a stated standard is dismissed and a new, harder standard is introduced so the conclusion never has to be reconsidered. That matters here because standards can be refined in good faith, especially when both sides notice a weak test. That is the exact slip in this case: the revision functions mainly to avoid conceding that the earlier standard was met.</x:v>
       </x:c>
       <x:c r="Y97" t="str"/>
       <x:c r="Z97" t="str"/>
@@ -7246,13 +7582,16 @@
         <x:v>Natural things can be wonderful, harmful, neutral, or context-dependent. Arsenic, viruses, and earthquakes are natural too. The relevant questions are evidence, outcomes, and tradeoffs, not whether something sounds untouched.</x:v>
       </x:c>
       <x:c r="V98" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. The fallacy here is Naturalistic fallacy: something is treated as good, safe, or morally preferable mainly because it is called natural, traditional, or closer to nature. That matters here because natural things can be wonderful, harmful, neutral, or context-dependent. A better analysis would remember that arsenic, viruses, and earthquakes are natural too.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="W98" t="str">
-        <x:v>The 2026 push to expand raw milk access often leaned on the idea that unprocessed equals healthier, despite repeated warnings from public-health officials that the safety risks are real and the claimed benefits remain unproven.</x:v>
+        <x:v>The 2026 push to expand raw milk access often leaned on the idea that unprocessed equals healthier, despite repeated warnings from public-health officials that the safety risks are real and the claimed benefits remain unproven. The fallacy here is Naturalistic fallacy: something is treated as good, safe, or morally preferable mainly because it is called natural, traditional, or closer to nature. That matters here because natural things can be wonderful, harmful, neutral, or context-dependent. A better analysis would remember that arsenic, viruses, and earthquakes are natural too.</x:v>
       </x:c>
       <x:c r="X98" t="str">
-        <x:v>Wellness marketing routinely sells herbs, supplements, detoxes, and hormone routines by invoking nature itself as if natural origin settled the medical question.</x:v>
+        <x:v>Wellness marketing routinely sells herbs, supplements, detoxes, and hormone routines by invoking nature itself as if natural origin settled the medical question. The fallacy here is Naturalistic fallacy: something is treated as good, safe, or morally preferable mainly because it is called natural, traditional, or closer to nature. That matters here because natural things can be wonderful, harmful, neutral, or context-dependent. A better analysis would remember that arsenic, viruses, and earthquakes are natural too.</x:v>
       </x:c>
       <x:c r="Y98" t="str"/>
       <x:c r="Z98" t="str"/>
@@ -7315,10 +7654,10 @@
         <x:v>The rational status of a claim depends on the evidence for it, not on whether someone has managed to close every imaginable contrary possibility.</x:v>
       </x:c>
       <x:c r="V99" t="str">
-        <x:v>Election, paranormal, and conspiracy claims often survive by saying 'you cannot prove it did not happen,' as if that absence of disproof supplied positive warrant.</x:v>
+        <x:v>Election, paranormal, and conspiracy claims often survive by saying 'you cannot prove it did not happen,' as if that absence of disproof supplied positive warrant. The fallacy here is Negative proof fallacy: a claim is treated as true because it has not been disproved, or false because it has not been proved. That matters here because the rational status of a claim depends on the evidence for it, not on whether someone has managed to close every imaginable contrary possibility. The better question is whether the conclusion really follows once the structure of the argument is stated plainly.</x:v>
       </x:c>
       <x:c r="W99" t="str">
-        <x:v>Skeptics can also commit the reverse mistake when they treat an unproved claim as definitively false rather than merely unestablished.</x:v>
+        <x:v>Skeptics can also commit the reverse mistake when they treat an unproved claim as definitively false rather than merely unestablished. The fallacy here is Negative proof fallacy: a claim is treated as true because it has not been disproved, or false because it has not been proved. That matters here because the rational status of a claim depends on the evidence for it, not on whether someone has managed to close every imaginable contrary possibility. The better question is whether the conclusion really follows once the structure of the argument is stated plainly.</x:v>
       </x:c>
       <x:c r="X99" t="str"/>
       <x:c r="Y99" t="str"/>
@@ -7382,10 +7721,10 @@
         <x:v>Most policies, tools, and institutions are partial fixes. The right question is often whether an option improves matters relative to feasible alternatives, not whether it achieves a flawless end state.</x:v>
       </x:c>
       <x:c r="V100" t="str">
-        <x:v>Critics of content moderation, election safeguards, AI guardrails, and climate policy often reject incremental measures on the grounds that bad cases will still exist, as if imperfection erased all value.</x:v>
+        <x:v>Critics of content moderation, election safeguards, AI guardrails, and climate policy often reject incremental measures on the grounds that bad cases will still exist, as if imperfection erased all value. The fallacy here is Nirvana fallacy: a realistic option is rejected because it does not solve a problem perfectly or because an imagined ideal is used as the standard of comparison. That matters here because most policies, tools, and institutions are partial fixes. A better analysis would remember that the right question is often whether an option improves matters relative to feasible alternatives, not whether it achieves a flawless end state.</x:v>
       </x:c>
       <x:c r="W100" t="str">
-        <x:v>Debates about public-health interventions frequently collapse into 'if it does not stop every case, it failed,' which compares reality to fantasy rather than to the available alternatives.</x:v>
+        <x:v>Debates about public-health interventions frequently collapse into 'if it does not stop every case, it failed,' which compares reality to fantasy rather than to the available alternatives. The fallacy here is Nirvana fallacy: a realistic option is rejected because it does not solve a problem perfectly or because an imagined ideal is used as the standard of comparison. That matters here because most policies, tools, and institutions are partial fixes. A better analysis would remember that the right question is often whether an option improves matters relative to feasible alternatives, not whether it achieves a flawless end state.</x:v>
       </x:c>
       <x:c r="X100" t="str"/>
       <x:c r="Y100" t="str"/>
@@ -7457,10 +7796,10 @@
         <x:v>Sometimes categories do have genuine criteria. The fallacy arises when the criteria are improvised only after a counterexample appears, so the definition changes to save the claim.</x:v>
       </x:c>
       <x:c r="V101" t="str">
-        <x:v>In 2024 intraparty fights, Republicans who backed Ukraine aid or accepted the 2020 certification were often dismissed as 'not real conservatives' instead of being treated as counterexamples within conservatism.</x:v>
+        <x:v>In 2024 intraparty fights, Republicans who backed Ukraine aid or accepted the 2020 certification were often dismissed as 'not real conservatives' instead of being treated as counterexamples within conservatism. The fallacy here is No True Scotsman: someone protects a generalization from counterexamples by redefining the group with an ad hoc 'real' or 'true' membership test. That matters here because sometimes categories do have genuine criteria. A better analysis would remember that the fallacy arises when the criteria are improvised only after a counterexample appears, so the definition changes to save the claim.</x:v>
       </x:c>
       <x:c r="W101" t="str">
-        <x:v>Religious and ideological arguments frequently insist that anyone whose behavior embarrasses the group was never a 'true' believer in the first place, which preserves group purity by redefinition.</x:v>
+        <x:v>Religious and ideological arguments frequently insist that anyone whose behavior embarrasses the group was never a 'true' believer in the first place, which preserves group purity by redefinition. The fallacy here is No True Scotsman: someone protects a generalization from counterexamples by redefining the group with an ad hoc 'real' or 'true' membership test. That matters here because sometimes categories do have genuine criteria. A better analysis would remember that the fallacy arises when the criteria are improvised only after a counterexample appears, so the definition changes to save the claim.</x:v>
       </x:c>
       <x:c r="X101" t="str"/>
       <x:c r="Y101" t="str"/>
@@ -7528,10 +7867,10 @@
         <x:v>A principle can have limits, but if the exceptions swallow the rule, the apparent commitment becomes mostly decorative.</x:v>
       </x:c>
       <x:c r="V102" t="str">
-        <x:v>Public commitments to transparency, merit, or local control often vanish once they threaten a favored outcome.</x:v>
+        <x:v>Public commitments to transparency, merit, or local control often vanish once they threaten a favored outcome. The fallacy here is Overwhelming exception: a general principle is padded with so many exceptions that it no longer guides action or says much of substance. That matters here because a principle can have limits, but if the exceptions swallow the rule, the apparent commitment becomes mostly decorative. The better question is whether the key term keeps the same meaning from one step of the argument to the next.</x:v>
       </x:c>
       <x:c r="W102" t="str">
-        <x:v>Organizations sometimes advertise simple values statements that become practically meaningless once the long list of carve-outs is revealed.</x:v>
+        <x:v>Organizations sometimes advertise simple values statements that become practically meaningless once the long list of carve-outs is revealed. The fallacy here is Overwhelming exception: a general principle is padded with so many exceptions that it no longer guides action or says much of substance. That matters here because a principle can have limits, but if the exceptions swallow the rule, the apparent commitment becomes mostly decorative. The better question is whether the key term keeps the same meaning from one step of the argument to the next.</x:v>
       </x:c>
       <x:c r="X102" t="str"/>
       <x:c r="Y102" t="str"/>
@@ -7595,13 +7934,16 @@
         <x:v>Some traits do cluster more often than chance would predict, but the cluster is not a logical necessity. A familiar package can make us overread what belongs together.</x:v>
       </x:c>
       <x:c r="V103" t="str">
-        <x:v>AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. — Associated Press | Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent | 2024-02-17 | https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
+        <x:v>Christian-nation idea fuels US conservative causes, but historians say it misreads founders' intent
+AP's February 17, 2024 article on Christian nationalism shows how selective quotations and compressed historical frames can turn a messy founding-era record into a neat ideological slogan. It is a rich case for misclassification, quotation out of context, and present-minded reinterpretation. The fallacy here is Package-deal fallacy: traits that are often bundled together by stereotype, tradition, or habit are treated as if they must always come as a package. That matters here because some traits do cluster more often than chance would predict, but the cluster is not a logical necessity. A better analysis would remember that a familiar package can make us overread what belongs together.
+Source: Associated Press | 2024-02-17
+https://apnews.com/article/4ea388e8d80c54016a6a4460cbef9b82</x:v>
       </x:c>
       <x:c r="W103" t="str">
-        <x:v>Campaign and media narratives often assume that working-class, rural, religious, or college-educated identities come with one full political bundle attached.</x:v>
+        <x:v>Campaign and media narratives often assume that working-class, rural, religious, or college-educated identities come with one full political bundle attached. The fallacy here is Package-deal fallacy: traits that are often bundled together by stereotype, tradition, or habit are treated as if they must always come as a package. That matters here because some traits do cluster more often than chance would predict, but the cluster is not a logical necessity. A better analysis would remember that a familiar package can make us overread what belongs together.</x:v>
       </x:c>
       <x:c r="X103" t="str">
-        <x:v>People frequently expect hobbies, musical taste, fashion, or ethnicity to drag a whole associated worldview behind them even when the individual breaks the pattern.</x:v>
+        <x:v>People frequently expect hobbies, musical taste, fashion, or ethnicity to drag a whole associated worldview behind them even when the individual breaks the pattern. The fallacy here is Package-deal fallacy: traits that are often bundled together by stereotype, tradition, or habit are treated as if they must always come as a package. That matters here because some traits do cluster more often than chance would predict, but the cluster is not a logical necessity. A better analysis would remember that a familiar package can make us overread what belongs together.</x:v>
       </x:c>
       <x:c r="Y103" t="str"/>
       <x:c r="Z103" t="str"/>
@@ -7668,10 +8010,10 @@
         <x:v>Personifying weather, markets, or algorithms can be a vivid metaphor, but it becomes fallacious when the metaphor is used as literal evidence.</x:v>
       </x:c>
       <x:c r="V104" t="str">
-        <x:v>People often say the algorithm hates them, loves outrage, or wants to silence them when the actual explanation is a mix of optimization rules and incentives.</x:v>
+        <x:v>People often say the algorithm hates them, loves outrage, or wants to silence them when the actual explanation is a mix of optimization rules and incentives. The fallacy here is Pathetic fallacy: human feelings, intentions, or judgments are projected onto impersonal things and then treated as if the projection explained reality. That matters here because personifying weather, markets, or algorithms can be a vivid metaphor, but it becomes fallacious when the metaphor is used as literal evidence. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W104" t="str">
-        <x:v>News coverage sometimes treats storms, markets, or viruses as if they were moral agents taking revenge, sending messages, or rewarding virtue.</x:v>
+        <x:v>News coverage sometimes treats storms, markets, or viruses as if they were moral agents taking revenge, sending messages, or rewarding virtue. The fallacy here is Pathetic fallacy: human feelings, intentions, or judgments are projected onto impersonal things and then treated as if the projection explained reality. That matters here because personifying weather, markets, or algorithms can be a vivid metaphor, but it becomes fallacious when the metaphor is used as literal evidence. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X104" t="str"/>
       <x:c r="Y104" t="str"/>
@@ -7737,10 +8079,10 @@
         <x:v>A partial improvement can still be worthwhile. The mistake is demanding perfection from one proposal when no realistic policy can eliminate the problem entirely.</x:v>
       </x:c>
       <x:c r="V105" t="str">
-        <x:v>Climate and transit proposals are often rejected because they will not solve emissions or congestion completely, as if incomplete progress counted as no progress.</x:v>
+        <x:v>Climate and transit proposals are often rejected because they will not solve emissions or congestion completely, as if incomplete progress counted as no progress. The fallacy here is Perfect solution fallacy: a useful solution is dismissed because it does not fully solve the problem or because some flaws would remain afterward. That matters here because a partial improvement can still be worthwhile. A better analysis would remember that the mistake is demanding perfection from one proposal when no realistic policy can eliminate the problem entirely.</x:v>
       </x:c>
       <x:c r="W105" t="str">
-        <x:v>Arguments about AI safety, gun policy, and public health often dismiss guardrails for failing to eliminate every bad case, rather than asking whether they would reduce harm.</x:v>
+        <x:v>Arguments about AI safety, gun policy, and public health often dismiss guardrails for failing to eliminate every bad case, rather than asking whether they would reduce harm. The fallacy here is Perfect solution fallacy: a useful solution is dismissed because it does not fully solve the problem or because some flaws would remain afterward. That matters here because a partial improvement can still be worthwhile. A better analysis would remember that the mistake is demanding perfection from one proposal when no realistic policy can eliminate the problem entirely.</x:v>
       </x:c>
       <x:c r="X105" t="str"/>
       <x:c r="Y105" t="str"/>
@@ -7800,13 +8142,16 @@
         <x:v>Many human traits and performances come in degrees. Treating any deviation from an ideal as proof of total failure destroys the resolution needed for fair judgment.</x:v>
       </x:c>
       <x:c r="V106" t="str">
-        <x:v>AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. — Associated Press | Why AP called the Arizona Senate race for Ruben Gallego | 2024-11-12 | https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
+        <x:v>Why AP called the Arizona Senate race for Ruben Gallego
+AP's explanation of why it called the Arizona Senate race for Ruben Gallego is a useful numbers-first counterexample to intuition-driven political certainty. It shows what it looks like to reason from remaining vote shares, path constraints, and actual denominators instead of headline impressions. The fallacy here is Perfect standard: a messy range of better and worse cases is collapsed into a rigid perfect-or-failed binary. That matters here because many human traits and performances come in degrees. A better analysis would remember that treating any deviation from an ideal as proof of total failure destroys the resolution needed for fair judgment.
+Source: Associated Press | 2024-11-12
+https://apnews.com/article/169d3ba60250c786b22668f415b6c505</x:v>
       </x:c>
       <x:c r="W106" t="str">
-        <x:v>Debates about media bias, moral character, and institutional trust often assume that if a person or outlet is not perfectly objective, then it is simply propaganda.</x:v>
+        <x:v>Debates about media bias, moral character, and institutional trust often assume that if a person or outlet is not perfectly objective, then it is simply propaganda. The fallacy here is Perfect standard: a messy range of better and worse cases is collapsed into a rigid perfect-or-failed binary. That matters here because many human traits and performances come in degrees. A better analysis would remember that treating any deviation from an ideal as proof of total failure destroys the resolution needed for fair judgment.</x:v>
       </x:c>
       <x:c r="X106" t="str">
-        <x:v>Public discussion of peace, tolerance, and fairness often ignores large improvements because some imperfection remains somewhere.</x:v>
+        <x:v>Public discussion of peace, tolerance, and fairness often ignores large improvements because some imperfection remains somewhere. The fallacy here is Perfect standard: a messy range of better and worse cases is collapsed into a rigid perfect-or-failed binary. That matters here because many human traits and performances come in degrees. A better analysis would remember that treating any deviation from an ideal as proof of total failure destroys the resolution needed for fair judgment.</x:v>
       </x:c>
       <x:c r="Y106" t="str"/>
       <x:c r="Z106" t="str"/>
@@ -7875,10 +8220,10 @@
         <x:v>An analogy usually highlights one structural similarity, not a one-to-one mapping of every detail.</x:v>
       </x:c>
       <x:c r="V107" t="str">
-        <x:v>Infrastructure analogies about bridges, firewalls, or guardrails are often attacked by demanding that every literal feature transfer over exactly.</x:v>
+        <x:v>Infrastructure analogies about bridges, firewalls, or guardrails are often attacked by demanding that every literal feature transfer over exactly. The fallacy here is Perverted analogy: an analogy is deliberately stretched past its intended point so it can be mocked or refuted. That matters here because an analogy usually highlights one structural similarity, not a one-to-one mapping of every detail. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="W107" t="str">
-        <x:v>Debaters sometimes turn an opponent's limited comparison into a cartoon version so they can say the analogy obviously fails.</x:v>
+        <x:v>Debaters sometimes turn an opponent's limited comparison into a cartoon version so they can say the analogy obviously fails. The fallacy here is Perverted analogy: an analogy is deliberately stretched past its intended point so it can be mocked or refuted. That matters here because an analogy usually highlights one structural similarity, not a one-to-one mapping of every detail. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="X107" t="str"/>
       <x:c r="Y107" t="str"/>
@@ -7938,10 +8283,10 @@
         <x:v>A true or well-supported detail can increase trust only where the claims are genuinely linked. Often the extra conclusion is just hitching a ride on evidence that belongs to something narrower.</x:v>
       </x:c>
       <x:c r="V108" t="str">
-        <x:v>After the September 2024 ABC debate, the fact that the lecterns differed in height was treated by some users as if it supported much broader unverified claims about secret coordination and leaked questions.</x:v>
+        <x:v>After the September 2024 ABC debate, the fact that the lecterns differed in height was treated by some users as if it supported much broader unverified claims about secret coordination and leaked questions. The fallacy here is Piggy-back assumption: evidence for one claim is illegitimately used as if it also confirmed a second claim that merely travels alongside it. That matters here because a true or well-supported detail can increase trust only where the claims are genuinely linked. A better analysis would remember that often the extra conclusion is just hitching a ride on evidence that belongs to something narrower.</x:v>
       </x:c>
       <x:c r="W108" t="str">
-        <x:v>Conspiracy arguments often point to one authentic photo, real location, or correct minor fact and then use that narrow success to smuggle in much larger unsupported conclusions.</x:v>
+        <x:v>Conspiracy arguments often point to one authentic photo, real location, or correct minor fact and then use that narrow success to smuggle in much larger unsupported conclusions. The fallacy here is Piggy-back assumption: evidence for one claim is illegitimately used as if it also confirmed a second claim that merely travels alongside it. That matters here because a true or well-supported detail can increase trust only where the claims are genuinely linked. A better analysis would remember that often the extra conclusion is just hitching a ride on evidence that belongs to something narrower.</x:v>
       </x:c>
       <x:c r="X108" t="str"/>
       <x:c r="Y108" t="str"/>
@@ -8007,10 +8352,10 @@
         <x:v>Source criticism can be relevant, but poisoning the well tries to make the audience stop listening before the argument or evidence is even on the table.</x:v>
       </x:c>
       <x:c r="V109" t="str">
-        <x:v>In political and media fights, audiences are often primed to treat a judge, journalist, scientist, or witness as corrupt before that person's specific evidence is even heard.</x:v>
+        <x:v>In political and media fights, audiences are often primed to treat a judge, journalist, scientist, or witness as corrupt before that person's specific evidence is even heard. The fallacy here is Poisoning the well: negative framing is introduced in advance so that whatever a person says next will be dismissed before it is fairly heard. That matters here because source criticism can be relevant, but poisoning the well tries to make the audience stop listening before the argument or evidence is even on the table. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="W109" t="str">
-        <x:v>After the September 2024 Harris-Trump debate, repeated claims that moderators and outlets were inherently rigged encouraged supporters to dismiss later fact-checks in advance rather than assess them on the merits.</x:v>
+        <x:v>After the September 2024 Harris-Trump debate, repeated claims that moderators and outlets were inherently rigged encouraged supporters to dismiss later fact-checks in advance rather than assess them on the merits. The fallacy here is Poisoning the well: negative framing is introduced in advance so that whatever a person says next will be dismissed before it is fairly heard. That matters here because source criticism can be relevant, but poisoning the well tries to make the audience stop listening before the argument or evidence is even on the table. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="X109" t="str"/>
       <x:c r="Y109" t="str"/>
@@ -8076,10 +8421,10 @@
         <x:v>Temporal order matters for causation, but it is only one ingredient. The improvement might be coincidence, regression to the mean, other background changes, or a different cause entirely.</x:v>
       </x:c>
       <x:c r="V110" t="str">
-        <x:v>Wellness and self-optimization discourse in 2024 routinely credited cold plunges, supplements, or glucose hacks for improvements that followed several simultaneous lifestyle changes.</x:v>
+        <x:v>Wellness and self-optimization discourse in 2024 routinely credited cold plunges, supplements, or glucose hacks for improvements that followed several simultaneous lifestyle changes. The fallacy here is Post hoc ergo propter hoc: someone infers that because one event happened before another, the earlier event caused the later one. That matters here because temporal order matters for causation, but it is only one ingredient. A better analysis would remember that the improvement might be coincidence, regression to the mean, other background changes, or a different cause entirely.</x:v>
       </x:c>
       <x:c r="W110" t="str">
-        <x:v>Politicians often claim that a policy worked because a good trend appeared soon after the policy was announced, even when the trend began earlier or other explanations remain stronger.</x:v>
+        <x:v>Politicians often claim that a policy worked because a good trend appeared soon after the policy was announced, even when the trend began earlier or other explanations remain stronger. The fallacy here is Post hoc ergo propter hoc: someone infers that because one event happened before another, the earlier event caused the later one. That matters here because temporal order matters for causation, but it is only one ingredient. A better analysis would remember that the improvement might be coincidence, regression to the mean, other background changes, or a different cause entirely.</x:v>
       </x:c>
       <x:c r="X110" t="str"/>
       <x:c r="Y110" t="str"/>
@@ -8145,16 +8490,22 @@
         <x:v>Examples can illustrate a claim, but they do not by themselves prove a universal proposition. The missing question is whether the example is representative.</x:v>
       </x:c>
       <x:c r="V111" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Google makes fixes to AI-generated search summaries after outlandish answers went viral
+When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. The fallacy here is Proof by example: one or a few examples are offered as if they were enough to establish a universal claim. That matters here because examples can illustrate a claim, but they do not by themselves prove a universal proposition. A better analysis would remember that the missing question is whether the example is representative.
+Source: Associated Press | 2024-05-31
+https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="W111" t="str">
-        <x:v>AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. — Associated Press | Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said | 2024-10-26 | https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
+        <x:v>Researchers say an AI-powered transcription tool used in hospitals invents things no one ever said
+AP's reporting on Whisper hallucinating in hospital transcripts is a sharp case of a polished output being treated as if accuracy followed from confidence and fluency. It also shows why one plausible-seeming example is not enough to certify a tool as reliable in high-stakes settings. The fallacy here is Proof by example: one or a few examples are offered as if they were enough to establish a universal claim. That matters here because examples can illustrate a claim, but they do not by themselves prove a universal proposition. A better analysis would remember that the missing question is whether the example is representative.
+Source: Associated Press | 2024-10-26
+https://apnews.com/article/90020cdf5fa16c79ca2e5b6c4c9bbb14</x:v>
       </x:c>
       <x:c r="X111" t="str">
-        <x:v>A single accurate prediction, one striking conversion story, or one dramatic crime clip is often treated as if it proved a broad thesis about markets, religion, or social decline.</x:v>
+        <x:v>A single accurate prediction, one striking conversion story, or one dramatic crime clip is often treated as if it proved a broad thesis about markets, religion, or social decline. The fallacy here is Proof by example: one or a few examples are offered as if they were enough to establish a universal claim. That matters here because examples can illustrate a claim, but they do not by themselves prove a universal proposition. A better analysis would remember that the missing question is whether the example is representative.</x:v>
       </x:c>
       <x:c r="Y111" t="str">
-        <x:v>Debates about AI often jump from one impressive demo or one embarrassing failure to a total conclusion about the technology as a whole.</x:v>
+        <x:v>Debates about AI often jump from one impressive demo or one embarrassing failure to a total conclusion about the technology as a whole. The fallacy here is Proof by example: one or a few examples are offered as if they were enough to establish a universal claim. That matters here because examples can illustrate a claim, but they do not by themselves prove a universal proposition. A better analysis would remember that the missing question is whether the example is representative.</x:v>
       </x:c>
       <x:c r="Z111" t="str"/>
       <x:c r="AA111" t="str">
@@ -8220,13 +8571,16 @@
         <x:v>Complexity is not itself a fallacy. The problem is using sprawl as a shield, making it costly to respond point by point and then treating any unanswered fragment as proof of victory.</x:v>
       </x:c>
       <x:c r="V112" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. The fallacy here is Proof by verbosity: a claim is protected by an avalanche of words, side points, jargon, or branching assertions that overwhelm reasonable scrutiny and create the illusion of depth. That matters here because complexity is not itself a fallacy. A better analysis would remember that the problem is using sprawl as a shield, making it costly to respond point by point and then treating any unanswered fragment as proof of victory.
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="W112" t="str">
-        <x:v>Podcast debates, marathon livestreams, and mega-threads often bury the central claim beneath so many tangents that audiences mistake exhaustion for concession.</x:v>
+        <x:v>Podcast debates, marathon livestreams, and mega-threads often bury the central claim beneath so many tangents that audiences mistake exhaustion for concession. The fallacy here is Proof by verbosity: a claim is protected by an avalanche of words, side points, jargon, or branching assertions that overwhelm reasonable scrutiny and create the illusion of depth. That matters here because complexity is not itself a fallacy. A better analysis would remember that the problem is using sprawl as a shield, making it costly to respond point by point and then treating any unanswered fragment as proof of victory.</x:v>
       </x:c>
       <x:c r="X112" t="str">
-        <x:v>AI-generated text makes this tactic cheaper by allowing people to produce long, confident, fast-moving argument dumps that sound comprehensive while remaining poorly grounded.</x:v>
+        <x:v>AI-generated text makes this tactic cheaper by allowing people to produce long, confident, fast-moving argument dumps that sound comprehensive while remaining poorly grounded. The fallacy here is Proof by verbosity: a claim is protected by an avalanche of words, side points, jargon, or branching assertions that overwhelm reasonable scrutiny and create the illusion of depth. That matters here because complexity is not itself a fallacy. A better analysis would remember that the problem is using sprawl as a shield, making it costly to respond point by point and then treating any unanswered fragment as proof of victory.</x:v>
       </x:c>
       <x:c r="Y112" t="str"/>
       <x:c r="Z112" t="str"/>
@@ -8289,10 +8643,10 @@
         <x:v>The missing piece is the base rate. Even a very accurate test can generate many false matches when the target condition is rare.</x:v>
       </x:c>
       <x:c r="V113" t="str">
-        <x:v>Crime and security debates often overstate the force of DNA, face-recognition, or screening matches by ignoring how many non-matching people were also in the pool.</x:v>
+        <x:v>Crime and security debates often overstate the force of DNA, face-recognition, or screening matches by ignoring how many non-matching people were also in the pool. The fallacy here is Prosecutor's fallacy: a low probability of a false match is confused with a low probability that a matched person is innocent. That matters here because the missing piece is the base rate. A better analysis would remember that even a very accurate test can generate many false matches when the target condition is rare.</x:v>
       </x:c>
       <x:c r="W113" t="str">
-        <x:v>A similar mistake appears whenever a diagnostic tool's false-positive rate is treated as if it directly gave the chance that any one flagged person is guilty, sick, or dangerous.</x:v>
+        <x:v>A similar mistake appears whenever a diagnostic tool's false-positive rate is treated as if it directly gave the chance that any one flagged person is guilty, sick, or dangerous. The fallacy here is Prosecutor's fallacy: a low probability of a false match is confused with a low probability that a matched person is innocent. That matters here because the missing piece is the base rate. A better analysis would remember that even a very accurate test can generate many false matches when the target condition is rare.</x:v>
       </x:c>
       <x:c r="X113" t="str"/>
       <x:c r="Y113" t="str"/>
@@ -8356,10 +8710,10 @@
         <x:v>Self-knowledge can be useful, but it is not a universal template. Other people may share some motives while differing sharply on others.</x:v>
       </x:c>
       <x:c r="V114" t="str">
-        <x:v>People often assume that because they would lie, panic, or seek status in a situation, anyone else in that situation must be driven by the same motive.</x:v>
+        <x:v>People often assume that because they would lie, panic, or seek status in a situation, anyone else in that situation must be driven by the same motive. The fallacy here is Psychologist's fallacy: someone projects their own motives, fears, or mental structure onto others and treats that projection as insight into those other people. That matters here because self-knowledge can be useful, but it is not a universal template. A better analysis would remember that other people may share some motives while differing sharply on others.</x:v>
       </x:c>
       <x:c r="W114" t="str">
-        <x:v>Political and religious debate is full of claims about what opponents 'really know' or 'really fear' that reflect the speaker's own psychology more than the target's.</x:v>
+        <x:v>Political and religious debate is full of claims about what opponents 'really know' or 'really fear' that reflect the speaker's own psychology more than the target's. The fallacy here is Psychologist's fallacy: someone projects their own motives, fears, or mental structure onto others and treats that projection as insight into those other people. That matters here because self-knowledge can be useful, but it is not a universal template. A better analysis would remember that other people may share some motives while differing sharply on others.</x:v>
       </x:c>
       <x:c r="X114" t="str"/>
       <x:c r="Y114" t="str"/>
@@ -8425,19 +8779,31 @@
         <x:v>Not every detour is fallacious; context can matter. The fallacy appears when the diversion substitutes for addressing the question that was actually on the table.</x:v>
       </x:c>
       <x:c r="V115" t="str">
-        <x:v>AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' — Associated Press | Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets | 2024-09-26 | https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
+        <x:v>Top Haitian official denounces false claim, repeated by Trump, that immigrants are eating pets
+AP's September 26, 2024 report on Haiti's transitional council president condemning the Springfield pet-eating rumor shows how quickly a sensational falsehood can travel from fringe posts to a presidential debate to the United Nations. The case is vivid enough to illustrate both emotional manipulation and the costs of repeating an unverified claim because it 'sounds like what the other side would do.' The fallacy here is Red herring: someone diverts attention from the unresolved issue by switching to a different issue that is easier, safer, or more emotionally useful. That matters here because not every detour is fallacious; context can matter. That is the exact slip in this case: the diversion substitutes for addressing the question that was actually on the table.
+Source: Associated Press | 2024-09-26
+https://apnews.com/article/7004bd6820a4d2f8bf07adf4f6dcf18b</x:v>
       </x:c>
       <x:c r="W115" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+        <x:v>Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement
+AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. The fallacy here is Red herring: someone diverts attention from the unresolved issue by switching to a different issue that is easier, safer, or more emotionally useful. That matters here because not every detour is fallacious; context can matter. That is the exact slip in this case: the diversion substitutes for addressing the question that was actually on the table.
+Source: Associated Press | 2024-09-10
+https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="X115" t="str">
-        <x:v>AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. — Associated Press | FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate | 2024-06-27 | https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
+        <x:v>FACT FOCUS: Here's a look at some of the false claims made during Biden and Trump's first debate
+AP's June 27, 2024 fact check of the first Biden-Trump debate is a dense collection of real argumentative shortcuts: statistics pulled loose from context, emotionally loaded immigration claims, and repeated assertions that did more rhetorical than evidential work. It is one of the best single-source stress tests in the library. The fallacy here is Red herring: someone diverts attention from the unresolved issue by switching to a different issue that is easier, safer, or more emotionally useful. That matters here because not every detour is fallacious; context can matter. That is the exact slip in this case: the diversion substitutes for addressing the question that was actually on the table.
+Source: Associated Press | 2024-06-27
+https://www.ap.org/news-highlights/spotlights/2024/fact-focus-heres-a-look-at-some-of-the-false-claims-made-during-biden-and-trumps-first-debate/</x:v>
       </x:c>
       <x:c r="Y115" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>AP Explains: Migration is more complex than politics show
+AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. The fallacy here is Red herring: someone diverts attention from the unresolved issue by switching to a different issue that is easier, safer, or more emotionally useful. That matters here because not every detour is fallacious; context can matter. That is the exact slip in this case: the diversion substitutes for addressing the question that was actually on the table.
+Source: Associated Press | 2024-09-20
+https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="Z115" t="str">
-        <x:v>In the June 27, 2024 Biden-Trump debate, answers about the economy, abortion, and January 6 often veered into immigration, personal fitness, or unrelated grievances instead of the question asked.</x:v>
+        <x:v>In the June 27, 2024 Biden-Trump debate, answers about the economy, abortion, and January 6 often veered into immigration, personal fitness, or unrelated grievances instead of the question asked. The fallacy here is Red herring: someone diverts attention from the unresolved issue by switching to a different issue that is easier, safer, or more emotionally useful. That matters here because not every detour is fallacious; context can matter. That is the exact slip in this case: the diversion substitutes for addressing the question that was actually on the table.</x:v>
       </x:c>
       <x:c r="AA115" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -8494,10 +8860,10 @@
         <x:v>Evidence matters for empirical claims, but it cannot rescue a contradiction. If the concept itself does not make sense, more observations do not repair it.</x:v>
       </x:c>
       <x:c r="V116" t="str">
-        <x:v>Some arguments define a being, force, or property in mutually incompatible ways and then insist critics still need field evidence before calling the view incoherent.</x:v>
+        <x:v>Some arguments define a being, force, or property in mutually incompatible ways and then insist critics still need field evidence before calling the view incoherent. The fallacy here is Redeeming illogic with evidence: someone demands empirical evidence before rejecting a concept that is already incoherent, self-contradictory, or logically impossible on its own terms. That matters here because evidence matters for empirical claims, but it cannot rescue a contradiction. A better analysis would remember that if the concept itself does not make sense, more observations do not repair it.</x:v>
       </x:c>
       <x:c r="W116" t="str">
-        <x:v>Online debate often treats every claim as if it deserved purely empirical testing, even when the real defect appears earlier at the level of definition or logical consistency.</x:v>
+        <x:v>Online debate often treats every claim as if it deserved purely empirical testing, even when the real defect appears earlier at the level of definition or logical consistency. The fallacy here is Redeeming illogic with evidence: someone demands empirical evidence before rejecting a concept that is already incoherent, self-contradictory, or logically impossible on its own terms. That matters here because evidence matters for empirical claims, but it cannot rescue a contradiction. A better analysis would remember that if the concept itself does not make sense, more observations do not repair it.</x:v>
       </x:c>
       <x:c r="X116" t="str"/>
       <x:c r="Y116" t="str"/>
@@ -8563,10 +8929,10 @@
         <x:v>After unusually high or low outcomes, partial reversion toward the average is often expected even without special causal forces.</x:v>
       </x:c>
       <x:c r="V117" t="str">
-        <x:v>Sports commentators routinely over-credit halftime speeches or rituals for rebounds that would be unsurprising after an extreme first-half performance.</x:v>
+        <x:v>Sports commentators routinely over-credit halftime speeches or rituals for rebounds that would be unsurprising after an extreme first-half performance. The fallacy here is Regression fallacy: movement back toward a normal range after an extreme result is credited to some intervention that may have had little or nothing to do with it. That matters here because after unusually high or low outcomes, partial reversion toward the average is often expected even without special causal forces. The better question is what alternative causes, missing mechanisms, or reversed directions still need to be ruled out.</x:v>
       </x:c>
       <x:c r="W117" t="str">
-        <x:v>Investors and managers often mistake a natural bounce after a terrible quarter for proof that a new slogan, consultant, or memo fixed the underlying problem.</x:v>
+        <x:v>Investors and managers often mistake a natural bounce after a terrible quarter for proof that a new slogan, consultant, or memo fixed the underlying problem. The fallacy here is Regression fallacy: movement back toward a normal range after an extreme result is credited to some intervention that may have had little or nothing to do with it. That matters here because after unusually high or low outcomes, partial reversion toward the average is often expected even without special causal forces. The better question is what alternative causes, missing mechanisms, or reversed directions still need to be ruled out.</x:v>
       </x:c>
       <x:c r="X117" t="str"/>
       <x:c r="Y117" t="str"/>
@@ -8636,10 +9002,10 @@
         <x:v>Metaphor can be useful shorthand, but the fallacy appears when agency, intention, or moral responsibility is attributed to an abstraction as though it literally possessed a mind of its own.</x:v>
       </x:c>
       <x:c r="V118" t="str">
-        <x:v>People talk as if capitalism, democracy, the algorithm, or history itself wants, fears, rewards, or punishes, which can hide the actual network of human choices and incentives underneath.</x:v>
+        <x:v>People talk as if capitalism, democracy, the algorithm, or history itself wants, fears, rewards, or punishes, which can hide the actual network of human choices and incentives underneath. The fallacy here is Reification: an abstraction is spoken of as if it were a concrete agent or thing in a way that misleads rather than merely using harmless metaphor. That matters here because metaphor can be useful shorthand, but the fallacy appears when agency, intention, or moral responsibility is attributed to an abstraction as though it literally possessed a mind of its own. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W118" t="str">
-        <x:v>AI discussions sometimes slide from 'the model produced this output' to 'the AI wants this outcome,' smuggling in a stronger picture of agency than the evidence supports.</x:v>
+        <x:v>AI discussions sometimes slide from 'the model produced this output' to 'the AI wants this outcome,' smuggling in a stronger picture of agency than the evidence supports. The fallacy here is Reification: an abstraction is spoken of as if it were a concrete agent or thing in a way that misleads rather than merely using harmless metaphor. That matters here because metaphor can be useful shorthand, but the fallacy appears when agency, intention, or moral responsibility is attributed to an abstraction as though it literally possessed a mind of its own. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X118" t="str"/>
       <x:c r="Y118" t="str"/>
@@ -8705,10 +9071,10 @@
         <x:v>An outcome can make a story feel inevitable in retrospect without ever having been inevitable in advance. Hindsight strips away the branching paths that were live at the time.</x:v>
       </x:c>
       <x:c r="V119" t="str">
-        <x:v>After elections, market crashes, and celebrity scandals, commentators often speak as if the final result had been written into the evidence from the start rather than emerging from many uncertain factors.</x:v>
+        <x:v>After elections, market crashes, and celebrity scandals, commentators often speak as if the final result had been written into the evidence from the start rather than emerging from many uncertain factors. The fallacy here is Retrospective determinism: occurs when, after an outcome happens, people claim it was inevitable or obvious all along even though the uncertainty beforehand was real. That matters here because an outcome can make a story feel inevitable in retrospect without ever having been inevitable in advance. A better analysis would remember that hindsight strips away the branching paths that were live at the time.</x:v>
       </x:c>
       <x:c r="W119" t="str">
-        <x:v>This fallacy regularly follows close races and volatile technologies, where later narratives overstate how clear the winning path supposedly was.</x:v>
+        <x:v>This fallacy regularly follows close races and volatile technologies, where later narratives overstate how clear the winning path supposedly was. The fallacy here is Retrospective determinism: occurs when, after an outcome happens, people claim it was inevitable or obvious all along even though the uncertainty beforehand was real. That matters here because an outcome can make a story feel inevitable in retrospect without ever having been inevitable in advance. A better analysis would remember that hindsight strips away the branching paths that were live at the time.</x:v>
       </x:c>
       <x:c r="X119" t="str"/>
       <x:c r="Y119" t="str"/>
@@ -8770,10 +9136,10 @@
         <x:v>Many concepts such as belief, risk, identity, and influence work by degree. Treating them as all-or-nothing can falsify the speaker's actual position.</x:v>
       </x:c>
       <x:c r="V120" t="str">
-        <x:v>Election, public-health, and AI debates often force nuanced confidence claims into binary boxes such as certain or uncertain, safe or unsafe, real or fake.</x:v>
+        <x:v>Election, public-health, and AI debates often force nuanced confidence claims into binary boxes such as certain or uncertain, safe or unsafe, real or fake. The fallacy here is Semantic pixelization: a fuzzy, graded, or probabilistic position is forced into unnaturally sharp categories so it becomes easier to attack. That matters here because many concepts such as belief, risk, identity, and influence work by degree. A better analysis would remember that treating them as all-or-nothing can falsify the speaker's actual position.</x:v>
       </x:c>
       <x:c r="W120" t="str">
-        <x:v>Arguments about what someone believes frequently replace a spectrum of confidence with a yes-or-no label that the original speaker never endorsed.</x:v>
+        <x:v>Arguments about what someone believes frequently replace a spectrum of confidence with a yes-or-no label that the original speaker never endorsed. The fallacy here is Semantic pixelization: a fuzzy, graded, or probabilistic position is forced into unnaturally sharp categories so it becomes easier to attack. That matters here because many concepts such as belief, risk, identity, and influence work by degree. A better analysis would remember that treating them as all-or-nothing can falsify the speaker's actual position.</x:v>
       </x:c>
       <x:c r="X120" t="str"/>
       <x:c r="Y120" t="str"/>
@@ -8841,10 +9207,10 @@
         <x:v>Emotional attraction can explain why we want a conclusion, but not whether the conclusion is supported. A heartwarming possibility can still be false or impractical.</x:v>
       </x:c>
       <x:c r="V121" t="str">
-        <x:v>Fundraising pitches, miracle-cure stories, and uplifting viral posts often rely on the emotional payoff of the conclusion to make scrutiny feel mean or unnecessary.</x:v>
+        <x:v>Fundraising pitches, miracle-cure stories, and uplifting viral posts often rely on the emotional payoff of the conclusion to make scrutiny feel mean or unnecessary. The fallacy here is Sentimental fallacy: the desirability, comfort, or emotional appeal of an outcome is treated as if that were evidence that the outcome is true, feasible, or justified. That matters here because emotional attraction can explain why we want a conclusion, but not whether the conclusion is supported. A better analysis would remember that a heartwarming possibility can still be false or impractical.</x:v>
       </x:c>
       <x:c r="W121" t="str">
-        <x:v>Public debate about policy sometimes slides from 'this would be compassionate' to 'therefore it must be workable and correct,' skipping the harder evidential and tradeoff questions.</x:v>
+        <x:v>Public debate about policy sometimes slides from 'this would be compassionate' to 'therefore it must be workable and correct,' skipping the harder evidential and tradeoff questions. The fallacy here is Sentimental fallacy: the desirability, comfort, or emotional appeal of an outcome is treated as if that were evidence that the outcome is true, feasible, or justified. That matters here because emotional attraction can explain why we want a conclusion, but not whether the conclusion is supported. A better analysis would remember that a heartwarming possibility can still be false or impractical.</x:v>
       </x:c>
       <x:c r="X121" t="str"/>
       <x:c r="Y121" t="str"/>
@@ -8912,16 +9278,22 @@
         <x:v>This is close to cherry picking, but the emphasis is on drawing the target around the bullet holes after the shots land. Post hoc pattern-hunting can make randomness, noise, or mixed data look like confirmation.</x:v>
       </x:c>
       <x:c r="V122" t="str">
-        <x:v>NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not
+NPR's October 12, 2024 fact check on noncitizen-voting claims is a good case study in the gap between isolated anecdotes and population-level conclusions. It shows how a few suspicious stories can feel decisive even when the base rates and verified counts point the other way. The fallacy here is Sharpshooter fallacy: someone highlights the data cluster that supports a favored story only after looking at the results, then treats that hand-picked pattern as if it had been the tested target all along. That matters here because this is close to cherry picking, but the emphasis is on drawing the target around the bullet holes after the shots land. A better analysis would remember that post hoc pattern-hunting can make randomness, noise, or mixed data look like confirmation.
+Source: NPR | 2024-10-12
+https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="W122" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+        <x:v>Survivorship bias
+Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. The fallacy here is Sharpshooter fallacy: someone highlights the data cluster that supports a favored story only after looking at the results, then treats that hand-picked pattern as if it had been the tested target all along. That matters here because this is close to cherry picking, but the emphasis is on drawing the target around the bullet holes after the shots land. A better analysis would remember that post hoc pattern-hunting can make randomness, noise, or mixed data look like confirmation.
+Source: Britannica | 2026-01-01
+https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
       <x:c r="X122" t="str">
-        <x:v>Economic and election commentary often selects the time window, county, or subgroup that flatters the preferred narrative after the fact, then presents that slice as the decisive measure.</x:v>
+        <x:v>Economic and election commentary often selects the time window, county, or subgroup that flatters the preferred narrative after the fact, then presents that slice as the decisive measure. The fallacy here is Sharpshooter fallacy: someone highlights the data cluster that supports a favored story only after looking at the results, then treats that hand-picked pattern as if it had been the tested target all along. That matters here because this is close to cherry picking, but the emphasis is on drawing the target around the bullet holes after the shots land. A better analysis would remember that post hoc pattern-hunting can make randomness, noise, or mixed data look like confirmation.</x:v>
       </x:c>
       <x:c r="Y122" t="str">
-        <x:v>AI benchmarking and startup marketing sometimes advertise the few tasks where a model shines while leaving out the wider distribution of tasks where the results are weaker or unstable.</x:v>
+        <x:v>AI benchmarking and startup marketing sometimes advertise the few tasks where a model shines while leaving out the wider distribution of tasks where the results are weaker or unstable. The fallacy here is Sharpshooter fallacy: someone highlights the data cluster that supports a favored story only after looking at the results, then treats that hand-picked pattern as if it had been the tested target all along. That matters here because this is close to cherry picking, but the emphasis is on drawing the target around the bullet holes after the shots land. A better analysis would remember that post hoc pattern-hunting can make randomness, noise, or mixed data look like confirmation.</x:v>
       </x:c>
       <x:c r="Z122" t="str"/>
       <x:c r="AA122" t="str">
@@ -8987,19 +9359,28 @@
         <x:v>Some causes are more important than others, and sometimes one factor really is dominant. The fallacy appears when a multi-causal phenomenon is flattened into a one-variable story without enough evidence.</x:v>
       </x:c>
       <x:c r="V123" t="str">
-        <x:v>AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. — Associated Press | AP Explains: Migration is more complex than politics show | 2024-09-20 | https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
+        <x:v>AP Explains: Migration is more complex than politics show
+AP's migration explainer from September 20, 2024 is useful because it deliberately widens the frame beyond debate slogans and viral rumors. That makes it a strong case for fallacies that depend on flattening a complicated policy landscape into one cause, one image, or one moral punchline. The fallacy here is Single cause fallacy: a complex outcome is explained as if one cause alone did the work, while other relevant causes are ignored or illegitimately minimized. That matters here because some causes are more important than others, and sometimes one factor really is dominant. That is the exact slip in this case: a multi-causal phenomenon is flattened into a one-variable story without enough evidence.
+Source: Associated Press | 2024-09-20
+https://apnews.com/article/e6cc90ee306bd6442c6c47a058bf43d5</x:v>
       </x:c>
       <x:c r="W123" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+        <x:v>AI seen cutting worker numbers, survey by staffing company Adecco shows
+Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. The fallacy here is Single cause fallacy: a complex outcome is explained as if one cause alone did the work, while other relevant causes are ignored or illegitimately minimized. That matters here because some causes are more important than others, and sometimes one factor really is dominant. That is the exact slip in this case: a multi-causal phenomenon is flattened into a one-variable story without enough evidence.
+Source: Reuters | 2024-04-05
+https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="X123" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>Analysis-US port strike throws spotlight on big union foe: automation
+Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. The fallacy here is Single cause fallacy: a complex outcome is explained as if one cause alone did the work, while other relevant causes are ignored or illegitimately minimized. That matters here because some causes are more important than others, and sometimes one factor really is dominant. That is the exact slip in this case: a multi-causal phenomenon is flattened into a one-variable story without enough evidence.
+Source: Reuters | 2024-10-04
+https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="Y123" t="str">
-        <x:v>Arguments about inflation, crime, housing costs, and educational decline often blame one villain such as immigrants, regulation, presidents, or social media, even when the outcome reflects multiple interacting causes.</x:v>
+        <x:v>Arguments about inflation, crime, housing costs, and educational decline often blame one villain such as immigrants, regulation, presidents, or social media, even when the outcome reflects multiple interacting causes. The fallacy here is Single cause fallacy: a complex outcome is explained as if one cause alone did the work, while other relevant causes are ignored or illegitimately minimized. That matters here because some causes are more important than others, and sometimes one factor really is dominant. That is the exact slip in this case: a multi-causal phenomenon is flattened into a one-variable story without enough evidence.</x:v>
       </x:c>
       <x:c r="Z123" t="str">
-        <x:v>After school shootings or viral episodes of unrest, public commentary regularly rushes to one master explanation instead of asking how incentives, access, institutions, culture, and personal history combine.</x:v>
+        <x:v>After school shootings or viral episodes of unrest, public commentary regularly rushes to one master explanation instead of asking how incentives, access, institutions, culture, and personal history combine. The fallacy here is Single cause fallacy: a complex outcome is explained as if one cause alone did the work, while other relevant causes are ignored or illegitimately minimized. That matters here because some causes are more important than others, and sometimes one factor really is dominant. That is the exact slip in this case: a multi-causal phenomenon is flattened into a one-variable story without enough evidence.</x:v>
       </x:c>
       <x:c r="AA123" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -9064,19 +9445,28 @@
         <x:v>Some slopes are real, especially when incentives, precedent, or institutional weakness make escalation predictable. The fallacy appears when the chain is asserted rather than argued for.</x:v>
       </x:c>
       <x:c r="V124" t="str">
-        <x:v>AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. — Associated Press | Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging | 2024-05-18 | https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
+        <x:v>Noncitizen voting, already illegal in federal elections, becomes a centerpiece of 2024 GOP messaging
+AP's May 18, 2024 overview of noncitizen-voting rhetoric documented how a politically useful intuition about election fraud kept being treated as if it were established by the evidence. The report is especially useful for seeing how tiny counts, suggestive language, and moral urgency can be stretched into system-wide claims. The fallacy here is Slippery slope: someone claims that a relatively small first step will trigger a chain of worsening outcomes without showing why that chain is likely, stable, or hard to stop. That matters here because some slopes are real, especially when incentives, precedent, or institutional weakness make escalation predictable. That is the exact slip in this case: the chain is asserted rather than argued for.
+Source: Associated Press | 2024-05-18
+https://apnews.com/article/1c65429c152c2a10514b5156eacf9ca7</x:v>
       </x:c>
       <x:c r="W124" t="str">
-        <x:v>Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. — Reuters | AI seen cutting worker numbers, survey by staffing company Adecco shows | 2024-04-05 | https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
+        <x:v>AI seen cutting worker numbers, survey by staffing company Adecco shows
+Reuters' April 5, 2024 report on the Adecco survey is a good reminder that expectations about job loss are not the same as demonstrated causal outcomes. It is useful wherever people slide from speculative trend talk to a confident story about what one technology will inevitably do to the labor market. The fallacy here is Slippery slope: someone claims that a relatively small first step will trigger a chain of worsening outcomes without showing why that chain is likely, stable, or hard to stop. That matters here because some slopes are real, especially when incentives, precedent, or institutional weakness make escalation predictable. That is the exact slip in this case: the chain is asserted rather than argued for.
+Source: Reuters | 2024-04-05
+https://uk.investing.com/news/stock-market-news/ai-seen-cutting-worker-numbers-survey-by-staffing-company-adecco-shows-3419149</x:v>
       </x:c>
       <x:c r="X124" t="str">
-        <x:v>Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. — Reuters | Analysis-US port strike throws spotlight on big union foe: automation | 2024-10-04 | https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
+        <x:v>Analysis-US port strike throws spotlight on big union foe: automation
+Reuters' October 4, 2024 analysis of the dockworker strike is valuable because it resists the easy story that automation is either an obvious job-killer or an obvious productivity savior. It exposes how often both sides of a public dispute compress tradeoffs into one emotionally convenient causal narrative. The fallacy here is Slippery slope: someone claims that a relatively small first step will trigger a chain of worsening outcomes without showing why that chain is likely, stable, or hard to stop. That matters here because some slopes are real, especially when incentives, precedent, or institutional weakness make escalation predictable. That is the exact slip in this case: the chain is asserted rather than argued for.
+Source: Reuters | 2024-10-04
+https://www.investing.com/news/stock-market-news/analysisus-port-strike-throws-spotlight-on-big-union-foe-automation-3648625</x:v>
       </x:c>
       <x:c r="Y124" t="str">
-        <x:v>In 2024 arguments over classroom AI, both enthusiasts and critics often predicted inevitable futures - either total educational collapse or total educational liberation - without showing why intermediate guardrails would fail.</x:v>
+        <x:v>In 2024 arguments over classroom AI, both enthusiasts and critics often predicted inevitable futures - either total educational collapse or total educational liberation - without showing why intermediate guardrails would fail. The fallacy here is Slippery slope: someone claims that a relatively small first step will trigger a chain of worsening outcomes without showing why that chain is likely, stable, or hard to stop. That matters here because some slopes are real, especially when incentives, precedent, or institutional weakness make escalation predictable. That is the exact slip in this case: the chain is asserted rather than argued for.</x:v>
       </x:c>
       <x:c r="Z124" t="str">
-        <x:v>Election rhetoric about mail voting, early voting, or routine administrative changes often predicts the total breakdown of legitimacy from one policy shift without evidence for the full cascade.</x:v>
+        <x:v>Election rhetoric about mail voting, early voting, or routine administrative changes often predicts the total breakdown of legitimacy from one policy shift without evidence for the full cascade. The fallacy here is Slippery slope: someone claims that a relatively small first step will trigger a chain of worsening outcomes without showing why that chain is likely, stable, or hard to stop. That matters here because some slopes are real, especially when incentives, precedent, or institutional weakness make escalation predictable. That is the exact slip in this case: the chain is asserted rather than argued for.</x:v>
       </x:c>
       <x:c r="AA124" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -9139,16 +9529,22 @@
         <x:v>Exceptions can be justified, but they need a principled reason. Mere attachment to the favored case is not enough.</x:v>
       </x:c>
       <x:c r="V125" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. The fallacy here is Special pleading: someone asks for an exception to a rule or standard but does not provide a relevant reason for why the favored case should be exempt. That matters here because exceptions can be justified, but they need a principled reason. A better analysis would remember that mere attachment to the favored case is not enough.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="W125" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. The fallacy here is Special pleading: someone asks for an exception to a rule or standard but does not provide a relevant reason for why the favored case should be exempt. That matters here because exceptions can be justified, but they need a principled reason. A better analysis would remember that mere attachment to the favored case is not enough.
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="X125" t="str">
-        <x:v>Political actors often demand strict accountability, civility, or transparency for opponents while inventing excuses for why their own side should be judged differently.</x:v>
+        <x:v>Political actors often demand strict accountability, civility, or transparency for opponents while inventing excuses for why their own side should be judged differently. The fallacy here is Special pleading: someone asks for an exception to a rule or standard but does not provide a relevant reason for why the favored case should be exempt. That matters here because exceptions can be justified, but they need a principled reason. A better analysis would remember that mere attachment to the favored case is not enough.</x:v>
       </x:c>
       <x:c r="Y125" t="str">
-        <x:v>Religious and ideological arguments often exempt cherished claims from the evidence standards applied to ordinary claims.</x:v>
+        <x:v>Religious and ideological arguments often exempt cherished claims from the evidence standards applied to ordinary claims. The fallacy here is Special pleading: someone asks for an exception to a rule or standard but does not provide a relevant reason for why the favored case should be exempt. That matters here because exceptions can be justified, but they need a principled reason. A better analysis would remember that mere attachment to the favored case is not enough.</x:v>
       </x:c>
       <x:c r="Z125" t="str"/>
       <x:c r="AA125" t="str">
@@ -9212,10 +9608,10 @@
         <x:v>Attention is selective. Media, algorithms, and memory amplify the dramatic cases, not the ordinary distribution.</x:v>
       </x:c>
       <x:c r="V126" t="str">
-        <x:v>Crime clips, campus incidents, and viral protest footage often dominate public perception far beyond their representativeness, making whole groups look more extreme than they are.</x:v>
+        <x:v>Crime clips, campus incidents, and viral protest footage often dominate public perception far beyond their representativeness, making whole groups look more extreme than they are. The fallacy here is Spotlight fallacy: the most visible or most covered cases in a category are treated as if they represent the category as a whole. That matters here because attention is selective. A better analysis would remember that media, algorithms, and memory amplify the dramatic cases, not the ordinary distribution.</x:v>
       </x:c>
       <x:c r="W126" t="str">
-        <x:v>People watching political interviews can easily conclude that a population is loud, combative, or theatrical without noticing that quieter members of the same population rarely become visible.</x:v>
+        <x:v>People watching political interviews can easily conclude that a population is loud, combative, or theatrical without noticing that quieter members of the same population rarely become visible. The fallacy here is Spotlight fallacy: the most visible or most covered cases in a category are treated as if they represent the category as a whole. That matters here because attention is selective. A better analysis would remember that media, algorithms, and memory amplify the dramatic cases, not the ordinary distribution.</x:v>
       </x:c>
       <x:c r="X126" t="str"/>
       <x:c r="Y126" t="str"/>
@@ -9279,10 +9675,10 @@
         <x:v>Sometimes the problem is deliberate obscurity; other times it is sincere confusion. Either way, complexity should not be mistaken for structure.</x:v>
       </x:c>
       <x:c r="V127" t="str">
-        <x:v>Conspiracy reasoning often spirals into self-sealing loops where every attempted refutation becomes fresh confirmation through an increasingly baroque chain of premises.</x:v>
+        <x:v>Conspiracy reasoning often spirals into self-sealing loops where every attempted refutation becomes fresh confirmation through an increasingly baroque chain of premises. The fallacy here is Square logic: an argument becomes so internally tangled that its pieces no longer form a coherent chain from premise to conclusion even though it sounds intricate. That matters here because sometimes the problem is deliberate obscurity; other times it is sincere confusion. A better analysis would remember that either way, complexity should not be mistaken for structure.</x:v>
       </x:c>
       <x:c r="W127" t="str">
-        <x:v>AI-generated argument dumps can produce this effect by chaining plausible-sounding clauses that never quite add up to a valid line of reasoning.</x:v>
+        <x:v>AI-generated argument dumps can produce this effect by chaining plausible-sounding clauses that never quite add up to a valid line of reasoning. The fallacy here is Square logic: an argument becomes so internally tangled that its pieces no longer form a coherent chain from premise to conclusion even though it sounds intricate. That matters here because sometimes the problem is deliberate obscurity; other times it is sincere confusion. A better analysis would remember that either way, complexity should not be mistaken for structure.</x:v>
       </x:c>
       <x:c r="X127" t="str"/>
       <x:c r="Y127" t="str"/>
@@ -9348,13 +9744,16 @@
         <x:v>A straw man can be created by exaggeration, selective quotation, or by ignoring the qualifying parts of the original claim. It is not enough that a reply is critical; the key problem is that the reply no longer addresses the real position.</x:v>
       </x:c>
       <x:c r="V128" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+        <x:v>Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement
+AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. The fallacy here is Straw man argument: someone replaces an opponent's actual position with a weaker, more extreme, or simplified version and then refutes that easier target. That matters here because a straw man can be created by exaggeration, selective quotation, or by ignoring the qualifying parts of the original claim. A better analysis would remember that it is not enough that a reply is critical; the key problem is that the reply no longer addresses the real position.
+Source: Associated Press | 2024-09-10
+https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="W128" t="str">
-        <x:v>During the September 10, 2024 Harris-Trump debate, claims about abortion rights were repeatedly recast into the far more extreme charge that Democrats support killing babies after birth, which is not the position being defended.</x:v>
+        <x:v>During the September 10, 2024 Harris-Trump debate, claims about abortion rights were repeatedly recast into the far more extreme charge that Democrats support killing babies after birth, which is not the position being defended. The fallacy here is Straw man argument: someone replaces an opponent's actual position with a weaker, more extreme, or simplified version and then refutes that easier target. That matters here because a straw man can be created by exaggeration, selective quotation, or by ignoring the qualifying parts of the original claim. A better analysis would remember that it is not enough that a reply is critical; the key problem is that the reply no longer addresses the real position.</x:v>
       </x:c>
       <x:c r="X128" t="str">
-        <x:v>Debates over campus speech and content moderation often turn a narrower argument about rules, incentives, or disclosure into the cartoon claim that one side 'wants censorship' or 'wants total chaos.'</x:v>
+        <x:v>Debates over campus speech and content moderation often turn a narrower argument about rules, incentives, or disclosure into the cartoon claim that one side 'wants censorship' or 'wants total chaos.' The fallacy here is Straw man argument: someone replaces an opponent's actual position with a weaker, more extreme, or simplified version and then refutes that easier target. That matters here because a straw man can be created by exaggeration, selective quotation, or by ignoring the qualifying parts of the original claim. A better analysis would remember that it is not enough that a reply is critical; the key problem is that the reply no longer addresses the real position.</x:v>
       </x:c>
       <x:c r="Y128" t="str"/>
       <x:c r="Z128" t="str"/>
@@ -9421,19 +9820,28 @@
         <x:v>Strong delivery can make good arguments easier to hear, but it can also camouflage weak ones. Audiences often remember certainty, rhythm, and applause longer than the actual reasoning.</x:v>
       </x:c>
       <x:c r="V129" t="str">
-        <x:v>AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. — Associated Press | AI experimentation is high risk, high reward for low-profile political campaigns | 2024-06-17 | https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
+        <x:v>AI experimentation is high risk, high reward for low-profile political campaigns
+AP reported that a PAC opposing Shreveport mayor Adrian Perkins used an AI-generated attack ad that put his face on a chastened student in a principal's office. The case is a clean example of vivid, emotionally loaded presentation doing persuasive work that policy argument still had to do for itself. The fallacy here is Style over substance fallacy: the polish, confidence, charisma, or dramatic force of a presentation is treated as if it established the quality of the argument itself. That matters here because strong delivery can make good arguments easier to hear, but it can also camouflage weak ones. A better analysis would remember that audiences often remember certainty, rhythm, and applause longer than the actual reasoning.
+Source: Associated Press | 2024-06-17
+https://apnews.com/article/33b527ba2785c850b6f473c401bf988b</x:v>
       </x:c>
       <x:c r="W129" t="str">
-        <x:v>AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. — Associated Press | To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery | 2023-11-08 | https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
+        <x:v>To help 2024 voters, Meta says it will begin labeling political ads that use AI-generated imagery
+AP's report on Meta's decision to label AI-generated political ads shows how much public trust can hang on surface cues such as labels, watermarks, and disclosure language. Those cues matter, but they are not substitutes for checking who made a claim or whether the substance is true. The fallacy here is Style over substance fallacy: the polish, confidence, charisma, or dramatic force of a presentation is treated as if it established the quality of the argument itself. That matters here because strong delivery can make good arguments easier to hear, but it can also camouflage weak ones. A better analysis would remember that audiences often remember certainty, rhythm, and applause longer than the actual reasoning.
+Source: Associated Press | 2023-11-08
+https://apnews.com/article/c4aec653d5043a09b1c78b4fb5dcd79b</x:v>
       </x:c>
       <x:c r="X129" t="str">
-        <x:v>AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. — Associated Press | Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots | 2024-11-15 | https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
+        <x:v>Ruben Gallego did better than most Democrats. He says his party needs to stoke working class roots
+AP's November 15, 2024 piece on Ruben Gallego is helpful because it distinguishes authentic narrative connection from cheap identity signaling. It lets a reader ask when biography is relevant evidence about trust and when it becomes a substitute for argument or policy detail. The fallacy here is Style over substance fallacy: the polish, confidence, charisma, or dramatic force of a presentation is treated as if it established the quality of the argument itself. That matters here because strong delivery can make good arguments easier to hear, but it can also camouflage weak ones. A better analysis would remember that audiences often remember certainty, rhythm, and applause longer than the actual reasoning.
+Source: Associated Press | 2024-11-15
+https://apnews.com/article/9f7a1d37047a1f12aad463b53918d735</x:v>
       </x:c>
       <x:c r="Y129" t="str">
-        <x:v>Coverage of the September 10, 2024 Harris-Trump debate often focused on who seemed stronger, calmer, or more in command, which matters politically but does not by itself settle whether the claims on stage were accurate.</x:v>
+        <x:v>Coverage of the September 10, 2024 Harris-Trump debate often focused on who seemed stronger, calmer, or more in command, which matters politically but does not by itself settle whether the claims on stage were accurate. The fallacy here is Style over substance fallacy: the polish, confidence, charisma, or dramatic force of a presentation is treated as if it established the quality of the argument itself. That matters here because strong delivery can make good arguments easier to hear, but it can also camouflage weak ones. A better analysis would remember that audiences often remember certainty, rhythm, and applause longer than the actual reasoning.</x:v>
       </x:c>
       <x:c r="Z129" t="str">
-        <x:v>Short-form video and podcast culture reward confidence, pace, and rhetorical dominance, making it easy for a slick performance to outperform a careful but less theatrical argument.</x:v>
+        <x:v>Short-form video and podcast culture reward confidence, pace, and rhetorical dominance, making it easy for a slick performance to outperform a careful but less theatrical argument. The fallacy here is Style over substance fallacy: the polish, confidence, charisma, or dramatic force of a presentation is treated as if it established the quality of the argument itself. That matters here because strong delivery can make good arguments easier to hear, but it can also camouflage weak ones. A better analysis would remember that audiences often remember certainty, rhythm, and applause longer than the actual reasoning.</x:v>
       </x:c>
       <x:c r="AA129" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -9496,10 +9904,10 @@
         <x:v>Correlative terms such as healthy and unhealthy, free and restricted, informed and uninformed, or biased and impartial depend on contrasts that can be weakened without disappearing.</x:v>
       </x:c>
       <x:c r="V130" t="str">
-        <x:v>Critics sometimes argue that because everyone has some bias, calling a report biased says nothing, as if degrees of distortion and unfairness were impossible.</x:v>
+        <x:v>Critics sometimes argue that because everyone has some bias, calling a report biased says nothing, as if degrees of distortion and unfairness were impossible. The fallacy here is Suppressed correlative: one term in a meaningful contrast is redefined so broadly or so narrowly that its opposing term can no longer do any work. That matters here because correlative terms such as healthy and unhealthy, free and restricted, informed and uninformed, or biased and impartial depend on contrasts that can be weakened without disappearing. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W130" t="str">
-        <x:v>Debates about freedom and censorship often set the positive term to an impossible ideal so that ordinary, useful distinctions collapse.</x:v>
+        <x:v>Debates about freedom and censorship often set the positive term to an impossible ideal so that ordinary, useful distinctions collapse. The fallacy here is Suppressed correlative: one term in a meaningful contrast is redefined so broadly or so narrowly that its opposing term can no longer do any work. That matters here because correlative terms such as healthy and unhealthy, free and restricted, informed and uninformed, or biased and impartial depend on contrasts that can be weakened without disappearing. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X130" t="str"/>
       <x:c r="Y130" t="str"/>
@@ -9565,13 +9973,16 @@
         <x:v>The visible winners are often the easiest cases to notice, but they are not the whole sample. Ignoring the many failed or filtered-out cases makes strategies look safer, smarter, or more effective than they really are.</x:v>
       </x:c>
       <x:c r="V131" t="str">
-        <x:v>Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. — Britannica | Survivorship bias | 2026-01-01 | https://www.britannica.com/science/survivorship-bias</x:v>
+        <x:v>Survivorship bias
+Britannica's overview of survivorship bias, especially its retelling of Abraham Wald's aircraft analysis, is a strong historical case of the visible sample misleading people about the full set. It earns its keep anywhere a page needs a real example of selection effects masquerading as a complete picture. The fallacy here is Survivorship bias: conclusions are drawn from the visible successes that made it through a filter while the failures, dropouts, or non-survivors are ignored. That matters here because the visible winners are often the easiest cases to notice, but they are not the whole sample. A better analysis would remember that ignoring the many failed or filtered-out cases makes strategies look safer, smarter, or more effective than they really are.
+Source: Britannica | 2026-01-01
+https://www.britannica.com/science/survivorship-bias</x:v>
       </x:c>
       <x:c r="W131" t="str">
-        <x:v>Startup and creator advice often highlights spectacular winners while the much larger number of people who copied the same strategy and failed remain largely invisible.</x:v>
+        <x:v>Startup and creator advice often highlights spectacular winners while the much larger number of people who copied the same strategy and failed remain largely invisible. The fallacy here is Survivorship bias: conclusions are drawn from the visible successes that made it through a filter while the failures, dropouts, or non-survivors are ignored. That matters here because the visible winners are often the easiest cases to notice, but they are not the whole sample. A better analysis would remember that ignoring the many failed or filtered-out cases makes strategies look safer, smarter, or more effective than they really are.</x:v>
       </x:c>
       <x:c r="X131" t="str">
-        <x:v>Investment talk routinely showcases the funds, traders, and backtests that survived long enough to look impressive while the dead funds and broken strategies quietly disappear.</x:v>
+        <x:v>Investment talk routinely showcases the funds, traders, and backtests that survived long enough to look impressive while the dead funds and broken strategies quietly disappear. The fallacy here is Survivorship bias: conclusions are drawn from the visible successes that made it through a filter while the failures, dropouts, or non-survivors are ignored. That matters here because the visible winners are often the easiest cases to notice, but they are not the whole sample. A better analysis would remember that ignoring the many failed or filtered-out cases makes strategies look safer, smarter, or more effective than they really are.</x:v>
       </x:c>
       <x:c r="Y131" t="str"/>
       <x:c r="Z131" t="str"/>
@@ -9634,10 +10045,10 @@
         <x:v>Some things really are designed for purposes, but purpose should not be assumed where it has not been shown. Processes can produce outcomes without aiming at them.</x:v>
       </x:c>
       <x:c r="V132" t="str">
-        <x:v>People often speak as if history is automatically bending toward justice, collapse, nationalism, or liberation, as though social change carried its own guaranteed destination.</x:v>
+        <x:v>People often speak as if history is automatically bending toward justice, collapse, nationalism, or liberation, as though social change carried its own guaranteed destination. The fallacy here is Teleological fallacy: a purpose, goal, or final destination is attributed to something without adequate evidence that such an end point was built into it. That matters here because some things really are designed for purposes, but purpose should not be assumed where it has not been shown. A better analysis would remember that processes can produce outcomes without aiming at them.</x:v>
       </x:c>
       <x:c r="W132" t="str">
-        <x:v>In technology debates, AI progress is sometimes framed as if it were inherently marching toward a single destined endpoint such as AGI rather than following contingent technical and social paths.</x:v>
+        <x:v>In technology debates, AI progress is sometimes framed as if it were inherently marching toward a single destined endpoint such as AGI rather than following contingent technical and social paths. The fallacy here is Teleological fallacy: a purpose, goal, or final destination is attributed to something without adequate evidence that such an end point was built into it. That matters here because some things really are designed for purposes, but purpose should not be assumed where it has not been shown. A better analysis would remember that processes can produce outcomes without aiming at them.</x:v>
       </x:c>
       <x:c r="X132" t="str"/>
       <x:c r="Y132" t="str"/>
@@ -9703,10 +10114,10 @@
         <x:v>Aphorisms can be wise shortcuts, but they become fallacious when they replace the reasoning that the situation still requires.</x:v>
       </x:c>
       <x:c r="V133" t="str">
-        <x:v>Phrases such as 'Do your own research,' 'common sense,' or 'if you know, you know' are often used online not to open inquiry but to make further questions look unnecessary or naive.</x:v>
+        <x:v>Phrases such as 'Do your own research,' 'common sense,' or 'if you know, you know' are often used online not to open inquiry but to make further questions look unnecessary or naive. The fallacy here is Thought-terminating cliché: a familiar slogan or stock phrase is used to stop inquiry, deflect scrutiny, or create the feeling that an issue has already been settled. That matters here because aphorisms can be wise shortcuts, but they become fallacious when they replace the reasoning that the situation still requires. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="W133" t="str">
-        <x:v>Political and religious arguments frequently end with slogans like 'Freedom is not free' or 'Only God knows,' which can be meaningful in some contexts but often function as conversation-stoppers.</x:v>
+        <x:v>Political and religious arguments frequently end with slogans like 'Freedom is not free' or 'Only God knows,' which can be meaningful in some contexts but often function as conversation-stoppers. The fallacy here is Thought-terminating cliché: a familiar slogan or stock phrase is used to stop inquiry, deflect scrutiny, or create the feeling that an issue has already been settled. That matters here because aphorisms can be wise shortcuts, but they become fallacious when they replace the reasoning that the situation still requires. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="X133" t="str"/>
       <x:c r="Y133" t="str"/>
@@ -9770,10 +10181,10 @@
         <x:v>A vivid case can motivate investigation, but it does not by itself justify a population-level conclusion.</x:v>
       </x:c>
       <x:c r="V134" t="str">
-        <x:v>Isolated crime stories are often turned into sweeping claims about immigrants, professions, age groups, or political movements.</x:v>
+        <x:v>Isolated crime stories are often turned into sweeping claims about immigrants, professions, age groups, or political movements. The fallacy here is Top-down condemnation: a negative trait found in one member of a group is used to condemn the group as a whole. That matters here because a vivid case can motivate investigation, but it does not by itself justify a population-level conclusion. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W134" t="str">
-        <x:v>A single corporate scandal can quickly become a claim that the entire industry is rotten in exactly the same way.</x:v>
+        <x:v>A single corporate scandal can quickly become a claim that the entire industry is rotten in exactly the same way. The fallacy here is Top-down condemnation: a negative trait found in one member of a group is used to condemn the group as a whole. That matters here because a vivid case can motivate investigation, but it does not by itself justify a population-level conclusion. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X134" t="str"/>
       <x:c r="Y134" t="str"/>
@@ -9845,10 +10256,10 @@
         <x:v>Generalizations are often default-pattern claims, not exceptionless universal laws.</x:v>
       </x:c>
       <x:c r="V135" t="str">
-        <x:v>Public-health advice is often dismissed by pointing to unusual edge cases even when the advice was clearly aimed at ordinary conditions.</x:v>
+        <x:v>Public-health advice is often dismissed by pointing to unusual edge cases even when the advice was clearly aimed at ordinary conditions. The fallacy here is Top-down faulty generalization: a reasonable generalization is attacked by demanding that it hold without relevant scope conditions or exceptions. That matters here because generalizations are often default-pattern claims, not exceptionless universal laws. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W135" t="str">
-        <x:v>Safety rules and economic patterns are frequently challenged by exceptions that do not actually undermine the broader tendency being described.</x:v>
+        <x:v>Safety rules and economic patterns are frequently challenged by exceptions that do not actually undermine the broader tendency being described. The fallacy here is Top-down faulty generalization: a reasonable generalization is attacked by demanding that it hold without relevant scope conditions or exceptions. That matters here because generalizations are often default-pattern claims, not exceptionless universal laws. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X135" t="str"/>
       <x:c r="Y135" t="str"/>
@@ -9912,10 +10323,10 @@
         <x:v>A favorable anecdote can remind us not to overgeneralize negatively, but it cannot prove that the larger class is generally positive.</x:v>
       </x:c>
       <x:c r="V136" t="str">
-        <x:v>One transparent politician or one ethical corporation is often used to imply that the surrounding system is healthier than the broader evidence suggests.</x:v>
+        <x:v>One transparent politician or one ethical corporation is often used to imply that the surrounding system is healthier than the broader evidence suggests. The fallacy here is Top-down justification: a positive trait found in one member of a group is used to justify a positive conclusion about the group as a whole. That matters here because a favorable anecdote can remind us not to overgeneralize negatively, but it cannot prove that the larger class is generally positive. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="W136" t="str">
-        <x:v>People frequently infer that an institution is trustworthy because they personally encountered one helpful employee inside it.</x:v>
+        <x:v>People frequently infer that an institution is trustworthy because they personally encountered one helpful employee inside it. The fallacy here is Top-down justification: a positive trait found in one member of a group is used to justify a positive conclusion about the group as a whole. That matters here because a favorable anecdote can remind us not to overgeneralize negatively, but it cannot prove that the larger class is generally positive. The better question is whether the category or definition still fits once the context or scale changes.</x:v>
       </x:c>
       <x:c r="X136" t="str"/>
       <x:c r="Y136" t="str"/>
@@ -9975,10 +10386,10 @@
         <x:v>A track record does not make contrary outcomes impossible, but it does affect rational priors. Ignoring repeated past failure forces every new case to borrow more credibility than it has earned.</x:v>
       </x:c>
       <x:c r="V137" t="str">
-        <x:v>Baseless claims about widespread noncitizen voting keep getting relaunched as if decades of rarity, audits, and failed alarms provide no reason for initial skepticism.</x:v>
+        <x:v>Baseless claims about widespread noncitizen voting keep getting relaunched as if decades of rarity, audits, and failed alarms provide no reason for initial skepticism. The fallacy here is Track-record reset: each new claim is treated as if the relevant history of prior failures, hoaxes, or false alarms did not exist and should confer no default expectation at all. That matters here because a track record does not make contrary outcomes impossible, but it does affect rational priors. A better analysis would remember that ignoring repeated past failure forces every new case to borrow more credibility than it has earned.</x:v>
       </x:c>
       <x:c r="W137" t="str">
-        <x:v>Every new blurry UFO clip, miracle cure, or ghost story is often pitched as if the long record of ordinary explanations should have zero effect on our starting expectations.</x:v>
+        <x:v>Every new blurry UFO clip, miracle cure, or ghost story is often pitched as if the long record of ordinary explanations should have zero effect on our starting expectations. The fallacy here is Track-record reset: each new claim is treated as if the relevant history of prior failures, hoaxes, or false alarms did not exist and should confer no default expectation at all. That matters here because a track record does not make contrary outcomes impossible, but it does affect rational priors. A better analysis would remember that ignoring repeated past failure forces every new case to borrow more credibility than it has earned.</x:v>
       </x:c>
       <x:c r="X137" t="str"/>
       <x:c r="Y137" t="str"/>
@@ -10048,13 +10459,16 @@
         <x:v>Hypocrisy can matter for trust, but it does not by itself answer whether the original claim, act, or argument was wrong.</x:v>
       </x:c>
       <x:c r="V138" t="str">
-        <x:v>AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. — Associated Press | Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement | 2024-09-10 | https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
+        <x:v>Key takeaways from a debate that featured tense clashes and closed with a Taylor Swift endorsement
+AP's September 10, 2024 debate takeaway piece captures how often nationally watched debates pivot on baiting, reframing, crowd-pleasing jabs, and memorable lines rather than patient argument. It is a compact real-world lab for straw manning, redirection, and emotionally charged reframing. The fallacy here is Tu quoque: criticism is answered not by engaging the issue, but by pointing to similar hypocrisy or wrongdoing elsewhere. That matters here because hypocrisy can matter for trust, but it does not by itself answer whether the original claim, act, or argument was wrong. The better question is whether the original claim has been answered rather than sidestepped or reframed.
+Source: Associated Press | 2024-09-10
+https://www.ap.org/news-highlights/elections/2024/key-takeaways-from-a-debate-that-featured-tense-clashes-and-closed-with-a-taylor-swift-endorsement/</x:v>
       </x:c>
       <x:c r="W138" t="str">
-        <x:v>In the June 27, 2024 Biden-Trump debate and the September 10, 2024 Harris-Trump debate, many charges were met with 'your side did it too' responses that redirected blame without addressing the original allegation.</x:v>
+        <x:v>In the June 27, 2024 Biden-Trump debate and the September 10, 2024 Harris-Trump debate, many charges were met with 'your side did it too' responses that redirected blame without addressing the original allegation. The fallacy here is Tu quoque: criticism is answered not by engaging the issue, but by pointing to similar hypocrisy or wrongdoing elsewhere. That matters here because hypocrisy can matter for trust, but it does not by itself answer whether the original claim, act, or argument was wrong. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="X138" t="str">
-        <x:v>Arguments about misinformation, climate, religion, and media bias often slide into scorekeeping about who is worse rather than whether the specific criticized claim is true or justified.</x:v>
+        <x:v>Arguments about misinformation, climate, religion, and media bias often slide into scorekeeping about who is worse rather than whether the specific criticized claim is true or justified. The fallacy here is Tu quoque: criticism is answered not by engaging the issue, but by pointing to similar hypocrisy or wrongdoing elsewhere. That matters here because hypocrisy can matter for trust, but it does not by itself answer whether the original claim, act, or argument was wrong. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="Y138" t="str"/>
       <x:c r="Z138" t="str"/>
@@ -10121,10 +10535,10 @@
         <x:v>Exposing hypocrisy can matter, but retaliation does not erase the original wrong or magically sanitize a copy of it.</x:v>
       </x:c>
       <x:c r="V139" t="str">
-        <x:v>In 2024 election discourse, misinformation was often excused with the claim that the other side lies too, as if symmetry or revenge transformed falsehood into fairness.</x:v>
+        <x:v>In 2024 election discourse, misinformation was often excused with the claim that the other side lies too, as if symmetry or revenge transformed falsehood into fairness. The fallacy here is Two wrongs make a right: someone treats one wrong act as justified because it responds to, retaliates against, or balances out another wrong. That matters here because exposing hypocrisy can matter, but retaliation does not erase the original wrong or magically sanitize a copy of it. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="W139" t="str">
-        <x:v>Debates about censorship, doxxing, and dirty campaign tactics often slide from condemnation into imitation, with each side treating the other's bad behavior as a license to do the same.</x:v>
+        <x:v>Debates about censorship, doxxing, and dirty campaign tactics often slide from condemnation into imitation, with each side treating the other's bad behavior as a license to do the same. The fallacy here is Two wrongs make a right: someone treats one wrong act as justified because it responds to, retaliates against, or balances out another wrong. That matters here because exposing hypocrisy can matter, but retaliation does not erase the original wrong or magically sanitize a copy of it. The better question is whether the original claim has been answered rather than sidestepped or reframed.</x:v>
       </x:c>
       <x:c r="X139" t="str"/>
       <x:c r="Y139" t="str"/>
@@ -10188,13 +10602,16 @@
         <x:v>Sharing a feature does not establish identity or class inclusion unless the shared feature actually covers the whole relevant group. A middle term can connect without unifying.</x:v>
       </x:c>
       <x:c r="V140" t="str">
-        <x:v>AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. — NPR | Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not | 2024-10-12 | https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
+        <x:v>Fact-check: Trump keeps claiming noncitizen voting is a big problem. It's not
+AP and NPR both showed how a few real or suspected ineligible votes were repeatedly used to argue that federal elections are broadly compromised. The jump from a narrow premise to a sweeping conclusion is exactly why formal discipline matters in public reasoning. The fallacy here is Undistributed middle: two things are linked to the same broader category and the argument wrongly infers that one of them must therefore be the other. That matters here because sharing a feature does not establish identity or class inclusion unless the shared feature actually covers the whole relevant group. A better analysis would remember that a middle term can connect without unifying.
+Source: NPR | 2024-10-12
+https://www.npr.org/2024/10/12/nx-s1-5147789/voting-election-2024-noncitizen-fact-check</x:v>
       </x:c>
       <x:c r="W140" t="str">
-        <x:v>Lifestyle and identity marketing often says 'the cool do X' and 'I do X,' then slides to 'therefore I am one of the cool,' even though the shared feature is too broad.</x:v>
+        <x:v>Lifestyle and identity marketing often says 'the cool do X' and 'I do X,' then slides to 'therefore I am one of the cool,' even though the shared feature is too broad. The fallacy here is Undistributed middle: two things are linked to the same broader category and the argument wrongly infers that one of them must therefore be the other. That matters here because sharing a feature does not establish identity or class inclusion unless the shared feature actually covers the whole relevant group. A better analysis would remember that a middle term can connect without unifying.</x:v>
       </x:c>
       <x:c r="X140" t="str">
-        <x:v>Political commentary frequently infers that because two camps are skeptical of the same institution or support the same policy, they must belong to the same underlying movement.</x:v>
+        <x:v>Political commentary frequently infers that because two camps are skeptical of the same institution or support the same policy, they must belong to the same underlying movement. The fallacy here is Undistributed middle: two things are linked to the same broader category and the argument wrongly infers that one of them must therefore be the other. That matters here because sharing a feature does not establish identity or class inclusion unless the shared feature actually covers the whole relevant group. A better analysis would remember that a middle term can connect without unifying.</x:v>
       </x:c>
       <x:c r="Y140" t="str"/>
       <x:c r="Z140" t="str"/>
@@ -10253,10 +10670,10 @@
         <x:v>Vagueness can be useful early in exploration, but it becomes fallacious when the fog is preserved to prevent serious evaluation. If key terms cannot be pinned down, the claim can keep slipping away from critique.</x:v>
       </x:c>
       <x:c r="V141" t="str">
-        <x:v>Alternative-health and wellness marketing often leans on words like 'toxins,' 'energy,' 'balance,' and 'boost' precisely because they sound scientific while remaining hard to falsify.</x:v>
+        <x:v>Alternative-health and wellness marketing often leans on words like 'toxins,' 'energy,' 'balance,' and 'boost' precisely because they sound scientific while remaining hard to falsify. The fallacy here is Vague insulators: vague, elastic, or undefined terms are chosen so that a position sounds meaningful while resisting clear testing or criticism. That matters here because vagueness can be useful early in exploration, but it becomes fallacious when the fog is preserved to prevent serious evaluation. A better analysis would remember that if key terms cannot be pinned down, the claim can keep slipping away from critique.</x:v>
       </x:c>
       <x:c r="W141" t="str">
-        <x:v>In arguments about spirituality, self-help, and even AI, flexible phrases can be stretched to fit almost any outcome, which makes the view feel resilient without making it well supported.</x:v>
+        <x:v>In arguments about spirituality, self-help, and even AI, flexible phrases can be stretched to fit almost any outcome, which makes the view feel resilient without making it well supported. The fallacy here is Vague insulators: vague, elastic, or undefined terms are chosen so that a position sounds meaningful while resisting clear testing or criticism. That matters here because vagueness can be useful early in exploration, but it becomes fallacious when the fog is preserved to prevent serious evaluation. A better analysis would remember that if key terms cannot be pinned down, the claim can keep slipping away from critique.</x:v>
       </x:c>
       <x:c r="X141" t="str"/>
       <x:c r="Y141" t="str"/>
@@ -10328,19 +10745,28 @@
         <x:v>Hope can sustain action, but it does not convert possibility into evidence. The stronger the desire, the easier it is to mistake wanting for warrant.</x:v>
       </x:c>
       <x:c r="V142" t="str">
-        <x:v>In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. — Associated Press | Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist | 2024-05-06 | https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
+        <x:v>Brad Parscale helped Trump win in 2016 using Facebook ads. Now he's back, and an AI evangelist
+In AP's profile of Brad Parscale's AI evangelism, campaign technology is repeatedly framed as inherently superior because it is new, disruptive, and supposedly closer to what voters really want. That is exactly the kind of setting where novelty, confidence, and prestige can outrun evidence. The fallacy here is Wishful thinking: a belief or decision is driven mainly by what would be pleasing, hopeful, or comforting if true rather than by what the evidence supports. That matters here because hope can sustain action, but it does not convert possibility into evidence. A better analysis would remember that the stronger the desire, the easier it is to mistake wanting for warrant.
+Source: Associated Press | 2024-05-06
+https://apnews.com/article/3ff2c8eba34b87754cc25e96aa257c9d</x:v>
       </x:c>
       <x:c r="W142" t="str">
-        <x:v>AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. — Associated Press | Raw milk from a California dairy is recalled after routine testing detected the bird flu virus | 2024-11-25 | https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
+        <x:v>Raw milk from a California dairy is recalled after routine testing detected the bird flu virus
+AP's November 25, 2024 report on raw milk recalled after bird-flu detection is a good case for arguments that romanticize the 'natural' while minimizing risk. It makes the tradeoff concrete: appeals to purity and tradition can feel reassuring even when the biological evidence points the other way. The fallacy here is Wishful thinking: a belief or decision is driven mainly by what would be pleasing, hopeful, or comforting if true rather than by what the evidence supports. That matters here because hope can sustain action, but it does not convert possibility into evidence. A better analysis would remember that the stronger the desire, the easier it is to mistake wanting for warrant.
+Source: Associated Press | 2024-11-25
+https://apnews.com/article/b7ac9c95db99d367b2932f0de16e5821</x:v>
       </x:c>
       <x:c r="X142" t="str">
-        <x:v>PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. — PolitiFact | How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online | 2024-09-20 | https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
+        <x:v>How an unsubstantiated, anonymous affidavit about the ABC presidential debate was amplified online
+PolitiFact's September 20, 2024 reconstruction of the fake ABC whistleblower affidavit is especially valuable because it shows how public figures shared the claim while conceding they did not know whether it was true. That is a live, well-documented case of conjecture and amplification outrunning authentication. The fallacy here is Wishful thinking: a belief or decision is driven mainly by what would be pleasing, hopeful, or comforting if true rather than by what the evidence supports. That matters here because hope can sustain action, but it does not convert possibility into evidence. A better analysis would remember that the stronger the desire, the easier it is to mistake wanting for warrant.
+Source: PolitiFact | 2024-09-20
+https://www.politifact.com/article/2024/sep/20/Fact-checking-ABC-debate-whistleblower-affidavit/</x:v>
       </x:c>
       <x:c r="Y142" t="str">
-        <x:v>Speculative markets, miracle-cure promises, and election-night narratives often run on the thought that a hoped-for outcome is somehow more likely because people badly want it.</x:v>
+        <x:v>Speculative markets, miracle-cure promises, and election-night narratives often run on the thought that a hoped-for outcome is somehow more likely because people badly want it. The fallacy here is Wishful thinking: a belief or decision is driven mainly by what would be pleasing, hopeful, or comforting if true rather than by what the evidence supports. That matters here because hope can sustain action, but it does not convert possibility into evidence. A better analysis would remember that the stronger the desire, the easier it is to mistake wanting for warrant.</x:v>
       </x:c>
       <x:c r="Z142" t="str">
-        <x:v>Beliefs about the afterlife, destiny, or technological salvation are often defended by saying life would feel bleak without them, which speaks to desire rather than truth.</x:v>
+        <x:v>Beliefs about the afterlife, destiny, or technological salvation are often defended by saying life would feel bleak without them, which speaks to desire rather than truth. The fallacy here is Wishful thinking: a belief or decision is driven mainly by what would be pleasing, hopeful, or comforting if true rather than by what the evidence supports. That matters here because hope can sustain action, but it does not convert possibility into evidence. A better analysis would remember that the stronger the desire, the easier it is to mistake wanting for warrant.</x:v>
       </x:c>
       <x:c r="AA142" t="str">
         <x:v>modernized-2026-pass</x:v>
@@ -10399,10 +10825,10 @@
         <x:v>Real corroboration requires accessible, independent testimony or records. Simply claiming that more witnesses exist adds almost nothing if the chain cannot be examined.</x:v>
       </x:c>
       <x:c r="V143" t="str">
-        <x:v>Paranormal, religious, and conspiracy stories often swell in authority by invoking unnamed doctors, secret insiders, or hundreds of silent observers who never become independently available.</x:v>
+        <x:v>Paranormal, religious, and conspiracy stories often swell in authority by invoking unnamed doctors, secret insiders, or hundreds of silent observers who never become independently available. The fallacy here is Witness chain: testimony is padded by unverifiable references to other alleged witnesses, creating the illusion of corroboration without actually providing independent support. That matters here because real corroboration requires accessible, independent testimony or records. A better analysis would remember that simply claiming that more witnesses exist adds almost nothing if the chain cannot be examined.</x:v>
       </x:c>
       <x:c r="W143" t="str">
-        <x:v>Historical arguments sometimes treat a late report that 'many people saw it' as if that were the same thing as actually having many separate testimonies.</x:v>
+        <x:v>Historical arguments sometimes treat a late report that 'many people saw it' as if that were the same thing as actually having many separate testimonies. The fallacy here is Witness chain: testimony is padded by unverifiable references to other alleged witnesses, creating the illusion of corroboration without actually providing independent support. That matters here because real corroboration requires accessible, independent testimony or records. A better analysis would remember that simply claiming that more witnesses exist adds almost nothing if the chain cannot be examined.</x:v>
       </x:c>
       <x:c r="X143" t="str"/>
       <x:c r="Y143" t="str"/>
@@ -10466,16 +10892,22 @@
         <x:v>Correlations can be real while still pointing the wrong way. Without evidence about timing, mechanism, and alternatives, reversing cause and effect is easy.</x:v>
       </x:c>
       <x:c r="V144" t="str">
-        <x:v>When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. — Associated Press | Google makes fixes to AI-generated search summaries after outlandish answers went viral | 2024-05-31 | https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
+        <x:v>Google makes fixes to AI-generated search summaries after outlandish answers went viral
+When AP covered Google's erroneous AI overviews, the central lesson was that a system can sound authoritative while still misreading queries, flattening context, or repeating bad source material. The episode is a strong real-world case of surface fluency masking evidential and conceptual weakness. The fallacy here is Wrong causal direction: a real association is noticed but the direction of causation is reversed. That matters here because correlations can be real while still pointing the wrong way. A better analysis would remember that without evidence about timing, mechanism, and alternatives, reversing cause and effect is easy.
+Source: Associated Press | 2024-05-31
+https://apnews.com/article/33060569d6cc01abe6c63d21665330d8</x:v>
       </x:c>
       <x:c r="W144" t="str">
-        <x:v>FactCheck.org's May 2024 H5N1 explainer is a strong illustration of why people n